<commit_message>
Update VETUSDT.json at 2024-04-16_05-27-54 bestfile_scores 0.000665353939689467 bestfile_sharp 0.1868295345238975
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -16197,10 +16197,10 @@
         <v>93</v>
       </c>
       <c r="F57">
-        <v>0.000154025130411517</v>
+        <v>0.001255627512428914</v>
       </c>
       <c r="G57">
-        <v>0.000154025130411517</v>
+        <v>0.001255627512428914</v>
       </c>
       <c r="H57">
         <v>0</v>
@@ -16209,10 +16209,10 @@
         <v>0</v>
       </c>
       <c r="J57">
-        <v>0.0001482679723446401</v>
+        <v>0.001511295891833742</v>
       </c>
       <c r="K57">
-        <v>0.0001482679723446401</v>
+        <v>0.001511295891833742</v>
       </c>
       <c r="L57">
         <v>0</v>
@@ -16221,34 +16221,34 @@
         <v>0</v>
       </c>
       <c r="N57">
-        <v>5.209460241521664</v>
+        <v>12.24399089471044</v>
       </c>
       <c r="O57">
         <v>0</v>
       </c>
       <c r="P57">
-        <v>0.9963190045831128</v>
+        <v>0.9895028336871218</v>
       </c>
       <c r="Q57">
         <v>1</v>
       </c>
       <c r="R57">
-        <v>0.00713668921833699</v>
+        <v>0.07141033092501393</v>
       </c>
       <c r="S57">
         <v>-0</v>
       </c>
       <c r="T57">
-        <v>0.1451708804264108</v>
+        <v>0.1944349051639195</v>
       </c>
       <c r="U57">
         <v>-0</v>
       </c>
       <c r="V57">
-        <v>0.999838157299978</v>
+        <v>0.9991155438640293</v>
       </c>
       <c r="W57">
-        <v>0.9674531602458458</v>
+        <v>0.8449450491025632</v>
       </c>
       <c r="X57">
         <v>1</v>
@@ -16257,22 +16257,22 @@
         <v>1</v>
       </c>
       <c r="Z57">
-        <v>0.8299040129128529</v>
+        <v>0.8055960619595565</v>
       </c>
       <c r="AB57">
-        <v>0.001212817412848336</v>
+        <v>0.005896068918155522</v>
       </c>
       <c r="AC57">
         <v>0</v>
       </c>
       <c r="AD57">
-        <v>0.999838157299978</v>
+        <v>0.9991155438640293</v>
       </c>
       <c r="AE57">
         <v>1</v>
       </c>
       <c r="AF57">
-        <v>0.001212817412848336</v>
+        <v>0.005896068918155522</v>
       </c>
       <c r="AG57">
         <v>0</v>
@@ -16281,55 +16281,55 @@
         <v>202</v>
       </c>
       <c r="AI57">
-        <v>0.005641087347138496</v>
+        <v>0.04413639627430367</v>
       </c>
       <c r="AJ57">
         <v>0</v>
       </c>
       <c r="AK57">
-        <v>-86.434132078</v>
+        <v>-1317.16180684</v>
       </c>
       <c r="AL57">
         <v>0</v>
       </c>
       <c r="AM57">
-        <v>11809.6029179222</v>
+        <v>38774.3858131602</v>
       </c>
       <c r="AN57">
         <v>10000</v>
       </c>
       <c r="AO57">
-        <v>11809.6029179222</v>
+        <v>38774.3858131602</v>
       </c>
       <c r="AP57">
         <v>10000</v>
       </c>
       <c r="AQ57">
-        <v>0.1809602917922204</v>
+        <v>2.877438581316019</v>
       </c>
       <c r="AR57">
         <v>0</v>
       </c>
       <c r="AS57">
-        <v>4.604462222222222</v>
+        <v>1.959059395956235</v>
       </c>
       <c r="AU57">
-        <v>130.25</v>
+        <v>116.6166666666667</v>
       </c>
       <c r="AW57">
-        <v>0</v>
+        <v>0.1259501256736581</v>
       </c>
       <c r="AX57">
         <v>1</v>
       </c>
       <c r="AY57">
-        <v>0</v>
+        <v>-4336.176133398528</v>
       </c>
       <c r="AZ57">
         <v>0</v>
       </c>
       <c r="BA57">
-        <v>2218</v>
+        <v>4105</v>
       </c>
       <c r="BB57">
         <v>0</v>
@@ -16338,37 +16338,37 @@
         <v>1079.958333333333</v>
       </c>
       <c r="BD57">
+        <v>9118</v>
+      </c>
+      <c r="BE57">
+        <v>0</v>
+      </c>
+      <c r="BF57">
+        <v>13223</v>
+      </c>
+      <c r="BG57">
+        <v>0</v>
+      </c>
+      <c r="BH57">
         <v>3408</v>
       </c>
-      <c r="BE57">
-        <v>0</v>
-      </c>
-      <c r="BF57">
-        <v>5626</v>
-      </c>
-      <c r="BG57">
-        <v>0</v>
-      </c>
-      <c r="BH57">
-        <v>2161</v>
-      </c>
       <c r="BI57">
         <v>0</v>
       </c>
       <c r="BJ57">
-        <v>2218</v>
+        <v>4025</v>
       </c>
       <c r="BK57">
         <v>0</v>
       </c>
       <c r="BL57">
-        <v>1247</v>
+        <v>5710</v>
       </c>
       <c r="BM57">
         <v>0</v>
       </c>
       <c r="BN57">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="BO57">
         <v>0</v>
@@ -16380,49 +16380,49 @@
         <v>0</v>
       </c>
       <c r="BR57">
-        <v>1809.602917921998</v>
+        <v>28774.38581315999</v>
       </c>
       <c r="BS57">
         <v>0</v>
       </c>
       <c r="BT57">
-        <v>0.06022724746414452</v>
+        <v>0.0555443318163657</v>
       </c>
       <c r="BU57">
         <v>100</v>
       </c>
       <c r="BV57">
-        <v>0.1691115204496482</v>
+        <v>0.2413107224056973</v>
       </c>
       <c r="BW57">
         <v>100</v>
       </c>
       <c r="BX57">
-        <v>0.02061302756247461</v>
+        <v>0.01048418681402411</v>
       </c>
       <c r="BY57">
         <v>100</v>
       </c>
       <c r="BZ57">
-        <v>0.01561218761449268</v>
+        <v>0.01042009946556962</v>
       </c>
       <c r="CA57">
         <v>1</v>
       </c>
       <c r="CB57">
-        <v>1896.037049999998</v>
+        <v>30091.54761999999</v>
       </c>
       <c r="CC57">
         <v>0</v>
       </c>
       <c r="CD57">
-        <v>1896.037049999998</v>
+        <v>34427.72375339852</v>
       </c>
       <c r="CE57">
         <v>0</v>
       </c>
       <c r="CF57">
-        <v>0.1513081642703564</v>
+        <v>0.1666791844316405</v>
       </c>
       <c r="CG57">
         <v>0</v>
@@ -16431,22 +16431,22 @@
         <v>10000</v>
       </c>
       <c r="CJ57">
-        <v>7.716049382716049E-05</v>
+        <v>0.006674382716049383</v>
       </c>
       <c r="CK57">
         <v>0</v>
       </c>
       <c r="CL57">
-        <v>984454.406228471</v>
+        <v>25924377.11451623</v>
       </c>
       <c r="CM57">
         <v>0</v>
       </c>
       <c r="CN57" s="2">
-        <v>45398.05377800363</v>
+        <v>45398.15244287193</v>
       </c>
       <c r="CO57">
-        <v>-0.9943954266380367</v>
+        <v>-0.7777179486581601</v>
       </c>
       <c r="CP57">
         <v>-0.9999999999999732</v>

</xml_diff>

<commit_message>
Update VETUSDT.json at 2024-04-16_10-21-11 bestfile_scores 0.000934310639338648 bestfile_sharp 0.2597294059399704
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="257">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -298,6 +298,9 @@
     <t>OCEANUSDT</t>
   </si>
   <si>
+    <t>VETUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -569,9 +572,6 @@
   </si>
   <si>
     <t>EOSUSDT</t>
-  </si>
-  <si>
-    <t>VETUSDT</t>
   </si>
   <si>
     <t>AXSUSDT</t>
@@ -1146,7 +1146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP57"/>
+  <dimension ref="A1:CP58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1435,16 +1435,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1701,16 +1701,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E3" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1967,13 +1967,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2233,16 +2233,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2499,16 +2499,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2765,16 +2765,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -3031,16 +3031,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3297,16 +3297,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3563,16 +3563,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3829,16 +3829,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E11" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -4095,16 +4095,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4361,16 +4361,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E13" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4627,16 +4627,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4893,16 +4893,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -5159,16 +5159,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D16" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E16" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5425,16 +5425,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D17" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5691,16 +5691,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5957,16 +5957,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E19" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6223,16 +6223,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E20" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6489,16 +6489,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D21" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6755,16 +6755,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -7021,16 +7021,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E23" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7287,16 +7287,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D24" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E24" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7553,16 +7553,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D25" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E25" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7819,16 +7819,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D26" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E26" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -8085,16 +8085,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E27" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8351,16 +8351,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D28" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8617,16 +8617,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D29" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E29" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8883,16 +8883,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D30" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E30" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -9149,16 +9149,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D31" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E31" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9415,16 +9415,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D32" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E32" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9681,16 +9681,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D33" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9947,16 +9947,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D34" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E34" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10219,16 +10219,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D35" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E35" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10491,16 +10491,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E36" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10763,16 +10763,16 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E37" t="s">
-        <v>185</v>
+        <v>94</v>
       </c>
       <c r="F37">
         <v>0.001640077</v>
@@ -11035,13 +11035,13 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E38" t="s">
         <v>186</v>
@@ -11307,13 +11307,13 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D39" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E39" t="s">
         <v>187</v>
@@ -11579,13 +11579,13 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C40" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D40" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E40" t="s">
         <v>188</v>
@@ -11851,13 +11851,13 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C41" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D41" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E41" t="s">
         <v>189</v>
@@ -12123,13 +12123,13 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E42" t="s">
         <v>190</v>
@@ -12395,13 +12395,13 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D43" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E43" t="s">
         <v>191</v>
@@ -12667,13 +12667,13 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D44" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E44" t="s">
         <v>192</v>
@@ -12939,13 +12939,13 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C45" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D45" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E45" t="s">
         <v>193</v>
@@ -13211,13 +13211,13 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D46" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E46" t="s">
         <v>194</v>
@@ -13483,13 +13483,13 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D47" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E47" t="s">
         <v>195</v>
@@ -13755,13 +13755,13 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E48" t="s">
         <v>196</v>
@@ -14027,13 +14027,13 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D49" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E49" t="s">
         <v>197</v>
@@ -14299,13 +14299,13 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D50" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E50" t="s">
         <v>198</v>
@@ -14571,13 +14571,13 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D51" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E51" t="s">
         <v>199</v>
@@ -14843,13 +14843,13 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D52" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E52" t="s">
         <v>200</v>
@@ -15115,13 +15115,13 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E53" t="s">
         <v>201</v>
@@ -15387,16 +15387,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C54" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15659,13 +15659,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C55" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E55" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15928,10 +15928,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E56" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16449,6 +16449,269 @@
         <v>-0.7777179486581601</v>
       </c>
       <c r="CP57">
+        <v>-0.9999999999999732</v>
+      </c>
+    </row>
+    <row r="58" spans="1:94">
+      <c r="A58" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E58" t="s">
+        <v>94</v>
+      </c>
+      <c r="F58">
+        <v>0.001364122639297527</v>
+      </c>
+      <c r="G58">
+        <v>0.001364122639297527</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>0</v>
+      </c>
+      <c r="J58">
+        <v>0.001297293119460341</v>
+      </c>
+      <c r="K58">
+        <v>0.001297293119460341</v>
+      </c>
+      <c r="L58">
+        <v>0</v>
+      </c>
+      <c r="M58">
+        <v>0</v>
+      </c>
+      <c r="N58">
+        <v>24.21316856536011</v>
+      </c>
+      <c r="O58">
+        <v>0</v>
+      </c>
+      <c r="P58">
+        <v>0.9997949931923897</v>
+      </c>
+      <c r="Q58">
+        <v>1</v>
+      </c>
+      <c r="R58">
+        <v>0.06237148478473695</v>
+      </c>
+      <c r="S58">
+        <v>-0</v>
+      </c>
+      <c r="T58">
+        <v>0.1539017749998078</v>
+      </c>
+      <c r="U58">
+        <v>-0</v>
+      </c>
+      <c r="V58">
+        <v>0.9992642599845767</v>
+      </c>
+      <c r="W58">
+        <v>0.8882982556401527</v>
+      </c>
+      <c r="X58">
+        <v>1</v>
+      </c>
+      <c r="Y58">
+        <v>1</v>
+      </c>
+      <c r="Z58">
+        <v>0.873386993376827</v>
+      </c>
+      <c r="AB58">
+        <v>0.005243039178105519</v>
+      </c>
+      <c r="AC58">
+        <v>0</v>
+      </c>
+      <c r="AD58">
+        <v>0.9992642599845767</v>
+      </c>
+      <c r="AE58">
+        <v>1</v>
+      </c>
+      <c r="AF58">
+        <v>0.005243039178105519</v>
+      </c>
+      <c r="AG58">
+        <v>0</v>
+      </c>
+      <c r="AH58" t="s">
+        <v>202</v>
+      </c>
+      <c r="AI58">
+        <v>0.03707838267375759</v>
+      </c>
+      <c r="AJ58">
+        <v>0</v>
+      </c>
+      <c r="AK58">
+        <v>-2866.9001878604</v>
+      </c>
+      <c r="AL58">
+        <v>0</v>
+      </c>
+      <c r="AM58">
+        <v>43528.4007141399</v>
+      </c>
+      <c r="AN58">
+        <v>10000</v>
+      </c>
+      <c r="AO58">
+        <v>43528.4007141399</v>
+      </c>
+      <c r="AP58">
+        <v>10000</v>
+      </c>
+      <c r="AQ58">
+        <v>3.35284007141399</v>
+      </c>
+      <c r="AR58">
+        <v>0</v>
+      </c>
+      <c r="AS58">
+        <v>0.9903358342265095</v>
+      </c>
+      <c r="AU58">
+        <v>83.95</v>
+      </c>
+      <c r="AW58">
+        <v>0.0715786876751517</v>
+      </c>
+      <c r="AX58">
+        <v>1</v>
+      </c>
+      <c r="AY58">
+        <v>-2805.97595243043</v>
+      </c>
+      <c r="AZ58">
+        <v>0</v>
+      </c>
+      <c r="BA58">
+        <v>10727</v>
+      </c>
+      <c r="BB58">
+        <v>0</v>
+      </c>
+      <c r="BC58">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BD58">
+        <v>15398</v>
+      </c>
+      <c r="BE58">
+        <v>0</v>
+      </c>
+      <c r="BF58">
+        <v>26125</v>
+      </c>
+      <c r="BG58">
+        <v>0</v>
+      </c>
+      <c r="BH58">
+        <v>10643</v>
+      </c>
+      <c r="BI58">
+        <v>0</v>
+      </c>
+      <c r="BJ58">
+        <v>10657</v>
+      </c>
+      <c r="BK58">
+        <v>0</v>
+      </c>
+      <c r="BL58">
+        <v>4755</v>
+      </c>
+      <c r="BM58">
+        <v>0</v>
+      </c>
+      <c r="BN58">
+        <v>70</v>
+      </c>
+      <c r="BO58">
+        <v>0</v>
+      </c>
+      <c r="BP58">
+        <v>0</v>
+      </c>
+      <c r="BQ58">
+        <v>0</v>
+      </c>
+      <c r="BR58">
+        <v>33528.4007141396</v>
+      </c>
+      <c r="BS58">
+        <v>0</v>
+      </c>
+      <c r="BT58">
+        <v>0.05244279254971655</v>
+      </c>
+      <c r="BU58">
+        <v>100</v>
+      </c>
+      <c r="BV58">
+        <v>0.1449461011079747</v>
+      </c>
+      <c r="BW58">
+        <v>100</v>
+      </c>
+      <c r="BX58">
+        <v>0.006422810151173568</v>
+      </c>
+      <c r="BY58">
+        <v>100</v>
+      </c>
+      <c r="BZ58">
+        <v>0.007638975474069304</v>
+      </c>
+      <c r="CA58">
+        <v>1</v>
+      </c>
+      <c r="CB58">
+        <v>36395.300902</v>
+      </c>
+      <c r="CC58">
+        <v>0</v>
+      </c>
+      <c r="CD58">
+        <v>39201.27685443043</v>
+      </c>
+      <c r="CE58">
+        <v>0</v>
+      </c>
+      <c r="CF58">
+        <v>0.1868295345238975</v>
+      </c>
+      <c r="CG58">
+        <v>0</v>
+      </c>
+      <c r="CH58">
+        <v>10000</v>
+      </c>
+      <c r="CJ58">
+        <v>0.01795644114921223</v>
+      </c>
+      <c r="CK58">
+        <v>0</v>
+      </c>
+      <c r="CL58">
+        <v>12238601.04739222</v>
+      </c>
+      <c r="CM58">
+        <v>0</v>
+      </c>
+      <c r="CN58" s="2">
+        <v>45398.22773080703</v>
+      </c>
+      <c r="CO58">
+        <v>-0.8048033596017621</v>
+      </c>
+      <c r="CP58">
         <v>-0.9999999999999732</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ZRXUSDT.json at 2024-04-16_12-39-23 bestfile_scores 0.0003379926573969627 bestfile_sharp 0.09035235399757573
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -16460,10 +16460,10 @@
         <v>94</v>
       </c>
       <c r="F58">
-        <v>0.001364122639297527</v>
+        <v>0.001990512544368439</v>
       </c>
       <c r="G58">
-        <v>0.001364122639297527</v>
+        <v>0.001990512544368439</v>
       </c>
       <c r="H58">
         <v>0</v>
@@ -16472,10 +16472,10 @@
         <v>0</v>
       </c>
       <c r="J58">
-        <v>0.001297293119460341</v>
+        <v>0.001746730012986153</v>
       </c>
       <c r="K58">
-        <v>0.001297293119460341</v>
+        <v>0.001746730012986153</v>
       </c>
       <c r="L58">
         <v>0</v>
@@ -16484,34 +16484,34 @@
         <v>0</v>
       </c>
       <c r="N58">
-        <v>24.21316856536011</v>
+        <v>22.10094612859626</v>
       </c>
       <c r="O58">
         <v>0</v>
       </c>
       <c r="P58">
-        <v>0.9997949931923897</v>
+        <v>0.9998179737541465</v>
       </c>
       <c r="Q58">
         <v>1</v>
       </c>
       <c r="R58">
-        <v>0.06237148478473695</v>
+        <v>0.06547405196275462</v>
       </c>
       <c r="S58">
         <v>-0</v>
       </c>
       <c r="T58">
-        <v>0.1539017749998078</v>
+        <v>0.1389462987035806</v>
       </c>
       <c r="U58">
         <v>-0</v>
       </c>
       <c r="V58">
-        <v>0.9992642599845767</v>
+        <v>0.9988224775774484</v>
       </c>
       <c r="W58">
-        <v>0.8882982556401527</v>
+        <v>0.873774578968785</v>
       </c>
       <c r="X58">
         <v>1</v>
@@ -16520,22 +16520,22 @@
         <v>1</v>
       </c>
       <c r="Z58">
-        <v>0.873386993376827</v>
+        <v>0.8610165007677734</v>
       </c>
       <c r="AB58">
-        <v>0.005243039178105519</v>
+        <v>0.007023704605228443</v>
       </c>
       <c r="AC58">
         <v>0</v>
       </c>
       <c r="AD58">
-        <v>0.9992642599845767</v>
+        <v>0.9988224775774484</v>
       </c>
       <c r="AE58">
         <v>1</v>
       </c>
       <c r="AF58">
-        <v>0.005243039178105519</v>
+        <v>0.007023704605228443</v>
       </c>
       <c r="AG58">
         <v>0</v>
@@ -16544,55 +16544,55 @@
         <v>202</v>
       </c>
       <c r="AI58">
-        <v>0.03707838267375759</v>
+        <v>0.05896463482078796</v>
       </c>
       <c r="AJ58">
         <v>0</v>
       </c>
       <c r="AK58">
-        <v>-2866.9001878604</v>
+        <v>-5773.774690739001</v>
       </c>
       <c r="AL58">
         <v>0</v>
       </c>
       <c r="AM58">
-        <v>43528.4007141399</v>
+        <v>85467.01657826123</v>
       </c>
       <c r="AN58">
         <v>10000</v>
       </c>
       <c r="AO58">
-        <v>43528.4007141399</v>
+        <v>85467.01657826123</v>
       </c>
       <c r="AP58">
         <v>10000</v>
       </c>
       <c r="AQ58">
-        <v>3.35284007141399</v>
+        <v>7.546701657826123</v>
       </c>
       <c r="AR58">
         <v>0</v>
       </c>
       <c r="AS58">
-        <v>0.9903358342265095</v>
+        <v>1.084998252603621</v>
       </c>
       <c r="AU58">
-        <v>83.95</v>
+        <v>90.8</v>
       </c>
       <c r="AW58">
-        <v>0.0715786876751517</v>
+        <v>0.03856515151480244</v>
       </c>
       <c r="AX58">
         <v>1</v>
       </c>
       <c r="AY58">
-        <v>-2805.97595243043</v>
+        <v>-3258.737115060647</v>
       </c>
       <c r="AZ58">
         <v>0</v>
       </c>
       <c r="BA58">
-        <v>10727</v>
+        <v>9362</v>
       </c>
       <c r="BB58">
         <v>0</v>
@@ -16601,37 +16601,37 @@
         <v>1078.958333333333</v>
       </c>
       <c r="BD58">
-        <v>15398</v>
+        <v>14484</v>
       </c>
       <c r="BE58">
         <v>0</v>
       </c>
       <c r="BF58">
-        <v>26125</v>
+        <v>23846</v>
       </c>
       <c r="BG58">
         <v>0</v>
       </c>
       <c r="BH58">
-        <v>10643</v>
+        <v>9049</v>
       </c>
       <c r="BI58">
         <v>0</v>
       </c>
       <c r="BJ58">
-        <v>10657</v>
+        <v>9303</v>
       </c>
       <c r="BK58">
         <v>0</v>
       </c>
       <c r="BL58">
-        <v>4755</v>
+        <v>5435</v>
       </c>
       <c r="BM58">
         <v>0</v>
       </c>
       <c r="BN58">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="BO58">
         <v>0</v>
@@ -16643,49 +16643,49 @@
         <v>0</v>
       </c>
       <c r="BR58">
-        <v>33528.4007141396</v>
+        <v>75467.01657826095</v>
       </c>
       <c r="BS58">
         <v>0</v>
       </c>
       <c r="BT58">
-        <v>0.05244279254971655</v>
+        <v>0.06570525378628353</v>
       </c>
       <c r="BU58">
         <v>100</v>
       </c>
       <c r="BV58">
-        <v>0.1449461011079747</v>
+        <v>0.1613998324263049</v>
       </c>
       <c r="BW58">
         <v>100</v>
       </c>
       <c r="BX58">
-        <v>0.006422810151173568</v>
+        <v>0.007022666204230724</v>
       </c>
       <c r="BY58">
         <v>100</v>
       </c>
       <c r="BZ58">
-        <v>0.007638975474069304</v>
+        <v>0.008974746013760164</v>
       </c>
       <c r="CA58">
         <v>1</v>
       </c>
       <c r="CB58">
-        <v>36395.300902</v>
+        <v>81240.79126899995</v>
       </c>
       <c r="CC58">
         <v>0</v>
       </c>
       <c r="CD58">
-        <v>39201.27685443043</v>
+        <v>84499.5283840606</v>
       </c>
       <c r="CE58">
         <v>0</v>
       </c>
       <c r="CF58">
-        <v>0.1868295345238975</v>
+        <v>0.2597294059399704</v>
       </c>
       <c r="CG58">
         <v>0</v>
@@ -16694,22 +16694,22 @@
         <v>10000</v>
       </c>
       <c r="CJ58">
-        <v>0.01795644114921223</v>
+        <v>0.02324683348779734</v>
       </c>
       <c r="CK58">
         <v>0</v>
       </c>
       <c r="CL58">
-        <v>12238601.04739222</v>
+        <v>30956738.30357938</v>
       </c>
       <c r="CM58">
         <v>0</v>
       </c>
       <c r="CN58" s="2">
-        <v>45398.22773080703</v>
+        <v>45398.43140524219</v>
       </c>
       <c r="CO58">
-        <v>-0.8048033596017621</v>
+        <v>-0.7757098341832183</v>
       </c>
       <c r="CP58">
         <v>-0.9999999999999732</v>

</xml_diff>

<commit_message>
Update ZRXUSDT.json at 2024-04-16_14-48-50 bestfile_scores 0.00038336066817075686 bestfile_sharp 0.12970028080537643
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="258">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>VETUSDT</t>
+  </si>
+  <si>
+    <t>ZRXUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1146,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP58"/>
+  <dimension ref="A1:CP59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1435,16 +1438,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1528,7 +1531,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1693,7 +1696,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1701,16 +1704,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1794,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1959,7 +1962,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1967,13 +1970,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2060,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2225,7 +2228,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2233,16 +2236,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2326,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2491,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2499,16 +2502,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2592,7 +2595,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2757,7 +2760,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2765,16 +2768,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2858,7 +2861,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3023,7 +3026,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3031,16 +3034,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3124,7 +3127,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3289,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3297,16 +3300,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3390,7 +3393,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3555,7 +3558,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3563,16 +3566,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3656,7 +3659,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3821,7 +3824,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3829,16 +3832,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E11" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3922,7 +3925,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4087,7 +4090,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4095,16 +4098,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E12" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4188,7 +4191,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4353,7 +4356,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4361,16 +4364,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E13" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4454,7 +4457,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4619,7 +4622,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4627,16 +4630,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4720,7 +4723,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4885,7 +4888,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4893,16 +4896,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -4986,7 +4989,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5151,7 +5154,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5159,16 +5162,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5252,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5417,7 +5420,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5425,16 +5428,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5518,7 +5521,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5683,7 +5686,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5691,16 +5694,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E18" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5784,7 +5787,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5949,7 +5952,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5957,16 +5960,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E19" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6050,7 +6053,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6215,7 +6218,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6223,16 +6226,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E20" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6316,7 +6319,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6481,7 +6484,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6489,16 +6492,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E21" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6582,7 +6585,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6747,7 +6750,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6755,16 +6758,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6848,7 +6851,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7013,7 +7016,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7021,16 +7024,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E23" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7114,7 +7117,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7279,7 +7282,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7287,16 +7290,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E24" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7380,7 +7383,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7545,7 +7548,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7553,16 +7556,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7646,7 +7649,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7811,7 +7814,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7819,16 +7822,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7912,7 +7915,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8077,7 +8080,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8085,16 +8088,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E27" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8178,7 +8181,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8343,7 +8346,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8351,16 +8354,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E28" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8444,7 +8447,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8609,7 +8612,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8617,16 +8620,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E29" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8710,7 +8713,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8875,7 +8878,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8883,16 +8886,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E30" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8976,7 +8979,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9141,7 +9144,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9149,16 +9152,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E31" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9242,7 +9245,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9407,7 +9410,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9415,16 +9418,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E32" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9508,7 +9511,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9673,7 +9676,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9681,16 +9684,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E33" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9774,7 +9777,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9939,7 +9942,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9947,16 +9950,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E34" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10040,7 +10043,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10205,7 +10208,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10219,16 +10222,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E35" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10312,7 +10315,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10477,7 +10480,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10491,16 +10494,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E36" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10584,7 +10587,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10749,7 +10752,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10763,13 +10766,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10856,7 +10859,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11021,7 +11024,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11035,16 +11038,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E38" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11128,7 +11131,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11293,7 +11296,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11307,16 +11310,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E39" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11400,7 +11403,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11565,7 +11568,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11579,16 +11582,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E40" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11672,7 +11675,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11837,7 +11840,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11851,16 +11854,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E41" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11944,7 +11947,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12109,7 +12112,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12123,16 +12126,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E42" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12216,7 +12219,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12381,7 +12384,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12395,16 +12398,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E43" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12488,7 +12491,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12653,7 +12656,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12667,16 +12670,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E44" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12760,7 +12763,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12925,7 +12928,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12939,16 +12942,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E45" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13032,7 +13035,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13197,7 +13200,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13211,16 +13214,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E46" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13304,7 +13307,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13469,7 +13472,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13483,16 +13486,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E47" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13576,7 +13579,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13741,7 +13744,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13755,16 +13758,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E48" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13848,7 +13851,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14013,7 +14016,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14027,16 +14030,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E49" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14120,7 +14123,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14285,7 +14288,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14299,16 +14302,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E50" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14392,7 +14395,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14557,7 +14560,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14571,16 +14574,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E51" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14664,7 +14667,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14829,7 +14832,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14843,16 +14846,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E52" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14936,7 +14939,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15101,7 +15104,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15115,16 +15118,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E53" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15208,7 +15211,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15373,7 +15376,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15387,16 +15390,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15480,7 +15483,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15645,7 +15648,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15659,13 +15662,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15749,7 +15752,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15914,7 +15917,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15928,10 +15931,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E56" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16015,7 +16018,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16180,7 +16183,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16278,7 +16281,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16541,7 +16544,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16712,6 +16715,269 @@
         <v>-0.7757098341832183</v>
       </c>
       <c r="CP58">
+        <v>-0.9999999999999732</v>
+      </c>
+    </row>
+    <row r="59" spans="1:94">
+      <c r="A59" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="E59" t="s">
+        <v>95</v>
+      </c>
+      <c r="F59">
+        <v>0.0004125392330109889</v>
+      </c>
+      <c r="G59">
+        <v>0.0004125392330109889</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>0</v>
+      </c>
+      <c r="J59">
+        <v>0.000939431396576862</v>
+      </c>
+      <c r="K59">
+        <v>0.000939431396576862</v>
+      </c>
+      <c r="L59">
+        <v>0</v>
+      </c>
+      <c r="M59">
+        <v>0</v>
+      </c>
+      <c r="N59">
+        <v>18.37478297773834</v>
+      </c>
+      <c r="O59">
+        <v>0</v>
+      </c>
+      <c r="P59">
+        <v>0.9998372399877068</v>
+      </c>
+      <c r="Q59">
+        <v>1</v>
+      </c>
+      <c r="R59">
+        <v>0.03439705019596732</v>
+      </c>
+      <c r="S59">
+        <v>-0</v>
+      </c>
+      <c r="T59">
+        <v>0.1880195642397774</v>
+      </c>
+      <c r="U59">
+        <v>-0</v>
+      </c>
+      <c r="V59">
+        <v>0.9995951677167287</v>
+      </c>
+      <c r="W59">
+        <v>0.870421341348077</v>
+      </c>
+      <c r="X59">
+        <v>1</v>
+      </c>
+      <c r="Y59">
+        <v>1</v>
+      </c>
+      <c r="Z59">
+        <v>0.8140400142554371</v>
+      </c>
+      <c r="AB59">
+        <v>0.004520013799245894</v>
+      </c>
+      <c r="AC59">
+        <v>0</v>
+      </c>
+      <c r="AD59">
+        <v>0.9995951677167287</v>
+      </c>
+      <c r="AE59">
+        <v>1</v>
+      </c>
+      <c r="AF59">
+        <v>0.004520013799245894</v>
+      </c>
+      <c r="AG59">
+        <v>0</v>
+      </c>
+      <c r="AH59" t="s">
+        <v>203</v>
+      </c>
+      <c r="AI59">
+        <v>0.01398045765943972</v>
+      </c>
+      <c r="AJ59">
+        <v>0</v>
+      </c>
+      <c r="AK59">
+        <v>-534.151894618</v>
+      </c>
+      <c r="AL59">
+        <v>0</v>
+      </c>
+      <c r="AM59">
+        <v>15611.66517538218</v>
+      </c>
+      <c r="AN59">
+        <v>10000</v>
+      </c>
+      <c r="AO59">
+        <v>15611.44061538218</v>
+      </c>
+      <c r="AP59">
+        <v>10000</v>
+      </c>
+      <c r="AQ59">
+        <v>0.5611665175382183</v>
+      </c>
+      <c r="AR59">
+        <v>0</v>
+      </c>
+      <c r="AS59">
+        <v>1.304975726116683</v>
+      </c>
+      <c r="AU59">
+        <v>83.75</v>
+      </c>
+      <c r="AW59">
+        <v>0.05192670508131355</v>
+      </c>
+      <c r="AX59">
+        <v>1</v>
+      </c>
+      <c r="AY59">
+        <v>-336.6111377548751</v>
+      </c>
+      <c r="AZ59">
+        <v>0</v>
+      </c>
+      <c r="BA59">
+        <v>9237</v>
+      </c>
+      <c r="BB59">
+        <v>0</v>
+      </c>
+      <c r="BC59">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BD59">
+        <v>10607</v>
+      </c>
+      <c r="BE59">
+        <v>0</v>
+      </c>
+      <c r="BF59">
+        <v>19844</v>
+      </c>
+      <c r="BG59">
+        <v>0</v>
+      </c>
+      <c r="BH59">
+        <v>8870</v>
+      </c>
+      <c r="BI59">
+        <v>0</v>
+      </c>
+      <c r="BJ59">
+        <v>9219</v>
+      </c>
+      <c r="BK59">
+        <v>0</v>
+      </c>
+      <c r="BL59">
+        <v>1737</v>
+      </c>
+      <c r="BM59">
+        <v>0</v>
+      </c>
+      <c r="BN59">
+        <v>18</v>
+      </c>
+      <c r="BO59">
+        <v>0</v>
+      </c>
+      <c r="BP59">
+        <v>0</v>
+      </c>
+      <c r="BQ59">
+        <v>0</v>
+      </c>
+      <c r="BR59">
+        <v>5611.665175381995</v>
+      </c>
+      <c r="BS59">
+        <v>0</v>
+      </c>
+      <c r="BT59">
+        <v>0.05109993742475609</v>
+      </c>
+      <c r="BU59">
+        <v>100</v>
+      </c>
+      <c r="BV59">
+        <v>0.2284358530268059</v>
+      </c>
+      <c r="BW59">
+        <v>100</v>
+      </c>
+      <c r="BX59">
+        <v>0.01316118008225159</v>
+      </c>
+      <c r="BY59">
+        <v>100</v>
+      </c>
+      <c r="BZ59">
+        <v>0.01081373991239444</v>
+      </c>
+      <c r="CA59">
+        <v>1</v>
+      </c>
+      <c r="CB59">
+        <v>6145.817069999996</v>
+      </c>
+      <c r="CC59">
+        <v>0</v>
+      </c>
+      <c r="CD59">
+        <v>6482.428207754871</v>
+      </c>
+      <c r="CE59">
+        <v>0</v>
+      </c>
+      <c r="CF59">
+        <v>0.09035235399757573</v>
+      </c>
+      <c r="CG59">
+        <v>0</v>
+      </c>
+      <c r="CH59">
+        <v>10000</v>
+      </c>
+      <c r="CJ59">
+        <v>0.00636574074074074</v>
+      </c>
+      <c r="CK59">
+        <v>0</v>
+      </c>
+      <c r="CL59">
+        <v>3838702.753107005</v>
+      </c>
+      <c r="CM59">
+        <v>0</v>
+      </c>
+      <c r="CN59" s="2">
+        <v>45398.52737637559</v>
+      </c>
+      <c r="CO59">
+        <v>-0.9202070805237382</v>
+      </c>
+      <c r="CP59">
         <v>-0.9999999999999732</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RUNEUSDT.json at 2024-04-16_16-45-24 bestfile_scores 0.000819656923567702 bestfile_sharp 0.13160863787509386
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -16726,10 +16726,10 @@
         <v>95</v>
       </c>
       <c r="F59">
-        <v>0.0004125392330109889</v>
+        <v>0.0005221982670147174</v>
       </c>
       <c r="G59">
-        <v>0.0004125392330109889</v>
+        <v>0.0005221982670147174</v>
       </c>
       <c r="H59">
         <v>0</v>
@@ -16738,10 +16738,10 @@
         <v>0</v>
       </c>
       <c r="J59">
-        <v>0.000939431396576862</v>
+        <v>0.00101124440566831</v>
       </c>
       <c r="K59">
-        <v>0.000939431396576862</v>
+        <v>0.00101124440566831</v>
       </c>
       <c r="L59">
         <v>0</v>
@@ -16750,34 +16750,34 @@
         <v>0</v>
       </c>
       <c r="N59">
-        <v>18.37478297773834</v>
+        <v>9.656854045294958</v>
       </c>
       <c r="O59">
         <v>0</v>
       </c>
       <c r="P59">
-        <v>0.9998372399877068</v>
+        <v>0.9998311515597478</v>
       </c>
       <c r="Q59">
         <v>1</v>
       </c>
       <c r="R59">
-        <v>0.03439705019596732</v>
+        <v>0.01018204657081445</v>
       </c>
       <c r="S59">
         <v>-0</v>
       </c>
       <c r="T59">
-        <v>0.1880195642397774</v>
+        <v>0.06380468843904037</v>
       </c>
       <c r="U59">
         <v>-0</v>
       </c>
       <c r="V59">
-        <v>0.9995951677167287</v>
+        <v>0.9998461805853679</v>
       </c>
       <c r="W59">
-        <v>0.870421341348077</v>
+        <v>0.9487031953275766</v>
       </c>
       <c r="X59">
         <v>1</v>
@@ -16786,22 +16786,22 @@
         <v>1</v>
       </c>
       <c r="Z59">
-        <v>0.8140400142554371</v>
+        <v>0.9363908211293905</v>
       </c>
       <c r="AB59">
-        <v>0.004520013799245894</v>
+        <v>0.001480967196344486</v>
       </c>
       <c r="AC59">
         <v>0</v>
       </c>
       <c r="AD59">
-        <v>0.9995951677167287</v>
+        <v>0.9998461805853679</v>
       </c>
       <c r="AE59">
         <v>1</v>
       </c>
       <c r="AF59">
-        <v>0.004520013799245894</v>
+        <v>0.001480967196344486</v>
       </c>
       <c r="AG59">
         <v>0</v>
@@ -16810,55 +16810,55 @@
         <v>203</v>
       </c>
       <c r="AI59">
-        <v>0.01398045765943972</v>
+        <v>0.008849841894546528</v>
       </c>
       <c r="AJ59">
         <v>0</v>
       </c>
       <c r="AK59">
-        <v>-534.151894618</v>
+        <v>-414.1426404160001</v>
       </c>
       <c r="AL59">
         <v>0</v>
       </c>
       <c r="AM59">
-        <v>15611.66517538218</v>
+        <v>17573.46803958403</v>
       </c>
       <c r="AN59">
         <v>10000</v>
       </c>
       <c r="AO59">
-        <v>15611.44061538218</v>
+        <v>17573.34147958403</v>
       </c>
       <c r="AP59">
         <v>10000</v>
       </c>
       <c r="AQ59">
-        <v>0.5611665175382183</v>
+        <v>0.757346803958403</v>
       </c>
       <c r="AR59">
         <v>0</v>
       </c>
       <c r="AS59">
-        <v>1.304975726116683</v>
+        <v>2.481317926096407</v>
       </c>
       <c r="AU59">
-        <v>83.75</v>
+        <v>107.7333333333333</v>
       </c>
       <c r="AW59">
-        <v>0.05192670508131355</v>
+        <v>0.00154643941367346</v>
       </c>
       <c r="AX59">
         <v>1</v>
       </c>
       <c r="AY59">
-        <v>-336.6111377548751</v>
+        <v>-12.37148773286695</v>
       </c>
       <c r="AZ59">
         <v>0</v>
       </c>
       <c r="BA59">
-        <v>9237</v>
+        <v>4982</v>
       </c>
       <c r="BB59">
         <v>0</v>
@@ -16867,37 +16867,37 @@
         <v>1079.958333333333</v>
       </c>
       <c r="BD59">
-        <v>10607</v>
+        <v>5447</v>
       </c>
       <c r="BE59">
         <v>0</v>
       </c>
       <c r="BF59">
-        <v>19844</v>
+        <v>10429</v>
       </c>
       <c r="BG59">
         <v>0</v>
       </c>
       <c r="BH59">
-        <v>8870</v>
+        <v>4516</v>
       </c>
       <c r="BI59">
         <v>0</v>
       </c>
       <c r="BJ59">
-        <v>9219</v>
+        <v>4980</v>
       </c>
       <c r="BK59">
         <v>0</v>
       </c>
       <c r="BL59">
-        <v>1737</v>
+        <v>931</v>
       </c>
       <c r="BM59">
         <v>0</v>
       </c>
       <c r="BN59">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="BO59">
         <v>0</v>
@@ -16909,49 +16909,49 @@
         <v>0</v>
       </c>
       <c r="BR59">
-        <v>5611.665175381995</v>
+        <v>7573.468039583999</v>
       </c>
       <c r="BS59">
         <v>0</v>
       </c>
       <c r="BT59">
-        <v>0.05109993742475609</v>
+        <v>0.04130282653539031</v>
       </c>
       <c r="BU59">
         <v>100</v>
       </c>
       <c r="BV59">
-        <v>0.2284358530268059</v>
+        <v>0.06791945164260231</v>
       </c>
       <c r="BW59">
         <v>100</v>
       </c>
       <c r="BX59">
-        <v>0.01316118008225159</v>
+        <v>0.0130829499029384</v>
       </c>
       <c r="BY59">
         <v>100</v>
       </c>
       <c r="BZ59">
-        <v>0.01081373991239444</v>
+        <v>0.01042956421249071</v>
       </c>
       <c r="CA59">
         <v>1</v>
       </c>
       <c r="CB59">
-        <v>6145.817069999996</v>
+        <v>7987.610679999999</v>
       </c>
       <c r="CC59">
         <v>0</v>
       </c>
       <c r="CD59">
-        <v>6482.428207754871</v>
+        <v>7999.982167732865</v>
       </c>
       <c r="CE59">
         <v>0</v>
       </c>
       <c r="CF59">
-        <v>0.09035235399757573</v>
+        <v>0.1297002808053764</v>
       </c>
       <c r="CG59">
         <v>0</v>
@@ -16960,22 +16960,22 @@
         <v>10000</v>
       </c>
       <c r="CJ59">
-        <v>0.00636574074074074</v>
+        <v>0.003009259259259259</v>
       </c>
       <c r="CK59">
         <v>0</v>
       </c>
       <c r="CL59">
-        <v>3838702.753107005</v>
+        <v>3327004.945222864</v>
       </c>
       <c r="CM59">
         <v>0</v>
       </c>
       <c r="CN59" s="2">
-        <v>45398.52737637559</v>
+        <v>45398.61726723986</v>
       </c>
       <c r="CO59">
-        <v>-0.9202070805237382</v>
+        <v>-0.9614802262041642</v>
       </c>
       <c r="CP59">
         <v>-0.9999999999999732</v>

</xml_diff>

<commit_message>
Update RUNEUSDT.json at 2024-04-16_19-26-30 bestfile_scores 0.0008482253794308781 bestfile_sharp 0.11880877385262616
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="259">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>ZRXUSDT</t>
+  </si>
+  <si>
+    <t>RUNEUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1149,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP59"/>
+  <dimension ref="A1:CP60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1438,16 +1441,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1531,7 +1534,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1696,7 +1699,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1704,16 +1707,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1797,7 +1800,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1962,7 +1965,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1970,13 +1973,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2063,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2228,7 +2231,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2236,16 +2239,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2329,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2494,7 +2497,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2502,16 +2505,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2595,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2760,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2768,16 +2771,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E7" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2861,7 +2864,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3026,7 +3029,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3034,16 +3037,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3127,7 +3130,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3292,7 +3295,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3300,16 +3303,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3393,7 +3396,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3558,7 +3561,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3566,16 +3569,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3659,7 +3662,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3824,7 +3827,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3832,16 +3835,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3925,7 +3928,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4090,7 +4093,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4098,16 +4101,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E12" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4191,7 +4194,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4356,7 +4359,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4364,16 +4367,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4457,7 +4460,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4622,7 +4625,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4630,16 +4633,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4723,7 +4726,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4888,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4896,16 +4899,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -4989,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5154,7 +5157,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5162,16 +5165,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E16" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5255,7 +5258,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5420,7 +5423,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5428,16 +5431,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E17" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5521,7 +5524,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5686,7 +5689,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5694,16 +5697,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5787,7 +5790,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5952,7 +5955,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5960,16 +5963,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E19" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6053,7 +6056,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6218,7 +6221,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6226,16 +6229,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E20" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6319,7 +6322,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6484,7 +6487,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6492,16 +6495,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6585,7 +6588,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6750,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6758,16 +6761,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6851,7 +6854,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7016,7 +7019,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7024,16 +7027,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E23" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7117,7 +7120,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7282,7 +7285,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7290,16 +7293,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7383,7 +7386,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7548,7 +7551,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7556,16 +7559,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E25" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7649,7 +7652,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7814,7 +7817,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7822,16 +7825,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E26" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7915,7 +7918,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8080,7 +8083,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8088,16 +8091,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8181,7 +8184,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8346,7 +8349,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8354,16 +8357,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E28" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8447,7 +8450,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8612,7 +8615,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8620,16 +8623,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E29" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8713,7 +8716,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8878,7 +8881,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8886,16 +8889,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E30" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8979,7 +8982,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9144,7 +9147,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9152,16 +9155,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E31" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9245,7 +9248,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9410,7 +9413,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9418,16 +9421,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E32" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9511,7 +9514,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9676,7 +9679,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9684,16 +9687,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E33" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9777,7 +9780,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9942,7 +9945,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9950,16 +9953,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E34" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10043,7 +10046,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10208,7 +10211,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10222,16 +10225,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E35" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10315,7 +10318,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10480,7 +10483,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10494,16 +10497,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E36" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10587,7 +10590,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10752,7 +10755,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10766,13 +10769,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10859,7 +10862,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11024,7 +11027,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11038,16 +11041,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E38" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11131,7 +11134,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11296,7 +11299,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11310,16 +11313,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E39" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11403,7 +11406,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11568,7 +11571,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11582,16 +11585,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E40" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11675,7 +11678,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11840,7 +11843,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11854,16 +11857,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11947,7 +11950,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12112,7 +12115,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12126,16 +12129,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E42" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12219,7 +12222,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12384,7 +12387,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12398,16 +12401,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E43" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12491,7 +12494,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12656,7 +12659,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12670,16 +12673,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E44" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12763,7 +12766,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12928,7 +12931,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12942,16 +12945,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E45" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13035,7 +13038,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13200,7 +13203,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13214,16 +13217,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E46" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13307,7 +13310,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13472,7 +13475,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13486,16 +13489,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E47" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13579,7 +13582,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13744,7 +13747,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13758,16 +13761,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E48" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13851,7 +13854,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14016,7 +14019,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14030,16 +14033,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E49" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14123,7 +14126,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14288,7 +14291,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14302,16 +14305,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E50" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14395,7 +14398,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14560,7 +14563,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14574,16 +14577,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E51" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14667,7 +14670,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14832,7 +14835,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14846,16 +14849,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E52" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14939,7 +14942,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15104,7 +15107,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15118,16 +15121,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E53" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15211,7 +15214,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15376,7 +15379,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15390,16 +15393,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15483,7 +15486,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15648,7 +15651,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15662,13 +15665,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15752,7 +15755,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15917,7 +15920,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15931,10 +15934,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E56" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16018,7 +16021,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16183,7 +16186,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16281,7 +16284,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16544,7 +16547,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16807,7 +16810,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -16978,6 +16981,269 @@
         <v>-0.9614802262041642</v>
       </c>
       <c r="CP59">
+        <v>-0.9999999999999732</v>
+      </c>
+    </row>
+    <row r="60" spans="1:94">
+      <c r="A60" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E60" t="s">
+        <v>96</v>
+      </c>
+      <c r="F60">
+        <v>0.001842869842314521</v>
+      </c>
+      <c r="G60">
+        <v>0.001842869842314521</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60">
+        <v>0</v>
+      </c>
+      <c r="J60">
+        <v>0.001435757851956287</v>
+      </c>
+      <c r="K60">
+        <v>0.001435757851956287</v>
+      </c>
+      <c r="L60">
+        <v>0</v>
+      </c>
+      <c r="M60">
+        <v>0</v>
+      </c>
+      <c r="N60">
+        <v>30.22061036305413</v>
+      </c>
+      <c r="O60">
+        <v>0</v>
+      </c>
+      <c r="P60">
+        <v>0.9997634667588731</v>
+      </c>
+      <c r="Q60">
+        <v>1</v>
+      </c>
+      <c r="R60">
+        <v>0.06384360816531744</v>
+      </c>
+      <c r="S60">
+        <v>-0</v>
+      </c>
+      <c r="T60">
+        <v>0.2371250312347759</v>
+      </c>
+      <c r="U60">
+        <v>-0</v>
+      </c>
+      <c r="V60">
+        <v>0.9989630934338973</v>
+      </c>
+      <c r="W60">
+        <v>0.8530849912726379</v>
+      </c>
+      <c r="X60">
+        <v>1</v>
+      </c>
+      <c r="Y60">
+        <v>1</v>
+      </c>
+      <c r="Z60">
+        <v>0.7591075655924593</v>
+      </c>
+      <c r="AB60">
+        <v>0.007021018525291578</v>
+      </c>
+      <c r="AC60">
+        <v>0</v>
+      </c>
+      <c r="AD60">
+        <v>0.9989630934338973</v>
+      </c>
+      <c r="AE60">
+        <v>1</v>
+      </c>
+      <c r="AF60">
+        <v>0.007021018525291578</v>
+      </c>
+      <c r="AG60">
+        <v>0</v>
+      </c>
+      <c r="AH60" t="s">
+        <v>204</v>
+      </c>
+      <c r="AI60">
+        <v>0.04101220453838832</v>
+      </c>
+      <c r="AJ60">
+        <v>0</v>
+      </c>
+      <c r="AK60">
+        <v>-4383.904282140001</v>
+      </c>
+      <c r="AL60">
+        <v>0</v>
+      </c>
+      <c r="AM60">
+        <v>73037.72772106039</v>
+      </c>
+      <c r="AN60">
+        <v>10000</v>
+      </c>
+      <c r="AO60">
+        <v>73038.47772106039</v>
+      </c>
+      <c r="AP60">
+        <v>10000</v>
+      </c>
+      <c r="AQ60">
+        <v>6.303772772106039</v>
+      </c>
+      <c r="AR60">
+        <v>0</v>
+      </c>
+      <c r="AS60">
+        <v>0.7939187808963517</v>
+      </c>
+      <c r="AU60">
+        <v>71.28333333333333</v>
+      </c>
+      <c r="AW60">
+        <v>0.01597019772342795</v>
+      </c>
+      <c r="AX60">
+        <v>1</v>
+      </c>
+      <c r="AY60">
+        <v>-1094.27710161459</v>
+      </c>
+      <c r="AZ60">
+        <v>0</v>
+      </c>
+      <c r="BA60">
+        <v>9360</v>
+      </c>
+      <c r="BB60">
+        <v>0</v>
+      </c>
+      <c r="BC60">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BD60">
+        <v>23277</v>
+      </c>
+      <c r="BE60">
+        <v>0</v>
+      </c>
+      <c r="BF60">
+        <v>32637</v>
+      </c>
+      <c r="BG60">
+        <v>0</v>
+      </c>
+      <c r="BH60">
+        <v>9274</v>
+      </c>
+      <c r="BI60">
+        <v>0</v>
+      </c>
+      <c r="BJ60">
+        <v>9302</v>
+      </c>
+      <c r="BK60">
+        <v>0</v>
+      </c>
+      <c r="BL60">
+        <v>14003</v>
+      </c>
+      <c r="BM60">
+        <v>0</v>
+      </c>
+      <c r="BN60">
+        <v>58</v>
+      </c>
+      <c r="BO60">
+        <v>0</v>
+      </c>
+      <c r="BP60">
+        <v>0</v>
+      </c>
+      <c r="BQ60">
+        <v>0</v>
+      </c>
+      <c r="BR60">
+        <v>63041.76561786002</v>
+      </c>
+      <c r="BS60">
+        <v>0</v>
+      </c>
+      <c r="BT60">
+        <v>0.06744789877399233</v>
+      </c>
+      <c r="BU60">
+        <v>100</v>
+      </c>
+      <c r="BV60">
+        <v>0.317505191869218</v>
+      </c>
+      <c r="BW60">
+        <v>100</v>
+      </c>
+      <c r="BX60">
+        <v>0.008272603297578847</v>
+      </c>
+      <c r="BY60">
+        <v>100</v>
+      </c>
+      <c r="BZ60">
+        <v>0.01200249805440164</v>
+      </c>
+      <c r="CA60">
+        <v>1</v>
+      </c>
+      <c r="CB60">
+        <v>67425.66990000002</v>
+      </c>
+      <c r="CC60">
+        <v>0</v>
+      </c>
+      <c r="CD60">
+        <v>68519.94700161461</v>
+      </c>
+      <c r="CE60">
+        <v>0</v>
+      </c>
+      <c r="CF60">
+        <v>0.1316086378750939</v>
+      </c>
+      <c r="CG60">
+        <v>0</v>
+      </c>
+      <c r="CH60">
+        <v>10000</v>
+      </c>
+      <c r="CJ60">
+        <v>0.01222993827160494</v>
+      </c>
+      <c r="CK60">
+        <v>0</v>
+      </c>
+      <c r="CL60">
+        <v>57288867.12987947</v>
+      </c>
+      <c r="CM60">
+        <v>0</v>
+      </c>
+      <c r="CN60" s="2">
+        <v>45398.698221018</v>
+      </c>
+      <c r="CO60">
+        <v>-0.7317367093387688</v>
+      </c>
+      <c r="CP60">
         <v>-0.9999999999999732</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ENSUSDT.json at 2024-04-17_01-58-55 bestfile_scores 0.0007093918081098438 bestfile_sharp 0.10487382837940669
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="260">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>RUNEUSDT</t>
+  </si>
+  <si>
+    <t>ENSUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1152,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP60"/>
+  <dimension ref="A1:CP61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1441,16 +1444,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1534,7 +1537,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1699,7 +1702,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1707,16 +1710,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1800,7 +1803,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1965,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1973,13 +1976,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2066,7 +2069,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2231,7 +2234,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2239,16 +2242,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2332,7 +2335,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2497,7 +2500,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2505,16 +2508,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2598,7 +2601,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2763,7 +2766,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2771,16 +2774,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2864,7 +2867,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3029,7 +3032,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3037,16 +3040,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3130,7 +3133,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3295,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3303,16 +3306,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3396,7 +3399,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3561,7 +3564,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3569,16 +3572,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3662,7 +3665,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3827,7 +3830,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3835,16 +3838,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3928,7 +3931,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4093,7 +4096,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4101,16 +4104,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E12" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4194,7 +4197,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4359,7 +4362,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4367,16 +4370,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E13" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4460,7 +4463,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4625,7 +4628,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4633,16 +4636,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4726,7 +4729,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4891,7 +4894,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4899,16 +4902,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -4992,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5157,7 +5160,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5165,16 +5168,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5258,7 +5261,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5423,7 +5426,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5431,16 +5434,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5524,7 +5527,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5689,7 +5692,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5697,16 +5700,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E18" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5790,7 +5793,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5955,7 +5958,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5963,16 +5966,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E19" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6056,7 +6059,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6221,7 +6224,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6229,16 +6232,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6322,7 +6325,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6487,7 +6490,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6495,16 +6498,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E21" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6588,7 +6591,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6753,7 +6756,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6761,16 +6764,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6854,7 +6857,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7019,7 +7022,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7027,16 +7030,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7120,7 +7123,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7285,7 +7288,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7293,16 +7296,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E24" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7386,7 +7389,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7551,7 +7554,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7559,16 +7562,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E25" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7652,7 +7655,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7817,7 +7820,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7825,16 +7828,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E26" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7918,7 +7921,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8083,7 +8086,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8091,16 +8094,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E27" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8184,7 +8187,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8349,7 +8352,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8357,16 +8360,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E28" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8450,7 +8453,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8615,7 +8618,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8623,16 +8626,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E29" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8716,7 +8719,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8881,7 +8884,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8889,16 +8892,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E30" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8982,7 +8985,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9147,7 +9150,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9155,16 +9158,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E31" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9248,7 +9251,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9413,7 +9416,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9421,16 +9424,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E32" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9514,7 +9517,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9679,7 +9682,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9687,16 +9690,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E33" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9780,7 +9783,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9945,7 +9948,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9953,16 +9956,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E34" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10046,7 +10049,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10211,7 +10214,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10225,16 +10228,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E35" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10318,7 +10321,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10483,7 +10486,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10497,16 +10500,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E36" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10590,7 +10593,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10755,7 +10758,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10769,13 +10772,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10862,7 +10865,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11027,7 +11030,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11041,16 +11044,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11134,7 +11137,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11299,7 +11302,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11313,16 +11316,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E39" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11406,7 +11409,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11571,7 +11574,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11585,16 +11588,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E40" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11678,7 +11681,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11843,7 +11846,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11857,16 +11860,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E41" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11950,7 +11953,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12115,7 +12118,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12129,16 +12132,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E42" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12222,7 +12225,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12387,7 +12390,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12401,16 +12404,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E43" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12494,7 +12497,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12659,7 +12662,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12673,16 +12676,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E44" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12766,7 +12769,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12931,7 +12934,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12945,16 +12948,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E45" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13038,7 +13041,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13203,7 +13206,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13217,16 +13220,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E46" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13310,7 +13313,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13475,7 +13478,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13489,16 +13492,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E47" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13582,7 +13585,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13747,7 +13750,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13761,16 +13764,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E48" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13854,7 +13857,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14019,7 +14022,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14033,16 +14036,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E49" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14126,7 +14129,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14291,7 +14294,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14305,16 +14308,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E50" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14398,7 +14401,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14563,7 +14566,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14577,16 +14580,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E51" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14670,7 +14673,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14835,7 +14838,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14849,16 +14852,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E52" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14942,7 +14945,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15107,7 +15110,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15121,16 +15124,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E53" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15214,7 +15217,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15379,7 +15382,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15393,16 +15396,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C54" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D54" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E54" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15486,7 +15489,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15651,7 +15654,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15665,13 +15668,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15755,7 +15758,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15920,7 +15923,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15934,10 +15937,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E56" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16021,7 +16024,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16186,7 +16189,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16284,7 +16287,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16547,7 +16550,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16810,7 +16813,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -17073,7 +17076,7 @@
         <v>0</v>
       </c>
       <c r="AH60" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="AI60">
         <v>0.04385278076244065</v>
@@ -17245,6 +17248,269 @@
       </c>
       <c r="CP60">
         <v>-0.9999999999999732</v>
+      </c>
+    </row>
+    <row r="61" spans="1:94">
+      <c r="A61" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E61" t="s">
+        <v>97</v>
+      </c>
+      <c r="F61">
+        <v>0.0006776201968474727</v>
+      </c>
+      <c r="G61">
+        <v>0.0006776201968474727</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61">
+        <v>0</v>
+      </c>
+      <c r="J61">
+        <v>0.002159947035591902</v>
+      </c>
+      <c r="K61">
+        <v>0.002159947035591902</v>
+      </c>
+      <c r="L61">
+        <v>0</v>
+      </c>
+      <c r="M61">
+        <v>0</v>
+      </c>
+      <c r="N61">
+        <v>11.66468215863261</v>
+      </c>
+      <c r="O61">
+        <v>0</v>
+      </c>
+      <c r="P61">
+        <v>0.9997527316258012</v>
+      </c>
+      <c r="Q61">
+        <v>1</v>
+      </c>
+      <c r="R61">
+        <v>0.04885741440964268</v>
+      </c>
+      <c r="S61">
+        <v>-0</v>
+      </c>
+      <c r="T61">
+        <v>0.09819379131032092</v>
+      </c>
+      <c r="U61">
+        <v>-0</v>
+      </c>
+      <c r="V61">
+        <v>0.9994157580646265</v>
+      </c>
+      <c r="W61">
+        <v>0.9104767476783258</v>
+      </c>
+      <c r="X61">
+        <v>1</v>
+      </c>
+      <c r="Y61">
+        <v>1</v>
+      </c>
+      <c r="Z61">
+        <v>0.903604907969178</v>
+      </c>
+      <c r="AB61">
+        <v>0.004950442936334854</v>
+      </c>
+      <c r="AC61">
+        <v>0</v>
+      </c>
+      <c r="AD61">
+        <v>0.9994157580646265</v>
+      </c>
+      <c r="AE61">
+        <v>1</v>
+      </c>
+      <c r="AF61">
+        <v>0.004950442936334854</v>
+      </c>
+      <c r="AG61">
+        <v>0</v>
+      </c>
+      <c r="AH61" t="s">
+        <v>205</v>
+      </c>
+      <c r="AI61">
+        <v>0.01757226731119264</v>
+      </c>
+      <c r="AJ61">
+        <v>0</v>
+      </c>
+      <c r="AK61">
+        <v>-297.73514308</v>
+      </c>
+      <c r="AL61">
+        <v>0</v>
+      </c>
+      <c r="AM61">
+        <v>18001.36045692012</v>
+      </c>
+      <c r="AN61">
+        <v>10000</v>
+      </c>
+      <c r="AO61">
+        <v>17999.65105692012</v>
+      </c>
+      <c r="AP61">
+        <v>10000</v>
+      </c>
+      <c r="AQ61">
+        <v>0.8001360456920124</v>
+      </c>
+      <c r="AR61">
+        <v>0</v>
+      </c>
+      <c r="AS61">
+        <v>2.05515543700191</v>
+      </c>
+      <c r="AU61">
+        <v>103.7</v>
+      </c>
+      <c r="AW61">
+        <v>0.02064680093933145</v>
+      </c>
+      <c r="AX61">
+        <v>1</v>
+      </c>
+      <c r="AY61">
+        <v>-174.9621842191654</v>
+      </c>
+      <c r="AZ61">
+        <v>0</v>
+      </c>
+      <c r="BA61">
+        <v>4808</v>
+      </c>
+      <c r="BB61">
+        <v>0</v>
+      </c>
+      <c r="BC61">
+        <v>867.8333333333334</v>
+      </c>
+      <c r="BD61">
+        <v>5315</v>
+      </c>
+      <c r="BE61">
+        <v>0</v>
+      </c>
+      <c r="BF61">
+        <v>10123</v>
+      </c>
+      <c r="BG61">
+        <v>0</v>
+      </c>
+      <c r="BH61">
+        <v>4461</v>
+      </c>
+      <c r="BI61">
+        <v>0</v>
+      </c>
+      <c r="BJ61">
+        <v>4794</v>
+      </c>
+      <c r="BK61">
+        <v>0</v>
+      </c>
+      <c r="BL61">
+        <v>854</v>
+      </c>
+      <c r="BM61">
+        <v>0</v>
+      </c>
+      <c r="BN61">
+        <v>14</v>
+      </c>
+      <c r="BO61">
+        <v>0</v>
+      </c>
+      <c r="BP61">
+        <v>0</v>
+      </c>
+      <c r="BQ61">
+        <v>0</v>
+      </c>
+      <c r="BR61">
+        <v>8001.360456920008</v>
+      </c>
+      <c r="BS61">
+        <v>0</v>
+      </c>
+      <c r="BT61">
+        <v>0.06370423493368013</v>
+      </c>
+      <c r="BU61">
+        <v>100</v>
+      </c>
+      <c r="BV61">
+        <v>0.1190143804060388</v>
+      </c>
+      <c r="BW61">
+        <v>100</v>
+      </c>
+      <c r="BX61">
+        <v>0.01507844201602131</v>
+      </c>
+      <c r="BY61">
+        <v>100</v>
+      </c>
+      <c r="BZ61">
+        <v>0.01252336458059134</v>
+      </c>
+      <c r="CA61">
+        <v>1</v>
+      </c>
+      <c r="CB61">
+        <v>8299.095600000008</v>
+      </c>
+      <c r="CC61">
+        <v>0</v>
+      </c>
+      <c r="CD61">
+        <v>8474.057784219172</v>
+      </c>
+      <c r="CE61">
+        <v>0</v>
+      </c>
+      <c r="CF61">
+        <v>0.1048738283794067</v>
+      </c>
+      <c r="CG61">
+        <v>0</v>
+      </c>
+      <c r="CH61">
+        <v>10000</v>
+      </c>
+      <c r="CJ61">
+        <v>0.003792788900091219</v>
+      </c>
+      <c r="CK61">
+        <v>0</v>
+      </c>
+      <c r="CL61">
+        <v>2650091.450559197</v>
+      </c>
+      <c r="CM61">
+        <v>0</v>
+      </c>
+      <c r="CN61" s="2">
+        <v>45398.97480032586</v>
+      </c>
+      <c r="CO61">
+        <v>-0.9240444127040541</v>
+      </c>
+      <c r="CP61">
+        <v>-0.9999999999999756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update OPUSDT.json at 2024-04-17_05-59-43 bestfile_scores 0.001434627938973232 bestfile_sharp 0.23745043899039642
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="261">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -308,6 +308,9 @@
   </si>
   <si>
     <t>ENSUSDT</t>
+  </si>
+  <si>
+    <t>OPUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1155,7 +1158,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP61"/>
+  <dimension ref="A1:CP62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1444,16 +1447,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1537,7 +1540,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1702,7 +1705,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1710,16 +1713,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1803,7 +1806,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1968,7 +1971,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1976,13 +1979,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2069,7 +2072,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2234,7 +2237,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2242,16 +2245,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2335,7 +2338,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2500,7 +2503,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2508,16 +2511,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2601,7 +2604,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2766,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2774,16 +2777,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E7" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2867,7 +2870,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3032,7 +3035,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3040,16 +3043,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3133,7 +3136,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3298,7 +3301,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3306,16 +3309,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3399,7 +3402,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3564,7 +3567,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3572,16 +3575,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3665,7 +3668,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3830,7 +3833,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3838,16 +3841,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E11" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3931,7 +3934,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4096,7 +4099,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4104,16 +4107,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E12" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4197,7 +4200,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4362,7 +4365,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4370,16 +4373,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E13" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4463,7 +4466,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4628,7 +4631,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4636,16 +4639,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4729,7 +4732,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4894,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4902,16 +4905,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -4995,7 +4998,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5160,7 +5163,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5168,16 +5171,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E16" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5261,7 +5264,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5426,7 +5429,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5434,16 +5437,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5527,7 +5530,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5692,7 +5695,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5700,16 +5703,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5793,7 +5796,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5958,7 +5961,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5966,16 +5969,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E19" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6059,7 +6062,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6224,7 +6227,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6232,16 +6235,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E20" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6325,7 +6328,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6490,7 +6493,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6498,16 +6501,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6591,7 +6594,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6756,7 +6759,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6764,16 +6767,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6857,7 +6860,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7022,7 +7025,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7030,16 +7033,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E23" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7123,7 +7126,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7288,7 +7291,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7296,16 +7299,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7389,7 +7392,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7554,7 +7557,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7562,16 +7565,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7655,7 +7658,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7820,7 +7823,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7828,16 +7831,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E26" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7921,7 +7924,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8086,7 +8089,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8094,16 +8097,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E27" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8187,7 +8190,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8352,7 +8355,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8360,16 +8363,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8453,7 +8456,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8618,7 +8621,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8626,16 +8629,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E29" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8719,7 +8722,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8884,7 +8887,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8892,16 +8895,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E30" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8985,7 +8988,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9150,7 +9153,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9158,16 +9161,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E31" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9251,7 +9254,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9416,7 +9419,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9424,16 +9427,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E32" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9517,7 +9520,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9682,7 +9685,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9690,16 +9693,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9783,7 +9786,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9948,7 +9951,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9956,16 +9959,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E34" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10049,7 +10052,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10214,7 +10217,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10228,16 +10231,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10321,7 +10324,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10486,7 +10489,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10500,16 +10503,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E36" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10593,7 +10596,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10758,7 +10761,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10772,13 +10775,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10865,7 +10868,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11030,7 +11033,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11044,16 +11047,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E38" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11137,7 +11140,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11302,7 +11305,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11316,16 +11319,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11409,7 +11412,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11574,7 +11577,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11588,16 +11591,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E40" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11681,7 +11684,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11846,7 +11849,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11860,16 +11863,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E41" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11953,7 +11956,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12118,7 +12121,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12132,16 +12135,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12225,7 +12228,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12390,7 +12393,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12404,16 +12407,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E43" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12497,7 +12500,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12662,7 +12665,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12676,16 +12679,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E44" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12769,7 +12772,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12934,7 +12937,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12948,16 +12951,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E45" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13041,7 +13044,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13206,7 +13209,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13220,16 +13223,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E46" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13313,7 +13316,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13478,7 +13481,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13492,16 +13495,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E47" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13585,7 +13588,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13750,7 +13753,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13764,16 +13767,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E48" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13857,7 +13860,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14022,7 +14025,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14036,16 +14039,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E49" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14129,7 +14132,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14294,7 +14297,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14308,16 +14311,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E50" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14401,7 +14404,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14566,7 +14569,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14580,16 +14583,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E51" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14673,7 +14676,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14838,7 +14841,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14852,16 +14855,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E52" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14945,7 +14948,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15110,7 +15113,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15124,16 +15127,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E53" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15217,7 +15220,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15382,7 +15385,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15396,16 +15399,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D54" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E54" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15489,7 +15492,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15654,7 +15657,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15668,13 +15671,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15758,7 +15761,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15923,7 +15926,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15937,10 +15940,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16024,7 +16027,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16189,7 +16192,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16287,7 +16290,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16550,7 +16553,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16813,7 +16816,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -17076,7 +17079,7 @@
         <v>0</v>
       </c>
       <c r="AH60" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI60">
         <v>0.04385278076244065</v>
@@ -17339,7 +17342,7 @@
         <v>0</v>
       </c>
       <c r="AH61" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AI61">
         <v>0.01757226731119264</v>
@@ -17511,6 +17514,269 @@
       </c>
       <c r="CP61">
         <v>-0.9999999999999756</v>
+      </c>
+    </row>
+    <row r="62" spans="1:94">
+      <c r="A62" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E62" t="s">
+        <v>98</v>
+      </c>
+      <c r="F62">
+        <v>0.00250141067802212</v>
+      </c>
+      <c r="G62">
+        <v>0.00250141067802212</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62">
+        <v>0</v>
+      </c>
+      <c r="J62">
+        <v>0.003237101077870807</v>
+      </c>
+      <c r="K62">
+        <v>0.003237101077870807</v>
+      </c>
+      <c r="L62">
+        <v>0</v>
+      </c>
+      <c r="M62">
+        <v>0</v>
+      </c>
+      <c r="N62">
+        <v>8.960000000000001</v>
+      </c>
+      <c r="O62">
+        <v>0</v>
+      </c>
+      <c r="P62">
+        <v>0.9999420271141708</v>
+      </c>
+      <c r="Q62">
+        <v>1</v>
+      </c>
+      <c r="R62">
+        <v>0.09851016914299447</v>
+      </c>
+      <c r="S62">
+        <v>-0</v>
+      </c>
+      <c r="T62">
+        <v>0.1398180750800546</v>
+      </c>
+      <c r="U62">
+        <v>-0</v>
+      </c>
+      <c r="V62">
+        <v>0.9985582588237153</v>
+      </c>
+      <c r="W62">
+        <v>0.8742736913374778</v>
+      </c>
+      <c r="X62">
+        <v>1</v>
+      </c>
+      <c r="Y62">
+        <v>1</v>
+      </c>
+      <c r="Z62">
+        <v>0.8603859408245278</v>
+      </c>
+      <c r="AB62">
+        <v>0.009572429424446747</v>
+      </c>
+      <c r="AC62">
+        <v>0</v>
+      </c>
+      <c r="AD62">
+        <v>0.9985582588237153</v>
+      </c>
+      <c r="AE62">
+        <v>1</v>
+      </c>
+      <c r="AF62">
+        <v>0.009572429424446747</v>
+      </c>
+      <c r="AG62">
+        <v>0</v>
+      </c>
+      <c r="AH62" t="s">
+        <v>206</v>
+      </c>
+      <c r="AI62">
+        <v>0.05512246253185499</v>
+      </c>
+      <c r="AJ62">
+        <v>0</v>
+      </c>
+      <c r="AK62">
+        <v>-1157.663383838</v>
+      </c>
+      <c r="AL62">
+        <v>0</v>
+      </c>
+      <c r="AM62">
+        <v>55276.64593101211</v>
+      </c>
+      <c r="AN62">
+        <v>10000</v>
+      </c>
+      <c r="AO62">
+        <v>55276.64593101211</v>
+      </c>
+      <c r="AP62">
+        <v>10000</v>
+      </c>
+      <c r="AQ62">
+        <v>4.527664593101211</v>
+      </c>
+      <c r="AR62">
+        <v>0</v>
+      </c>
+      <c r="AS62">
+        <v>2.672130701897461</v>
+      </c>
+      <c r="AU62">
+        <v>112.4833333333333</v>
+      </c>
+      <c r="AW62">
+        <v>0.04086166432447337</v>
+      </c>
+      <c r="AX62">
+        <v>1</v>
+      </c>
+      <c r="AY62">
+        <v>-1978.212075419069</v>
+      </c>
+      <c r="AZ62">
+        <v>0</v>
+      </c>
+      <c r="BA62">
+        <v>2171</v>
+      </c>
+      <c r="BB62">
+        <v>0</v>
+      </c>
+      <c r="BC62">
+        <v>684.375</v>
+      </c>
+      <c r="BD62">
+        <v>3961</v>
+      </c>
+      <c r="BE62">
+        <v>0</v>
+      </c>
+      <c r="BF62">
+        <v>6132</v>
+      </c>
+      <c r="BG62">
+        <v>0</v>
+      </c>
+      <c r="BH62">
+        <v>969</v>
+      </c>
+      <c r="BI62">
+        <v>0</v>
+      </c>
+      <c r="BJ62">
+        <v>2128</v>
+      </c>
+      <c r="BK62">
+        <v>0</v>
+      </c>
+      <c r="BL62">
+        <v>2992</v>
+      </c>
+      <c r="BM62">
+        <v>0</v>
+      </c>
+      <c r="BN62">
+        <v>43</v>
+      </c>
+      <c r="BO62">
+        <v>0</v>
+      </c>
+      <c r="BP62">
+        <v>0</v>
+      </c>
+      <c r="BQ62">
+        <v>0</v>
+      </c>
+      <c r="BR62">
+        <v>45276.54503616201</v>
+      </c>
+      <c r="BS62">
+        <v>0</v>
+      </c>
+      <c r="BT62">
+        <v>0.09214985016754507</v>
+      </c>
+      <c r="BU62">
+        <v>100</v>
+      </c>
+      <c r="BV62">
+        <v>0.1622612110792429</v>
+      </c>
+      <c r="BW62">
+        <v>100</v>
+      </c>
+      <c r="BX62">
+        <v>0.01034667864108584</v>
+      </c>
+      <c r="BY62">
+        <v>100</v>
+      </c>
+      <c r="BZ62">
+        <v>0.01444960997114174</v>
+      </c>
+      <c r="CA62">
+        <v>1</v>
+      </c>
+      <c r="CB62">
+        <v>46434.20842000001</v>
+      </c>
+      <c r="CC62">
+        <v>0</v>
+      </c>
+      <c r="CD62">
+        <v>48412.42049541908</v>
+      </c>
+      <c r="CE62">
+        <v>0</v>
+      </c>
+      <c r="CF62">
+        <v>0.2374504389903964</v>
+      </c>
+      <c r="CG62">
+        <v>0</v>
+      </c>
+      <c r="CH62">
+        <v>10000</v>
+      </c>
+      <c r="CJ62">
+        <v>0.02782174601241933</v>
+      </c>
+      <c r="CK62">
+        <v>0</v>
+      </c>
+      <c r="CL62">
+        <v>26351531.43582868</v>
+      </c>
+      <c r="CM62">
+        <v>0</v>
+      </c>
+      <c r="CN62" s="2">
+        <v>45399.16874621194</v>
+      </c>
+      <c r="CO62">
+        <v>-0.6213262971882773</v>
+      </c>
+      <c r="CP62">
+        <v>-0.9999999999999784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update UNIUSDT.json at 2024-04-17_10-10-17 bestfile_scores 0.0004870442371008088 bestfile_sharp 0.1841131057155104
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="262">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -311,6 +311,9 @@
   </si>
   <si>
     <t>OPUSDT</t>
+  </si>
+  <si>
+    <t>UNIUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1158,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP62"/>
+  <dimension ref="A1:CP63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1447,16 +1450,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1540,7 +1543,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1705,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1713,16 +1716,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1806,7 +1809,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1971,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1979,13 +1982,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2072,7 +2075,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2237,7 +2240,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2245,16 +2248,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2338,7 +2341,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2503,7 +2506,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2511,16 +2514,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2604,7 +2607,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2769,7 +2772,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2777,16 +2780,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2870,7 +2873,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3035,7 +3038,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3043,16 +3046,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3136,7 +3139,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3301,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3309,16 +3312,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3402,7 +3405,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3567,7 +3570,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3575,16 +3578,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3668,7 +3671,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3833,7 +3836,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3841,16 +3844,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E11" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3934,7 +3937,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4099,7 +4102,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4107,16 +4110,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4200,7 +4203,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4365,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4373,16 +4376,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4466,7 +4469,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4631,7 +4634,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4639,16 +4642,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4732,7 +4735,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4897,7 +4900,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4905,16 +4908,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -4998,7 +5001,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5163,7 +5166,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5171,16 +5174,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5264,7 +5267,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5429,7 +5432,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5437,16 +5440,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E17" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5530,7 +5533,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5695,7 +5698,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5703,16 +5706,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E18" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5796,7 +5799,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5961,7 +5964,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5969,16 +5972,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E19" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6062,7 +6065,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6227,7 +6230,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6235,16 +6238,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6328,7 +6331,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6493,7 +6496,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6501,16 +6504,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6594,7 +6597,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6759,7 +6762,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6767,16 +6770,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E22" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6860,7 +6863,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7025,7 +7028,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7033,16 +7036,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7126,7 +7129,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7291,7 +7294,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7299,16 +7302,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7392,7 +7395,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7557,7 +7560,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7565,16 +7568,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7658,7 +7661,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7823,7 +7826,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7831,16 +7834,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E26" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7924,7 +7927,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8089,7 +8092,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8097,16 +8100,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E27" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8190,7 +8193,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8355,7 +8358,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8363,16 +8366,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8456,7 +8459,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8621,7 +8624,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8629,16 +8632,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E29" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8722,7 +8725,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8887,7 +8890,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8895,16 +8898,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8988,7 +8991,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9153,7 +9156,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9161,16 +9164,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E31" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9254,7 +9257,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9419,7 +9422,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9427,16 +9430,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E32" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9520,7 +9523,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9685,7 +9688,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9693,16 +9696,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9786,7 +9789,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9951,7 +9954,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9959,16 +9962,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E34" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10052,7 +10055,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10217,7 +10220,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10231,16 +10234,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E35" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10324,7 +10327,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10489,7 +10492,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10503,16 +10506,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E36" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10596,7 +10599,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10761,7 +10764,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10775,13 +10778,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10868,7 +10871,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11033,7 +11036,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11047,16 +11050,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E38" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11140,7 +11143,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11305,7 +11308,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11319,16 +11322,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E39" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11412,7 +11415,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11577,7 +11580,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11591,16 +11594,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E40" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11684,7 +11687,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11849,7 +11852,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11863,16 +11866,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E41" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11956,7 +11959,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12121,7 +12124,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12135,16 +12138,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E42" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12228,7 +12231,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12393,7 +12396,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12407,16 +12410,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E43" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12500,7 +12503,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12665,7 +12668,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12679,16 +12682,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E44" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12772,7 +12775,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12937,7 +12940,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12951,16 +12954,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E45" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13044,7 +13047,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13209,7 +13212,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13223,16 +13226,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E46" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13316,7 +13319,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13481,7 +13484,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13495,16 +13498,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E47" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13588,7 +13591,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13753,7 +13756,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13767,16 +13770,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E48" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13860,7 +13863,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14025,7 +14028,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14039,16 +14042,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14132,7 +14135,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14297,7 +14300,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14311,16 +14314,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E50" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14404,7 +14407,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14569,7 +14572,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14583,16 +14586,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E51" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14676,7 +14679,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14841,7 +14844,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14855,16 +14858,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E52" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14948,7 +14951,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15113,7 +15116,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15127,16 +15130,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E53" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15220,7 +15223,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15385,7 +15388,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15399,16 +15402,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15492,7 +15495,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15657,7 +15660,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15671,13 +15674,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C55" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E55" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15761,7 +15764,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15926,7 +15929,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15940,10 +15943,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16027,7 +16030,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16192,7 +16195,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16290,7 +16293,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16553,7 +16556,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16816,7 +16819,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -17079,7 +17082,7 @@
         <v>0</v>
       </c>
       <c r="AH60" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI60">
         <v>0.04385278076244065</v>
@@ -17342,7 +17345,7 @@
         <v>0</v>
       </c>
       <c r="AH61" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI61">
         <v>0.01757226731119264</v>
@@ -17605,7 +17608,7 @@
         <v>0</v>
       </c>
       <c r="AH62" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="AI62">
         <v>0.05512246253185499</v>
@@ -17777,6 +17780,269 @@
       </c>
       <c r="CP62">
         <v>-0.9999999999999784</v>
+      </c>
+    </row>
+    <row r="63" spans="1:94">
+      <c r="A63" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E63" t="s">
+        <v>99</v>
+      </c>
+      <c r="F63">
+        <v>0.0005530662709798406</v>
+      </c>
+      <c r="G63">
+        <v>0.0005530662709798406</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63">
+        <v>0</v>
+      </c>
+      <c r="J63">
+        <v>0.001129672679885241</v>
+      </c>
+      <c r="K63">
+        <v>0.001129672679885241</v>
+      </c>
+      <c r="L63">
+        <v>0</v>
+      </c>
+      <c r="M63">
+        <v>0</v>
+      </c>
+      <c r="N63">
+        <v>14.08210079165862</v>
+      </c>
+      <c r="O63">
+        <v>0</v>
+      </c>
+      <c r="P63">
+        <v>0.9963022005820252</v>
+      </c>
+      <c r="Q63">
+        <v>1</v>
+      </c>
+      <c r="R63">
+        <v>0.01876950593364631</v>
+      </c>
+      <c r="S63">
+        <v>-0</v>
+      </c>
+      <c r="T63">
+        <v>0.1156042952559239</v>
+      </c>
+      <c r="U63">
+        <v>-0</v>
+      </c>
+      <c r="V63">
+        <v>0.9997300260474141</v>
+      </c>
+      <c r="W63">
+        <v>0.9022408584663015</v>
+      </c>
+      <c r="X63">
+        <v>1</v>
+      </c>
+      <c r="Y63">
+        <v>1</v>
+      </c>
+      <c r="Z63">
+        <v>0.8845697945429987</v>
+      </c>
+      <c r="AB63">
+        <v>0.003161635495886697</v>
+      </c>
+      <c r="AC63">
+        <v>0</v>
+      </c>
+      <c r="AD63">
+        <v>0.9997300260474141</v>
+      </c>
+      <c r="AE63">
+        <v>1</v>
+      </c>
+      <c r="AF63">
+        <v>0.003161635495886697</v>
+      </c>
+      <c r="AG63">
+        <v>0</v>
+      </c>
+      <c r="AH63" t="s">
+        <v>207</v>
+      </c>
+      <c r="AI63">
+        <v>0.01271959061682842</v>
+      </c>
+      <c r="AJ63">
+        <v>0</v>
+      </c>
+      <c r="AK63">
+        <v>-460.58132618</v>
+      </c>
+      <c r="AL63">
+        <v>0</v>
+      </c>
+      <c r="AM63">
+        <v>18158.8055738202</v>
+      </c>
+      <c r="AN63">
+        <v>10000</v>
+      </c>
+      <c r="AO63">
+        <v>18157.7495738202</v>
+      </c>
+      <c r="AP63">
+        <v>10000</v>
+      </c>
+      <c r="AQ63">
+        <v>0.8158805573820203</v>
+      </c>
+      <c r="AR63">
+        <v>0</v>
+      </c>
+      <c r="AS63">
+        <v>1.701641106649992</v>
+      </c>
+      <c r="AU63">
+        <v>97.15000000000001</v>
+      </c>
+      <c r="AW63">
+        <v>0.0002407443116559062</v>
+      </c>
+      <c r="AX63">
+        <v>1</v>
+      </c>
+      <c r="AY63">
+        <v>-2.075568047337285</v>
+      </c>
+      <c r="AZ63">
+        <v>0</v>
+      </c>
+      <c r="BA63">
+        <v>6613</v>
+      </c>
+      <c r="BB63">
+        <v>0</v>
+      </c>
+      <c r="BC63">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BD63">
+        <v>8581</v>
+      </c>
+      <c r="BE63">
+        <v>0</v>
+      </c>
+      <c r="BF63">
+        <v>15194</v>
+      </c>
+      <c r="BG63">
+        <v>0</v>
+      </c>
+      <c r="BH63">
+        <v>6669</v>
+      </c>
+      <c r="BI63">
+        <v>0</v>
+      </c>
+      <c r="BJ63">
+        <v>6612</v>
+      </c>
+      <c r="BK63">
+        <v>0</v>
+      </c>
+      <c r="BL63">
+        <v>1912</v>
+      </c>
+      <c r="BM63">
+        <v>0</v>
+      </c>
+      <c r="BN63">
+        <v>1</v>
+      </c>
+      <c r="BO63">
+        <v>0</v>
+      </c>
+      <c r="BP63">
+        <v>0</v>
+      </c>
+      <c r="BQ63">
+        <v>0</v>
+      </c>
+      <c r="BR63">
+        <v>8158.805573819994</v>
+      </c>
+      <c r="BS63">
+        <v>0</v>
+      </c>
+      <c r="BT63">
+        <v>0.04165887397552461</v>
+      </c>
+      <c r="BU63">
+        <v>100</v>
+      </c>
+      <c r="BV63">
+        <v>0.1303899207540317</v>
+      </c>
+      <c r="BW63">
+        <v>100</v>
+      </c>
+      <c r="BX63">
+        <v>0.01161459349193769</v>
+      </c>
+      <c r="BY63">
+        <v>100</v>
+      </c>
+      <c r="BZ63">
+        <v>0.009174774953634677</v>
+      </c>
+      <c r="CA63">
+        <v>1</v>
+      </c>
+      <c r="CB63">
+        <v>8619.386899999994</v>
+      </c>
+      <c r="CC63">
+        <v>0</v>
+      </c>
+      <c r="CD63">
+        <v>8621.462468047332</v>
+      </c>
+      <c r="CE63">
+        <v>0</v>
+      </c>
+      <c r="CF63">
+        <v>0.1359713694556786</v>
+      </c>
+      <c r="CG63">
+        <v>0</v>
+      </c>
+      <c r="CH63">
+        <v>10000</v>
+      </c>
+      <c r="CJ63">
+        <v>0.004209144269385233</v>
+      </c>
+      <c r="CK63">
+        <v>0</v>
+      </c>
+      <c r="CL63">
+        <v>1792278.455560063</v>
+      </c>
+      <c r="CM63">
+        <v>0</v>
+      </c>
+      <c r="CN63" s="2">
+        <v>45399.31942677312</v>
+      </c>
+      <c r="CO63">
+        <v>-0.951306289405574</v>
+      </c>
+      <c r="CP63">
+        <v>-0.9999999999999732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AUDIOUSDT.json at 2024-04-17_15-35-43 bestfile_scores 0.0007268723635037832 bestfile_sharp 0.15393394657768714
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="263">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -314,6 +314,9 @@
   </si>
   <si>
     <t>UNIUSDT</t>
+  </si>
+  <si>
+    <t>AUDIOUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1161,7 +1164,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP63"/>
+  <dimension ref="A1:CP64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1450,16 +1453,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1543,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1708,7 +1711,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1716,16 +1719,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1809,7 +1812,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1974,7 +1977,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1982,13 +1985,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2075,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2240,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2248,16 +2251,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2341,7 +2344,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2506,7 +2509,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2514,16 +2517,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2607,7 +2610,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2772,7 +2775,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2780,16 +2783,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E7" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2873,7 +2876,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3038,7 +3041,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3046,16 +3049,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3139,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3304,7 +3307,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3312,16 +3315,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3405,7 +3408,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3570,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3578,16 +3581,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3671,7 +3674,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3836,7 +3839,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3844,16 +3847,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3937,7 +3940,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4102,7 +4105,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4110,16 +4113,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E12" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4203,7 +4206,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4368,7 +4371,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4376,16 +4379,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4469,7 +4472,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4634,7 +4637,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4642,16 +4645,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4735,7 +4738,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4900,7 +4903,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4908,16 +4911,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -5001,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5166,7 +5169,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5174,16 +5177,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5267,7 +5270,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5432,7 +5435,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5440,16 +5443,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5533,7 +5536,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5698,7 +5701,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5706,16 +5709,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5799,7 +5802,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5964,7 +5967,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5972,16 +5975,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6065,7 +6068,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6230,7 +6233,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6238,16 +6241,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6331,7 +6334,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6496,7 +6499,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6504,16 +6507,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6597,7 +6600,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6762,7 +6765,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6770,16 +6773,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E22" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6863,7 +6866,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7028,7 +7031,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7036,16 +7039,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7129,7 +7132,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7294,7 +7297,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7302,16 +7305,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7395,7 +7398,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7560,7 +7563,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7568,16 +7571,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E25" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7661,7 +7664,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7826,7 +7829,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7834,16 +7837,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7927,7 +7930,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8092,7 +8095,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8100,16 +8103,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E27" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8193,7 +8196,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8358,7 +8361,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8366,16 +8369,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E28" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8459,7 +8462,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8624,7 +8627,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8632,16 +8635,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E29" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8725,7 +8728,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8890,7 +8893,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8898,16 +8901,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E30" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8991,7 +8994,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9156,7 +9159,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9164,16 +9167,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E31" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9257,7 +9260,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9422,7 +9425,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9430,16 +9433,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E32" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9523,7 +9526,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9688,7 +9691,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9696,16 +9699,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9789,7 +9792,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9954,7 +9957,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9962,16 +9965,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E34" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10055,7 +10058,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10220,7 +10223,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10234,16 +10237,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E35" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10327,7 +10330,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10492,7 +10495,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10506,16 +10509,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E36" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10599,7 +10602,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10764,7 +10767,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10778,13 +10781,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10871,7 +10874,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11036,7 +11039,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11050,16 +11053,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E38" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11143,7 +11146,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11308,7 +11311,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11322,16 +11325,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E39" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11415,7 +11418,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11580,7 +11583,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11594,16 +11597,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E40" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11687,7 +11690,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11852,7 +11855,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11866,16 +11869,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E41" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11959,7 +11962,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12124,7 +12127,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12138,16 +12141,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E42" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12231,7 +12234,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12396,7 +12399,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12410,16 +12413,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E43" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12503,7 +12506,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12668,7 +12671,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12682,16 +12685,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E44" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12775,7 +12778,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12940,7 +12943,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12954,16 +12957,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E45" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13047,7 +13050,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13212,7 +13215,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13226,16 +13229,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E46" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13319,7 +13322,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13484,7 +13487,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13498,16 +13501,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E47" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13591,7 +13594,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13756,7 +13759,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13770,16 +13773,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E48" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13863,7 +13866,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14028,7 +14031,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14042,16 +14045,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E49" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14135,7 +14138,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14300,7 +14303,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14314,16 +14317,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E50" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14407,7 +14410,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14572,7 +14575,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14586,16 +14589,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E51" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14679,7 +14682,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14844,7 +14847,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14858,16 +14861,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E52" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14951,7 +14954,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15116,7 +15119,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15130,16 +15133,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E53" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15223,7 +15226,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15388,7 +15391,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15402,16 +15405,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15495,7 +15498,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15660,7 +15663,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15674,13 +15677,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C55" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E55" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15764,7 +15767,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15929,7 +15932,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15943,10 +15946,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16030,7 +16033,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16195,7 +16198,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16293,7 +16296,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16556,7 +16559,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16819,7 +16822,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -17082,7 +17085,7 @@
         <v>0</v>
       </c>
       <c r="AH60" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI60">
         <v>0.04385278076244065</v>
@@ -17345,7 +17348,7 @@
         <v>0</v>
       </c>
       <c r="AH61" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI61">
         <v>0.01757226731119264</v>
@@ -17608,7 +17611,7 @@
         <v>0</v>
       </c>
       <c r="AH62" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI62">
         <v>0.05512246253185499</v>
@@ -17790,10 +17793,10 @@
         <v>99</v>
       </c>
       <c r="F63">
-        <v>0.0005530662709798406</v>
+        <v>0.0007538484415952063</v>
       </c>
       <c r="G63">
-        <v>0.0005530662709798406</v>
+        <v>0.0007538484415952063</v>
       </c>
       <c r="H63">
         <v>0</v>
@@ -17802,10 +17805,10 @@
         <v>0</v>
       </c>
       <c r="J63">
-        <v>0.001129672679885241</v>
+        <v>0.001194328506808029</v>
       </c>
       <c r="K63">
-        <v>0.001129672679885241</v>
+        <v>0.001194328506808029</v>
       </c>
       <c r="L63">
         <v>0</v>
@@ -17814,34 +17817,34 @@
         <v>0</v>
       </c>
       <c r="N63">
-        <v>14.08210079165862</v>
+        <v>10.28121258930295</v>
       </c>
       <c r="O63">
         <v>0</v>
       </c>
       <c r="P63">
-        <v>0.9963022005820252</v>
+        <v>0.9988084877990421</v>
       </c>
       <c r="Q63">
         <v>1</v>
       </c>
       <c r="R63">
-        <v>0.01876950593364631</v>
+        <v>0.016215050225833</v>
       </c>
       <c r="S63">
         <v>-0</v>
       </c>
       <c r="T63">
-        <v>0.1156042952559239</v>
+        <v>0.08196493183702271</v>
       </c>
       <c r="U63">
         <v>-0</v>
       </c>
       <c r="V63">
-        <v>0.9997300260474141</v>
+        <v>0.9997487613235339</v>
       </c>
       <c r="W63">
-        <v>0.9022408584663015</v>
+        <v>0.9357181143437892</v>
       </c>
       <c r="X63">
         <v>1</v>
@@ -17850,79 +17853,79 @@
         <v>1</v>
       </c>
       <c r="Z63">
-        <v>0.8845697945429987</v>
+        <v>0.911643612727801</v>
       </c>
       <c r="AB63">
-        <v>0.003161635495886697</v>
+        <v>0.002312921726475302</v>
       </c>
       <c r="AC63">
         <v>0</v>
       </c>
       <c r="AD63">
-        <v>0.9997300260474141</v>
+        <v>0.9997487613235339</v>
       </c>
       <c r="AE63">
         <v>1</v>
       </c>
       <c r="AF63">
-        <v>0.003161635495886697</v>
+        <v>0.002312921726475302</v>
       </c>
       <c r="AG63">
         <v>0</v>
       </c>
       <c r="AH63" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AI63">
-        <v>0.01271959061682842</v>
+        <v>0.0157574961492794</v>
       </c>
       <c r="AJ63">
         <v>0</v>
       </c>
       <c r="AK63">
-        <v>-460.58132618</v>
+        <v>-540.00893688</v>
       </c>
       <c r="AL63">
         <v>0</v>
       </c>
       <c r="AM63">
-        <v>18158.8055738202</v>
+        <v>22548.07566312009</v>
       </c>
       <c r="AN63">
         <v>10000</v>
       </c>
       <c r="AO63">
-        <v>18157.7495738202</v>
+        <v>22546.75566312009</v>
       </c>
       <c r="AP63">
         <v>10000</v>
       </c>
       <c r="AQ63">
-        <v>0.8158805573820203</v>
+        <v>1.254807566312009</v>
       </c>
       <c r="AR63">
         <v>0</v>
       </c>
       <c r="AS63">
-        <v>1.701641106649992</v>
+        <v>2.330613655487438</v>
       </c>
       <c r="AU63">
-        <v>97.15000000000001</v>
+        <v>105.4666666666667</v>
       </c>
       <c r="AW63">
-        <v>0.0002407443116559062</v>
+        <v>0.003306849891246448</v>
       </c>
       <c r="AX63">
         <v>1</v>
       </c>
       <c r="AY63">
-        <v>-2.075568047337285</v>
+        <v>-43.42392754621802</v>
       </c>
       <c r="AZ63">
         <v>0</v>
       </c>
       <c r="BA63">
-        <v>6613</v>
+        <v>4729</v>
       </c>
       <c r="BB63">
         <v>0</v>
@@ -17931,37 +17934,37 @@
         <v>1078.958333333333</v>
       </c>
       <c r="BD63">
-        <v>8581</v>
+        <v>6364</v>
       </c>
       <c r="BE63">
         <v>0</v>
       </c>
       <c r="BF63">
-        <v>15194</v>
+        <v>11093</v>
       </c>
       <c r="BG63">
         <v>0</v>
       </c>
       <c r="BH63">
-        <v>6669</v>
+        <v>4596</v>
       </c>
       <c r="BI63">
         <v>0</v>
       </c>
       <c r="BJ63">
-        <v>6612</v>
+        <v>4726</v>
       </c>
       <c r="BK63">
         <v>0</v>
       </c>
       <c r="BL63">
-        <v>1912</v>
+        <v>1768</v>
       </c>
       <c r="BM63">
         <v>0</v>
       </c>
       <c r="BN63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BO63">
         <v>0</v>
@@ -17973,49 +17976,49 @@
         <v>0</v>
       </c>
       <c r="BR63">
-        <v>8158.805573819994</v>
+        <v>12548.07566312</v>
       </c>
       <c r="BS63">
         <v>0</v>
       </c>
       <c r="BT63">
-        <v>0.04165887397552461</v>
+        <v>0.03680360457320977</v>
       </c>
       <c r="BU63">
         <v>100</v>
       </c>
       <c r="BV63">
-        <v>0.1303899207540317</v>
+        <v>0.09691074381991542</v>
       </c>
       <c r="BW63">
         <v>100</v>
       </c>
       <c r="BX63">
-        <v>0.01161459349193769</v>
+        <v>0.0107543703593493</v>
       </c>
       <c r="BY63">
         <v>100</v>
       </c>
       <c r="BZ63">
-        <v>0.009174774953634677</v>
+        <v>0.008572137443375455</v>
       </c>
       <c r="CA63">
         <v>1</v>
       </c>
       <c r="CB63">
-        <v>8619.386899999994</v>
+        <v>13088.0846</v>
       </c>
       <c r="CC63">
         <v>0</v>
       </c>
       <c r="CD63">
-        <v>8621.462468047332</v>
+        <v>13131.50852754622</v>
       </c>
       <c r="CE63">
         <v>0</v>
       </c>
       <c r="CF63">
-        <v>0.1359713694556786</v>
+        <v>0.1841131057155104</v>
       </c>
       <c r="CG63">
         <v>0</v>
@@ -18024,25 +18027,288 @@
         <v>10000</v>
       </c>
       <c r="CJ63">
-        <v>0.004209144269385233</v>
+        <v>0.005135928328699413</v>
       </c>
       <c r="CK63">
         <v>0</v>
       </c>
       <c r="CL63">
-        <v>1792278.455560063</v>
+        <v>3150529.607220278</v>
       </c>
       <c r="CM63">
         <v>0</v>
       </c>
       <c r="CN63" s="2">
-        <v>45399.31942677312</v>
+        <v>45399.42382790972</v>
       </c>
       <c r="CO63">
-        <v>-0.951306289405574</v>
+        <v>-0.9477002142299265</v>
       </c>
       <c r="CP63">
         <v>-0.9999999999999732</v>
+      </c>
+    </row>
+    <row r="64" spans="1:94">
+      <c r="A64" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E64" t="s">
+        <v>100</v>
+      </c>
+      <c r="F64">
+        <v>0.0006414899820990083</v>
+      </c>
+      <c r="G64">
+        <v>0.0006414899820990083</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64">
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <v>0.001328477660574801</v>
+      </c>
+      <c r="K64">
+        <v>0.001328477660574801</v>
+      </c>
+      <c r="L64">
+        <v>0</v>
+      </c>
+      <c r="M64">
+        <v>0</v>
+      </c>
+      <c r="N64">
+        <v>15.29171668667467</v>
+      </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64">
+        <v>0.9956453799384687</v>
+      </c>
+      <c r="Q64">
+        <v>1</v>
+      </c>
+      <c r="R64">
+        <v>0.05327124279558383</v>
+      </c>
+      <c r="S64">
+        <v>-0</v>
+      </c>
+      <c r="T64">
+        <v>0.1677595162566009</v>
+      </c>
+      <c r="U64">
+        <v>-0</v>
+      </c>
+      <c r="V64">
+        <v>0.9994199173917235</v>
+      </c>
+      <c r="W64">
+        <v>0.889240642842745</v>
+      </c>
+      <c r="X64">
+        <v>1</v>
+      </c>
+      <c r="Y64">
+        <v>1</v>
+      </c>
+      <c r="Z64">
+        <v>0.8323823485208039</v>
+      </c>
+      <c r="AB64">
+        <v>0.005183375682018007</v>
+      </c>
+      <c r="AC64">
+        <v>0</v>
+      </c>
+      <c r="AD64">
+        <v>0.9994199173917235</v>
+      </c>
+      <c r="AE64">
+        <v>1</v>
+      </c>
+      <c r="AF64">
+        <v>0.005183375682018007</v>
+      </c>
+      <c r="AG64">
+        <v>0</v>
+      </c>
+      <c r="AH64" t="s">
+        <v>208</v>
+      </c>
+      <c r="AI64">
+        <v>0.02035482894247531</v>
+      </c>
+      <c r="AJ64">
+        <v>0</v>
+      </c>
+      <c r="AK64">
+        <v>-456.56203922</v>
+      </c>
+      <c r="AL64">
+        <v>0</v>
+      </c>
+      <c r="AM64">
+        <v>18649.26186078061</v>
+      </c>
+      <c r="AN64">
+        <v>10000</v>
+      </c>
+      <c r="AO64">
+        <v>18648.34386078061</v>
+      </c>
+      <c r="AP64">
+        <v>10000</v>
+      </c>
+      <c r="AQ64">
+        <v>0.864926186078061</v>
+      </c>
+      <c r="AR64">
+        <v>0</v>
+      </c>
+      <c r="AS64">
+        <v>1.568561013907582</v>
+      </c>
+      <c r="AU64">
+        <v>108.6</v>
+      </c>
+      <c r="AW64">
+        <v>0.07372553707385335</v>
+      </c>
+      <c r="AX64">
+        <v>1</v>
+      </c>
+      <c r="AY64">
+        <v>-724.7654819357329</v>
+      </c>
+      <c r="AZ64">
+        <v>0</v>
+      </c>
+      <c r="BA64">
+        <v>6553</v>
+      </c>
+      <c r="BB64">
+        <v>0</v>
+      </c>
+      <c r="BC64">
+        <v>971.8333333333334</v>
+      </c>
+      <c r="BD64">
+        <v>8308</v>
+      </c>
+      <c r="BE64">
+        <v>0</v>
+      </c>
+      <c r="BF64">
+        <v>14861</v>
+      </c>
+      <c r="BG64">
+        <v>0</v>
+      </c>
+      <c r="BH64">
+        <v>6063</v>
+      </c>
+      <c r="BI64">
+        <v>0</v>
+      </c>
+      <c r="BJ64">
+        <v>6351</v>
+      </c>
+      <c r="BK64">
+        <v>0</v>
+      </c>
+      <c r="BL64">
+        <v>2245</v>
+      </c>
+      <c r="BM64">
+        <v>0</v>
+      </c>
+      <c r="BN64">
+        <v>202</v>
+      </c>
+      <c r="BO64">
+        <v>0</v>
+      </c>
+      <c r="BP64">
+        <v>0</v>
+      </c>
+      <c r="BQ64">
+        <v>0</v>
+      </c>
+      <c r="BR64">
+        <v>8649.261860780012</v>
+      </c>
+      <c r="BS64">
+        <v>0</v>
+      </c>
+      <c r="BT64">
+        <v>0.05626650540821408</v>
+      </c>
+      <c r="BU64">
+        <v>100</v>
+      </c>
+      <c r="BV64">
+        <v>0.201350385218753</v>
+      </c>
+      <c r="BW64">
+        <v>100</v>
+      </c>
+      <c r="BX64">
+        <v>0.01397581437787464</v>
+      </c>
+      <c r="BY64">
+        <v>100</v>
+      </c>
+      <c r="BZ64">
+        <v>0.0108258941514361</v>
+      </c>
+      <c r="CA64">
+        <v>1</v>
+      </c>
+      <c r="CB64">
+        <v>9105.823900000012</v>
+      </c>
+      <c r="CC64">
+        <v>0</v>
+      </c>
+      <c r="CD64">
+        <v>9830.589381935744</v>
+      </c>
+      <c r="CE64">
+        <v>0</v>
+      </c>
+      <c r="CF64">
+        <v>0.1025748473838637</v>
+      </c>
+      <c r="CG64">
+        <v>0</v>
+      </c>
+      <c r="CH64">
+        <v>10000</v>
+      </c>
+      <c r="CJ64">
+        <v>0.009517684887459807</v>
+      </c>
+      <c r="CK64">
+        <v>0</v>
+      </c>
+      <c r="CL64">
+        <v>7007359.345300732</v>
+      </c>
+      <c r="CM64">
+        <v>0</v>
+      </c>
+      <c r="CN64" s="2">
+        <v>45399.52560670529</v>
+      </c>
+      <c r="CO64">
+        <v>-0.8719527819991274</v>
+      </c>
+      <c r="CP64">
+        <v>-0.9999999999999741</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update LINKUSDT.json at 2024-04-17_21-43-00 bestfile_scores 0.0007332365388133643 bestfile_sharp 0.13850074425602726
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="264">
   <si>
     <t>Unnamed: 0.2</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>AUDIOUSDT</t>
+  </si>
+  <si>
+    <t>LINKUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1164,7 +1167,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CP64"/>
+  <dimension ref="A1:CP65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:94">
@@ -1453,16 +1456,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F2">
         <v>0.0009987329999999999</v>
@@ -1546,7 +1549,7 @@
         <v>0</v>
       </c>
       <c r="AH2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI2">
         <v>0.049606857</v>
@@ -1711,7 +1714,7 @@
         <v>0</v>
       </c>
       <c r="CN2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3" spans="1:94">
@@ -1719,16 +1722,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F3">
         <v>0.001058605</v>
@@ -1812,7 +1815,7 @@
         <v>0</v>
       </c>
       <c r="AH3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI3">
         <v>0.04006526</v>
@@ -1977,7 +1980,7 @@
         <v>0</v>
       </c>
       <c r="CN3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="4" spans="1:94">
@@ -1985,13 +1988,13 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
         <v>93</v>
@@ -2078,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="AH4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI4">
         <v>0.092575794</v>
@@ -2243,7 +2246,7 @@
         <v>0</v>
       </c>
       <c r="CN4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5" spans="1:94">
@@ -2251,16 +2254,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F5">
         <v>0.001186265</v>
@@ -2344,7 +2347,7 @@
         <v>0</v>
       </c>
       <c r="AH5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI5">
         <v>0.027448502</v>
@@ -2509,7 +2512,7 @@
         <v>0</v>
       </c>
       <c r="CN5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:94">
@@ -2517,16 +2520,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F6">
         <v>0.001076751</v>
@@ -2610,7 +2613,7 @@
         <v>0</v>
       </c>
       <c r="AH6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI6">
         <v>0.083929868</v>
@@ -2775,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="CN6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:94">
@@ -2783,16 +2786,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E7" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F7">
         <v>-0.000540801</v>
@@ -2876,7 +2879,7 @@
         <v>0</v>
       </c>
       <c r="AH7" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI7">
         <v>0.145376251</v>
@@ -3041,7 +3044,7 @@
         <v>0</v>
       </c>
       <c r="CN7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:94">
@@ -3049,16 +3052,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F8">
         <v>0.001278948</v>
@@ -3142,7 +3145,7 @@
         <v>0</v>
       </c>
       <c r="AH8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI8">
         <v>0.087987204</v>
@@ -3307,7 +3310,7 @@
         <v>0</v>
       </c>
       <c r="CN8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="9" spans="1:94">
@@ -3315,16 +3318,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F9">
         <v>0.000266144</v>
@@ -3408,7 +3411,7 @@
         <v>0</v>
       </c>
       <c r="AH9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI9">
         <v>0.118237951</v>
@@ -3573,7 +3576,7 @@
         <v>0</v>
       </c>
       <c r="CN9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" spans="1:94">
@@ -3581,16 +3584,16 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F10">
         <v>0.001013204</v>
@@ -3674,7 +3677,7 @@
         <v>0</v>
       </c>
       <c r="AH10" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI10">
         <v>0.08106915200000001</v>
@@ -3839,7 +3842,7 @@
         <v>0</v>
       </c>
       <c r="CN10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:94">
@@ -3847,16 +3850,16 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E11" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F11">
         <v>0.001228309</v>
@@ -3940,7 +3943,7 @@
         <v>0</v>
       </c>
       <c r="AH11" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI11">
         <v>0.027960571</v>
@@ -4105,7 +4108,7 @@
         <v>0</v>
       </c>
       <c r="CN11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:94">
@@ -4113,16 +4116,16 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F12">
         <v>0.0009776030000000001</v>
@@ -4206,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="AH12" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI12">
         <v>0.032951036</v>
@@ -4371,7 +4374,7 @@
         <v>0</v>
       </c>
       <c r="CN12" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:94">
@@ -4379,16 +4382,16 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F13">
         <v>-2.89E-05</v>
@@ -4472,7 +4475,7 @@
         <v>0</v>
       </c>
       <c r="AH13" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI13">
         <v>0.179185242</v>
@@ -4637,7 +4640,7 @@
         <v>0</v>
       </c>
       <c r="CN13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="1:94">
@@ -4645,16 +4648,16 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F14">
         <v>0.000431045</v>
@@ -4738,7 +4741,7 @@
         <v>0</v>
       </c>
       <c r="AH14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI14">
         <v>0.143233482</v>
@@ -4903,7 +4906,7 @@
         <v>0</v>
       </c>
       <c r="CN14" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" spans="1:94">
@@ -4911,16 +4914,16 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F15">
         <v>0.000327551</v>
@@ -5004,7 +5007,7 @@
         <v>0</v>
       </c>
       <c r="AH15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI15">
         <v>0.138115134</v>
@@ -5169,7 +5172,7 @@
         <v>0</v>
       </c>
       <c r="CN15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" spans="1:94">
@@ -5177,16 +5180,16 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F16">
         <v>0.001162093</v>
@@ -5270,7 +5273,7 @@
         <v>0</v>
       </c>
       <c r="AH16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI16">
         <v>0.09650975000000001</v>
@@ -5435,7 +5438,7 @@
         <v>0</v>
       </c>
       <c r="CN16" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="1:92">
@@ -5443,16 +5446,16 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D17" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F17">
         <v>0.00141042</v>
@@ -5536,7 +5539,7 @@
         <v>0</v>
       </c>
       <c r="AH17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI17">
         <v>0.060693695</v>
@@ -5701,7 +5704,7 @@
         <v>0</v>
       </c>
       <c r="CN17" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" spans="1:92">
@@ -5709,16 +5712,16 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D18" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E18" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F18">
         <v>0.000897625</v>
@@ -5802,7 +5805,7 @@
         <v>0</v>
       </c>
       <c r="AH18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI18">
         <v>0.107514363</v>
@@ -5967,7 +5970,7 @@
         <v>0</v>
       </c>
       <c r="CN18" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="19" spans="1:92">
@@ -5975,16 +5978,16 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F19">
         <v>0.000473511</v>
@@ -6068,7 +6071,7 @@
         <v>0</v>
       </c>
       <c r="AH19" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI19">
         <v>0.014898256</v>
@@ -6233,7 +6236,7 @@
         <v>0</v>
       </c>
       <c r="CN19" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="20" spans="1:92">
@@ -6241,16 +6244,16 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F20">
         <v>0.00029592</v>
@@ -6334,7 +6337,7 @@
         <v>0</v>
       </c>
       <c r="AH20" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI20">
         <v>0.02858403</v>
@@ -6499,7 +6502,7 @@
         <v>0</v>
       </c>
       <c r="CN20" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21" spans="1:92">
@@ -6507,16 +6510,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D21" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E21" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F21">
         <v>0.000354958</v>
@@ -6600,7 +6603,7 @@
         <v>0</v>
       </c>
       <c r="AH21" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI21">
         <v>0.082273481</v>
@@ -6765,7 +6768,7 @@
         <v>0</v>
       </c>
       <c r="CN21" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="22" spans="1:92">
@@ -6773,16 +6776,16 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F22">
         <v>0.000513154</v>
@@ -6866,7 +6869,7 @@
         <v>0</v>
       </c>
       <c r="AH22" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI22">
         <v>0.012592558</v>
@@ -7031,7 +7034,7 @@
         <v>0</v>
       </c>
       <c r="CN22" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" spans="1:92">
@@ -7039,16 +7042,16 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D23" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E23" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F23">
         <v>0.000263694</v>
@@ -7132,7 +7135,7 @@
         <v>0</v>
       </c>
       <c r="AH23" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI23">
         <v>0.00903967</v>
@@ -7297,7 +7300,7 @@
         <v>0</v>
       </c>
       <c r="CN23" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="24" spans="1:92">
@@ -7305,16 +7308,16 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F24">
         <v>0.00048524</v>
@@ -7398,7 +7401,7 @@
         <v>0</v>
       </c>
       <c r="AH24" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI24">
         <v>0.030046089</v>
@@ -7563,7 +7566,7 @@
         <v>0</v>
       </c>
       <c r="CN24" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:92">
@@ -7571,16 +7574,16 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E25" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F25">
         <v>0.000308954</v>
@@ -7664,7 +7667,7 @@
         <v>0</v>
       </c>
       <c r="AH25" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI25">
         <v>0.010607012</v>
@@ -7829,7 +7832,7 @@
         <v>0</v>
       </c>
       <c r="CN25" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="26" spans="1:92">
@@ -7837,16 +7840,16 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D26" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E26" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F26">
         <v>0.001706564</v>
@@ -7930,7 +7933,7 @@
         <v>0</v>
       </c>
       <c r="AH26" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI26">
         <v>0.053096335</v>
@@ -8095,7 +8098,7 @@
         <v>0</v>
       </c>
       <c r="CN26" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="27" spans="1:92">
@@ -8103,16 +8106,16 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D27" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E27" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F27">
         <v>0.001293263</v>
@@ -8196,7 +8199,7 @@
         <v>0</v>
       </c>
       <c r="AH27" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI27">
         <v>0.092674047</v>
@@ -8361,7 +8364,7 @@
         <v>0</v>
       </c>
       <c r="CN27" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="28" spans="1:92">
@@ -8369,16 +8372,16 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D28" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E28" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F28">
         <v>0.001493963</v>
@@ -8462,7 +8465,7 @@
         <v>0</v>
       </c>
       <c r="AH28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI28">
         <v>0.03099706</v>
@@ -8627,7 +8630,7 @@
         <v>0</v>
       </c>
       <c r="CN28" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="29" spans="1:92">
@@ -8635,16 +8638,16 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D29" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E29" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F29">
         <v>0.001124522</v>
@@ -8728,7 +8731,7 @@
         <v>0</v>
       </c>
       <c r="AH29" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI29">
         <v>0.069423731</v>
@@ -8893,7 +8896,7 @@
         <v>0</v>
       </c>
       <c r="CN29" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:92">
@@ -8901,16 +8904,16 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D30" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F30">
         <v>0.001194286</v>
@@ -8994,7 +8997,7 @@
         <v>0</v>
       </c>
       <c r="AH30" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI30">
         <v>0.060424834</v>
@@ -9159,7 +9162,7 @@
         <v>0</v>
       </c>
       <c r="CN30" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="31" spans="1:92">
@@ -9167,16 +9170,16 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D31" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E31" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F31">
         <v>0.002038684</v>
@@ -9260,7 +9263,7 @@
         <v>0</v>
       </c>
       <c r="AH31" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI31">
         <v>0.056666776</v>
@@ -9425,7 +9428,7 @@
         <v>0</v>
       </c>
       <c r="CN31" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="32" spans="1:92">
@@ -9433,16 +9436,16 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E32" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F32">
         <v>0.003509328</v>
@@ -9526,7 +9529,7 @@
         <v>0</v>
       </c>
       <c r="AH32" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI32">
         <v>0.098888062</v>
@@ -9691,7 +9694,7 @@
         <v>0</v>
       </c>
       <c r="CN32" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="33" spans="1:94">
@@ -9699,16 +9702,16 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F33">
         <v>0.001020607</v>
@@ -9792,7 +9795,7 @@
         <v>0</v>
       </c>
       <c r="AH33" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI33">
         <v>0.035815903</v>
@@ -9957,7 +9960,7 @@
         <v>0</v>
       </c>
       <c r="CN33" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" spans="1:94">
@@ -9965,16 +9968,16 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E34" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F34">
         <v>0.001036188</v>
@@ -10058,7 +10061,7 @@
         <v>0</v>
       </c>
       <c r="AH34" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI34">
         <v>0.037311133</v>
@@ -10223,7 +10226,7 @@
         <v>0</v>
       </c>
       <c r="CN34" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="CO34">
         <v>-0.814742818</v>
@@ -10237,16 +10240,16 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E35" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F35">
         <v>0.001410503</v>
@@ -10330,7 +10333,7 @@
         <v>0</v>
       </c>
       <c r="AH35" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI35">
         <v>0.041330496</v>
@@ -10495,7 +10498,7 @@
         <v>0</v>
       </c>
       <c r="CN35" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="CO35">
         <v>-0.753066891</v>
@@ -10509,16 +10512,16 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D36" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F36">
         <v>0.00072725</v>
@@ -10602,7 +10605,7 @@
         <v>0</v>
       </c>
       <c r="AH36" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI36">
         <v>0.047772102</v>
@@ -10767,7 +10770,7 @@
         <v>0</v>
       </c>
       <c r="CN36" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CO36">
         <v>-0.872335259</v>
@@ -10781,13 +10784,13 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D37" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -10874,7 +10877,7 @@
         <v>0</v>
       </c>
       <c r="AH37" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI37">
         <v>0.060484521</v>
@@ -11039,7 +11042,7 @@
         <v>0</v>
       </c>
       <c r="CN37" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="CO37">
         <v>-0.759885442</v>
@@ -11053,16 +11056,16 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E38" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F38">
         <v>0.000951107</v>
@@ -11146,7 +11149,7 @@
         <v>0</v>
       </c>
       <c r="AH38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI38">
         <v>0.061007062</v>
@@ -11311,7 +11314,7 @@
         <v>0</v>
       </c>
       <c r="CN38" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CO38">
         <v>-0.838900609</v>
@@ -11325,16 +11328,16 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D39" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E39" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F39">
         <v>0.001738925</v>
@@ -11418,7 +11421,7 @@
         <v>0</v>
       </c>
       <c r="AH39" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI39">
         <v>0.025236369</v>
@@ -11583,7 +11586,7 @@
         <v>0</v>
       </c>
       <c r="CN39" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CO39">
         <v>-0.780218664</v>
@@ -11597,16 +11600,16 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E40" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F40">
         <v>0.001263071</v>
@@ -11690,7 +11693,7 @@
         <v>0</v>
       </c>
       <c r="AH40" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI40">
         <v>0.031804424</v>
@@ -11855,7 +11858,7 @@
         <v>0</v>
       </c>
       <c r="CN40" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CO40">
         <v>-0.79992089</v>
@@ -11869,16 +11872,16 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D41" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E41" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F41">
         <v>0.002702281</v>
@@ -11962,7 +11965,7 @@
         <v>0</v>
       </c>
       <c r="AH41" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI41">
         <v>0.072404657</v>
@@ -12127,7 +12130,7 @@
         <v>0</v>
       </c>
       <c r="CN41" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CO41">
         <v>-0.528089775</v>
@@ -12141,16 +12144,16 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E42" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F42">
         <v>0.001559412</v>
@@ -12234,7 +12237,7 @@
         <v>0</v>
       </c>
       <c r="AH42" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI42">
         <v>0.06821192299999999</v>
@@ -12399,7 +12402,7 @@
         <v>0</v>
       </c>
       <c r="CN42" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CO42">
         <v>-0.754849911</v>
@@ -12413,16 +12416,16 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C43" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D43" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E43" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F43">
         <v>0.001270244</v>
@@ -12506,7 +12509,7 @@
         <v>0</v>
       </c>
       <c r="AH43" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI43">
         <v>0.069326524</v>
@@ -12671,7 +12674,7 @@
         <v>0</v>
       </c>
       <c r="CN43" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CO43">
         <v>-0.7655395739999999</v>
@@ -12685,16 +12688,16 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D44" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E44" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F44">
         <v>0.0009943969999999999</v>
@@ -12778,7 +12781,7 @@
         <v>0</v>
       </c>
       <c r="AH44" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI44">
         <v>0.036991009</v>
@@ -12943,7 +12946,7 @@
         <v>0</v>
       </c>
       <c r="CN44" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CO44">
         <v>-0.829764531</v>
@@ -12957,16 +12960,16 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C45" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D45" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E45" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F45">
         <v>0.002384052</v>
@@ -13050,7 +13053,7 @@
         <v>0</v>
       </c>
       <c r="AH45" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI45">
         <v>0.036729519</v>
@@ -13215,7 +13218,7 @@
         <v>0</v>
       </c>
       <c r="CN45" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CO45">
         <v>-0.404237806</v>
@@ -13229,16 +13232,16 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C46" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D46" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E46" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F46">
         <v>0.001488019</v>
@@ -13322,7 +13325,7 @@
         <v>0</v>
       </c>
       <c r="AH46" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI46">
         <v>0.045071814</v>
@@ -13487,7 +13490,7 @@
         <v>0</v>
       </c>
       <c r="CN46" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CO46">
         <v>-0.703677808</v>
@@ -13501,16 +13504,16 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D47" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E47" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F47">
         <v>0.001436084</v>
@@ -13594,7 +13597,7 @@
         <v>0</v>
       </c>
       <c r="AH47" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI47">
         <v>0.0580535</v>
@@ -13759,7 +13762,7 @@
         <v>0</v>
       </c>
       <c r="CN47" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CO47">
         <v>-0.753715321</v>
@@ -13773,16 +13776,16 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E48" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F48">
         <v>0.001379037</v>
@@ -13866,7 +13869,7 @@
         <v>0</v>
       </c>
       <c r="AH48" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI48">
         <v>0.056639031</v>
@@ -14031,7 +14034,7 @@
         <v>0</v>
       </c>
       <c r="CN48" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CO48">
         <v>-0.71793867</v>
@@ -14045,16 +14048,16 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C49" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E49" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F49">
         <v>0.00225795</v>
@@ -14138,7 +14141,7 @@
         <v>0</v>
       </c>
       <c r="AH49" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI49">
         <v>0.074241638</v>
@@ -14303,7 +14306,7 @@
         <v>0</v>
       </c>
       <c r="CN49" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CO49">
         <v>-0.655169358</v>
@@ -14317,16 +14320,16 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D50" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E50" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F50">
         <v>0.002405425</v>
@@ -14410,7 +14413,7 @@
         <v>0</v>
       </c>
       <c r="AH50" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI50">
         <v>0.05430774</v>
@@ -14575,7 +14578,7 @@
         <v>0</v>
       </c>
       <c r="CN50" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CO50">
         <v>-0.6872439380000001</v>
@@ -14589,16 +14592,16 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D51" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E51" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F51">
         <v>0.00267884</v>
@@ -14682,7 +14685,7 @@
         <v>0</v>
       </c>
       <c r="AH51" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI51">
         <v>0.080539377</v>
@@ -14847,7 +14850,7 @@
         <v>0</v>
       </c>
       <c r="CN51" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CO51">
         <v>-0.596275172</v>
@@ -14861,16 +14864,16 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D52" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E52" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F52">
         <v>0.001221159</v>
@@ -14954,7 +14957,7 @@
         <v>0</v>
       </c>
       <c r="AH52" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI52">
         <v>0.032588051</v>
@@ -15119,7 +15122,7 @@
         <v>0</v>
       </c>
       <c r="CN52" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CO52">
         <v>-0.808081961</v>
@@ -15133,16 +15136,16 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E53" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F53">
         <v>0.00093247</v>
@@ -15226,7 +15229,7 @@
         <v>0</v>
       </c>
       <c r="AH53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI53">
         <v>0.026475554</v>
@@ -15391,7 +15394,7 @@
         <v>0</v>
       </c>
       <c r="CN53" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="CO53">
         <v>-0.77227813</v>
@@ -15405,16 +15408,16 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C54" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D54" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E54" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F54">
         <v>0.0008229381467956</v>
@@ -15498,7 +15501,7 @@
         <v>0</v>
       </c>
       <c r="AH54" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI54">
         <v>0.0245106310926154</v>
@@ -15663,7 +15666,7 @@
         <v>0</v>
       </c>
       <c r="CN54" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CO54">
         <v>-0.8664117478627688</v>
@@ -15677,13 +15680,13 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F55">
         <v>0.0022239398231451</v>
@@ -15767,7 +15770,7 @@
         <v>0</v>
       </c>
       <c r="AH55" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI55">
         <v>0.0779439577559576</v>
@@ -15932,7 +15935,7 @@
         <v>0</v>
       </c>
       <c r="CN55" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="CO55">
         <v>-0.7108907987632488</v>
@@ -15946,10 +15949,10 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E56" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F56">
         <v>0.0018211096217568</v>
@@ -16033,7 +16036,7 @@
         <v>0</v>
       </c>
       <c r="AH56" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI56">
         <v>0.0402740604837066</v>
@@ -16198,7 +16201,7 @@
         <v>0</v>
       </c>
       <c r="CN56" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="CO56">
         <v>-0.7447372903525753</v>
@@ -16296,7 +16299,7 @@
         <v>0</v>
       </c>
       <c r="AH57" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI57">
         <v>0.04413639627430367</v>
@@ -16559,7 +16562,7 @@
         <v>0</v>
       </c>
       <c r="AH58" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI58">
         <v>0.05896463482078796</v>
@@ -16822,7 +16825,7 @@
         <v>0</v>
       </c>
       <c r="AH59" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI59">
         <v>0.008849841894546528</v>
@@ -17085,7 +17088,7 @@
         <v>0</v>
       </c>
       <c r="AH60" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI60">
         <v>0.04385278076244065</v>
@@ -17348,7 +17351,7 @@
         <v>0</v>
       </c>
       <c r="AH61" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI61">
         <v>0.01757226731119264</v>
@@ -17611,7 +17614,7 @@
         <v>0</v>
       </c>
       <c r="AH62" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI62">
         <v>0.05512246253185499</v>
@@ -17874,7 +17877,7 @@
         <v>0</v>
       </c>
       <c r="AH63" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI63">
         <v>0.0157574961492794</v>
@@ -18056,10 +18059,10 @@
         <v>100</v>
       </c>
       <c r="F64">
-        <v>0.0006414899820990083</v>
+        <v>0.001241696258706959</v>
       </c>
       <c r="G64">
-        <v>0.0006414899820990083</v>
+        <v>0.001241696258706959</v>
       </c>
       <c r="H64">
         <v>0</v>
@@ -18068,10 +18071,10 @@
         <v>0</v>
       </c>
       <c r="J64">
-        <v>0.001328477660574801</v>
+        <v>0.001665793195308174</v>
       </c>
       <c r="K64">
-        <v>0.001328477660574801</v>
+        <v>0.001665793195308174</v>
       </c>
       <c r="L64">
         <v>0</v>
@@ -18080,34 +18083,34 @@
         <v>0</v>
       </c>
       <c r="N64">
-        <v>15.29171668667467</v>
+        <v>9.308180415023152</v>
       </c>
       <c r="O64">
         <v>0</v>
       </c>
       <c r="P64">
-        <v>0.9956453799384687</v>
+        <v>0.9997315917944116</v>
       </c>
       <c r="Q64">
         <v>1</v>
       </c>
       <c r="R64">
-        <v>0.05327124279558383</v>
+        <v>0.06699082525840623</v>
       </c>
       <c r="S64">
         <v>-0</v>
       </c>
       <c r="T64">
-        <v>0.1677595162566009</v>
+        <v>0.1784430053360573</v>
       </c>
       <c r="U64">
         <v>-0</v>
       </c>
       <c r="V64">
-        <v>0.9994199173917235</v>
+        <v>0.9990865515256721</v>
       </c>
       <c r="W64">
-        <v>0.889240642842745</v>
+        <v>0.8675881375992838</v>
       </c>
       <c r="X64">
         <v>1</v>
@@ -18116,79 +18119,79 @@
         <v>1</v>
       </c>
       <c r="Z64">
-        <v>0.8323823485208039</v>
+        <v>0.8217073848222994</v>
       </c>
       <c r="AB64">
-        <v>0.005183375682018007</v>
+        <v>0.006931332671059251</v>
       </c>
       <c r="AC64">
         <v>0</v>
       </c>
       <c r="AD64">
-        <v>0.9994199173917235</v>
+        <v>0.9990865515256721</v>
       </c>
       <c r="AE64">
         <v>1</v>
       </c>
       <c r="AF64">
-        <v>0.005183375682018007</v>
+        <v>0.006931332671059251</v>
       </c>
       <c r="AG64">
         <v>0</v>
       </c>
       <c r="AH64" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AI64">
-        <v>0.02035482894247531</v>
+        <v>0.03487751847262728</v>
       </c>
       <c r="AJ64">
         <v>0</v>
       </c>
       <c r="AK64">
-        <v>-456.56203922</v>
+        <v>-819.7335469</v>
       </c>
       <c r="AL64">
         <v>0</v>
       </c>
       <c r="AM64">
-        <v>18649.26186078061</v>
+        <v>33400.08135309993</v>
       </c>
       <c r="AN64">
         <v>10000</v>
       </c>
       <c r="AO64">
-        <v>18648.34386078061</v>
+        <v>33398.14335309993</v>
       </c>
       <c r="AP64">
         <v>10000</v>
       </c>
       <c r="AQ64">
-        <v>0.864926186078061</v>
+        <v>2.340008135309993</v>
       </c>
       <c r="AR64">
         <v>0</v>
       </c>
       <c r="AS64">
-        <v>1.568561013907582</v>
+        <v>2.57595909342178</v>
       </c>
       <c r="AU64">
-        <v>108.6</v>
+        <v>117.25</v>
       </c>
       <c r="AW64">
-        <v>0.07372553707385335</v>
+        <v>0.04735158662886915</v>
       </c>
       <c r="AX64">
         <v>1</v>
       </c>
       <c r="AY64">
-        <v>-724.7654819357329</v>
+        <v>-1203.850914225728</v>
       </c>
       <c r="AZ64">
         <v>0</v>
       </c>
       <c r="BA64">
-        <v>6553</v>
+        <v>3915</v>
       </c>
       <c r="BB64">
         <v>0</v>
@@ -18197,37 +18200,37 @@
         <v>971.8333333333334</v>
       </c>
       <c r="BD64">
-        <v>8308</v>
+        <v>5131</v>
       </c>
       <c r="BE64">
         <v>0</v>
       </c>
       <c r="BF64">
-        <v>14861</v>
+        <v>9046</v>
       </c>
       <c r="BG64">
         <v>0</v>
       </c>
       <c r="BH64">
-        <v>6063</v>
+        <v>3281</v>
       </c>
       <c r="BI64">
         <v>0</v>
       </c>
       <c r="BJ64">
-        <v>6351</v>
+        <v>3799</v>
       </c>
       <c r="BK64">
         <v>0</v>
       </c>
       <c r="BL64">
-        <v>2245</v>
+        <v>1850</v>
       </c>
       <c r="BM64">
         <v>0</v>
       </c>
       <c r="BN64">
-        <v>202</v>
+        <v>116</v>
       </c>
       <c r="BO64">
         <v>0</v>
@@ -18239,49 +18242,49 @@
         <v>0</v>
       </c>
       <c r="BR64">
-        <v>8649.261860780012</v>
+        <v>23400.08135309999</v>
       </c>
       <c r="BS64">
         <v>0</v>
       </c>
       <c r="BT64">
-        <v>0.05626650540821408</v>
+        <v>0.06942761561462818</v>
       </c>
       <c r="BU64">
         <v>100</v>
       </c>
       <c r="BV64">
-        <v>0.201350385218753</v>
+        <v>0.216926037777943</v>
       </c>
       <c r="BW64">
         <v>100</v>
       </c>
       <c r="BX64">
-        <v>0.01397581437787464</v>
+        <v>0.01235704956127353</v>
       </c>
       <c r="BY64">
         <v>100</v>
       </c>
       <c r="BZ64">
-        <v>0.0108258941514361</v>
+        <v>0.01130768892999977</v>
       </c>
       <c r="CA64">
         <v>1</v>
       </c>
       <c r="CB64">
-        <v>9105.823900000012</v>
+        <v>24219.81489999999</v>
       </c>
       <c r="CC64">
         <v>0</v>
       </c>
       <c r="CD64">
-        <v>9830.589381935744</v>
+        <v>25423.66581422572</v>
       </c>
       <c r="CE64">
         <v>0</v>
       </c>
       <c r="CF64">
-        <v>0.1025748473838637</v>
+        <v>0.1539339465776871</v>
       </c>
       <c r="CG64">
         <v>0</v>
@@ -18290,25 +18293,288 @@
         <v>10000</v>
       </c>
       <c r="CJ64">
-        <v>0.009517684887459807</v>
+        <v>0.01491961414790997</v>
       </c>
       <c r="CK64">
         <v>0</v>
       </c>
       <c r="CL64">
-        <v>7007359.345300732</v>
+        <v>9382168.591397652</v>
       </c>
       <c r="CM64">
         <v>0</v>
       </c>
       <c r="CN64" s="2">
-        <v>45399.52560670529</v>
+        <v>45399.64982165807</v>
       </c>
       <c r="CO64">
-        <v>-0.8719527819991274</v>
+        <v>-0.7774025388699596</v>
       </c>
       <c r="CP64">
         <v>-0.9999999999999741</v>
+      </c>
+    </row>
+    <row r="65" spans="1:94">
+      <c r="A65" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E65" t="s">
+        <v>101</v>
+      </c>
+      <c r="F65">
+        <v>0.001648760113822867</v>
+      </c>
+      <c r="G65">
+        <v>0.001648760113822867</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <v>0.001362680305489894</v>
+      </c>
+      <c r="K65">
+        <v>0.001362680305489894</v>
+      </c>
+      <c r="L65">
+        <v>0</v>
+      </c>
+      <c r="M65">
+        <v>0</v>
+      </c>
+      <c r="N65">
+        <v>18.57756857903469</v>
+      </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65">
+        <v>0.9922517427670731</v>
+      </c>
+      <c r="Q65">
+        <v>1</v>
+      </c>
+      <c r="R65">
+        <v>0.08779594975698457</v>
+      </c>
+      <c r="S65">
+        <v>-0</v>
+      </c>
+      <c r="T65">
+        <v>0.2242944291876719</v>
+      </c>
+      <c r="U65">
+        <v>-0</v>
+      </c>
+      <c r="V65">
+        <v>0.9980133893870992</v>
+      </c>
+      <c r="W65">
+        <v>0.819569238235362</v>
+      </c>
+      <c r="X65">
+        <v>1</v>
+      </c>
+      <c r="Y65">
+        <v>1</v>
+      </c>
+      <c r="Z65">
+        <v>0.77579243929262</v>
+      </c>
+      <c r="AB65">
+        <v>0.0103684090772033</v>
+      </c>
+      <c r="AC65">
+        <v>0</v>
+      </c>
+      <c r="AD65">
+        <v>0.9980133893870992</v>
+      </c>
+      <c r="AE65">
+        <v>1</v>
+      </c>
+      <c r="AF65">
+        <v>0.0103684090772033</v>
+      </c>
+      <c r="AG65">
+        <v>0</v>
+      </c>
+      <c r="AH65" t="s">
+        <v>209</v>
+      </c>
+      <c r="AI65">
+        <v>0.06734990601851573</v>
+      </c>
+      <c r="AJ65">
+        <v>0</v>
+      </c>
+      <c r="AK65">
+        <v>-1984.794300448</v>
+      </c>
+      <c r="AL65">
+        <v>0</v>
+      </c>
+      <c r="AM65">
+        <v>59246.75699955177</v>
+      </c>
+      <c r="AN65">
+        <v>10000</v>
+      </c>
+      <c r="AO65">
+        <v>59246.82651955177</v>
+      </c>
+      <c r="AP65">
+        <v>10000</v>
+      </c>
+      <c r="AQ65">
+        <v>4.924675699955177</v>
+      </c>
+      <c r="AR65">
+        <v>0</v>
+      </c>
+      <c r="AS65">
+        <v>1.291053567274781</v>
+      </c>
+      <c r="AU65">
+        <v>91.53333333333333</v>
+      </c>
+      <c r="AW65">
+        <v>0.004982011324640392</v>
+      </c>
+      <c r="AX65">
+        <v>1</v>
+      </c>
+      <c r="AY65">
+        <v>-256.5141250313314</v>
+      </c>
+      <c r="AZ65">
+        <v>0</v>
+      </c>
+      <c r="BA65">
+        <v>6521</v>
+      </c>
+      <c r="BB65">
+        <v>0</v>
+      </c>
+      <c r="BC65">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BD65">
+        <v>13542</v>
+      </c>
+      <c r="BE65">
+        <v>0</v>
+      </c>
+      <c r="BF65">
+        <v>20063</v>
+      </c>
+      <c r="BG65">
+        <v>0</v>
+      </c>
+      <c r="BH65">
+        <v>5487</v>
+      </c>
+      <c r="BI65">
+        <v>0</v>
+      </c>
+      <c r="BJ65">
+        <v>6300</v>
+      </c>
+      <c r="BK65">
+        <v>0</v>
+      </c>
+      <c r="BL65">
+        <v>8055</v>
+      </c>
+      <c r="BM65">
+        <v>0</v>
+      </c>
+      <c r="BN65">
+        <v>221</v>
+      </c>
+      <c r="BO65">
+        <v>0</v>
+      </c>
+      <c r="BP65">
+        <v>0</v>
+      </c>
+      <c r="BQ65">
+        <v>0</v>
+      </c>
+      <c r="BR65">
+        <v>49246.756999552</v>
+      </c>
+      <c r="BS65">
+        <v>0</v>
+      </c>
+      <c r="BT65">
+        <v>0.09451401541946781</v>
+      </c>
+      <c r="BU65">
+        <v>100</v>
+      </c>
+      <c r="BV65">
+        <v>0.2889986808518486</v>
+      </c>
+      <c r="BW65">
+        <v>100</v>
+      </c>
+      <c r="BX65">
+        <v>0.0112665637005338</v>
+      </c>
+      <c r="BY65">
+        <v>100</v>
+      </c>
+      <c r="BZ65">
+        <v>0.01216878539459997</v>
+      </c>
+      <c r="CA65">
+        <v>1</v>
+      </c>
+      <c r="CB65">
+        <v>51231.55129999999</v>
+      </c>
+      <c r="CC65">
+        <v>0</v>
+      </c>
+      <c r="CD65">
+        <v>51488.06542503132</v>
+      </c>
+      <c r="CE65">
+        <v>0</v>
+      </c>
+      <c r="CF65">
+        <v>0.1238768379243737</v>
+      </c>
+      <c r="CG65">
+        <v>0</v>
+      </c>
+      <c r="CH65">
+        <v>10000</v>
+      </c>
+      <c r="CJ65">
+        <v>0.03831018518518518</v>
+      </c>
+      <c r="CK65">
+        <v>0</v>
+      </c>
+      <c r="CL65">
+        <v>45028078.73791471</v>
+      </c>
+      <c r="CM65">
+        <v>0</v>
+      </c>
+      <c r="CN65" s="2">
+        <v>45399.7561074746</v>
+      </c>
+      <c r="CO65">
+        <v>-0.7425340385328522</v>
+      </c>
+      <c r="CP65">
+        <v>-0.9999999999999732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update APEUSDT.json at 2024-04-18_01-41-22 bestfile_scores 0.0015429960144150046 bestfile_sharp 0.1544186673226351
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -18322,10 +18322,10 @@
         <v>101</v>
       </c>
       <c r="F65">
-        <v>0.001648760113822867</v>
+        <v>0.001598448309925837</v>
       </c>
       <c r="G65">
-        <v>0.001648760113822867</v>
+        <v>0.001598448309925837</v>
       </c>
       <c r="H65">
         <v>0</v>
@@ -18334,10 +18334,10 @@
         <v>0</v>
       </c>
       <c r="J65">
-        <v>0.001362680305489894</v>
+        <v>0.00133449784532762</v>
       </c>
       <c r="K65">
-        <v>0.001362680305489894</v>
+        <v>0.00133449784532762</v>
       </c>
       <c r="L65">
         <v>0</v>
@@ -18346,34 +18346,34 @@
         <v>0</v>
       </c>
       <c r="N65">
-        <v>18.57756857903469</v>
+        <v>12.17732165592808</v>
       </c>
       <c r="O65">
         <v>0</v>
       </c>
       <c r="P65">
-        <v>0.9922517427670731</v>
+        <v>0.9927512129224491</v>
       </c>
       <c r="Q65">
         <v>1</v>
       </c>
       <c r="R65">
-        <v>0.08779594975698457</v>
+        <v>0.09460417156557985</v>
       </c>
       <c r="S65">
         <v>-0</v>
       </c>
       <c r="T65">
-        <v>0.2242944291876719</v>
+        <v>0.213999537681425</v>
       </c>
       <c r="U65">
         <v>-0</v>
       </c>
       <c r="V65">
-        <v>0.9980133893870992</v>
+        <v>0.9979153312582629</v>
       </c>
       <c r="W65">
-        <v>0.819569238235362</v>
+        <v>0.8324903736256853</v>
       </c>
       <c r="X65">
         <v>1</v>
@@ -18382,22 +18382,22 @@
         <v>1</v>
       </c>
       <c r="Z65">
-        <v>0.77579243929262</v>
+        <v>0.7848792202190936</v>
       </c>
       <c r="AB65">
-        <v>0.0103684090772033</v>
+        <v>0.01117791231201725</v>
       </c>
       <c r="AC65">
         <v>0</v>
       </c>
       <c r="AD65">
-        <v>0.9980133893870992</v>
+        <v>0.9979153312582629</v>
       </c>
       <c r="AE65">
         <v>1</v>
       </c>
       <c r="AF65">
-        <v>0.0103684090772033</v>
+        <v>0.01117791231201725</v>
       </c>
       <c r="AG65">
         <v>0</v>
@@ -18406,55 +18406,55 @@
         <v>209</v>
       </c>
       <c r="AI65">
-        <v>0.06734990601851573</v>
+        <v>0.0617007650932976</v>
       </c>
       <c r="AJ65">
         <v>0</v>
       </c>
       <c r="AK65">
-        <v>-1984.794300448</v>
+        <v>-1863.186851128</v>
       </c>
       <c r="AL65">
         <v>0</v>
       </c>
       <c r="AM65">
-        <v>59246.75699955177</v>
+        <v>56118.44056887188</v>
       </c>
       <c r="AN65">
         <v>10000</v>
       </c>
       <c r="AO65">
-        <v>59246.82651955177</v>
+        <v>56117.56280887187</v>
       </c>
       <c r="AP65">
         <v>10000</v>
       </c>
       <c r="AQ65">
-        <v>4.924675699955177</v>
+        <v>4.611844056887188</v>
       </c>
       <c r="AR65">
         <v>0</v>
       </c>
       <c r="AS65">
-        <v>1.291053567274781</v>
+        <v>1.969069708491762</v>
       </c>
       <c r="AU65">
-        <v>91.53333333333333</v>
+        <v>77.91666666666667</v>
       </c>
       <c r="AW65">
-        <v>0.004982011324640392</v>
+        <v>0.004564030846676962</v>
       </c>
       <c r="AX65">
         <v>1</v>
       </c>
       <c r="AY65">
-        <v>-256.5141250313314</v>
+        <v>-219.9936855857287</v>
       </c>
       <c r="AZ65">
         <v>0</v>
       </c>
       <c r="BA65">
-        <v>6521</v>
+        <v>5031</v>
       </c>
       <c r="BB65">
         <v>0</v>
@@ -18463,37 +18463,37 @@
         <v>1079.958333333333</v>
       </c>
       <c r="BD65">
-        <v>13542</v>
+        <v>8120</v>
       </c>
       <c r="BE65">
         <v>0</v>
       </c>
       <c r="BF65">
-        <v>20063</v>
+        <v>13151</v>
       </c>
       <c r="BG65">
         <v>0</v>
       </c>
       <c r="BH65">
-        <v>5487</v>
+        <v>4803</v>
       </c>
       <c r="BI65">
         <v>0</v>
       </c>
       <c r="BJ65">
-        <v>6300</v>
+        <v>4992</v>
       </c>
       <c r="BK65">
         <v>0</v>
       </c>
       <c r="BL65">
-        <v>8055</v>
+        <v>3317</v>
       </c>
       <c r="BM65">
         <v>0</v>
       </c>
       <c r="BN65">
-        <v>221</v>
+        <v>39</v>
       </c>
       <c r="BO65">
         <v>0</v>
@@ -18505,49 +18505,49 @@
         <v>0</v>
       </c>
       <c r="BR65">
-        <v>49246.756999552</v>
+        <v>46118.44056887203</v>
       </c>
       <c r="BS65">
         <v>0</v>
       </c>
       <c r="BT65">
-        <v>0.09451401541946781</v>
+        <v>0.1020856288784739</v>
       </c>
       <c r="BU65">
         <v>100</v>
       </c>
       <c r="BV65">
-        <v>0.2889986808518486</v>
+        <v>0.2740559761527905</v>
       </c>
       <c r="BW65">
         <v>100</v>
       </c>
       <c r="BX65">
-        <v>0.0112665637005338</v>
+        <v>0.0121205208840009</v>
       </c>
       <c r="BY65">
         <v>100</v>
       </c>
       <c r="BZ65">
-        <v>0.01216878539459997</v>
+        <v>0.01316140176020784</v>
       </c>
       <c r="CA65">
         <v>1</v>
       </c>
       <c r="CB65">
-        <v>51231.55129999999</v>
+        <v>47981.62742000003</v>
       </c>
       <c r="CC65">
         <v>0</v>
       </c>
       <c r="CD65">
-        <v>51488.06542503132</v>
+        <v>48201.62110558576</v>
       </c>
       <c r="CE65">
         <v>0</v>
       </c>
       <c r="CF65">
-        <v>0.1238768379243737</v>
+        <v>0.1385007442560273</v>
       </c>
       <c r="CG65">
         <v>0</v>
@@ -18556,22 +18556,22 @@
         <v>10000</v>
       </c>
       <c r="CJ65">
-        <v>0.03831018518518518</v>
+        <v>0.03557098765432098</v>
       </c>
       <c r="CK65">
         <v>0</v>
       </c>
       <c r="CL65">
-        <v>45028078.73791471</v>
+        <v>13895500.92838126</v>
       </c>
       <c r="CM65">
         <v>0</v>
       </c>
       <c r="CN65" s="2">
-        <v>45399.7561074746</v>
+        <v>45399.90488704533</v>
       </c>
       <c r="CO65">
-        <v>-0.7425340385328522</v>
+        <v>-0.8140402180385446</v>
       </c>
       <c r="CP65">
         <v>-0.9999999999999732</v>

</xml_diff>

<commit_message>
Update KSMUSDT.json at 2024-04-18_10-42-41 bestfile_scores 0.0003989488073321612 bestfile_sharp 0.09526260076783863
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -18816,268 +18816,268 @@
         <v>94</v>
       </c>
       <c r="G66">
-        <v>0.001961133454451369</v>
+        <v>0.002475543019398341</v>
       </c>
       <c r="H66">
-        <v>0.0009805667272256846</v>
+        <v>0.00123777150969917</v>
       </c>
       <c r="I66">
-        <v>0.001456453477897801</v>
+        <v>0.002666291574861868</v>
       </c>
       <c r="J66">
-        <v>0.001456453477897801</v>
+        <v>0.002666291574861868</v>
       </c>
       <c r="K66">
-        <v>0.004767794115462154</v>
+        <v>0.006191730177007426</v>
       </c>
       <c r="L66">
-        <v>0.002383897057731077</v>
+        <v>0.003095865088503713</v>
       </c>
       <c r="M66">
-        <v>0.001351066794805456</v>
+        <v>0.002224541514668066</v>
       </c>
       <c r="N66">
-        <v>0.001351066794805456</v>
+        <v>0.002224541514668066</v>
       </c>
       <c r="O66">
-        <v>34.26094570928196</v>
+        <v>10.23336252189142</v>
       </c>
       <c r="P66">
-        <v>19.09676007005254</v>
+        <v>19.53021015761821</v>
       </c>
       <c r="Q66">
-        <v>0.4445311686338452</v>
+        <v>0.4473841595028464</v>
       </c>
       <c r="R66">
-        <v>0.5019127124297752</v>
+        <v>0.636906873305635</v>
       </c>
       <c r="S66">
-        <v>0.03999142926048058</v>
+        <v>0.04048297718732324</v>
       </c>
       <c r="T66">
-        <v>0.09288085922456882</v>
+        <v>0.0891402572621659</v>
       </c>
       <c r="U66">
-        <v>0.1638747636881711</v>
+        <v>0.1086999689042422</v>
       </c>
       <c r="V66">
-        <v>0.2491474583714446</v>
+        <v>0.1789711743861446</v>
       </c>
       <c r="W66">
-        <v>0.9996548524216143</v>
+        <v>0.9997404602444955</v>
       </c>
       <c r="X66">
-        <v>0.9089758609609809</v>
+        <v>0.9204435938834532</v>
       </c>
       <c r="Y66">
-        <v>0.7928407610137149</v>
+        <v>0.8435321711440263</v>
       </c>
       <c r="Z66">
-        <v>0.9977170792731698</v>
+        <v>0.9975264032405107</v>
       </c>
       <c r="AA66">
-        <v>0.7922206819930464</v>
+        <v>0.7953278973769896</v>
       </c>
       <c r="AB66">
-        <v>0.7509364804626362</v>
+        <v>0.8209055440456304</v>
       </c>
       <c r="AC66">
-        <v>0.002448301082287046</v>
+        <v>0.002542330315294323</v>
       </c>
       <c r="AD66">
-        <v>0.01087253808693166</v>
+        <v>0.01083306576401342</v>
       </c>
       <c r="AE66">
-        <v>0.9996548524216143</v>
+        <v>0.9997404602444955</v>
       </c>
       <c r="AF66">
-        <v>0.9977170792731698</v>
+        <v>0.9975264032405107</v>
       </c>
       <c r="AG66">
-        <v>0.002448301082287046</v>
+        <v>0.002542330315294323</v>
       </c>
       <c r="AH66">
-        <v>0.01087253808693166</v>
+        <v>0.01083306576401342</v>
       </c>
       <c r="AI66" t="s">
         <v>212</v>
       </c>
       <c r="AJ66">
-        <v>0.01299794879664704</v>
+        <v>0.01228964656713829</v>
       </c>
       <c r="AK66">
-        <v>0.075429806682414</v>
+        <v>0.09024694460460349</v>
       </c>
       <c r="AL66">
-        <v>-2611.67281266</v>
+        <v>-2628.71634146</v>
       </c>
       <c r="AM66">
-        <v>-2945.00469136</v>
+        <v>-2633.4802084</v>
       </c>
       <c r="AN66">
-        <v>44442.63308733977</v>
+        <v>65691.49795854004</v>
       </c>
       <c r="AO66">
-        <v>30284.16490863989</v>
+        <v>75930.64399160004</v>
       </c>
       <c r="AP66">
-        <v>44440.41308733977</v>
+        <v>65691.49795854004</v>
       </c>
       <c r="AQ66">
-        <v>30241.52650863989</v>
+        <v>75725.47639160004</v>
       </c>
       <c r="AR66">
-        <v>3.444263308733977</v>
+        <v>5.569149795854004</v>
       </c>
       <c r="AS66">
-        <v>2.028416490863989</v>
+        <v>6.593064399160004</v>
       </c>
       <c r="AT66">
-        <v>0.6995463200807678</v>
+        <v>2.34375053487377</v>
       </c>
       <c r="AU66">
-        <v>1.253850827715871</v>
+        <v>1.22765895435387</v>
       </c>
       <c r="AV66">
-        <v>87.7</v>
+        <v>115.4833333333333</v>
       </c>
       <c r="AW66">
-        <v>119.3333333333333</v>
+        <v>97.81666666666666</v>
       </c>
       <c r="AX66">
-        <v>0.02371218174737122</v>
+        <v>0.04008462811781553</v>
       </c>
       <c r="AY66">
-        <v>0.01066582853855195</v>
+        <v>0</v>
       </c>
       <c r="AZ66">
-        <v>-899.9788992513356</v>
+        <v>-2435.364794068255</v>
       </c>
       <c r="BA66">
-        <v>-250.4293768409455</v>
+        <v>0</v>
       </c>
       <c r="BB66">
-        <v>11210</v>
+        <v>3123</v>
       </c>
       <c r="BC66">
-        <v>6442</v>
+        <v>6617</v>
       </c>
       <c r="BD66">
         <v>761.3333333333334</v>
       </c>
       <c r="BE66">
-        <v>14874</v>
+        <v>4668</v>
       </c>
       <c r="BF66">
-        <v>8097</v>
+        <v>8252</v>
       </c>
       <c r="BG66">
-        <v>26084</v>
+        <v>7791</v>
       </c>
       <c r="BH66">
-        <v>14539</v>
+        <v>14869</v>
       </c>
       <c r="BI66">
-        <v>11127</v>
+        <v>2463</v>
       </c>
       <c r="BJ66">
-        <v>6417</v>
+        <v>4550</v>
       </c>
       <c r="BK66">
-        <v>11190</v>
+        <v>3089</v>
       </c>
       <c r="BL66">
-        <v>6430</v>
+        <v>6617</v>
       </c>
       <c r="BM66">
-        <v>3641</v>
+        <v>2068</v>
       </c>
       <c r="BN66">
-        <v>1680</v>
+        <v>3702</v>
       </c>
       <c r="BO66">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="BP66">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="BQ66">
-        <v>106</v>
+        <v>137</v>
       </c>
       <c r="BR66">
         <v>0</v>
       </c>
       <c r="BS66">
-        <v>34442.63308733996</v>
+        <v>55691.49795854005</v>
       </c>
       <c r="BT66">
-        <v>20284.16490864001</v>
+        <v>65930.64399159997</v>
       </c>
       <c r="BU66">
-        <v>0.02962572059445111</v>
+        <v>0.02546789158839128</v>
       </c>
       <c r="BV66">
-        <v>0.08787186933944816</v>
+        <v>0.08139585643292656</v>
       </c>
       <c r="BW66">
-        <v>0.08906833053975084</v>
+        <v>0.05726307434505765</v>
       </c>
       <c r="BX66">
-        <v>0.1982745922405625</v>
+        <v>0.1519563865655393</v>
       </c>
       <c r="BY66">
-        <v>0.0105701980200897</v>
+        <v>0.007683797017581389</v>
       </c>
       <c r="BZ66">
-        <v>0.0131629555514272</v>
+        <v>0.0102698422326152</v>
       </c>
       <c r="CA66">
-        <v>0.00696540151154724</v>
+        <v>0.006191502740431796</v>
       </c>
       <c r="CB66">
-        <v>0.01463033437010301</v>
+        <v>0.01126058911142145</v>
       </c>
       <c r="CC66">
-        <v>37054.30589999996</v>
+        <v>58320.21430000005</v>
       </c>
       <c r="CD66">
-        <v>23229.16960000001</v>
+        <v>68564.12419999996</v>
       </c>
       <c r="CE66">
-        <v>37954.2847992513</v>
+        <v>60755.57909406831</v>
       </c>
       <c r="CF66">
-        <v>23479.59897684096</v>
+        <v>68564.12419999996</v>
       </c>
       <c r="CG66">
-        <v>0.1544186673226351</v>
+        <v>0.1647857813081419</v>
       </c>
       <c r="CH66">
-        <v>0.08142804639025134</v>
+        <v>0.1491322394877734</v>
       </c>
       <c r="CI66">
         <v>10000</v>
       </c>
       <c r="CK66">
-        <v>0.0007661577190390194</v>
+        <v>0.002681552016636568</v>
       </c>
       <c r="CL66">
-        <v>0.008044656049909702</v>
+        <v>0.03239752640507853</v>
       </c>
       <c r="CM66">
-        <v>13686665.26837973</v>
+        <v>34082601.71958958</v>
       </c>
       <c r="CN66">
-        <v>12392869.99238669</v>
+        <v>28802806.1197283</v>
       </c>
       <c r="CO66" s="2">
-        <v>45400.07041536496</v>
+        <v>45400.24312405257</v>
       </c>
       <c r="CP66">
-        <v>-0.830161895070457</v>
+        <v>-0.7661604887809055</v>
       </c>
       <c r="CQ66">
-        <v>-0.4972522286795623</v>
+        <v>-0.4563890361669725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update KSMUSDT.json at 2024-04-18_15-37-26 bestfile_scores 0.0008446797928198357 bestfile_sharp 0.14958437200352093
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="277">
   <si>
     <t>Unnamed: 0.3</t>
   </si>
@@ -299,6 +299,9 @@
   </si>
   <si>
     <t>APEUSDT</t>
+  </si>
+  <si>
+    <t>KSMUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1203,7 +1206,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CQ66"/>
+  <dimension ref="A1:CQ67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:95">
@@ -1495,19 +1498,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G2">
         <v>0.0009987329999999999</v>
@@ -1591,7 +1594,7 @@
         <v>0</v>
       </c>
       <c r="AI2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ2">
         <v>0.049606857</v>
@@ -1756,7 +1759,7 @@
         <v>0</v>
       </c>
       <c r="CO2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3" spans="1:95">
@@ -1764,19 +1767,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G3">
         <v>0.001058605</v>
@@ -1860,7 +1863,7 @@
         <v>0</v>
       </c>
       <c r="AI3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ3">
         <v>0.04006526</v>
@@ -2025,7 +2028,7 @@
         <v>0</v>
       </c>
       <c r="CO3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" spans="1:95">
@@ -2033,19 +2036,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G4">
         <v>0.000882894</v>
@@ -2129,7 +2132,7 @@
         <v>0</v>
       </c>
       <c r="AI4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ4">
         <v>0.092575794</v>
@@ -2294,7 +2297,7 @@
         <v>0</v>
       </c>
       <c r="CO4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:95">
@@ -2302,19 +2305,19 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G5">
         <v>0.001186265</v>
@@ -2398,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="AI5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ5">
         <v>0.027448502</v>
@@ -2563,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="CO5" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:95">
@@ -2571,19 +2574,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G6">
         <v>0.001076751</v>
@@ -2667,7 +2670,7 @@
         <v>0</v>
       </c>
       <c r="AI6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ6">
         <v>0.083929868</v>
@@ -2832,7 +2835,7 @@
         <v>0</v>
       </c>
       <c r="CO6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:95">
@@ -2840,19 +2843,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G7">
         <v>-0.000540801</v>
@@ -2936,7 +2939,7 @@
         <v>0</v>
       </c>
       <c r="AI7" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ7">
         <v>0.145376251</v>
@@ -3101,7 +3104,7 @@
         <v>0</v>
       </c>
       <c r="CO7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:95">
@@ -3109,19 +3112,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E8" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G8">
         <v>0.001278948</v>
@@ -3205,7 +3208,7 @@
         <v>0</v>
       </c>
       <c r="AI8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ8">
         <v>0.087987204</v>
@@ -3370,7 +3373,7 @@
         <v>0</v>
       </c>
       <c r="CO8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:95">
@@ -3378,19 +3381,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F9" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G9">
         <v>0.000266144</v>
@@ -3474,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="AI9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ9">
         <v>0.118237951</v>
@@ -3639,7 +3642,7 @@
         <v>0</v>
       </c>
       <c r="CO9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:95">
@@ -3647,19 +3650,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G10">
         <v>0.001013204</v>
@@ -3743,7 +3746,7 @@
         <v>0</v>
       </c>
       <c r="AI10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ10">
         <v>0.08106915200000001</v>
@@ -3908,7 +3911,7 @@
         <v>0</v>
       </c>
       <c r="CO10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:95">
@@ -3916,19 +3919,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F11" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G11">
         <v>0.001228309</v>
@@ -4012,7 +4015,7 @@
         <v>0</v>
       </c>
       <c r="AI11" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ11">
         <v>0.027960571</v>
@@ -4177,7 +4180,7 @@
         <v>0</v>
       </c>
       <c r="CO11" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:95">
@@ -4185,19 +4188,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F12" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G12">
         <v>0.0009776030000000001</v>
@@ -4281,7 +4284,7 @@
         <v>0</v>
       </c>
       <c r="AI12" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ12">
         <v>0.032951036</v>
@@ -4446,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="CO12" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:95">
@@ -4454,19 +4457,19 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E13" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G13">
         <v>-2.89E-05</v>
@@ -4550,7 +4553,7 @@
         <v>0</v>
       </c>
       <c r="AI13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ13">
         <v>0.179185242</v>
@@ -4715,7 +4718,7 @@
         <v>0</v>
       </c>
       <c r="CO13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="14" spans="1:95">
@@ -4723,19 +4726,19 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G14">
         <v>0.000431045</v>
@@ -4819,7 +4822,7 @@
         <v>0</v>
       </c>
       <c r="AI14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ14">
         <v>0.143233482</v>
@@ -4984,7 +4987,7 @@
         <v>0</v>
       </c>
       <c r="CO14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:95">
@@ -4992,19 +4995,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G15">
         <v>0.000327551</v>
@@ -5088,7 +5091,7 @@
         <v>0</v>
       </c>
       <c r="AI15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ15">
         <v>0.138115134</v>
@@ -5253,7 +5256,7 @@
         <v>0</v>
       </c>
       <c r="CO15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:95">
@@ -5261,19 +5264,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G16">
         <v>0.001162093</v>
@@ -5357,7 +5360,7 @@
         <v>0</v>
       </c>
       <c r="AI16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ16">
         <v>0.09650975000000001</v>
@@ -5522,7 +5525,7 @@
         <v>0</v>
       </c>
       <c r="CO16" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="17" spans="1:93">
@@ -5530,19 +5533,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E17" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F17" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G17">
         <v>0.00141042</v>
@@ -5626,7 +5629,7 @@
         <v>0</v>
       </c>
       <c r="AI17" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ17">
         <v>0.060693695</v>
@@ -5791,7 +5794,7 @@
         <v>0</v>
       </c>
       <c r="CO17" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="18" spans="1:93">
@@ -5799,19 +5802,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G18">
         <v>0.000897625</v>
@@ -5895,7 +5898,7 @@
         <v>0</v>
       </c>
       <c r="AI18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ18">
         <v>0.107514363</v>
@@ -6060,7 +6063,7 @@
         <v>0</v>
       </c>
       <c r="CO18" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="1:93">
@@ -6068,19 +6071,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F19" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G19">
         <v>0.000473511</v>
@@ -6164,7 +6167,7 @@
         <v>0</v>
       </c>
       <c r="AI19" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ19">
         <v>0.014898256</v>
@@ -6329,7 +6332,7 @@
         <v>0</v>
       </c>
       <c r="CO19" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" spans="1:93">
@@ -6337,19 +6340,19 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G20">
         <v>0.00029592</v>
@@ -6433,7 +6436,7 @@
         <v>0</v>
       </c>
       <c r="AI20" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ20">
         <v>0.02858403</v>
@@ -6598,7 +6601,7 @@
         <v>0</v>
       </c>
       <c r="CO20" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="21" spans="1:93">
@@ -6606,19 +6609,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G21">
         <v>0.000354958</v>
@@ -6702,7 +6705,7 @@
         <v>0</v>
       </c>
       <c r="AI21" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ21">
         <v>0.082273481</v>
@@ -6867,7 +6870,7 @@
         <v>0</v>
       </c>
       <c r="CO21" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="22" spans="1:93">
@@ -6875,19 +6878,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F22" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G22">
         <v>0.000513154</v>
@@ -6971,7 +6974,7 @@
         <v>0</v>
       </c>
       <c r="AI22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ22">
         <v>0.012592558</v>
@@ -7136,7 +7139,7 @@
         <v>0</v>
       </c>
       <c r="CO22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:93">
@@ -7144,19 +7147,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F23" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G23">
         <v>0.000263694</v>
@@ -7240,7 +7243,7 @@
         <v>0</v>
       </c>
       <c r="AI23" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ23">
         <v>0.00903967</v>
@@ -7405,7 +7408,7 @@
         <v>0</v>
       </c>
       <c r="CO23" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" spans="1:93">
@@ -7413,19 +7416,19 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E24" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G24">
         <v>0.00048524</v>
@@ -7509,7 +7512,7 @@
         <v>0</v>
       </c>
       <c r="AI24" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ24">
         <v>0.030046089</v>
@@ -7674,7 +7677,7 @@
         <v>0</v>
       </c>
       <c r="CO24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="25" spans="1:93">
@@ -7682,19 +7685,19 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F25" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G25">
         <v>0.000308954</v>
@@ -7778,7 +7781,7 @@
         <v>0</v>
       </c>
       <c r="AI25" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ25">
         <v>0.010607012</v>
@@ -7943,7 +7946,7 @@
         <v>0</v>
       </c>
       <c r="CO25" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:93">
@@ -7951,19 +7954,19 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E26" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G26">
         <v>0.001706564</v>
@@ -8047,7 +8050,7 @@
         <v>0</v>
       </c>
       <c r="AI26" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ26">
         <v>0.053096335</v>
@@ -8212,7 +8215,7 @@
         <v>0</v>
       </c>
       <c r="CO26" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="27" spans="1:93">
@@ -8220,19 +8223,19 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E27" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F27" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G27">
         <v>0.001293263</v>
@@ -8316,7 +8319,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ27">
         <v>0.092674047</v>
@@ -8481,7 +8484,7 @@
         <v>0</v>
       </c>
       <c r="CO27" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="28" spans="1:93">
@@ -8489,19 +8492,19 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F28" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G28">
         <v>0.001493963</v>
@@ -8585,7 +8588,7 @@
         <v>0</v>
       </c>
       <c r="AI28" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ28">
         <v>0.03099706</v>
@@ -8750,7 +8753,7 @@
         <v>0</v>
       </c>
       <c r="CO28" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="29" spans="1:93">
@@ -8758,19 +8761,19 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E29" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G29">
         <v>0.001124522</v>
@@ -8854,7 +8857,7 @@
         <v>0</v>
       </c>
       <c r="AI29" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ29">
         <v>0.069423731</v>
@@ -9019,7 +9022,7 @@
         <v>0</v>
       </c>
       <c r="CO29" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="30" spans="1:93">
@@ -9027,19 +9030,19 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E30" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F30" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G30">
         <v>0.001194286</v>
@@ -9123,7 +9126,7 @@
         <v>0</v>
       </c>
       <c r="AI30" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ30">
         <v>0.060424834</v>
@@ -9288,7 +9291,7 @@
         <v>0</v>
       </c>
       <c r="CO30" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="31" spans="1:93">
@@ -9296,19 +9299,19 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E31" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F31" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G31">
         <v>0.002038684</v>
@@ -9392,7 +9395,7 @@
         <v>0</v>
       </c>
       <c r="AI31" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ31">
         <v>0.056666776</v>
@@ -9557,7 +9560,7 @@
         <v>0</v>
       </c>
       <c r="CO31" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="32" spans="1:93">
@@ -9565,19 +9568,19 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E32" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F32" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G32">
         <v>0.003509328</v>
@@ -9661,7 +9664,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ32">
         <v>0.098888062</v>
@@ -9826,7 +9829,7 @@
         <v>0</v>
       </c>
       <c r="CO32" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33" spans="1:95">
@@ -9834,19 +9837,19 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E33" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F33" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G33">
         <v>0.001020607</v>
@@ -9930,7 +9933,7 @@
         <v>0</v>
       </c>
       <c r="AI33" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ33">
         <v>0.035815903</v>
@@ -10095,7 +10098,7 @@
         <v>0</v>
       </c>
       <c r="CO33" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="34" spans="1:95">
@@ -10103,19 +10106,19 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E34" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F34" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G34">
         <v>0.001036188</v>
@@ -10199,7 +10202,7 @@
         <v>0</v>
       </c>
       <c r="AI34" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ34">
         <v>0.037311133</v>
@@ -10364,7 +10367,7 @@
         <v>0</v>
       </c>
       <c r="CO34" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="CP34">
         <v>-0.814742818</v>
@@ -10378,19 +10381,19 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E35" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F35" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G35">
         <v>0.001410503</v>
@@ -10474,7 +10477,7 @@
         <v>0</v>
       </c>
       <c r="AI35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ35">
         <v>0.041330496</v>
@@ -10639,7 +10642,7 @@
         <v>0</v>
       </c>
       <c r="CO35" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CP35">
         <v>-0.753066891</v>
@@ -10653,19 +10656,19 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F36" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G36">
         <v>0.00072725</v>
@@ -10749,7 +10752,7 @@
         <v>0</v>
       </c>
       <c r="AI36" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ36">
         <v>0.047772102</v>
@@ -10914,7 +10917,7 @@
         <v>0</v>
       </c>
       <c r="CO36" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CP36">
         <v>-0.872335259</v>
@@ -10928,19 +10931,19 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F37" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G37">
         <v>0.001640077</v>
@@ -11024,7 +11027,7 @@
         <v>0</v>
       </c>
       <c r="AI37" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ37">
         <v>0.060484521</v>
@@ -11189,7 +11192,7 @@
         <v>0</v>
       </c>
       <c r="CO37" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CP37">
         <v>-0.759885442</v>
@@ -11203,19 +11206,19 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F38" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G38">
         <v>0.000951107</v>
@@ -11299,7 +11302,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ38">
         <v>0.061007062</v>
@@ -11464,7 +11467,7 @@
         <v>0</v>
       </c>
       <c r="CO38" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CP38">
         <v>-0.838900609</v>
@@ -11478,19 +11481,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E39" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F39" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G39">
         <v>0.001738925</v>
@@ -11574,7 +11577,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ39">
         <v>0.025236369</v>
@@ -11739,7 +11742,7 @@
         <v>0</v>
       </c>
       <c r="CO39" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CP39">
         <v>-0.780218664</v>
@@ -11753,19 +11756,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E40" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F40" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G40">
         <v>0.001263071</v>
@@ -11849,7 +11852,7 @@
         <v>0</v>
       </c>
       <c r="AI40" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ40">
         <v>0.031804424</v>
@@ -12014,7 +12017,7 @@
         <v>0</v>
       </c>
       <c r="CO40" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CP40">
         <v>-0.79992089</v>
@@ -12028,19 +12031,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F41" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G41">
         <v>0.002702281</v>
@@ -12124,7 +12127,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ41">
         <v>0.072404657</v>
@@ -12289,7 +12292,7 @@
         <v>0</v>
       </c>
       <c r="CO41" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CP41">
         <v>-0.528089775</v>
@@ -12303,19 +12306,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E42" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F42" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G42">
         <v>0.001559412</v>
@@ -12399,7 +12402,7 @@
         <v>0</v>
       </c>
       <c r="AI42" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ42">
         <v>0.06821192299999999</v>
@@ -12564,7 +12567,7 @@
         <v>0</v>
       </c>
       <c r="CO42" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CP42">
         <v>-0.754849911</v>
@@ -12578,19 +12581,19 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E43" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F43" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G43">
         <v>0.001270244</v>
@@ -12674,7 +12677,7 @@
         <v>0</v>
       </c>
       <c r="AI43" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ43">
         <v>0.069326524</v>
@@ -12839,7 +12842,7 @@
         <v>0</v>
       </c>
       <c r="CO43" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CP43">
         <v>-0.7655395739999999</v>
@@ -12853,19 +12856,19 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F44" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G44">
         <v>0.0009943969999999999</v>
@@ -12949,7 +12952,7 @@
         <v>0</v>
       </c>
       <c r="AI44" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ44">
         <v>0.036991009</v>
@@ -13114,7 +13117,7 @@
         <v>0</v>
       </c>
       <c r="CO44" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CP44">
         <v>-0.829764531</v>
@@ -13128,19 +13131,19 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E45" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F45" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G45">
         <v>0.002384052</v>
@@ -13224,7 +13227,7 @@
         <v>0</v>
       </c>
       <c r="AI45" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ45">
         <v>0.036729519</v>
@@ -13389,7 +13392,7 @@
         <v>0</v>
       </c>
       <c r="CO45" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CP45">
         <v>-0.404237806</v>
@@ -13403,19 +13406,19 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E46" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F46" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G46">
         <v>0.001488019</v>
@@ -13499,7 +13502,7 @@
         <v>0</v>
       </c>
       <c r="AI46" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ46">
         <v>0.045071814</v>
@@ -13664,7 +13667,7 @@
         <v>0</v>
       </c>
       <c r="CO46" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CP46">
         <v>-0.703677808</v>
@@ -13678,19 +13681,19 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F47" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G47">
         <v>0.001436084</v>
@@ -13774,7 +13777,7 @@
         <v>0</v>
       </c>
       <c r="AI47" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ47">
         <v>0.0580535</v>
@@ -13939,7 +13942,7 @@
         <v>0</v>
       </c>
       <c r="CO47" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CP47">
         <v>-0.753715321</v>
@@ -13953,19 +13956,19 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E48" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F48" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G48">
         <v>0.001379037</v>
@@ -14049,7 +14052,7 @@
         <v>0</v>
       </c>
       <c r="AI48" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ48">
         <v>0.056639031</v>
@@ -14214,7 +14217,7 @@
         <v>0</v>
       </c>
       <c r="CO48" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CP48">
         <v>-0.71793867</v>
@@ -14228,19 +14231,19 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E49" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F49" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G49">
         <v>0.00225795</v>
@@ -14324,7 +14327,7 @@
         <v>0</v>
       </c>
       <c r="AI49" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ49">
         <v>0.074241638</v>
@@ -14489,7 +14492,7 @@
         <v>0</v>
       </c>
       <c r="CO49" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CP49">
         <v>-0.655169358</v>
@@ -14503,19 +14506,19 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E50" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F50" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G50">
         <v>0.002405425</v>
@@ -14599,7 +14602,7 @@
         <v>0</v>
       </c>
       <c r="AI50" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ50">
         <v>0.05430774</v>
@@ -14764,7 +14767,7 @@
         <v>0</v>
       </c>
       <c r="CO50" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="CP50">
         <v>-0.6872439380000001</v>
@@ -14778,19 +14781,19 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E51" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F51" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G51">
         <v>0.00267884</v>
@@ -14874,7 +14877,7 @@
         <v>0</v>
       </c>
       <c r="AI51" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ51">
         <v>0.080539377</v>
@@ -15039,7 +15042,7 @@
         <v>0</v>
       </c>
       <c r="CO51" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="CP51">
         <v>-0.596275172</v>
@@ -15053,19 +15056,19 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E52" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F52" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G52">
         <v>0.001221159</v>
@@ -15149,7 +15152,7 @@
         <v>0</v>
       </c>
       <c r="AI52" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ52">
         <v>0.032588051</v>
@@ -15314,7 +15317,7 @@
         <v>0</v>
       </c>
       <c r="CO52" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="CP52">
         <v>-0.808081961</v>
@@ -15328,19 +15331,19 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E53" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F53" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G53">
         <v>0.00093247</v>
@@ -15424,7 +15427,7 @@
         <v>0</v>
       </c>
       <c r="AI53" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ53">
         <v>0.026475554</v>
@@ -15589,7 +15592,7 @@
         <v>0</v>
       </c>
       <c r="CO53" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="CP53">
         <v>-0.77227813</v>
@@ -15603,19 +15606,19 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D54" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G54">
         <v>0.0008229381467956</v>
@@ -15699,7 +15702,7 @@
         <v>0</v>
       </c>
       <c r="AI54" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ54">
         <v>0.0245106310926154</v>
@@ -15864,7 +15867,7 @@
         <v>0</v>
       </c>
       <c r="CO54" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="CP54">
         <v>-0.8664117478627688</v>
@@ -15878,16 +15881,16 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C55" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F55" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G55">
         <v>0.0022239398231451</v>
@@ -15971,7 +15974,7 @@
         <v>0</v>
       </c>
       <c r="AI55" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ55">
         <v>0.0779439577559576</v>
@@ -16136,7 +16139,7 @@
         <v>0</v>
       </c>
       <c r="CO55" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="CP55">
         <v>-0.7108907987632488</v>
@@ -16150,13 +16153,13 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C56" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F56" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G56">
         <v>0.0018211096217568</v>
@@ -16240,7 +16243,7 @@
         <v>0</v>
       </c>
       <c r="AI56" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ56">
         <v>0.0402740604837066</v>
@@ -16405,7 +16408,7 @@
         <v>0</v>
       </c>
       <c r="CO56" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="CP56">
         <v>-0.7447372903525753</v>
@@ -16419,10 +16422,10 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F57" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G57">
         <v>0.0012556275124289</v>
@@ -16506,7 +16509,7 @@
         <v>0</v>
       </c>
       <c r="AI57" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ57">
         <v>0.0441363962743036</v>
@@ -16671,7 +16674,7 @@
         <v>0</v>
       </c>
       <c r="CO57" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="CP57">
         <v>-0.7777179486581601</v>
@@ -16685,10 +16688,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F58" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G58">
         <v>0.0019905125443684</v>
@@ -16772,7 +16775,7 @@
         <v>0</v>
       </c>
       <c r="AI58" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ58">
         <v>0.0589646348207879</v>
@@ -16937,7 +16940,7 @@
         <v>0</v>
       </c>
       <c r="CO58" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="CP58">
         <v>-0.7757098341832183</v>
@@ -16951,10 +16954,10 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F59" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G59">
         <v>0.0005221982670147</v>
@@ -17038,7 +17041,7 @@
         <v>0</v>
       </c>
       <c r="AI59" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ59">
         <v>0.0088498418945465</v>
@@ -17203,7 +17206,7 @@
         <v>0</v>
       </c>
       <c r="CO59" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="CP59">
         <v>-0.9614802262041642</v>
@@ -17217,10 +17220,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F60" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G60">
         <v>0.0018105477499388</v>
@@ -17304,7 +17307,7 @@
         <v>0</v>
       </c>
       <c r="AI60" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ60">
         <v>0.0438527807624406</v>
@@ -17469,7 +17472,7 @@
         <v>0</v>
       </c>
       <c r="CO60" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="CP60">
         <v>-0.6569921650581255</v>
@@ -17483,10 +17486,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G61">
         <v>0.0006776201968474</v>
@@ -17570,7 +17573,7 @@
         <v>0</v>
       </c>
       <c r="AI61" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ61">
         <v>0.0175722673111926</v>
@@ -17735,7 +17738,7 @@
         <v>0</v>
       </c>
       <c r="CO61" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="CP61">
         <v>-0.924044412704054</v>
@@ -17749,10 +17752,10 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F62" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G62">
         <v>0.0025014106780221</v>
@@ -17836,7 +17839,7 @@
         <v>0</v>
       </c>
       <c r="AI62" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ62">
         <v>0.0551224625318549</v>
@@ -18001,7 +18004,7 @@
         <v>0</v>
       </c>
       <c r="CO62" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="CP62">
         <v>-0.6213262971882773</v>
@@ -18015,10 +18018,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G63">
         <v>0.0007538484415952</v>
@@ -18102,7 +18105,7 @@
         <v>0</v>
       </c>
       <c r="AI63" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ63">
         <v>0.0157574961492794</v>
@@ -18267,7 +18270,7 @@
         <v>0</v>
       </c>
       <c r="CO63" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="CP63">
         <v>-0.9477002142299265</v>
@@ -18281,10 +18284,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F64" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G64">
         <v>0.0012416962587069</v>
@@ -18368,7 +18371,7 @@
         <v>0</v>
       </c>
       <c r="AI64" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ64">
         <v>0.0348775184726272</v>
@@ -18533,7 +18536,7 @@
         <v>0</v>
       </c>
       <c r="CO64" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="CP64">
         <v>-0.7774025388699596</v>
@@ -18547,10 +18550,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F65" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G65">
         <v>0.0015984483099258</v>
@@ -18634,7 +18637,7 @@
         <v>0</v>
       </c>
       <c r="AI65" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ65">
         <v>0.0617007650932976</v>
@@ -18799,7 +18802,7 @@
         <v>0</v>
       </c>
       <c r="CO65" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="CP65">
         <v>-0.8140402180385446</v>
@@ -18900,7 +18903,7 @@
         <v>0.01083306576401342</v>
       </c>
       <c r="AI66" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AJ66">
         <v>0.01228964656713829</v>
@@ -19078,6 +19081,278 @@
       </c>
       <c r="CQ66">
         <v>-0.4563890361669725</v>
+      </c>
+    </row>
+    <row r="67" spans="1:95">
+      <c r="A67" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F67" t="s">
+        <v>95</v>
+      </c>
+      <c r="G67">
+        <v>0.00056011030166081</v>
+      </c>
+      <c r="H67">
+        <v>0.000280055150830405</v>
+      </c>
+      <c r="I67">
+        <v>0.0005323724967918331</v>
+      </c>
+      <c r="J67">
+        <v>0.0005323724967918331</v>
+      </c>
+      <c r="K67">
+        <v>0.0005299767451950821</v>
+      </c>
+      <c r="L67">
+        <v>0.0002649883725975411</v>
+      </c>
+      <c r="M67">
+        <v>0.0005183792091088657</v>
+      </c>
+      <c r="N67">
+        <v>0.0005183792091088657</v>
+      </c>
+      <c r="O67">
+        <v>6.826955010619812</v>
+      </c>
+      <c r="P67">
+        <v>80.56752268777757</v>
+      </c>
+      <c r="Q67">
+        <v>0.1934702067902953</v>
+      </c>
+      <c r="R67">
+        <v>0.6913463586662338</v>
+      </c>
+      <c r="S67">
+        <v>0.04922616529601365</v>
+      </c>
+      <c r="T67">
+        <v>0.05632829461020863</v>
+      </c>
+      <c r="U67">
+        <v>0.2492126659834974</v>
+      </c>
+      <c r="V67">
+        <v>0.1681379894765381</v>
+      </c>
+      <c r="W67">
+        <v>0.9992532685397598</v>
+      </c>
+      <c r="X67">
+        <v>0.7713642102943742</v>
+      </c>
+      <c r="Y67">
+        <v>0.8629550739619983</v>
+      </c>
+      <c r="Z67">
+        <v>0.9990616425958897</v>
+      </c>
+      <c r="AA67">
+        <v>0.6906940270786949</v>
+      </c>
+      <c r="AB67">
+        <v>0.8319806730494639</v>
+      </c>
+      <c r="AC67">
+        <v>0.006939600861191607</v>
+      </c>
+      <c r="AD67">
+        <v>0.006330898137423144</v>
+      </c>
+      <c r="AE67">
+        <v>0.9992532685397598</v>
+      </c>
+      <c r="AF67">
+        <v>0.9990616425958897</v>
+      </c>
+      <c r="AG67">
+        <v>0.006939600861191607</v>
+      </c>
+      <c r="AH67">
+        <v>0.006330898137423144</v>
+      </c>
+      <c r="AI67" t="s">
+        <v>213</v>
+      </c>
+      <c r="AJ67">
+        <v>0.01145649975565328</v>
+      </c>
+      <c r="AK67">
+        <v>0.03972890520267203</v>
+      </c>
+      <c r="AL67">
+        <v>-334.1096595</v>
+      </c>
+      <c r="AM67">
+        <v>-1782.60515798</v>
+      </c>
+      <c r="AN67">
+        <v>18297.26484050013</v>
+      </c>
+      <c r="AO67">
+        <v>17758.06874202069</v>
+      </c>
+      <c r="AP67">
+        <v>18297.26484050013</v>
+      </c>
+      <c r="AQ67">
+        <v>17754.61674202069</v>
+      </c>
+      <c r="AR67">
+        <v>0.8297264840500127</v>
+      </c>
+      <c r="AS67">
+        <v>0.7758068742020692</v>
+      </c>
+      <c r="AT67">
+        <v>3.5124485177642</v>
+      </c>
+      <c r="AU67">
+        <v>0.2974221961470029</v>
+      </c>
+      <c r="AV67">
+        <v>116.2166666666667</v>
+      </c>
+      <c r="AW67">
+        <v>72.96666666666667</v>
+      </c>
+      <c r="AX67">
+        <v>0</v>
+      </c>
+      <c r="AY67">
+        <v>0.06771692854276455</v>
+      </c>
+      <c r="AZ67">
+        <v>0</v>
+      </c>
+      <c r="BA67">
+        <v>-692.9924531679723</v>
+      </c>
+      <c r="BB67">
+        <v>2388</v>
+      </c>
+      <c r="BC67">
+        <v>32498</v>
+      </c>
+      <c r="BD67">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BE67">
+        <v>4978</v>
+      </c>
+      <c r="BF67">
+        <v>54431</v>
+      </c>
+      <c r="BG67">
+        <v>7366</v>
+      </c>
+      <c r="BH67">
+        <v>86929</v>
+      </c>
+      <c r="BI67">
+        <v>2417</v>
+      </c>
+      <c r="BJ67">
+        <v>32466</v>
+      </c>
+      <c r="BK67">
+        <v>2388</v>
+      </c>
+      <c r="BL67">
+        <v>32478</v>
+      </c>
+      <c r="BM67">
+        <v>2561</v>
+      </c>
+      <c r="BN67">
+        <v>21965</v>
+      </c>
+      <c r="BO67">
+        <v>0</v>
+      </c>
+      <c r="BP67">
+        <v>20</v>
+      </c>
+      <c r="BQ67">
+        <v>0</v>
+      </c>
+      <c r="BR67">
+        <v>0</v>
+      </c>
+      <c r="BS67">
+        <v>8297.264840500002</v>
+      </c>
+      <c r="BT67">
+        <v>7758.068742020041</v>
+      </c>
+      <c r="BU67">
+        <v>0.06209707867837869</v>
+      </c>
+      <c r="BV67">
+        <v>0.05190579309141474</v>
+      </c>
+      <c r="BW67">
+        <v>0.1698648815502474</v>
+      </c>
+      <c r="BX67">
+        <v>0.1438424379430342</v>
+      </c>
+      <c r="BY67">
+        <v>0.01469946116115529</v>
+      </c>
+      <c r="BZ67">
+        <v>0.007914910662209703</v>
+      </c>
+      <c r="CA67">
+        <v>0.01320236875139543</v>
+      </c>
+      <c r="CB67">
+        <v>0.007020582081390735</v>
+      </c>
+      <c r="CC67">
+        <v>8631.374500000002</v>
+      </c>
+      <c r="CD67">
+        <v>9540.673900000042</v>
+      </c>
+      <c r="CE67">
+        <v>8631.374500000002</v>
+      </c>
+      <c r="CF67">
+        <v>10233.66635316801</v>
+      </c>
+      <c r="CG67">
+        <v>0.09526260076783863</v>
+      </c>
+      <c r="CH67">
+        <v>0.06455064908909733</v>
+      </c>
+      <c r="CI67">
+        <v>10000</v>
+      </c>
+      <c r="CK67">
+        <v>3.861600247142416E-05</v>
+      </c>
+      <c r="CL67">
+        <v>0.01058078467717022</v>
+      </c>
+      <c r="CM67">
+        <v>4452642.888408865</v>
+      </c>
+      <c r="CN67">
+        <v>20248746.97476565</v>
+      </c>
+      <c r="CO67" s="2">
+        <v>45400.44633041293</v>
+      </c>
+      <c r="CP67">
+        <v>-0.9266047568089176</v>
+      </c>
+      <c r="CQ67">
+        <v>-0.8084849743699738</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update WAVESUSDT.json at 2024-04-18_20-53-50 bestfile_scores 0.0005239110052792928 bestfile_sharp 0.14880821909343891
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -19091,190 +19091,190 @@
         <v>95</v>
       </c>
       <c r="G67">
-        <v>0.00056011030166081</v>
+        <v>0.001208944261057887</v>
       </c>
       <c r="H67">
-        <v>0.000280055150830405</v>
+        <v>0.0006044721305289436</v>
       </c>
       <c r="I67">
-        <v>0.0005323724967918331</v>
+        <v>0.001076431801899203</v>
       </c>
       <c r="J67">
-        <v>0.0005323724967918331</v>
+        <v>0.001076431801899203</v>
       </c>
       <c r="K67">
-        <v>0.0005299767451950821</v>
+        <v>0.001363571017074561</v>
       </c>
       <c r="L67">
-        <v>0.0002649883725975411</v>
+        <v>0.0006817855085372804</v>
       </c>
       <c r="M67">
-        <v>0.0005183792091088657</v>
+        <v>0.001016029730313916</v>
       </c>
       <c r="N67">
-        <v>0.0005183792091088657</v>
+        <v>0.001016029730313916</v>
       </c>
       <c r="O67">
-        <v>6.826955010619812</v>
+        <v>11.53519984553003</v>
       </c>
       <c r="P67">
-        <v>80.56752268777757</v>
+        <v>17.64386947287121</v>
       </c>
       <c r="Q67">
-        <v>0.1934702067902953</v>
+        <v>0.1921915300742149</v>
       </c>
       <c r="R67">
-        <v>0.6913463586662338</v>
+        <v>0.6315686411541986</v>
       </c>
       <c r="S67">
-        <v>0.04922616529601365</v>
+        <v>0.03340021876453157</v>
       </c>
       <c r="T67">
-        <v>0.05632829461020863</v>
+        <v>0.08997286145615917</v>
       </c>
       <c r="U67">
-        <v>0.2492126659834974</v>
+        <v>0.2481923527352983</v>
       </c>
       <c r="V67">
-        <v>0.1681379894765381</v>
+        <v>0.2290751915085273</v>
       </c>
       <c r="W67">
-        <v>0.9992532685397598</v>
+        <v>0.9993769932147427</v>
       </c>
       <c r="X67">
-        <v>0.7713642102943742</v>
+        <v>0.8574736912308205</v>
       </c>
       <c r="Y67">
-        <v>0.8629550739619983</v>
+        <v>0.823463484029076</v>
       </c>
       <c r="Z67">
-        <v>0.9990616425958897</v>
+        <v>0.99855022013794</v>
       </c>
       <c r="AA67">
-        <v>0.6906940270786949</v>
+        <v>0.7492246730842103</v>
       </c>
       <c r="AB67">
-        <v>0.8319806730494639</v>
+        <v>0.7791528923885436</v>
       </c>
       <c r="AC67">
-        <v>0.006939600861191607</v>
+        <v>0.004364776711903726</v>
       </c>
       <c r="AD67">
-        <v>0.006330898137423144</v>
+        <v>0.009662114019183791</v>
       </c>
       <c r="AE67">
-        <v>0.9992532685397598</v>
+        <v>0.9993769932147427</v>
       </c>
       <c r="AF67">
-        <v>0.9990616425958897</v>
+        <v>0.99855022013794</v>
       </c>
       <c r="AG67">
-        <v>0.006939600861191607</v>
+        <v>0.004364776711903726</v>
       </c>
       <c r="AH67">
-        <v>0.006330898137423144</v>
+        <v>0.009662114019183791</v>
       </c>
       <c r="AI67" t="s">
         <v>213</v>
       </c>
       <c r="AJ67">
-        <v>0.01145649975565328</v>
+        <v>0.01570755211730832</v>
       </c>
       <c r="AK67">
-        <v>0.03972890520267203</v>
+        <v>0.04655778477343839</v>
       </c>
       <c r="AL67">
-        <v>-334.1096595</v>
+        <v>-1446.64548588</v>
       </c>
       <c r="AM67">
-        <v>-1782.60515798</v>
+        <v>-1142.02995452</v>
       </c>
       <c r="AN67">
-        <v>18297.26484050013</v>
+        <v>36825.76511411995</v>
       </c>
       <c r="AO67">
-        <v>17758.06874202069</v>
+        <v>31924.87564548021</v>
       </c>
       <c r="AP67">
-        <v>18297.26484050013</v>
+        <v>36825.76511411995</v>
       </c>
       <c r="AQ67">
-        <v>17754.61674202069</v>
+        <v>31920.08064548021</v>
       </c>
       <c r="AR67">
-        <v>0.8297264840500127</v>
+        <v>2.682576511411995</v>
       </c>
       <c r="AS67">
-        <v>0.7758068742020692</v>
+        <v>2.192487564548021</v>
       </c>
       <c r="AT67">
-        <v>3.5124485177642</v>
+        <v>2.078761216017142</v>
       </c>
       <c r="AU67">
-        <v>0.2974221961470029</v>
+        <v>1.359766582615396</v>
       </c>
       <c r="AV67">
-        <v>116.2166666666667</v>
+        <v>88.76666666666667</v>
       </c>
       <c r="AW67">
         <v>72.96666666666667</v>
       </c>
       <c r="AX67">
-        <v>0</v>
+        <v>0.005782377739628801</v>
       </c>
       <c r="AY67">
-        <v>0.06771692854276455</v>
+        <v>0.03444884271750963</v>
       </c>
       <c r="AZ67">
-        <v>0</v>
+        <v>-164.4325689253092</v>
       </c>
       <c r="BA67">
-        <v>-692.9924531679723</v>
+        <v>-822.9788727409277</v>
       </c>
       <c r="BB67">
-        <v>2388</v>
+        <v>5173</v>
       </c>
       <c r="BC67">
-        <v>32498</v>
+        <v>5822</v>
       </c>
       <c r="BD67">
         <v>1078.958333333333</v>
       </c>
       <c r="BE67">
-        <v>4978</v>
+        <v>7273</v>
       </c>
       <c r="BF67">
-        <v>54431</v>
+        <v>13215</v>
       </c>
       <c r="BG67">
-        <v>7366</v>
+        <v>12446</v>
       </c>
       <c r="BH67">
-        <v>86929</v>
+        <v>19037</v>
       </c>
       <c r="BI67">
-        <v>2417</v>
+        <v>4995</v>
       </c>
       <c r="BJ67">
-        <v>32466</v>
+        <v>5520</v>
       </c>
       <c r="BK67">
-        <v>2388</v>
+        <v>5166</v>
       </c>
       <c r="BL67">
-        <v>32478</v>
+        <v>5735</v>
       </c>
       <c r="BM67">
-        <v>2561</v>
+        <v>2278</v>
       </c>
       <c r="BN67">
-        <v>21965</v>
+        <v>7695</v>
       </c>
       <c r="BO67">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="BP67">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="BQ67">
         <v>0</v>
@@ -19283,76 +19283,76 @@
         <v>0</v>
       </c>
       <c r="BS67">
-        <v>8297.264840500002</v>
+        <v>26825.76511412003</v>
       </c>
       <c r="BT67">
-        <v>7758.068742020041</v>
+        <v>21924.87564548</v>
       </c>
       <c r="BU67">
-        <v>0.06209707867837869</v>
+        <v>0.04634944445717447</v>
       </c>
       <c r="BV67">
-        <v>0.05190579309141474</v>
+        <v>0.07607454946414445</v>
       </c>
       <c r="BW67">
-        <v>0.1698648815502474</v>
+        <v>0.1432460464407948</v>
       </c>
       <c r="BX67">
-        <v>0.1438424379430342</v>
+        <v>0.1807909664363859</v>
       </c>
       <c r="BY67">
-        <v>0.01469946116115529</v>
+        <v>0.01080919951278491</v>
       </c>
       <c r="BZ67">
-        <v>0.007914910662209703</v>
+        <v>0.007841900883603476</v>
       </c>
       <c r="CA67">
-        <v>0.01320236875139543</v>
+        <v>0.009389131100047909</v>
       </c>
       <c r="CB67">
-        <v>0.007020582081390735</v>
+        <v>0.01070112247275361</v>
       </c>
       <c r="CC67">
-        <v>8631.374500000002</v>
+        <v>28272.41060000003</v>
       </c>
       <c r="CD67">
-        <v>9540.673900000042</v>
+        <v>23066.9056</v>
       </c>
       <c r="CE67">
-        <v>8631.374500000002</v>
+        <v>28436.84316892534</v>
       </c>
       <c r="CF67">
-        <v>10233.66635316801</v>
+        <v>23889.88447274093</v>
       </c>
       <c r="CG67">
-        <v>0.09526260076783863</v>
+        <v>0.1495843720035209</v>
       </c>
       <c r="CH67">
-        <v>0.06455064908909733</v>
+        <v>0.1057817975684645</v>
       </c>
       <c r="CI67">
         <v>10000</v>
       </c>
       <c r="CK67">
-        <v>3.861600247142416E-05</v>
+        <v>0.001158480074142725</v>
       </c>
       <c r="CL67">
-        <v>0.01058078467717022</v>
+        <v>0.02320821748532592</v>
       </c>
       <c r="CM67">
-        <v>4452642.888408865</v>
+        <v>8548919.458356148</v>
       </c>
       <c r="CN67">
-        <v>20248746.97476565</v>
+        <v>12816652.38654841</v>
       </c>
       <c r="CO67" s="2">
-        <v>45400.44633041293</v>
+        <v>45400.65101744193</v>
       </c>
       <c r="CP67">
-        <v>-0.9266047568089176</v>
+        <v>-0.843107865610227</v>
       </c>
       <c r="CQ67">
-        <v>-0.8084849743699738</v>
+        <v>-0.7145783115530381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update WAVESUSDT.json at 2024-04-19_00-55-17 bestfile_scores 0.0006206608637614436 bestfile_sharp 0.07658637489399542
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="278">
   <si>
     <t>Unnamed: 0.3</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>KSMUSDT</t>
+  </si>
+  <si>
+    <t>WAVESUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1206,7 +1209,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CQ67"/>
+  <dimension ref="A1:CQ68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:95">
@@ -1498,19 +1501,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G2">
         <v>0.0009987329999999999</v>
@@ -1594,7 +1597,7 @@
         <v>0</v>
       </c>
       <c r="AI2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ2">
         <v>0.049606857</v>
@@ -1759,7 +1762,7 @@
         <v>0</v>
       </c>
       <c r="CO2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:95">
@@ -1767,19 +1770,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G3">
         <v>0.001058605</v>
@@ -1863,7 +1866,7 @@
         <v>0</v>
       </c>
       <c r="AI3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ3">
         <v>0.04006526</v>
@@ -2028,7 +2031,7 @@
         <v>0</v>
       </c>
       <c r="CO3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:95">
@@ -2036,19 +2039,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G4">
         <v>0.000882894</v>
@@ -2132,7 +2135,7 @@
         <v>0</v>
       </c>
       <c r="AI4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ4">
         <v>0.092575794</v>
@@ -2297,7 +2300,7 @@
         <v>0</v>
       </c>
       <c r="CO4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" spans="1:95">
@@ -2305,19 +2308,19 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G5">
         <v>0.001186265</v>
@@ -2401,7 +2404,7 @@
         <v>0</v>
       </c>
       <c r="AI5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ5">
         <v>0.027448502</v>
@@ -2566,7 +2569,7 @@
         <v>0</v>
       </c>
       <c r="CO5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:95">
@@ -2574,19 +2577,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G6">
         <v>0.001076751</v>
@@ -2670,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="AI6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ6">
         <v>0.083929868</v>
@@ -2835,7 +2838,7 @@
         <v>0</v>
       </c>
       <c r="CO6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="7" spans="1:95">
@@ -2843,19 +2846,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G7">
         <v>-0.000540801</v>
@@ -2939,7 +2942,7 @@
         <v>0</v>
       </c>
       <c r="AI7" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ7">
         <v>0.145376251</v>
@@ -3104,7 +3107,7 @@
         <v>0</v>
       </c>
       <c r="CO7" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:95">
@@ -3112,19 +3115,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E8" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F8" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G8">
         <v>0.001278948</v>
@@ -3208,7 +3211,7 @@
         <v>0</v>
       </c>
       <c r="AI8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ8">
         <v>0.087987204</v>
@@ -3373,7 +3376,7 @@
         <v>0</v>
       </c>
       <c r="CO8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:95">
@@ -3381,19 +3384,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G9">
         <v>0.000266144</v>
@@ -3477,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="AI9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ9">
         <v>0.118237951</v>
@@ -3642,7 +3645,7 @@
         <v>0</v>
       </c>
       <c r="CO9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" spans="1:95">
@@ -3650,19 +3653,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E10" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G10">
         <v>0.001013204</v>
@@ -3746,7 +3749,7 @@
         <v>0</v>
       </c>
       <c r="AI10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ10">
         <v>0.08106915200000001</v>
@@ -3911,7 +3914,7 @@
         <v>0</v>
       </c>
       <c r="CO10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:95">
@@ -3919,19 +3922,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F11" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G11">
         <v>0.001228309</v>
@@ -4015,7 +4018,7 @@
         <v>0</v>
       </c>
       <c r="AI11" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ11">
         <v>0.027960571</v>
@@ -4180,7 +4183,7 @@
         <v>0</v>
       </c>
       <c r="CO11" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:95">
@@ -4188,19 +4191,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F12" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G12">
         <v>0.0009776030000000001</v>
@@ -4284,7 +4287,7 @@
         <v>0</v>
       </c>
       <c r="AI12" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ12">
         <v>0.032951036</v>
@@ -4449,7 +4452,7 @@
         <v>0</v>
       </c>
       <c r="CO12" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" spans="1:95">
@@ -4457,19 +4460,19 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E13" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G13">
         <v>-2.89E-05</v>
@@ -4553,7 +4556,7 @@
         <v>0</v>
       </c>
       <c r="AI13" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ13">
         <v>0.179185242</v>
@@ -4718,7 +4721,7 @@
         <v>0</v>
       </c>
       <c r="CO13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" spans="1:95">
@@ -4726,19 +4729,19 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G14">
         <v>0.000431045</v>
@@ -4822,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="AI14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ14">
         <v>0.143233482</v>
@@ -4987,7 +4990,7 @@
         <v>0</v>
       </c>
       <c r="CO14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="15" spans="1:95">
@@ -4995,19 +4998,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G15">
         <v>0.000327551</v>
@@ -5091,7 +5094,7 @@
         <v>0</v>
       </c>
       <c r="AI15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ15">
         <v>0.138115134</v>
@@ -5256,7 +5259,7 @@
         <v>0</v>
       </c>
       <c r="CO15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" spans="1:95">
@@ -5264,19 +5267,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E16" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G16">
         <v>0.001162093</v>
@@ -5360,7 +5363,7 @@
         <v>0</v>
       </c>
       <c r="AI16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ16">
         <v>0.09650975000000001</v>
@@ -5525,7 +5528,7 @@
         <v>0</v>
       </c>
       <c r="CO16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17" spans="1:93">
@@ -5533,19 +5536,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E17" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G17">
         <v>0.00141042</v>
@@ -5629,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="AI17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ17">
         <v>0.060693695</v>
@@ -5794,7 +5797,7 @@
         <v>0</v>
       </c>
       <c r="CO17" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="18" spans="1:93">
@@ -5802,19 +5805,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G18">
         <v>0.000897625</v>
@@ -5898,7 +5901,7 @@
         <v>0</v>
       </c>
       <c r="AI18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ18">
         <v>0.107514363</v>
@@ -6063,7 +6066,7 @@
         <v>0</v>
       </c>
       <c r="CO18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" spans="1:93">
@@ -6071,19 +6074,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F19" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G19">
         <v>0.000473511</v>
@@ -6167,7 +6170,7 @@
         <v>0</v>
       </c>
       <c r="AI19" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ19">
         <v>0.014898256</v>
@@ -6332,7 +6335,7 @@
         <v>0</v>
       </c>
       <c r="CO19" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="1:93">
@@ -6340,19 +6343,19 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E20" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F20" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G20">
         <v>0.00029592</v>
@@ -6436,7 +6439,7 @@
         <v>0</v>
       </c>
       <c r="AI20" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ20">
         <v>0.02858403</v>
@@ -6601,7 +6604,7 @@
         <v>0</v>
       </c>
       <c r="CO20" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="21" spans="1:93">
@@ -6609,19 +6612,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G21">
         <v>0.000354958</v>
@@ -6705,7 +6708,7 @@
         <v>0</v>
       </c>
       <c r="AI21" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ21">
         <v>0.082273481</v>
@@ -6870,7 +6873,7 @@
         <v>0</v>
       </c>
       <c r="CO21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:93">
@@ -6878,19 +6881,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F22" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G22">
         <v>0.000513154</v>
@@ -6974,7 +6977,7 @@
         <v>0</v>
       </c>
       <c r="AI22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ22">
         <v>0.012592558</v>
@@ -7139,7 +7142,7 @@
         <v>0</v>
       </c>
       <c r="CO22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" spans="1:93">
@@ -7147,19 +7150,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F23" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G23">
         <v>0.000263694</v>
@@ -7243,7 +7246,7 @@
         <v>0</v>
       </c>
       <c r="AI23" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ23">
         <v>0.00903967</v>
@@ -7408,7 +7411,7 @@
         <v>0</v>
       </c>
       <c r="CO23" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="24" spans="1:93">
@@ -7416,19 +7419,19 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F24" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G24">
         <v>0.00048524</v>
@@ -7512,7 +7515,7 @@
         <v>0</v>
       </c>
       <c r="AI24" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ24">
         <v>0.030046089</v>
@@ -7677,7 +7680,7 @@
         <v>0</v>
       </c>
       <c r="CO24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="25" spans="1:93">
@@ -7685,19 +7688,19 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E25" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F25" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G25">
         <v>0.000308954</v>
@@ -7781,7 +7784,7 @@
         <v>0</v>
       </c>
       <c r="AI25" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ25">
         <v>0.010607012</v>
@@ -7946,7 +7949,7 @@
         <v>0</v>
       </c>
       <c r="CO25" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:93">
@@ -7954,19 +7957,19 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E26" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F26" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G26">
         <v>0.001706564</v>
@@ -8050,7 +8053,7 @@
         <v>0</v>
       </c>
       <c r="AI26" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ26">
         <v>0.053096335</v>
@@ -8215,7 +8218,7 @@
         <v>0</v>
       </c>
       <c r="CO26" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="27" spans="1:93">
@@ -8223,19 +8226,19 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F27" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G27">
         <v>0.001293263</v>
@@ -8319,7 +8322,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ27">
         <v>0.092674047</v>
@@ -8484,7 +8487,7 @@
         <v>0</v>
       </c>
       <c r="CO27" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" spans="1:93">
@@ -8492,19 +8495,19 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F28" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G28">
         <v>0.001493963</v>
@@ -8588,7 +8591,7 @@
         <v>0</v>
       </c>
       <c r="AI28" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ28">
         <v>0.03099706</v>
@@ -8753,7 +8756,7 @@
         <v>0</v>
       </c>
       <c r="CO28" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" spans="1:93">
@@ -8761,19 +8764,19 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F29" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G29">
         <v>0.001124522</v>
@@ -8857,7 +8860,7 @@
         <v>0</v>
       </c>
       <c r="AI29" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ29">
         <v>0.069423731</v>
@@ -9022,7 +9025,7 @@
         <v>0</v>
       </c>
       <c r="CO29" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="30" spans="1:93">
@@ -9030,19 +9033,19 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E30" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F30" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G30">
         <v>0.001194286</v>
@@ -9126,7 +9129,7 @@
         <v>0</v>
       </c>
       <c r="AI30" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ30">
         <v>0.060424834</v>
@@ -9291,7 +9294,7 @@
         <v>0</v>
       </c>
       <c r="CO30" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="31" spans="1:93">
@@ -9299,19 +9302,19 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E31" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F31" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G31">
         <v>0.002038684</v>
@@ -9395,7 +9398,7 @@
         <v>0</v>
       </c>
       <c r="AI31" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ31">
         <v>0.056666776</v>
@@ -9560,7 +9563,7 @@
         <v>0</v>
       </c>
       <c r="CO31" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="32" spans="1:93">
@@ -9568,19 +9571,19 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E32" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F32" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G32">
         <v>0.003509328</v>
@@ -9664,7 +9667,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ32">
         <v>0.098888062</v>
@@ -9829,7 +9832,7 @@
         <v>0</v>
       </c>
       <c r="CO32" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="33" spans="1:95">
@@ -9837,19 +9840,19 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E33" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F33" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G33">
         <v>0.001020607</v>
@@ -9933,7 +9936,7 @@
         <v>0</v>
       </c>
       <c r="AI33" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ33">
         <v>0.035815903</v>
@@ -10098,7 +10101,7 @@
         <v>0</v>
       </c>
       <c r="CO33" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" spans="1:95">
@@ -10106,19 +10109,19 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E34" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F34" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G34">
         <v>0.001036188</v>
@@ -10202,7 +10205,7 @@
         <v>0</v>
       </c>
       <c r="AI34" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ34">
         <v>0.037311133</v>
@@ -10367,7 +10370,7 @@
         <v>0</v>
       </c>
       <c r="CO34" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="CP34">
         <v>-0.814742818</v>
@@ -10381,19 +10384,19 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E35" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F35" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G35">
         <v>0.001410503</v>
@@ -10477,7 +10480,7 @@
         <v>0</v>
       </c>
       <c r="AI35" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ35">
         <v>0.041330496</v>
@@ -10642,7 +10645,7 @@
         <v>0</v>
       </c>
       <c r="CO35" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CP35">
         <v>-0.753066891</v>
@@ -10656,19 +10659,19 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F36" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G36">
         <v>0.00072725</v>
@@ -10752,7 +10755,7 @@
         <v>0</v>
       </c>
       <c r="AI36" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ36">
         <v>0.047772102</v>
@@ -10917,7 +10920,7 @@
         <v>0</v>
       </c>
       <c r="CO36" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CP36">
         <v>-0.872335259</v>
@@ -10931,19 +10934,19 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G37">
         <v>0.001640077</v>
@@ -11027,7 +11030,7 @@
         <v>0</v>
       </c>
       <c r="AI37" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ37">
         <v>0.060484521</v>
@@ -11192,7 +11195,7 @@
         <v>0</v>
       </c>
       <c r="CO37" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CP37">
         <v>-0.759885442</v>
@@ -11206,19 +11209,19 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F38" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G38">
         <v>0.000951107</v>
@@ -11302,7 +11305,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ38">
         <v>0.061007062</v>
@@ -11467,7 +11470,7 @@
         <v>0</v>
       </c>
       <c r="CO38" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CP38">
         <v>-0.838900609</v>
@@ -11481,19 +11484,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E39" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F39" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G39">
         <v>0.001738925</v>
@@ -11577,7 +11580,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ39">
         <v>0.025236369</v>
@@ -11742,7 +11745,7 @@
         <v>0</v>
       </c>
       <c r="CO39" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CP39">
         <v>-0.780218664</v>
@@ -11756,19 +11759,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F40" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G40">
         <v>0.001263071</v>
@@ -11852,7 +11855,7 @@
         <v>0</v>
       </c>
       <c r="AI40" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ40">
         <v>0.031804424</v>
@@ -12017,7 +12020,7 @@
         <v>0</v>
       </c>
       <c r="CO40" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CP40">
         <v>-0.79992089</v>
@@ -12031,19 +12034,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E41" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F41" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G41">
         <v>0.002702281</v>
@@ -12127,7 +12130,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ41">
         <v>0.072404657</v>
@@ -12292,7 +12295,7 @@
         <v>0</v>
       </c>
       <c r="CO41" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CP41">
         <v>-0.528089775</v>
@@ -12306,19 +12309,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E42" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F42" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G42">
         <v>0.001559412</v>
@@ -12402,7 +12405,7 @@
         <v>0</v>
       </c>
       <c r="AI42" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ42">
         <v>0.06821192299999999</v>
@@ -12567,7 +12570,7 @@
         <v>0</v>
       </c>
       <c r="CO42" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CP42">
         <v>-0.754849911</v>
@@ -12581,19 +12584,19 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E43" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F43" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G43">
         <v>0.001270244</v>
@@ -12677,7 +12680,7 @@
         <v>0</v>
       </c>
       <c r="AI43" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ43">
         <v>0.069326524</v>
@@ -12842,7 +12845,7 @@
         <v>0</v>
       </c>
       <c r="CO43" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CP43">
         <v>-0.7655395739999999</v>
@@ -12856,19 +12859,19 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E44" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F44" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G44">
         <v>0.0009943969999999999</v>
@@ -12952,7 +12955,7 @@
         <v>0</v>
       </c>
       <c r="AI44" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ44">
         <v>0.036991009</v>
@@ -13117,7 +13120,7 @@
         <v>0</v>
       </c>
       <c r="CO44" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CP44">
         <v>-0.829764531</v>
@@ -13131,19 +13134,19 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E45" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F45" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G45">
         <v>0.002384052</v>
@@ -13227,7 +13230,7 @@
         <v>0</v>
       </c>
       <c r="AI45" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ45">
         <v>0.036729519</v>
@@ -13392,7 +13395,7 @@
         <v>0</v>
       </c>
       <c r="CO45" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CP45">
         <v>-0.404237806</v>
@@ -13406,19 +13409,19 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E46" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F46" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G46">
         <v>0.001488019</v>
@@ -13502,7 +13505,7 @@
         <v>0</v>
       </c>
       <c r="AI46" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ46">
         <v>0.045071814</v>
@@ -13667,7 +13670,7 @@
         <v>0</v>
       </c>
       <c r="CO46" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CP46">
         <v>-0.703677808</v>
@@ -13681,19 +13684,19 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F47" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G47">
         <v>0.001436084</v>
@@ -13777,7 +13780,7 @@
         <v>0</v>
       </c>
       <c r="AI47" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ47">
         <v>0.0580535</v>
@@ -13942,7 +13945,7 @@
         <v>0</v>
       </c>
       <c r="CO47" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CP47">
         <v>-0.753715321</v>
@@ -13956,19 +13959,19 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E48" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F48" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G48">
         <v>0.001379037</v>
@@ -14052,7 +14055,7 @@
         <v>0</v>
       </c>
       <c r="AI48" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ48">
         <v>0.056639031</v>
@@ -14217,7 +14220,7 @@
         <v>0</v>
       </c>
       <c r="CO48" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CP48">
         <v>-0.71793867</v>
@@ -14231,19 +14234,19 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E49" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F49" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G49">
         <v>0.00225795</v>
@@ -14327,7 +14330,7 @@
         <v>0</v>
       </c>
       <c r="AI49" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ49">
         <v>0.074241638</v>
@@ -14492,7 +14495,7 @@
         <v>0</v>
       </c>
       <c r="CO49" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="CP49">
         <v>-0.655169358</v>
@@ -14506,19 +14509,19 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E50" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F50" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G50">
         <v>0.002405425</v>
@@ -14602,7 +14605,7 @@
         <v>0</v>
       </c>
       <c r="AI50" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ50">
         <v>0.05430774</v>
@@ -14767,7 +14770,7 @@
         <v>0</v>
       </c>
       <c r="CO50" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="CP50">
         <v>-0.6872439380000001</v>
@@ -14781,19 +14784,19 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F51" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G51">
         <v>0.00267884</v>
@@ -14877,7 +14880,7 @@
         <v>0</v>
       </c>
       <c r="AI51" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ51">
         <v>0.080539377</v>
@@ -15042,7 +15045,7 @@
         <v>0</v>
       </c>
       <c r="CO51" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="CP51">
         <v>-0.596275172</v>
@@ -15056,19 +15059,19 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E52" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F52" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G52">
         <v>0.001221159</v>
@@ -15152,7 +15155,7 @@
         <v>0</v>
       </c>
       <c r="AI52" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ52">
         <v>0.032588051</v>
@@ -15317,7 +15320,7 @@
         <v>0</v>
       </c>
       <c r="CO52" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="CP52">
         <v>-0.808081961</v>
@@ -15331,19 +15334,19 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F53" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G53">
         <v>0.00093247</v>
@@ -15427,7 +15430,7 @@
         <v>0</v>
       </c>
       <c r="AI53" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ53">
         <v>0.026475554</v>
@@ -15592,7 +15595,7 @@
         <v>0</v>
       </c>
       <c r="CO53" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="CP53">
         <v>-0.77227813</v>
@@ -15606,19 +15609,19 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E54" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F54" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G54">
         <v>0.0008229381467956</v>
@@ -15702,7 +15705,7 @@
         <v>0</v>
       </c>
       <c r="AI54" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ54">
         <v>0.0245106310926154</v>
@@ -15867,7 +15870,7 @@
         <v>0</v>
       </c>
       <c r="CO54" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="CP54">
         <v>-0.8664117478627688</v>
@@ -15881,16 +15884,16 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C55" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F55" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G55">
         <v>0.0022239398231451</v>
@@ -15974,7 +15977,7 @@
         <v>0</v>
       </c>
       <c r="AI55" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ55">
         <v>0.0779439577559576</v>
@@ -16139,7 +16142,7 @@
         <v>0</v>
       </c>
       <c r="CO55" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="CP55">
         <v>-0.7108907987632488</v>
@@ -16153,13 +16156,13 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F56" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G56">
         <v>0.0018211096217568</v>
@@ -16243,7 +16246,7 @@
         <v>0</v>
       </c>
       <c r="AI56" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ56">
         <v>0.0402740604837066</v>
@@ -16408,7 +16411,7 @@
         <v>0</v>
       </c>
       <c r="CO56" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="CP56">
         <v>-0.7447372903525753</v>
@@ -16422,10 +16425,10 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F57" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G57">
         <v>0.0012556275124289</v>
@@ -16509,7 +16512,7 @@
         <v>0</v>
       </c>
       <c r="AI57" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ57">
         <v>0.0441363962743036</v>
@@ -16674,7 +16677,7 @@
         <v>0</v>
       </c>
       <c r="CO57" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="CP57">
         <v>-0.7777179486581601</v>
@@ -16688,10 +16691,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F58" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G58">
         <v>0.0019905125443684</v>
@@ -16775,7 +16778,7 @@
         <v>0</v>
       </c>
       <c r="AI58" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ58">
         <v>0.0589646348207879</v>
@@ -16940,7 +16943,7 @@
         <v>0</v>
       </c>
       <c r="CO58" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="CP58">
         <v>-0.7757098341832183</v>
@@ -16954,10 +16957,10 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F59" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G59">
         <v>0.0005221982670147</v>
@@ -17041,7 +17044,7 @@
         <v>0</v>
       </c>
       <c r="AI59" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ59">
         <v>0.0088498418945465</v>
@@ -17206,7 +17209,7 @@
         <v>0</v>
       </c>
       <c r="CO59" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="CP59">
         <v>-0.9614802262041642</v>
@@ -17220,10 +17223,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F60" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G60">
         <v>0.0018105477499388</v>
@@ -17307,7 +17310,7 @@
         <v>0</v>
       </c>
       <c r="AI60" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ60">
         <v>0.0438527807624406</v>
@@ -17472,7 +17475,7 @@
         <v>0</v>
       </c>
       <c r="CO60" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="CP60">
         <v>-0.6569921650581255</v>
@@ -17486,10 +17489,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F61" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G61">
         <v>0.0006776201968474</v>
@@ -17573,7 +17576,7 @@
         <v>0</v>
       </c>
       <c r="AI61" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ61">
         <v>0.0175722673111926</v>
@@ -17738,7 +17741,7 @@
         <v>0</v>
       </c>
       <c r="CO61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="CP61">
         <v>-0.924044412704054</v>
@@ -17752,10 +17755,10 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F62" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G62">
         <v>0.0025014106780221</v>
@@ -17839,7 +17842,7 @@
         <v>0</v>
       </c>
       <c r="AI62" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ62">
         <v>0.0551224625318549</v>
@@ -18004,7 +18007,7 @@
         <v>0</v>
       </c>
       <c r="CO62" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="CP62">
         <v>-0.6213262971882773</v>
@@ -18018,10 +18021,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F63" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G63">
         <v>0.0007538484415952</v>
@@ -18105,7 +18108,7 @@
         <v>0</v>
       </c>
       <c r="AI63" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ63">
         <v>0.0157574961492794</v>
@@ -18270,7 +18273,7 @@
         <v>0</v>
       </c>
       <c r="CO63" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="CP63">
         <v>-0.9477002142299265</v>
@@ -18284,10 +18287,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F64" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G64">
         <v>0.0012416962587069</v>
@@ -18371,7 +18374,7 @@
         <v>0</v>
       </c>
       <c r="AI64" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ64">
         <v>0.0348775184726272</v>
@@ -18536,7 +18539,7 @@
         <v>0</v>
       </c>
       <c r="CO64" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="CP64">
         <v>-0.7774025388699596</v>
@@ -18550,10 +18553,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F65" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G65">
         <v>0.0015984483099258</v>
@@ -18637,7 +18640,7 @@
         <v>0</v>
       </c>
       <c r="AI65" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ65">
         <v>0.0617007650932976</v>
@@ -18802,7 +18805,7 @@
         <v>0</v>
       </c>
       <c r="CO65" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="CP65">
         <v>-0.8140402180385446</v>
@@ -18903,7 +18906,7 @@
         <v>0.01083306576401342</v>
       </c>
       <c r="AI66" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ66">
         <v>0.01228964656713829</v>
@@ -19175,7 +19178,7 @@
         <v>0.009662114019183791</v>
       </c>
       <c r="AI67" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="AJ67">
         <v>0.01570755211730832</v>
@@ -19353,6 +19356,278 @@
       </c>
       <c r="CQ67">
         <v>-0.7145783115530381</v>
+      </c>
+    </row>
+    <row r="68" spans="1:95">
+      <c r="A68" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F68" t="s">
+        <v>96</v>
+      </c>
+      <c r="G68">
+        <v>0.002061850314947877</v>
+      </c>
+      <c r="H68">
+        <v>0.001030925157473939</v>
+      </c>
+      <c r="I68">
+        <v>7.107723924004716E-05</v>
+      </c>
+      <c r="J68">
+        <v>7.107723924004716E-05</v>
+      </c>
+      <c r="K68">
+        <v>0.001858655949149446</v>
+      </c>
+      <c r="L68">
+        <v>0.000929327974574723</v>
+      </c>
+      <c r="M68">
+        <v>6.431364982846244E-05</v>
+      </c>
+      <c r="N68">
+        <v>6.431364982846244E-05</v>
+      </c>
+      <c r="O68">
+        <v>27.47976387977931</v>
+      </c>
+      <c r="P68">
+        <v>9.967977159612641</v>
+      </c>
+      <c r="Q68">
+        <v>0.3118846619681307</v>
+      </c>
+      <c r="R68">
+        <v>0.6549017130688074</v>
+      </c>
+      <c r="S68">
+        <v>0.05563539154102014</v>
+      </c>
+      <c r="T68">
+        <v>0.03720610615413493</v>
+      </c>
+      <c r="U68">
+        <v>0.228288217183206</v>
+      </c>
+      <c r="V68">
+        <v>0.1472777633712802</v>
+      </c>
+      <c r="W68">
+        <v>0.9990802021173822</v>
+      </c>
+      <c r="X68">
+        <v>0.8489305139893405</v>
+      </c>
+      <c r="Y68">
+        <v>0.8823861606045551</v>
+      </c>
+      <c r="Z68">
+        <v>0.9995669677422319</v>
+      </c>
+      <c r="AA68">
+        <v>0.7696643364670031</v>
+      </c>
+      <c r="AB68">
+        <v>0.8412757804485351</v>
+      </c>
+      <c r="AC68">
+        <v>0.006599833996922164</v>
+      </c>
+      <c r="AD68">
+        <v>0.0042384051582964</v>
+      </c>
+      <c r="AE68">
+        <v>0.9990802021173822</v>
+      </c>
+      <c r="AF68">
+        <v>0.9995669677422319</v>
+      </c>
+      <c r="AG68">
+        <v>0.006599833996922164</v>
+      </c>
+      <c r="AH68">
+        <v>0.0042384051582964</v>
+      </c>
+      <c r="AI68" t="s">
+        <v>214</v>
+      </c>
+      <c r="AJ68">
+        <v>0.02239499395527291</v>
+      </c>
+      <c r="AK68">
+        <v>0.005853361308655457</v>
+      </c>
+      <c r="AL68">
+        <v>-6759.284227964001</v>
+      </c>
+      <c r="AM68">
+        <v>-132.198697914</v>
+      </c>
+      <c r="AN68">
+        <v>92481.17399203611</v>
+      </c>
+      <c r="AO68">
+        <v>10797.80445208634</v>
+      </c>
+      <c r="AP68">
+        <v>92460.19837203612</v>
+      </c>
+      <c r="AQ68">
+        <v>10796.26557208634</v>
+      </c>
+      <c r="AR68">
+        <v>8.248117399203611</v>
+      </c>
+      <c r="AS68">
+        <v>0.07978044520863414</v>
+      </c>
+      <c r="AT68">
+        <v>0.8720879947881565</v>
+      </c>
+      <c r="AU68">
+        <v>2.404584726867335</v>
+      </c>
+      <c r="AV68">
+        <v>90.33333333333333</v>
+      </c>
+      <c r="AW68">
+        <v>149.2166666666667</v>
+      </c>
+      <c r="AX68">
+        <v>0.001647948110206856</v>
+      </c>
+      <c r="AY68">
+        <v>0.1351813016870194</v>
+      </c>
+      <c r="AZ68">
+        <v>-147.3063977774817</v>
+      </c>
+      <c r="BA68">
+        <v>-145.3703957086861</v>
+      </c>
+      <c r="BB68">
+        <v>13761</v>
+      </c>
+      <c r="BC68">
+        <v>5150</v>
+      </c>
+      <c r="BD68">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BE68">
+        <v>15916</v>
+      </c>
+      <c r="BF68">
+        <v>5615</v>
+      </c>
+      <c r="BG68">
+        <v>29677</v>
+      </c>
+      <c r="BH68">
+        <v>10765</v>
+      </c>
+      <c r="BI68">
+        <v>13381</v>
+      </c>
+      <c r="BJ68">
+        <v>5139</v>
+      </c>
+      <c r="BK68">
+        <v>13759</v>
+      </c>
+      <c r="BL68">
+        <v>5146</v>
+      </c>
+      <c r="BM68">
+        <v>2535</v>
+      </c>
+      <c r="BN68">
+        <v>476</v>
+      </c>
+      <c r="BO68">
+        <v>2</v>
+      </c>
+      <c r="BP68">
+        <v>4</v>
+      </c>
+      <c r="BQ68">
+        <v>0</v>
+      </c>
+      <c r="BR68">
+        <v>0</v>
+      </c>
+      <c r="BS68">
+        <v>82481.17399203603</v>
+      </c>
+      <c r="BT68">
+        <v>797.8044520860029</v>
+      </c>
+      <c r="BU68">
+        <v>0.04290348885869012</v>
+      </c>
+      <c r="BV68">
+        <v>0.1202504257169967</v>
+      </c>
+      <c r="BW68">
+        <v>0.1301127205652294</v>
+      </c>
+      <c r="BX68">
+        <v>0.3002543371297677</v>
+      </c>
+      <c r="BY68">
+        <v>0.01256117148226153</v>
+      </c>
+      <c r="BZ68">
+        <v>0.02331681240673363</v>
+      </c>
+      <c r="CA68">
+        <v>0.009269061591935608</v>
+      </c>
+      <c r="CB68">
+        <v>0.02354928426964311</v>
+      </c>
+      <c r="CC68">
+        <v>89240.45822000003</v>
+      </c>
+      <c r="CD68">
+        <v>930.003150000003</v>
+      </c>
+      <c r="CE68">
+        <v>89387.76461777752</v>
+      </c>
+      <c r="CF68">
+        <v>1075.373545708689</v>
+      </c>
+      <c r="CG68">
+        <v>0.1488082190934389</v>
+      </c>
+      <c r="CH68">
+        <v>0.0245119584945619</v>
+      </c>
+      <c r="CI68">
+        <v>10000</v>
+      </c>
+      <c r="CK68">
+        <v>0.007908950617283951</v>
+      </c>
+      <c r="CL68">
+        <v>0.0005401234567901234</v>
+      </c>
+      <c r="CM68">
+        <v>32434223.01659032</v>
+      </c>
+      <c r="CN68">
+        <v>472313.986333131</v>
+      </c>
+      <c r="CO68" s="2">
+        <v>45400.87074471051</v>
+      </c>
+      <c r="CP68">
+        <v>-0.773596014638592</v>
+      </c>
+      <c r="CQ68">
+        <v>-0.9674897044232793</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SNXUSDT.json at 2024-04-19_06-04-32 bestfile_scores 0.0005580163220426926 bestfile_sharp 0.15066585191293586
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -19366,191 +19366,191 @@
         <v>96</v>
       </c>
       <c r="G68">
-        <v>0.002061850314947877</v>
+        <v>0.002384997880270134</v>
       </c>
       <c r="H68">
-        <v>0.001030925157473939</v>
+        <v>0.001192498940135067</v>
       </c>
       <c r="I68">
-        <v>7.107723924004716E-05</v>
+        <v>0.0001369232758667849</v>
       </c>
       <c r="J68">
-        <v>7.107723924004716E-05</v>
+        <v>0.0001369232758667849</v>
       </c>
       <c r="K68">
-        <v>0.001858655949149446</v>
+        <v>0.002084353096736957</v>
       </c>
       <c r="L68">
-        <v>0.000929327974574723</v>
+        <v>0.001042176548368479</v>
       </c>
       <c r="M68">
-        <v>6.431364982846244E-05</v>
+        <v>0.0001110446906754437</v>
       </c>
       <c r="N68">
-        <v>6.431364982846244E-05</v>
+        <v>0.0001110446906754437</v>
       </c>
       <c r="O68">
-        <v>27.47976387977931</v>
+        <v>15.31262780199853</v>
       </c>
       <c r="P68">
-        <v>9.967977159612641</v>
+        <v>4.285350515066168</v>
       </c>
       <c r="Q68">
-        <v>0.3118846619681307</v>
+        <v>0.3921937840912242</v>
       </c>
       <c r="R68">
-        <v>0.6549017130688074</v>
+        <v>0.6814421672614276</v>
       </c>
       <c r="S68">
-        <v>0.05563539154102014</v>
+        <v>0.06030421445049951</v>
       </c>
       <c r="T68">
-        <v>0.03720610615413493</v>
+        <v>0.08934913887221584</v>
       </c>
       <c r="U68">
-        <v>0.228288217183206</v>
+        <v>0.1810605090122995</v>
       </c>
       <c r="V68">
-        <v>0.1472777633712802</v>
+        <v>0.2049664233577391</v>
       </c>
       <c r="W68">
-        <v>0.9990802021173822</v>
+        <v>0.9992070102014501</v>
       </c>
       <c r="X68">
-        <v>0.8489305139893405</v>
+        <v>0.8409978808730804</v>
       </c>
       <c r="Y68">
-        <v>0.8823861606045551</v>
+        <v>0.8251755172559925</v>
       </c>
       <c r="Z68">
-        <v>0.9995669677422319</v>
+        <v>0.9987725466043624</v>
       </c>
       <c r="AA68">
-        <v>0.7696643364670031</v>
+        <v>0.8192838730879928</v>
       </c>
       <c r="AB68">
-        <v>0.8412757804485351</v>
+        <v>0.8040986864817953</v>
       </c>
       <c r="AC68">
-        <v>0.006599833996922164</v>
+        <v>0.006951764164820487</v>
       </c>
       <c r="AD68">
-        <v>0.0042384051582964</v>
+        <v>0.009682496602030617</v>
       </c>
       <c r="AE68">
-        <v>0.9990802021173822</v>
+        <v>0.9992070102014501</v>
       </c>
       <c r="AF68">
-        <v>0.9995669677422319</v>
+        <v>0.9987725466043624</v>
       </c>
       <c r="AG68">
-        <v>0.006599833996922164</v>
+        <v>0.006951764164820487</v>
       </c>
       <c r="AH68">
-        <v>0.0042384051582964</v>
+        <v>0.009682496602030617</v>
       </c>
       <c r="AI68" t="s">
         <v>214</v>
       </c>
       <c r="AJ68">
-        <v>0.02239499395527291</v>
+        <v>0.01945380747640302</v>
       </c>
       <c r="AK68">
-        <v>0.005853361308655457</v>
+        <v>0.01123642261824176</v>
       </c>
       <c r="AL68">
-        <v>-6759.284227964001</v>
+        <v>-7075.875342406</v>
       </c>
       <c r="AM68">
-        <v>-132.198697914</v>
+        <v>-85.11522094200001</v>
       </c>
       <c r="AN68">
-        <v>92481.17399203611</v>
+        <v>131002.5496813422</v>
       </c>
       <c r="AO68">
-        <v>10797.80445208634</v>
+        <v>11593.52094905808</v>
       </c>
       <c r="AP68">
-        <v>92460.19837203612</v>
+        <v>131003.4904913422</v>
       </c>
       <c r="AQ68">
-        <v>10796.26557208634</v>
+        <v>11592.08020905808</v>
       </c>
       <c r="AR68">
-        <v>8.248117399203611</v>
+        <v>12.10025496813422</v>
       </c>
       <c r="AS68">
-        <v>0.07978044520863414</v>
+        <v>0.1593520949058076</v>
       </c>
       <c r="AT68">
-        <v>0.8720879947881565</v>
+        <v>1.567110143525238</v>
       </c>
       <c r="AU68">
-        <v>2.404584726867335</v>
+        <v>5.59649520927887</v>
       </c>
       <c r="AV68">
-        <v>90.33333333333333</v>
+        <v>103.05</v>
       </c>
       <c r="AW68">
-        <v>149.2166666666667</v>
+        <v>117.5166666666667</v>
       </c>
       <c r="AX68">
-        <v>0.001647948110206856</v>
+        <v>0.006801762965061194</v>
       </c>
       <c r="AY68">
-        <v>0.1351813016870194</v>
+        <v>0.08550935360130708</v>
       </c>
       <c r="AZ68">
-        <v>-147.3063977774817</v>
+        <v>-877.1949729437605</v>
       </c>
       <c r="BA68">
-        <v>-145.3703957086861</v>
+        <v>-156.9607019970486</v>
       </c>
       <c r="BB68">
-        <v>13761</v>
+        <v>7204</v>
       </c>
       <c r="BC68">
-        <v>5150</v>
+        <v>2079</v>
       </c>
       <c r="BD68">
         <v>1079.958333333333</v>
       </c>
       <c r="BE68">
-        <v>15916</v>
+        <v>9333</v>
       </c>
       <c r="BF68">
-        <v>5615</v>
+        <v>2549</v>
       </c>
       <c r="BG68">
-        <v>29677</v>
+        <v>16537</v>
       </c>
       <c r="BH68">
-        <v>10765</v>
+        <v>4628</v>
       </c>
       <c r="BI68">
-        <v>13381</v>
+        <v>6913</v>
       </c>
       <c r="BJ68">
-        <v>5139</v>
+        <v>2069</v>
       </c>
       <c r="BK68">
-        <v>13759</v>
+        <v>7176</v>
       </c>
       <c r="BL68">
-        <v>5146</v>
+        <v>2077</v>
       </c>
       <c r="BM68">
-        <v>2535</v>
+        <v>2420</v>
       </c>
       <c r="BN68">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="BO68">
+        <v>28</v>
+      </c>
+      <c r="BP68">
         <v>2</v>
       </c>
-      <c r="BP68">
-        <v>4</v>
-      </c>
       <c r="BQ68">
         <v>0</v>
       </c>
@@ -19558,76 +19558,76 @@
         <v>0</v>
       </c>
       <c r="BS68">
-        <v>82481.17399203603</v>
+        <v>121012.7547875938</v>
       </c>
       <c r="BT68">
-        <v>797.8044520860029</v>
+        <v>1593.520949057997</v>
       </c>
       <c r="BU68">
-        <v>0.04290348885869012</v>
+        <v>0.03949514773523077</v>
       </c>
       <c r="BV68">
-        <v>0.1202504257169967</v>
+        <v>0.1951523328490107</v>
       </c>
       <c r="BW68">
-        <v>0.1301127205652294</v>
+        <v>0.09930444694169656</v>
       </c>
       <c r="BX68">
-        <v>0.3002543371297677</v>
+        <v>0.3544594630018181</v>
       </c>
       <c r="BY68">
-        <v>0.01256117148226153</v>
+        <v>0.009892178926767569</v>
       </c>
       <c r="BZ68">
-        <v>0.02331681240673363</v>
+        <v>0.0253863983548441</v>
       </c>
       <c r="CA68">
-        <v>0.009269061591935608</v>
+        <v>0.008418919720083295</v>
       </c>
       <c r="CB68">
-        <v>0.02354928426964311</v>
+        <v>0.03322396890846473</v>
       </c>
       <c r="CC68">
-        <v>89240.45822000003</v>
+        <v>128088.6301299998</v>
       </c>
       <c r="CD68">
-        <v>930.003150000003</v>
+        <v>1678.636169999997</v>
       </c>
       <c r="CE68">
-        <v>89387.76461777752</v>
+        <v>128965.8251029435</v>
       </c>
       <c r="CF68">
-        <v>1075.373545708689</v>
+        <v>1835.596871997046</v>
       </c>
       <c r="CG68">
-        <v>0.1488082190934389</v>
+        <v>0.07658637489399542</v>
       </c>
       <c r="CH68">
-        <v>0.0245119584945619</v>
+        <v>0.02477651048744884</v>
       </c>
       <c r="CI68">
         <v>10000</v>
       </c>
       <c r="CK68">
-        <v>0.007908950617283951</v>
+        <v>0.008796296296296297</v>
       </c>
       <c r="CL68">
-        <v>0.0005401234567901234</v>
+        <v>0.001003086419753086</v>
       </c>
       <c r="CM68">
-        <v>32434223.01659032</v>
+        <v>43578601.99423853</v>
       </c>
       <c r="CN68">
-        <v>472313.986333131</v>
+        <v>362119.31393403</v>
       </c>
       <c r="CO68" s="2">
-        <v>45400.87074471051</v>
+        <v>45401.03841700275</v>
       </c>
       <c r="CP68">
-        <v>-0.773596014638592</v>
+        <v>-0.7040504011377985</v>
       </c>
       <c r="CQ68">
-        <v>-0.9674897044232793</v>
+        <v>-0.889563108338023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SNXUSDT.json at 2024-04-19_10-47-22 bestfile_scores 0.0008198038258348695 bestfile_sharp 0.15963030037681575
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="279">
   <si>
     <t>Unnamed: 0.3</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>WAVESUSDT</t>
+  </si>
+  <si>
+    <t>SNXUSDT</t>
   </si>
   <si>
     <t>0</t>
@@ -1209,7 +1212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CQ68"/>
+  <dimension ref="A1:CQ69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:95">
@@ -1501,19 +1504,19 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G2">
         <v>0.0009987329999999999</v>
@@ -1597,7 +1600,7 @@
         <v>0</v>
       </c>
       <c r="AI2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ2">
         <v>0.049606857</v>
@@ -1762,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="CO2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" spans="1:95">
@@ -1770,19 +1773,19 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G3">
         <v>0.001058605</v>
@@ -1866,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="AI3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ3">
         <v>0.04006526</v>
@@ -2031,7 +2034,7 @@
         <v>0</v>
       </c>
       <c r="CO3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:95">
@@ -2039,19 +2042,19 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G4">
         <v>0.000882894</v>
@@ -2135,7 +2138,7 @@
         <v>0</v>
       </c>
       <c r="AI4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ4">
         <v>0.092575794</v>
@@ -2300,7 +2303,7 @@
         <v>0</v>
       </c>
       <c r="CO4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="5" spans="1:95">
@@ -2308,19 +2311,19 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G5">
         <v>0.001186265</v>
@@ -2404,7 +2407,7 @@
         <v>0</v>
       </c>
       <c r="AI5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ5">
         <v>0.027448502</v>
@@ -2569,7 +2572,7 @@
         <v>0</v>
       </c>
       <c r="CO5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:95">
@@ -2577,19 +2580,19 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G6">
         <v>0.001076751</v>
@@ -2673,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="AI6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ6">
         <v>0.083929868</v>
@@ -2838,7 +2841,7 @@
         <v>0</v>
       </c>
       <c r="CO6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:95">
@@ -2846,19 +2849,19 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="G7">
         <v>-0.000540801</v>
@@ -2942,7 +2945,7 @@
         <v>0</v>
       </c>
       <c r="AI7" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ7">
         <v>0.145376251</v>
@@ -3107,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="CO7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" spans="1:95">
@@ -3115,19 +3118,19 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F8" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G8">
         <v>0.001278948</v>
@@ -3211,7 +3214,7 @@
         <v>0</v>
       </c>
       <c r="AI8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ8">
         <v>0.087987204</v>
@@ -3376,7 +3379,7 @@
         <v>0</v>
       </c>
       <c r="CO8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:95">
@@ -3384,19 +3387,19 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G9">
         <v>0.000266144</v>
@@ -3480,7 +3483,7 @@
         <v>0</v>
       </c>
       <c r="AI9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ9">
         <v>0.118237951</v>
@@ -3645,7 +3648,7 @@
         <v>0</v>
       </c>
       <c r="CO9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:95">
@@ -3653,19 +3656,19 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G10">
         <v>0.001013204</v>
@@ -3749,7 +3752,7 @@
         <v>0</v>
       </c>
       <c r="AI10" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ10">
         <v>0.08106915200000001</v>
@@ -3914,7 +3917,7 @@
         <v>0</v>
       </c>
       <c r="CO10" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" spans="1:95">
@@ -3922,19 +3925,19 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F11" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="G11">
         <v>0.001228309</v>
@@ -4018,7 +4021,7 @@
         <v>0</v>
       </c>
       <c r="AI11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ11">
         <v>0.027960571</v>
@@ -4183,7 +4186,7 @@
         <v>0</v>
       </c>
       <c r="CO11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="12" spans="1:95">
@@ -4191,19 +4194,19 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E12" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F12" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G12">
         <v>0.0009776030000000001</v>
@@ -4287,7 +4290,7 @@
         <v>0</v>
       </c>
       <c r="AI12" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ12">
         <v>0.032951036</v>
@@ -4452,7 +4455,7 @@
         <v>0</v>
       </c>
       <c r="CO12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="13" spans="1:95">
@@ -4460,19 +4463,19 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E13" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="G13">
         <v>-2.89E-05</v>
@@ -4556,7 +4559,7 @@
         <v>0</v>
       </c>
       <c r="AI13" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ13">
         <v>0.179185242</v>
@@ -4721,7 +4724,7 @@
         <v>0</v>
       </c>
       <c r="CO13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="14" spans="1:95">
@@ -4729,19 +4732,19 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G14">
         <v>0.000431045</v>
@@ -4825,7 +4828,7 @@
         <v>0</v>
       </c>
       <c r="AI14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ14">
         <v>0.143233482</v>
@@ -4990,7 +4993,7 @@
         <v>0</v>
       </c>
       <c r="CO14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:95">
@@ -4998,19 +5001,19 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="G15">
         <v>0.000327551</v>
@@ -5094,7 +5097,7 @@
         <v>0</v>
       </c>
       <c r="AI15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ15">
         <v>0.138115134</v>
@@ -5259,7 +5262,7 @@
         <v>0</v>
       </c>
       <c r="CO15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" spans="1:95">
@@ -5267,19 +5270,19 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G16">
         <v>0.001162093</v>
@@ -5363,7 +5366,7 @@
         <v>0</v>
       </c>
       <c r="AI16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ16">
         <v>0.09650975000000001</v>
@@ -5528,7 +5531,7 @@
         <v>0</v>
       </c>
       <c r="CO16" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:93">
@@ -5536,19 +5539,19 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F17" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G17">
         <v>0.00141042</v>
@@ -5632,7 +5635,7 @@
         <v>0</v>
       </c>
       <c r="AI17" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ17">
         <v>0.060693695</v>
@@ -5797,7 +5800,7 @@
         <v>0</v>
       </c>
       <c r="CO17" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:93">
@@ -5805,19 +5808,19 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F18" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G18">
         <v>0.000897625</v>
@@ -5901,7 +5904,7 @@
         <v>0</v>
       </c>
       <c r="AI18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ18">
         <v>0.107514363</v>
@@ -6066,7 +6069,7 @@
         <v>0</v>
       </c>
       <c r="CO18" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="19" spans="1:93">
@@ -6074,19 +6077,19 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F19" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="G19">
         <v>0.000473511</v>
@@ -6170,7 +6173,7 @@
         <v>0</v>
       </c>
       <c r="AI19" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ19">
         <v>0.014898256</v>
@@ -6335,7 +6338,7 @@
         <v>0</v>
       </c>
       <c r="CO19" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="20" spans="1:93">
@@ -6343,19 +6346,19 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F20" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G20">
         <v>0.00029592</v>
@@ -6439,7 +6442,7 @@
         <v>0</v>
       </c>
       <c r="AI20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ20">
         <v>0.02858403</v>
@@ -6604,7 +6607,7 @@
         <v>0</v>
       </c>
       <c r="CO20" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="21" spans="1:93">
@@ -6612,19 +6615,19 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F21" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G21">
         <v>0.000354958</v>
@@ -6708,7 +6711,7 @@
         <v>0</v>
       </c>
       <c r="AI21" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ21">
         <v>0.082273481</v>
@@ -6873,7 +6876,7 @@
         <v>0</v>
       </c>
       <c r="CO21" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="22" spans="1:93">
@@ -6881,19 +6884,19 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F22" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G22">
         <v>0.000513154</v>
@@ -6977,7 +6980,7 @@
         <v>0</v>
       </c>
       <c r="AI22" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ22">
         <v>0.012592558</v>
@@ -7142,7 +7145,7 @@
         <v>0</v>
       </c>
       <c r="CO22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="23" spans="1:93">
@@ -7150,19 +7153,19 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G23">
         <v>0.000263694</v>
@@ -7246,7 +7249,7 @@
         <v>0</v>
       </c>
       <c r="AI23" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ23">
         <v>0.00903967</v>
@@ -7411,7 +7414,7 @@
         <v>0</v>
       </c>
       <c r="CO23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24" spans="1:93">
@@ -7419,19 +7422,19 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F24" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G24">
         <v>0.00048524</v>
@@ -7515,7 +7518,7 @@
         <v>0</v>
       </c>
       <c r="AI24" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ24">
         <v>0.030046089</v>
@@ -7680,7 +7683,7 @@
         <v>0</v>
       </c>
       <c r="CO24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:93">
@@ -7688,19 +7691,19 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E25" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F25" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G25">
         <v>0.000308954</v>
@@ -7784,7 +7787,7 @@
         <v>0</v>
       </c>
       <c r="AI25" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ25">
         <v>0.010607012</v>
@@ -7949,7 +7952,7 @@
         <v>0</v>
       </c>
       <c r="CO25" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" spans="1:93">
@@ -7957,19 +7960,19 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E26" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F26" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G26">
         <v>0.001706564</v>
@@ -8053,7 +8056,7 @@
         <v>0</v>
       </c>
       <c r="AI26" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ26">
         <v>0.053096335</v>
@@ -8218,7 +8221,7 @@
         <v>0</v>
       </c>
       <c r="CO26" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="27" spans="1:93">
@@ -8226,19 +8229,19 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E27" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F27" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G27">
         <v>0.001293263</v>
@@ -8322,7 +8325,7 @@
         <v>0</v>
       </c>
       <c r="AI27" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ27">
         <v>0.092674047</v>
@@ -8487,7 +8490,7 @@
         <v>0</v>
       </c>
       <c r="CO27" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" spans="1:93">
@@ -8495,19 +8498,19 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E28" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F28" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="G28">
         <v>0.001493963</v>
@@ -8591,7 +8594,7 @@
         <v>0</v>
       </c>
       <c r="AI28" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ28">
         <v>0.03099706</v>
@@ -8756,7 +8759,7 @@
         <v>0</v>
       </c>
       <c r="CO28" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:93">
@@ -8764,19 +8767,19 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E29" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F29" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G29">
         <v>0.001124522</v>
@@ -8860,7 +8863,7 @@
         <v>0</v>
       </c>
       <c r="AI29" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ29">
         <v>0.069423731</v>
@@ -9025,7 +9028,7 @@
         <v>0</v>
       </c>
       <c r="CO29" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" spans="1:93">
@@ -9033,19 +9036,19 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E30" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F30" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G30">
         <v>0.001194286</v>
@@ -9129,7 +9132,7 @@
         <v>0</v>
       </c>
       <c r="AI30" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ30">
         <v>0.060424834</v>
@@ -9294,7 +9297,7 @@
         <v>0</v>
       </c>
       <c r="CO30" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" spans="1:93">
@@ -9302,19 +9305,19 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E31" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F31" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G31">
         <v>0.002038684</v>
@@ -9398,7 +9401,7 @@
         <v>0</v>
       </c>
       <c r="AI31" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ31">
         <v>0.056666776</v>
@@ -9563,7 +9566,7 @@
         <v>0</v>
       </c>
       <c r="CO31" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="1:93">
@@ -9571,19 +9574,19 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E32" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F32" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G32">
         <v>0.003509328</v>
@@ -9667,7 +9670,7 @@
         <v>0</v>
       </c>
       <c r="AI32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ32">
         <v>0.098888062</v>
@@ -9832,7 +9835,7 @@
         <v>0</v>
       </c>
       <c r="CO32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" spans="1:95">
@@ -9840,19 +9843,19 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E33" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F33" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G33">
         <v>0.001020607</v>
@@ -9936,7 +9939,7 @@
         <v>0</v>
       </c>
       <c r="AI33" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ33">
         <v>0.035815903</v>
@@ -10101,7 +10104,7 @@
         <v>0</v>
       </c>
       <c r="CO33" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="34" spans="1:95">
@@ -10109,19 +10112,19 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E34" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F34" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G34">
         <v>0.001036188</v>
@@ -10205,7 +10208,7 @@
         <v>0</v>
       </c>
       <c r="AI34" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ34">
         <v>0.037311133</v>
@@ -10370,7 +10373,7 @@
         <v>0</v>
       </c>
       <c r="CO34" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="CP34">
         <v>-0.814742818</v>
@@ -10384,19 +10387,19 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E35" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F35" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="G35">
         <v>0.001410503</v>
@@ -10480,7 +10483,7 @@
         <v>0</v>
       </c>
       <c r="AI35" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ35">
         <v>0.041330496</v>
@@ -10645,7 +10648,7 @@
         <v>0</v>
       </c>
       <c r="CO35" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="CP35">
         <v>-0.753066891</v>
@@ -10659,19 +10662,19 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F36" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G36">
         <v>0.00072725</v>
@@ -10755,7 +10758,7 @@
         <v>0</v>
       </c>
       <c r="AI36" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ36">
         <v>0.047772102</v>
@@ -10920,7 +10923,7 @@
         <v>0</v>
       </c>
       <c r="CO36" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="CP36">
         <v>-0.872335259</v>
@@ -10934,19 +10937,19 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F37" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G37">
         <v>0.001640077</v>
@@ -11030,7 +11033,7 @@
         <v>0</v>
       </c>
       <c r="AI37" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ37">
         <v>0.060484521</v>
@@ -11195,7 +11198,7 @@
         <v>0</v>
       </c>
       <c r="CO37" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="CP37">
         <v>-0.759885442</v>
@@ -11209,19 +11212,19 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F38" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G38">
         <v>0.000951107</v>
@@ -11305,7 +11308,7 @@
         <v>0</v>
       </c>
       <c r="AI38" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ38">
         <v>0.061007062</v>
@@ -11470,7 +11473,7 @@
         <v>0</v>
       </c>
       <c r="CO38" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="CP38">
         <v>-0.838900609</v>
@@ -11484,19 +11487,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F39" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G39">
         <v>0.001738925</v>
@@ -11580,7 +11583,7 @@
         <v>0</v>
       </c>
       <c r="AI39" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ39">
         <v>0.025236369</v>
@@ -11745,7 +11748,7 @@
         <v>0</v>
       </c>
       <c r="CO39" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="CP39">
         <v>-0.780218664</v>
@@ -11759,19 +11762,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E40" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F40" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G40">
         <v>0.001263071</v>
@@ -11855,7 +11858,7 @@
         <v>0</v>
       </c>
       <c r="AI40" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ40">
         <v>0.031804424</v>
@@ -12020,7 +12023,7 @@
         <v>0</v>
       </c>
       <c r="CO40" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="CP40">
         <v>-0.79992089</v>
@@ -12034,19 +12037,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E41" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F41" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G41">
         <v>0.002702281</v>
@@ -12130,7 +12133,7 @@
         <v>0</v>
       </c>
       <c r="AI41" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ41">
         <v>0.072404657</v>
@@ -12295,7 +12298,7 @@
         <v>0</v>
       </c>
       <c r="CO41" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="CP41">
         <v>-0.528089775</v>
@@ -12309,19 +12312,19 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E42" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F42" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G42">
         <v>0.001559412</v>
@@ -12405,7 +12408,7 @@
         <v>0</v>
       </c>
       <c r="AI42" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ42">
         <v>0.06821192299999999</v>
@@ -12570,7 +12573,7 @@
         <v>0</v>
       </c>
       <c r="CO42" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="CP42">
         <v>-0.754849911</v>
@@ -12584,19 +12587,19 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E43" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F43" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G43">
         <v>0.001270244</v>
@@ -12680,7 +12683,7 @@
         <v>0</v>
       </c>
       <c r="AI43" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ43">
         <v>0.069326524</v>
@@ -12845,7 +12848,7 @@
         <v>0</v>
       </c>
       <c r="CO43" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="CP43">
         <v>-0.7655395739999999</v>
@@ -12859,19 +12862,19 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E44" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F44" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G44">
         <v>0.0009943969999999999</v>
@@ -12955,7 +12958,7 @@
         <v>0</v>
       </c>
       <c r="AI44" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ44">
         <v>0.036991009</v>
@@ -13120,7 +13123,7 @@
         <v>0</v>
       </c>
       <c r="CO44" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="CP44">
         <v>-0.829764531</v>
@@ -13134,19 +13137,19 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E45" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F45" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G45">
         <v>0.002384052</v>
@@ -13230,7 +13233,7 @@
         <v>0</v>
       </c>
       <c r="AI45" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ45">
         <v>0.036729519</v>
@@ -13395,7 +13398,7 @@
         <v>0</v>
       </c>
       <c r="CO45" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="CP45">
         <v>-0.404237806</v>
@@ -13409,19 +13412,19 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E46" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F46" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G46">
         <v>0.001488019</v>
@@ -13505,7 +13508,7 @@
         <v>0</v>
       </c>
       <c r="AI46" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ46">
         <v>0.045071814</v>
@@ -13670,7 +13673,7 @@
         <v>0</v>
       </c>
       <c r="CO46" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="CP46">
         <v>-0.703677808</v>
@@ -13684,19 +13687,19 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F47" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G47">
         <v>0.001436084</v>
@@ -13780,7 +13783,7 @@
         <v>0</v>
       </c>
       <c r="AI47" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ47">
         <v>0.0580535</v>
@@ -13945,7 +13948,7 @@
         <v>0</v>
       </c>
       <c r="CO47" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="CP47">
         <v>-0.753715321</v>
@@ -13959,19 +13962,19 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E48" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F48" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G48">
         <v>0.001379037</v>
@@ -14055,7 +14058,7 @@
         <v>0</v>
       </c>
       <c r="AI48" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ48">
         <v>0.056639031</v>
@@ -14220,7 +14223,7 @@
         <v>0</v>
       </c>
       <c r="CO48" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="CP48">
         <v>-0.71793867</v>
@@ -14234,19 +14237,19 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E49" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F49" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="G49">
         <v>0.00225795</v>
@@ -14330,7 +14333,7 @@
         <v>0</v>
       </c>
       <c r="AI49" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ49">
         <v>0.074241638</v>
@@ -14495,7 +14498,7 @@
         <v>0</v>
       </c>
       <c r="CO49" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="CP49">
         <v>-0.655169358</v>
@@ -14509,19 +14512,19 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E50" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F50" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G50">
         <v>0.002405425</v>
@@ -14605,7 +14608,7 @@
         <v>0</v>
       </c>
       <c r="AI50" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ50">
         <v>0.05430774</v>
@@ -14770,7 +14773,7 @@
         <v>0</v>
       </c>
       <c r="CO50" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="CP50">
         <v>-0.6872439380000001</v>
@@ -14784,19 +14787,19 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E51" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F51" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G51">
         <v>0.00267884</v>
@@ -14880,7 +14883,7 @@
         <v>0</v>
       </c>
       <c r="AI51" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ51">
         <v>0.080539377</v>
@@ -15045,7 +15048,7 @@
         <v>0</v>
       </c>
       <c r="CO51" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="CP51">
         <v>-0.596275172</v>
@@ -15059,19 +15062,19 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E52" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F52" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G52">
         <v>0.001221159</v>
@@ -15155,7 +15158,7 @@
         <v>0</v>
       </c>
       <c r="AI52" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ52">
         <v>0.032588051</v>
@@ -15320,7 +15323,7 @@
         <v>0</v>
       </c>
       <c r="CO52" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="CP52">
         <v>-0.808081961</v>
@@ -15334,19 +15337,19 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F53" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G53">
         <v>0.00093247</v>
@@ -15430,7 +15433,7 @@
         <v>0</v>
       </c>
       <c r="AI53" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ53">
         <v>0.026475554</v>
@@ -15595,7 +15598,7 @@
         <v>0</v>
       </c>
       <c r="CO53" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="CP53">
         <v>-0.77227813</v>
@@ -15609,19 +15612,19 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C54" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D54" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G54">
         <v>0.0008229381467956</v>
@@ -15705,7 +15708,7 @@
         <v>0</v>
       </c>
       <c r="AI54" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ54">
         <v>0.0245106310926154</v>
@@ -15870,7 +15873,7 @@
         <v>0</v>
       </c>
       <c r="CO54" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="CP54">
         <v>-0.8664117478627688</v>
@@ -15884,16 +15887,16 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C55" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D55" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F55" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G55">
         <v>0.0022239398231451</v>
@@ -15977,7 +15980,7 @@
         <v>0</v>
       </c>
       <c r="AI55" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ55">
         <v>0.0779439577559576</v>
@@ -16142,7 +16145,7 @@
         <v>0</v>
       </c>
       <c r="CO55" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="CP55">
         <v>-0.7108907987632488</v>
@@ -16156,13 +16159,13 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C56" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F56" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G56">
         <v>0.0018211096217568</v>
@@ -16246,7 +16249,7 @@
         <v>0</v>
       </c>
       <c r="AI56" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ56">
         <v>0.0402740604837066</v>
@@ -16411,7 +16414,7 @@
         <v>0</v>
       </c>
       <c r="CO56" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="CP56">
         <v>-0.7447372903525753</v>
@@ -16425,10 +16428,10 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F57" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G57">
         <v>0.0012556275124289</v>
@@ -16512,7 +16515,7 @@
         <v>0</v>
       </c>
       <c r="AI57" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ57">
         <v>0.0441363962743036</v>
@@ -16677,7 +16680,7 @@
         <v>0</v>
       </c>
       <c r="CO57" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="CP57">
         <v>-0.7777179486581601</v>
@@ -16691,10 +16694,10 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F58" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G58">
         <v>0.0019905125443684</v>
@@ -16778,7 +16781,7 @@
         <v>0</v>
       </c>
       <c r="AI58" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ58">
         <v>0.0589646348207879</v>
@@ -16943,7 +16946,7 @@
         <v>0</v>
       </c>
       <c r="CO58" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="CP58">
         <v>-0.7757098341832183</v>
@@ -16957,10 +16960,10 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F59" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G59">
         <v>0.0005221982670147</v>
@@ -17044,7 +17047,7 @@
         <v>0</v>
       </c>
       <c r="AI59" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ59">
         <v>0.0088498418945465</v>
@@ -17209,7 +17212,7 @@
         <v>0</v>
       </c>
       <c r="CO59" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="CP59">
         <v>-0.9614802262041642</v>
@@ -17223,10 +17226,10 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F60" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G60">
         <v>0.0018105477499388</v>
@@ -17310,7 +17313,7 @@
         <v>0</v>
       </c>
       <c r="AI60" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ60">
         <v>0.0438527807624406</v>
@@ -17475,7 +17478,7 @@
         <v>0</v>
       </c>
       <c r="CO60" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="CP60">
         <v>-0.6569921650581255</v>
@@ -17489,10 +17492,10 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F61" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G61">
         <v>0.0006776201968474</v>
@@ -17576,7 +17579,7 @@
         <v>0</v>
       </c>
       <c r="AI61" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ61">
         <v>0.0175722673111926</v>
@@ -17741,7 +17744,7 @@
         <v>0</v>
       </c>
       <c r="CO61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="CP61">
         <v>-0.924044412704054</v>
@@ -17755,10 +17758,10 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G62">
         <v>0.0025014106780221</v>
@@ -17842,7 +17845,7 @@
         <v>0</v>
       </c>
       <c r="AI62" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ62">
         <v>0.0551224625318549</v>
@@ -18007,7 +18010,7 @@
         <v>0</v>
       </c>
       <c r="CO62" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="CP62">
         <v>-0.6213262971882773</v>
@@ -18021,10 +18024,10 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F63" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G63">
         <v>0.0007538484415952</v>
@@ -18108,7 +18111,7 @@
         <v>0</v>
       </c>
       <c r="AI63" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ63">
         <v>0.0157574961492794</v>
@@ -18273,7 +18276,7 @@
         <v>0</v>
       </c>
       <c r="CO63" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="CP63">
         <v>-0.9477002142299265</v>
@@ -18287,10 +18290,10 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F64" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G64">
         <v>0.0012416962587069</v>
@@ -18374,7 +18377,7 @@
         <v>0</v>
       </c>
       <c r="AI64" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ64">
         <v>0.0348775184726272</v>
@@ -18539,7 +18542,7 @@
         <v>0</v>
       </c>
       <c r="CO64" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="CP64">
         <v>-0.7774025388699596</v>
@@ -18553,10 +18556,10 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F65" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="G65">
         <v>0.0015984483099258</v>
@@ -18640,7 +18643,7 @@
         <v>0</v>
       </c>
       <c r="AI65" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ65">
         <v>0.0617007650932976</v>
@@ -18805,7 +18808,7 @@
         <v>0</v>
       </c>
       <c r="CO65" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="CP65">
         <v>-0.8140402180385446</v>
@@ -18906,7 +18909,7 @@
         <v>0.01083306576401342</v>
       </c>
       <c r="AI66" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ66">
         <v>0.01228964656713829</v>
@@ -19178,7 +19181,7 @@
         <v>0.009662114019183791</v>
       </c>
       <c r="AI67" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ67">
         <v>0.01570755211730832</v>
@@ -19450,7 +19453,7 @@
         <v>0.009682496602030617</v>
       </c>
       <c r="AI68" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AJ68">
         <v>0.01945380747640302</v>
@@ -19628,6 +19631,278 @@
       </c>
       <c r="CQ68">
         <v>-0.889563108338023</v>
+      </c>
+    </row>
+    <row r="69" spans="1:95">
+      <c r="A69" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F69" t="s">
+        <v>97</v>
+      </c>
+      <c r="G69">
+        <v>0.001608957414964252</v>
+      </c>
+      <c r="H69">
+        <v>0.0008044787074821258</v>
+      </c>
+      <c r="I69">
+        <v>0.0003571463938587538</v>
+      </c>
+      <c r="J69">
+        <v>0.0003571463938587538</v>
+      </c>
+      <c r="K69">
+        <v>0.001603286941914916</v>
+      </c>
+      <c r="L69">
+        <v>0.0008016434709574582</v>
+      </c>
+      <c r="M69">
+        <v>0.0002687967158724325</v>
+      </c>
+      <c r="N69">
+        <v>0.0002687967158724325</v>
+      </c>
+      <c r="O69">
+        <v>16.40656497393319</v>
+      </c>
+      <c r="P69">
+        <v>5.073411855570574</v>
+      </c>
+      <c r="Q69">
+        <v>0.2697152126036517</v>
+      </c>
+      <c r="R69">
+        <v>0.6266762319713819</v>
+      </c>
+      <c r="S69">
+        <v>0.08883818203683971</v>
+      </c>
+      <c r="T69">
+        <v>0.04489116784346199</v>
+      </c>
+      <c r="U69">
+        <v>0.2495207077372677</v>
+      </c>
+      <c r="V69">
+        <v>0.2094378518612111</v>
+      </c>
+      <c r="W69">
+        <v>0.9978219926990421</v>
+      </c>
+      <c r="X69">
+        <v>0.7881744606169196</v>
+      </c>
+      <c r="Y69">
+        <v>0.8192834571553508</v>
+      </c>
+      <c r="Z69">
+        <v>0.9993986490679695</v>
+      </c>
+      <c r="AA69">
+        <v>0.7599514521940335</v>
+      </c>
+      <c r="AB69">
+        <v>0.7972078777545685</v>
+      </c>
+      <c r="AC69">
+        <v>0.01024003797240197</v>
+      </c>
+      <c r="AD69">
+        <v>0.006816341845870443</v>
+      </c>
+      <c r="AE69">
+        <v>0.9978219926990421</v>
+      </c>
+      <c r="AF69">
+        <v>0.9993986490679695</v>
+      </c>
+      <c r="AG69">
+        <v>0.01024003797240197</v>
+      </c>
+      <c r="AH69">
+        <v>0.006816341845870443</v>
+      </c>
+      <c r="AI69" t="s">
+        <v>215</v>
+      </c>
+      <c r="AJ69">
+        <v>0.03948313241528283</v>
+      </c>
+      <c r="AK69">
+        <v>0.01485127720624749</v>
+      </c>
+      <c r="AL69">
+        <v>-2387.37729948</v>
+      </c>
+      <c r="AM69">
+        <v>-182.3800568</v>
+      </c>
+      <c r="AN69">
+        <v>56666.77310052046</v>
+      </c>
+      <c r="AO69">
+        <v>14700.21875206001</v>
+      </c>
+      <c r="AP69">
+        <v>56643.45350052046</v>
+      </c>
+      <c r="AQ69">
+        <v>14700.39215206001</v>
+      </c>
+      <c r="AR69">
+        <v>4.666677310052046</v>
+      </c>
+      <c r="AS69">
+        <v>0.4700218752060012</v>
+      </c>
+      <c r="AT69">
+        <v>1.461674481667702</v>
+      </c>
+      <c r="AU69">
+        <v>4.726807357329923</v>
+      </c>
+      <c r="AV69">
+        <v>84.83333333333333</v>
+      </c>
+      <c r="AW69">
+        <v>116.2</v>
+      </c>
+      <c r="AX69">
+        <v>0.01830746773368767</v>
+      </c>
+      <c r="AY69">
+        <v>0.05152826515925592</v>
+      </c>
+      <c r="AZ69">
+        <v>-914.8050393927592</v>
+      </c>
+      <c r="BA69">
+        <v>-265.3143236894216</v>
+      </c>
+      <c r="BB69">
+        <v>6928</v>
+      </c>
+      <c r="BC69">
+        <v>2263</v>
+      </c>
+      <c r="BD69">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BE69">
+        <v>10774</v>
+      </c>
+      <c r="BF69">
+        <v>3211</v>
+      </c>
+      <c r="BG69">
+        <v>17702</v>
+      </c>
+      <c r="BH69">
+        <v>5474</v>
+      </c>
+      <c r="BI69">
+        <v>6536</v>
+      </c>
+      <c r="BJ69">
+        <v>2208</v>
+      </c>
+      <c r="BK69">
+        <v>6923</v>
+      </c>
+      <c r="BL69">
+        <v>2259</v>
+      </c>
+      <c r="BM69">
+        <v>4238</v>
+      </c>
+      <c r="BN69">
+        <v>1003</v>
+      </c>
+      <c r="BO69">
+        <v>5</v>
+      </c>
+      <c r="BP69">
+        <v>4</v>
+      </c>
+      <c r="BQ69">
+        <v>0</v>
+      </c>
+      <c r="BR69">
+        <v>0</v>
+      </c>
+      <c r="BS69">
+        <v>46666.77310051995</v>
+      </c>
+      <c r="BT69">
+        <v>4701.214143200003</v>
+      </c>
+      <c r="BU69">
+        <v>0.06929158494601359</v>
+      </c>
+      <c r="BV69">
+        <v>0.0669357108338629</v>
+      </c>
+      <c r="BW69">
+        <v>0.1587398401351162</v>
+      </c>
+      <c r="BX69">
+        <v>0.1685995849649735</v>
+      </c>
+      <c r="BY69">
+        <v>0.01391394865496849</v>
+      </c>
+      <c r="BZ69">
+        <v>0.01749637562093771</v>
+      </c>
+      <c r="CA69">
+        <v>0.01140419033963007</v>
+      </c>
+      <c r="CB69">
+        <v>0.01454621944057001</v>
+      </c>
+      <c r="CC69">
+        <v>49054.15039999995</v>
+      </c>
+      <c r="CD69">
+        <v>4883.594200000003</v>
+      </c>
+      <c r="CE69">
+        <v>49968.95543939271</v>
+      </c>
+      <c r="CF69">
+        <v>5148.908523689424</v>
+      </c>
+      <c r="CG69">
+        <v>0.1506658519129359</v>
+      </c>
+      <c r="CH69">
+        <v>0.04590873357131624</v>
+      </c>
+      <c r="CI69">
+        <v>10000</v>
+      </c>
+      <c r="CK69">
+        <v>0.001506024096385542</v>
+      </c>
+      <c r="CL69">
+        <v>0.003166512202656781</v>
+      </c>
+      <c r="CM69">
+        <v>19230472.27697121</v>
+      </c>
+      <c r="CN69">
+        <v>1162734.066962649</v>
+      </c>
+      <c r="CO69" s="2">
+        <v>45401.25317957817</v>
+      </c>
+      <c r="CP69">
+        <v>-0.6790216377125027</v>
+      </c>
+      <c r="CQ69">
+        <v>-0.8261410353744627</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MATICUSDT.json at 2024-04-19_14-53-52 bestfile_scores 0.0009654249405869036 bestfile_sharp 0.038748918495049724
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -19641,190 +19641,190 @@
         <v>97</v>
       </c>
       <c r="G69">
-        <v>0.001608957414964252</v>
+        <v>0.002050883476106824</v>
       </c>
       <c r="H69">
-        <v>0.0008044787074821258</v>
+        <v>0.001025441738053412</v>
       </c>
       <c r="I69">
-        <v>0.0003571463938587538</v>
+        <v>0.0007475161254359985</v>
       </c>
       <c r="J69">
-        <v>0.0003571463938587538</v>
+        <v>0.0007475161254359985</v>
       </c>
       <c r="K69">
-        <v>0.001603286941914916</v>
+        <v>0.001872874017962722</v>
       </c>
       <c r="L69">
-        <v>0.0008016434709574582</v>
+        <v>0.0009364370089813612</v>
       </c>
       <c r="M69">
-        <v>0.0002687967158724325</v>
+        <v>0.000569820430868706</v>
       </c>
       <c r="N69">
-        <v>0.0002687967158724325</v>
+        <v>0.000569820430868706</v>
       </c>
       <c r="O69">
-        <v>16.40656497393319</v>
+        <v>12.62699362811354</v>
       </c>
       <c r="P69">
-        <v>5.073411855570574</v>
+        <v>6.830662290017378</v>
       </c>
       <c r="Q69">
-        <v>0.2697152126036517</v>
+        <v>0.2672148819739805</v>
       </c>
       <c r="R69">
-        <v>0.6266762319713819</v>
+        <v>0.6069758053114781</v>
       </c>
       <c r="S69">
-        <v>0.08883818203683971</v>
+        <v>0.09274541918400059</v>
       </c>
       <c r="T69">
-        <v>0.04489116784346199</v>
+        <v>0.08682770305057673</v>
       </c>
       <c r="U69">
-        <v>0.2495207077372677</v>
+        <v>0.2410199269924077</v>
       </c>
       <c r="V69">
-        <v>0.2094378518612111</v>
+        <v>0.233509923362278</v>
       </c>
       <c r="W69">
-        <v>0.9978219926990421</v>
+        <v>0.9975191552500322</v>
       </c>
       <c r="X69">
-        <v>0.7881744606169196</v>
+        <v>0.8087933235498754</v>
       </c>
       <c r="Y69">
-        <v>0.8192834571553508</v>
+        <v>0.8039615175759266</v>
       </c>
       <c r="Z69">
-        <v>0.9993986490679695</v>
+        <v>0.9985600812219979</v>
       </c>
       <c r="AA69">
-        <v>0.7599514521940335</v>
+        <v>0.7590487591739689</v>
       </c>
       <c r="AB69">
-        <v>0.7972078777545685</v>
+        <v>0.7787257794378143</v>
       </c>
       <c r="AC69">
-        <v>0.01024003797240197</v>
+        <v>0.01019384000883422</v>
       </c>
       <c r="AD69">
-        <v>0.006816341845870443</v>
+        <v>0.009502809785555974</v>
       </c>
       <c r="AE69">
-        <v>0.9978219926990421</v>
+        <v>0.9975191552500322</v>
       </c>
       <c r="AF69">
-        <v>0.9993986490679695</v>
+        <v>0.9985600812219979</v>
       </c>
       <c r="AG69">
-        <v>0.01024003797240197</v>
+        <v>0.01019384000883422</v>
       </c>
       <c r="AH69">
-        <v>0.006816341845870443</v>
+        <v>0.009502809785555974</v>
       </c>
       <c r="AI69" t="s">
         <v>215</v>
       </c>
       <c r="AJ69">
-        <v>0.03948313241528283</v>
+        <v>0.04679962694772061</v>
       </c>
       <c r="AK69">
-        <v>0.01485127720624749</v>
+        <v>0.03778110269298413</v>
       </c>
       <c r="AL69">
-        <v>-2387.37729948</v>
+        <v>-2767.31383998</v>
       </c>
       <c r="AM69">
-        <v>-182.3800568</v>
+        <v>-520.9325969600001</v>
       </c>
       <c r="AN69">
-        <v>56666.77310052046</v>
+        <v>91207.47826001985</v>
       </c>
       <c r="AO69">
-        <v>14700.21875206001</v>
+        <v>22394.66017984009</v>
       </c>
       <c r="AP69">
-        <v>56643.45350052046</v>
+        <v>91168.93766001986</v>
       </c>
       <c r="AQ69">
-        <v>14700.39215206001</v>
+        <v>22394.17117984009</v>
       </c>
       <c r="AR69">
-        <v>4.666677310052046</v>
+        <v>8.120747826001985</v>
       </c>
       <c r="AS69">
-        <v>0.4700218752060012</v>
+        <v>1.239466017984009</v>
       </c>
       <c r="AT69">
-        <v>1.461674481667702</v>
+        <v>1.899856859722528</v>
       </c>
       <c r="AU69">
-        <v>4.726807357329923</v>
+        <v>3.513136110734157</v>
       </c>
       <c r="AV69">
-        <v>84.83333333333333</v>
+        <v>104.4333333333333</v>
       </c>
       <c r="AW69">
-        <v>116.2</v>
+        <v>118.75</v>
       </c>
       <c r="AX69">
-        <v>0.01830746773368767</v>
+        <v>0.06825567338459632</v>
       </c>
       <c r="AY69">
-        <v>0.05152826515925592</v>
+        <v>0.1015446510087083</v>
       </c>
       <c r="AZ69">
-        <v>-914.8050393927592</v>
+        <v>-6151.64033564636</v>
       </c>
       <c r="BA69">
-        <v>-265.3143236894216</v>
+        <v>-1460.074453297303</v>
       </c>
       <c r="BB69">
-        <v>6928</v>
+        <v>4766</v>
       </c>
       <c r="BC69">
-        <v>2263</v>
+        <v>3091</v>
       </c>
       <c r="BD69">
         <v>1078.958333333333</v>
       </c>
       <c r="BE69">
-        <v>10774</v>
+        <v>8858</v>
       </c>
       <c r="BF69">
-        <v>3211</v>
+        <v>4279</v>
       </c>
       <c r="BG69">
-        <v>17702</v>
+        <v>13624</v>
       </c>
       <c r="BH69">
-        <v>5474</v>
+        <v>7370</v>
       </c>
       <c r="BI69">
-        <v>6536</v>
+        <v>4236</v>
       </c>
       <c r="BJ69">
-        <v>2208</v>
+        <v>2947</v>
       </c>
       <c r="BK69">
-        <v>6923</v>
+        <v>4740</v>
       </c>
       <c r="BL69">
-        <v>2259</v>
+        <v>3050</v>
       </c>
       <c r="BM69">
-        <v>4238</v>
+        <v>4622</v>
       </c>
       <c r="BN69">
-        <v>1003</v>
+        <v>1332</v>
       </c>
       <c r="BO69">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="BP69">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="BQ69">
         <v>0</v>
@@ -19833,76 +19833,76 @@
         <v>0</v>
       </c>
       <c r="BS69">
-        <v>46666.77310051995</v>
+        <v>81207.47826001993</v>
       </c>
       <c r="BT69">
-        <v>4701.214143200003</v>
+        <v>12397.63760304</v>
       </c>
       <c r="BU69">
-        <v>0.06929158494601359</v>
+        <v>0.06472944544205009</v>
       </c>
       <c r="BV69">
-        <v>0.0669357108338629</v>
+        <v>0.08449359486621975</v>
       </c>
       <c r="BW69">
-        <v>0.1587398401351162</v>
+        <v>0.1369613061020943</v>
       </c>
       <c r="BX69">
-        <v>0.1685995849649735</v>
+        <v>0.1811825401044125</v>
       </c>
       <c r="BY69">
-        <v>0.01391394865496849</v>
+        <v>0.01432038218044533</v>
       </c>
       <c r="BZ69">
-        <v>0.01749637562093771</v>
+        <v>0.01704466126997548</v>
       </c>
       <c r="CA69">
-        <v>0.01140419033963007</v>
+        <v>0.01127103045173808</v>
       </c>
       <c r="CB69">
-        <v>0.01454621944057001</v>
+        <v>0.01476436301747337</v>
       </c>
       <c r="CC69">
-        <v>49054.15039999995</v>
+        <v>83974.79209999992</v>
       </c>
       <c r="CD69">
-        <v>4883.594200000003</v>
+        <v>12918.57019999999</v>
       </c>
       <c r="CE69">
-        <v>49968.95543939271</v>
+        <v>90126.43243564627</v>
       </c>
       <c r="CF69">
-        <v>5148.908523689424</v>
+        <v>14378.6446532973</v>
       </c>
       <c r="CG69">
-        <v>0.1506658519129359</v>
+        <v>0.1596303003768157</v>
       </c>
       <c r="CH69">
-        <v>0.04590873357131624</v>
+        <v>0.06926056623035046</v>
       </c>
       <c r="CI69">
         <v>10000</v>
       </c>
       <c r="CK69">
-        <v>0.001506024096385542</v>
+        <v>0.002664504170528267</v>
       </c>
       <c r="CL69">
-        <v>0.003166512202656781</v>
+        <v>0.008456904541241891</v>
       </c>
       <c r="CM69">
-        <v>19230472.27697121</v>
+        <v>31206714.64650577</v>
       </c>
       <c r="CN69">
-        <v>1162734.066962649</v>
+        <v>3444392.687119505</v>
       </c>
       <c r="CO69" s="2">
-        <v>45401.25317957817</v>
+        <v>45401.44958580234</v>
       </c>
       <c r="CP69">
-        <v>-0.6790216377125027</v>
+        <v>-0.5814104972412503</v>
       </c>
       <c r="CQ69">
-        <v>-0.8261410353744627</v>
+        <v>-0.7012550955960412</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AVAXUSDT.json at 2024-04-20_09-52-20 bestfile_scores 0.0005777979452188831 bestfile_sharp 0.1494920524603618
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -20165,190 +20165,190 @@
         <v>95</v>
       </c>
       <c r="H70">
-        <v>0.003197292110093786</v>
+        <v>0.004410416036765064</v>
       </c>
       <c r="I70">
-        <v>0.001598646055046893</v>
+        <v>0.002205208018382532</v>
       </c>
       <c r="J70">
-        <v>0.0007810938403536305</v>
+        <v>0.0007758914468987133</v>
       </c>
       <c r="K70">
-        <v>0.0007810938403536305</v>
+        <v>0.0007758914468987133</v>
       </c>
       <c r="L70">
-        <v>0.002008615794338797</v>
+        <v>0.002181850582277911</v>
       </c>
       <c r="M70">
-        <v>0.001004307897169399</v>
+        <v>0.001090925291138956</v>
       </c>
       <c r="N70">
-        <v>0.0004776519697776927</v>
+        <v>0.0005097741760766716</v>
       </c>
       <c r="O70">
-        <v>0.0004776519697776927</v>
+        <v>0.0005097741760766716</v>
       </c>
       <c r="P70">
-        <v>41.27870245221085</v>
+        <v>13.1608418613632</v>
       </c>
       <c r="Q70">
-        <v>16.90797451245414</v>
+        <v>23.81370921027225</v>
       </c>
       <c r="R70">
-        <v>0.3988818621456781</v>
+        <v>0.3886053375468781</v>
       </c>
       <c r="S70">
-        <v>0.5954072982543913</v>
+        <v>0.6270108615110761</v>
       </c>
       <c r="T70">
-        <v>0.01056349609370588</v>
+        <v>0.0500358317632592</v>
       </c>
       <c r="U70">
-        <v>0.09306890296499781</v>
+        <v>0.09533166990064181</v>
       </c>
       <c r="V70">
-        <v>0.1266041159985717</v>
+        <v>0.2201260714374058</v>
       </c>
       <c r="W70">
-        <v>0.2346535458716338</v>
+        <v>0.2201688859977751</v>
       </c>
       <c r="X70">
-        <v>0.9998505645626301</v>
+        <v>0.9991582184589494</v>
       </c>
       <c r="Y70">
-        <v>0.9147634322457596</v>
+        <v>0.8137804555398892</v>
       </c>
       <c r="Z70">
-        <v>0.7884447887873871</v>
+        <v>0.809870664784014</v>
       </c>
       <c r="AA70">
-        <v>0.9984740719203027</v>
+        <v>0.9980130122355819</v>
       </c>
       <c r="AB70">
-        <v>0.8627130938519509</v>
+        <v>0.7332150459198449</v>
       </c>
       <c r="AC70">
-        <v>0.7662821743387359</v>
+        <v>0.7892375070519728</v>
       </c>
       <c r="AD70">
-        <v>0.002223460458959708</v>
+        <v>0.006833369621658581</v>
       </c>
       <c r="AE70">
-        <v>0.01034518536521765</v>
+        <v>0.01003757165240989</v>
       </c>
       <c r="AF70">
-        <v>0.9998505645626301</v>
+        <v>0.9991582184589494</v>
       </c>
       <c r="AG70">
-        <v>0.9984740719203027</v>
+        <v>0.9980130122355819</v>
       </c>
       <c r="AH70">
-        <v>0.002223460458959708</v>
+        <v>0.006833369621658581</v>
       </c>
       <c r="AI70">
-        <v>0.01034518536521765</v>
+        <v>0.01003757165240989</v>
       </c>
       <c r="AJ70" t="s">
         <v>226</v>
       </c>
       <c r="AK70">
-        <v>0.006729657638389397</v>
+        <v>0.0260012684361012</v>
       </c>
       <c r="AL70">
-        <v>0.04123834186308471</v>
+        <v>0.05899741597904416</v>
       </c>
       <c r="AM70">
-        <v>-34473.276135334</v>
+        <v>-54683.400538804</v>
       </c>
       <c r="AN70">
-        <v>-1009.91150606</v>
+        <v>-1534.434274444</v>
       </c>
       <c r="AO70">
-        <v>313195.271052465</v>
+        <v>1153755.044321193</v>
       </c>
       <c r="AP70">
-        <v>23220.22885394001</v>
+        <v>23090.35580555591</v>
       </c>
       <c r="AQ70">
-        <v>313184.1200524649</v>
+        <v>1153583.740621193</v>
       </c>
       <c r="AR70">
-        <v>23218.51165394002</v>
+        <v>23087.34630555591</v>
       </c>
       <c r="AS70">
-        <v>30.3195271052465</v>
+        <v>114.3755044321193</v>
       </c>
       <c r="AT70">
-        <v>1.322022885394001</v>
+        <v>1.309035580555591</v>
       </c>
       <c r="AU70">
-        <v>0.5808821878438153</v>
+        <v>1.821888865413057</v>
       </c>
       <c r="AV70">
-        <v>1.418469283338815</v>
+        <v>1.007097912531299</v>
       </c>
       <c r="AW70">
-        <v>67.45</v>
+        <v>85.68333333333334</v>
       </c>
       <c r="AX70">
-        <v>112.65</v>
+        <v>108.2166666666667</v>
       </c>
       <c r="AY70">
-        <v>0.0002936325718988755</v>
+        <v>0.001816227246539547</v>
       </c>
       <c r="AZ70">
-        <v>0.008562780961992802</v>
+        <v>0.1144259642161577</v>
       </c>
       <c r="BA70">
-        <v>-99.18152393743236</v>
+        <v>-2180.597016570432</v>
       </c>
       <c r="BB70">
-        <v>-122.9019575029915</v>
+        <v>-1889.684700253975</v>
       </c>
       <c r="BC70">
-        <v>20198</v>
+        <v>6300</v>
       </c>
       <c r="BD70">
-        <v>8405</v>
+        <v>11140</v>
       </c>
       <c r="BE70">
         <v>1078.958333333333</v>
       </c>
       <c r="BF70">
-        <v>24340</v>
+        <v>7900</v>
       </c>
       <c r="BG70">
-        <v>9838</v>
+        <v>14554</v>
       </c>
       <c r="BH70">
-        <v>44538</v>
+        <v>14200</v>
       </c>
       <c r="BI70">
-        <v>18243</v>
+        <v>25694</v>
       </c>
       <c r="BJ70">
-        <v>19991</v>
+        <v>5652</v>
       </c>
       <c r="BK70">
-        <v>8207</v>
+        <v>11061</v>
       </c>
       <c r="BL70">
-        <v>20193</v>
+        <v>6282</v>
       </c>
       <c r="BM70">
-        <v>8206</v>
+        <v>11096</v>
       </c>
       <c r="BN70">
-        <v>4349</v>
+        <v>2248</v>
       </c>
       <c r="BO70">
-        <v>1631</v>
+        <v>3493</v>
       </c>
       <c r="BP70">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="BQ70">
-        <v>199</v>
+        <v>44</v>
       </c>
       <c r="BR70">
         <v>0</v>
@@ -20357,76 +20357,76 @@
         <v>0</v>
       </c>
       <c r="BT70">
-        <v>303201.7997946653</v>
+        <v>1143755.044321196</v>
       </c>
       <c r="BU70">
-        <v>13220.22885393998</v>
+        <v>13090.35580555596</v>
       </c>
       <c r="BV70">
-        <v>0.02018660178594265</v>
+        <v>0.04328865773378397</v>
       </c>
       <c r="BW70">
-        <v>0.08325059723983033</v>
+        <v>0.08044988179076616</v>
       </c>
       <c r="BX70">
-        <v>0.06736077986163409</v>
+        <v>0.1234707060681545</v>
       </c>
       <c r="BY70">
-        <v>0.1890248146561201</v>
+        <v>0.1740696259184592</v>
       </c>
       <c r="BZ70">
-        <v>0.005944566715605079</v>
+        <v>0.009285771563490365</v>
       </c>
       <c r="CA70">
-        <v>0.01788193827177928</v>
+        <v>0.01630172262815842</v>
       </c>
       <c r="CB70">
-        <v>0.004868492323286427</v>
+        <v>0.008341415513819126</v>
       </c>
       <c r="CC70">
-        <v>0.01315967622066296</v>
+        <v>0.01169230847462865</v>
       </c>
       <c r="CD70">
-        <v>337675.0759299993</v>
+        <v>1198438.44486</v>
       </c>
       <c r="CE70">
-        <v>14230.14035999998</v>
+        <v>14624.79007999996</v>
       </c>
       <c r="CF70">
-        <v>337774.2574539367</v>
+        <v>1200619.04187657</v>
       </c>
       <c r="CG70">
-        <v>14353.04231750297</v>
+        <v>16514.47478025394</v>
       </c>
       <c r="CH70">
-        <v>0.03874891849504972</v>
+        <v>0.04296369618829193</v>
       </c>
       <c r="CI70">
-        <v>0.08045108644220864</v>
+        <v>0.08046611845312036</v>
       </c>
       <c r="CJ70">
         <v>10000</v>
       </c>
       <c r="CL70">
-        <v>0.001776336113685511</v>
+        <v>0.006912264442384924</v>
       </c>
       <c r="CM70">
-        <v>0.01706827309236948</v>
+        <v>0.01672072907012666</v>
       </c>
       <c r="CN70">
-        <v>128402449.1105698</v>
+        <v>369252754.6086284</v>
       </c>
       <c r="CO70">
-        <v>6336875.528540782</v>
+        <v>8020410.490554446</v>
       </c>
       <c r="CP70" s="2">
-        <v>45401.62075843258</v>
+        <v>45401.84767321962</v>
       </c>
       <c r="CQ70">
-        <v>-0.3418779213839334</v>
+        <v>-0.1225754953154068</v>
       </c>
       <c r="CR70">
-        <v>-0.7885323258390414</v>
+        <v>-0.7733579091455093</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SUSHIUSDT.json at 2024-04-21_01-45-27 bestfile_scores 0.000507899072581916 bestfile_sharp 0.1019064101175263
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="303">
   <si>
     <t>Unnamed: 0.6</t>
   </si>
@@ -310,6 +310,9 @@
     <t>SANDUSDT</t>
   </si>
   <si>
+    <t>GMTUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -578,9 +581,6 @@
   </si>
   <si>
     <t>RNDRUSDT</t>
-  </si>
-  <si>
-    <t>GMTUSDT</t>
   </si>
   <si>
     <t>SUSHIUSDT</t>
@@ -1284,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CT72"/>
+  <dimension ref="A1:CT73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:98">
@@ -1585,28 +1585,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J2">
         <v>0.0009987329999999999</v>
@@ -1863,28 +1863,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J3">
         <v>0.001058605</v>
@@ -2141,28 +2141,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J4">
         <v>0.000882894</v>
@@ -2419,28 +2419,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I5" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J5">
         <v>0.001186265</v>
@@ -2697,25 +2697,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I6" t="s">
         <v>97</v>
@@ -2975,28 +2975,28 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I7" t="s">
-        <v>188</v>
+        <v>98</v>
       </c>
       <c r="J7">
         <v>-0.000540801</v>
@@ -3253,25 +3253,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I8" t="s">
         <v>189</v>
@@ -3531,25 +3531,25 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I9" t="s">
         <v>190</v>
@@ -3809,25 +3809,25 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I10" t="s">
         <v>191</v>
@@ -4087,25 +4087,25 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I11" t="s">
         <v>192</v>
@@ -4365,25 +4365,25 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I12" t="s">
         <v>193</v>
@@ -4643,25 +4643,25 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H13" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I13" t="s">
         <v>194</v>
@@ -4921,25 +4921,25 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I14" t="s">
         <v>195</v>
@@ -5199,28 +5199,28 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J15">
         <v>0.000327551</v>
@@ -5477,25 +5477,25 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I16" t="s">
         <v>196</v>
@@ -5755,25 +5755,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H17" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I17" t="s">
         <v>197</v>
@@ -6033,25 +6033,25 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H18" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I18" t="s">
         <v>198</v>
@@ -6311,25 +6311,25 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I19" t="s">
         <v>199</v>
@@ -6589,25 +6589,25 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H20" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I20" t="s">
         <v>200</v>
@@ -6867,25 +6867,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I21" t="s">
         <v>201</v>
@@ -7145,25 +7145,25 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I22" t="s">
         <v>202</v>
@@ -7423,25 +7423,25 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I23" t="s">
         <v>203</v>
@@ -7701,25 +7701,25 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I24" t="s">
         <v>204</v>
@@ -7979,25 +7979,25 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H25" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I25" t="s">
         <v>205</v>
@@ -8257,25 +8257,25 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I26" t="s">
         <v>206</v>
@@ -8535,25 +8535,25 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I27" t="s">
         <v>207</v>
@@ -8813,25 +8813,25 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H28" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I28" t="s">
         <v>208</v>
@@ -9091,25 +9091,25 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H29" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I29" t="s">
         <v>209</v>
@@ -9369,25 +9369,25 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H30" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I30" t="s">
         <v>210</v>
@@ -9647,25 +9647,25 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H31" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I31" t="s">
         <v>211</v>
@@ -9925,25 +9925,25 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H32" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I32" t="s">
         <v>212</v>
@@ -10203,25 +10203,25 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H33" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I33" t="s">
         <v>213</v>
@@ -10481,25 +10481,25 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H34" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I34" t="s">
         <v>214</v>
@@ -10765,25 +10765,25 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H35" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I35" t="s">
         <v>215</v>
@@ -11049,25 +11049,25 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H36" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I36" t="s">
         <v>216</v>
@@ -11333,28 +11333,28 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J37">
         <v>0.001640077</v>
@@ -11617,25 +11617,25 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I38" t="s">
         <v>217</v>
@@ -11901,25 +11901,25 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H39" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I39" t="s">
         <v>218</v>
@@ -12185,25 +12185,25 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H40" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I40" t="s">
         <v>219</v>
@@ -12469,25 +12469,25 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H41" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I41" t="s">
         <v>220</v>
@@ -12753,25 +12753,25 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H42" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I42" t="s">
         <v>221</v>
@@ -13037,25 +13037,25 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H43" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I43" t="s">
         <v>222</v>
@@ -13321,25 +13321,25 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H44" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I44" t="s">
         <v>223</v>
@@ -13605,25 +13605,25 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H45" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I45" t="s">
         <v>224</v>
@@ -13889,25 +13889,25 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H46" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I46" t="s">
         <v>225</v>
@@ -14173,25 +14173,25 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I47" t="s">
         <v>226</v>
@@ -14457,25 +14457,25 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I48" t="s">
         <v>227</v>
@@ -14741,25 +14741,25 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H49" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I49" t="s">
         <v>228</v>
@@ -15025,25 +15025,25 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H50" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I50" t="s">
         <v>229</v>
@@ -15309,25 +15309,25 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H51" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I51" t="s">
         <v>230</v>
@@ -15593,25 +15593,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H52" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I52" t="s">
         <v>231</v>
@@ -15877,25 +15877,25 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I53" t="s">
         <v>232</v>
@@ -16161,28 +16161,28 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H54" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I54" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J54">
         <v>0.0008229381467956</v>
@@ -16445,25 +16445,25 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F55" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G55" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I55" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J55">
         <v>0.0022239398231451</v>
@@ -16726,22 +16726,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E56" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F56" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I56" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J56">
         <v>0.0018211096217568</v>
@@ -17004,19 +17004,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C57" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D57" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I57" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J57">
         <v>0.0012556275124289</v>
@@ -17279,19 +17279,19 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C58" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D58" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E58" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I58" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J58">
         <v>0.0019905125443684</v>
@@ -17554,19 +17554,19 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C59" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D59" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E59" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I59" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J59">
         <v>0.0005221982670147</v>
@@ -17829,19 +17829,19 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C60" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D60" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E60" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I60" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J60">
         <v>0.0018105477499388</v>
@@ -18104,19 +18104,19 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C61" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D61" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E61" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I61" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J61">
         <v>0.0006776201968474</v>
@@ -18379,19 +18379,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C62" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D62" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E62" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I62" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J62">
         <v>0.0025014106780221</v>
@@ -18654,19 +18654,19 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C63" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D63" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E63" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I63" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J63">
         <v>0.0007538484415952</v>
@@ -18929,19 +18929,19 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C64" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D64" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I64" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J64">
         <v>0.0012416962587069</v>
@@ -19204,19 +19204,19 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E65" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I65" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J65">
         <v>0.0015984483099258</v>
@@ -19479,16 +19479,16 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D66" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I66" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J66">
         <v>0.0024755430193983</v>
@@ -19760,16 +19760,16 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C67" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D67" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I67" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J67">
         <v>0.0012089442610578</v>
@@ -20041,16 +20041,16 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C68" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J68">
         <v>0.0023849978802701</v>
@@ -20322,16 +20322,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D69" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I69" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J69">
         <v>0.0020508834761068</v>
@@ -20603,13 +20603,13 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J70">
         <v>0.004410416036765</v>
@@ -20881,10 +20881,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I71" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J71">
         <v>0.0006414105255352</v>
@@ -21421,6 +21421,278 @@
       </c>
       <c r="CT72">
         <v>-0.8267377140365109</v>
+      </c>
+    </row>
+    <row r="73" spans="1:98">
+      <c r="A73" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="I73" t="s">
+        <v>98</v>
+      </c>
+      <c r="J73">
+        <v>0.0008003654809294325</v>
+      </c>
+      <c r="K73">
+        <v>0.0004001827404647162</v>
+      </c>
+      <c r="L73">
+        <v>0.0009080051794412292</v>
+      </c>
+      <c r="M73">
+        <v>0.0009080051794412292</v>
+      </c>
+      <c r="N73">
+        <v>0.001403506335296334</v>
+      </c>
+      <c r="O73">
+        <v>0.000701753167648167</v>
+      </c>
+      <c r="P73">
+        <v>0.0006834692895637984</v>
+      </c>
+      <c r="Q73">
+        <v>0.0006834692895637984</v>
+      </c>
+      <c r="R73">
+        <v>9.338912133891213</v>
+      </c>
+      <c r="S73">
+        <v>8.187360756398414</v>
+      </c>
+      <c r="T73">
+        <v>0.4696363824789076</v>
+      </c>
+      <c r="U73">
+        <v>0.6211499875764427</v>
+      </c>
+      <c r="V73">
+        <v>0.02438056944607176</v>
+      </c>
+      <c r="W73">
+        <v>0.06968726177731056</v>
+      </c>
+      <c r="X73">
+        <v>0.06035648903810926</v>
+      </c>
+      <c r="Y73">
+        <v>0.213957138080325</v>
+      </c>
+      <c r="Z73">
+        <v>0.9995852632927549</v>
+      </c>
+      <c r="AA73">
+        <v>0.9468551850535822</v>
+      </c>
+      <c r="AB73">
+        <v>0.7973403754763994</v>
+      </c>
+      <c r="AC73">
+        <v>0.9992200806611152</v>
+      </c>
+      <c r="AD73">
+        <v>0.9255257257600396</v>
+      </c>
+      <c r="AE73">
+        <v>0.786115888961936</v>
+      </c>
+      <c r="AF73">
+        <v>0.002768659761224431</v>
+      </c>
+      <c r="AG73">
+        <v>0.008671749707596748</v>
+      </c>
+      <c r="AH73">
+        <v>0.9995852632927549</v>
+      </c>
+      <c r="AI73">
+        <v>0.9992200806611152</v>
+      </c>
+      <c r="AJ73">
+        <v>0.002768659761224431</v>
+      </c>
+      <c r="AK73">
+        <v>0.008671749707596748</v>
+      </c>
+      <c r="AL73" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM73">
+        <v>0.008922434565822774</v>
+      </c>
+      <c r="AN73">
+        <v>0.01630495131483891</v>
+      </c>
+      <c r="AO73">
+        <v>-417.86963052</v>
+      </c>
+      <c r="AP73">
+        <v>-528.657206662</v>
+      </c>
+      <c r="AQ73">
+        <v>18468.25306499995</v>
+      </c>
+      <c r="AR73">
+        <v>20055.83210333804</v>
+      </c>
+      <c r="AS73">
+        <v>18468.25306499995</v>
+      </c>
+      <c r="AT73">
+        <v>20054.23000333804</v>
+      </c>
+      <c r="AU73">
+        <v>0.8468253064999947</v>
+      </c>
+      <c r="AV73">
+        <v>1.005583210333804</v>
+      </c>
+      <c r="AW73">
+        <v>2.560125698324022</v>
+      </c>
+      <c r="AX73">
+        <v>2.925734161754554</v>
+      </c>
+      <c r="AY73">
+        <v>107.7666666666667</v>
+      </c>
+      <c r="AZ73">
+        <v>99.78333333333333</v>
+      </c>
+      <c r="BA73">
+        <v>0.004034017084883299</v>
+      </c>
+      <c r="BB73">
+        <v>0</v>
+      </c>
+      <c r="BC73">
+        <v>-35.99675641842089</v>
+      </c>
+      <c r="BD73">
+        <v>0</v>
+      </c>
+      <c r="BE73">
+        <v>3188</v>
+      </c>
+      <c r="BF73">
+        <v>2983</v>
+      </c>
+      <c r="BG73">
+        <v>766.7916666666666</v>
+      </c>
+      <c r="BH73">
+        <v>3973</v>
+      </c>
+      <c r="BI73">
+        <v>3295</v>
+      </c>
+      <c r="BJ73">
+        <v>7161</v>
+      </c>
+      <c r="BK73">
+        <v>6278</v>
+      </c>
+      <c r="BL73">
+        <v>3027</v>
+      </c>
+      <c r="BM73">
+        <v>2635</v>
+      </c>
+      <c r="BN73">
+        <v>3185</v>
+      </c>
+      <c r="BO73">
+        <v>2983</v>
+      </c>
+      <c r="BP73">
+        <v>946</v>
+      </c>
+      <c r="BQ73">
+        <v>660</v>
+      </c>
+      <c r="BR73">
+        <v>3</v>
+      </c>
+      <c r="BS73">
+        <v>0</v>
+      </c>
+      <c r="BT73">
+        <v>0</v>
+      </c>
+      <c r="BU73">
+        <v>0</v>
+      </c>
+      <c r="BV73">
+        <v>8469.436529480003</v>
+      </c>
+      <c r="BW73">
+        <v>10055.832103338</v>
+      </c>
+      <c r="BX73">
+        <v>0.05025982571559835</v>
+      </c>
+      <c r="BY73">
+        <v>0.07055195206044632</v>
+      </c>
+      <c r="BZ73">
+        <v>0.09258390607789721</v>
+      </c>
+      <c r="CA73">
+        <v>0.1761685228835807</v>
+      </c>
+      <c r="CB73">
+        <v>0.01285972929328954</v>
+      </c>
+      <c r="CC73">
+        <v>0.01389522542302284</v>
+      </c>
+      <c r="CD73">
+        <v>0.0111093109771639</v>
+      </c>
+      <c r="CE73">
+        <v>0.01376759628427725</v>
+      </c>
+      <c r="CF73">
+        <v>8887.306160000002</v>
+      </c>
+      <c r="CG73">
+        <v>10584.48931</v>
+      </c>
+      <c r="CH73">
+        <v>8923.302916418423</v>
+      </c>
+      <c r="CI73">
+        <v>10584.48931</v>
+      </c>
+      <c r="CJ73">
+        <v>0.1335940871248117</v>
+      </c>
+      <c r="CK73">
+        <v>0.08571463977379885</v>
+      </c>
+      <c r="CL73">
+        <v>10000</v>
+      </c>
+      <c r="CN73">
+        <v>0.0003803520973701369</v>
+      </c>
+      <c r="CO73">
+        <v>0.009726146489893502</v>
+      </c>
+      <c r="CP73">
+        <v>2617479.238699115</v>
+      </c>
+      <c r="CQ73">
+        <v>4050354.030474017</v>
+      </c>
+      <c r="CR73" s="2">
+        <v>45402.82553006194</v>
+      </c>
+      <c r="CS73">
+        <v>-0.9011542748767547</v>
+      </c>
+      <c r="CT73">
+        <v>-0.7124209679360802</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update LTCUSDT.json at 2024-04-21_07-26-23 bestfile_scores 0.0005842704100873035 bestfile_sharp 0.04831082400635559
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="303">
   <si>
     <t>Unnamed: 0.6</t>
   </si>
@@ -313,6 +313,9 @@
     <t>GMTUSDT</t>
   </si>
   <si>
+    <t>SUSHIUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -581,9 +584,6 @@
   </si>
   <si>
     <t>RNDRUSDT</t>
-  </si>
-  <si>
-    <t>SUSHIUSDT</t>
   </si>
   <si>
     <t>LTCUSDT</t>
@@ -1284,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CT73"/>
+  <dimension ref="A1:CT74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:98">
@@ -1585,28 +1585,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J2">
         <v>0.0009987329999999999</v>
@@ -1863,28 +1863,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J3">
         <v>0.001058605</v>
@@ -2141,28 +2141,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J4">
         <v>0.000882894</v>
@@ -2419,28 +2419,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J5">
         <v>0.001186265</v>
@@ -2697,25 +2697,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I6" t="s">
         <v>97</v>
@@ -2975,25 +2975,25 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I7" t="s">
         <v>98</v>
@@ -3253,28 +3253,28 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I8" t="s">
-        <v>189</v>
+        <v>99</v>
       </c>
       <c r="J8">
         <v>0.001278948</v>
@@ -3531,25 +3531,25 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I9" t="s">
         <v>190</v>
@@ -3809,25 +3809,25 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
         <v>191</v>
@@ -4087,25 +4087,25 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I11" t="s">
         <v>192</v>
@@ -4365,25 +4365,25 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I12" t="s">
         <v>193</v>
@@ -4643,25 +4643,25 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I13" t="s">
         <v>194</v>
@@ -4921,25 +4921,25 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I14" t="s">
         <v>195</v>
@@ -5199,28 +5199,28 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J15">
         <v>0.000327551</v>
@@ -5477,25 +5477,25 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
         <v>196</v>
@@ -5755,25 +5755,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
         <v>197</v>
@@ -6033,25 +6033,25 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I18" t="s">
         <v>198</v>
@@ -6311,25 +6311,25 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s">
         <v>199</v>
@@ -6589,25 +6589,25 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I20" t="s">
         <v>200</v>
@@ -6867,25 +6867,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I21" t="s">
         <v>201</v>
@@ -7145,25 +7145,25 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I22" t="s">
         <v>202</v>
@@ -7423,25 +7423,25 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I23" t="s">
         <v>203</v>
@@ -7701,25 +7701,25 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I24" t="s">
         <v>204</v>
@@ -7979,25 +7979,25 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I25" t="s">
         <v>205</v>
@@ -8257,25 +8257,25 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I26" t="s">
         <v>206</v>
@@ -8535,25 +8535,25 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I27" t="s">
         <v>207</v>
@@ -8813,25 +8813,25 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I28" t="s">
         <v>208</v>
@@ -9091,25 +9091,25 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I29" t="s">
         <v>209</v>
@@ -9369,25 +9369,25 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I30" t="s">
         <v>210</v>
@@ -9647,25 +9647,25 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I31" t="s">
         <v>211</v>
@@ -9925,25 +9925,25 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I32" t="s">
         <v>212</v>
@@ -10203,25 +10203,25 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I33" t="s">
         <v>213</v>
@@ -10481,25 +10481,25 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I34" t="s">
         <v>214</v>
@@ -10765,25 +10765,25 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I35" t="s">
         <v>215</v>
@@ -11049,25 +11049,25 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I36" t="s">
         <v>216</v>
@@ -11333,28 +11333,28 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J37">
         <v>0.001640077</v>
@@ -11617,25 +11617,25 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I38" t="s">
         <v>217</v>
@@ -11901,25 +11901,25 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I39" t="s">
         <v>218</v>
@@ -12185,25 +12185,25 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I40" t="s">
         <v>219</v>
@@ -12469,25 +12469,25 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I41" t="s">
         <v>220</v>
@@ -12753,25 +12753,25 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I42" t="s">
         <v>221</v>
@@ -13037,25 +13037,25 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I43" t="s">
         <v>222</v>
@@ -13321,25 +13321,25 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I44" t="s">
         <v>223</v>
@@ -13605,25 +13605,25 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I45" t="s">
         <v>224</v>
@@ -13889,25 +13889,25 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I46" t="s">
         <v>225</v>
@@ -14173,25 +14173,25 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
         <v>226</v>
@@ -14457,25 +14457,25 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I48" t="s">
         <v>227</v>
@@ -14741,25 +14741,25 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I49" t="s">
         <v>228</v>
@@ -15025,25 +15025,25 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I50" t="s">
         <v>229</v>
@@ -15309,25 +15309,25 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I51" t="s">
         <v>230</v>
@@ -15593,25 +15593,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I52" t="s">
         <v>231</v>
@@ -15877,25 +15877,25 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I53" t="s">
         <v>232</v>
@@ -16161,28 +16161,28 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H54" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I54" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J54">
         <v>0.0008229381467956</v>
@@ -16445,25 +16445,25 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G55" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I55" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J55">
         <v>0.0022239398231451</v>
@@ -16726,22 +16726,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F56" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I56" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J56">
         <v>0.0018211096217568</v>
@@ -17004,19 +17004,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E57" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I57" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J57">
         <v>0.0012556275124289</v>
@@ -17279,19 +17279,19 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E58" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I58" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J58">
         <v>0.0019905125443684</v>
@@ -17554,19 +17554,19 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E59" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I59" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J59">
         <v>0.0005221982670147</v>
@@ -17829,19 +17829,19 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E60" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I60" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J60">
         <v>0.0018105477499388</v>
@@ -18104,19 +18104,19 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E61" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I61" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J61">
         <v>0.0006776201968474</v>
@@ -18379,19 +18379,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E62" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I62" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J62">
         <v>0.0025014106780221</v>
@@ -18654,19 +18654,19 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E63" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I63" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J63">
         <v>0.0007538484415952</v>
@@ -18929,19 +18929,19 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E64" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I64" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J64">
         <v>0.0012416962587069</v>
@@ -19204,19 +19204,19 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I65" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J65">
         <v>0.0015984483099258</v>
@@ -19479,16 +19479,16 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D66" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I66" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J66">
         <v>0.0024755430193983</v>
@@ -19760,16 +19760,16 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D67" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I67" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J67">
         <v>0.0012089442610578</v>
@@ -20041,16 +20041,16 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D68" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I68" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J68">
         <v>0.0023849978802701</v>
@@ -20322,16 +20322,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D69" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I69" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J69">
         <v>0.0020508834761068</v>
@@ -20603,13 +20603,13 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I70" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J70">
         <v>0.004410416036765</v>
@@ -20881,10 +20881,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="I71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J71">
         <v>0.0006414105255352</v>
@@ -21693,6 +21693,278 @@
       </c>
       <c r="CT73">
         <v>-0.7124209679360802</v>
+      </c>
+    </row>
+    <row r="74" spans="1:98">
+      <c r="A74" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="I74" t="s">
+        <v>99</v>
+      </c>
+      <c r="J74">
+        <v>0.001155136088498043</v>
+      </c>
+      <c r="K74">
+        <v>0.0005775680442490216</v>
+      </c>
+      <c r="L74">
+        <v>0.0001073640905211448</v>
+      </c>
+      <c r="M74">
+        <v>0.0001073640905211448</v>
+      </c>
+      <c r="N74">
+        <v>0.002543767194464075</v>
+      </c>
+      <c r="O74">
+        <v>0.001271883597232037</v>
+      </c>
+      <c r="P74">
+        <v>7.478055832546015E-05</v>
+      </c>
+      <c r="Q74">
+        <v>7.478055832546015E-05</v>
+      </c>
+      <c r="R74">
+        <v>15.86450094525252</v>
+      </c>
+      <c r="S74">
+        <v>4.938153478143447</v>
+      </c>
+      <c r="T74">
+        <v>0.4242291987797702</v>
+      </c>
+      <c r="U74">
+        <v>1</v>
+      </c>
+      <c r="V74">
+        <v>0.02425287323856219</v>
+      </c>
+      <c r="W74">
+        <v>0.0597509545587419</v>
+      </c>
+      <c r="X74">
+        <v>0.1120946896073946</v>
+      </c>
+      <c r="Y74">
+        <v>0.154588362501109</v>
+      </c>
+      <c r="Z74">
+        <v>0.9995310719108732</v>
+      </c>
+      <c r="AA74">
+        <v>0.9559570094699298</v>
+      </c>
+      <c r="AB74">
+        <v>0.8736280250465894</v>
+      </c>
+      <c r="AC74">
+        <v>0.9988786592651285</v>
+      </c>
+      <c r="AD74">
+        <v>0.7622309189210518</v>
+      </c>
+      <c r="AE74">
+        <v>0.8455253816406558</v>
+      </c>
+      <c r="AF74">
+        <v>0.002165243474043214</v>
+      </c>
+      <c r="AG74">
+        <v>0.006128769940808926</v>
+      </c>
+      <c r="AH74">
+        <v>0.9995310719108732</v>
+      </c>
+      <c r="AI74">
+        <v>0.9988786592651285</v>
+      </c>
+      <c r="AJ74">
+        <v>0.002165243474043214</v>
+      </c>
+      <c r="AK74">
+        <v>0.006128769940808926</v>
+      </c>
+      <c r="AL74" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM74">
+        <v>0.01004442064624554</v>
+      </c>
+      <c r="AN74">
+        <v>0.01443848204083306</v>
+      </c>
+      <c r="AO74">
+        <v>-1121.2526495</v>
+      </c>
+      <c r="AP74">
+        <v>-71.05295434000001</v>
+      </c>
+      <c r="AQ74">
+        <v>34791.18245049971</v>
+      </c>
+      <c r="AR74">
+        <v>11229.31324566018</v>
+      </c>
+      <c r="AS74">
+        <v>34783.33845049971</v>
+      </c>
+      <c r="AT74">
+        <v>11228.44094566018</v>
+      </c>
+      <c r="AU74">
+        <v>2.479118245049971</v>
+      </c>
+      <c r="AV74">
+        <v>0.1229313245660175</v>
+      </c>
+      <c r="AW74">
+        <v>1.511473655537396</v>
+      </c>
+      <c r="AX74">
+        <v>4.853835333833459</v>
+      </c>
+      <c r="AY74">
+        <v>116.05</v>
+      </c>
+      <c r="AZ74">
+        <v>127.5666666666667</v>
+      </c>
+      <c r="BA74">
+        <v>0.05467713029987305</v>
+      </c>
+      <c r="BB74">
+        <v>0.1291951059170759</v>
+      </c>
+      <c r="BC74">
+        <v>-1498.765803475317</v>
+      </c>
+      <c r="BD74">
+        <v>-192.9260504638221</v>
+      </c>
+      <c r="BE74">
+        <v>8097</v>
+      </c>
+      <c r="BF74">
+        <v>2373</v>
+      </c>
+      <c r="BG74">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BH74">
+        <v>9036</v>
+      </c>
+      <c r="BI74">
+        <v>2960</v>
+      </c>
+      <c r="BJ74">
+        <v>17133</v>
+      </c>
+      <c r="BK74">
+        <v>5333</v>
+      </c>
+      <c r="BL74">
+        <v>7938</v>
+      </c>
+      <c r="BM74">
+        <v>2371</v>
+      </c>
+      <c r="BN74">
+        <v>8094</v>
+      </c>
+      <c r="BO74">
+        <v>2371</v>
+      </c>
+      <c r="BP74">
+        <v>1098</v>
+      </c>
+      <c r="BQ74">
+        <v>589</v>
+      </c>
+      <c r="BR74">
+        <v>3</v>
+      </c>
+      <c r="BS74">
+        <v>2</v>
+      </c>
+      <c r="BT74">
+        <v>0</v>
+      </c>
+      <c r="BU74">
+        <v>0</v>
+      </c>
+      <c r="BV74">
+        <v>24791.18245049998</v>
+      </c>
+      <c r="BW74">
+        <v>1229.31324566</v>
+      </c>
+      <c r="BX74">
+        <v>0.06311245099897179</v>
+      </c>
+      <c r="BY74">
+        <v>0.1660018047011206</v>
+      </c>
+      <c r="BZ74">
+        <v>0.2173823585641193</v>
+      </c>
+      <c r="CA74">
+        <v>0.2573331724056189</v>
+      </c>
+      <c r="CB74">
+        <v>0.01623894846040772</v>
+      </c>
+      <c r="CC74">
+        <v>0.02969657001740581</v>
+      </c>
+      <c r="CD74">
+        <v>0.01327787179992364</v>
+      </c>
+      <c r="CE74">
+        <v>0.02711724092887033</v>
+      </c>
+      <c r="CF74">
+        <v>25912.43509999998</v>
+      </c>
+      <c r="CG74">
+        <v>1300.3662</v>
+      </c>
+      <c r="CH74">
+        <v>27411.2009034753</v>
+      </c>
+      <c r="CI74">
+        <v>1493.292250463822</v>
+      </c>
+      <c r="CJ74">
+        <v>0.1019064101175263</v>
+      </c>
+      <c r="CK74">
+        <v>0.02894417017774548</v>
+      </c>
+      <c r="CL74">
+        <v>10000</v>
+      </c>
+      <c r="CN74">
+        <v>7.716049382716049E-05</v>
+      </c>
+      <c r="CO74">
+        <v>0</v>
+      </c>
+      <c r="CP74">
+        <v>5152305.117252609</v>
+      </c>
+      <c r="CQ74">
+        <v>284228.7150822567</v>
+      </c>
+      <c r="CR74" s="2">
+        <v>45403.0739103215</v>
+      </c>
+      <c r="CS74">
+        <v>-0.9022640234515125</v>
+      </c>
+      <c r="CT74">
+        <v>-0.9353148225259252</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GALUSDT.json at 2024-04-21_11-12-19 bestfile_scores 0.0018980673168523087 bestfile_sharp 0.0891982496445387
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="303">
   <si>
     <t>Unnamed: 0.6</t>
   </si>
@@ -316,6 +316,9 @@
     <t>SUSHIUSDT</t>
   </si>
   <si>
+    <t>LTCUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -584,9 +587,6 @@
   </si>
   <si>
     <t>RNDRUSDT</t>
-  </si>
-  <si>
-    <t>LTCUSDT</t>
   </si>
   <si>
     <t>GALUSDT</t>
@@ -1284,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CT74"/>
+  <dimension ref="A1:CT75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:98">
@@ -1585,28 +1585,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J2">
         <v>0.0009987329999999999</v>
@@ -1863,28 +1863,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J3">
         <v>0.001058605</v>
@@ -2141,28 +2141,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J4">
         <v>0.000882894</v>
@@ -2419,28 +2419,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J5">
         <v>0.001186265</v>
@@ -2697,25 +2697,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I6" t="s">
         <v>97</v>
@@ -2975,25 +2975,25 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I7" t="s">
         <v>98</v>
@@ -3253,25 +3253,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I8" t="s">
         <v>99</v>
@@ -3531,28 +3531,28 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I9" t="s">
-        <v>190</v>
+        <v>100</v>
       </c>
       <c r="J9">
         <v>0.000266144</v>
@@ -3809,25 +3809,25 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I10" t="s">
         <v>191</v>
@@ -4087,25 +4087,25 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I11" t="s">
         <v>192</v>
@@ -4365,25 +4365,25 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I12" t="s">
         <v>193</v>
@@ -4643,25 +4643,25 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I13" t="s">
         <v>194</v>
@@ -4921,25 +4921,25 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I14" t="s">
         <v>195</v>
@@ -5199,28 +5199,28 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J15">
         <v>0.000327551</v>
@@ -5477,25 +5477,25 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I16" t="s">
         <v>196</v>
@@ -5755,25 +5755,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H17" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I17" t="s">
         <v>197</v>
@@ -6033,25 +6033,25 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H18" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I18" t="s">
         <v>198</v>
@@ -6311,25 +6311,25 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I19" t="s">
         <v>199</v>
@@ -6589,25 +6589,25 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I20" t="s">
         <v>200</v>
@@ -6867,25 +6867,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I21" t="s">
         <v>201</v>
@@ -7145,25 +7145,25 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I22" t="s">
         <v>202</v>
@@ -7423,25 +7423,25 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I23" t="s">
         <v>203</v>
@@ -7701,25 +7701,25 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I24" t="s">
         <v>204</v>
@@ -7979,25 +7979,25 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H25" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I25" t="s">
         <v>205</v>
@@ -8257,25 +8257,25 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H26" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I26" t="s">
         <v>206</v>
@@ -8535,25 +8535,25 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H27" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I27" t="s">
         <v>207</v>
@@ -8813,25 +8813,25 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H28" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I28" t="s">
         <v>208</v>
@@ -9091,25 +9091,25 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H29" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I29" t="s">
         <v>209</v>
@@ -9369,25 +9369,25 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H30" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I30" t="s">
         <v>210</v>
@@ -9647,25 +9647,25 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H31" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I31" t="s">
         <v>211</v>
@@ -9925,25 +9925,25 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H32" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I32" t="s">
         <v>212</v>
@@ -10203,25 +10203,25 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I33" t="s">
         <v>213</v>
@@ -10481,25 +10481,25 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H34" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I34" t="s">
         <v>214</v>
@@ -10765,25 +10765,25 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H35" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I35" t="s">
         <v>215</v>
@@ -11049,25 +11049,25 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H36" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I36" t="s">
         <v>216</v>
@@ -11333,28 +11333,28 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H37" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J37">
         <v>0.001640077</v>
@@ -11617,25 +11617,25 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I38" t="s">
         <v>217</v>
@@ -11901,25 +11901,25 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H39" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I39" t="s">
         <v>218</v>
@@ -12185,25 +12185,25 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I40" t="s">
         <v>219</v>
@@ -12469,25 +12469,25 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I41" t="s">
         <v>220</v>
@@ -12753,25 +12753,25 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H42" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I42" t="s">
         <v>221</v>
@@ -13037,25 +13037,25 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H43" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I43" t="s">
         <v>222</v>
@@ -13321,25 +13321,25 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H44" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I44" t="s">
         <v>223</v>
@@ -13605,25 +13605,25 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H45" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I45" t="s">
         <v>224</v>
@@ -13889,25 +13889,25 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H46" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I46" t="s">
         <v>225</v>
@@ -14173,25 +14173,25 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I47" t="s">
         <v>226</v>
@@ -14457,25 +14457,25 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I48" t="s">
         <v>227</v>
@@ -14741,25 +14741,25 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H49" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I49" t="s">
         <v>228</v>
@@ -15025,25 +15025,25 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H50" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I50" t="s">
         <v>229</v>
@@ -15309,25 +15309,25 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H51" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I51" t="s">
         <v>230</v>
@@ -15593,25 +15593,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H52" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I52" t="s">
         <v>231</v>
@@ -15877,25 +15877,25 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I53" t="s">
         <v>232</v>
@@ -16161,28 +16161,28 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G54" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H54" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I54" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J54">
         <v>0.0008229381467956</v>
@@ -16445,25 +16445,25 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F55" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G55" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I55" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J55">
         <v>0.0022239398231451</v>
@@ -16726,22 +16726,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E56" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F56" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I56" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J56">
         <v>0.0018211096217568</v>
@@ -17004,19 +17004,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C57" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D57" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E57" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I57" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J57">
         <v>0.0012556275124289</v>
@@ -17279,19 +17279,19 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C58" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D58" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E58" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I58" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J58">
         <v>0.0019905125443684</v>
@@ -17554,19 +17554,19 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C59" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D59" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E59" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I59" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J59">
         <v>0.0005221982670147</v>
@@ -17829,19 +17829,19 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C60" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D60" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E60" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I60" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J60">
         <v>0.0018105477499388</v>
@@ -18104,19 +18104,19 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C61" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D61" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E61" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I61" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J61">
         <v>0.0006776201968474</v>
@@ -18379,19 +18379,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D62" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E62" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I62" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J62">
         <v>0.0025014106780221</v>
@@ -18654,19 +18654,19 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E63" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I63" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J63">
         <v>0.0007538484415952</v>
@@ -18929,19 +18929,19 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E64" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I64" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J64">
         <v>0.0012416962587069</v>
@@ -19204,19 +19204,19 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D65" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E65" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="I65" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J65">
         <v>0.0015984483099258</v>
@@ -19479,16 +19479,16 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C66" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D66" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I66" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J66">
         <v>0.0024755430193983</v>
@@ -19760,16 +19760,16 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D67" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I67" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J67">
         <v>0.0012089442610578</v>
@@ -20041,16 +20041,16 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C68" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D68" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I68" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J68">
         <v>0.0023849978802701</v>
@@ -20322,16 +20322,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C69" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D69" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I69" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J69">
         <v>0.0020508834761068</v>
@@ -20603,13 +20603,13 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I70" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J70">
         <v>0.004410416036765</v>
@@ -20881,10 +20881,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="I71" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J71">
         <v>0.0006414105255352</v>
@@ -21965,6 +21965,278 @@
       </c>
       <c r="CT74">
         <v>-0.9353148225259252</v>
+      </c>
+    </row>
+    <row r="75" spans="1:98">
+      <c r="A75" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I75" t="s">
+        <v>100</v>
+      </c>
+      <c r="J75">
+        <v>0.001355651330368079</v>
+      </c>
+      <c r="K75">
+        <v>0.0006778256651840397</v>
+      </c>
+      <c r="L75">
+        <v>0.0006208133408187599</v>
+      </c>
+      <c r="M75">
+        <v>0.0006208133408187599</v>
+      </c>
+      <c r="N75">
+        <v>0.001023720234109393</v>
+      </c>
+      <c r="O75">
+        <v>0.0005118601170546966</v>
+      </c>
+      <c r="P75">
+        <v>0.0005265825172917182</v>
+      </c>
+      <c r="Q75">
+        <v>0.0005265825172917182</v>
+      </c>
+      <c r="R75">
+        <v>11.26271480980884</v>
+      </c>
+      <c r="S75">
+        <v>28.82317049623479</v>
+      </c>
+      <c r="T75">
+        <v>0.3831050339835673</v>
+      </c>
+      <c r="U75">
+        <v>0.6757380418240518</v>
+      </c>
+      <c r="V75">
+        <v>0.01869289994651518</v>
+      </c>
+      <c r="W75">
+        <v>0.07377767183841726</v>
+      </c>
+      <c r="X75">
+        <v>0.1223610723643727</v>
+      </c>
+      <c r="Y75">
+        <v>0.1358322110405941</v>
+      </c>
+      <c r="Z75">
+        <v>0.9996653263959692</v>
+      </c>
+      <c r="AA75">
+        <v>0.9084219597032094</v>
+      </c>
+      <c r="AB75">
+        <v>0.8852299119821746</v>
+      </c>
+      <c r="AC75">
+        <v>0.9979086379804013</v>
+      </c>
+      <c r="AD75">
+        <v>0.8779416373082003</v>
+      </c>
+      <c r="AE75">
+        <v>0.8652729566955598</v>
+      </c>
+      <c r="AF75">
+        <v>0.002536599412627556</v>
+      </c>
+      <c r="AG75">
+        <v>0.009112086818146913</v>
+      </c>
+      <c r="AH75">
+        <v>0.9996653263959692</v>
+      </c>
+      <c r="AI75">
+        <v>0.9979086379804013</v>
+      </c>
+      <c r="AJ75">
+        <v>0.002536599412627556</v>
+      </c>
+      <c r="AK75">
+        <v>0.009112086818146913</v>
+      </c>
+      <c r="AL75" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM75">
+        <v>0.01058859886288484</v>
+      </c>
+      <c r="AN75">
+        <v>0.06503152839823989</v>
+      </c>
+      <c r="AO75">
+        <v>-1611.136905998</v>
+      </c>
+      <c r="AP75">
+        <v>-1291.004818746</v>
+      </c>
+      <c r="AQ75">
+        <v>43132.89100400215</v>
+      </c>
+      <c r="AR75">
+        <v>19535.02457083993</v>
+      </c>
+      <c r="AS75">
+        <v>43129.76400400215</v>
+      </c>
+      <c r="AT75">
+        <v>19535.02457083993</v>
+      </c>
+      <c r="AU75">
+        <v>3.313289100400215</v>
+      </c>
+      <c r="AV75">
+        <v>0.9535024570839927</v>
+      </c>
+      <c r="AW75">
+        <v>2.129812361122541</v>
+      </c>
+      <c r="AX75">
+        <v>0.8319109481853066</v>
+      </c>
+      <c r="AY75">
+        <v>110.6833333333333</v>
+      </c>
+      <c r="AZ75">
+        <v>103.3666666666667</v>
+      </c>
+      <c r="BA75">
+        <v>0.0134996077893301</v>
+      </c>
+      <c r="BB75">
+        <v>0.009886799560081332</v>
+      </c>
+      <c r="BC75">
+        <v>-475.4491265385896</v>
+      </c>
+      <c r="BD75">
+        <v>-108.1111789337186</v>
+      </c>
+      <c r="BE75">
+        <v>5439</v>
+      </c>
+      <c r="BF75">
+        <v>14375</v>
+      </c>
+      <c r="BG75">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BH75">
+        <v>6713</v>
+      </c>
+      <c r="BI75">
+        <v>16724</v>
+      </c>
+      <c r="BJ75">
+        <v>12152</v>
+      </c>
+      <c r="BK75">
+        <v>31099</v>
+      </c>
+      <c r="BL75">
+        <v>5425</v>
+      </c>
+      <c r="BM75">
+        <v>12790</v>
+      </c>
+      <c r="BN75">
+        <v>5434</v>
+      </c>
+      <c r="BO75">
+        <v>14342</v>
+      </c>
+      <c r="BP75">
+        <v>1288</v>
+      </c>
+      <c r="BQ75">
+        <v>3934</v>
+      </c>
+      <c r="BR75">
+        <v>5</v>
+      </c>
+      <c r="BS75">
+        <v>33</v>
+      </c>
+      <c r="BT75">
+        <v>0</v>
+      </c>
+      <c r="BU75">
+        <v>0</v>
+      </c>
+      <c r="BV75">
+        <v>33132.89100400206</v>
+      </c>
+      <c r="BW75">
+        <v>9535.785461253998</v>
+      </c>
+      <c r="BX75">
+        <v>0.03772402923596588</v>
+      </c>
+      <c r="BY75">
+        <v>0.07445012696152829</v>
+      </c>
+      <c r="BZ75">
+        <v>0.07109716719701913</v>
+      </c>
+      <c r="CA75">
+        <v>0.1209471737664159</v>
+      </c>
+      <c r="CB75">
+        <v>0.009633862714460361</v>
+      </c>
+      <c r="CC75">
+        <v>0.009511778452406574</v>
+      </c>
+      <c r="CD75">
+        <v>0.00817255237240296</v>
+      </c>
+      <c r="CE75">
+        <v>0.01226775390154929</v>
+      </c>
+      <c r="CF75">
+        <v>34744.02791000006</v>
+      </c>
+      <c r="CG75">
+        <v>10826.79028</v>
+      </c>
+      <c r="CH75">
+        <v>35219.47703653864</v>
+      </c>
+      <c r="CI75">
+        <v>10934.90145893372</v>
+      </c>
+      <c r="CJ75">
+        <v>0.04831082400635559</v>
+      </c>
+      <c r="CK75">
+        <v>0.08379970580071765</v>
+      </c>
+      <c r="CL75">
+        <v>10000</v>
+      </c>
+      <c r="CN75">
+        <v>0.0006178560395427865</v>
+      </c>
+      <c r="CO75">
+        <v>0.02915508186592524</v>
+      </c>
+      <c r="CP75">
+        <v>5603280.617032995</v>
+      </c>
+      <c r="CQ75">
+        <v>9238253.926865038</v>
+      </c>
+      <c r="CR75" s="2">
+        <v>45403.31058760947</v>
+      </c>
+      <c r="CS75">
+        <v>-0.8442464713130005</v>
+      </c>
+      <c r="CT75">
+        <v>-0.8173346670588505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update XRPUSDT.json at 2024-04-22_04-54-13 bestfile_scores 0.0009103263782603566 bestfile_sharp 0.1849399280056099
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="303">
   <si>
     <t>Unnamed: 0.6</t>
   </si>
@@ -319,6 +319,12 @@
     <t>LTCUSDT</t>
   </si>
   <si>
+    <t>GALUSDT</t>
+  </si>
+  <si>
+    <t>XRPUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -589,13 +595,7 @@
     <t>RNDRUSDT</t>
   </si>
   <si>
-    <t>GALUSDT</t>
-  </si>
-  <si>
     <t>INJUSDT</t>
-  </si>
-  <si>
-    <t>XRPUSDT</t>
   </si>
   <si>
     <t>KAVAUSDT</t>
@@ -1284,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CT75"/>
+  <dimension ref="A1:CT77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:98">
@@ -1585,28 +1585,28 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J2">
         <v>0.0009987329999999999</v>
@@ -1863,28 +1863,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="J3">
         <v>0.001058605</v>
@@ -2141,28 +2141,28 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I4" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J4">
         <v>0.000882894</v>
@@ -2419,28 +2419,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="J5">
         <v>0.001186265</v>
@@ -2697,25 +2697,25 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I6" t="s">
         <v>97</v>
@@ -2975,25 +2975,25 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I7" t="s">
         <v>98</v>
@@ -3253,25 +3253,25 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I8" t="s">
         <v>99</v>
@@ -3531,25 +3531,25 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H9" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I9" t="s">
         <v>100</v>
@@ -3809,28 +3809,28 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H10" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="I10" t="s">
-        <v>191</v>
+        <v>101</v>
       </c>
       <c r="J10">
         <v>0.001013204</v>
@@ -4087,28 +4087,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I11" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J11">
         <v>0.001228309</v>
@@ -4365,28 +4365,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I12" t="s">
-        <v>193</v>
+        <v>102</v>
       </c>
       <c r="J12">
         <v>0.0009776030000000001</v>
@@ -4643,25 +4643,25 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H13" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="I13" t="s">
         <v>194</v>
@@ -4921,25 +4921,25 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="G14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="I14" t="s">
         <v>195</v>
@@ -5199,28 +5199,28 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="I15" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J15">
         <v>0.000327551</v>
@@ -5477,25 +5477,25 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I16" t="s">
         <v>196</v>
@@ -5755,25 +5755,25 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H17" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I17" t="s">
         <v>197</v>
@@ -6033,25 +6033,25 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H18" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I18" t="s">
         <v>198</v>
@@ -6311,25 +6311,25 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H19" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I19" t="s">
         <v>199</v>
@@ -6589,25 +6589,25 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="E20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I20" t="s">
         <v>200</v>
@@ -6867,25 +6867,25 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I21" t="s">
         <v>201</v>
@@ -7145,25 +7145,25 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="I22" t="s">
         <v>202</v>
@@ -7423,25 +7423,25 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="I23" t="s">
         <v>203</v>
@@ -7701,25 +7701,25 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I24" t="s">
         <v>204</v>
@@ -7979,25 +7979,25 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H25" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I25" t="s">
         <v>205</v>
@@ -8257,25 +8257,25 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H26" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I26" t="s">
         <v>206</v>
@@ -8535,25 +8535,25 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H27" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I27" t="s">
         <v>207</v>
@@ -8813,25 +8813,25 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H28" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I28" t="s">
         <v>208</v>
@@ -9091,25 +9091,25 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H29" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I29" t="s">
         <v>209</v>
@@ -9369,25 +9369,25 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H30" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I30" t="s">
         <v>210</v>
@@ -9647,25 +9647,25 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H31" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="I31" t="s">
         <v>211</v>
@@ -9925,25 +9925,25 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I32" t="s">
         <v>212</v>
@@ -10203,25 +10203,25 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="I33" t="s">
         <v>213</v>
@@ -10481,25 +10481,25 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H34" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I34" t="s">
         <v>214</v>
@@ -10765,25 +10765,25 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H35" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I35" t="s">
         <v>215</v>
@@ -11049,25 +11049,25 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="I36" t="s">
         <v>216</v>
@@ -11333,28 +11333,28 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I37" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J37">
         <v>0.001640077</v>
@@ -11617,25 +11617,25 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I38" t="s">
         <v>217</v>
@@ -11901,25 +11901,25 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="E39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H39" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="I39" t="s">
         <v>218</v>
@@ -12185,25 +12185,25 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="E40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H40" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I40" t="s">
         <v>219</v>
@@ -12469,25 +12469,25 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="I41" t="s">
         <v>220</v>
@@ -12753,25 +12753,25 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H42" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I42" t="s">
         <v>221</v>
@@ -13037,25 +13037,25 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H43" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I43" t="s">
         <v>222</v>
@@ -13321,25 +13321,25 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="I44" t="s">
         <v>223</v>
@@ -13605,25 +13605,25 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I45" t="s">
         <v>224</v>
@@ -13889,25 +13889,25 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="E46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H46" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I46" t="s">
         <v>225</v>
@@ -14173,25 +14173,25 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H47" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I47" t="s">
         <v>226</v>
@@ -14457,25 +14457,25 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H48" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="I48" t="s">
         <v>227</v>
@@ -14741,25 +14741,25 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H49" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I49" t="s">
         <v>228</v>
@@ -15025,25 +15025,25 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="E50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H50" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I50" t="s">
         <v>229</v>
@@ -15309,25 +15309,25 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H51" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="I51" t="s">
         <v>230</v>
@@ -15593,25 +15593,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H52" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="I52" t="s">
         <v>231</v>
@@ -15877,25 +15877,25 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I53" t="s">
         <v>232</v>
@@ -16161,28 +16161,28 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H54" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I54" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="J54">
         <v>0.0008229381467956</v>
@@ -16445,25 +16445,25 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G55" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="I55" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="J55">
         <v>0.0022239398231451</v>
@@ -16726,22 +16726,22 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C56" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D56" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E56" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F56" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="I56" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="J56">
         <v>0.0018211096217568</v>
@@ -17004,19 +17004,19 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C57" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D57" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E57" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I57" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J57">
         <v>0.0012556275124289</v>
@@ -17279,19 +17279,19 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C58" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D58" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E58" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="I58" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J58">
         <v>0.0019905125443684</v>
@@ -17554,19 +17554,19 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C59" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D59" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E59" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I59" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="J59">
         <v>0.0005221982670147</v>
@@ -17829,19 +17829,19 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C60" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D60" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E60" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="I60" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="J60">
         <v>0.0018105477499388</v>
@@ -18104,19 +18104,19 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C61" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D61" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E61" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="I61" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="J61">
         <v>0.0006776201968474</v>
@@ -18379,19 +18379,19 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D62" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E62" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I62" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="J62">
         <v>0.0025014106780221</v>
@@ -18654,19 +18654,19 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C63" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D63" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E63" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="I63" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J63">
         <v>0.0007538484415952</v>
@@ -18929,19 +18929,19 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E64" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I64" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="J64">
         <v>0.0012416962587069</v>
@@ -19204,19 +19204,19 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C65" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D65" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E65" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I65" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J65">
         <v>0.0015984483099258</v>
@@ -19479,16 +19479,16 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C66" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D66" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="I66" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J66">
         <v>0.0024755430193983</v>
@@ -19760,16 +19760,16 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C67" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D67" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="I67" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="J67">
         <v>0.0012089442610578</v>
@@ -20041,16 +20041,16 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C68" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D68" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="I68" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J68">
         <v>0.0023849978802701</v>
@@ -20322,16 +20322,16 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C69" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D69" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="I69" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J69">
         <v>0.0020508834761068</v>
@@ -20603,13 +20603,13 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C70" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I70" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="J70">
         <v>0.004410416036765</v>
@@ -20881,10 +20881,10 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="I71" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J71">
         <v>0.0006414105255352</v>
@@ -22237,6 +22237,550 @@
       </c>
       <c r="CT75">
         <v>-0.8173346670588505</v>
+      </c>
+    </row>
+    <row r="76" spans="1:98">
+      <c r="A76" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I76" t="s">
+        <v>101</v>
+      </c>
+      <c r="J76">
+        <v>0.0007409682940759943</v>
+      </c>
+      <c r="K76">
+        <v>0.0003704841470379971</v>
+      </c>
+      <c r="L76">
+        <v>0.002960797138407356</v>
+      </c>
+      <c r="M76">
+        <v>0.002960797138407356</v>
+      </c>
+      <c r="N76">
+        <v>0.001901088706588672</v>
+      </c>
+      <c r="O76">
+        <v>0.0009505443532943358</v>
+      </c>
+      <c r="P76">
+        <v>0.003310443628669546</v>
+      </c>
+      <c r="Q76">
+        <v>0.003310443628669546</v>
+      </c>
+      <c r="R76">
+        <v>17.49711689673248</v>
+      </c>
+      <c r="S76">
+        <v>8.424951948278874</v>
+      </c>
+      <c r="T76">
+        <v>0.4537569547382341</v>
+      </c>
+      <c r="U76">
+        <v>0.4284247769425286</v>
+      </c>
+      <c r="V76">
+        <v>0.01522613033274777</v>
+      </c>
+      <c r="W76">
+        <v>0.09608383229720328</v>
+      </c>
+      <c r="X76">
+        <v>0.0363170182279708</v>
+      </c>
+      <c r="Y76">
+        <v>0.2397838567462378</v>
+      </c>
+      <c r="Z76">
+        <v>0.9997390302721156</v>
+      </c>
+      <c r="AA76">
+        <v>0.9661423879352263</v>
+      </c>
+      <c r="AB76">
+        <v>0.7888904604326938</v>
+      </c>
+      <c r="AC76">
+        <v>0.9975178008184862</v>
+      </c>
+      <c r="AD76">
+        <v>0.9092327020636333</v>
+      </c>
+      <c r="AE76">
+        <v>0.7590555595337336</v>
+      </c>
+      <c r="AF76">
+        <v>0.001783016439642901</v>
+      </c>
+      <c r="AG76">
+        <v>0.01203321461475726</v>
+      </c>
+      <c r="AH76">
+        <v>0.9997390302721156</v>
+      </c>
+      <c r="AI76">
+        <v>0.9975178008184862</v>
+      </c>
+      <c r="AJ76">
+        <v>0.001783016439642901</v>
+      </c>
+      <c r="AK76">
+        <v>0.01203321461475726</v>
+      </c>
+      <c r="AL76" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM76">
+        <v>0.005689041712621093</v>
+      </c>
+      <c r="AN76">
+        <v>0.09436460040480206</v>
+      </c>
+      <c r="AO76">
+        <v>-518.98541786</v>
+      </c>
+      <c r="AP76">
+        <v>-1682.3227202</v>
+      </c>
+      <c r="AQ76">
+        <v>16987.18099886027</v>
+      </c>
+      <c r="AR76">
+        <v>82891.78139551562</v>
+      </c>
+      <c r="AS76">
+        <v>16987.18099886027</v>
+      </c>
+      <c r="AT76">
+        <v>83272.23981962049</v>
+      </c>
+      <c r="AU76">
+        <v>0.6987180998860272</v>
+      </c>
+      <c r="AV76">
+        <v>7.289178139551561</v>
+      </c>
+      <c r="AW76">
+        <v>1.370148876105252</v>
+      </c>
+      <c r="AX76">
+        <v>2.835792123022458</v>
+      </c>
+      <c r="AY76">
+        <v>76.63333333333334</v>
+      </c>
+      <c r="AZ76">
+        <v>105.55</v>
+      </c>
+      <c r="BA76">
+        <v>0</v>
+      </c>
+      <c r="BB76">
+        <v>0.005658229509505465</v>
+      </c>
+      <c r="BC76">
+        <v>0</v>
+      </c>
+      <c r="BD76">
+        <v>-426.9140032690848</v>
+      </c>
+      <c r="BE76">
+        <v>6021</v>
+      </c>
+      <c r="BF76">
+        <v>3824</v>
+      </c>
+      <c r="BG76">
+        <v>715.375</v>
+      </c>
+      <c r="BH76">
+        <v>6496</v>
+      </c>
+      <c r="BI76">
+        <v>2203</v>
+      </c>
+      <c r="BJ76">
+        <v>12517</v>
+      </c>
+      <c r="BK76">
+        <v>6027</v>
+      </c>
+      <c r="BL76">
+        <v>5981</v>
+      </c>
+      <c r="BM76">
+        <v>1078</v>
+      </c>
+      <c r="BN76">
+        <v>6021</v>
+      </c>
+      <c r="BO76">
+        <v>2116</v>
+      </c>
+      <c r="BP76">
+        <v>515</v>
+      </c>
+      <c r="BQ76">
+        <v>1125</v>
+      </c>
+      <c r="BR76">
+        <v>0</v>
+      </c>
+      <c r="BS76">
+        <v>1708</v>
+      </c>
+      <c r="BT76">
+        <v>0</v>
+      </c>
+      <c r="BU76">
+        <v>0</v>
+      </c>
+      <c r="BV76">
+        <v>6988.73088214</v>
+      </c>
+      <c r="BW76">
+        <v>73340.86697980002</v>
+      </c>
+      <c r="BX76">
+        <v>0.05087466185282001</v>
+      </c>
+      <c r="BY76">
+        <v>0.08647750155435711</v>
+      </c>
+      <c r="BZ76">
+        <v>0.07071724023909719</v>
+      </c>
+      <c r="CA76">
+        <v>0.1941341861364861</v>
+      </c>
+      <c r="CB76">
+        <v>0.01536938017749344</v>
+      </c>
+      <c r="CC76">
+        <v>0.01199368660763904</v>
+      </c>
+      <c r="CD76">
+        <v>0.0124231069502814</v>
+      </c>
+      <c r="CE76">
+        <v>0.01351115597404425</v>
+      </c>
+      <c r="CF76">
+        <v>7507.7163</v>
+      </c>
+      <c r="CG76">
+        <v>75023.18970000002</v>
+      </c>
+      <c r="CH76">
+        <v>7507.7163</v>
+      </c>
+      <c r="CI76">
+        <v>75450.10370326909</v>
+      </c>
+      <c r="CJ76">
+        <v>0.08919824964453869</v>
+      </c>
+      <c r="CK76">
+        <v>0.1766374307868145</v>
+      </c>
+      <c r="CL76">
+        <v>10000</v>
+      </c>
+      <c r="CN76">
+        <v>5.824111822947E-05</v>
+      </c>
+      <c r="CO76">
+        <v>0.03995340710541642</v>
+      </c>
+      <c r="CP76">
+        <v>1797194.663885087</v>
+      </c>
+      <c r="CQ76">
+        <v>103761437.1558867</v>
+      </c>
+      <c r="CR76" s="2">
+        <v>45403.46751435161</v>
+      </c>
+      <c r="CS76">
+        <v>-0.9172425776350783</v>
+      </c>
+      <c r="CT76">
+        <v>-0.4507750361317039</v>
+      </c>
+    </row>
+    <row r="77" spans="1:98">
+      <c r="A77" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="I77" t="s">
+        <v>102</v>
+      </c>
+      <c r="J77">
+        <v>0.002416373053874654</v>
+      </c>
+      <c r="K77">
+        <v>0.001208186526937327</v>
+      </c>
+      <c r="L77">
+        <v>0.0005491112143227728</v>
+      </c>
+      <c r="M77">
+        <v>0.0005491112143227728</v>
+      </c>
+      <c r="N77">
+        <v>0.002176127952708162</v>
+      </c>
+      <c r="O77">
+        <v>0.001088063976354081</v>
+      </c>
+      <c r="P77">
+        <v>0.0004095275761893058</v>
+      </c>
+      <c r="Q77">
+        <v>0.0004095275761893058</v>
+      </c>
+      <c r="R77">
+        <v>29.44372853890968</v>
+      </c>
+      <c r="S77">
+        <v>9.855935799992285</v>
+      </c>
+      <c r="T77">
+        <v>0.3742276255140405</v>
+      </c>
+      <c r="U77">
+        <v>0.49778565600006</v>
+      </c>
+      <c r="V77">
+        <v>0.04611916480610084</v>
+      </c>
+      <c r="W77">
+        <v>0.09592003681836131</v>
+      </c>
+      <c r="X77">
+        <v>0.1852922032541665</v>
+      </c>
+      <c r="Y77">
+        <v>0.2144601712394749</v>
+      </c>
+      <c r="Z77">
+        <v>0.9994357454171765</v>
+      </c>
+      <c r="AA77">
+        <v>0.8463602095543351</v>
+      </c>
+      <c r="AB77">
+        <v>0.8051896603247478</v>
+      </c>
+      <c r="AC77">
+        <v>0.9989642575166992</v>
+      </c>
+      <c r="AD77">
+        <v>0.7728040851551814</v>
+      </c>
+      <c r="AE77">
+        <v>0.7932527508134306</v>
+      </c>
+      <c r="AF77">
+        <v>0.005780200053586797</v>
+      </c>
+      <c r="AG77">
+        <v>0.009980777925547546</v>
+      </c>
+      <c r="AH77">
+        <v>0.9994357454171765</v>
+      </c>
+      <c r="AI77">
+        <v>0.9989642575166992</v>
+      </c>
+      <c r="AJ77">
+        <v>0.005780200053586797</v>
+      </c>
+      <c r="AK77">
+        <v>0.009980777925547546</v>
+      </c>
+      <c r="AL77" t="s">
+        <v>233</v>
+      </c>
+      <c r="AM77">
+        <v>0.0213191472253164</v>
+      </c>
+      <c r="AN77">
+        <v>0.02913323696838731</v>
+      </c>
+      <c r="AO77">
+        <v>-10155.939895032</v>
+      </c>
+      <c r="AP77">
+        <v>-411.276049242</v>
+      </c>
+      <c r="AQ77">
+        <v>135506.4874049671</v>
+      </c>
+      <c r="AR77">
+        <v>18091.45212075794</v>
+      </c>
+      <c r="AS77">
+        <v>135506.4874049671</v>
+      </c>
+      <c r="AT77">
+        <v>18027.85332075794</v>
+      </c>
+      <c r="AU77">
+        <v>12.55064874049671</v>
+      </c>
+      <c r="AV77">
+        <v>0.8091452120757943</v>
+      </c>
+      <c r="AW77">
+        <v>0.8133267289366921</v>
+      </c>
+      <c r="AX77">
+        <v>2.431255285163958</v>
+      </c>
+      <c r="AY77">
+        <v>65.36666666666666</v>
+      </c>
+      <c r="AZ77">
+        <v>97.8</v>
+      </c>
+      <c r="BA77">
+        <v>0.008651058379411866</v>
+      </c>
+      <c r="BB77">
+        <v>0.09174956868434567</v>
+      </c>
+      <c r="BC77">
+        <v>-1183.865265994496</v>
+      </c>
+      <c r="BD77">
+        <v>-858.9279072597677</v>
+      </c>
+      <c r="BE77">
+        <v>11617</v>
+      </c>
+      <c r="BF77">
+        <v>3288</v>
+      </c>
+      <c r="BG77">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BH77">
+        <v>20181</v>
+      </c>
+      <c r="BI77">
+        <v>7356</v>
+      </c>
+      <c r="BJ77">
+        <v>31798</v>
+      </c>
+      <c r="BK77">
+        <v>10644</v>
+      </c>
+      <c r="BL77">
+        <v>10204</v>
+      </c>
+      <c r="BM77">
+        <v>2577</v>
+      </c>
+      <c r="BN77">
+        <v>11598</v>
+      </c>
+      <c r="BO77">
+        <v>3265</v>
+      </c>
+      <c r="BP77">
+        <v>9977</v>
+      </c>
+      <c r="BQ77">
+        <v>4779</v>
+      </c>
+      <c r="BR77">
+        <v>19</v>
+      </c>
+      <c r="BS77">
+        <v>23</v>
+      </c>
+      <c r="BT77">
+        <v>0</v>
+      </c>
+      <c r="BU77">
+        <v>0</v>
+      </c>
+      <c r="BV77">
+        <v>125506.4874049681</v>
+      </c>
+      <c r="BW77">
+        <v>8091.452120758007</v>
+      </c>
+      <c r="BX77">
+        <v>0.02920839054061308</v>
+      </c>
+      <c r="BY77">
+        <v>0.07629258210080538</v>
+      </c>
+      <c r="BZ77">
+        <v>0.100440321043834</v>
+      </c>
+      <c r="CA77">
+        <v>0.1713254251374956</v>
+      </c>
+      <c r="CB77">
+        <v>0.003615990904406083</v>
+      </c>
+      <c r="CC77">
+        <v>0.01070558514090266</v>
+      </c>
+      <c r="CD77">
+        <v>0.004520851532863802</v>
+      </c>
+      <c r="CE77">
+        <v>0.01042350463065131</v>
+      </c>
+      <c r="CF77">
+        <v>135662.4273000001</v>
+      </c>
+      <c r="CG77">
+        <v>8502.728170000008</v>
+      </c>
+      <c r="CH77">
+        <v>136846.2925659946</v>
+      </c>
+      <c r="CI77">
+        <v>9361.656077259775</v>
+      </c>
+      <c r="CJ77">
+        <v>0.1157853283667048</v>
+      </c>
+      <c r="CK77">
+        <v>0.04901352504422727</v>
+      </c>
+      <c r="CL77">
+        <v>10000</v>
+      </c>
+      <c r="CN77">
+        <v>0.00628858024691358</v>
+      </c>
+      <c r="CO77">
+        <v>0.009027777777777777</v>
+      </c>
+      <c r="CP77">
+        <v>90295518.62573735</v>
+      </c>
+      <c r="CQ77">
+        <v>11075597.03060125</v>
+      </c>
+      <c r="CR77" s="2">
+        <v>45403.78684908099</v>
+      </c>
+      <c r="CS77">
+        <v>-0.7048134977852135</v>
+      </c>
+      <c r="CT77">
+        <v>-0.7166260014620679</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RNDRUSDT.json at 2024-04-22_13-42-22 bestfile_scores 0.002220562748914326 bestfile_sharp 0.25400339440161745
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="311">
   <si>
     <t>Unnamed: 0.7</t>
   </si>
@@ -313,6 +313,9 @@
     <t>XRPUSDT</t>
   </si>
   <si>
+    <t>XTZUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -593,9 +596,6 @@
   </si>
   <si>
     <t>APTUSDT</t>
-  </si>
-  <si>
-    <t>XTZUSDT</t>
   </si>
   <si>
     <t>RNDRUSDT</t>
@@ -1308,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU78"/>
+  <dimension ref="A1:CU79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1612,31 +1612,31 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K2">
         <v>0.0009987329999999999</v>
@@ -1893,31 +1893,31 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J3" t="s">
-        <v>193</v>
+        <v>99</v>
       </c>
       <c r="K3">
         <v>0.001058605</v>
@@ -2174,31 +2174,31 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K4">
         <v>0.000882894</v>
@@ -2455,28 +2455,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J5" t="s">
         <v>194</v>
@@ -2736,31 +2736,31 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K6">
         <v>0.001076751</v>
@@ -3017,31 +3017,31 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K7">
         <v>-0.000540801</v>
@@ -3298,31 +3298,31 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K8">
         <v>0.001278948</v>
@@ -3579,31 +3579,31 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J9" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K9">
         <v>0.000266144</v>
@@ -3860,31 +3860,31 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K10">
         <v>0.001013204</v>
@@ -4141,28 +4141,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J11" t="s">
         <v>195</v>
@@ -4422,28 +4422,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J12" t="s">
         <v>98</v>
@@ -4703,28 +4703,28 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J13" t="s">
         <v>196</v>
@@ -4984,28 +4984,28 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J14" t="s">
         <v>197</v>
@@ -5265,31 +5265,31 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K15">
         <v>0.000327551</v>
@@ -5546,28 +5546,28 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J16" t="s">
         <v>198</v>
@@ -5827,28 +5827,28 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I17" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J17" t="s">
         <v>199</v>
@@ -6108,28 +6108,28 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I18" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J18" t="s">
         <v>200</v>
@@ -6389,28 +6389,28 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J19" t="s">
         <v>201</v>
@@ -6670,28 +6670,28 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I20" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J20" t="s">
         <v>202</v>
@@ -6951,28 +6951,28 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I21" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J21" t="s">
         <v>203</v>
@@ -7232,28 +7232,28 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J22" t="s">
         <v>204</v>
@@ -7513,28 +7513,28 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I23" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J23" t="s">
         <v>205</v>
@@ -7794,28 +7794,28 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J24" t="s">
         <v>206</v>
@@ -8075,28 +8075,28 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I25" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J25" t="s">
         <v>207</v>
@@ -8356,28 +8356,28 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I26" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J26" t="s">
         <v>208</v>
@@ -8637,28 +8637,28 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I27" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J27" t="s">
         <v>209</v>
@@ -8918,28 +8918,28 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I28" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J28" t="s">
         <v>210</v>
@@ -9199,28 +9199,28 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I29" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J29" t="s">
         <v>211</v>
@@ -9480,28 +9480,28 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I30" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J30" t="s">
         <v>212</v>
@@ -9761,28 +9761,28 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I31" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J31" t="s">
         <v>213</v>
@@ -10042,28 +10042,28 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I32" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J32" t="s">
         <v>214</v>
@@ -10323,28 +10323,28 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I33" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J33" t="s">
         <v>215</v>
@@ -10604,28 +10604,28 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J34" t="s">
         <v>216</v>
@@ -10891,28 +10891,28 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I35" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J35" t="s">
         <v>217</v>
@@ -11178,28 +11178,28 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I36" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J36" t="s">
         <v>218</v>
@@ -11465,31 +11465,31 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J37" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K37">
         <v>0.001640077</v>
@@ -11752,28 +11752,28 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I38" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J38" t="s">
         <v>219</v>
@@ -12039,28 +12039,28 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I39" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J39" t="s">
         <v>220</v>
@@ -12326,28 +12326,28 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I40" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J40" t="s">
         <v>221</v>
@@ -12613,28 +12613,28 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I41" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J41" t="s">
         <v>222</v>
@@ -12900,28 +12900,28 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I42" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J42" t="s">
         <v>223</v>
@@ -13187,28 +13187,28 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I43" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J43" t="s">
         <v>224</v>
@@ -13474,28 +13474,28 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I44" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J44" t="s">
         <v>225</v>
@@ -13761,28 +13761,28 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I45" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J45" t="s">
         <v>226</v>
@@ -14048,28 +14048,28 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I46" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J46" t="s">
         <v>227</v>
@@ -14335,28 +14335,28 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J47" t="s">
         <v>228</v>
@@ -14622,28 +14622,28 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I48" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J48" t="s">
         <v>229</v>
@@ -14909,28 +14909,28 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I49" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J49" t="s">
         <v>230</v>
@@ -15196,28 +15196,28 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I50" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J50" t="s">
         <v>231</v>
@@ -15483,28 +15483,28 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J51" t="s">
         <v>232</v>
@@ -15770,28 +15770,28 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I52" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J52" t="s">
         <v>233</v>
@@ -16057,28 +16057,28 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I53" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J53" t="s">
         <v>234</v>
@@ -16344,31 +16344,31 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H54" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I54" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J54" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K54">
         <v>0.0008229381467956</v>
@@ -16631,28 +16631,28 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G55" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H55" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J55" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K55">
         <v>0.0022239398231451</v>
@@ -16915,25 +16915,25 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F56" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G56" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J56" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K56">
         <v>0.0018211096217568</v>
@@ -17196,22 +17196,22 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E57" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F57" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J57" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K57">
         <v>0.0012556275124289</v>
@@ -17474,22 +17474,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E58" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F58" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J58" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K58">
         <v>0.0019905125443684</v>
@@ -17752,22 +17752,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E59" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F59" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J59" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K59">
         <v>0.0005221982670147</v>
@@ -18030,22 +18030,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E60" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F60" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J60" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K60">
         <v>0.0018105477499388</v>
@@ -18308,22 +18308,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E61" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F61" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J61" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K61">
         <v>0.0006776201968474</v>
@@ -18586,22 +18586,22 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F62" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J62" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K62">
         <v>0.0025014106780221</v>
@@ -18864,22 +18864,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F63" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J63" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K63">
         <v>0.0007538484415952</v>
@@ -19142,22 +19142,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F64" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J64" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K64">
         <v>0.0012416962587069</v>
@@ -19420,22 +19420,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F65" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J65" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K65">
         <v>0.0015984483099258</v>
@@ -19698,19 +19698,19 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D66" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E66" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J66" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K66">
         <v>0.0024755430193983</v>
@@ -19982,19 +19982,19 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E67" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J67" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K67">
         <v>0.0012089442610578</v>
@@ -20266,19 +20266,19 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D68" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E68" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J68" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K68">
         <v>0.0023849978802701</v>
@@ -20550,19 +20550,19 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D69" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E69" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J69" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K69">
         <v>0.0020508834761068</v>
@@ -20834,16 +20834,16 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C70" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K70">
         <v>0.004410416036765</v>
@@ -21115,13 +21115,13 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C71" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J71" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K71">
         <v>0.0006414105255352</v>
@@ -21393,10 +21393,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="J72" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K72">
         <v>0.0014224236350091</v>
@@ -21668,10 +21668,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="J73" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="K73">
         <v>0.0008003654809294</v>
@@ -21943,10 +21943,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J74" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="K74">
         <v>0.001155136088498</v>
@@ -22218,10 +22218,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J75" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K75">
         <v>0.001355651330368</v>
@@ -22493,10 +22493,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J76" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K76">
         <v>0.0007409682940759</v>
@@ -23308,6 +23308,278 @@
       </c>
       <c r="CU78">
         <v>-0.8021491961550891</v>
+      </c>
+    </row>
+    <row r="79" spans="1:99">
+      <c r="A79" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J79" t="s">
+        <v>99</v>
+      </c>
+      <c r="K79">
+        <v>0.0023022492949476</v>
+      </c>
+      <c r="L79">
+        <v>0.0011511246474738</v>
+      </c>
+      <c r="M79">
+        <v>0.001132809470618446</v>
+      </c>
+      <c r="N79">
+        <v>0.001132809470618446</v>
+      </c>
+      <c r="O79">
+        <v>0.001320341103277967</v>
+      </c>
+      <c r="P79">
+        <v>0.0006601705516389833</v>
+      </c>
+      <c r="Q79">
+        <v>0.0009297039817541374</v>
+      </c>
+      <c r="R79">
+        <v>0.0009297039817541374</v>
+      </c>
+      <c r="S79">
+        <v>6.044719057733153</v>
+      </c>
+      <c r="T79">
+        <v>18.28986290789728</v>
+      </c>
+      <c r="U79">
+        <v>0.3408549281555267</v>
+      </c>
+      <c r="V79">
+        <v>0.744649803226329</v>
+      </c>
+      <c r="W79">
+        <v>0.08486726489436318</v>
+      </c>
+      <c r="X79">
+        <v>0.05002306106166224</v>
+      </c>
+      <c r="Y79">
+        <v>0.2005157685450449</v>
+      </c>
+      <c r="Z79">
+        <v>0.1223006915905091</v>
+      </c>
+      <c r="AA79">
+        <v>0.9991162835274094</v>
+      </c>
+      <c r="AB79">
+        <v>0.8412472807924374</v>
+      </c>
+      <c r="AC79">
+        <v>0.8971580909746162</v>
+      </c>
+      <c r="AD79">
+        <v>0.9991372938699528</v>
+      </c>
+      <c r="AE79">
+        <v>0.7997387517786095</v>
+      </c>
+      <c r="AF79">
+        <v>0.8779248708082366</v>
+      </c>
+      <c r="AG79">
+        <v>0.008438748641480366</v>
+      </c>
+      <c r="AH79">
+        <v>0.005215146972682691</v>
+      </c>
+      <c r="AI79">
+        <v>0.9991162835274094</v>
+      </c>
+      <c r="AJ79">
+        <v>0.9991372938699528</v>
+      </c>
+      <c r="AK79">
+        <v>0.008438748641480366</v>
+      </c>
+      <c r="AL79">
+        <v>0.005215146972682691</v>
+      </c>
+      <c r="AM79" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN79">
+        <v>0.01877497112173667</v>
+      </c>
+      <c r="AO79">
+        <v>0.04654771507522337</v>
+      </c>
+      <c r="AP79">
+        <v>-3850.77647392</v>
+      </c>
+      <c r="AQ79">
+        <v>-1535.82957572</v>
+      </c>
+      <c r="AR79">
+        <v>119553.1577260801</v>
+      </c>
+      <c r="AS79">
+        <v>33924.84182428</v>
+      </c>
+      <c r="AT79">
+        <v>119553.1577260801</v>
+      </c>
+      <c r="AU79">
+        <v>33649.75422428</v>
+      </c>
+      <c r="AV79">
+        <v>10.95531577260801</v>
+      </c>
+      <c r="AW79">
+        <v>2.392484182427999</v>
+      </c>
+      <c r="AX79">
+        <v>3.960095588611154</v>
+      </c>
+      <c r="AY79">
+        <v>1.31079410125171</v>
+      </c>
+      <c r="AZ79">
+        <v>148.2666666666667</v>
+      </c>
+      <c r="BA79">
+        <v>113.1833333333333</v>
+      </c>
+      <c r="BB79">
+        <v>0.0190701963167496</v>
+      </c>
+      <c r="BC79">
+        <v>0.0514758727695607</v>
+      </c>
+      <c r="BD79">
+        <v>-2204.678948651953</v>
+      </c>
+      <c r="BE79">
+        <v>-1381.73636704508</v>
+      </c>
+      <c r="BF79">
+        <v>2308</v>
+      </c>
+      <c r="BG79">
+        <v>6780</v>
+      </c>
+      <c r="BH79">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI79">
+        <v>4214</v>
+      </c>
+      <c r="BJ79">
+        <v>12954</v>
+      </c>
+      <c r="BK79">
+        <v>6522</v>
+      </c>
+      <c r="BL79">
+        <v>19734</v>
+      </c>
+      <c r="BM79">
+        <v>2236</v>
+      </c>
+      <c r="BN79">
+        <v>6500</v>
+      </c>
+      <c r="BO79">
+        <v>2301</v>
+      </c>
+      <c r="BP79">
+        <v>6737</v>
+      </c>
+      <c r="BQ79">
+        <v>1978</v>
+      </c>
+      <c r="BR79">
+        <v>6454</v>
+      </c>
+      <c r="BS79">
+        <v>7</v>
+      </c>
+      <c r="BT79">
+        <v>43</v>
+      </c>
+      <c r="BU79">
+        <v>0</v>
+      </c>
+      <c r="BV79">
+        <v>0</v>
+      </c>
+      <c r="BW79">
+        <v>109553.1577260801</v>
+      </c>
+      <c r="BX79">
+        <v>23924.84182427999</v>
+      </c>
+      <c r="BY79">
+        <v>0.04418845432014045</v>
+      </c>
+      <c r="BZ79">
+        <v>0.04451638722632226</v>
+      </c>
+      <c r="CA79">
+        <v>0.1112417378984985</v>
+      </c>
+      <c r="CB79">
+        <v>0.1087884404396345</v>
+      </c>
+      <c r="CC79">
+        <v>0.0083758688712897</v>
+      </c>
+      <c r="CD79">
+        <v>0.009364121757474026</v>
+      </c>
+      <c r="CE79">
+        <v>0.008577394640126919</v>
+      </c>
+      <c r="CF79">
+        <v>0.006982197247215908</v>
+      </c>
+      <c r="CG79">
+        <v>113403.9342000001</v>
+      </c>
+      <c r="CH79">
+        <v>25460.67139999999</v>
+      </c>
+      <c r="CI79">
+        <v>115608.613148652</v>
+      </c>
+      <c r="CJ79">
+        <v>26842.40776704507</v>
+      </c>
+      <c r="CK79">
+        <v>0.06218119599475105</v>
+      </c>
+      <c r="CL79">
+        <v>0.1911733449218872</v>
+      </c>
+      <c r="CM79">
+        <v>10000</v>
+      </c>
+      <c r="CO79">
+        <v>0.01065801668211307</v>
+      </c>
+      <c r="CP79">
+        <v>0.01714550509731233</v>
+      </c>
+      <c r="CQ79">
+        <v>20364169.57193603</v>
+      </c>
+      <c r="CR79">
+        <v>13794144.77050867</v>
+      </c>
+      <c r="CS79" s="2">
+        <v>45404.46191518348</v>
+      </c>
+      <c r="CT79">
+        <v>-0.6546270123512354</v>
+      </c>
+      <c r="CU79">
+        <v>-0.8511473034125144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update CHRUSDT.json at 2024-04-23_20-16-28 bestfile_scores 0.0011775010367306548 bestfile_sharp 0.08042047244351958
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="311">
   <si>
     <t>Unnamed: 0.7</t>
   </si>
@@ -325,6 +325,9 @@
     <t>KAVAUSDT</t>
   </si>
   <si>
+    <t>ONEUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -605,9 +608,6 @@
   </si>
   <si>
     <t>APTUSDT</t>
-  </si>
-  <si>
-    <t>ONEUSDT</t>
   </si>
   <si>
     <t>CHRUSDT</t>
@@ -1308,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU82"/>
+  <dimension ref="A1:CU83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1612,31 +1612,31 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K2">
         <v>0.0009987329999999999</v>
@@ -1893,28 +1893,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J3" t="s">
         <v>99</v>
@@ -2174,31 +2174,31 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K4">
         <v>0.000882894</v>
@@ -2455,28 +2455,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J5" t="s">
         <v>100</v>
@@ -2736,31 +2736,31 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K6">
         <v>0.001076751</v>
@@ -3017,31 +3017,31 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K7">
         <v>-0.000540801</v>
@@ -3298,31 +3298,31 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K8">
         <v>0.001278948</v>
@@ -3579,31 +3579,31 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K9">
         <v>0.000266144</v>
@@ -3860,31 +3860,31 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K10">
         <v>0.001013204</v>
@@ -4141,28 +4141,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J11" t="s">
         <v>101</v>
@@ -4422,28 +4422,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I12" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J12" t="s">
         <v>98</v>
@@ -4703,28 +4703,28 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J13" t="s">
         <v>102</v>
@@ -4984,31 +4984,31 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J14" t="s">
-        <v>197</v>
+        <v>103</v>
       </c>
       <c r="K14">
         <v>0.000431045</v>
@@ -5265,31 +5265,31 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K15">
         <v>0.000327551</v>
@@ -5546,28 +5546,28 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J16" t="s">
         <v>198</v>
@@ -5827,28 +5827,28 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J17" t="s">
         <v>199</v>
@@ -6108,28 +6108,28 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J18" t="s">
         <v>200</v>
@@ -6389,28 +6389,28 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J19" t="s">
         <v>201</v>
@@ -6670,28 +6670,28 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I20" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J20" t="s">
         <v>202</v>
@@ -6951,28 +6951,28 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J21" t="s">
         <v>203</v>
@@ -7232,28 +7232,28 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J22" t="s">
         <v>204</v>
@@ -7513,28 +7513,28 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I23" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J23" t="s">
         <v>205</v>
@@ -7794,28 +7794,28 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I24" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J24" t="s">
         <v>206</v>
@@ -8075,28 +8075,28 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J25" t="s">
         <v>207</v>
@@ -8356,28 +8356,28 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J26" t="s">
         <v>208</v>
@@ -8637,28 +8637,28 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I27" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J27" t="s">
         <v>209</v>
@@ -8918,28 +8918,28 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I28" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J28" t="s">
         <v>210</v>
@@ -9199,28 +9199,28 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I29" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J29" t="s">
         <v>211</v>
@@ -9480,28 +9480,28 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J30" t="s">
         <v>212</v>
@@ -9761,28 +9761,28 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I31" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J31" t="s">
         <v>213</v>
@@ -10042,28 +10042,28 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I32" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J32" t="s">
         <v>214</v>
@@ -10323,28 +10323,28 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I33" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J33" t="s">
         <v>215</v>
@@ -10604,28 +10604,28 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J34" t="s">
         <v>216</v>
@@ -10891,28 +10891,28 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J35" t="s">
         <v>217</v>
@@ -11178,28 +11178,28 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J36" t="s">
         <v>218</v>
@@ -11465,31 +11465,31 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J37" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K37">
         <v>0.001640077</v>
@@ -11752,28 +11752,28 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J38" t="s">
         <v>219</v>
@@ -12039,28 +12039,28 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J39" t="s">
         <v>220</v>
@@ -12326,28 +12326,28 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I40" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J40" t="s">
         <v>221</v>
@@ -12613,28 +12613,28 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J41" t="s">
         <v>222</v>
@@ -12900,28 +12900,28 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I42" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J42" t="s">
         <v>223</v>
@@ -13187,28 +13187,28 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I43" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J43" t="s">
         <v>224</v>
@@ -13474,28 +13474,28 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I44" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J44" t="s">
         <v>225</v>
@@ -13761,28 +13761,28 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I45" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J45" t="s">
         <v>226</v>
@@ -14048,28 +14048,28 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I46" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J46" t="s">
         <v>227</v>
@@ -14335,28 +14335,28 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I47" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J47" t="s">
         <v>228</v>
@@ -14622,28 +14622,28 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J48" t="s">
         <v>229</v>
@@ -14909,28 +14909,28 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I49" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J49" t="s">
         <v>230</v>
@@ -15196,28 +15196,28 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I50" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J50" t="s">
         <v>231</v>
@@ -15483,28 +15483,28 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I51" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J51" t="s">
         <v>232</v>
@@ -15770,28 +15770,28 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J52" t="s">
         <v>233</v>
@@ -16057,28 +16057,28 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I53" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J53" t="s">
         <v>234</v>
@@ -16344,31 +16344,31 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H54" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I54" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J54" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K54">
         <v>0.0008229381467956</v>
@@ -16631,28 +16631,28 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G55" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H55" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J55" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K55">
         <v>0.0022239398231451</v>
@@ -16915,25 +16915,25 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G56" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J56" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K56">
         <v>0.0018211096217568</v>
@@ -17196,22 +17196,22 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E57" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F57" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J57" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K57">
         <v>0.0012556275124289</v>
@@ -17474,22 +17474,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E58" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F58" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J58" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K58">
         <v>0.0019905125443684</v>
@@ -17752,22 +17752,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E59" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F59" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J59" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K59">
         <v>0.0005221982670147</v>
@@ -18030,22 +18030,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E60" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F60" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J60" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K60">
         <v>0.0018105477499388</v>
@@ -18308,22 +18308,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F61" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J61" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K61">
         <v>0.0006776201968474</v>
@@ -18586,22 +18586,22 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C62" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D62" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E62" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F62" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J62" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K62">
         <v>0.0025014106780221</v>
@@ -18864,22 +18864,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E63" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F63" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J63" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K63">
         <v>0.0007538484415952</v>
@@ -19142,22 +19142,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E64" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F64" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J64" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K64">
         <v>0.0012416962587069</v>
@@ -19420,22 +19420,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F65" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J65" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K65">
         <v>0.0015984483099258</v>
@@ -19698,19 +19698,19 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E66" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J66" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K66">
         <v>0.0024755430193983</v>
@@ -19982,19 +19982,19 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C67" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D67" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E67" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J67" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K67">
         <v>0.0012089442610578</v>
@@ -20266,19 +20266,19 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D68" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E68" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J68" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K68">
         <v>0.0023849978802701</v>
@@ -20550,19 +20550,19 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C69" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D69" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E69" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J69" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K69">
         <v>0.0020508834761068</v>
@@ -20834,16 +20834,16 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C70" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D70" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J70" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K70">
         <v>0.004410416036765</v>
@@ -21115,13 +21115,13 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C71" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J71" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K71">
         <v>0.0006414105255352</v>
@@ -21393,10 +21393,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J72" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="K72">
         <v>0.0014224236350091</v>
@@ -21668,10 +21668,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J73" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K73">
         <v>0.0008003654809294</v>
@@ -21943,10 +21943,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J74" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K74">
         <v>0.001155136088498</v>
@@ -22218,10 +22218,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J75" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K75">
         <v>0.001355651330368</v>
@@ -22493,10 +22493,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J76" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K76">
         <v>0.0007409682940759</v>
@@ -24396,6 +24396,278 @@
       </c>
       <c r="CU82">
         <v>-0.92167062843021</v>
+      </c>
+    </row>
+    <row r="83" spans="1:99">
+      <c r="A83" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="J83" t="s">
+        <v>103</v>
+      </c>
+      <c r="K83">
+        <v>0.001187602923088615</v>
+      </c>
+      <c r="L83">
+        <v>0.0005938014615443077</v>
+      </c>
+      <c r="M83">
+        <v>0.001104573885329696</v>
+      </c>
+      <c r="N83">
+        <v>0.001104573885329696</v>
+      </c>
+      <c r="O83">
+        <v>0.002329194404699808</v>
+      </c>
+      <c r="P83">
+        <v>0.001164597202349904</v>
+      </c>
+      <c r="Q83">
+        <v>0.0009013350891015071</v>
+      </c>
+      <c r="R83">
+        <v>0.0009013350891015071</v>
+      </c>
+      <c r="S83">
+        <v>17.77013002044832</v>
+      </c>
+      <c r="T83">
+        <v>10.97171958794707</v>
+      </c>
+      <c r="U83">
+        <v>0.3761781647122883</v>
+      </c>
+      <c r="V83">
+        <v>0.7000871404316595</v>
+      </c>
+      <c r="W83">
+        <v>0.02791427353052018</v>
+      </c>
+      <c r="X83">
+        <v>0.07560341498902283</v>
+      </c>
+      <c r="Y83">
+        <v>0.2258151777299673</v>
+      </c>
+      <c r="Z83">
+        <v>0.1638142652492838</v>
+      </c>
+      <c r="AA83">
+        <v>0.9996414709266825</v>
+      </c>
+      <c r="AB83">
+        <v>0.8198941368241861</v>
+      </c>
+      <c r="AC83">
+        <v>0.8568990908092247</v>
+      </c>
+      <c r="AD83">
+        <v>0.9987294425076463</v>
+      </c>
+      <c r="AE83">
+        <v>0.7385702114406039</v>
+      </c>
+      <c r="AF83">
+        <v>0.8336253034592219</v>
+      </c>
+      <c r="AG83">
+        <v>0.004946317301240458</v>
+      </c>
+      <c r="AH83">
+        <v>0.008361015861965755</v>
+      </c>
+      <c r="AI83">
+        <v>0.9996414709266825</v>
+      </c>
+      <c r="AJ83">
+        <v>0.9987294425076463</v>
+      </c>
+      <c r="AK83">
+        <v>0.004946317301240458</v>
+      </c>
+      <c r="AL83">
+        <v>0.008361015861965755</v>
+      </c>
+      <c r="AM83" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN83">
+        <v>0.007589587709628477</v>
+      </c>
+      <c r="AO83">
+        <v>0.03498808921949439</v>
+      </c>
+      <c r="AP83">
+        <v>-1475.75506598</v>
+      </c>
+      <c r="AQ83">
+        <v>-974.5887138200001</v>
+      </c>
+      <c r="AR83">
+        <v>36031.21989402001</v>
+      </c>
+      <c r="AS83">
+        <v>32944.37490618024</v>
+      </c>
+      <c r="AT83">
+        <v>36031.21989402001</v>
+      </c>
+      <c r="AU83">
+        <v>32943.32994618025</v>
+      </c>
+      <c r="AV83">
+        <v>2.603121989402001</v>
+      </c>
+      <c r="AW83">
+        <v>2.294437490618024</v>
+      </c>
+      <c r="AX83">
+        <v>1.348377627236408</v>
+      </c>
+      <c r="AY83">
+        <v>2.186101733063246</v>
+      </c>
+      <c r="AZ83">
+        <v>108.15</v>
+      </c>
+      <c r="BA83">
+        <v>106.7166666666667</v>
+      </c>
+      <c r="BB83">
+        <v>0.01622597094488962</v>
+      </c>
+      <c r="BC83">
+        <v>0.03482233864432707</v>
+      </c>
+      <c r="BD83">
+        <v>-453.6889197120319</v>
+      </c>
+      <c r="BE83">
+        <v>-862.9647002263624</v>
+      </c>
+      <c r="BF83">
+        <v>8729</v>
+      </c>
+      <c r="BG83">
+        <v>4538</v>
+      </c>
+      <c r="BH83">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI83">
+        <v>10462</v>
+      </c>
+      <c r="BJ83">
+        <v>7311</v>
+      </c>
+      <c r="BK83">
+        <v>19191</v>
+      </c>
+      <c r="BL83">
+        <v>11849</v>
+      </c>
+      <c r="BM83">
+        <v>8701</v>
+      </c>
+      <c r="BN83">
+        <v>3472</v>
+      </c>
+      <c r="BO83">
+        <v>8724</v>
+      </c>
+      <c r="BP83">
+        <v>4439</v>
+      </c>
+      <c r="BQ83">
+        <v>1761</v>
+      </c>
+      <c r="BR83">
+        <v>3839</v>
+      </c>
+      <c r="BS83">
+        <v>5</v>
+      </c>
+      <c r="BT83">
+        <v>99</v>
+      </c>
+      <c r="BU83">
+        <v>0</v>
+      </c>
+      <c r="BV83">
+        <v>0</v>
+      </c>
+      <c r="BW83">
+        <v>26031.21989401999</v>
+      </c>
+      <c r="BX83">
+        <v>22944.37490618002</v>
+      </c>
+      <c r="BY83">
+        <v>0.04042037732965634</v>
+      </c>
+      <c r="BZ83">
+        <v>0.07910254587964398</v>
+      </c>
+      <c r="CA83">
+        <v>0.1247808654181507</v>
+      </c>
+      <c r="CB83">
+        <v>0.1426253155070022</v>
+      </c>
+      <c r="CC83">
+        <v>0.01271395191331906</v>
+      </c>
+      <c r="CD83">
+        <v>0.01026658671436477</v>
+      </c>
+      <c r="CE83">
+        <v>0.009826740856113184</v>
+      </c>
+      <c r="CF83">
+        <v>0.01485384705810866</v>
+      </c>
+      <c r="CG83">
+        <v>27506.97495999999</v>
+      </c>
+      <c r="CH83">
+        <v>23918.96362000002</v>
+      </c>
+      <c r="CI83">
+        <v>27960.66387971202</v>
+      </c>
+      <c r="CJ83">
+        <v>24781.92832022638</v>
+      </c>
+      <c r="CK83">
+        <v>0.07271148486064086</v>
+      </c>
+      <c r="CL83">
+        <v>0.1218400209194586</v>
+      </c>
+      <c r="CM83">
+        <v>10000</v>
+      </c>
+      <c r="CO83">
+        <v>0.002430555555555556</v>
+      </c>
+      <c r="CP83">
+        <v>0.01018518518518519</v>
+      </c>
+      <c r="CQ83">
+        <v>5450725.921064924</v>
+      </c>
+      <c r="CR83">
+        <v>9553962.229671104</v>
+      </c>
+      <c r="CS83" s="2">
+        <v>45405.59739121774</v>
+      </c>
+      <c r="CT83">
+        <v>-0.7975627900619038</v>
+      </c>
+      <c r="CU83">
+        <v>-0.7661869296895436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SKLUSDT.json at 2024-04-24_05-28-36 bestfile_scores 0.0003008670739450048 bestfile_sharp 0.10704115393542822
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="856" uniqueCount="311">
   <si>
     <t>Unnamed: 0.7</t>
   </si>
@@ -328,6 +328,9 @@
     <t>ONEUSDT</t>
   </si>
   <si>
+    <t>CHRUSDT</t>
+  </si>
+  <si>
     <t>0</t>
   </si>
   <si>
@@ -608,9 +611,6 @@
   </si>
   <si>
     <t>APTUSDT</t>
-  </si>
-  <si>
-    <t>CHRUSDT</t>
   </si>
   <si>
     <t>SKLUSDT</t>
@@ -1308,7 +1308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU83"/>
+  <dimension ref="A1:CU84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1612,31 +1612,31 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K2">
         <v>0.0009987329999999999</v>
@@ -1893,28 +1893,28 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J3" t="s">
         <v>99</v>
@@ -2174,31 +2174,31 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K4">
         <v>0.000882894</v>
@@ -2455,28 +2455,28 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="G5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J5" t="s">
         <v>100</v>
@@ -2736,31 +2736,31 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K6">
         <v>0.001076751</v>
@@ -3017,31 +3017,31 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="I7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="J7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K7">
         <v>-0.000540801</v>
@@ -3298,31 +3298,31 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J8" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K8">
         <v>0.001278948</v>
@@ -3579,31 +3579,31 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J9" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K9">
         <v>0.000266144</v>
@@ -3860,31 +3860,31 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I10" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="J10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K10">
         <v>0.001013204</v>
@@ -4141,28 +4141,28 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I11" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J11" t="s">
         <v>101</v>
@@ -4422,28 +4422,28 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J12" t="s">
         <v>98</v>
@@ -4703,28 +4703,28 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J13" t="s">
         <v>102</v>
@@ -4984,28 +4984,28 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J14" t="s">
         <v>103</v>
@@ -5265,31 +5265,31 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I15" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="J15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K15">
         <v>0.000327551</v>
@@ -5546,31 +5546,31 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J16" t="s">
-        <v>198</v>
+        <v>104</v>
       </c>
       <c r="K16">
         <v>0.001162093</v>
@@ -5827,28 +5827,28 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I17" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J17" t="s">
         <v>199</v>
@@ -6108,28 +6108,28 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I18" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J18" t="s">
         <v>200</v>
@@ -6389,28 +6389,28 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="G19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J19" t="s">
         <v>201</v>
@@ -6670,28 +6670,28 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I20" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J20" t="s">
         <v>202</v>
@@ -6951,28 +6951,28 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I21" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J21" t="s">
         <v>203</v>
@@ -7232,28 +7232,28 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J22" t="s">
         <v>204</v>
@@ -7513,28 +7513,28 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I23" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J23" t="s">
         <v>205</v>
@@ -7794,28 +7794,28 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J24" t="s">
         <v>206</v>
@@ -8075,28 +8075,28 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J25" t="s">
         <v>207</v>
@@ -8356,28 +8356,28 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J26" t="s">
         <v>208</v>
@@ -8637,28 +8637,28 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I27" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J27" t="s">
         <v>209</v>
@@ -8918,28 +8918,28 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I28" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J28" t="s">
         <v>210</v>
@@ -9199,28 +9199,28 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I29" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J29" t="s">
         <v>211</v>
@@ -9480,28 +9480,28 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="I30" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J30" t="s">
         <v>212</v>
@@ -9761,28 +9761,28 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I31" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J31" t="s">
         <v>213</v>
@@ -10042,28 +10042,28 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I32" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J32" t="s">
         <v>214</v>
@@ -10323,28 +10323,28 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J33" t="s">
         <v>215</v>
@@ -10604,28 +10604,28 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I34" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="J34" t="s">
         <v>216</v>
@@ -10891,28 +10891,28 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I35" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J35" t="s">
         <v>217</v>
@@ -11178,28 +11178,28 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I36" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J36" t="s">
         <v>218</v>
@@ -11465,31 +11465,31 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J37" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K37">
         <v>0.001640077</v>
@@ -11752,28 +11752,28 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I38" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="J38" t="s">
         <v>219</v>
@@ -12039,28 +12039,28 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I39" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J39" t="s">
         <v>220</v>
@@ -12326,28 +12326,28 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I40" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J40" t="s">
         <v>221</v>
@@ -12613,28 +12613,28 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I41" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J41" t="s">
         <v>222</v>
@@ -12900,28 +12900,28 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I42" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="J42" t="s">
         <v>223</v>
@@ -13187,28 +13187,28 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I43" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J43" t="s">
         <v>224</v>
@@ -13474,28 +13474,28 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I44" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J44" t="s">
         <v>225</v>
@@ -13761,28 +13761,28 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I45" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J45" t="s">
         <v>226</v>
@@ -14048,28 +14048,28 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I46" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J46" t="s">
         <v>227</v>
@@ -14335,28 +14335,28 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I47" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="J47" t="s">
         <v>228</v>
@@ -14622,28 +14622,28 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="E48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I48" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J48" t="s">
         <v>229</v>
@@ -14909,28 +14909,28 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I49" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J49" t="s">
         <v>230</v>
@@ -15196,28 +15196,28 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="I50" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="J50" t="s">
         <v>231</v>
@@ -15483,28 +15483,28 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="G51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I51" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J51" t="s">
         <v>232</v>
@@ -15770,28 +15770,28 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J52" t="s">
         <v>233</v>
@@ -16057,28 +16057,28 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J53" t="s">
         <v>234</v>
@@ -16344,31 +16344,31 @@
         <v>52</v>
       </c>
       <c r="B54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I54" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="J54" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K54">
         <v>0.0008229381467956</v>
@@ -16631,28 +16631,28 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="G55" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H55" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J55" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="K55">
         <v>0.0022239398231451</v>
@@ -16915,25 +16915,25 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F56" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G56" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="J56" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K56">
         <v>0.0018211096217568</v>
@@ -17196,22 +17196,22 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E57" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F57" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="J57" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K57">
         <v>0.0012556275124289</v>
@@ -17474,22 +17474,22 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E58" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J58" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K58">
         <v>0.0019905125443684</v>
@@ -17752,22 +17752,22 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E59" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F59" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J59" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K59">
         <v>0.0005221982670147</v>
@@ -18030,22 +18030,22 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E60" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F60" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J60" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="K60">
         <v>0.0018105477499388</v>
@@ -18308,22 +18308,22 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C61" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D61" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E61" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F61" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J61" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="K61">
         <v>0.0006776201968474</v>
@@ -18586,22 +18586,22 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E62" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F62" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J62" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K62">
         <v>0.0025014106780221</v>
@@ -18864,22 +18864,22 @@
         <v>61</v>
       </c>
       <c r="B63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E63" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F63" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="J63" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K63">
         <v>0.0007538484415952</v>
@@ -19142,22 +19142,22 @@
         <v>62</v>
       </c>
       <c r="B64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E64" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F64" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="J64" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K64">
         <v>0.0012416962587069</v>
@@ -19420,22 +19420,22 @@
         <v>63</v>
       </c>
       <c r="B65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E65" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F65" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="J65" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="K65">
         <v>0.0015984483099258</v>
@@ -19698,19 +19698,19 @@
         <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E66" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J66" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K66">
         <v>0.0024755430193983</v>
@@ -19982,19 +19982,19 @@
         <v>65</v>
       </c>
       <c r="B67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E67" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="J67" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="K67">
         <v>0.0012089442610578</v>
@@ -20266,19 +20266,19 @@
         <v>66</v>
       </c>
       <c r="B68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D68" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E68" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J68" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="K68">
         <v>0.0023849978802701</v>
@@ -20550,19 +20550,19 @@
         <v>67</v>
       </c>
       <c r="B69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D69" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E69" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="J69" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="K69">
         <v>0.0020508834761068</v>
@@ -20834,16 +20834,16 @@
         <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C70" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D70" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="J70" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K70">
         <v>0.004410416036765</v>
@@ -21115,13 +21115,13 @@
         <v>69</v>
       </c>
       <c r="B71" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C71" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J71" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K71">
         <v>0.0006414105255352</v>
@@ -21393,10 +21393,10 @@
         <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J72" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K72">
         <v>0.0014224236350091</v>
@@ -21668,10 +21668,10 @@
         <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="J73" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K73">
         <v>0.0008003654809294</v>
@@ -21943,10 +21943,10 @@
         <v>72</v>
       </c>
       <c r="B74" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="J74" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="K74">
         <v>0.001155136088498</v>
@@ -22218,10 +22218,10 @@
         <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J75" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="K75">
         <v>0.001355651330368</v>
@@ -22493,10 +22493,10 @@
         <v>74</v>
       </c>
       <c r="B76" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="J76" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K76">
         <v>0.0007409682940759</v>
@@ -24668,6 +24668,278 @@
       </c>
       <c r="CU83">
         <v>-0.7661869296895436</v>
+      </c>
+    </row>
+    <row r="84" spans="1:99">
+      <c r="A84" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="J84" t="s">
+        <v>104</v>
+      </c>
+      <c r="K84">
+        <v>0.002638660691366201</v>
+      </c>
+      <c r="L84">
+        <v>0.001319330345683101</v>
+      </c>
+      <c r="M84">
+        <v>0.00127972002567045</v>
+      </c>
+      <c r="N84">
+        <v>0.00127972002567045</v>
+      </c>
+      <c r="O84">
+        <v>0.001811065451283778</v>
+      </c>
+      <c r="P84">
+        <v>0.0009055327256418888</v>
+      </c>
+      <c r="Q84">
+        <v>0.00120542104992718</v>
+      </c>
+      <c r="R84">
+        <v>0.00120542104992718</v>
+      </c>
+      <c r="S84">
+        <v>14.21628920868861</v>
+      </c>
+      <c r="T84">
+        <v>14.25980940622709</v>
+      </c>
+      <c r="U84">
+        <v>0.3726516823622893</v>
+      </c>
+      <c r="V84">
+        <v>0.5248393896377442</v>
+      </c>
+      <c r="W84">
+        <v>0.06735869831013411</v>
+      </c>
+      <c r="X84">
+        <v>0.09846212321720701</v>
+      </c>
+      <c r="Y84">
+        <v>0.2245726252191716</v>
+      </c>
+      <c r="Z84">
+        <v>0.2364561081292338</v>
+      </c>
+      <c r="AA84">
+        <v>0.998686831131235</v>
+      </c>
+      <c r="AB84">
+        <v>0.8279502967434699</v>
+      </c>
+      <c r="AC84">
+        <v>0.7956644460699689</v>
+      </c>
+      <c r="AD84">
+        <v>0.9978293798970223</v>
+      </c>
+      <c r="AE84">
+        <v>0.7757324464033544</v>
+      </c>
+      <c r="AF84">
+        <v>0.7635502252737323</v>
+      </c>
+      <c r="AG84">
+        <v>0.008096419998446866</v>
+      </c>
+      <c r="AH84">
+        <v>0.01101026659927736</v>
+      </c>
+      <c r="AI84">
+        <v>0.998686831131235</v>
+      </c>
+      <c r="AJ84">
+        <v>0.9978293798970223</v>
+      </c>
+      <c r="AK84">
+        <v>0.008096419998446866</v>
+      </c>
+      <c r="AL84">
+        <v>0.01101026659927736</v>
+      </c>
+      <c r="AM84" t="s">
+        <v>235</v>
+      </c>
+      <c r="AN84">
+        <v>0.02891294155673375</v>
+      </c>
+      <c r="AO84">
+        <v>0.05598633660165474</v>
+      </c>
+      <c r="AP84">
+        <v>-8425.582709600001</v>
+      </c>
+      <c r="AQ84">
+        <v>-1552.14576944</v>
+      </c>
+      <c r="AR84">
+        <v>172168.8488618802</v>
+      </c>
+      <c r="AS84">
+        <v>39795.18153056001</v>
+      </c>
+      <c r="AT84">
+        <v>172168.2800618802</v>
+      </c>
+      <c r="AU84">
+        <v>39732.68923056001</v>
+      </c>
+      <c r="AV84">
+        <v>16.21688488618802</v>
+      </c>
+      <c r="AW84">
+        <v>2.979518153056001</v>
+      </c>
+      <c r="AX84">
+        <v>1.687768151815181</v>
+      </c>
+      <c r="AY84">
+        <v>1.680365608156374</v>
+      </c>
+      <c r="AZ84">
+        <v>119.4166666666667</v>
+      </c>
+      <c r="BA84">
+        <v>111.35</v>
+      </c>
+      <c r="BB84">
+        <v>0</v>
+      </c>
+      <c r="BC84">
+        <v>0.02158773431953568</v>
+      </c>
+      <c r="BD84">
+        <v>0</v>
+      </c>
+      <c r="BE84">
+        <v>-691.6489062095777</v>
+      </c>
+      <c r="BF84">
+        <v>7124</v>
+      </c>
+      <c r="BG84">
+        <v>6727</v>
+      </c>
+      <c r="BH84">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI84">
+        <v>8229</v>
+      </c>
+      <c r="BJ84">
+        <v>8673</v>
+      </c>
+      <c r="BK84">
+        <v>15353</v>
+      </c>
+      <c r="BL84">
+        <v>15400</v>
+      </c>
+      <c r="BM84">
+        <v>6427</v>
+      </c>
+      <c r="BN84">
+        <v>6367</v>
+      </c>
+      <c r="BO84">
+        <v>7124</v>
+      </c>
+      <c r="BP84">
+        <v>6703</v>
+      </c>
+      <c r="BQ84">
+        <v>1802</v>
+      </c>
+      <c r="BR84">
+        <v>2306</v>
+      </c>
+      <c r="BS84">
+        <v>0</v>
+      </c>
+      <c r="BT84">
+        <v>24</v>
+      </c>
+      <c r="BU84">
+        <v>0</v>
+      </c>
+      <c r="BV84">
+        <v>0</v>
+      </c>
+      <c r="BW84">
+        <v>162184.0130903996</v>
+      </c>
+      <c r="BX84">
+        <v>29795.18153056</v>
+      </c>
+      <c r="BY84">
+        <v>0.0548054404427499</v>
+      </c>
+      <c r="BZ84">
+        <v>0.09018642574593751</v>
+      </c>
+      <c r="CA84">
+        <v>0.1262542343082536</v>
+      </c>
+      <c r="CB84">
+        <v>0.1912093402454063</v>
+      </c>
+      <c r="CC84">
+        <v>0.01338068051328788</v>
+      </c>
+      <c r="CD84">
+        <v>0.01746251592383252</v>
+      </c>
+      <c r="CE84">
+        <v>0.01111179224969334</v>
+      </c>
+      <c r="CF84">
+        <v>0.01392197242052187</v>
+      </c>
+      <c r="CG84">
+        <v>170609.5957999996</v>
+      </c>
+      <c r="CH84">
+        <v>31347.3273</v>
+      </c>
+      <c r="CI84">
+        <v>170609.5957999996</v>
+      </c>
+      <c r="CJ84">
+        <v>32038.97620620958</v>
+      </c>
+      <c r="CK84">
+        <v>0.08042047244351958</v>
+      </c>
+      <c r="CL84">
+        <v>0.127088106073291</v>
+      </c>
+      <c r="CM84">
+        <v>10000</v>
+      </c>
+      <c r="CO84">
+        <v>0.009452160493827161</v>
+      </c>
+      <c r="CP84">
+        <v>0.02029320987654321</v>
+      </c>
+      <c r="CQ84">
+        <v>67308493.07961167</v>
+      </c>
+      <c r="CR84">
+        <v>9017755.465507763</v>
+      </c>
+      <c r="CS84" s="2">
+        <v>45405.84478857185</v>
+      </c>
+      <c r="CT84">
+        <v>-0.641321453686593</v>
+      </c>
+      <c r="CU84">
+        <v>-0.7042240923869452</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ALGOUSDT.json at 2024-04-24_16-01-58 bestfile_scores 0.0009323985701347958 bestfile_sharp 0.23291520735270765
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU85"/>
+  <dimension ref="A1:CU86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -25254,6 +25254,275 @@
       </c>
       <c r="CU85">
         <v>-0.9921334262355667</v>
+      </c>
+    </row>
+    <row r="86" spans="1:99">
+      <c r="J86" t="s">
+        <v>207</v>
+      </c>
+      <c r="K86">
+        <v>0.000719801002360354</v>
+      </c>
+      <c r="L86">
+        <v>0.000359900501180177</v>
+      </c>
+      <c r="M86">
+        <v>0.000637401956996797</v>
+      </c>
+      <c r="N86">
+        <v>0.000637401956996797</v>
+      </c>
+      <c r="O86">
+        <v>0.0013183991269901</v>
+      </c>
+      <c r="P86">
+        <v>0.0006591995634950498</v>
+      </c>
+      <c r="Q86">
+        <v>0.0004523278044736845</v>
+      </c>
+      <c r="R86">
+        <v>0.0004523278044736845</v>
+      </c>
+      <c r="S86">
+        <v>18.74771191349681</v>
+      </c>
+      <c r="T86">
+        <v>4.577563236145974</v>
+      </c>
+      <c r="U86">
+        <v>0.4583932449374378</v>
+      </c>
+      <c r="V86">
+        <v>0.6162713998360264</v>
+      </c>
+      <c r="W86">
+        <v>0.00657175881030223</v>
+      </c>
+      <c r="X86">
+        <v>0.05057931728939506</v>
+      </c>
+      <c r="Y86">
+        <v>0.02483082236983788</v>
+      </c>
+      <c r="Z86">
+        <v>0.2324818094860823</v>
+      </c>
+      <c r="AA86">
+        <v>0.9998194243284108</v>
+      </c>
+      <c r="AB86">
+        <v>0.9792172343240961</v>
+      </c>
+      <c r="AC86">
+        <v>0.8025415429063898</v>
+      </c>
+      <c r="AD86">
+        <v>0.9992549900252792</v>
+      </c>
+      <c r="AE86">
+        <v>0.88501828738166</v>
+      </c>
+      <c r="AF86">
+        <v>0.7702115727040658</v>
+      </c>
+      <c r="AG86">
+        <v>0.0008157732201142562</v>
+      </c>
+      <c r="AH86">
+        <v>0.006933964625650903</v>
+      </c>
+      <c r="AI86">
+        <v>0.9998194243284108</v>
+      </c>
+      <c r="AJ86">
+        <v>0.9992549900252792</v>
+      </c>
+      <c r="AK86">
+        <v>0.0008157732201142562</v>
+      </c>
+      <c r="AL86">
+        <v>0.006933964625650903</v>
+      </c>
+      <c r="AM86" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN86">
+        <v>0.004679842077409701</v>
+      </c>
+      <c r="AO86">
+        <v>0.02024489568608402</v>
+      </c>
+      <c r="AP86">
+        <v>-957.645106786</v>
+      </c>
+      <c r="AQ86">
+        <v>-556.247589178</v>
+      </c>
+      <c r="AR86">
+        <v>21735.37256321382</v>
+      </c>
+      <c r="AS86">
+        <v>19887.59477082206</v>
+      </c>
+      <c r="AT86">
+        <v>21735.37256321382</v>
+      </c>
+      <c r="AU86">
+        <v>19863.54394082206</v>
+      </c>
+      <c r="AV86">
+        <v>1.173537256321382</v>
+      </c>
+      <c r="AW86">
+        <v>0.9887594770822064</v>
+      </c>
+      <c r="AX86">
+        <v>1.279440846393435</v>
+      </c>
+      <c r="AY86">
+        <v>5.233934116376401</v>
+      </c>
+      <c r="AZ86">
+        <v>116.9333333333333</v>
+      </c>
+      <c r="BA86">
+        <v>140.4833333333333</v>
+      </c>
+      <c r="BB86">
+        <v>2.244295838938429E-05</v>
+      </c>
+      <c r="BC86">
+        <v>0.03318049485384934</v>
+      </c>
+      <c r="BD86">
+        <v>-0.2848752608471553</v>
+      </c>
+      <c r="BE86">
+        <v>-358.4245620158542</v>
+      </c>
+      <c r="BF86">
+        <v>9772</v>
+      </c>
+      <c r="BG86">
+        <v>2599</v>
+      </c>
+      <c r="BH86">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI86">
+        <v>10456</v>
+      </c>
+      <c r="BJ86">
+        <v>2340</v>
+      </c>
+      <c r="BK86">
+        <v>20228</v>
+      </c>
+      <c r="BL86">
+        <v>4939</v>
+      </c>
+      <c r="BM86">
+        <v>9764</v>
+      </c>
+      <c r="BN86">
+        <v>2029</v>
+      </c>
+      <c r="BO86">
+        <v>9771</v>
+      </c>
+      <c r="BP86">
+        <v>2559</v>
+      </c>
+      <c r="BQ86">
+        <v>692</v>
+      </c>
+      <c r="BR86">
+        <v>311</v>
+      </c>
+      <c r="BS86">
+        <v>1</v>
+      </c>
+      <c r="BT86">
+        <v>40</v>
+      </c>
+      <c r="BU86">
+        <v>0</v>
+      </c>
+      <c r="BV86">
+        <v>0</v>
+      </c>
+      <c r="BW86">
+        <v>11735.37256321402</v>
+      </c>
+      <c r="BX86">
+        <v>9887.594770822006</v>
+      </c>
+      <c r="BY86">
+        <v>0.04920145046583688</v>
+      </c>
+      <c r="BZ86">
+        <v>0.08215959776497388</v>
+      </c>
+      <c r="CA86">
+        <v>0.06100216665928337</v>
+      </c>
+      <c r="CB86">
+        <v>0.2044290433384323</v>
+      </c>
+      <c r="CC86">
+        <v>0.01751584063849812</v>
+      </c>
+      <c r="CD86">
+        <v>0.01920326125056007</v>
+      </c>
+      <c r="CE86">
+        <v>0.01264241928644005</v>
+      </c>
+      <c r="CF86">
+        <v>0.01756754747362051</v>
+      </c>
+      <c r="CG86">
+        <v>12693.01767000002</v>
+      </c>
+      <c r="CH86">
+        <v>10443.84236000001</v>
+      </c>
+      <c r="CI86">
+        <v>12693.30254526086</v>
+      </c>
+      <c r="CJ86">
+        <v>10802.26692201586</v>
+      </c>
+      <c r="CK86">
+        <v>0.09397133728198301</v>
+      </c>
+      <c r="CL86">
+        <v>0.06430922481210541</v>
+      </c>
+      <c r="CM86">
+        <v>10000</v>
+      </c>
+      <c r="CO86">
+        <v>0</v>
+      </c>
+      <c r="CP86">
+        <v>0.007105344454742045</v>
+      </c>
+      <c r="CQ86">
+        <v>2851692.203283581</v>
+      </c>
+      <c r="CR86">
+        <v>5470308.140646266</v>
+      </c>
+      <c r="CS86" s="2">
+        <v>45406.40391306597</v>
+      </c>
+      <c r="CT86">
+        <v>-0.9414869172232342</v>
+      </c>
+      <c r="CU86">
+        <v>-0.7676228035631731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update TRXUSDT.json at 2024-04-24_22-50-03 bestfile_scores 0.00047670195575126025 bestfile_sharp 0.03541781069694058
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="944" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU86"/>
+  <dimension ref="A1:CU87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -25523,6 +25523,275 @@
       </c>
       <c r="CU86">
         <v>-0.7676228035631731</v>
+      </c>
+    </row>
+    <row r="87" spans="1:99">
+      <c r="J87" t="s">
+        <v>208</v>
+      </c>
+      <c r="K87">
+        <v>0.001624155024458451</v>
+      </c>
+      <c r="L87">
+        <v>0.0008120775122292256</v>
+      </c>
+      <c r="M87">
+        <v>0.001051197730107978</v>
+      </c>
+      <c r="N87">
+        <v>0.001051197730107978</v>
+      </c>
+      <c r="O87">
+        <v>0.001916401223087316</v>
+      </c>
+      <c r="P87">
+        <v>0.0009582006115436581</v>
+      </c>
+      <c r="Q87">
+        <v>0.000908118426658322</v>
+      </c>
+      <c r="R87">
+        <v>0.000908118426658322</v>
+      </c>
+      <c r="S87">
+        <v>16.18968912917552</v>
+      </c>
+      <c r="T87">
+        <v>19.06190384244063</v>
+      </c>
+      <c r="U87">
+        <v>0.3802594395960561</v>
+      </c>
+      <c r="V87">
+        <v>0.2613210782536639</v>
+      </c>
+      <c r="W87">
+        <v>0.02883657147746224</v>
+      </c>
+      <c r="X87">
+        <v>0.07291873600276512</v>
+      </c>
+      <c r="Y87">
+        <v>0.1504300536148817</v>
+      </c>
+      <c r="Z87">
+        <v>0.1527780010251412</v>
+      </c>
+      <c r="AA87">
+        <v>0.9994133334721068</v>
+      </c>
+      <c r="AB87">
+        <v>0.8817195160820253</v>
+      </c>
+      <c r="AC87">
+        <v>0.8603563337356448</v>
+      </c>
+      <c r="AD87">
+        <v>0.9982243188666013</v>
+      </c>
+      <c r="AE87">
+        <v>0.8287006246158564</v>
+      </c>
+      <c r="AF87">
+        <v>0.7551034210926815</v>
+      </c>
+      <c r="AG87">
+        <v>0.003669933078920623</v>
+      </c>
+      <c r="AH87">
+        <v>0.008430389570990215</v>
+      </c>
+      <c r="AI87">
+        <v>0.9994133334721068</v>
+      </c>
+      <c r="AJ87">
+        <v>0.9982243188666013</v>
+      </c>
+      <c r="AK87">
+        <v>0.003669933078920623</v>
+      </c>
+      <c r="AL87">
+        <v>0.008430389570990215</v>
+      </c>
+      <c r="AM87" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN87">
+        <v>0.02205487622276112</v>
+      </c>
+      <c r="AO87">
+        <v>0.05952022851450087</v>
+      </c>
+      <c r="AP87">
+        <v>-2418.036095292</v>
+      </c>
+      <c r="AQ87">
+        <v>-2251.408181426</v>
+      </c>
+      <c r="AR87">
+        <v>57602.10713259</v>
+      </c>
+      <c r="AS87">
+        <v>31068.29754857417</v>
+      </c>
+      <c r="AT87">
+        <v>57602.99060259001</v>
+      </c>
+      <c r="AU87">
+        <v>31045.27956857417</v>
+      </c>
+      <c r="AV87">
+        <v>4.760210713259</v>
+      </c>
+      <c r="AW87">
+        <v>2.106829754857417</v>
+      </c>
+      <c r="AX87">
+        <v>1.481718860327093</v>
+      </c>
+      <c r="AY87">
+        <v>1.25739651204253</v>
+      </c>
+      <c r="AZ87">
+        <v>91.75</v>
+      </c>
+      <c r="BA87">
+        <v>93.45</v>
+      </c>
+      <c r="BB87">
+        <v>0.05875303032050968</v>
+      </c>
+      <c r="BC87">
+        <v>0.03462616469254681</v>
+      </c>
+      <c r="BD87">
+        <v>-3122.576355556558</v>
+      </c>
+      <c r="BE87">
+        <v>-836.434489579409</v>
+      </c>
+      <c r="BF87">
+        <v>5956</v>
+      </c>
+      <c r="BG87">
+        <v>9208</v>
+      </c>
+      <c r="BH87">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI87">
+        <v>11512</v>
+      </c>
+      <c r="BJ87">
+        <v>11359</v>
+      </c>
+      <c r="BK87">
+        <v>17468</v>
+      </c>
+      <c r="BL87">
+        <v>20567</v>
+      </c>
+      <c r="BM87">
+        <v>5894</v>
+      </c>
+      <c r="BN87">
+        <v>8894</v>
+      </c>
+      <c r="BO87">
+        <v>5912</v>
+      </c>
+      <c r="BP87">
+        <v>9130</v>
+      </c>
+      <c r="BQ87">
+        <v>5618</v>
+      </c>
+      <c r="BR87">
+        <v>2465</v>
+      </c>
+      <c r="BS87">
+        <v>44</v>
+      </c>
+      <c r="BT87">
+        <v>78</v>
+      </c>
+      <c r="BU87">
+        <v>0</v>
+      </c>
+      <c r="BV87">
+        <v>0</v>
+      </c>
+      <c r="BW87">
+        <v>47606.88204470804</v>
+      </c>
+      <c r="BX87">
+        <v>21068.29754857396</v>
+      </c>
+      <c r="BY87">
+        <v>0.0321269761468897</v>
+      </c>
+      <c r="BZ87">
+        <v>0.0747313262752913</v>
+      </c>
+      <c r="CA87">
+        <v>0.08122410679064272</v>
+      </c>
+      <c r="CB87">
+        <v>0.1324687469813762</v>
+      </c>
+      <c r="CC87">
+        <v>0.0107549236807208</v>
+      </c>
+      <c r="CD87">
+        <v>0.01188640490787263</v>
+      </c>
+      <c r="CE87">
+        <v>0.007744210937119617</v>
+      </c>
+      <c r="CF87">
+        <v>0.01244205564162896</v>
+      </c>
+      <c r="CG87">
+        <v>50024.91814000005</v>
+      </c>
+      <c r="CH87">
+        <v>23319.70572999996</v>
+      </c>
+      <c r="CI87">
+        <v>53147.4944955566</v>
+      </c>
+      <c r="CJ87">
+        <v>24156.14021957937</v>
+      </c>
+      <c r="CK87">
+        <v>0.2329152073527077</v>
+      </c>
+      <c r="CL87">
+        <v>0.1243263724852883</v>
+      </c>
+      <c r="CM87">
+        <v>10000</v>
+      </c>
+      <c r="CO87">
+        <v>0.002355576150756874</v>
+      </c>
+      <c r="CP87">
+        <v>0.02038924930491195</v>
+      </c>
+      <c r="CQ87">
+        <v>25347102.27661829</v>
+      </c>
+      <c r="CR87">
+        <v>10570112.91971009</v>
+      </c>
+      <c r="CS87" s="2">
+        <v>45406.66806319206</v>
+      </c>
+      <c r="CT87">
+        <v>-0.8207903291654746</v>
+      </c>
+      <c r="CU87">
+        <v>-0.7904342151277074</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ALPHAUSDT.json at 2024-04-25_03-14-25 bestfile_scores 0.00028485309351874153 bestfile_sharp 0.07099934652871313
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="946" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU87"/>
+  <dimension ref="A1:CU88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -25792,6 +25792,275 @@
       </c>
       <c r="CU87">
         <v>-0.7904342151277074</v>
+      </c>
+    </row>
+    <row r="88" spans="1:99">
+      <c r="J88" t="s">
+        <v>209</v>
+      </c>
+      <c r="K88">
+        <v>0.001951100188842814</v>
+      </c>
+      <c r="L88">
+        <v>0.0009755500944214068</v>
+      </c>
+      <c r="M88">
+        <v>0.0004361834836490441</v>
+      </c>
+      <c r="N88">
+        <v>0.0004361834836490441</v>
+      </c>
+      <c r="O88">
+        <v>0.000552609306919627</v>
+      </c>
+      <c r="P88">
+        <v>0.0002763046534598135</v>
+      </c>
+      <c r="Q88">
+        <v>0.0002187695914747767</v>
+      </c>
+      <c r="R88">
+        <v>0.0002187695914747767</v>
+      </c>
+      <c r="S88">
+        <v>35.90416296925036</v>
+      </c>
+      <c r="T88">
+        <v>8.846637601759328</v>
+      </c>
+      <c r="U88">
+        <v>0.4147199697740905</v>
+      </c>
+      <c r="V88">
+        <v>0.8170853037821222</v>
+      </c>
+      <c r="W88">
+        <v>0.09104593447847015</v>
+      </c>
+      <c r="X88">
+        <v>0.04307341288567829</v>
+      </c>
+      <c r="Y88">
+        <v>0.1675266118164311</v>
+      </c>
+      <c r="Z88">
+        <v>0.09129972272437749</v>
+      </c>
+      <c r="AA88">
+        <v>0.9979024079376395</v>
+      </c>
+      <c r="AB88">
+        <v>0.8435441426189658</v>
+      </c>
+      <c r="AC88">
+        <v>0.9336163213380239</v>
+      </c>
+      <c r="AD88">
+        <v>0.9987761683940237</v>
+      </c>
+      <c r="AE88">
+        <v>0.8334748408071527</v>
+      </c>
+      <c r="AF88">
+        <v>0.9087457883974269</v>
+      </c>
+      <c r="AG88">
+        <v>0.01115713454172098</v>
+      </c>
+      <c r="AH88">
+        <v>0.004685861692206245</v>
+      </c>
+      <c r="AI88">
+        <v>0.9979024079376395</v>
+      </c>
+      <c r="AJ88">
+        <v>0.9987761683940237</v>
+      </c>
+      <c r="AK88">
+        <v>0.01115713454172098</v>
+      </c>
+      <c r="AL88">
+        <v>0.004685861692206245</v>
+      </c>
+      <c r="AM88" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN88">
+        <v>0.05149354256962412</v>
+      </c>
+      <c r="AO88">
+        <v>0.05893934496251729</v>
+      </c>
+      <c r="AP88">
+        <v>-8770.210119714</v>
+      </c>
+      <c r="AQ88">
+        <v>-290.529522364</v>
+      </c>
+      <c r="AR88">
+        <v>82075.46120028623</v>
+      </c>
+      <c r="AS88">
+        <v>16015.26574763606</v>
+      </c>
+      <c r="AT88">
+        <v>82072.27956028623</v>
+      </c>
+      <c r="AU88">
+        <v>15995.40830763606</v>
+      </c>
+      <c r="AV88">
+        <v>7.207546120028622</v>
+      </c>
+      <c r="AW88">
+        <v>0.6015265747636063</v>
+      </c>
+      <c r="AX88">
+        <v>0.6681466102714878</v>
+      </c>
+      <c r="AY88">
+        <v>2.710380683205974</v>
+      </c>
+      <c r="AZ88">
+        <v>82.55</v>
+      </c>
+      <c r="BA88">
+        <v>166.3166666666667</v>
+      </c>
+      <c r="BB88">
+        <v>0.00204112613254108</v>
+      </c>
+      <c r="BC88">
+        <v>0.1258734590673847</v>
+      </c>
+      <c r="BD88">
+        <v>-165.3537202335606</v>
+      </c>
+      <c r="BE88">
+        <v>-908.0290159806948</v>
+      </c>
+      <c r="BF88">
+        <v>17223</v>
+      </c>
+      <c r="BG88">
+        <v>2408</v>
+      </c>
+      <c r="BH88">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI88">
+        <v>21552</v>
+      </c>
+      <c r="BJ88">
+        <v>7146</v>
+      </c>
+      <c r="BK88">
+        <v>38775</v>
+      </c>
+      <c r="BL88">
+        <v>9554</v>
+      </c>
+      <c r="BM88">
+        <v>16770</v>
+      </c>
+      <c r="BN88">
+        <v>2365</v>
+      </c>
+      <c r="BO88">
+        <v>17125</v>
+      </c>
+      <c r="BP88">
+        <v>2388</v>
+      </c>
+      <c r="BQ88">
+        <v>4782</v>
+      </c>
+      <c r="BR88">
+        <v>4781</v>
+      </c>
+      <c r="BS88">
+        <v>98</v>
+      </c>
+      <c r="BT88">
+        <v>20</v>
+      </c>
+      <c r="BU88">
+        <v>0</v>
+      </c>
+      <c r="BV88">
+        <v>0</v>
+      </c>
+      <c r="BW88">
+        <v>72075.46120028601</v>
+      </c>
+      <c r="BX88">
+        <v>6015.265747635984</v>
+      </c>
+      <c r="BY88">
+        <v>0.04712604707456167</v>
+      </c>
+      <c r="BZ88">
+        <v>0.04379688717384538</v>
+      </c>
+      <c r="CA88">
+        <v>0.09048708205366365</v>
+      </c>
+      <c r="CB88">
+        <v>0.08362306487729781</v>
+      </c>
+      <c r="CC88">
+        <v>0.006997698323338252</v>
+      </c>
+      <c r="CD88">
+        <v>0.01081197607590412</v>
+      </c>
+      <c r="CE88">
+        <v>0.006543541917764676</v>
+      </c>
+      <c r="CF88">
+        <v>0.007632383834101261</v>
+      </c>
+      <c r="CG88">
+        <v>80845.67132000001</v>
+      </c>
+      <c r="CH88">
+        <v>6305.795269999983</v>
+      </c>
+      <c r="CI88">
+        <v>81011.02504023357</v>
+      </c>
+      <c r="CJ88">
+        <v>7213.824285980678</v>
+      </c>
+      <c r="CK88">
+        <v>0.03541781069694058</v>
+      </c>
+      <c r="CL88">
+        <v>0.07839911226633609</v>
+      </c>
+      <c r="CM88">
+        <v>10000</v>
+      </c>
+      <c r="CO88">
+        <v>0.03919753086419753</v>
+      </c>
+      <c r="CP88">
+        <v>0.007330246913580247</v>
+      </c>
+      <c r="CQ88">
+        <v>65046152.47826129</v>
+      </c>
+      <c r="CR88">
+        <v>5725644.496349121</v>
+      </c>
+      <c r="CS88" s="2">
+        <v>45406.95144454927</v>
+      </c>
+      <c r="CT88">
+        <v>-0.561712415905279</v>
+      </c>
+      <c r="CU88">
+        <v>-0.8810999866388021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update DOTUSDT.json at 2024-04-25_10-14-59 bestfile_scores 0.0005331148753909055 bestfile_sharp 0.1914875660755673
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU88"/>
+  <dimension ref="A1:CU89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -26061,6 +26061,275 @@
       </c>
       <c r="CU88">
         <v>-0.8810999866388021</v>
+      </c>
+    </row>
+    <row r="89" spans="1:99">
+      <c r="J89" t="s">
+        <v>210</v>
+      </c>
+      <c r="K89">
+        <v>0.000345514979697592</v>
+      </c>
+      <c r="L89">
+        <v>0.000172757489848796</v>
+      </c>
+      <c r="M89">
+        <v>0.0004188519801897606</v>
+      </c>
+      <c r="N89">
+        <v>0.0004188519801897606</v>
+      </c>
+      <c r="O89">
+        <v>0.0003504759606676844</v>
+      </c>
+      <c r="P89">
+        <v>0.0001752379803338422</v>
+      </c>
+      <c r="Q89">
+        <v>0.0003725649237025674</v>
+      </c>
+      <c r="R89">
+        <v>0.0003725649237025674</v>
+      </c>
+      <c r="S89">
+        <v>9.694818472934914</v>
+      </c>
+      <c r="T89">
+        <v>8.337358694394075</v>
+      </c>
+      <c r="U89">
+        <v>0.785622210643986</v>
+      </c>
+      <c r="V89">
+        <v>0.3531398136783446</v>
+      </c>
+      <c r="W89">
+        <v>0.04777185505613632</v>
+      </c>
+      <c r="X89">
+        <v>0.0276333107701373</v>
+      </c>
+      <c r="Y89">
+        <v>0.2498925884880395</v>
+      </c>
+      <c r="Z89">
+        <v>0.1730721018834004</v>
+      </c>
+      <c r="AA89">
+        <v>0.9987374559444938</v>
+      </c>
+      <c r="AB89">
+        <v>0.9060789840452804</v>
+      </c>
+      <c r="AC89">
+        <v>0.8644157745489677</v>
+      </c>
+      <c r="AD89">
+        <v>0.9995026615670642</v>
+      </c>
+      <c r="AE89">
+        <v>0.6304052078287954</v>
+      </c>
+      <c r="AF89">
+        <v>0.8270933050451624</v>
+      </c>
+      <c r="AG89">
+        <v>0.005738986784779263</v>
+      </c>
+      <c r="AH89">
+        <v>0.003993921576659855</v>
+      </c>
+      <c r="AI89">
+        <v>0.9987374559444938</v>
+      </c>
+      <c r="AJ89">
+        <v>0.9995026615670642</v>
+      </c>
+      <c r="AK89">
+        <v>0.005738986784779263</v>
+      </c>
+      <c r="AL89">
+        <v>0.003993921576659855</v>
+      </c>
+      <c r="AM89" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN89">
+        <v>0.01222205876457107</v>
+      </c>
+      <c r="AO89">
+        <v>0.01516571123341925</v>
+      </c>
+      <c r="AP89">
+        <v>-505.904061722</v>
+      </c>
+      <c r="AQ89">
+        <v>-296.465975534</v>
+      </c>
+      <c r="AR89">
+        <v>14521.96638827791</v>
+      </c>
+      <c r="AS89">
+        <v>15718.41686446591</v>
+      </c>
+      <c r="AT89">
+        <v>14521.96638827791</v>
+      </c>
+      <c r="AU89">
+        <v>15717.82943446592</v>
+      </c>
+      <c r="AV89">
+        <v>0.4521966388277914</v>
+      </c>
+      <c r="AW89">
+        <v>0.5718416864465914</v>
+      </c>
+      <c r="AX89">
+        <v>2.473275066068074</v>
+      </c>
+      <c r="AY89">
+        <v>2.874671405827687</v>
+      </c>
+      <c r="AZ89">
+        <v>118.2</v>
+      </c>
+      <c r="BA89">
+        <v>105.85</v>
+      </c>
+      <c r="BB89">
+        <v>0</v>
+      </c>
+      <c r="BC89">
+        <v>0.01080387928835819</v>
+      </c>
+      <c r="BD89">
+        <v>0</v>
+      </c>
+      <c r="BE89">
+        <v>-65.6938161971628</v>
+      </c>
+      <c r="BF89">
+        <v>4766</v>
+      </c>
+      <c r="BG89">
+        <v>3632</v>
+      </c>
+      <c r="BH89">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI89">
+        <v>5704</v>
+      </c>
+      <c r="BJ89">
+        <v>5372</v>
+      </c>
+      <c r="BK89">
+        <v>10470</v>
+      </c>
+      <c r="BL89">
+        <v>9004</v>
+      </c>
+      <c r="BM89">
+        <v>4757</v>
+      </c>
+      <c r="BN89">
+        <v>3567</v>
+      </c>
+      <c r="BO89">
+        <v>4766</v>
+      </c>
+      <c r="BP89">
+        <v>3630</v>
+      </c>
+      <c r="BQ89">
+        <v>947</v>
+      </c>
+      <c r="BR89">
+        <v>1805</v>
+      </c>
+      <c r="BS89">
+        <v>0</v>
+      </c>
+      <c r="BT89">
+        <v>2</v>
+      </c>
+      <c r="BU89">
+        <v>0</v>
+      </c>
+      <c r="BV89">
+        <v>0</v>
+      </c>
+      <c r="BW89">
+        <v>4521.966388278002</v>
+      </c>
+      <c r="BX89">
+        <v>5718.416864466</v>
+      </c>
+      <c r="BY89">
+        <v>0.123292181954453</v>
+      </c>
+      <c r="BZ89">
+        <v>0.07700249077917144</v>
+      </c>
+      <c r="CA89">
+        <v>0.3289185936591047</v>
+      </c>
+      <c r="CB89">
+        <v>0.1937089202640401</v>
+      </c>
+      <c r="CC89">
+        <v>0.02907279399408242</v>
+      </c>
+      <c r="CD89">
+        <v>0.01246025811077574</v>
+      </c>
+      <c r="CE89">
+        <v>0.02513362567230389</v>
+      </c>
+      <c r="CF89">
+        <v>0.01423019557634262</v>
+      </c>
+      <c r="CG89">
+        <v>5027.870450000002</v>
+      </c>
+      <c r="CH89">
+        <v>6014.88284</v>
+      </c>
+      <c r="CI89">
+        <v>5027.870450000002</v>
+      </c>
+      <c r="CJ89">
+        <v>6080.576656197163</v>
+      </c>
+      <c r="CK89">
+        <v>0.07099934652871313</v>
+      </c>
+      <c r="CL89">
+        <v>0.1223424692253783</v>
+      </c>
+      <c r="CM89">
+        <v>10000</v>
+      </c>
+      <c r="CO89">
+        <v>0</v>
+      </c>
+      <c r="CP89">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="CQ89">
+        <v>2347413.70669186</v>
+      </c>
+      <c r="CR89">
+        <v>1429804.32644608</v>
+      </c>
+      <c r="CS89" s="2">
+        <v>45407.13503203569</v>
+      </c>
+      <c r="CT89">
+        <v>-0.9176379634509605</v>
+      </c>
+      <c r="CU89">
+        <v>-0.9519924246039231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update BNBUSDT.json at 2024-04-25_13-26-24 bestfile_scores 0.0006084488908330382 bestfile_sharp 0.07768922232911872
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU89"/>
+  <dimension ref="A1:CU90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -26330,6 +26330,275 @@
       </c>
       <c r="CU89">
         <v>-0.9519924246039231</v>
+      </c>
+    </row>
+    <row r="90" spans="1:99">
+      <c r="J90" t="s">
+        <v>211</v>
+      </c>
+      <c r="K90">
+        <v>0.0008756469377746434</v>
+      </c>
+      <c r="L90">
+        <v>0.0004378234688873217</v>
+      </c>
+      <c r="M90">
+        <v>0.0007190461570929507</v>
+      </c>
+      <c r="N90">
+        <v>0.0007190461570929507</v>
+      </c>
+      <c r="O90">
+        <v>0.000699412291548862</v>
+      </c>
+      <c r="P90">
+        <v>0.000349706145774431</v>
+      </c>
+      <c r="Q90">
+        <v>0.0006258837298089182</v>
+      </c>
+      <c r="R90">
+        <v>0.0006258837298089182</v>
+      </c>
+      <c r="S90">
+        <v>15.82452210851516</v>
+      </c>
+      <c r="T90">
+        <v>22.10650704769261</v>
+      </c>
+      <c r="U90">
+        <v>0.2017754151508146</v>
+      </c>
+      <c r="V90">
+        <v>0.7668742582283157</v>
+      </c>
+      <c r="W90">
+        <v>0.02594764317832158</v>
+      </c>
+      <c r="X90">
+        <v>0.03376262774361775</v>
+      </c>
+      <c r="Y90">
+        <v>0.2445223406477499</v>
+      </c>
+      <c r="Z90">
+        <v>0.1220461898359423</v>
+      </c>
+      <c r="AA90">
+        <v>0.9993058097321195</v>
+      </c>
+      <c r="AB90">
+        <v>0.8482608240318938</v>
+      </c>
+      <c r="AC90">
+        <v>0.9234170423947164</v>
+      </c>
+      <c r="AD90">
+        <v>0.9989578178398208</v>
+      </c>
+      <c r="AE90">
+        <v>0.7424683830885809</v>
+      </c>
+      <c r="AF90">
+        <v>0.8780287691666064</v>
+      </c>
+      <c r="AG90">
+        <v>0.004015493407745043</v>
+      </c>
+      <c r="AH90">
+        <v>0.004208875897774582</v>
+      </c>
+      <c r="AI90">
+        <v>0.9993058097321195</v>
+      </c>
+      <c r="AJ90">
+        <v>0.9989578178398208</v>
+      </c>
+      <c r="AK90">
+        <v>0.004015493407745043</v>
+      </c>
+      <c r="AL90">
+        <v>0.004208875897774582</v>
+      </c>
+      <c r="AM90" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN90">
+        <v>0.01993903091124403</v>
+      </c>
+      <c r="AO90">
+        <v>0.04435378584014773</v>
+      </c>
+      <c r="AP90">
+        <v>-1081.84641128</v>
+      </c>
+      <c r="AQ90">
+        <v>-981.8358141200001</v>
+      </c>
+      <c r="AR90">
+        <v>25712.01121441974</v>
+      </c>
+      <c r="AS90">
+        <v>21717.69018588066</v>
+      </c>
+      <c r="AT90">
+        <v>25698.97261441974</v>
+      </c>
+      <c r="AU90">
+        <v>21717.76518588066</v>
+      </c>
+      <c r="AV90">
+        <v>1.571201121441974</v>
+      </c>
+      <c r="AW90">
+        <v>1.171769018588066</v>
+      </c>
+      <c r="AX90">
+        <v>1.515448368769402</v>
+      </c>
+      <c r="AY90">
+        <v>1.084869257752994</v>
+      </c>
+      <c r="AZ90">
+        <v>90.13333333333334</v>
+      </c>
+      <c r="BA90">
+        <v>97.34999999999999</v>
+      </c>
+      <c r="BB90">
+        <v>0.008355052366600437</v>
+      </c>
+      <c r="BC90">
+        <v>0.02407995277807922</v>
+      </c>
+      <c r="BD90">
+        <v>-141.495306703019</v>
+      </c>
+      <c r="BE90">
+        <v>-313.3494257593116</v>
+      </c>
+      <c r="BF90">
+        <v>6688</v>
+      </c>
+      <c r="BG90">
+        <v>10299</v>
+      </c>
+      <c r="BH90">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI90">
+        <v>10386</v>
+      </c>
+      <c r="BJ90">
+        <v>13553</v>
+      </c>
+      <c r="BK90">
+        <v>17074</v>
+      </c>
+      <c r="BL90">
+        <v>23852</v>
+      </c>
+      <c r="BM90">
+        <v>6560</v>
+      </c>
+      <c r="BN90">
+        <v>10016</v>
+      </c>
+      <c r="BO90">
+        <v>6683</v>
+      </c>
+      <c r="BP90">
+        <v>10286</v>
+      </c>
+      <c r="BQ90">
+        <v>3826</v>
+      </c>
+      <c r="BR90">
+        <v>3537</v>
+      </c>
+      <c r="BS90">
+        <v>5</v>
+      </c>
+      <c r="BT90">
+        <v>13</v>
+      </c>
+      <c r="BU90">
+        <v>0</v>
+      </c>
+      <c r="BV90">
+        <v>0</v>
+      </c>
+      <c r="BW90">
+        <v>15711.95688871998</v>
+      </c>
+      <c r="BX90">
+        <v>11717.69018587999</v>
+      </c>
+      <c r="BY90">
+        <v>0.04566966227758523</v>
+      </c>
+      <c r="BZ90">
+        <v>0.06310609304114541</v>
+      </c>
+      <c r="CA90">
+        <v>0.138839632515019</v>
+      </c>
+      <c r="CB90">
+        <v>0.1087017396169696</v>
+      </c>
+      <c r="CC90">
+        <v>0.009785696885523155</v>
+      </c>
+      <c r="CD90">
+        <v>0.009562698974271314</v>
+      </c>
+      <c r="CE90">
+        <v>0.008159381925781374</v>
+      </c>
+      <c r="CF90">
+        <v>0.009404092876252964</v>
+      </c>
+      <c r="CG90">
+        <v>16793.80329999998</v>
+      </c>
+      <c r="CH90">
+        <v>12699.52599999999</v>
+      </c>
+      <c r="CI90">
+        <v>16935.298606703</v>
+      </c>
+      <c r="CJ90">
+        <v>13012.8754257593</v>
+      </c>
+      <c r="CK90">
+        <v>0.1914875660755673</v>
+      </c>
+      <c r="CL90">
+        <v>0.1414721828491605</v>
+      </c>
+      <c r="CM90">
+        <v>10000</v>
+      </c>
+      <c r="CO90">
+        <v>0.0001930800123571208</v>
+      </c>
+      <c r="CP90">
+        <v>0.004595304294099475</v>
+      </c>
+      <c r="CQ90">
+        <v>6695372.633398985</v>
+      </c>
+      <c r="CR90">
+        <v>4722406.067514317</v>
+      </c>
+      <c r="CS90" s="2">
+        <v>45407.42709660172</v>
+      </c>
+      <c r="CT90">
+        <v>-0.9278452363120948</v>
+      </c>
+      <c r="CU90">
+        <v>-0.8892615252973167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update NEARUSDT.json at 2024-04-25_17-12-43 bestfile_scores 0.0005582132883607066 bestfile_sharp 0.1406503759723267
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU90"/>
+  <dimension ref="A1:CU91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -26599,6 +26599,275 @@
       </c>
       <c r="CU90">
         <v>-0.8892615252973167</v>
+      </c>
+    </row>
+    <row r="91" spans="1:99">
+      <c r="J91" t="s">
+        <v>212</v>
+      </c>
+      <c r="K91">
+        <v>0.001948887318000692</v>
+      </c>
+      <c r="L91">
+        <v>0.0009744436590003458</v>
+      </c>
+      <c r="M91">
+        <v>0.0004303003853498577</v>
+      </c>
+      <c r="N91">
+        <v>0.0004303003853498577</v>
+      </c>
+      <c r="O91">
+        <v>0.001203436898563637</v>
+      </c>
+      <c r="P91">
+        <v>0.0006017184492818183</v>
+      </c>
+      <c r="Q91">
+        <v>0.000427333069700131</v>
+      </c>
+      <c r="R91">
+        <v>0.000427333069700131</v>
+      </c>
+      <c r="S91">
+        <v>13.73849299741502</v>
+      </c>
+      <c r="T91">
+        <v>9.195725143716965</v>
+      </c>
+      <c r="U91">
+        <v>0.3790723163683974</v>
+      </c>
+      <c r="V91">
+        <v>0.7772121617424494</v>
+      </c>
+      <c r="W91">
+        <v>0.0154512178498121</v>
+      </c>
+      <c r="X91">
+        <v>0.08078635804422347</v>
+      </c>
+      <c r="Y91">
+        <v>0.2432533784607171</v>
+      </c>
+      <c r="Z91">
+        <v>0.1197389404776264</v>
+      </c>
+      <c r="AA91">
+        <v>0.9997653065443706</v>
+      </c>
+      <c r="AB91">
+        <v>0.8515329665424067</v>
+      </c>
+      <c r="AC91">
+        <v>0.8866436871596282</v>
+      </c>
+      <c r="AD91">
+        <v>0.9985381705305694</v>
+      </c>
+      <c r="AE91">
+        <v>0.7553505825879112</v>
+      </c>
+      <c r="AF91">
+        <v>0.8806206630839274</v>
+      </c>
+      <c r="AG91">
+        <v>0.003644361140770225</v>
+      </c>
+      <c r="AH91">
+        <v>0.009060300267909488</v>
+      </c>
+      <c r="AI91">
+        <v>0.9997653065443706</v>
+      </c>
+      <c r="AJ91">
+        <v>0.9985381705305694</v>
+      </c>
+      <c r="AK91">
+        <v>0.003644361140770225</v>
+      </c>
+      <c r="AL91">
+        <v>0.009060300267909488</v>
+      </c>
+      <c r="AM91" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN91">
+        <v>0.01303355243598029</v>
+      </c>
+      <c r="AO91">
+        <v>0.04664074832858237</v>
+      </c>
+      <c r="AP91">
+        <v>-4761.432402603999</v>
+      </c>
+      <c r="AQ91">
+        <v>-477.10161386</v>
+      </c>
+      <c r="AR91">
+        <v>81879.93159485537</v>
+      </c>
+      <c r="AS91">
+        <v>15913.87908614014</v>
+      </c>
+      <c r="AT91">
+        <v>81875.92719485537</v>
+      </c>
+      <c r="AU91">
+        <v>15913.74258614014</v>
+      </c>
+      <c r="AV91">
+        <v>7.187993159485536</v>
+      </c>
+      <c r="AW91">
+        <v>0.5913879086140146</v>
+      </c>
+      <c r="AX91">
+        <v>1.744735777837692</v>
+      </c>
+      <c r="AY91">
+        <v>2.607383350117489</v>
+      </c>
+      <c r="AZ91">
+        <v>112.1</v>
+      </c>
+      <c r="BA91">
+        <v>112.7</v>
+      </c>
+      <c r="BB91">
+        <v>0.002817071625238198</v>
+      </c>
+      <c r="BC91">
+        <v>0.04674747718068686</v>
+      </c>
+      <c r="BD91">
+        <v>-216.53243045216</v>
+      </c>
+      <c r="BE91">
+        <v>-313.413515604291</v>
+      </c>
+      <c r="BF91">
+        <v>5090</v>
+      </c>
+      <c r="BG91">
+        <v>3721</v>
+      </c>
+      <c r="BH91">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI91">
+        <v>9747</v>
+      </c>
+      <c r="BJ91">
+        <v>6210</v>
+      </c>
+      <c r="BK91">
+        <v>14837</v>
+      </c>
+      <c r="BL91">
+        <v>9931</v>
+      </c>
+      <c r="BM91">
+        <v>4954</v>
+      </c>
+      <c r="BN91">
+        <v>3687</v>
+      </c>
+      <c r="BO91">
+        <v>4980</v>
+      </c>
+      <c r="BP91">
+        <v>3686</v>
+      </c>
+      <c r="BQ91">
+        <v>4793</v>
+      </c>
+      <c r="BR91">
+        <v>2523</v>
+      </c>
+      <c r="BS91">
+        <v>110</v>
+      </c>
+      <c r="BT91">
+        <v>35</v>
+      </c>
+      <c r="BU91">
+        <v>0</v>
+      </c>
+      <c r="BV91">
+        <v>0</v>
+      </c>
+      <c r="BW91">
+        <v>71886.40329739601</v>
+      </c>
+      <c r="BX91">
+        <v>5913.879086140008</v>
+      </c>
+      <c r="BY91">
+        <v>0.0196277116121691</v>
+      </c>
+      <c r="BZ91">
+        <v>0.0726977021545096</v>
+      </c>
+      <c r="CA91">
+        <v>0.1383826142690789</v>
+      </c>
+      <c r="CB91">
+        <v>0.1066255581236546</v>
+      </c>
+      <c r="CC91">
+        <v>0.005188438409837917</v>
+      </c>
+      <c r="CD91">
+        <v>0.007068375658577656</v>
+      </c>
+      <c r="CE91">
+        <v>0.004689981969634566</v>
+      </c>
+      <c r="CF91">
+        <v>0.009911989499410225</v>
+      </c>
+      <c r="CG91">
+        <v>76647.83570000001</v>
+      </c>
+      <c r="CH91">
+        <v>6390.980700000008</v>
+      </c>
+      <c r="CI91">
+        <v>76864.36813045217</v>
+      </c>
+      <c r="CJ91">
+        <v>6704.394215604299</v>
+      </c>
+      <c r="CK91">
+        <v>0.07768922232911872</v>
+      </c>
+      <c r="CL91">
+        <v>0.05864366153782942</v>
+      </c>
+      <c r="CM91">
+        <v>10000</v>
+      </c>
+      <c r="CO91">
+        <v>0.002083333333333333</v>
+      </c>
+      <c r="CP91">
+        <v>0.02986111111111111</v>
+      </c>
+      <c r="CQ91">
+        <v>42240364.06965576</v>
+      </c>
+      <c r="CR91">
+        <v>2899232.912138085</v>
+      </c>
+      <c r="CS91" s="2">
+        <v>45407.56002666696</v>
+      </c>
+      <c r="CT91">
+        <v>-0.8179686291978085</v>
+      </c>
+      <c r="CU91">
+        <v>-0.8477823365237495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update OMGUSDT.json at 2024-04-25_22-58-30 bestfile_scores 0.0012997716641754836 bestfile_sharp 0.17253138556708225
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU91"/>
+  <dimension ref="A1:CU92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -26868,6 +26868,275 @@
       </c>
       <c r="CU91">
         <v>-0.8477823365237495</v>
+      </c>
+    </row>
+    <row r="92" spans="1:99">
+      <c r="J92" t="s">
+        <v>213</v>
+      </c>
+      <c r="K92">
+        <v>0.001089776280603916</v>
+      </c>
+      <c r="L92">
+        <v>0.0005448881403019579</v>
+      </c>
+      <c r="M92">
+        <v>0.0004368410351580643</v>
+      </c>
+      <c r="N92">
+        <v>0.0004368410351580643</v>
+      </c>
+      <c r="O92">
+        <v>0.001567206405684973</v>
+      </c>
+      <c r="P92">
+        <v>0.0007836032028424866</v>
+      </c>
+      <c r="Q92">
+        <v>0.0004675207751403176</v>
+      </c>
+      <c r="R92">
+        <v>0.0004675207751403176</v>
+      </c>
+      <c r="S92">
+        <v>54.31320652802963</v>
+      </c>
+      <c r="T92">
+        <v>11.49025811180987</v>
+      </c>
+      <c r="U92">
+        <v>0.3326157401522471</v>
+      </c>
+      <c r="V92">
+        <v>0.5453067833644851</v>
+      </c>
+      <c r="W92">
+        <v>0.05708149232224951</v>
+      </c>
+      <c r="X92">
+        <v>0.02617880608410247</v>
+      </c>
+      <c r="Y92">
+        <v>0.1486995593659856</v>
+      </c>
+      <c r="Z92">
+        <v>0.2493525993897033</v>
+      </c>
+      <c r="AA92">
+        <v>0.9988313662268823</v>
+      </c>
+      <c r="AB92">
+        <v>0.8727414674897824</v>
+      </c>
+      <c r="AC92">
+        <v>0.9226903960618744</v>
+      </c>
+      <c r="AD92">
+        <v>0.9992978112478876</v>
+      </c>
+      <c r="AE92">
+        <v>0.8529386319575794</v>
+      </c>
+      <c r="AF92">
+        <v>0.6698350846733409</v>
+      </c>
+      <c r="AG92">
+        <v>0.006385670264302784</v>
+      </c>
+      <c r="AH92">
+        <v>0.003427885323264733</v>
+      </c>
+      <c r="AI92">
+        <v>0.9988313662268823</v>
+      </c>
+      <c r="AJ92">
+        <v>0.9992978112478876</v>
+      </c>
+      <c r="AK92">
+        <v>0.006385670264302784</v>
+      </c>
+      <c r="AL92">
+        <v>0.003427885323264733</v>
+      </c>
+      <c r="AM92" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN92">
+        <v>0.02672263152296682</v>
+      </c>
+      <c r="AO92">
+        <v>0.0220624049464632</v>
+      </c>
+      <c r="AP92">
+        <v>-3655.3825404</v>
+      </c>
+      <c r="AQ92">
+        <v>-365.34624272</v>
+      </c>
+      <c r="AR92">
+        <v>32422.64985960016</v>
+      </c>
+      <c r="AS92">
+        <v>16026.6377132799</v>
+      </c>
+      <c r="AT92">
+        <v>32399.07385960016</v>
+      </c>
+      <c r="AU92">
+        <v>16026.6377132799</v>
+      </c>
+      <c r="AV92">
+        <v>2.242264985960016</v>
+      </c>
+      <c r="AW92">
+        <v>0.6026637713279897</v>
+      </c>
+      <c r="AX92">
+        <v>0.44167959537408</v>
+      </c>
+      <c r="AY92">
+        <v>2.085912314635719</v>
+      </c>
+      <c r="AZ92">
+        <v>82.11666666666666</v>
+      </c>
+      <c r="BA92">
+        <v>98.8</v>
+      </c>
+      <c r="BB92">
+        <v>0.005782246374329844</v>
+      </c>
+      <c r="BC92">
+        <v>0.007992930888510873</v>
+      </c>
+      <c r="BD92">
+        <v>-151.6665818374931</v>
+      </c>
+      <c r="BE92">
+        <v>-51.50217502366311</v>
+      </c>
+      <c r="BF92">
+        <v>26582</v>
+      </c>
+      <c r="BG92">
+        <v>5301</v>
+      </c>
+      <c r="BH92">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI92">
+        <v>32074</v>
+      </c>
+      <c r="BJ92">
+        <v>7108</v>
+      </c>
+      <c r="BK92">
+        <v>58656</v>
+      </c>
+      <c r="BL92">
+        <v>12409</v>
+      </c>
+      <c r="BM92">
+        <v>26562</v>
+      </c>
+      <c r="BN92">
+        <v>5298</v>
+      </c>
+      <c r="BO92">
+        <v>26576</v>
+      </c>
+      <c r="BP92">
+        <v>5297</v>
+      </c>
+      <c r="BQ92">
+        <v>5512</v>
+      </c>
+      <c r="BR92">
+        <v>1810</v>
+      </c>
+      <c r="BS92">
+        <v>6</v>
+      </c>
+      <c r="BT92">
+        <v>4</v>
+      </c>
+      <c r="BU92">
+        <v>0</v>
+      </c>
+      <c r="BV92">
+        <v>0</v>
+      </c>
+      <c r="BW92">
+        <v>22422.6498596</v>
+      </c>
+      <c r="BX92">
+        <v>6026.61715728</v>
+      </c>
+      <c r="BY92">
+        <v>0.0478985240126962</v>
+      </c>
+      <c r="BZ92">
+        <v>0.07174263600471449</v>
+      </c>
+      <c r="CA92">
+        <v>0.1043944746605658</v>
+      </c>
+      <c r="CB92">
+        <v>0.1994089391792258</v>
+      </c>
+      <c r="CC92">
+        <v>0.01236589961736039</v>
+      </c>
+      <c r="CD92">
+        <v>0.01511603778788603</v>
+      </c>
+      <c r="CE92">
+        <v>0.008333224599895273</v>
+      </c>
+      <c r="CF92">
+        <v>0.01295437640661317</v>
+      </c>
+      <c r="CG92">
+        <v>26078.0324</v>
+      </c>
+      <c r="CH92">
+        <v>6391.963400000001</v>
+      </c>
+      <c r="CI92">
+        <v>26229.69898183749</v>
+      </c>
+      <c r="CJ92">
+        <v>6443.465575023663</v>
+      </c>
+      <c r="CK92">
+        <v>0.1406503759723267</v>
+      </c>
+      <c r="CL92">
+        <v>0.09972378566007177</v>
+      </c>
+      <c r="CM92">
+        <v>10000</v>
+      </c>
+      <c r="CO92">
+        <v>0.003935185185185185</v>
+      </c>
+      <c r="CP92">
+        <v>0.001658950617283951</v>
+      </c>
+      <c r="CQ92">
+        <v>13857426.11025287</v>
+      </c>
+      <c r="CR92">
+        <v>1448171.53934798</v>
+      </c>
+      <c r="CS92" s="2">
+        <v>45407.71719204811</v>
+      </c>
+      <c r="CT92">
+        <v>-0.8215150584575165</v>
+      </c>
+      <c r="CU92">
+        <v>-0.9176181622791028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update COTIUSDT.json at 2024-04-26_03-42-58 bestfile_scores 0.000548406816724295 bestfile_sharp 0.1620874533203581
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU92"/>
+  <dimension ref="A1:CU93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -27137,6 +27137,275 @@
       </c>
       <c r="CU92">
         <v>-0.9176181622791028</v>
+      </c>
+    </row>
+    <row r="93" spans="1:99">
+      <c r="J93" t="s">
+        <v>214</v>
+      </c>
+      <c r="K93">
+        <v>0.002274117335452575</v>
+      </c>
+      <c r="L93">
+        <v>0.001137058667726287</v>
+      </c>
+      <c r="M93">
+        <v>0.000971470573771116</v>
+      </c>
+      <c r="N93">
+        <v>0.000971470573771116</v>
+      </c>
+      <c r="O93">
+        <v>0.004066230996926134</v>
+      </c>
+      <c r="P93">
+        <v>0.002033115498463067</v>
+      </c>
+      <c r="Q93">
+        <v>0.001057441916741464</v>
+      </c>
+      <c r="R93">
+        <v>0.001057441916741464</v>
+      </c>
+      <c r="S93">
+        <v>9.730930977275358</v>
+      </c>
+      <c r="T93">
+        <v>21.15266792700336</v>
+      </c>
+      <c r="U93">
+        <v>0.3985287712051558</v>
+      </c>
+      <c r="V93">
+        <v>0.5664476733243975</v>
+      </c>
+      <c r="W93">
+        <v>0.03741804864667954</v>
+      </c>
+      <c r="X93">
+        <v>0.07848340372438393</v>
+      </c>
+      <c r="Y93">
+        <v>0.1300337711453541</v>
+      </c>
+      <c r="Z93">
+        <v>0.2381585106412399</v>
+      </c>
+      <c r="AA93">
+        <v>0.9993070762456537</v>
+      </c>
+      <c r="AB93">
+        <v>0.8964120319053887</v>
+      </c>
+      <c r="AC93">
+        <v>0.820385693081384</v>
+      </c>
+      <c r="AD93">
+        <v>0.9990281823949684</v>
+      </c>
+      <c r="AE93">
+        <v>0.8282310159855727</v>
+      </c>
+      <c r="AF93">
+        <v>0.7619178180695421</v>
+      </c>
+      <c r="AG93">
+        <v>0.004394592950889599</v>
+      </c>
+      <c r="AH93">
+        <v>0.007880160120817952</v>
+      </c>
+      <c r="AI93">
+        <v>0.9993070762456537</v>
+      </c>
+      <c r="AJ93">
+        <v>0.9990281823949684</v>
+      </c>
+      <c r="AK93">
+        <v>0.004394592950889599</v>
+      </c>
+      <c r="AL93">
+        <v>0.007880160120817952</v>
+      </c>
+      <c r="AM93" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN93">
+        <v>0.02213931289331737</v>
+      </c>
+      <c r="AO93">
+        <v>0.03200406812725923</v>
+      </c>
+      <c r="AP93">
+        <v>-3070.964633272</v>
+      </c>
+      <c r="AQ93">
+        <v>-1026.565408268</v>
+      </c>
+      <c r="AR93">
+        <v>116250.660416728</v>
+      </c>
+      <c r="AS93">
+        <v>28537.62969173201</v>
+      </c>
+      <c r="AT93">
+        <v>115838.403266728</v>
+      </c>
+      <c r="AU93">
+        <v>28537.62969173201</v>
+      </c>
+      <c r="AV93">
+        <v>10.6250660416728</v>
+      </c>
+      <c r="AW93">
+        <v>1.8537629691732</v>
+      </c>
+      <c r="AX93">
+        <v>2.46396872224337</v>
+      </c>
+      <c r="AY93">
+        <v>1.132924017569204</v>
+      </c>
+      <c r="AZ93">
+        <v>93.34999999999999</v>
+      </c>
+      <c r="BA93">
+        <v>73.55</v>
+      </c>
+      <c r="BB93">
+        <v>0.0131578031150078</v>
+      </c>
+      <c r="BC93">
+        <v>0.05767463398980652</v>
+      </c>
+      <c r="BD93">
+        <v>-1457.611382205865</v>
+      </c>
+      <c r="BE93">
+        <v>-1197.418463301198</v>
+      </c>
+      <c r="BF93">
+        <v>4429</v>
+      </c>
+      <c r="BG93">
+        <v>6637</v>
+      </c>
+      <c r="BH93">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI93">
+        <v>6080</v>
+      </c>
+      <c r="BJ93">
+        <v>16207</v>
+      </c>
+      <c r="BK93">
+        <v>10509</v>
+      </c>
+      <c r="BL93">
+        <v>22844</v>
+      </c>
+      <c r="BM93">
+        <v>4193</v>
+      </c>
+      <c r="BN93">
+        <v>6528</v>
+      </c>
+      <c r="BO93">
+        <v>4409</v>
+      </c>
+      <c r="BP93">
+        <v>6588</v>
+      </c>
+      <c r="BQ93">
+        <v>1887</v>
+      </c>
+      <c r="BR93">
+        <v>9679</v>
+      </c>
+      <c r="BS93">
+        <v>20</v>
+      </c>
+      <c r="BT93">
+        <v>49</v>
+      </c>
+      <c r="BU93">
+        <v>0</v>
+      </c>
+      <c r="BV93">
+        <v>0</v>
+      </c>
+      <c r="BW93">
+        <v>106250.6604167281</v>
+      </c>
+      <c r="BX93">
+        <v>18537.62969173198</v>
+      </c>
+      <c r="BY93">
+        <v>0.03892936006459703</v>
+      </c>
+      <c r="BZ93">
+        <v>0.06460153239297101</v>
+      </c>
+      <c r="CA93">
+        <v>0.0693951352338226</v>
+      </c>
+      <c r="CB93">
+        <v>0.1919129342134135</v>
+      </c>
+      <c r="CC93">
+        <v>0.01065139962831592</v>
+      </c>
+      <c r="CD93">
+        <v>0.009370656536507519</v>
+      </c>
+      <c r="CE93">
+        <v>0.008753658195568843</v>
+      </c>
+      <c r="CF93">
+        <v>0.0089890040516395</v>
+      </c>
+      <c r="CG93">
+        <v>109321.6250500001</v>
+      </c>
+      <c r="CH93">
+        <v>19564.19509999998</v>
+      </c>
+      <c r="CI93">
+        <v>110779.2364322059</v>
+      </c>
+      <c r="CJ93">
+        <v>20761.61356330118</v>
+      </c>
+      <c r="CK93">
+        <v>0.1725313855670823</v>
+      </c>
+      <c r="CL93">
+        <v>0.08513042212819663</v>
+      </c>
+      <c r="CM93">
+        <v>10000</v>
+      </c>
+      <c r="CO93">
+        <v>0.002816358024691358</v>
+      </c>
+      <c r="CP93">
+        <v>0.01531635802469136</v>
+      </c>
+      <c r="CQ93">
+        <v>17088360.3131318</v>
+      </c>
+      <c r="CR93">
+        <v>16635452.15900955</v>
+      </c>
+      <c r="CS93" s="2">
+        <v>45407.95732689535</v>
+      </c>
+      <c r="CT93">
+        <v>-0.7542388832888753</v>
+      </c>
+      <c r="CU93">
+        <v>-0.6981424011030314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GRTUSDT.json at 2024-04-26_10-00-32 bestfile_scores 0.0007813744979330378 bestfile_sharp 0.16060683983137639
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="958" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU93"/>
+  <dimension ref="A1:CU94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -27406,6 +27406,275 @@
       </c>
       <c r="CU93">
         <v>-0.6981424011030314</v>
+      </c>
+    </row>
+    <row r="94" spans="1:99">
+      <c r="J94" t="s">
+        <v>215</v>
+      </c>
+      <c r="K94">
+        <v>0.001162689504127901</v>
+      </c>
+      <c r="L94">
+        <v>0.0005813447520639503</v>
+      </c>
+      <c r="M94">
+        <v>0.000332639083723052</v>
+      </c>
+      <c r="N94">
+        <v>0.000332639083723052</v>
+      </c>
+      <c r="O94">
+        <v>0.001792260464903261</v>
+      </c>
+      <c r="P94">
+        <v>0.0008961302324516307</v>
+      </c>
+      <c r="Q94">
+        <v>0.0003835131986585472</v>
+      </c>
+      <c r="R94">
+        <v>0.0003835131986585472</v>
+      </c>
+      <c r="S94">
+        <v>8.734596242138972</v>
+      </c>
+      <c r="T94">
+        <v>0.4481654384814229</v>
+      </c>
+      <c r="U94">
+        <v>0.1990900354041484</v>
+      </c>
+      <c r="V94">
+        <v>1</v>
+      </c>
+      <c r="W94">
+        <v>0.03924051553656326</v>
+      </c>
+      <c r="X94">
+        <v>0.1025032525175916</v>
+      </c>
+      <c r="Y94">
+        <v>0.2279370786049078</v>
+      </c>
+      <c r="Z94">
+        <v>0.1445310896990829</v>
+      </c>
+      <c r="AA94">
+        <v>0.9993559783985878</v>
+      </c>
+      <c r="AB94">
+        <v>0.8546748358229734</v>
+      </c>
+      <c r="AC94">
+        <v>0.8614248747277495</v>
+      </c>
+      <c r="AD94">
+        <v>0.9957367177201037</v>
+      </c>
+      <c r="AE94">
+        <v>0.7718529845755485</v>
+      </c>
+      <c r="AF94">
+        <v>0.8555119147679715</v>
+      </c>
+      <c r="AG94">
+        <v>0.005153398436948856</v>
+      </c>
+      <c r="AH94">
+        <v>0.01483584540071084</v>
+      </c>
+      <c r="AI94">
+        <v>0.9993559783985878</v>
+      </c>
+      <c r="AJ94">
+        <v>0.9957367177201037</v>
+      </c>
+      <c r="AK94">
+        <v>0.005153398436948856</v>
+      </c>
+      <c r="AL94">
+        <v>0.01483584540071084</v>
+      </c>
+      <c r="AM94" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN94">
+        <v>0.01428951294373429</v>
+      </c>
+      <c r="AO94">
+        <v>0.03274006077863804</v>
+      </c>
+      <c r="AP94">
+        <v>-1010.288615934</v>
+      </c>
+      <c r="AQ94">
+        <v>-33.389716666</v>
+      </c>
+      <c r="AR94">
+        <v>35075.81663406604</v>
+      </c>
+      <c r="AS94">
+        <v>14321.49719333403</v>
+      </c>
+      <c r="AT94">
+        <v>35020.76159406604</v>
+      </c>
+      <c r="AU94">
+        <v>14321.49719333403</v>
+      </c>
+      <c r="AV94">
+        <v>2.507581663406604</v>
+      </c>
+      <c r="AW94">
+        <v>0.4321497193334032</v>
+      </c>
+      <c r="AX94">
+        <v>2.746624964659316</v>
+      </c>
+      <c r="AY94">
+        <v>53.56149068322981</v>
+      </c>
+      <c r="AZ94">
+        <v>103.7</v>
+      </c>
+      <c r="BA94">
+        <v>1697.65</v>
+      </c>
+      <c r="BB94">
+        <v>0.005990740388638407</v>
+      </c>
+      <c r="BC94">
+        <v>0</v>
+      </c>
+      <c r="BD94">
+        <v>-157.2169301164739</v>
+      </c>
+      <c r="BE94">
+        <v>0</v>
+      </c>
+      <c r="BF94">
+        <v>4279</v>
+      </c>
+      <c r="BG94">
+        <v>182</v>
+      </c>
+      <c r="BH94">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI94">
+        <v>5154</v>
+      </c>
+      <c r="BJ94">
+        <v>302</v>
+      </c>
+      <c r="BK94">
+        <v>9433</v>
+      </c>
+      <c r="BL94">
+        <v>484</v>
+      </c>
+      <c r="BM94">
+        <v>4075</v>
+      </c>
+      <c r="BN94">
+        <v>182</v>
+      </c>
+      <c r="BO94">
+        <v>4257</v>
+      </c>
+      <c r="BP94">
+        <v>182</v>
+      </c>
+      <c r="BQ94">
+        <v>1079</v>
+      </c>
+      <c r="BR94">
+        <v>120</v>
+      </c>
+      <c r="BS94">
+        <v>22</v>
+      </c>
+      <c r="BT94">
+        <v>0</v>
+      </c>
+      <c r="BU94">
+        <v>0</v>
+      </c>
+      <c r="BV94">
+        <v>0</v>
+      </c>
+      <c r="BW94">
+        <v>25075.816634066</v>
+      </c>
+      <c r="BX94">
+        <v>4321.497193334001</v>
+      </c>
+      <c r="BY94">
+        <v>0.05318612413192853</v>
+      </c>
+      <c r="BZ94">
+        <v>0.2879076057409029</v>
+      </c>
+      <c r="CA94">
+        <v>0.1287157647971915</v>
+      </c>
+      <c r="CB94">
+        <v>0.3650179069702904</v>
+      </c>
+      <c r="CC94">
+        <v>0.01605827666794758</v>
+      </c>
+      <c r="CD94">
+        <v>0.05760247258158167</v>
+      </c>
+      <c r="CE94">
+        <v>0.01301242077861819</v>
+      </c>
+      <c r="CF94">
+        <v>0.0613083157428105</v>
+      </c>
+      <c r="CG94">
+        <v>26086.10525</v>
+      </c>
+      <c r="CH94">
+        <v>4354.886910000001</v>
+      </c>
+      <c r="CI94">
+        <v>26243.32218011647</v>
+      </c>
+      <c r="CJ94">
+        <v>4354.886910000001</v>
+      </c>
+      <c r="CK94">
+        <v>0.1620874533203581</v>
+      </c>
+      <c r="CL94">
+        <v>0.04437679609204329</v>
+      </c>
+      <c r="CM94">
+        <v>10000</v>
+      </c>
+      <c r="CO94">
+        <v>0.005054012345679012</v>
+      </c>
+      <c r="CP94">
+        <v>0</v>
+      </c>
+      <c r="CQ94">
+        <v>7032166.179724406</v>
+      </c>
+      <c r="CR94">
+        <v>118847.66881</v>
+      </c>
+      <c r="CS94" s="2">
+        <v>45408.15486152974</v>
+      </c>
+      <c r="CT94">
+        <v>-0.8706219162560768</v>
+      </c>
+      <c r="CU94">
+        <v>-0.7950532923358701</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update EGLDUSDT.json at 2024-04-26_16-41-49 bestfile_scores 0.0008604368236225762 bestfile_sharp 0.11059252413400326
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="960" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU94"/>
+  <dimension ref="A1:CU95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -27675,6 +27675,275 @@
       </c>
       <c r="CU94">
         <v>-0.7950532923358701</v>
+      </c>
+    </row>
+    <row r="95" spans="1:99">
+      <c r="J95" t="s">
+        <v>216</v>
+      </c>
+      <c r="K95">
+        <v>0.001499306927317701</v>
+      </c>
+      <c r="L95">
+        <v>0.0007496534636588503</v>
+      </c>
+      <c r="M95">
+        <v>0.0008683833705553923</v>
+      </c>
+      <c r="N95">
+        <v>0.0008683833705553923</v>
+      </c>
+      <c r="O95">
+        <v>0.001306031199455782</v>
+      </c>
+      <c r="P95">
+        <v>0.0006530155997278908</v>
+      </c>
+      <c r="Q95">
+        <v>0.0008544455577900179</v>
+      </c>
+      <c r="R95">
+        <v>0.0008544455577900179</v>
+      </c>
+      <c r="S95">
+        <v>17.05997296775439</v>
+      </c>
+      <c r="T95">
+        <v>35.06993628113536</v>
+      </c>
+      <c r="U95">
+        <v>0.2498310292462481</v>
+      </c>
+      <c r="V95">
+        <v>0.6601917397290639</v>
+      </c>
+      <c r="W95">
+        <v>0.06212642577452348</v>
+      </c>
+      <c r="X95">
+        <v>0.06723535471394455</v>
+      </c>
+      <c r="Y95">
+        <v>0.2374123057838232</v>
+      </c>
+      <c r="Z95">
+        <v>0.182148965207665</v>
+      </c>
+      <c r="AA95">
+        <v>0.9987795385819245</v>
+      </c>
+      <c r="AB95">
+        <v>0.7894348636622911</v>
+      </c>
+      <c r="AC95">
+        <v>0.8371482723401872</v>
+      </c>
+      <c r="AD95">
+        <v>0.9984183459466792</v>
+      </c>
+      <c r="AE95">
+        <v>0.7348031533459354</v>
+      </c>
+      <c r="AF95">
+        <v>0.8188666168917597</v>
+      </c>
+      <c r="AG95">
+        <v>0.007722804295804008</v>
+      </c>
+      <c r="AH95">
+        <v>0.007773072690660088</v>
+      </c>
+      <c r="AI95">
+        <v>0.9987795385819245</v>
+      </c>
+      <c r="AJ95">
+        <v>0.9984183459466792</v>
+      </c>
+      <c r="AK95">
+        <v>0.007722804295804008</v>
+      </c>
+      <c r="AL95">
+        <v>0.007773072690660088</v>
+      </c>
+      <c r="AM95" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN95">
+        <v>0.02834543237532101</v>
+      </c>
+      <c r="AO95">
+        <v>0.04688995272311564</v>
+      </c>
+      <c r="AP95">
+        <v>-1785.487037248</v>
+      </c>
+      <c r="AQ95">
+        <v>-1790.421098006</v>
+      </c>
+      <c r="AR95">
+        <v>50353.25681275198</v>
+      </c>
+      <c r="AS95">
+        <v>25511.46571199437</v>
+      </c>
+      <c r="AT95">
+        <v>49902.89260275198</v>
+      </c>
+      <c r="AU95">
+        <v>25511.46571199437</v>
+      </c>
+      <c r="AV95">
+        <v>4.035325681275198</v>
+      </c>
+      <c r="AW95">
+        <v>1.551146571199437</v>
+      </c>
+      <c r="AX95">
+        <v>1.40504726719548</v>
+      </c>
+      <c r="AY95">
+        <v>0.6831465722289761</v>
+      </c>
+      <c r="AZ95">
+        <v>101.2333333333333</v>
+      </c>
+      <c r="BA95">
+        <v>110.1</v>
+      </c>
+      <c r="BB95">
+        <v>0.0004871527174277262</v>
+      </c>
+      <c r="BC95">
+        <v>0.03427588175739515</v>
+      </c>
+      <c r="BD95">
+        <v>-20.53800872227807</v>
+      </c>
+      <c r="BE95">
+        <v>-614.0857572849952</v>
+      </c>
+      <c r="BF95">
+        <v>5579</v>
+      </c>
+      <c r="BG95">
+        <v>17064</v>
+      </c>
+      <c r="BH95">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI95">
+        <v>12828</v>
+      </c>
+      <c r="BJ95">
+        <v>20775</v>
+      </c>
+      <c r="BK95">
+        <v>18407</v>
+      </c>
+      <c r="BL95">
+        <v>37839</v>
+      </c>
+      <c r="BM95">
+        <v>5050</v>
+      </c>
+      <c r="BN95">
+        <v>16380</v>
+      </c>
+      <c r="BO95">
+        <v>5573</v>
+      </c>
+      <c r="BP95">
+        <v>17030</v>
+      </c>
+      <c r="BQ95">
+        <v>7778</v>
+      </c>
+      <c r="BR95">
+        <v>4395</v>
+      </c>
+      <c r="BS95">
+        <v>6</v>
+      </c>
+      <c r="BT95">
+        <v>34</v>
+      </c>
+      <c r="BU95">
+        <v>0</v>
+      </c>
+      <c r="BV95">
+        <v>0</v>
+      </c>
+      <c r="BW95">
+        <v>40353.25681275215</v>
+      </c>
+      <c r="BX95">
+        <v>15511.46571199399</v>
+      </c>
+      <c r="BY95">
+        <v>0.05117799654778413</v>
+      </c>
+      <c r="BZ95">
+        <v>0.08654141177703327</v>
+      </c>
+      <c r="CA95">
+        <v>0.1337247748407561</v>
+      </c>
+      <c r="CB95">
+        <v>0.1593936634287124</v>
+      </c>
+      <c r="CC95">
+        <v>0.01066858140973019</v>
+      </c>
+      <c r="CD95">
+        <v>0.01182109013417778</v>
+      </c>
+      <c r="CE95">
+        <v>0.008886996883406066</v>
+      </c>
+      <c r="CF95">
+        <v>0.01426132454462175</v>
+      </c>
+      <c r="CG95">
+        <v>42138.74385000015</v>
+      </c>
+      <c r="CH95">
+        <v>17301.88680999999</v>
+      </c>
+      <c r="CI95">
+        <v>42159.28185872243</v>
+      </c>
+      <c r="CJ95">
+        <v>17915.97256728498</v>
+      </c>
+      <c r="CK95">
+        <v>0.1606068398313764</v>
+      </c>
+      <c r="CL95">
+        <v>0.08155549848396061</v>
+      </c>
+      <c r="CM95">
+        <v>10000</v>
+      </c>
+      <c r="CO95">
+        <v>0.002857584182885388</v>
+      </c>
+      <c r="CP95">
+        <v>0.01421068890948409</v>
+      </c>
+      <c r="CQ95">
+        <v>35909902.46144007</v>
+      </c>
+      <c r="CR95">
+        <v>9989976.067409206</v>
+      </c>
+      <c r="CS95" s="2">
+        <v>45408.41706631281</v>
+      </c>
+      <c r="CT95">
+        <v>-0.7702665229627835</v>
+      </c>
+      <c r="CU95">
+        <v>-0.731704477344099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update COMPUSDT.json at 2024-04-26_21-09-40 bestfile_scores 0.0007011963640319308 bestfile_sharp 0.1480658534303749
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU95"/>
+  <dimension ref="A1:CU96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -27944,6 +27944,275 @@
       </c>
       <c r="CU95">
         <v>-0.731704477344099</v>
+      </c>
+    </row>
+    <row r="96" spans="1:99">
+      <c r="J96" t="s">
+        <v>217</v>
+      </c>
+      <c r="K96">
+        <v>0.002539278300601966</v>
+      </c>
+      <c r="L96">
+        <v>0.001269639150300983</v>
+      </c>
+      <c r="M96">
+        <v>0.0005314235230478026</v>
+      </c>
+      <c r="N96">
+        <v>0.0005314235230478026</v>
+      </c>
+      <c r="O96">
+        <v>0.00229225736152594</v>
+      </c>
+      <c r="P96">
+        <v>0.00114612868076297</v>
+      </c>
+      <c r="Q96">
+        <v>0.0004945559403785494</v>
+      </c>
+      <c r="R96">
+        <v>0.0004945559403785494</v>
+      </c>
+      <c r="S96">
+        <v>12.92549866893013</v>
+      </c>
+      <c r="T96">
+        <v>13.9922064894479</v>
+      </c>
+      <c r="U96">
+        <v>0.424841677049249</v>
+      </c>
+      <c r="V96">
+        <v>0.7756574951829108</v>
+      </c>
+      <c r="W96">
+        <v>0.08827953607599785</v>
+      </c>
+      <c r="X96">
+        <v>0.04550760366060576</v>
+      </c>
+      <c r="Y96">
+        <v>0.2404397899036964</v>
+      </c>
+      <c r="Z96">
+        <v>0.1173502987683091</v>
+      </c>
+      <c r="AA96">
+        <v>0.9983102839267268</v>
+      </c>
+      <c r="AB96">
+        <v>0.7832123550604194</v>
+      </c>
+      <c r="AC96">
+        <v>0.9035242120859002</v>
+      </c>
+      <c r="AD96">
+        <v>0.9991060690688153</v>
+      </c>
+      <c r="AE96">
+        <v>0.7564940396853471</v>
+      </c>
+      <c r="AF96">
+        <v>0.8564902259381001</v>
+      </c>
+      <c r="AG96">
+        <v>0.009919225671231555</v>
+      </c>
+      <c r="AH96">
+        <v>0.005069566938105054</v>
+      </c>
+      <c r="AI96">
+        <v>0.9983102839267268</v>
+      </c>
+      <c r="AJ96">
+        <v>0.9991060690688153</v>
+      </c>
+      <c r="AK96">
+        <v>0.009919225671231555</v>
+      </c>
+      <c r="AL96">
+        <v>0.005069566938105054</v>
+      </c>
+      <c r="AM96" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN96">
+        <v>0.03788820385254356</v>
+      </c>
+      <c r="AO96">
+        <v>0.03352346003151505</v>
+      </c>
+      <c r="AP96">
+        <v>-6955.243381</v>
+      </c>
+      <c r="AQ96">
+        <v>-493.2768356</v>
+      </c>
+      <c r="AR96">
+        <v>154690.135019</v>
+      </c>
+      <c r="AS96">
+        <v>17749.3325644002</v>
+      </c>
+      <c r="AT96">
+        <v>154657.2120189999</v>
+      </c>
+      <c r="AU96">
+        <v>17743.1265644002</v>
+      </c>
+      <c r="AV96">
+        <v>14.4690135019</v>
+      </c>
+      <c r="AW96">
+        <v>0.7749332564400195</v>
+      </c>
+      <c r="AX96">
+        <v>1.854520704972059</v>
+      </c>
+      <c r="AY96">
+        <v>1.713165673946614</v>
+      </c>
+      <c r="AZ96">
+        <v>117.8333333333333</v>
+      </c>
+      <c r="BA96">
+        <v>107.4333333333333</v>
+      </c>
+      <c r="BB96">
+        <v>0.05396993055804236</v>
+      </c>
+      <c r="BC96">
+        <v>0.04269633519742689</v>
+      </c>
+      <c r="BD96">
+        <v>-8651.194931387108</v>
+      </c>
+      <c r="BE96">
+        <v>-367.6254743226546</v>
+      </c>
+      <c r="BF96">
+        <v>5778</v>
+      </c>
+      <c r="BG96">
+        <v>6414</v>
+      </c>
+      <c r="BH96">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI96">
+        <v>8181</v>
+      </c>
+      <c r="BJ96">
+        <v>8697</v>
+      </c>
+      <c r="BK96">
+        <v>13959</v>
+      </c>
+      <c r="BL96">
+        <v>15111</v>
+      </c>
+      <c r="BM96">
+        <v>4860</v>
+      </c>
+      <c r="BN96">
+        <v>5999</v>
+      </c>
+      <c r="BO96">
+        <v>5747</v>
+      </c>
+      <c r="BP96">
+        <v>6355</v>
+      </c>
+      <c r="BQ96">
+        <v>3321</v>
+      </c>
+      <c r="BR96">
+        <v>2698</v>
+      </c>
+      <c r="BS96">
+        <v>31</v>
+      </c>
+      <c r="BT96">
+        <v>59</v>
+      </c>
+      <c r="BU96">
+        <v>0</v>
+      </c>
+      <c r="BV96">
+        <v>0</v>
+      </c>
+      <c r="BW96">
+        <v>144690.135019</v>
+      </c>
+      <c r="BX96">
+        <v>7749.332564399994</v>
+      </c>
+      <c r="BY96">
+        <v>0.05396592735622123</v>
+      </c>
+      <c r="BZ96">
+        <v>0.05484583981158555</v>
+      </c>
+      <c r="CA96">
+        <v>0.1386176222653542</v>
+      </c>
+      <c r="CB96">
+        <v>0.1048783493486045</v>
+      </c>
+      <c r="CC96">
+        <v>0.01433473643869187</v>
+      </c>
+      <c r="CD96">
+        <v>0.01227089830967895</v>
+      </c>
+      <c r="CE96">
+        <v>0.01059481628834019</v>
+      </c>
+      <c r="CF96">
+        <v>0.009074025572870348</v>
+      </c>
+      <c r="CG96">
+        <v>151645.3784</v>
+      </c>
+      <c r="CH96">
+        <v>8242.609399999994</v>
+      </c>
+      <c r="CI96">
+        <v>160296.5733313871</v>
+      </c>
+      <c r="CJ96">
+        <v>8610.234874322648</v>
+      </c>
+      <c r="CK96">
+        <v>0.1105925241340033</v>
+      </c>
+      <c r="CL96">
+        <v>0.09599992971661729</v>
+      </c>
+      <c r="CM96">
+        <v>10000</v>
+      </c>
+      <c r="CO96">
+        <v>0.006674382716049383</v>
+      </c>
+      <c r="CP96">
+        <v>0.006134259259259259</v>
+      </c>
+      <c r="CQ96">
+        <v>86047374.08980072</v>
+      </c>
+      <c r="CR96">
+        <v>4195010.116009732</v>
+      </c>
+      <c r="CS96" s="2">
+        <v>45408.69572966039</v>
+      </c>
+      <c r="CT96">
+        <v>-0.6208027078099908</v>
+      </c>
+      <c r="CU96">
+        <v>-0.8947084492298638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update HBARUSDT.json at 2024-04-27_15-06-18 bestfile_scores 0.0004960221137870924 bestfile_sharp 0.11315580755943838
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="964" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU96"/>
+  <dimension ref="A1:CU98"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -28213,6 +28213,544 @@
       </c>
       <c r="CU96">
         <v>-0.8947084492298638</v>
+      </c>
+    </row>
+    <row r="97" spans="10:99">
+      <c r="J97" t="s">
+        <v>218</v>
+      </c>
+      <c r="K97">
+        <v>0.001705731004323807</v>
+      </c>
+      <c r="L97">
+        <v>0.0008528655021619036</v>
+      </c>
+      <c r="M97">
+        <v>0.0005346146862532652</v>
+      </c>
+      <c r="N97">
+        <v>0.0005346146862532652</v>
+      </c>
+      <c r="O97">
+        <v>0.00184031072287496</v>
+      </c>
+      <c r="P97">
+        <v>0.0009201553614374802</v>
+      </c>
+      <c r="Q97">
+        <v>0.000497149906275074</v>
+      </c>
+      <c r="R97">
+        <v>0.000497149906275074</v>
+      </c>
+      <c r="S97">
+        <v>14.982059493036</v>
+      </c>
+      <c r="T97">
+        <v>6.322466144527182</v>
+      </c>
+      <c r="U97">
+        <v>0.3440941021059319</v>
+      </c>
+      <c r="V97">
+        <v>0.5978958985125707</v>
+      </c>
+      <c r="W97">
+        <v>0.0927524150605276</v>
+      </c>
+      <c r="X97">
+        <v>0.09877477938010616</v>
+      </c>
+      <c r="Y97">
+        <v>0.2367789739395751</v>
+      </c>
+      <c r="Z97">
+        <v>0.2403500104274805</v>
+      </c>
+      <c r="AA97">
+        <v>0.9976227692285655</v>
+      </c>
+      <c r="AB97">
+        <v>0.8380292580079706</v>
+      </c>
+      <c r="AC97">
+        <v>0.7848544254371177</v>
+      </c>
+      <c r="AD97">
+        <v>0.9980859889856024</v>
+      </c>
+      <c r="AE97">
+        <v>0.7631919502711668</v>
+      </c>
+      <c r="AF97">
+        <v>0.760104906583483</v>
+      </c>
+      <c r="AG97">
+        <v>0.01028762272041012</v>
+      </c>
+      <c r="AH97">
+        <v>0.01091810348006776</v>
+      </c>
+      <c r="AI97">
+        <v>0.9976227692285655</v>
+      </c>
+      <c r="AJ97">
+        <v>0.9980859889856024</v>
+      </c>
+      <c r="AK97">
+        <v>0.01028762272041012</v>
+      </c>
+      <c r="AL97">
+        <v>0.01091810348006776</v>
+      </c>
+      <c r="AM97" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN97">
+        <v>0.04644791623814626</v>
+      </c>
+      <c r="AO97">
+        <v>0.04106026414724349</v>
+      </c>
+      <c r="AP97">
+        <v>-3504.23270673</v>
+      </c>
+      <c r="AQ97">
+        <v>-386.5970702440001</v>
+      </c>
+      <c r="AR97">
+        <v>62999.96750327018</v>
+      </c>
+      <c r="AS97">
+        <v>17810.57532975603</v>
+      </c>
+      <c r="AT97">
+        <v>62881.78788327018</v>
+      </c>
+      <c r="AU97">
+        <v>17808.72786975603</v>
+      </c>
+      <c r="AV97">
+        <v>5.299996750327018</v>
+      </c>
+      <c r="AW97">
+        <v>0.7810575329756029</v>
+      </c>
+      <c r="AX97">
+        <v>1.600281228753322</v>
+      </c>
+      <c r="AY97">
+        <v>3.790964796640789</v>
+      </c>
+      <c r="AZ97">
+        <v>97.21666666666667</v>
+      </c>
+      <c r="BA97">
+        <v>109.9833333333333</v>
+      </c>
+      <c r="BB97">
+        <v>0.02970247799363397</v>
+      </c>
+      <c r="BC97">
+        <v>0.004732253267724571</v>
+      </c>
+      <c r="BD97">
+        <v>-1729.690868234953</v>
+      </c>
+      <c r="BE97">
+        <v>-38.97553799303052</v>
+      </c>
+      <c r="BF97">
+        <v>6554</v>
+      </c>
+      <c r="BG97">
+        <v>2856</v>
+      </c>
+      <c r="BH97">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI97">
+        <v>9626</v>
+      </c>
+      <c r="BJ97">
+        <v>3972</v>
+      </c>
+      <c r="BK97">
+        <v>16180</v>
+      </c>
+      <c r="BL97">
+        <v>6828</v>
+      </c>
+      <c r="BM97">
+        <v>6520</v>
+      </c>
+      <c r="BN97">
+        <v>2838</v>
+      </c>
+      <c r="BO97">
+        <v>6523</v>
+      </c>
+      <c r="BP97">
+        <v>2843</v>
+      </c>
+      <c r="BQ97">
+        <v>3106</v>
+      </c>
+      <c r="BR97">
+        <v>1134</v>
+      </c>
+      <c r="BS97">
+        <v>31</v>
+      </c>
+      <c r="BT97">
+        <v>13</v>
+      </c>
+      <c r="BU97">
+        <v>0</v>
+      </c>
+      <c r="BV97">
+        <v>0</v>
+      </c>
+      <c r="BW97">
+        <v>52999.96750327004</v>
+      </c>
+      <c r="BX97">
+        <v>7810.575329756003</v>
+      </c>
+      <c r="BY97">
+        <v>0.0589682310975323</v>
+      </c>
+      <c r="BZ97">
+        <v>0.1041801250845643</v>
+      </c>
+      <c r="CA97">
+        <v>0.1342880370338898</v>
+      </c>
+      <c r="CB97">
+        <v>0.1934653782906826</v>
+      </c>
+      <c r="CC97">
+        <v>0.0145024922053075</v>
+      </c>
+      <c r="CD97">
+        <v>0.01765107645517801</v>
+      </c>
+      <c r="CE97">
+        <v>0.010873260012217</v>
+      </c>
+      <c r="CF97">
+        <v>0.01688933598555118</v>
+      </c>
+      <c r="CG97">
+        <v>56504.20021000004</v>
+      </c>
+      <c r="CH97">
+        <v>8197.172400000003</v>
+      </c>
+      <c r="CI97">
+        <v>58233.89107823499</v>
+      </c>
+      <c r="CJ97">
+        <v>8236.147937993033</v>
+      </c>
+      <c r="CK97">
+        <v>0.1480658534303749</v>
+      </c>
+      <c r="CL97">
+        <v>0.06553555579824208</v>
+      </c>
+      <c r="CM97">
+        <v>10000</v>
+      </c>
+      <c r="CO97">
+        <v>0.005285493827160494</v>
+      </c>
+      <c r="CP97">
+        <v>0.00783179012345679</v>
+      </c>
+      <c r="CQ97">
+        <v>20034291.58056061</v>
+      </c>
+      <c r="CR97">
+        <v>1753546.300271091</v>
+      </c>
+      <c r="CS97" s="2">
+        <v>45408.88173610321</v>
+      </c>
+      <c r="CT97">
+        <v>-0.6637406607330143</v>
+      </c>
+      <c r="CU97">
+        <v>-0.7970155689698759</v>
+      </c>
+    </row>
+    <row r="98" spans="10:99">
+      <c r="J98" t="s">
+        <v>219</v>
+      </c>
+      <c r="K98">
+        <v>0.002466194294380886</v>
+      </c>
+      <c r="L98">
+        <v>0.001233097147190443</v>
+      </c>
+      <c r="M98">
+        <v>0.0005044525214208395</v>
+      </c>
+      <c r="N98">
+        <v>0.0005044525214208395</v>
+      </c>
+      <c r="O98">
+        <v>0.001688079614177496</v>
+      </c>
+      <c r="P98">
+        <v>0.0008440398070887478</v>
+      </c>
+      <c r="Q98">
+        <v>0.0005040832515054383</v>
+      </c>
+      <c r="R98">
+        <v>0.0005040832515054383</v>
+      </c>
+      <c r="S98">
+        <v>16.1015471275898</v>
+      </c>
+      <c r="T98">
+        <v>42.22477719047803</v>
+      </c>
+      <c r="U98">
+        <v>0.4101919941835988</v>
+      </c>
+      <c r="V98">
+        <v>0.7591079898604071</v>
+      </c>
+      <c r="W98">
+        <v>0.02133605574293554</v>
+      </c>
+      <c r="X98">
+        <v>0.07227383812146021</v>
+      </c>
+      <c r="Y98">
+        <v>0.1630719686112306</v>
+      </c>
+      <c r="Z98">
+        <v>0.1610599210507703</v>
+      </c>
+      <c r="AA98">
+        <v>0.9996277172763187</v>
+      </c>
+      <c r="AB98">
+        <v>0.8723494802839665</v>
+      </c>
+      <c r="AC98">
+        <v>0.8615575950705384</v>
+      </c>
+      <c r="AD98">
+        <v>0.999037032967601</v>
+      </c>
+      <c r="AE98">
+        <v>0.8199751609486819</v>
+      </c>
+      <c r="AF98">
+        <v>0.8474945899931438</v>
+      </c>
+      <c r="AG98">
+        <v>0.003599773286937066</v>
+      </c>
+      <c r="AH98">
+        <v>0.007356135213002895</v>
+      </c>
+      <c r="AI98">
+        <v>0.9996277172763187</v>
+      </c>
+      <c r="AJ98">
+        <v>0.999037032967601</v>
+      </c>
+      <c r="AK98">
+        <v>0.003599773286937066</v>
+      </c>
+      <c r="AL98">
+        <v>0.007356135213002895</v>
+      </c>
+      <c r="AM98" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN98">
+        <v>0.01299733286067653</v>
+      </c>
+      <c r="AO98">
+        <v>0.03285892641896526</v>
+      </c>
+      <c r="AP98">
+        <v>-7663.278154528</v>
+      </c>
+      <c r="AQ98">
+        <v>-1337.08297556</v>
+      </c>
+      <c r="AR98">
+        <v>142978.3682054722</v>
+      </c>
+      <c r="AS98">
+        <v>17240.05462444073</v>
+      </c>
+      <c r="AT98">
+        <v>142962.8882054721</v>
+      </c>
+      <c r="AU98">
+        <v>17238.92882444073</v>
+      </c>
+      <c r="AV98">
+        <v>13.29783682054722</v>
+      </c>
+      <c r="AW98">
+        <v>0.724005462444073</v>
+      </c>
+      <c r="AX98">
+        <v>1.489265585461238</v>
+      </c>
+      <c r="AY98">
+        <v>0.5679239766081872</v>
+      </c>
+      <c r="AZ98">
+        <v>86.13333333333334</v>
+      </c>
+      <c r="BA98">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="BB98">
+        <v>0.008499853999672593</v>
+      </c>
+      <c r="BC98">
+        <v>0.07917318323592999</v>
+      </c>
+      <c r="BD98">
+        <v>-1205.681577714251</v>
+      </c>
+      <c r="BE98">
+        <v>-737.466887889925</v>
+      </c>
+      <c r="BF98">
+        <v>8078</v>
+      </c>
+      <c r="BG98">
+        <v>20980</v>
+      </c>
+      <c r="BH98">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI98">
+        <v>9311</v>
+      </c>
+      <c r="BJ98">
+        <v>24621</v>
+      </c>
+      <c r="BK98">
+        <v>17389</v>
+      </c>
+      <c r="BL98">
+        <v>45601</v>
+      </c>
+      <c r="BM98">
+        <v>7579</v>
+      </c>
+      <c r="BN98">
+        <v>20207</v>
+      </c>
+      <c r="BO98">
+        <v>8051</v>
+      </c>
+      <c r="BP98">
+        <v>20910</v>
+      </c>
+      <c r="BQ98">
+        <v>1732</v>
+      </c>
+      <c r="BR98">
+        <v>4414</v>
+      </c>
+      <c r="BS98">
+        <v>27</v>
+      </c>
+      <c r="BT98">
+        <v>70</v>
+      </c>
+      <c r="BU98">
+        <v>0</v>
+      </c>
+      <c r="BV98">
+        <v>0</v>
+      </c>
+      <c r="BW98">
+        <v>132978.368205472</v>
+      </c>
+      <c r="BX98">
+        <v>7240.054624440002</v>
+      </c>
+      <c r="BY98">
+        <v>0.03453169624631488</v>
+      </c>
+      <c r="BZ98">
+        <v>0.07017913309538087</v>
+      </c>
+      <c r="CA98">
+        <v>0.08893281438107985</v>
+      </c>
+      <c r="CB98">
+        <v>0.1413100704695084</v>
+      </c>
+      <c r="CC98">
+        <v>0.009795481970643513</v>
+      </c>
+      <c r="CD98">
+        <v>0.008861399332615755</v>
+      </c>
+      <c r="CE98">
+        <v>0.00779104086638735</v>
+      </c>
+      <c r="CF98">
+        <v>0.009251780235869525</v>
+      </c>
+      <c r="CG98">
+        <v>140641.64636</v>
+      </c>
+      <c r="CH98">
+        <v>8577.137600000002</v>
+      </c>
+      <c r="CI98">
+        <v>141847.3279377143</v>
+      </c>
+      <c r="CJ98">
+        <v>9314.604487889927</v>
+      </c>
+      <c r="CK98">
+        <v>0.0439565535038046</v>
+      </c>
+      <c r="CL98">
+        <v>0.08609282173737862</v>
+      </c>
+      <c r="CM98">
+        <v>10000</v>
+      </c>
+      <c r="CO98">
+        <v>0.002700617283950617</v>
+      </c>
+      <c r="CP98">
+        <v>0.01087962962962963</v>
+      </c>
+      <c r="CQ98">
+        <v>54716860.54549867</v>
+      </c>
+      <c r="CR98">
+        <v>8525723.260530123</v>
+      </c>
+      <c r="CS98" s="2">
+        <v>45409.44021866774</v>
+      </c>
+      <c r="CT98">
+        <v>-0.6066396906320848</v>
+      </c>
+      <c r="CU98">
+        <v>-0.8752543116523225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FETUSDT.json at 2024-04-27_17-01-38 bestfile_scores 0.002494905704451547 bestfile_sharp 0.12303288331650838
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU98"/>
+  <dimension ref="A1:CU99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -28751,6 +28751,275 @@
       </c>
       <c r="CU98">
         <v>-0.8752543116523225</v>
+      </c>
+    </row>
+    <row r="99" spans="10:99">
+      <c r="J99" t="s">
+        <v>220</v>
+      </c>
+      <c r="K99">
+        <v>0.001904643854209187</v>
+      </c>
+      <c r="L99">
+        <v>0.0009523219271045935</v>
+      </c>
+      <c r="M99">
+        <v>0.000139634041835146</v>
+      </c>
+      <c r="N99">
+        <v>0.000139634041835146</v>
+      </c>
+      <c r="O99">
+        <v>0.001410138339224965</v>
+      </c>
+      <c r="P99">
+        <v>0.0007050691696124823</v>
+      </c>
+      <c r="Q99">
+        <v>0.0001870633165961477</v>
+      </c>
+      <c r="R99">
+        <v>0.0001870633165961477</v>
+      </c>
+      <c r="S99">
+        <v>6.504880589528917</v>
+      </c>
+      <c r="T99">
+        <v>5.652069910104557</v>
+      </c>
+      <c r="U99">
+        <v>0.3678676944222574</v>
+      </c>
+      <c r="V99">
+        <v>0.806918318196289</v>
+      </c>
+      <c r="W99">
+        <v>0.03400655204622841</v>
+      </c>
+      <c r="X99">
+        <v>0.006420290217923527</v>
+      </c>
+      <c r="Y99">
+        <v>0.08522677615986263</v>
+      </c>
+      <c r="Z99">
+        <v>0.07115733982724726</v>
+      </c>
+      <c r="AA99">
+        <v>0.999306590597236</v>
+      </c>
+      <c r="AB99">
+        <v>0.9200664419365733</v>
+      </c>
+      <c r="AC99">
+        <v>0.9624039704872572</v>
+      </c>
+      <c r="AD99">
+        <v>0.9998528638546477</v>
+      </c>
+      <c r="AE99">
+        <v>0.7620288997348975</v>
+      </c>
+      <c r="AF99">
+        <v>0.9156932234417878</v>
+      </c>
+      <c r="AG99">
+        <v>0.00390693604999059</v>
+      </c>
+      <c r="AH99">
+        <v>0.001048376461190725</v>
+      </c>
+      <c r="AI99">
+        <v>0.999306590597236</v>
+      </c>
+      <c r="AJ99">
+        <v>0.9998528638546477</v>
+      </c>
+      <c r="AK99">
+        <v>0.00390693604999059</v>
+      </c>
+      <c r="AL99">
+        <v>0.001048376461190725</v>
+      </c>
+      <c r="AM99" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN99">
+        <v>0.02240953925806517</v>
+      </c>
+      <c r="AO99">
+        <v>0.006246780490074177</v>
+      </c>
+      <c r="AP99">
+        <v>-1800.71544278</v>
+      </c>
+      <c r="AQ99">
+        <v>-105.976210196</v>
+      </c>
+      <c r="AR99">
+        <v>78066.78777721986</v>
+      </c>
+      <c r="AS99">
+        <v>11627.50616980406</v>
+      </c>
+      <c r="AT99">
+        <v>77950.98611721986</v>
+      </c>
+      <c r="AU99">
+        <v>11627.50616980406</v>
+      </c>
+      <c r="AV99">
+        <v>6.806678777721985</v>
+      </c>
+      <c r="AW99">
+        <v>0.1627506169804063</v>
+      </c>
+      <c r="AX99">
+        <v>3.68378416856492</v>
+      </c>
+      <c r="AY99">
+        <v>4.239324922169425</v>
+      </c>
+      <c r="AZ99">
+        <v>117.5333333333333</v>
+      </c>
+      <c r="BA99">
+        <v>117.35</v>
+      </c>
+      <c r="BB99">
+        <v>0</v>
+      </c>
+      <c r="BC99">
+        <v>0</v>
+      </c>
+      <c r="BD99">
+        <v>0</v>
+      </c>
+      <c r="BE99">
+        <v>0</v>
+      </c>
+      <c r="BF99">
+        <v>2415</v>
+      </c>
+      <c r="BG99">
+        <v>2664</v>
+      </c>
+      <c r="BH99">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI99">
+        <v>4610</v>
+      </c>
+      <c r="BJ99">
+        <v>3440</v>
+      </c>
+      <c r="BK99">
+        <v>7025</v>
+      </c>
+      <c r="BL99">
+        <v>6104</v>
+      </c>
+      <c r="BM99">
+        <v>1902</v>
+      </c>
+      <c r="BN99">
+        <v>2657</v>
+      </c>
+      <c r="BO99">
+        <v>2415</v>
+      </c>
+      <c r="BP99">
+        <v>2663</v>
+      </c>
+      <c r="BQ99">
+        <v>2708</v>
+      </c>
+      <c r="BR99">
+        <v>783</v>
+      </c>
+      <c r="BS99">
+        <v>0</v>
+      </c>
+      <c r="BT99">
+        <v>1</v>
+      </c>
+      <c r="BU99">
+        <v>0</v>
+      </c>
+      <c r="BV99">
+        <v>0</v>
+      </c>
+      <c r="BW99">
+        <v>68066.78777722</v>
+      </c>
+      <c r="BX99">
+        <v>1627.506169804002</v>
+      </c>
+      <c r="BY99">
+        <v>0.04459078537378716</v>
+      </c>
+      <c r="BZ99">
+        <v>0.04776951700658841</v>
+      </c>
+      <c r="CA99">
+        <v>0.08671112269136108</v>
+      </c>
+      <c r="CB99">
+        <v>0.08201852555874979</v>
+      </c>
+      <c r="CC99">
+        <v>0.009595270536980954</v>
+      </c>
+      <c r="CD99">
+        <v>0.01707862459881886</v>
+      </c>
+      <c r="CE99">
+        <v>0.008347364322256233</v>
+      </c>
+      <c r="CF99">
+        <v>0.0124917739686979</v>
+      </c>
+      <c r="CG99">
+        <v>69867.50322</v>
+      </c>
+      <c r="CH99">
+        <v>1733.482380000002</v>
+      </c>
+      <c r="CI99">
+        <v>69867.50322</v>
+      </c>
+      <c r="CJ99">
+        <v>1733.482380000002</v>
+      </c>
+      <c r="CK99">
+        <v>0.1131558075594384</v>
+      </c>
+      <c r="CL99">
+        <v>0.1111649299944669</v>
+      </c>
+      <c r="CM99">
+        <v>10000</v>
+      </c>
+      <c r="CO99">
+        <v>0.0001157407407407407</v>
+      </c>
+      <c r="CP99">
+        <v>7.716049382716049E-05</v>
+      </c>
+      <c r="CQ99">
+        <v>20021841.69786059</v>
+      </c>
+      <c r="CR99">
+        <v>555000.5818001842</v>
+      </c>
+      <c r="CS99" s="2">
+        <v>45409.62940216029</v>
+      </c>
+      <c r="CT99">
+        <v>-0.7930559623825889</v>
+      </c>
+      <c r="CU99">
+        <v>-0.9922124347773956</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update CRVUSDT.json at 2024-04-27_22-51-50 bestfile_scores 0.00033985414138660024 bestfile_sharp 0.068882578547734
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU99"/>
+  <dimension ref="A1:CU100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -29020,6 +29020,275 @@
       </c>
       <c r="CU99">
         <v>-0.9922124347773956</v>
+      </c>
+    </row>
+    <row r="100" spans="10:99">
+      <c r="J100" t="s">
+        <v>221</v>
+      </c>
+      <c r="K100">
+        <v>0.001927664146863739</v>
+      </c>
+      <c r="L100">
+        <v>0.0009638320734318695</v>
+      </c>
+      <c r="M100">
+        <v>0.002330707350674199</v>
+      </c>
+      <c r="N100">
+        <v>0.002330707350674199</v>
+      </c>
+      <c r="O100">
+        <v>0.005921679765900012</v>
+      </c>
+      <c r="P100">
+        <v>0.002960839882950006</v>
+      </c>
+      <c r="Q100">
+        <v>0.003724243510750114</v>
+      </c>
+      <c r="R100">
+        <v>0.003724243510750114</v>
+      </c>
+      <c r="S100">
+        <v>32.94231285215992</v>
+      </c>
+      <c r="T100">
+        <v>21.05285752616045</v>
+      </c>
+      <c r="U100">
+        <v>0.4453135954162409</v>
+      </c>
+      <c r="V100">
+        <v>0.8043597552982236</v>
+      </c>
+      <c r="W100">
+        <v>0.007279588621229223</v>
+      </c>
+      <c r="X100">
+        <v>0.02883556913316065</v>
+      </c>
+      <c r="Y100">
+        <v>0.06991449476328819</v>
+      </c>
+      <c r="Z100">
+        <v>0.07721555145363306</v>
+      </c>
+      <c r="AA100">
+        <v>0.9996035337617997</v>
+      </c>
+      <c r="AB100">
+        <v>0.9707791562731835</v>
+      </c>
+      <c r="AC100">
+        <v>0.9332527375842909</v>
+      </c>
+      <c r="AD100">
+        <v>0.9995676926073706</v>
+      </c>
+      <c r="AE100">
+        <v>0.9304205838176882</v>
+      </c>
+      <c r="AF100">
+        <v>0.9190872477901054</v>
+      </c>
+      <c r="AG100">
+        <v>0.001261427466810674</v>
+      </c>
+      <c r="AH100">
+        <v>0.003422720658006529</v>
+      </c>
+      <c r="AI100">
+        <v>0.9996035337617997</v>
+      </c>
+      <c r="AJ100">
+        <v>0.9995676926073706</v>
+      </c>
+      <c r="AK100">
+        <v>0.001261427466810674</v>
+      </c>
+      <c r="AL100">
+        <v>0.003422720658006529</v>
+      </c>
+      <c r="AM100" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN100">
+        <v>0.01203565385830771</v>
+      </c>
+      <c r="AO100">
+        <v>0.02369614773541375</v>
+      </c>
+      <c r="AP100">
+        <v>-696.4070824</v>
+      </c>
+      <c r="AQ100">
+        <v>-1148.22042206</v>
+      </c>
+      <c r="AR100">
+        <v>24526.91701760042</v>
+      </c>
+      <c r="AS100">
+        <v>29581.22827794016</v>
+      </c>
+      <c r="AT100">
+        <v>24511.66291760042</v>
+      </c>
+      <c r="AU100">
+        <v>29581.22827794016</v>
+      </c>
+      <c r="AV100">
+        <v>1.452691701760042</v>
+      </c>
+      <c r="AW100">
+        <v>1.958122827794016</v>
+      </c>
+      <c r="AX100">
+        <v>0.7279247578087666</v>
+      </c>
+      <c r="AY100">
+        <v>1.137395057951803</v>
+      </c>
+      <c r="AZ100">
+        <v>97.2</v>
+      </c>
+      <c r="BA100">
+        <v>93.7</v>
+      </c>
+      <c r="BB100">
+        <v>0</v>
+      </c>
+      <c r="BC100">
+        <v>0.0008734463648607701</v>
+      </c>
+      <c r="BD100">
+        <v>0</v>
+      </c>
+      <c r="BE100">
+        <v>-18.12189011162523</v>
+      </c>
+      <c r="BF100">
+        <v>6920</v>
+      </c>
+      <c r="BG100">
+        <v>3991</v>
+      </c>
+      <c r="BH100">
+        <v>465.875</v>
+      </c>
+      <c r="BI100">
+        <v>8427</v>
+      </c>
+      <c r="BJ100">
+        <v>5817</v>
+      </c>
+      <c r="BK100">
+        <v>15347</v>
+      </c>
+      <c r="BL100">
+        <v>9808</v>
+      </c>
+      <c r="BM100">
+        <v>6916</v>
+      </c>
+      <c r="BN100">
+        <v>3274</v>
+      </c>
+      <c r="BO100">
+        <v>6919</v>
+      </c>
+      <c r="BP100">
+        <v>3987</v>
+      </c>
+      <c r="BQ100">
+        <v>1511</v>
+      </c>
+      <c r="BR100">
+        <v>2543</v>
+      </c>
+      <c r="BS100">
+        <v>1</v>
+      </c>
+      <c r="BT100">
+        <v>4</v>
+      </c>
+      <c r="BU100">
+        <v>0</v>
+      </c>
+      <c r="BV100">
+        <v>0</v>
+      </c>
+      <c r="BW100">
+        <v>14526.9170176</v>
+      </c>
+      <c r="BX100">
+        <v>19581.22827794001</v>
+      </c>
+      <c r="BY100">
+        <v>0.03841665594891724</v>
+      </c>
+      <c r="BZ100">
+        <v>0.04136129648179634</v>
+      </c>
+      <c r="CA100">
+        <v>0.0462686505272458</v>
+      </c>
+      <c r="CB100">
+        <v>0.07484513389269476</v>
+      </c>
+      <c r="CC100">
+        <v>0.01535233635040644</v>
+      </c>
+      <c r="CD100">
+        <v>0.006793004406480699</v>
+      </c>
+      <c r="CE100">
+        <v>0.009459484517917191</v>
+      </c>
+      <c r="CF100">
+        <v>0.00835469396394469</v>
+      </c>
+      <c r="CG100">
+        <v>15223.3241</v>
+      </c>
+      <c r="CH100">
+        <v>20729.44870000001</v>
+      </c>
+      <c r="CI100">
+        <v>15223.3241</v>
+      </c>
+      <c r="CJ100">
+        <v>20747.57059011164</v>
+      </c>
+      <c r="CK100">
+        <v>0.1230328833165084</v>
+      </c>
+      <c r="CL100">
+        <v>0.3119010752537739</v>
+      </c>
+      <c r="CM100">
+        <v>10000</v>
+      </c>
+      <c r="CO100">
+        <v>0.0004471472008585226</v>
+      </c>
+      <c r="CP100">
+        <v>0.01010552673940261</v>
+      </c>
+      <c r="CQ100">
+        <v>2568699.750780469</v>
+      </c>
+      <c r="CR100">
+        <v>8829982.660321526</v>
+      </c>
+      <c r="CS100" s="2">
+        <v>45409.70949660632</v>
+      </c>
+      <c r="CT100">
+        <v>-0.8625963918106255</v>
+      </c>
+      <c r="CU100">
+        <v>-0.7644627443434996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MANAUSDT.json at 2024-04-28_02-24-53 bestfile_scores 0.0005320316342185966 bestfile_sharp 0.08808200187362383
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="972" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU100"/>
+  <dimension ref="A1:CU101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -29289,6 +29289,275 @@
       </c>
       <c r="CU100">
         <v>-0.7644627443434996</v>
+      </c>
+    </row>
+    <row r="101" spans="10:99">
+      <c r="J101" t="s">
+        <v>222</v>
+      </c>
+      <c r="K101">
+        <v>0.0006590659869258886</v>
+      </c>
+      <c r="L101">
+        <v>0.0003295329934629443</v>
+      </c>
+      <c r="M101">
+        <v>0.0005030850930884956</v>
+      </c>
+      <c r="N101">
+        <v>0.0005030850930884956</v>
+      </c>
+      <c r="O101">
+        <v>0.0004104813007887786</v>
+      </c>
+      <c r="P101">
+        <v>0.0002052406503943893</v>
+      </c>
+      <c r="Q101">
+        <v>0.0003215578286005716</v>
+      </c>
+      <c r="R101">
+        <v>0.0003215578286005716</v>
+      </c>
+      <c r="S101">
+        <v>20.1618889617655</v>
+      </c>
+      <c r="T101">
+        <v>23.06755661869671</v>
+      </c>
+      <c r="U101">
+        <v>0.6938060539392945</v>
+      </c>
+      <c r="V101">
+        <v>0.7724397879288504</v>
+      </c>
+      <c r="W101">
+        <v>0.06719557602005968</v>
+      </c>
+      <c r="X101">
+        <v>0.01817679112504592</v>
+      </c>
+      <c r="Y101">
+        <v>0.2356048934149554</v>
+      </c>
+      <c r="Z101">
+        <v>0.1094944971213034</v>
+      </c>
+      <c r="AA101">
+        <v>0.9981596081058777</v>
+      </c>
+      <c r="AB101">
+        <v>0.816794210098631</v>
+      </c>
+      <c r="AC101">
+        <v>0.9236226078872566</v>
+      </c>
+      <c r="AD101">
+        <v>0.9995898093475288</v>
+      </c>
+      <c r="AE101">
+        <v>0.7557843707566519</v>
+      </c>
+      <c r="AF101">
+        <v>0.8906788368119825</v>
+      </c>
+      <c r="AG101">
+        <v>0.008113378368000364</v>
+      </c>
+      <c r="AH101">
+        <v>0.002451216814968625</v>
+      </c>
+      <c r="AI101">
+        <v>0.9981596081058777</v>
+      </c>
+      <c r="AJ101">
+        <v>0.9995898093475288</v>
+      </c>
+      <c r="AK101">
+        <v>0.008113378368000364</v>
+      </c>
+      <c r="AL101">
+        <v>0.002451216814968625</v>
+      </c>
+      <c r="AM101" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN101">
+        <v>0.02371480284020294</v>
+      </c>
+      <c r="AO101">
+        <v>0.01978873312947207</v>
+      </c>
+      <c r="AP101">
+        <v>-868.68920354</v>
+      </c>
+      <c r="AQ101">
+        <v>-747.4953056000001</v>
+      </c>
+      <c r="AR101">
+        <v>20371.04339645985</v>
+      </c>
+      <c r="AS101">
+        <v>17214.6266944001</v>
+      </c>
+      <c r="AT101">
+        <v>20367.39779645985</v>
+      </c>
+      <c r="AU101">
+        <v>17214.0332944001</v>
+      </c>
+      <c r="AV101">
+        <v>1.037104339645985</v>
+      </c>
+      <c r="AW101">
+        <v>0.7214626694400104</v>
+      </c>
+      <c r="AX101">
+        <v>1.18770189378282</v>
+      </c>
+      <c r="AY101">
+        <v>1.039486572197021</v>
+      </c>
+      <c r="AZ101">
+        <v>150.0333333333333</v>
+      </c>
+      <c r="BA101">
+        <v>99.43333333333334</v>
+      </c>
+      <c r="BB101">
+        <v>0.01990805050714554</v>
+      </c>
+      <c r="BC101">
+        <v>0.00419297621006568</v>
+      </c>
+      <c r="BD101">
+        <v>-228.3062975911539</v>
+      </c>
+      <c r="BE101">
+        <v>-33.52556000316297</v>
+      </c>
+      <c r="BF101">
+        <v>8877</v>
+      </c>
+      <c r="BG101">
+        <v>11473</v>
+      </c>
+      <c r="BH101">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI101">
+        <v>12897</v>
+      </c>
+      <c r="BJ101">
+        <v>13439</v>
+      </c>
+      <c r="BK101">
+        <v>21774</v>
+      </c>
+      <c r="BL101">
+        <v>24912</v>
+      </c>
+      <c r="BM101">
+        <v>8841</v>
+      </c>
+      <c r="BN101">
+        <v>11309</v>
+      </c>
+      <c r="BO101">
+        <v>8869</v>
+      </c>
+      <c r="BP101">
+        <v>11471</v>
+      </c>
+      <c r="BQ101">
+        <v>4056</v>
+      </c>
+      <c r="BR101">
+        <v>2130</v>
+      </c>
+      <c r="BS101">
+        <v>8</v>
+      </c>
+      <c r="BT101">
+        <v>2</v>
+      </c>
+      <c r="BU101">
+        <v>0</v>
+      </c>
+      <c r="BV101">
+        <v>0</v>
+      </c>
+      <c r="BW101">
+        <v>10371.04339645998</v>
+      </c>
+      <c r="BX101">
+        <v>7214.6266944</v>
+      </c>
+      <c r="BY101">
+        <v>0.09812673689620358</v>
+      </c>
+      <c r="BZ101">
+        <v>0.04467018124666684</v>
+      </c>
+      <c r="CA101">
+        <v>0.2162790320138415</v>
+      </c>
+      <c r="CB101">
+        <v>0.09853717343290397</v>
+      </c>
+      <c r="CC101">
+        <v>0.02055497814823072</v>
+      </c>
+      <c r="CD101">
+        <v>0.01243602382530077</v>
+      </c>
+      <c r="CE101">
+        <v>0.01575305393079747</v>
+      </c>
+      <c r="CF101">
+        <v>0.009151227796929836</v>
+      </c>
+      <c r="CG101">
+        <v>11239.73259999998</v>
+      </c>
+      <c r="CH101">
+        <v>7962.122</v>
+      </c>
+      <c r="CI101">
+        <v>11468.03889759113</v>
+      </c>
+      <c r="CJ101">
+        <v>7995.647560003164</v>
+      </c>
+      <c r="CK101">
+        <v>0.068882578547734</v>
+      </c>
+      <c r="CL101">
+        <v>0.1581455233325068</v>
+      </c>
+      <c r="CM101">
+        <v>10000</v>
+      </c>
+      <c r="CO101">
+        <v>0</v>
+      </c>
+      <c r="CP101">
+        <v>0.002816358024691358</v>
+      </c>
+      <c r="CQ101">
+        <v>7775586.179986647</v>
+      </c>
+      <c r="CR101">
+        <v>3109464.939265249</v>
+      </c>
+      <c r="CS101" s="2">
+        <v>45409.95268396772</v>
+      </c>
+      <c r="CT101">
+        <v>-0.8320151516141147</v>
+      </c>
+      <c r="CU101">
+        <v>-0.9612574350521926</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FTMUSDT.json at 2024-04-28_06-30-18 bestfile_scores 0.0006908067957055008 bestfile_sharp 0.0712883361735744
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU101"/>
+  <dimension ref="A1:CU102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -29558,6 +29558,275 @@
       </c>
       <c r="CU101">
         <v>-0.9612574350521926</v>
+      </c>
+    </row>
+    <row r="102" spans="10:99">
+      <c r="J102" t="s">
+        <v>223</v>
+      </c>
+      <c r="K102">
+        <v>0.001141810493367146</v>
+      </c>
+      <c r="L102">
+        <v>0.0005709052466835729</v>
+      </c>
+      <c r="M102">
+        <v>0.0004038368310985696</v>
+      </c>
+      <c r="N102">
+        <v>0.0004038368310985696</v>
+      </c>
+      <c r="O102">
+        <v>0.001841158394997078</v>
+      </c>
+      <c r="P102">
+        <v>0.0009205791974985389</v>
+      </c>
+      <c r="Q102">
+        <v>0.0002328052615937049</v>
+      </c>
+      <c r="R102">
+        <v>0.0002328052615937049</v>
+      </c>
+      <c r="S102">
+        <v>24.21945291099194</v>
+      </c>
+      <c r="T102">
+        <v>5.515027585940816</v>
+      </c>
+      <c r="U102">
+        <v>0.3274412692468422</v>
+      </c>
+      <c r="V102">
+        <v>0.5960294392258227</v>
+      </c>
+      <c r="W102">
+        <v>0.006304188258278291</v>
+      </c>
+      <c r="X102">
+        <v>0.009499962412590783</v>
+      </c>
+      <c r="Y102">
+        <v>0.0759006491185369</v>
+      </c>
+      <c r="Z102">
+        <v>0.07127258026016152</v>
+      </c>
+      <c r="AA102">
+        <v>0.9998960000842839</v>
+      </c>
+      <c r="AB102">
+        <v>0.9409871524587657</v>
+      </c>
+      <c r="AC102">
+        <v>0.9638066853214451</v>
+      </c>
+      <c r="AD102">
+        <v>0.9997043332417299</v>
+      </c>
+      <c r="AE102">
+        <v>0.8240639188140662</v>
+      </c>
+      <c r="AF102">
+        <v>0.9243131411179735</v>
+      </c>
+      <c r="AG102">
+        <v>0.001425260922186125</v>
+      </c>
+      <c r="AH102">
+        <v>0.001313652318793831</v>
+      </c>
+      <c r="AI102">
+        <v>0.9998960000842839</v>
+      </c>
+      <c r="AJ102">
+        <v>0.9997043332417299</v>
+      </c>
+      <c r="AK102">
+        <v>0.001425260922186125</v>
+      </c>
+      <c r="AL102">
+        <v>0.001313652318793831</v>
+      </c>
+      <c r="AM102" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN102">
+        <v>0.00395972548026189</v>
+      </c>
+      <c r="AO102">
+        <v>0.01079946062967898</v>
+      </c>
+      <c r="AP102">
+        <v>-2091.63947524</v>
+      </c>
+      <c r="AQ102">
+        <v>-267.94375262</v>
+      </c>
+      <c r="AR102">
+        <v>34294.65112475909</v>
+      </c>
+      <c r="AS102">
+        <v>15465.68974737985</v>
+      </c>
+      <c r="AT102">
+        <v>34295.10652475909</v>
+      </c>
+      <c r="AU102">
+        <v>15465.68974737985</v>
+      </c>
+      <c r="AV102">
+        <v>2.429465112475909</v>
+      </c>
+      <c r="AW102">
+        <v>0.5465689747379852</v>
+      </c>
+      <c r="AX102">
+        <v>0.9903262601159752</v>
+      </c>
+      <c r="AY102">
+        <v>4.34335852225021</v>
+      </c>
+      <c r="AZ102">
+        <v>101.6333333333333</v>
+      </c>
+      <c r="BA102">
+        <v>118.2</v>
+      </c>
+      <c r="BB102">
+        <v>0.0009617602890207441</v>
+      </c>
+      <c r="BC102">
+        <v>0</v>
+      </c>
+      <c r="BD102">
+        <v>-25.40171683616734</v>
+      </c>
+      <c r="BE102">
+        <v>0</v>
+      </c>
+      <c r="BF102">
+        <v>12374</v>
+      </c>
+      <c r="BG102">
+        <v>2738</v>
+      </c>
+      <c r="BH102">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI102">
+        <v>13782</v>
+      </c>
+      <c r="BJ102">
+        <v>3218</v>
+      </c>
+      <c r="BK102">
+        <v>26156</v>
+      </c>
+      <c r="BL102">
+        <v>5956</v>
+      </c>
+      <c r="BM102">
+        <v>12351</v>
+      </c>
+      <c r="BN102">
+        <v>2670</v>
+      </c>
+      <c r="BO102">
+        <v>12372</v>
+      </c>
+      <c r="BP102">
+        <v>2738</v>
+      </c>
+      <c r="BQ102">
+        <v>1431</v>
+      </c>
+      <c r="BR102">
+        <v>548</v>
+      </c>
+      <c r="BS102">
+        <v>2</v>
+      </c>
+      <c r="BT102">
+        <v>0</v>
+      </c>
+      <c r="BU102">
+        <v>0</v>
+      </c>
+      <c r="BV102">
+        <v>0</v>
+      </c>
+      <c r="BW102">
+        <v>24294.65112476002</v>
+      </c>
+      <c r="BX102">
+        <v>5465.689747380001</v>
+      </c>
+      <c r="BY102">
+        <v>0.02939592294047228</v>
+      </c>
+      <c r="BZ102">
+        <v>0.07424968929253103</v>
+      </c>
+      <c r="CA102">
+        <v>0.0424986144881274</v>
+      </c>
+      <c r="CB102">
+        <v>0.1454596819859194</v>
+      </c>
+      <c r="CC102">
+        <v>0.009901271238412994</v>
+      </c>
+      <c r="CD102">
+        <v>0.01694801805916242</v>
+      </c>
+      <c r="CE102">
+        <v>0.00756081763249433</v>
+      </c>
+      <c r="CF102">
+        <v>0.01540162304544166</v>
+      </c>
+      <c r="CG102">
+        <v>26386.29060000002</v>
+      </c>
+      <c r="CH102">
+        <v>5733.633500000001</v>
+      </c>
+      <c r="CI102">
+        <v>26411.69231683619</v>
+      </c>
+      <c r="CJ102">
+        <v>5733.633500000001</v>
+      </c>
+      <c r="CK102">
+        <v>0.08808200187362383</v>
+      </c>
+      <c r="CL102">
+        <v>0.1685275112826306</v>
+      </c>
+      <c r="CM102">
+        <v>10000</v>
+      </c>
+      <c r="CO102">
+        <v>0.001080246913580247</v>
+      </c>
+      <c r="CP102">
+        <v>0.0005787037037037037</v>
+      </c>
+      <c r="CQ102">
+        <v>6561850.585549068</v>
+      </c>
+      <c r="CR102">
+        <v>1199182.410839436</v>
+      </c>
+      <c r="CS102" s="2">
+        <v>45410.10063387676</v>
+      </c>
+      <c r="CT102">
+        <v>-0.9034091343725907</v>
+      </c>
+      <c r="CU102">
+        <v>-0.9732638426030944</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update EOSUSDT.json at 2024-04-28_11-14-20 bestfile_scores 0.0007518066026225734 bestfile_sharp 0.14832807639722262
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="976" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="978" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU102"/>
+  <dimension ref="A1:CU103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -29827,6 +29827,275 @@
       </c>
       <c r="CU102">
         <v>-0.9732638426030944</v>
+      </c>
+    </row>
+    <row r="103" spans="10:99">
+      <c r="J103" t="s">
+        <v>224</v>
+      </c>
+      <c r="K103">
+        <v>0.00119003024969655</v>
+      </c>
+      <c r="L103">
+        <v>0.0005950151248482749</v>
+      </c>
+      <c r="M103">
+        <v>0.0007957399963407497</v>
+      </c>
+      <c r="N103">
+        <v>0.0007957399963407497</v>
+      </c>
+      <c r="O103">
+        <v>0.00131053771795453</v>
+      </c>
+      <c r="P103">
+        <v>0.0006552688589772648</v>
+      </c>
+      <c r="Q103">
+        <v>0.0007172032026557141</v>
+      </c>
+      <c r="R103">
+        <v>0.0007172032026557141</v>
+      </c>
+      <c r="S103">
+        <v>21.17319945935509</v>
+      </c>
+      <c r="T103">
+        <v>17.39826221278239</v>
+      </c>
+      <c r="U103">
+        <v>0.434376412305491</v>
+      </c>
+      <c r="V103">
+        <v>0.7252427292906195</v>
+      </c>
+      <c r="W103">
+        <v>0.02447751475053921</v>
+      </c>
+      <c r="X103">
+        <v>0.01949319935603695</v>
+      </c>
+      <c r="Y103">
+        <v>0.1620646973060086</v>
+      </c>
+      <c r="Z103">
+        <v>0.1073843570349158</v>
+      </c>
+      <c r="AA103">
+        <v>0.9996849773002762</v>
+      </c>
+      <c r="AB103">
+        <v>0.8659360878197271</v>
+      </c>
+      <c r="AC103">
+        <v>0.9148277528931772</v>
+      </c>
+      <c r="AD103">
+        <v>0.999626177816024</v>
+      </c>
+      <c r="AE103">
+        <v>0.8382705861165679</v>
+      </c>
+      <c r="AF103">
+        <v>0.8927916427205046</v>
+      </c>
+      <c r="AG103">
+        <v>0.00411457990882796</v>
+      </c>
+      <c r="AH103">
+        <v>0.002666022979249212</v>
+      </c>
+      <c r="AI103">
+        <v>0.9996849773002762</v>
+      </c>
+      <c r="AJ103">
+        <v>0.999626177816024</v>
+      </c>
+      <c r="AK103">
+        <v>0.00411457990882796</v>
+      </c>
+      <c r="AL103">
+        <v>0.002666022979249212</v>
+      </c>
+      <c r="AM103" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN103">
+        <v>0.006275468914856508</v>
+      </c>
+      <c r="AO103">
+        <v>0.01683186095188041</v>
+      </c>
+      <c r="AP103">
+        <v>-1872.380595522</v>
+      </c>
+      <c r="AQ103">
+        <v>-990.723025596</v>
+      </c>
+      <c r="AR103">
+        <v>36082.74445447791</v>
+      </c>
+      <c r="AS103">
+        <v>23589.78961440436</v>
+      </c>
+      <c r="AT103">
+        <v>36082.74445447791</v>
+      </c>
+      <c r="AU103">
+        <v>23589.78961440436</v>
+      </c>
+      <c r="AV103">
+        <v>2.608274445447791</v>
+      </c>
+      <c r="AW103">
+        <v>1.358978961440436</v>
+      </c>
+      <c r="AX103">
+        <v>1.133353032160159</v>
+      </c>
+      <c r="AY103">
+        <v>1.378217285529096</v>
+      </c>
+      <c r="AZ103">
+        <v>91.61666666666666</v>
+      </c>
+      <c r="BA103">
+        <v>117.5833333333333</v>
+      </c>
+      <c r="BB103">
+        <v>0.01075464633552679</v>
+      </c>
+      <c r="BC103">
+        <v>0.03223555878407724</v>
+      </c>
+      <c r="BD103">
+        <v>-303.9159921898887</v>
+      </c>
+      <c r="BE103">
+        <v>-485.6667100913197</v>
+      </c>
+      <c r="BF103">
+        <v>10859</v>
+      </c>
+      <c r="BG103">
+        <v>8877</v>
+      </c>
+      <c r="BH103">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI103">
+        <v>11986</v>
+      </c>
+      <c r="BJ103">
+        <v>9895</v>
+      </c>
+      <c r="BK103">
+        <v>22845</v>
+      </c>
+      <c r="BL103">
+        <v>18772</v>
+      </c>
+      <c r="BM103">
+        <v>10804</v>
+      </c>
+      <c r="BN103">
+        <v>8538</v>
+      </c>
+      <c r="BO103">
+        <v>10819</v>
+      </c>
+      <c r="BP103">
+        <v>8848</v>
+      </c>
+      <c r="BQ103">
+        <v>1182</v>
+      </c>
+      <c r="BR103">
+        <v>1357</v>
+      </c>
+      <c r="BS103">
+        <v>40</v>
+      </c>
+      <c r="BT103">
+        <v>29</v>
+      </c>
+      <c r="BU103">
+        <v>0</v>
+      </c>
+      <c r="BV103">
+        <v>0</v>
+      </c>
+      <c r="BW103">
+        <v>26082.74445447801</v>
+      </c>
+      <c r="BX103">
+        <v>13589.78961440401</v>
+      </c>
+      <c r="BY103">
+        <v>0.04253707060674984</v>
+      </c>
+      <c r="BZ103">
+        <v>0.05282370034353917</v>
+      </c>
+      <c r="CA103">
+        <v>0.08794790866976307</v>
+      </c>
+      <c r="CB103">
+        <v>0.0968117340700573</v>
+      </c>
+      <c r="CC103">
+        <v>0.01416398854736472</v>
+      </c>
+      <c r="CD103">
+        <v>0.01372604118772669</v>
+      </c>
+      <c r="CE103">
+        <v>0.01075841036298861</v>
+      </c>
+      <c r="CF103">
+        <v>0.01138198108102824</v>
+      </c>
+      <c r="CG103">
+        <v>27955.12505000001</v>
+      </c>
+      <c r="CH103">
+        <v>14580.51264000001</v>
+      </c>
+      <c r="CI103">
+        <v>28259.0410421899</v>
+      </c>
+      <c r="CJ103">
+        <v>15066.17935009133</v>
+      </c>
+      <c r="CK103">
+        <v>0.0712883361735744</v>
+      </c>
+      <c r="CL103">
+        <v>0.2227065491209557</v>
+      </c>
+      <c r="CM103">
+        <v>10000</v>
+      </c>
+      <c r="CO103">
+        <v>0.00251004016064257</v>
+      </c>
+      <c r="CP103">
+        <v>0.005020080321285141</v>
+      </c>
+      <c r="CQ103">
+        <v>7056587.606235802</v>
+      </c>
+      <c r="CR103">
+        <v>5608278.16173986</v>
+      </c>
+      <c r="CS103" s="2">
+        <v>45410.27105927056</v>
+      </c>
+      <c r="CT103">
+        <v>-0.8495964311677586</v>
+      </c>
+      <c r="CU103">
+        <v>-0.9372184121885635</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AAVEUSDT.json at 2024-04-29_01-19-35 bestfile_scores 0.0006175618540669836 bestfile_sharp 0.04271624393225256
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="980" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU104"/>
+  <dimension ref="A1:CU105"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -30365,6 +30365,275 @@
       </c>
       <c r="CU104">
         <v>-0.670303567439911</v>
+      </c>
+    </row>
+    <row r="105" spans="10:99">
+      <c r="J105" t="s">
+        <v>226</v>
+      </c>
+      <c r="K105">
+        <v>0.0009090305436314505</v>
+      </c>
+      <c r="L105">
+        <v>0.0004545152718157253</v>
+      </c>
+      <c r="M105">
+        <v>0.0007417202666315514</v>
+      </c>
+      <c r="N105">
+        <v>0.0007417202666315514</v>
+      </c>
+      <c r="O105">
+        <v>0.0006842854275498578</v>
+      </c>
+      <c r="P105">
+        <v>0.0003421427137749289</v>
+      </c>
+      <c r="Q105">
+        <v>0.0004551994539658155</v>
+      </c>
+      <c r="R105">
+        <v>0.0004551994539658155</v>
+      </c>
+      <c r="S105">
+        <v>13.72089972606968</v>
+      </c>
+      <c r="T105">
+        <v>11.73008217909642</v>
+      </c>
+      <c r="U105">
+        <v>0.4087654934560896</v>
+      </c>
+      <c r="V105">
+        <v>0.2390741279549037</v>
+      </c>
+      <c r="W105">
+        <v>0.05599479054013765</v>
+      </c>
+      <c r="X105">
+        <v>0.07521021827532988</v>
+      </c>
+      <c r="Y105">
+        <v>0.1364709291217586</v>
+      </c>
+      <c r="Z105">
+        <v>0.245896375102084</v>
+      </c>
+      <c r="AA105">
+        <v>0.9989080176430586</v>
+      </c>
+      <c r="AB105">
+        <v>0.8881671096511858</v>
+      </c>
+      <c r="AC105">
+        <v>0.7911825617797408</v>
+      </c>
+      <c r="AD105">
+        <v>0.9991709928114206</v>
+      </c>
+      <c r="AE105">
+        <v>0.7925819995790636</v>
+      </c>
+      <c r="AF105">
+        <v>0.2970520619048237</v>
+      </c>
+      <c r="AG105">
+        <v>0.004779146039613252</v>
+      </c>
+      <c r="AH105">
+        <v>0.009010283759930291</v>
+      </c>
+      <c r="AI105">
+        <v>0.9989080176430586</v>
+      </c>
+      <c r="AJ105">
+        <v>0.9991709928114206</v>
+      </c>
+      <c r="AK105">
+        <v>0.004779146039613252</v>
+      </c>
+      <c r="AL105">
+        <v>0.009010283759930291</v>
+      </c>
+      <c r="AM105" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN105">
+        <v>0.02160876907266873</v>
+      </c>
+      <c r="AO105">
+        <v>0.01987737015118875</v>
+      </c>
+      <c r="AP105">
+        <v>-1168.0424578</v>
+      </c>
+      <c r="AQ105">
+        <v>-601.025981</v>
+      </c>
+      <c r="AR105">
+        <v>26678.40054220002</v>
+      </c>
+      <c r="AS105">
+        <v>22271.66301900009</v>
+      </c>
+      <c r="AT105">
+        <v>26673.26454220002</v>
+      </c>
+      <c r="AU105">
+        <v>22268.50201900009</v>
+      </c>
+      <c r="AV105">
+        <v>1.667840054220002</v>
+      </c>
+      <c r="AW105">
+        <v>1.227166301900009</v>
+      </c>
+      <c r="AX105">
+        <v>1.74787518840971</v>
+      </c>
+      <c r="AY105">
+        <v>2.04288045051446</v>
+      </c>
+      <c r="AZ105">
+        <v>107.1333333333333</v>
+      </c>
+      <c r="BA105">
+        <v>89.90000000000001</v>
+      </c>
+      <c r="BB105">
+        <v>0.07635018217762098</v>
+      </c>
+      <c r="BC105">
+        <v>0.04643347432102433</v>
+      </c>
+      <c r="BD105">
+        <v>-1475.211869239558</v>
+      </c>
+      <c r="BE105">
+        <v>-626.8295478371909</v>
+      </c>
+      <c r="BF105">
+        <v>6253</v>
+      </c>
+      <c r="BG105">
+        <v>4506</v>
+      </c>
+      <c r="BH105">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI105">
+        <v>8565</v>
+      </c>
+      <c r="BJ105">
+        <v>8162</v>
+      </c>
+      <c r="BK105">
+        <v>14818</v>
+      </c>
+      <c r="BL105">
+        <v>12668</v>
+      </c>
+      <c r="BM105">
+        <v>6262</v>
+      </c>
+      <c r="BN105">
+        <v>3881</v>
+      </c>
+      <c r="BO105">
+        <v>6240</v>
+      </c>
+      <c r="BP105">
+        <v>4489</v>
+      </c>
+      <c r="BQ105">
+        <v>2303</v>
+      </c>
+      <c r="BR105">
+        <v>4281</v>
+      </c>
+      <c r="BS105">
+        <v>13</v>
+      </c>
+      <c r="BT105">
+        <v>17</v>
+      </c>
+      <c r="BU105">
+        <v>0</v>
+      </c>
+      <c r="BV105">
+        <v>0</v>
+      </c>
+      <c r="BW105">
+        <v>16678.4005422</v>
+      </c>
+      <c r="BX105">
+        <v>12271.66301900002</v>
+      </c>
+      <c r="BY105">
+        <v>0.05399167443921493</v>
+      </c>
+      <c r="BZ105">
+        <v>0.06932115595886859</v>
+      </c>
+      <c r="CA105">
+        <v>0.1054371157335934</v>
+      </c>
+      <c r="CB105">
+        <v>0.1966692048761269</v>
+      </c>
+      <c r="CC105">
+        <v>0.01895426743586637</v>
+      </c>
+      <c r="CD105">
+        <v>0.01109189749929689</v>
+      </c>
+      <c r="CE105">
+        <v>0.01199984809464267</v>
+      </c>
+      <c r="CF105">
+        <v>0.01137461073218787</v>
+      </c>
+      <c r="CG105">
+        <v>17846.44300000001</v>
+      </c>
+      <c r="CH105">
+        <v>12872.68900000002</v>
+      </c>
+      <c r="CI105">
+        <v>19321.65486923957</v>
+      </c>
+      <c r="CJ105">
+        <v>13499.51854783722</v>
+      </c>
+      <c r="CK105">
+        <v>0.1095667880976366</v>
+      </c>
+      <c r="CL105">
+        <v>0.1039902108061576</v>
+      </c>
+      <c r="CM105">
+        <v>10000</v>
+      </c>
+      <c r="CO105">
+        <v>0.001118827160493827</v>
+      </c>
+      <c r="CP105">
+        <v>0.008449074074074074</v>
+      </c>
+      <c r="CQ105">
+        <v>6441318.236132834</v>
+      </c>
+      <c r="CR105">
+        <v>10577375.81046865</v>
+      </c>
+      <c r="CS105" s="2">
+        <v>45410.86880564898</v>
+      </c>
+      <c r="CT105">
+        <v>-0.8842562871250494</v>
+      </c>
+      <c r="CU105">
+        <v>-0.8332615644573296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update CHZUSDT.json at 2024-04-29_04-57-20 bestfile_scores 0.0007860662763049864 bestfile_sharp 0.048312461980297365
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU105"/>
+  <dimension ref="A1:CU106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -30634,6 +30634,275 @@
       </c>
       <c r="CU105">
         <v>-0.8332615644573296</v>
+      </c>
+    </row>
+    <row r="106" spans="10:99">
+      <c r="J106" t="s">
+        <v>227</v>
+      </c>
+      <c r="K106">
+        <v>0.0009978406305031218</v>
+      </c>
+      <c r="L106">
+        <v>0.0004989203152515609</v>
+      </c>
+      <c r="M106">
+        <v>0.0005596173403421556</v>
+      </c>
+      <c r="N106">
+        <v>0.0005596173403421556</v>
+      </c>
+      <c r="O106">
+        <v>0.0009496932983324325</v>
+      </c>
+      <c r="P106">
+        <v>0.0004748466491662162</v>
+      </c>
+      <c r="Q106">
+        <v>0.0009368631115080017</v>
+      </c>
+      <c r="R106">
+        <v>0.0009368631115080017</v>
+      </c>
+      <c r="S106">
+        <v>10.19020795555384</v>
+      </c>
+      <c r="T106">
+        <v>22.16937381843436</v>
+      </c>
+      <c r="U106">
+        <v>0.3596967054957878</v>
+      </c>
+      <c r="V106">
+        <v>0.7732888810334636</v>
+      </c>
+      <c r="W106">
+        <v>0.0205488615302067</v>
+      </c>
+      <c r="X106">
+        <v>0.04643158470702363</v>
+      </c>
+      <c r="Y106">
+        <v>0.1515384109676206</v>
+      </c>
+      <c r="Z106">
+        <v>0.1167513491525133</v>
+      </c>
+      <c r="AA106">
+        <v>0.9996685020998253</v>
+      </c>
+      <c r="AB106">
+        <v>0.8720605815568616</v>
+      </c>
+      <c r="AC106">
+        <v>0.8976106300668285</v>
+      </c>
+      <c r="AD106">
+        <v>0.9994277022655204</v>
+      </c>
+      <c r="AE106">
+        <v>0.8488011174494496</v>
+      </c>
+      <c r="AF106">
+        <v>0.8832732181924509</v>
+      </c>
+      <c r="AG106">
+        <v>0.003275880730895938</v>
+      </c>
+      <c r="AH106">
+        <v>0.005099596721639506</v>
+      </c>
+      <c r="AI106">
+        <v>0.9996685020998253</v>
+      </c>
+      <c r="AJ106">
+        <v>0.9994277022655204</v>
+      </c>
+      <c r="AK106">
+        <v>0.003275880730895938</v>
+      </c>
+      <c r="AL106">
+        <v>0.005099596721639506</v>
+      </c>
+      <c r="AM106" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN106">
+        <v>0.006466382887901134</v>
+      </c>
+      <c r="AO106">
+        <v>0.01930226798361626</v>
+      </c>
+      <c r="AP106">
+        <v>-781.2431152</v>
+      </c>
+      <c r="AQ106">
+        <v>-898.7571398</v>
+      </c>
+      <c r="AR106">
+        <v>29361.20088480043</v>
+      </c>
+      <c r="AS106">
+        <v>18297.77486019978</v>
+      </c>
+      <c r="AT106">
+        <v>29361.20088480043</v>
+      </c>
+      <c r="AU106">
+        <v>18295.66786019978</v>
+      </c>
+      <c r="AV106">
+        <v>1.936120088480043</v>
+      </c>
+      <c r="AW106">
+        <v>0.8297774860199778</v>
+      </c>
+      <c r="AX106">
+        <v>2.351872046528535</v>
+      </c>
+      <c r="AY106">
+        <v>1.081919440847639</v>
+      </c>
+      <c r="AZ106">
+        <v>101.4333333333333</v>
+      </c>
+      <c r="BA106">
+        <v>70.83333333333333</v>
+      </c>
+      <c r="BB106">
+        <v>0.005297048272647058</v>
+      </c>
+      <c r="BC106">
+        <v>0.003966375016581499</v>
+      </c>
+      <c r="BD106">
+        <v>-107.263679083095</v>
+      </c>
+      <c r="BE106">
+        <v>-36.62215195255033</v>
+      </c>
+      <c r="BF106">
+        <v>5024</v>
+      </c>
+      <c r="BG106">
+        <v>11676</v>
+      </c>
+      <c r="BH106">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI106">
+        <v>5981</v>
+      </c>
+      <c r="BJ106">
+        <v>12266</v>
+      </c>
+      <c r="BK106">
+        <v>11005</v>
+      </c>
+      <c r="BL106">
+        <v>23942</v>
+      </c>
+      <c r="BM106">
+        <v>5006</v>
+      </c>
+      <c r="BN106">
+        <v>10898</v>
+      </c>
+      <c r="BO106">
+        <v>5021</v>
+      </c>
+      <c r="BP106">
+        <v>11575</v>
+      </c>
+      <c r="BQ106">
+        <v>975</v>
+      </c>
+      <c r="BR106">
+        <v>1368</v>
+      </c>
+      <c r="BS106">
+        <v>3</v>
+      </c>
+      <c r="BT106">
+        <v>101</v>
+      </c>
+      <c r="BU106">
+        <v>0</v>
+      </c>
+      <c r="BV106">
+        <v>0</v>
+      </c>
+      <c r="BW106">
+        <v>19361.2008848</v>
+      </c>
+      <c r="BX106">
+        <v>8297.774860199999</v>
+      </c>
+      <c r="BY106">
+        <v>0.04631702428001695</v>
+      </c>
+      <c r="BZ106">
+        <v>0.0464950220390535</v>
+      </c>
+      <c r="CA106">
+        <v>0.09520180003383732</v>
+      </c>
+      <c r="CB106">
+        <v>0.1041431500436597</v>
+      </c>
+      <c r="CC106">
+        <v>0.0157171389954733</v>
+      </c>
+      <c r="CD106">
+        <v>0.01132268831108308</v>
+      </c>
+      <c r="CE106">
+        <v>0.01145306615537105</v>
+      </c>
+      <c r="CF106">
+        <v>0.009545550708330269</v>
+      </c>
+      <c r="CG106">
+        <v>20142.444</v>
+      </c>
+      <c r="CH106">
+        <v>9196.531999999999</v>
+      </c>
+      <c r="CI106">
+        <v>20249.70767908309</v>
+      </c>
+      <c r="CJ106">
+        <v>9233.154151952549</v>
+      </c>
+      <c r="CK106">
+        <v>0.04271624393225256</v>
+      </c>
+      <c r="CL106">
+        <v>0.1065739711428937</v>
+      </c>
+      <c r="CM106">
+        <v>10000</v>
+      </c>
+      <c r="CO106">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="CP106">
+        <v>0.0128858024691358</v>
+      </c>
+      <c r="CQ106">
+        <v>2980115.038919296</v>
+      </c>
+      <c r="CR106">
+        <v>8161103.390277231</v>
+      </c>
+      <c r="CS106" s="2">
+        <v>45411.05529123368</v>
+      </c>
+      <c r="CT106">
+        <v>-0.8751724322696175</v>
+      </c>
+      <c r="CU106">
+        <v>-0.9210512865130351</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GALAUSDT.json at 2024-04-29_10-10-57 bestfile_scores 0.0004951012575865222 bestfile_sharp 0.27664587689666126
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU106"/>
+  <dimension ref="A1:CU107"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -30903,6 +30903,275 @@
       </c>
       <c r="CU106">
         <v>-0.9210512865130351</v>
+      </c>
+    </row>
+    <row r="107" spans="10:99">
+      <c r="J107" t="s">
+        <v>228</v>
+      </c>
+      <c r="K107">
+        <v>0.0008493175385022589</v>
+      </c>
+      <c r="L107">
+        <v>0.0004246587692511294</v>
+      </c>
+      <c r="M107">
+        <v>0.001296802890626614</v>
+      </c>
+      <c r="N107">
+        <v>0.001296802890626614</v>
+      </c>
+      <c r="O107">
+        <v>0.0004013918019895258</v>
+      </c>
+      <c r="P107">
+        <v>0.0002006959009947629</v>
+      </c>
+      <c r="Q107">
+        <v>0.001222107544347439</v>
+      </c>
+      <c r="R107">
+        <v>0.001222107544347439</v>
+      </c>
+      <c r="S107">
+        <v>8.263525777177062</v>
+      </c>
+      <c r="T107">
+        <v>14.05800347557444</v>
+      </c>
+      <c r="U107">
+        <v>0.4274942013775844</v>
+      </c>
+      <c r="V107">
+        <v>0.4133115203878119</v>
+      </c>
+      <c r="W107">
+        <v>0.009336802124667046</v>
+      </c>
+      <c r="X107">
+        <v>0.07544480327596814</v>
+      </c>
+      <c r="Y107">
+        <v>0.1236855588620039</v>
+      </c>
+      <c r="Z107">
+        <v>0.2194298639587536</v>
+      </c>
+      <c r="AA107">
+        <v>0.9998052908445882</v>
+      </c>
+      <c r="AB107">
+        <v>0.9398006154354451</v>
+      </c>
+      <c r="AC107">
+        <v>0.826076275155307</v>
+      </c>
+      <c r="AD107">
+        <v>0.9990091236777774</v>
+      </c>
+      <c r="AE107">
+        <v>0.7106930350336186</v>
+      </c>
+      <c r="AF107">
+        <v>0.7804518785383673</v>
+      </c>
+      <c r="AG107">
+        <v>0.001558413424836683</v>
+      </c>
+      <c r="AH107">
+        <v>0.008368149950938715</v>
+      </c>
+      <c r="AI107">
+        <v>0.9998052908445882</v>
+      </c>
+      <c r="AJ107">
+        <v>0.9990091236777774</v>
+      </c>
+      <c r="AK107">
+        <v>0.001558413424836683</v>
+      </c>
+      <c r="AL107">
+        <v>0.008368149950938715</v>
+      </c>
+      <c r="AM107" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN107">
+        <v>0.004456259320547247</v>
+      </c>
+      <c r="AO107">
+        <v>0.02863925861128914</v>
+      </c>
+      <c r="AP107">
+        <v>-724.7509722780001</v>
+      </c>
+      <c r="AQ107">
+        <v>-1875.798319906</v>
+      </c>
+      <c r="AR107">
+        <v>24992.46553772193</v>
+      </c>
+      <c r="AS107">
+        <v>40482.70805009406</v>
+      </c>
+      <c r="AT107">
+        <v>24983.04713772193</v>
+      </c>
+      <c r="AU107">
+        <v>40482.56245009405</v>
+      </c>
+      <c r="AV107">
+        <v>1.499246553772193</v>
+      </c>
+      <c r="AW107">
+        <v>3.048270805009405</v>
+      </c>
+      <c r="AX107">
+        <v>2.899306412413535</v>
+      </c>
+      <c r="AY107">
+        <v>1.705239445286917</v>
+      </c>
+      <c r="AZ107">
+        <v>135.15</v>
+      </c>
+      <c r="BA107">
+        <v>101.05</v>
+      </c>
+      <c r="BB107">
+        <v>0</v>
+      </c>
+      <c r="BC107">
+        <v>0.02778519236941406</v>
+      </c>
+      <c r="BD107">
+        <v>0</v>
+      </c>
+      <c r="BE107">
+        <v>-924.7825863386652</v>
+      </c>
+      <c r="BF107">
+        <v>4052</v>
+      </c>
+      <c r="BG107">
+        <v>6663</v>
+      </c>
+      <c r="BH107">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI107">
+        <v>4864</v>
+      </c>
+      <c r="BJ107">
+        <v>8505</v>
+      </c>
+      <c r="BK107">
+        <v>8916</v>
+      </c>
+      <c r="BL107">
+        <v>15168</v>
+      </c>
+      <c r="BM107">
+        <v>3987</v>
+      </c>
+      <c r="BN107">
+        <v>6542</v>
+      </c>
+      <c r="BO107">
+        <v>4052</v>
+      </c>
+      <c r="BP107">
+        <v>6541</v>
+      </c>
+      <c r="BQ107">
+        <v>877</v>
+      </c>
+      <c r="BR107">
+        <v>1963</v>
+      </c>
+      <c r="BS107">
+        <v>0</v>
+      </c>
+      <c r="BT107">
+        <v>122</v>
+      </c>
+      <c r="BU107">
+        <v>0</v>
+      </c>
+      <c r="BV107">
+        <v>0</v>
+      </c>
+      <c r="BW107">
+        <v>14992.465537722</v>
+      </c>
+      <c r="BX107">
+        <v>30482.70805009403</v>
+      </c>
+      <c r="BY107">
+        <v>0.04724515053479349</v>
+      </c>
+      <c r="BZ107">
+        <v>0.06799921524687715</v>
+      </c>
+      <c r="CA107">
+        <v>0.1644516139751596</v>
+      </c>
+      <c r="CB107">
+        <v>0.1800013382682261</v>
+      </c>
+      <c r="CC107">
+        <v>0.01569962811001999</v>
+      </c>
+      <c r="CD107">
+        <v>0.009575228215714882</v>
+      </c>
+      <c r="CE107">
+        <v>0.01215001504511067</v>
+      </c>
+      <c r="CF107">
+        <v>0.01018602577120633</v>
+      </c>
+      <c r="CG107">
+        <v>15717.21651</v>
+      </c>
+      <c r="CH107">
+        <v>32358.50637000003</v>
+      </c>
+      <c r="CI107">
+        <v>15717.21651</v>
+      </c>
+      <c r="CJ107">
+        <v>33283.28895633869</v>
+      </c>
+      <c r="CK107">
+        <v>0.04831246198029737</v>
+      </c>
+      <c r="CL107">
+        <v>0.1316618896414333</v>
+      </c>
+      <c r="CM107">
+        <v>10000</v>
+      </c>
+      <c r="CO107">
+        <v>0</v>
+      </c>
+      <c r="CP107">
+        <v>0.02081402533209762</v>
+      </c>
+      <c r="CQ107">
+        <v>3119970.627969288</v>
+      </c>
+      <c r="CR107">
+        <v>8562542.046147738</v>
+      </c>
+      <c r="CS107" s="2">
+        <v>45411.20650358612</v>
+      </c>
+      <c r="CT107">
+        <v>-0.9169005340500025</v>
+      </c>
+      <c r="CU107">
+        <v>-0.733125809699902</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update DYDXUSDT.json at 2024-04-29_12-40-31 bestfile_scores 0.000987887281094449 bestfile_sharp 0.17343950633665128
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU107"/>
+  <dimension ref="A1:CU108"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -31172,6 +31172,275 @@
       </c>
       <c r="CU107">
         <v>-0.733125809699902</v>
+      </c>
+    </row>
+    <row r="108" spans="10:99">
+      <c r="J108" t="s">
+        <v>229</v>
+      </c>
+      <c r="K108">
+        <v>0.002358555198053169</v>
+      </c>
+      <c r="L108">
+        <v>0.001179277599026585</v>
+      </c>
+      <c r="M108">
+        <v>6.870773686551424E-05</v>
+      </c>
+      <c r="N108">
+        <v>6.870773686551424E-05</v>
+      </c>
+      <c r="O108">
+        <v>0.003453807423228028</v>
+      </c>
+      <c r="P108">
+        <v>0.001726903711614014</v>
+      </c>
+      <c r="Q108">
+        <v>-0.0009944840171600244</v>
+      </c>
+      <c r="R108">
+        <v>-0.0009944840171600244</v>
+      </c>
+      <c r="S108">
+        <v>12.63389889802344</v>
+      </c>
+      <c r="T108">
+        <v>2.898723106524401</v>
+      </c>
+      <c r="U108">
+        <v>0.3450900085852832</v>
+      </c>
+      <c r="V108">
+        <v>0.6242653469186185</v>
+      </c>
+      <c r="W108">
+        <v>0.02717834102349045</v>
+      </c>
+      <c r="X108">
+        <v>0.2741607522699891</v>
+      </c>
+      <c r="Y108">
+        <v>0.2487023604903259</v>
+      </c>
+      <c r="Z108">
+        <v>0.3031180764167488</v>
+      </c>
+      <c r="AA108">
+        <v>0.9996594464560882</v>
+      </c>
+      <c r="AB108">
+        <v>0.8256406376211082</v>
+      </c>
+      <c r="AC108">
+        <v>0.9495483422167847</v>
+      </c>
+      <c r="AD108">
+        <v>0.9970232020683971</v>
+      </c>
+      <c r="AE108">
+        <v>0.7512807670539819</v>
+      </c>
+      <c r="AF108">
+        <v>0.8830639637121247</v>
+      </c>
+      <c r="AG108">
+        <v>0.004781350004079243</v>
+      </c>
+      <c r="AH108">
+        <v>0.006561839929481642</v>
+      </c>
+      <c r="AI108">
+        <v>0.9996594464560882</v>
+      </c>
+      <c r="AJ108">
+        <v>0.9970232020683971</v>
+      </c>
+      <c r="AK108">
+        <v>0.004781350004079243</v>
+      </c>
+      <c r="AL108">
+        <v>0.006561839929481642</v>
+      </c>
+      <c r="AM108" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN108">
+        <v>0.01159707595130376</v>
+      </c>
+      <c r="AO108">
+        <v>0.1681600411831147</v>
+      </c>
+      <c r="AP108">
+        <v>-3235.578466720001</v>
+      </c>
+      <c r="AQ108">
+        <v>-854.1129363520001</v>
+      </c>
+      <c r="AR108">
+        <v>94372.43813328003</v>
+      </c>
+      <c r="AS108">
+        <v>10676.55126364799</v>
+      </c>
+      <c r="AT108">
+        <v>94372.43813328003</v>
+      </c>
+      <c r="AU108">
+        <v>10657.00984364799</v>
+      </c>
+      <c r="AV108">
+        <v>8.437243813328003</v>
+      </c>
+      <c r="AW108">
+        <v>0.06765512636479887</v>
+      </c>
+      <c r="AX108">
+        <v>1.897823377918086</v>
+      </c>
+      <c r="AY108">
+        <v>8.273518049016056</v>
+      </c>
+      <c r="AZ108">
+        <v>81.40000000000001</v>
+      </c>
+      <c r="BA108">
+        <v>276.4166666666667</v>
+      </c>
+      <c r="BB108">
+        <v>0.0001321236847862487</v>
+      </c>
+      <c r="BC108">
+        <v>0.9647578908168699</v>
+      </c>
+      <c r="BD108">
+        <v>-11.57662351616318</v>
+      </c>
+      <c r="BE108">
+        <v>-41902.15623779324</v>
+      </c>
+      <c r="BF108">
+        <v>4818</v>
+      </c>
+      <c r="BG108">
+        <v>1710</v>
+      </c>
+      <c r="BH108">
+        <v>952.8333333333334</v>
+      </c>
+      <c r="BI108">
+        <v>7220</v>
+      </c>
+      <c r="BJ108">
+        <v>1052</v>
+      </c>
+      <c r="BK108">
+        <v>12038</v>
+      </c>
+      <c r="BL108">
+        <v>2762</v>
+      </c>
+      <c r="BM108">
+        <v>4406</v>
+      </c>
+      <c r="BN108">
+        <v>666</v>
+      </c>
+      <c r="BO108">
+        <v>4815</v>
+      </c>
+      <c r="BP108">
+        <v>1530</v>
+      </c>
+      <c r="BQ108">
+        <v>2814</v>
+      </c>
+      <c r="BR108">
+        <v>386</v>
+      </c>
+      <c r="BS108">
+        <v>3</v>
+      </c>
+      <c r="BT108">
+        <v>180</v>
+      </c>
+      <c r="BU108">
+        <v>0</v>
+      </c>
+      <c r="BV108">
+        <v>0</v>
+      </c>
+      <c r="BW108">
+        <v>84372.43813328</v>
+      </c>
+      <c r="BX108">
+        <v>676.5512636479918</v>
+      </c>
+      <c r="BY108">
+        <v>0.02979170655854042</v>
+      </c>
+      <c r="BZ108">
+        <v>0.09500109658037856</v>
+      </c>
+      <c r="CA108">
+        <v>0.1419803888470431</v>
+      </c>
+      <c r="CB108">
+        <v>0.1211812598831656</v>
+      </c>
+      <c r="CC108">
+        <v>0.007550050625862209</v>
+      </c>
+      <c r="CD108">
+        <v>0.02457744833974514</v>
+      </c>
+      <c r="CE108">
+        <v>0.006767718263651968</v>
+      </c>
+      <c r="CF108">
+        <v>0.0192732709606726</v>
+      </c>
+      <c r="CG108">
+        <v>87608.0166</v>
+      </c>
+      <c r="CH108">
+        <v>1530.664199999992</v>
+      </c>
+      <c r="CI108">
+        <v>87619.59322351616</v>
+      </c>
+      <c r="CJ108">
+        <v>43432.82043779323</v>
+      </c>
+      <c r="CK108">
+        <v>0.2766458768966613</v>
+      </c>
+      <c r="CL108">
+        <v>0.01411478486153202</v>
+      </c>
+      <c r="CM108">
+        <v>10000</v>
+      </c>
+      <c r="CO108">
+        <v>0.003629367265730902</v>
+      </c>
+      <c r="CP108">
+        <v>0.0003935458480913026</v>
+      </c>
+      <c r="CQ108">
+        <v>24257875.97869808</v>
+      </c>
+      <c r="CR108">
+        <v>5094802.189709073</v>
+      </c>
+      <c r="CS108" s="2">
+        <v>45411.42429172888</v>
+      </c>
+      <c r="CT108">
+        <v>-0.807087633056609</v>
+      </c>
+      <c r="CU108">
+        <v>-0.4803236705766102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 1INCHUSDT.json at 2024-04-29_19-53-24 bestfile_scores 0.0007731213383090268 bestfile_sharp 0.0566298889510846
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU108"/>
+  <dimension ref="A1:CU109"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -31441,6 +31441,275 @@
       </c>
       <c r="CU108">
         <v>-0.4803236705766102</v>
+      </c>
+    </row>
+    <row r="109" spans="10:99">
+      <c r="J109" t="s">
+        <v>230</v>
+      </c>
+      <c r="K109">
+        <v>0.002110636643427588</v>
+      </c>
+      <c r="L109">
+        <v>0.001055318321713794</v>
+      </c>
+      <c r="M109">
+        <v>0.0009939963433207577</v>
+      </c>
+      <c r="N109">
+        <v>0.0009939963433207577</v>
+      </c>
+      <c r="O109">
+        <v>0.002345747620953298</v>
+      </c>
+      <c r="P109">
+        <v>0.001172873810476649</v>
+      </c>
+      <c r="Q109">
+        <v>0.0007293606488665949</v>
+      </c>
+      <c r="R109">
+        <v>0.0007293606488665949</v>
+      </c>
+      <c r="S109">
+        <v>28.06931207762953</v>
+      </c>
+      <c r="T109">
+        <v>9.475654132732629</v>
+      </c>
+      <c r="U109">
+        <v>0.3661710030358916</v>
+      </c>
+      <c r="V109">
+        <v>0.7035911728171333</v>
+      </c>
+      <c r="W109">
+        <v>0.09005332217043512</v>
+      </c>
+      <c r="X109">
+        <v>0.02723420946687281</v>
+      </c>
+      <c r="Y109">
+        <v>0.1960762890306705</v>
+      </c>
+      <c r="Z109">
+        <v>0.1400125520981206</v>
+      </c>
+      <c r="AA109">
+        <v>0.9973805332386905</v>
+      </c>
+      <c r="AB109">
+        <v>0.8316215015142282</v>
+      </c>
+      <c r="AC109">
+        <v>0.883783675325408</v>
+      </c>
+      <c r="AD109">
+        <v>0.9996884155056633</v>
+      </c>
+      <c r="AE109">
+        <v>0.810568401229796</v>
+      </c>
+      <c r="AF109">
+        <v>0.8601673895143028</v>
+      </c>
+      <c r="AG109">
+        <v>0.009712845170598517</v>
+      </c>
+      <c r="AH109">
+        <v>0.003928384818884289</v>
+      </c>
+      <c r="AI109">
+        <v>0.9973805332386905</v>
+      </c>
+      <c r="AJ109">
+        <v>0.9996884155056633</v>
+      </c>
+      <c r="AK109">
+        <v>0.009712845170598517</v>
+      </c>
+      <c r="AL109">
+        <v>0.003928384818884289</v>
+      </c>
+      <c r="AM109" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN109">
+        <v>0.05061223839241435</v>
+      </c>
+      <c r="AO109">
+        <v>0.01369574182018806</v>
+      </c>
+      <c r="AP109">
+        <v>-7615.73086304</v>
+      </c>
+      <c r="AQ109">
+        <v>-696.5465467</v>
+      </c>
+      <c r="AR109">
+        <v>75984.27413696013</v>
+      </c>
+      <c r="AS109">
+        <v>26001.8857533</v>
+      </c>
+      <c r="AT109">
+        <v>75905.46413696013</v>
+      </c>
+      <c r="AU109">
+        <v>26001.8857533</v>
+      </c>
+      <c r="AV109">
+        <v>6.598427413696013</v>
+      </c>
+      <c r="AW109">
+        <v>1.60018857533</v>
+      </c>
+      <c r="AX109">
+        <v>0.853141089750713</v>
+      </c>
+      <c r="AY109">
+        <v>2.530723508540913</v>
+      </c>
+      <c r="AZ109">
+        <v>117.6</v>
+      </c>
+      <c r="BA109">
+        <v>88.8</v>
+      </c>
+      <c r="BB109">
+        <v>0.03112459094845468</v>
+      </c>
+      <c r="BC109">
+        <v>0.02293919028502044</v>
+      </c>
+      <c r="BD109">
+        <v>-2364.359780450724</v>
+      </c>
+      <c r="BE109">
+        <v>-392.0416336245963</v>
+      </c>
+      <c r="BF109">
+        <v>12661</v>
+      </c>
+      <c r="BG109">
+        <v>3804</v>
+      </c>
+      <c r="BH109">
+        <v>961.8333333333334</v>
+      </c>
+      <c r="BI109">
+        <v>14337</v>
+      </c>
+      <c r="BJ109">
+        <v>5310</v>
+      </c>
+      <c r="BK109">
+        <v>26998</v>
+      </c>
+      <c r="BL109">
+        <v>9114</v>
+      </c>
+      <c r="BM109">
+        <v>12642</v>
+      </c>
+      <c r="BN109">
+        <v>3777</v>
+      </c>
+      <c r="BO109">
+        <v>12643</v>
+      </c>
+      <c r="BP109">
+        <v>3789</v>
+      </c>
+      <c r="BQ109">
+        <v>1695</v>
+      </c>
+      <c r="BR109">
+        <v>1533</v>
+      </c>
+      <c r="BS109">
+        <v>18</v>
+      </c>
+      <c r="BT109">
+        <v>15</v>
+      </c>
+      <c r="BU109">
+        <v>0</v>
+      </c>
+      <c r="BV109">
+        <v>0</v>
+      </c>
+      <c r="BW109">
+        <v>65984.27413695995</v>
+      </c>
+      <c r="BX109">
+        <v>16001.88575329999</v>
+      </c>
+      <c r="BY109">
+        <v>0.06357771855036264</v>
+      </c>
+      <c r="BZ109">
+        <v>0.03846779790619466</v>
+      </c>
+      <c r="CA109">
+        <v>0.1233370044997575</v>
+      </c>
+      <c r="CB109">
+        <v>0.1226592141701881</v>
+      </c>
+      <c r="CC109">
+        <v>0.01856592059729292</v>
+      </c>
+      <c r="CD109">
+        <v>0.009315443790002584</v>
+      </c>
+      <c r="CE109">
+        <v>0.01259773349858223</v>
+      </c>
+      <c r="CF109">
+        <v>0.008553173744726143</v>
+      </c>
+      <c r="CG109">
+        <v>73600.00499999995</v>
+      </c>
+      <c r="CH109">
+        <v>16698.43229999999</v>
+      </c>
+      <c r="CI109">
+        <v>75964.36478045068</v>
+      </c>
+      <c r="CJ109">
+        <v>17090.47393362459</v>
+      </c>
+      <c r="CK109">
+        <v>0.1734395063366513</v>
+      </c>
+      <c r="CL109">
+        <v>0.1385806051725335</v>
+      </c>
+      <c r="CM109">
+        <v>10000</v>
+      </c>
+      <c r="CO109">
+        <v>0.00697422568767598</v>
+      </c>
+      <c r="CP109">
+        <v>0.006324453108078839</v>
+      </c>
+      <c r="CQ109">
+        <v>23973844.34944462</v>
+      </c>
+      <c r="CR109">
+        <v>2688942.923710383</v>
+      </c>
+      <c r="CS109" s="2">
+        <v>45411.52816553663</v>
+      </c>
+      <c r="CT109">
+        <v>-0.6156032480827009</v>
+      </c>
+      <c r="CU109">
+        <v>-0.8372228480576703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ENJUSDT.json at 2024-04-30_01-12-36 bestfile_scores 0.0005411798402292251 bestfile_sharp 0.132917788464223
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU109"/>
+  <dimension ref="A1:CU110"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -31710,6 +31710,275 @@
       </c>
       <c r="CU109">
         <v>-0.8372228480576703</v>
+      </c>
+    </row>
+    <row r="110" spans="10:99">
+      <c r="J110" t="s">
+        <v>231</v>
+      </c>
+      <c r="K110">
+        <v>0.001846607075694839</v>
+      </c>
+      <c r="L110">
+        <v>0.0009233035378474197</v>
+      </c>
+      <c r="M110">
+        <v>0.0007599892218528304</v>
+      </c>
+      <c r="N110">
+        <v>0.0007599892218528304</v>
+      </c>
+      <c r="O110">
+        <v>0.001381508919844099</v>
+      </c>
+      <c r="P110">
+        <v>0.0006907544599220495</v>
+      </c>
+      <c r="Q110">
+        <v>0.0007184381336138079</v>
+      </c>
+      <c r="R110">
+        <v>0.0007184381336138079</v>
+      </c>
+      <c r="S110">
+        <v>25.85377522280952</v>
+      </c>
+      <c r="T110">
+        <v>18.62108877657317</v>
+      </c>
+      <c r="U110">
+        <v>0.3978432476901825</v>
+      </c>
+      <c r="V110">
+        <v>0.430086549433453</v>
+      </c>
+      <c r="W110">
+        <v>0.09441061233248833</v>
+      </c>
+      <c r="X110">
+        <v>0.0896320968687775</v>
+      </c>
+      <c r="Y110">
+        <v>0.1647321872354172</v>
+      </c>
+      <c r="Z110">
+        <v>0.2468761141882611</v>
+      </c>
+      <c r="AA110">
+        <v>0.9990902063228789</v>
+      </c>
+      <c r="AB110">
+        <v>0.8717757768098162</v>
+      </c>
+      <c r="AC110">
+        <v>0.8035371632508073</v>
+      </c>
+      <c r="AD110">
+        <v>0.9970920803673445</v>
+      </c>
+      <c r="AE110">
+        <v>0.7779331690573085</v>
+      </c>
+      <c r="AF110">
+        <v>0.675857247404426</v>
+      </c>
+      <c r="AG110">
+        <v>0.007364103476617579</v>
+      </c>
+      <c r="AH110">
+        <v>0.01105750185738948</v>
+      </c>
+      <c r="AI110">
+        <v>0.9990902063228789</v>
+      </c>
+      <c r="AJ110">
+        <v>0.9970920803673445</v>
+      </c>
+      <c r="AK110">
+        <v>0.007364103476617579</v>
+      </c>
+      <c r="AL110">
+        <v>0.01105750185738948</v>
+      </c>
+      <c r="AM110" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN110">
+        <v>0.01824080739261039</v>
+      </c>
+      <c r="AO110">
+        <v>0.06122122643536942</v>
+      </c>
+      <c r="AP110">
+        <v>-5206.326603060001</v>
+      </c>
+      <c r="AQ110">
+        <v>-545.90296238</v>
+      </c>
+      <c r="AR110">
+        <v>73332.56279693999</v>
+      </c>
+      <c r="AS110">
+        <v>22715.10362548051</v>
+      </c>
+      <c r="AT110">
+        <v>73305.78509693999</v>
+      </c>
+      <c r="AU110">
+        <v>22715.15662548051</v>
+      </c>
+      <c r="AV110">
+        <v>6.333256279693999</v>
+      </c>
+      <c r="AW110">
+        <v>1.271510362548051</v>
+      </c>
+      <c r="AX110">
+        <v>0.9276862464183382</v>
+      </c>
+      <c r="AY110">
+        <v>1.286886468745338</v>
+      </c>
+      <c r="AZ110">
+        <v>69.16666666666667</v>
+      </c>
+      <c r="BA110">
+        <v>105.1166666666667</v>
+      </c>
+      <c r="BB110">
+        <v>0.04534554877839644</v>
+      </c>
+      <c r="BC110">
+        <v>0</v>
+      </c>
+      <c r="BD110">
+        <v>-3255.558645882625</v>
+      </c>
+      <c r="BE110">
+        <v>0</v>
+      </c>
+      <c r="BF110">
+        <v>12398</v>
+      </c>
+      <c r="BG110">
+        <v>5203</v>
+      </c>
+      <c r="BH110">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI110">
+        <v>15523</v>
+      </c>
+      <c r="BJ110">
+        <v>14907</v>
+      </c>
+      <c r="BK110">
+        <v>27921</v>
+      </c>
+      <c r="BL110">
+        <v>20110</v>
+      </c>
+      <c r="BM110">
+        <v>12366</v>
+      </c>
+      <c r="BN110">
+        <v>5203</v>
+      </c>
+      <c r="BO110">
+        <v>12383</v>
+      </c>
+      <c r="BP110">
+        <v>5203</v>
+      </c>
+      <c r="BQ110">
+        <v>3157</v>
+      </c>
+      <c r="BR110">
+        <v>9704</v>
+      </c>
+      <c r="BS110">
+        <v>15</v>
+      </c>
+      <c r="BT110">
+        <v>0</v>
+      </c>
+      <c r="BU110">
+        <v>0</v>
+      </c>
+      <c r="BV110">
+        <v>0</v>
+      </c>
+      <c r="BW110">
+        <v>63332.56279694012</v>
+      </c>
+      <c r="BX110">
+        <v>12716.14493761999</v>
+      </c>
+      <c r="BY110">
+        <v>0.05168325347808871</v>
+      </c>
+      <c r="BZ110">
+        <v>0.1202877902871604</v>
+      </c>
+      <c r="CA110">
+        <v>0.1092477396555746</v>
+      </c>
+      <c r="CB110">
+        <v>0.1978939551960537</v>
+      </c>
+      <c r="CC110">
+        <v>0.008284602778212469</v>
+      </c>
+      <c r="CD110">
+        <v>0.01552353208118639</v>
+      </c>
+      <c r="CE110">
+        <v>0.008424188358683768</v>
+      </c>
+      <c r="CF110">
+        <v>0.0190230569823722</v>
+      </c>
+      <c r="CG110">
+        <v>68538.88940000012</v>
+      </c>
+      <c r="CH110">
+        <v>13262.04789999999</v>
+      </c>
+      <c r="CI110">
+        <v>71794.44804588275</v>
+      </c>
+      <c r="CJ110">
+        <v>13262.04789999999</v>
+      </c>
+      <c r="CK110">
+        <v>0.0566298889510846</v>
+      </c>
+      <c r="CL110">
+        <v>0.08931899997439623</v>
+      </c>
+      <c r="CM110">
+        <v>10000</v>
+      </c>
+      <c r="CO110">
+        <v>0.003047839506172839</v>
+      </c>
+      <c r="CP110">
+        <v>0.002199074074074074</v>
+      </c>
+      <c r="CQ110">
+        <v>18344950.30516516</v>
+      </c>
+      <c r="CR110">
+        <v>7113237.577421894</v>
+      </c>
+      <c r="CS110" s="2">
+        <v>45411.82878898195</v>
+      </c>
+      <c r="CT110">
+        <v>-0.7629790982692873</v>
+      </c>
+      <c r="CU110">
+        <v>-0.8021612595391501</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SXPUSDT.json at 2024-04-30_05-39-16 bestfile_scores 0.0006630297133322832 bestfile_sharp 0.03550210994387869
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="992" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="994" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU110"/>
+  <dimension ref="A1:CU111"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -31979,6 +31979,275 @@
       </c>
       <c r="CU110">
         <v>-0.8021612595391501</v>
+      </c>
+    </row>
+    <row r="111" spans="10:99">
+      <c r="J111" t="s">
+        <v>232</v>
+      </c>
+      <c r="K111">
+        <v>0.0009582217292736228</v>
+      </c>
+      <c r="L111">
+        <v>0.0004791108646368114</v>
+      </c>
+      <c r="M111">
+        <v>0.0006702327939247521</v>
+      </c>
+      <c r="N111">
+        <v>0.0006702327939247521</v>
+      </c>
+      <c r="O111">
+        <v>0.001028644879699292</v>
+      </c>
+      <c r="P111">
+        <v>0.000514322439849646</v>
+      </c>
+      <c r="Q111">
+        <v>0.0005010532625056907</v>
+      </c>
+      <c r="R111">
+        <v>0.0005010532625056907</v>
+      </c>
+      <c r="S111">
+        <v>31.67159226822023</v>
+      </c>
+      <c r="T111">
+        <v>7.474362436822409</v>
+      </c>
+      <c r="U111">
+        <v>0.3690865070932836</v>
+      </c>
+      <c r="V111">
+        <v>0.7195246020799009</v>
+      </c>
+      <c r="W111">
+        <v>0.05195456388008537</v>
+      </c>
+      <c r="X111">
+        <v>0.09919794284577033</v>
+      </c>
+      <c r="Y111">
+        <v>0.1728659068393492</v>
+      </c>
+      <c r="Z111">
+        <v>0.1691839681782611</v>
+      </c>
+      <c r="AA111">
+        <v>0.999304719549694</v>
+      </c>
+      <c r="AB111">
+        <v>0.8478097928238977</v>
+      </c>
+      <c r="AC111">
+        <v>0.8646173161734547</v>
+      </c>
+      <c r="AD111">
+        <v>0.9987063145401199</v>
+      </c>
+      <c r="AE111">
+        <v>0.781205317417011</v>
+      </c>
+      <c r="AF111">
+        <v>0.8542342617159226</v>
+      </c>
+      <c r="AG111">
+        <v>0.006205423909049068</v>
+      </c>
+      <c r="AH111">
+        <v>0.007921163194322988</v>
+      </c>
+      <c r="AI111">
+        <v>0.999304719549694</v>
+      </c>
+      <c r="AJ111">
+        <v>0.9987063145401199</v>
+      </c>
+      <c r="AK111">
+        <v>0.006205423909049068</v>
+      </c>
+      <c r="AL111">
+        <v>0.007921163194322988</v>
+      </c>
+      <c r="AM111" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN111">
+        <v>0.01606655986286077</v>
+      </c>
+      <c r="AO111">
+        <v>0.03713636322961943</v>
+      </c>
+      <c r="AP111">
+        <v>-2258.599607892</v>
+      </c>
+      <c r="AQ111">
+        <v>-780.9264503600001</v>
+      </c>
+      <c r="AR111">
+        <v>28132.60287210782</v>
+      </c>
+      <c r="AS111">
+        <v>20618.03394963989</v>
+      </c>
+      <c r="AT111">
+        <v>28087.78177210782</v>
+      </c>
+      <c r="AU111">
+        <v>20618.03394963989</v>
+      </c>
+      <c r="AV111">
+        <v>1.813260287210782</v>
+      </c>
+      <c r="AW111">
+        <v>1.061803394963989</v>
+      </c>
+      <c r="AX111">
+        <v>0.7572610589714353</v>
+      </c>
+      <c r="AY111">
+        <v>3.204834179985958</v>
+      </c>
+      <c r="AZ111">
+        <v>113.0833333333333</v>
+      </c>
+      <c r="BA111">
+        <v>117.7333333333333</v>
+      </c>
+      <c r="BB111">
+        <v>0.02956285531938887</v>
+      </c>
+      <c r="BC111">
+        <v>0.08045726669695755</v>
+      </c>
+      <c r="BD111">
+        <v>-621.1862066584471</v>
+      </c>
+      <c r="BE111">
+        <v>-997.3752863844445</v>
+      </c>
+      <c r="BF111">
+        <v>15618</v>
+      </c>
+      <c r="BG111">
+        <v>3553</v>
+      </c>
+      <c r="BH111">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI111">
+        <v>18586</v>
+      </c>
+      <c r="BJ111">
+        <v>4519</v>
+      </c>
+      <c r="BK111">
+        <v>34204</v>
+      </c>
+      <c r="BL111">
+        <v>8072</v>
+      </c>
+      <c r="BM111">
+        <v>15469</v>
+      </c>
+      <c r="BN111">
+        <v>3025</v>
+      </c>
+      <c r="BO111">
+        <v>15601</v>
+      </c>
+      <c r="BP111">
+        <v>3532</v>
+      </c>
+      <c r="BQ111">
+        <v>3117</v>
+      </c>
+      <c r="BR111">
+        <v>1494</v>
+      </c>
+      <c r="BS111">
+        <v>17</v>
+      </c>
+      <c r="BT111">
+        <v>21</v>
+      </c>
+      <c r="BU111">
+        <v>0</v>
+      </c>
+      <c r="BV111">
+        <v>0</v>
+      </c>
+      <c r="BW111">
+        <v>18132.602872108</v>
+      </c>
+      <c r="BX111">
+        <v>10618.03394963999</v>
+      </c>
+      <c r="BY111">
+        <v>0.04007506262414946</v>
+      </c>
+      <c r="BZ111">
+        <v>0.07081252701906551</v>
+      </c>
+      <c r="CA111">
+        <v>0.0943761244394027</v>
+      </c>
+      <c r="CB111">
+        <v>0.127220868059645</v>
+      </c>
+      <c r="CC111">
+        <v>0.01130282847294496</v>
+      </c>
+      <c r="CD111">
+        <v>0.01815636747480773</v>
+      </c>
+      <c r="CE111">
+        <v>0.008348271237715114</v>
+      </c>
+      <c r="CF111">
+        <v>0.01441204207218206</v>
+      </c>
+      <c r="CG111">
+        <v>20391.20248</v>
+      </c>
+      <c r="CH111">
+        <v>11398.96039999999</v>
+      </c>
+      <c r="CI111">
+        <v>21012.38868665845</v>
+      </c>
+      <c r="CJ111">
+        <v>12396.33568638443</v>
+      </c>
+      <c r="CK111">
+        <v>0.132917788464223</v>
+      </c>
+      <c r="CL111">
+        <v>0.1327060571103286</v>
+      </c>
+      <c r="CM111">
+        <v>10000</v>
+      </c>
+      <c r="CO111">
+        <v>0.004513888888888888</v>
+      </c>
+      <c r="CP111">
+        <v>0.00933641975308642</v>
+      </c>
+      <c r="CQ111">
+        <v>10638257.28362185</v>
+      </c>
+      <c r="CR111">
+        <v>7296357.590261763</v>
+      </c>
+      <c r="CS111" s="2">
+        <v>45412.0504430569</v>
+      </c>
+      <c r="CT111">
+        <v>-0.8942723506201351</v>
+      </c>
+      <c r="CU111">
+        <v>-0.8923344605000599</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ROSEUSDT.json at 2024-04-30_09-00-31 bestfile_scores 0.0009232218530796171 bestfile_sharp 0.09616839260939938
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="994" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU111"/>
+  <dimension ref="A1:CU112"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -32248,6 +32248,275 @@
       </c>
       <c r="CU111">
         <v>-0.8923344605000599</v>
+      </c>
+    </row>
+    <row r="112" spans="10:99">
+      <c r="J112" t="s">
+        <v>233</v>
+      </c>
+      <c r="K112">
+        <v>0.003320376059487318</v>
+      </c>
+      <c r="L112">
+        <v>0.001660188029743659</v>
+      </c>
+      <c r="M112">
+        <v>0.0001480573897612025</v>
+      </c>
+      <c r="N112">
+        <v>0.0001480573897612025</v>
+      </c>
+      <c r="O112">
+        <v>0.001453710486382431</v>
+      </c>
+      <c r="P112">
+        <v>0.0007268552431912156</v>
+      </c>
+      <c r="Q112">
+        <v>0.0001170181906330558</v>
+      </c>
+      <c r="R112">
+        <v>0.0001170181906330558</v>
+      </c>
+      <c r="S112">
+        <v>14.26653794168759</v>
+      </c>
+      <c r="T112">
+        <v>9.539756709789536</v>
+      </c>
+      <c r="U112">
+        <v>0.3188284588613518</v>
+      </c>
+      <c r="V112">
+        <v>0.5915705401019734</v>
+      </c>
+      <c r="W112">
+        <v>0.07354837407521488</v>
+      </c>
+      <c r="X112">
+        <v>0.03621449565347842</v>
+      </c>
+      <c r="Y112">
+        <v>0.2423490982678377</v>
+      </c>
+      <c r="Z112">
+        <v>0.2014046000575335</v>
+      </c>
+      <c r="AA112">
+        <v>0.9980556331534561</v>
+      </c>
+      <c r="AB112">
+        <v>0.7947859260636987</v>
+      </c>
+      <c r="AC112">
+        <v>0.8557156628753676</v>
+      </c>
+      <c r="AD112">
+        <v>0.9992390720386227</v>
+      </c>
+      <c r="AE112">
+        <v>0.726895897733762</v>
+      </c>
+      <c r="AF112">
+        <v>0.7987354500694386</v>
+      </c>
+      <c r="AG112">
+        <v>0.009007048414043884</v>
+      </c>
+      <c r="AH112">
+        <v>0.004568222877433296</v>
+      </c>
+      <c r="AI112">
+        <v>0.9980556331534561</v>
+      </c>
+      <c r="AJ112">
+        <v>0.9992390720386227</v>
+      </c>
+      <c r="AK112">
+        <v>0.009007048414043884</v>
+      </c>
+      <c r="AL112">
+        <v>0.004568222877433296</v>
+      </c>
+      <c r="AM112" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN112">
+        <v>0.03788640692690706</v>
+      </c>
+      <c r="AO112">
+        <v>0.01608034889519972</v>
+      </c>
+      <c r="AP112">
+        <v>-25613.42765624</v>
+      </c>
+      <c r="AQ112">
+        <v>-160.86939412</v>
+      </c>
+      <c r="AR112">
+        <v>357522.3733154715</v>
+      </c>
+      <c r="AS112">
+        <v>11732.01022588004</v>
+      </c>
+      <c r="AT112">
+        <v>357264.4956154714</v>
+      </c>
+      <c r="AU112">
+        <v>11732.01022588004</v>
+      </c>
+      <c r="AV112">
+        <v>34.75223733154714</v>
+      </c>
+      <c r="AW112">
+        <v>0.1732010225880043</v>
+      </c>
+      <c r="AX112">
+        <v>1.681055093555093</v>
+      </c>
+      <c r="AY112">
+        <v>2.514976033164918</v>
+      </c>
+      <c r="AZ112">
+        <v>114.15</v>
+      </c>
+      <c r="BA112">
+        <v>107.45</v>
+      </c>
+      <c r="BB112">
+        <v>0.001596348996378763</v>
+      </c>
+      <c r="BC112">
+        <v>0.01071666776174045</v>
+      </c>
+      <c r="BD112">
+        <v>-596.6038049829068</v>
+      </c>
+      <c r="BE112">
+        <v>-20.50510843502616</v>
+      </c>
+      <c r="BF112">
+        <v>6874</v>
+      </c>
+      <c r="BG112">
+        <v>4609</v>
+      </c>
+      <c r="BH112">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI112">
+        <v>8519</v>
+      </c>
+      <c r="BJ112">
+        <v>5684</v>
+      </c>
+      <c r="BK112">
+        <v>15393</v>
+      </c>
+      <c r="BL112">
+        <v>10293</v>
+      </c>
+      <c r="BM112">
+        <v>6403</v>
+      </c>
+      <c r="BN112">
+        <v>4599</v>
+      </c>
+      <c r="BO112">
+        <v>6872</v>
+      </c>
+      <c r="BP112">
+        <v>4607</v>
+      </c>
+      <c r="BQ112">
+        <v>2116</v>
+      </c>
+      <c r="BR112">
+        <v>1085</v>
+      </c>
+      <c r="BS112">
+        <v>2</v>
+      </c>
+      <c r="BT112">
+        <v>2</v>
+      </c>
+      <c r="BU112">
+        <v>0</v>
+      </c>
+      <c r="BV112">
+        <v>0</v>
+      </c>
+      <c r="BW112">
+        <v>347520.1530637604</v>
+      </c>
+      <c r="BX112">
+        <v>1732.010225880002</v>
+      </c>
+      <c r="BY112">
+        <v>0.06953197861765564</v>
+      </c>
+      <c r="BZ112">
+        <v>0.1026866653693641</v>
+      </c>
+      <c r="CA112">
+        <v>0.1998330895050714</v>
+      </c>
+      <c r="CB112">
+        <v>0.2068365363378705</v>
+      </c>
+      <c r="CC112">
+        <v>0.01258492189810615</v>
+      </c>
+      <c r="CD112">
+        <v>0.01928834649781472</v>
+      </c>
+      <c r="CE112">
+        <v>0.01244393713106901</v>
+      </c>
+      <c r="CF112">
+        <v>0.01669259792065725</v>
+      </c>
+      <c r="CG112">
+        <v>373133.5807200004</v>
+      </c>
+      <c r="CH112">
+        <v>1892.879620000002</v>
+      </c>
+      <c r="CI112">
+        <v>373730.1845249833</v>
+      </c>
+      <c r="CJ112">
+        <v>1913.384728435028</v>
+      </c>
+      <c r="CK112">
+        <v>0.03550210994387869</v>
+      </c>
+      <c r="CL112">
+        <v>0.03133142036678326</v>
+      </c>
+      <c r="CM112">
+        <v>10000</v>
+      </c>
+      <c r="CO112">
+        <v>0.001119864071671301</v>
+      </c>
+      <c r="CP112">
+        <v>0.0008495520543713315</v>
+      </c>
+      <c r="CQ112">
+        <v>132703067.4248272</v>
+      </c>
+      <c r="CR112">
+        <v>646350.5069878154</v>
+      </c>
+      <c r="CS112" s="2">
+        <v>45412.23562108146</v>
+      </c>
+      <c r="CT112">
+        <v>-0.09166218257655467</v>
+      </c>
+      <c r="CU112">
+        <v>-0.9193280040552687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ARUSDT.json at 2024-04-30_12-47-56 bestfile_scores 0.0006554293782343679 bestfile_sharp 0.17072112134046277
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU112"/>
+  <dimension ref="A1:CU113"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -32517,6 +32517,275 @@
       </c>
       <c r="CU112">
         <v>-0.9193280040552687</v>
+      </c>
+    </row>
+    <row r="113" spans="10:99">
+      <c r="J113" t="s">
+        <v>234</v>
+      </c>
+      <c r="K113">
+        <v>0.0009101809236724545</v>
+      </c>
+      <c r="L113">
+        <v>0.0004550904618362273</v>
+      </c>
+      <c r="M113">
+        <v>0.001277328705284075</v>
+      </c>
+      <c r="N113">
+        <v>0.001277328705284075</v>
+      </c>
+      <c r="O113">
+        <v>0.001475798817459917</v>
+      </c>
+      <c r="P113">
+        <v>0.0007378994087299584</v>
+      </c>
+      <c r="Q113">
+        <v>0.001222568836468207</v>
+      </c>
+      <c r="R113">
+        <v>0.001222568836468207</v>
+      </c>
+      <c r="S113">
+        <v>15.49597960384389</v>
+      </c>
+      <c r="T113">
+        <v>12.32712296528731</v>
+      </c>
+      <c r="U113">
+        <v>0.4079344617764494</v>
+      </c>
+      <c r="V113">
+        <v>0.6447407973854092</v>
+      </c>
+      <c r="W113">
+        <v>0.02821099005744313</v>
+      </c>
+      <c r="X113">
+        <v>0.0991724782794786</v>
+      </c>
+      <c r="Y113">
+        <v>0.2413388627114259</v>
+      </c>
+      <c r="Z113">
+        <v>0.2043229390166602</v>
+      </c>
+      <c r="AA113">
+        <v>0.9994808983467547</v>
+      </c>
+      <c r="AB113">
+        <v>0.7999707790799354</v>
+      </c>
+      <c r="AC113">
+        <v>0.8349064777109861</v>
+      </c>
+      <c r="AD113">
+        <v>0.9984843604211638</v>
+      </c>
+      <c r="AE113">
+        <v>0.7589542621870838</v>
+      </c>
+      <c r="AF113">
+        <v>0.7964123613015145</v>
+      </c>
+      <c r="AG113">
+        <v>0.0061072219578577</v>
+      </c>
+      <c r="AH113">
+        <v>0.01035402435129395</v>
+      </c>
+      <c r="AI113">
+        <v>0.9994808983467547</v>
+      </c>
+      <c r="AJ113">
+        <v>0.9984843604211638</v>
+      </c>
+      <c r="AK113">
+        <v>0.0061072219578577</v>
+      </c>
+      <c r="AL113">
+        <v>0.01035402435129395</v>
+      </c>
+      <c r="AM113" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN113">
+        <v>0.01234200770842877</v>
+      </c>
+      <c r="AO113">
+        <v>0.04372538639913001</v>
+      </c>
+      <c r="AP113">
+        <v>-717.552314256</v>
+      </c>
+      <c r="AQ113">
+        <v>-1650.30649039</v>
+      </c>
+      <c r="AR113">
+        <v>21665.80868574392</v>
+      </c>
+      <c r="AS113">
+        <v>29589.18471960996</v>
+      </c>
+      <c r="AT113">
+        <v>21650.60002574392</v>
+      </c>
+      <c r="AU113">
+        <v>29589.18471960996</v>
+      </c>
+      <c r="AV113">
+        <v>1.166580868574392</v>
+      </c>
+      <c r="AW113">
+        <v>1.958918471960996</v>
+      </c>
+      <c r="AX113">
+        <v>1.545928260429324</v>
+      </c>
+      <c r="AY113">
+        <v>1.943392203659507</v>
+      </c>
+      <c r="AZ113">
+        <v>119.3833333333333</v>
+      </c>
+      <c r="BA113">
+        <v>100.6333333333333</v>
+      </c>
+      <c r="BB113">
+        <v>0.004260379490934279</v>
+      </c>
+      <c r="BC113">
+        <v>0.03431160673559609</v>
+      </c>
+      <c r="BD113">
+        <v>-52.98354725130179</v>
+      </c>
+      <c r="BE113">
+        <v>-754.6544773083301</v>
+      </c>
+      <c r="BF113">
+        <v>5490</v>
+      </c>
+      <c r="BG113">
+        <v>5599</v>
+      </c>
+      <c r="BH113">
+        <v>849.8333333333334</v>
+      </c>
+      <c r="BI113">
+        <v>7679</v>
+      </c>
+      <c r="BJ113">
+        <v>4877</v>
+      </c>
+      <c r="BK113">
+        <v>13169</v>
+      </c>
+      <c r="BL113">
+        <v>10476</v>
+      </c>
+      <c r="BM113">
+        <v>5484</v>
+      </c>
+      <c r="BN113">
+        <v>4001</v>
+      </c>
+      <c r="BO113">
+        <v>5489</v>
+      </c>
+      <c r="BP113">
+        <v>5521</v>
+      </c>
+      <c r="BQ113">
+        <v>2195</v>
+      </c>
+      <c r="BR113">
+        <v>876</v>
+      </c>
+      <c r="BS113">
+        <v>1</v>
+      </c>
+      <c r="BT113">
+        <v>78</v>
+      </c>
+      <c r="BU113">
+        <v>0</v>
+      </c>
+      <c r="BV113">
+        <v>0</v>
+      </c>
+      <c r="BW113">
+        <v>11665.808685744</v>
+      </c>
+      <c r="BX113">
+        <v>19589.18471961</v>
+      </c>
+      <c r="BY113">
+        <v>0.04315197247791526</v>
+      </c>
+      <c r="BZ113">
+        <v>0.08480155539681701</v>
+      </c>
+      <c r="CA113">
+        <v>0.1370203478366124</v>
+      </c>
+      <c r="CB113">
+        <v>0.1681986830656868</v>
+      </c>
+      <c r="CC113">
+        <v>0.012820006006728</v>
+      </c>
+      <c r="CD113">
+        <v>0.01170281694767721</v>
+      </c>
+      <c r="CE113">
+        <v>0.009452487276740324</v>
+      </c>
+      <c r="CF113">
+        <v>0.01483794154268238</v>
+      </c>
+      <c r="CG113">
+        <v>12383.361</v>
+      </c>
+      <c r="CH113">
+        <v>21239.49121</v>
+      </c>
+      <c r="CI113">
+        <v>12436.3445472513</v>
+      </c>
+      <c r="CJ113">
+        <v>21994.14568730833</v>
+      </c>
+      <c r="CK113">
+        <v>0.09616839260939938</v>
+      </c>
+      <c r="CL113">
+        <v>0.1273965447156222</v>
+      </c>
+      <c r="CM113">
+        <v>10000</v>
+      </c>
+      <c r="CO113">
+        <v>0.001470804530077953</v>
+      </c>
+      <c r="CP113">
+        <v>0.02711183017110359</v>
+      </c>
+      <c r="CQ113">
+        <v>3799926.369570356</v>
+      </c>
+      <c r="CR113">
+        <v>16980708.42353759</v>
+      </c>
+      <c r="CS113" s="2">
+        <v>45412.37538809028</v>
+      </c>
+      <c r="CT113">
+        <v>-0.8006705745635164</v>
+      </c>
+      <c r="CU113">
+        <v>-0.7122306825923299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ATOMUSDT.json at 2024-05-01_02-57-41 bestfile_scores 0.0009212141254985901 bestfile_sharp 0.16944021001401996
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="998" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU113"/>
+  <dimension ref="A1:CU115"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -32786,6 +32786,544 @@
       </c>
       <c r="CU113">
         <v>-0.7122306825923299</v>
+      </c>
+    </row>
+    <row r="114" spans="10:99">
+      <c r="J114" t="s">
+        <v>235</v>
+      </c>
+      <c r="K114">
+        <v>0.001332892770804062</v>
+      </c>
+      <c r="L114">
+        <v>0.0006664463854020308</v>
+      </c>
+      <c r="M114">
+        <v>0.000347571566597038</v>
+      </c>
+      <c r="N114">
+        <v>0.000347571566597038</v>
+      </c>
+      <c r="O114">
+        <v>0.002109399332369444</v>
+      </c>
+      <c r="P114">
+        <v>0.001054699666184722</v>
+      </c>
+      <c r="Q114">
+        <v>0.0005529998947536807</v>
+      </c>
+      <c r="R114">
+        <v>0.0005529998947536807</v>
+      </c>
+      <c r="S114">
+        <v>12.02328452989945</v>
+      </c>
+      <c r="T114">
+        <v>6.269888869289116</v>
+      </c>
+      <c r="U114">
+        <v>0.3710688912941193</v>
+      </c>
+      <c r="V114">
+        <v>0.5690346895849001</v>
+      </c>
+      <c r="W114">
+        <v>0.08708000276170821</v>
+      </c>
+      <c r="X114">
+        <v>0.05172318852651109</v>
+      </c>
+      <c r="Y114">
+        <v>0.2354164285065531</v>
+      </c>
+      <c r="Z114">
+        <v>0.2220945909507399</v>
+      </c>
+      <c r="AA114">
+        <v>0.9992487709361478</v>
+      </c>
+      <c r="AB114">
+        <v>0.8005659627676538</v>
+      </c>
+      <c r="AC114">
+        <v>0.8172297407556183</v>
+      </c>
+      <c r="AD114">
+        <v>0.9990207531239762</v>
+      </c>
+      <c r="AE114">
+        <v>0.7659980520567966</v>
+      </c>
+      <c r="AF114">
+        <v>0.7780192756202823</v>
+      </c>
+      <c r="AG114">
+        <v>0.007020209487453265</v>
+      </c>
+      <c r="AH114">
+        <v>0.006483902172103396</v>
+      </c>
+      <c r="AI114">
+        <v>0.9992487709361478</v>
+      </c>
+      <c r="AJ114">
+        <v>0.9990207531239762</v>
+      </c>
+      <c r="AK114">
+        <v>0.007020209487453265</v>
+      </c>
+      <c r="AL114">
+        <v>0.006483902172103396</v>
+      </c>
+      <c r="AM114" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN114">
+        <v>0.01639215161744757</v>
+      </c>
+      <c r="AO114">
+        <v>0.01765530710928148</v>
+      </c>
+      <c r="AP114">
+        <v>-1447.13170248</v>
+      </c>
+      <c r="AQ114">
+        <v>-184.18012836</v>
+      </c>
+      <c r="AR114">
+        <v>35202.18169751958</v>
+      </c>
+      <c r="AS114">
+        <v>13886.6123716398</v>
+      </c>
+      <c r="AT114">
+        <v>35202.18169751958</v>
+      </c>
+      <c r="AU114">
+        <v>13883.4948716398</v>
+      </c>
+      <c r="AV114">
+        <v>2.520218169751959</v>
+      </c>
+      <c r="AW114">
+        <v>0.3886612371639797</v>
+      </c>
+      <c r="AX114">
+        <v>1.992794260058104</v>
+      </c>
+      <c r="AY114">
+        <v>3.824565254094209</v>
+      </c>
+      <c r="AZ114">
+        <v>103.3833333333333</v>
+      </c>
+      <c r="BA114">
+        <v>101.7</v>
+      </c>
+      <c r="BB114">
+        <v>0.07344354398813382</v>
+      </c>
+      <c r="BC114">
+        <v>0.02217448527738178</v>
+      </c>
+      <c r="BD114">
+        <v>-2112.359164136457</v>
+      </c>
+      <c r="BE114">
+        <v>-92.31476065965876</v>
+      </c>
+      <c r="BF114">
+        <v>4616</v>
+      </c>
+      <c r="BG114">
+        <v>2679</v>
+      </c>
+      <c r="BH114">
+        <v>944.8333333333334</v>
+      </c>
+      <c r="BI114">
+        <v>6744</v>
+      </c>
+      <c r="BJ114">
+        <v>3245</v>
+      </c>
+      <c r="BK114">
+        <v>11360</v>
+      </c>
+      <c r="BL114">
+        <v>5924</v>
+      </c>
+      <c r="BM114">
+        <v>4514</v>
+      </c>
+      <c r="BN114">
+        <v>2654</v>
+      </c>
+      <c r="BO114">
+        <v>4584</v>
+      </c>
+      <c r="BP114">
+        <v>2671</v>
+      </c>
+      <c r="BQ114">
+        <v>2230</v>
+      </c>
+      <c r="BR114">
+        <v>591</v>
+      </c>
+      <c r="BS114">
+        <v>32</v>
+      </c>
+      <c r="BT114">
+        <v>8</v>
+      </c>
+      <c r="BU114">
+        <v>0</v>
+      </c>
+      <c r="BV114">
+        <v>0</v>
+      </c>
+      <c r="BW114">
+        <v>25202.18169751999</v>
+      </c>
+      <c r="BX114">
+        <v>3886.612371639999</v>
+      </c>
+      <c r="BY114">
+        <v>0.04713910443059481</v>
+      </c>
+      <c r="BZ114">
+        <v>0.1331273979846798</v>
+      </c>
+      <c r="CA114">
+        <v>0.1324658375463523</v>
+      </c>
+      <c r="CB114">
+        <v>0.185760551100755</v>
+      </c>
+      <c r="CC114">
+        <v>0.008901683112434283</v>
+      </c>
+      <c r="CD114">
+        <v>0.01982772971514233</v>
+      </c>
+      <c r="CE114">
+        <v>0.009351256826871969</v>
+      </c>
+      <c r="CF114">
+        <v>0.02264025183175318</v>
+      </c>
+      <c r="CG114">
+        <v>26649.3134</v>
+      </c>
+      <c r="CH114">
+        <v>4070.792499999999</v>
+      </c>
+      <c r="CI114">
+        <v>28761.67256413645</v>
+      </c>
+      <c r="CJ114">
+        <v>4163.107260659657</v>
+      </c>
+      <c r="CK114">
+        <v>0.1707211213404628</v>
+      </c>
+      <c r="CL114">
+        <v>0.06628332839888486</v>
+      </c>
+      <c r="CM114">
+        <v>10000</v>
+      </c>
+      <c r="CO114">
+        <v>0.002778145257309168</v>
+      </c>
+      <c r="CP114">
+        <v>0.004630242095515279</v>
+      </c>
+      <c r="CQ114">
+        <v>7607086.794297621</v>
+      </c>
+      <c r="CR114">
+        <v>778558.4127862654</v>
+      </c>
+      <c r="CS114" s="2">
+        <v>45412.53331743644</v>
+      </c>
+      <c r="CT114">
+        <v>-0.7935423347142916</v>
+      </c>
+      <c r="CU114">
+        <v>-0.9129370942470093</v>
+      </c>
+    </row>
+    <row r="115" spans="10:99">
+      <c r="J115" t="s">
+        <v>236</v>
+      </c>
+      <c r="K115">
+        <v>0.0011764066703146</v>
+      </c>
+      <c r="L115">
+        <v>0.0005882033351573002</v>
+      </c>
+      <c r="M115">
+        <v>0.001023786990567377</v>
+      </c>
+      <c r="N115">
+        <v>0.001023786990567377</v>
+      </c>
+      <c r="O115">
+        <v>0.0007126653475587163</v>
+      </c>
+      <c r="P115">
+        <v>0.0003563326737793582</v>
+      </c>
+      <c r="Q115">
+        <v>0.0009153344400036456</v>
+      </c>
+      <c r="R115">
+        <v>0.0009153344400036456</v>
+      </c>
+      <c r="S115">
+        <v>31.09471816042286</v>
+      </c>
+      <c r="T115">
+        <v>33.90223388248003</v>
+      </c>
+      <c r="U115">
+        <v>0.4149413448324196</v>
+      </c>
+      <c r="V115">
+        <v>0.6844309575576462</v>
+      </c>
+      <c r="W115">
+        <v>0.02345340730515126</v>
+      </c>
+      <c r="X115">
+        <v>0.09754487625873115</v>
+      </c>
+      <c r="Y115">
+        <v>0.1494496435073214</v>
+      </c>
+      <c r="Z115">
+        <v>0.1825139991471437</v>
+      </c>
+      <c r="AA115">
+        <v>0.999455486528507</v>
+      </c>
+      <c r="AB115">
+        <v>0.8751465945165627</v>
+      </c>
+      <c r="AC115">
+        <v>0.8522833270181041</v>
+      </c>
+      <c r="AD115">
+        <v>0.9970942901237999</v>
+      </c>
+      <c r="AE115">
+        <v>0.8508861639137382</v>
+      </c>
+      <c r="AF115">
+        <v>0.8191104170810597</v>
+      </c>
+      <c r="AG115">
+        <v>0.004020137648003813</v>
+      </c>
+      <c r="AH115">
+        <v>0.01151219780637629</v>
+      </c>
+      <c r="AI115">
+        <v>0.999455486528507</v>
+      </c>
+      <c r="AJ115">
+        <v>0.9970942901237999</v>
+      </c>
+      <c r="AK115">
+        <v>0.004020137648003813</v>
+      </c>
+      <c r="AL115">
+        <v>0.01151219780637629</v>
+      </c>
+      <c r="AM115" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN115">
+        <v>0.01228333733755324</v>
+      </c>
+      <c r="AO115">
+        <v>0.08630833368542579</v>
+      </c>
+      <c r="AP115">
+        <v>-2563.38316448</v>
+      </c>
+      <c r="AQ115">
+        <v>-1340.363133152</v>
+      </c>
+      <c r="AR115">
+        <v>35598.68043552066</v>
+      </c>
+      <c r="AS115">
+        <v>30194.71162684839</v>
+      </c>
+      <c r="AT115">
+        <v>35596.95387552065</v>
+      </c>
+      <c r="AU115">
+        <v>30191.52255684839</v>
+      </c>
+      <c r="AV115">
+        <v>2.559868043552065</v>
+      </c>
+      <c r="AW115">
+        <v>2.019471162684839</v>
+      </c>
+      <c r="AX115">
+        <v>0.7709921580305736</v>
+      </c>
+      <c r="AY115">
+        <v>0.7072867730070287</v>
+      </c>
+      <c r="AZ115">
+        <v>120.2666666666667</v>
+      </c>
+      <c r="BA115">
+        <v>108</v>
+      </c>
+      <c r="BB115">
+        <v>0.0003186614014887787</v>
+      </c>
+      <c r="BC115">
+        <v>0.04155436371207163</v>
+      </c>
+      <c r="BD115">
+        <v>-8.977023286413763</v>
+      </c>
+      <c r="BE115">
+        <v>-933.6745823264008</v>
+      </c>
+      <c r="BF115">
+        <v>15966</v>
+      </c>
+      <c r="BG115">
+        <v>9603</v>
+      </c>
+      <c r="BH115">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI115">
+        <v>17615</v>
+      </c>
+      <c r="BJ115">
+        <v>27010</v>
+      </c>
+      <c r="BK115">
+        <v>33581</v>
+      </c>
+      <c r="BL115">
+        <v>36613</v>
+      </c>
+      <c r="BM115">
+        <v>15955</v>
+      </c>
+      <c r="BN115">
+        <v>8326</v>
+      </c>
+      <c r="BO115">
+        <v>15965</v>
+      </c>
+      <c r="BP115">
+        <v>9574</v>
+      </c>
+      <c r="BQ115">
+        <v>1660</v>
+      </c>
+      <c r="BR115">
+        <v>18684</v>
+      </c>
+      <c r="BS115">
+        <v>1</v>
+      </c>
+      <c r="BT115">
+        <v>29</v>
+      </c>
+      <c r="BU115">
+        <v>0</v>
+      </c>
+      <c r="BV115">
+        <v>0</v>
+      </c>
+      <c r="BW115">
+        <v>25598.68043551999</v>
+      </c>
+      <c r="BX115">
+        <v>20194.71162684798</v>
+      </c>
+      <c r="BY115">
+        <v>0.04642701133194607</v>
+      </c>
+      <c r="BZ115">
+        <v>0.08882340233564429</v>
+      </c>
+      <c r="CA115">
+        <v>0.08053877815937154</v>
+      </c>
+      <c r="CB115">
+        <v>0.1531770329222444</v>
+      </c>
+      <c r="CC115">
+        <v>0.01637970055109596</v>
+      </c>
+      <c r="CD115">
+        <v>0.009657645357842229</v>
+      </c>
+      <c r="CE115">
+        <v>0.01086609564332599</v>
+      </c>
+      <c r="CF115">
+        <v>0.01351477954456124</v>
+      </c>
+      <c r="CG115">
+        <v>28162.06359999999</v>
+      </c>
+      <c r="CH115">
+        <v>21535.07475999998</v>
+      </c>
+      <c r="CI115">
+        <v>28171.0406232864</v>
+      </c>
+      <c r="CJ115">
+        <v>22468.74934232638</v>
+      </c>
+      <c r="CK115">
+        <v>0.05013848635342553</v>
+      </c>
+      <c r="CL115">
+        <v>0.08603903262552468</v>
+      </c>
+      <c r="CM115">
+        <v>10000</v>
+      </c>
+      <c r="CO115">
+        <v>0.001658950617283951</v>
+      </c>
+      <c r="CP115">
+        <v>0.01161265432098765</v>
+      </c>
+      <c r="CQ115">
+        <v>8081982.566677582</v>
+      </c>
+      <c r="CR115">
+        <v>22312718.74654885</v>
+      </c>
+      <c r="CS115" s="2">
+        <v>45412.79877642162</v>
+      </c>
+      <c r="CT115">
+        <v>-0.833943178203995</v>
+      </c>
+      <c r="CU115">
+        <v>-0.679446363535763</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ETCUSDT.json at 2024-05-01_08-50-20 bestfile_scores 0.0008917861688722051 bestfile_sharp 0.0536201652151181
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU115"/>
+  <dimension ref="A1:CU116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -33324,6 +33324,275 @@
       </c>
       <c r="CU115">
         <v>-0.679446363535763</v>
+      </c>
+    </row>
+    <row r="116" spans="10:99">
+      <c r="J116" t="s">
+        <v>237</v>
+      </c>
+      <c r="K116">
+        <v>0.001602260593513094</v>
+      </c>
+      <c r="L116">
+        <v>0.000801130296756547</v>
+      </c>
+      <c r="M116">
+        <v>0.001450036051263259</v>
+      </c>
+      <c r="N116">
+        <v>0.001450036051263259</v>
+      </c>
+      <c r="O116">
+        <v>0.001316897982484488</v>
+      </c>
+      <c r="P116">
+        <v>0.0006584489912422442</v>
+      </c>
+      <c r="Q116">
+        <v>0.0007752411627323097</v>
+      </c>
+      <c r="R116">
+        <v>0.0007752411627323097</v>
+      </c>
+      <c r="S116">
+        <v>22.19437478297774</v>
+      </c>
+      <c r="T116">
+        <v>30.18264593541418</v>
+      </c>
+      <c r="U116">
+        <v>0.2916283437389677</v>
+      </c>
+      <c r="V116">
+        <v>0.6960496214562415</v>
+      </c>
+      <c r="W116">
+        <v>0.0757921519905654</v>
+      </c>
+      <c r="X116">
+        <v>0.0845818751314278</v>
+      </c>
+      <c r="Y116">
+        <v>0.2219436271046168</v>
+      </c>
+      <c r="Z116">
+        <v>0.1788494926315526</v>
+      </c>
+      <c r="AA116">
+        <v>0.9988791794011113</v>
+      </c>
+      <c r="AB116">
+        <v>0.8007267351187684</v>
+      </c>
+      <c r="AC116">
+        <v>0.849076768561113</v>
+      </c>
+      <c r="AD116">
+        <v>0.9986499609779006</v>
+      </c>
+      <c r="AE116">
+        <v>0.7743912808155745</v>
+      </c>
+      <c r="AF116">
+        <v>0.8307477509788787</v>
+      </c>
+      <c r="AG116">
+        <v>0.009109850615393149</v>
+      </c>
+      <c r="AH116">
+        <v>0.008557563814572426</v>
+      </c>
+      <c r="AI116">
+        <v>0.9988791794011113</v>
+      </c>
+      <c r="AJ116">
+        <v>0.9986499609779006</v>
+      </c>
+      <c r="AK116">
+        <v>0.009109850615393149</v>
+      </c>
+      <c r="AL116">
+        <v>0.008557563814572426</v>
+      </c>
+      <c r="AM116" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN116">
+        <v>0.02536547490544452</v>
+      </c>
+      <c r="AO116">
+        <v>0.05531176656181399</v>
+      </c>
+      <c r="AP116">
+        <v>-7485.262525222</v>
+      </c>
+      <c r="AQ116">
+        <v>-2103.052164396</v>
+      </c>
+      <c r="AR116">
+        <v>56349.5918047778</v>
+      </c>
+      <c r="AS116">
+        <v>47819.30096560418</v>
+      </c>
+      <c r="AT116">
+        <v>56349.5918047778</v>
+      </c>
+      <c r="AU116">
+        <v>47814.34227560418</v>
+      </c>
+      <c r="AV116">
+        <v>4.634959180477781</v>
+      </c>
+      <c r="AW116">
+        <v>3.781930096560418</v>
+      </c>
+      <c r="AX116">
+        <v>1.080298731642189</v>
+      </c>
+      <c r="AY116">
+        <v>0.7947445927289462</v>
+      </c>
+      <c r="AZ116">
+        <v>116.8833333333333</v>
+      </c>
+      <c r="BA116">
+        <v>83.75</v>
+      </c>
+      <c r="BB116">
+        <v>0.006273788133967209</v>
+      </c>
+      <c r="BC116">
+        <v>0.1096291240312252</v>
+      </c>
+      <c r="BD116">
+        <v>-339.8808104851926</v>
+      </c>
+      <c r="BE116">
+        <v>-4915.538817624845</v>
+      </c>
+      <c r="BF116">
+        <v>11374</v>
+      </c>
+      <c r="BG116">
+        <v>9056</v>
+      </c>
+      <c r="BH116">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI116">
+        <v>12595</v>
+      </c>
+      <c r="BJ116">
+        <v>23540</v>
+      </c>
+      <c r="BK116">
+        <v>23969</v>
+      </c>
+      <c r="BL116">
+        <v>32596</v>
+      </c>
+      <c r="BM116">
+        <v>11329</v>
+      </c>
+      <c r="BN116">
+        <v>7639</v>
+      </c>
+      <c r="BO116">
+        <v>11335</v>
+      </c>
+      <c r="BP116">
+        <v>8954</v>
+      </c>
+      <c r="BQ116">
+        <v>1266</v>
+      </c>
+      <c r="BR116">
+        <v>15901</v>
+      </c>
+      <c r="BS116">
+        <v>39</v>
+      </c>
+      <c r="BT116">
+        <v>102</v>
+      </c>
+      <c r="BU116">
+        <v>0</v>
+      </c>
+      <c r="BV116">
+        <v>0</v>
+      </c>
+      <c r="BW116">
+        <v>46349.59180477803</v>
+      </c>
+      <c r="BX116">
+        <v>37819.30096560407</v>
+      </c>
+      <c r="BY116">
+        <v>0.04953408649051043</v>
+      </c>
+      <c r="BZ116">
+        <v>0.069002043344828</v>
+      </c>
+      <c r="CA116">
+        <v>0.1270990220745482</v>
+      </c>
+      <c r="CB116">
+        <v>0.1447513491842313</v>
+      </c>
+      <c r="CC116">
+        <v>0.01224062090051484</v>
+      </c>
+      <c r="CD116">
+        <v>0.009224494405355782</v>
+      </c>
+      <c r="CE116">
+        <v>0.01036379640413962</v>
+      </c>
+      <c r="CF116">
+        <v>0.00874171200185909</v>
+      </c>
+      <c r="CG116">
+        <v>53834.85433000003</v>
+      </c>
+      <c r="CH116">
+        <v>39922.35313000008</v>
+      </c>
+      <c r="CI116">
+        <v>54174.73514048522</v>
+      </c>
+      <c r="CJ116">
+        <v>44837.89194762492</v>
+      </c>
+      <c r="CK116">
+        <v>0.16944021001402</v>
+      </c>
+      <c r="CL116">
+        <v>0.1636354035588614</v>
+      </c>
+      <c r="CM116">
+        <v>10000</v>
+      </c>
+      <c r="CO116">
+        <v>0.01076388888888889</v>
+      </c>
+      <c r="CP116">
+        <v>0.02611882716049383</v>
+      </c>
+      <c r="CQ116">
+        <v>23700316.72310792</v>
+      </c>
+      <c r="CR116">
+        <v>55051148.20247716</v>
+      </c>
+      <c r="CS116" s="2">
+        <v>45413.12341573772</v>
+      </c>
+      <c r="CT116">
+        <v>-0.7450076808546802</v>
+      </c>
+      <c r="CU116">
+        <v>-0.731628038523951</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update IMXUSDT.json at 2024-05-01_12-33-49 bestfile_scores 0.0006775413019645016 bestfile_sharp 0.14823706357858993
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU116"/>
+  <dimension ref="A1:CU117"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -33593,6 +33593,275 @@
       </c>
       <c r="CU116">
         <v>-0.731628038523951</v>
+      </c>
+    </row>
+    <row r="117" spans="10:99">
+      <c r="J117" t="s">
+        <v>238</v>
+      </c>
+      <c r="K117">
+        <v>0.002588371817037638</v>
+      </c>
+      <c r="L117">
+        <v>0.001294185908518819</v>
+      </c>
+      <c r="M117">
+        <v>0.0004942776023173501</v>
+      </c>
+      <c r="N117">
+        <v>0.0004942776023173501</v>
+      </c>
+      <c r="O117">
+        <v>0.002805644880524572</v>
+      </c>
+      <c r="P117">
+        <v>0.001402822440262286</v>
+      </c>
+      <c r="Q117">
+        <v>0.0003758587243903655</v>
+      </c>
+      <c r="R117">
+        <v>0.0003758587243903655</v>
+      </c>
+      <c r="S117">
+        <v>50.66182660745318</v>
+      </c>
+      <c r="T117">
+        <v>76.4626375748214</v>
+      </c>
+      <c r="U117">
+        <v>0.3747403029156091</v>
+      </c>
+      <c r="V117">
+        <v>0.6491281549053534</v>
+      </c>
+      <c r="W117">
+        <v>0.08753511642839872</v>
+      </c>
+      <c r="X117">
+        <v>0.06417873757640563</v>
+      </c>
+      <c r="Y117">
+        <v>0.2336348609708445</v>
+      </c>
+      <c r="Z117">
+        <v>0.1819060149657591</v>
+      </c>
+      <c r="AA117">
+        <v>0.9991798487966487</v>
+      </c>
+      <c r="AB117">
+        <v>0.816011856348867</v>
+      </c>
+      <c r="AC117">
+        <v>0.8332340310231882</v>
+      </c>
+      <c r="AD117">
+        <v>0.9990890839750988</v>
+      </c>
+      <c r="AE117">
+        <v>0.7666778888905852</v>
+      </c>
+      <c r="AF117">
+        <v>0.8185963672901637</v>
+      </c>
+      <c r="AG117">
+        <v>0.007870567990945843</v>
+      </c>
+      <c r="AH117">
+        <v>0.007355055002484102</v>
+      </c>
+      <c r="AI117">
+        <v>0.9991798487966487</v>
+      </c>
+      <c r="AJ117">
+        <v>0.9990890839750988</v>
+      </c>
+      <c r="AK117">
+        <v>0.007870567990945843</v>
+      </c>
+      <c r="AL117">
+        <v>0.007355055002484102</v>
+      </c>
+      <c r="AM117" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN117">
+        <v>0.01898391796554559</v>
+      </c>
+      <c r="AO117">
+        <v>0.02847792630469306</v>
+      </c>
+      <c r="AP117">
+        <v>-21214.949442558</v>
+      </c>
+      <c r="AQ117">
+        <v>-1956.10907142</v>
+      </c>
+      <c r="AR117">
+        <v>162669.7916274428</v>
+      </c>
+      <c r="AS117">
+        <v>17043.31890858102</v>
+      </c>
+      <c r="AT117">
+        <v>162669.7916274428</v>
+      </c>
+      <c r="AU117">
+        <v>17039.90806858102</v>
+      </c>
+      <c r="AV117">
+        <v>15.26697916274427</v>
+      </c>
+      <c r="AW117">
+        <v>0.704331890858102</v>
+      </c>
+      <c r="AX117">
+        <v>0.4734942036674533</v>
+      </c>
+      <c r="AY117">
+        <v>0.3135995587825307</v>
+      </c>
+      <c r="AZ117">
+        <v>59.98333333333333</v>
+      </c>
+      <c r="BA117">
+        <v>63.33333333333334</v>
+      </c>
+      <c r="BB117">
+        <v>0.02460980564259875</v>
+      </c>
+      <c r="BC117">
+        <v>0.03174906024003513</v>
+      </c>
+      <c r="BD117">
+        <v>-4387.238775519522</v>
+      </c>
+      <c r="BE117">
+        <v>-295.0922837562236</v>
+      </c>
+      <c r="BF117">
+        <v>25279</v>
+      </c>
+      <c r="BG117">
+        <v>38498</v>
+      </c>
+      <c r="BH117">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI117">
+        <v>29383</v>
+      </c>
+      <c r="BJ117">
+        <v>44002</v>
+      </c>
+      <c r="BK117">
+        <v>54662</v>
+      </c>
+      <c r="BL117">
+        <v>82500</v>
+      </c>
+      <c r="BM117">
+        <v>25140</v>
+      </c>
+      <c r="BN117">
+        <v>38312</v>
+      </c>
+      <c r="BO117">
+        <v>25182</v>
+      </c>
+      <c r="BP117">
+        <v>38414</v>
+      </c>
+      <c r="BQ117">
+        <v>4243</v>
+      </c>
+      <c r="BR117">
+        <v>5690</v>
+      </c>
+      <c r="BS117">
+        <v>97</v>
+      </c>
+      <c r="BT117">
+        <v>84</v>
+      </c>
+      <c r="BU117">
+        <v>0</v>
+      </c>
+      <c r="BV117">
+        <v>0</v>
+      </c>
+      <c r="BW117">
+        <v>152669.7916274422</v>
+      </c>
+      <c r="BX117">
+        <v>7043.318908580002</v>
+      </c>
+      <c r="BY117">
+        <v>0.03728433373666599</v>
+      </c>
+      <c r="BZ117">
+        <v>0.06907914298395479</v>
+      </c>
+      <c r="CA117">
+        <v>0.132031062170961</v>
+      </c>
+      <c r="CB117">
+        <v>0.1542351160507225</v>
+      </c>
+      <c r="CC117">
+        <v>0.005954208521050854</v>
+      </c>
+      <c r="CD117">
+        <v>0.008228572727710446</v>
+      </c>
+      <c r="CE117">
+        <v>0.006652357466780163</v>
+      </c>
+      <c r="CF117">
+        <v>0.009058681671161613</v>
+      </c>
+      <c r="CG117">
+        <v>173884.7410700002</v>
+      </c>
+      <c r="CH117">
+        <v>8999.427980000002</v>
+      </c>
+      <c r="CI117">
+        <v>178271.9798455197</v>
+      </c>
+      <c r="CJ117">
+        <v>9294.520263756225</v>
+      </c>
+      <c r="CK117">
+        <v>0.0536201652151181</v>
+      </c>
+      <c r="CL117">
+        <v>0.07418276535382101</v>
+      </c>
+      <c r="CM117">
+        <v>10000</v>
+      </c>
+      <c r="CO117">
+        <v>0.01224127278344146</v>
+      </c>
+      <c r="CP117">
+        <v>0.01007877664504171</v>
+      </c>
+      <c r="CQ117">
+        <v>91063086.28766407</v>
+      </c>
+      <c r="CR117">
+        <v>7593228.666961946</v>
+      </c>
+      <c r="CS117" s="2">
+        <v>45413.36830803961</v>
+      </c>
+      <c r="CT117">
+        <v>-0.5920454049159357</v>
+      </c>
+      <c r="CU117">
+        <v>-0.8501899077399586</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ANKRUSDT.json at 2024-05-01_16-13-34 bestfile_scores 0.0006027320153614652 bestfile_sharp 0.11012474330193417
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU117"/>
+  <dimension ref="A1:CU118"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -33862,6 +33862,275 @@
       </c>
       <c r="CU117">
         <v>-0.8501899077399586</v>
+      </c>
+    </row>
+    <row r="118" spans="10:99">
+      <c r="J118" t="s">
+        <v>239</v>
+      </c>
+      <c r="K118">
+        <v>0.0007855416203648158</v>
+      </c>
+      <c r="L118">
+        <v>0.0003927708101824079</v>
+      </c>
+      <c r="M118">
+        <v>0.0008271423402952394</v>
+      </c>
+      <c r="N118">
+        <v>0.0008271423402952394</v>
+      </c>
+      <c r="O118">
+        <v>0.001616415754485079</v>
+      </c>
+      <c r="P118">
+        <v>0.0008082078772425394</v>
+      </c>
+      <c r="Q118">
+        <v>0.0006820441801378196</v>
+      </c>
+      <c r="R118">
+        <v>0.0006820441801378196</v>
+      </c>
+      <c r="S118">
+        <v>6.96563078822803</v>
+      </c>
+      <c r="T118">
+        <v>7.855937435686354</v>
+      </c>
+      <c r="U118">
+        <v>0.4849341436243124</v>
+      </c>
+      <c r="V118">
+        <v>0.7246979754694026</v>
+      </c>
+      <c r="W118">
+        <v>0.01251436909255606</v>
+      </c>
+      <c r="X118">
+        <v>0.06877541536742211</v>
+      </c>
+      <c r="Y118">
+        <v>0.04985784787440725</v>
+      </c>
+      <c r="Z118">
+        <v>0.1338662756941098</v>
+      </c>
+      <c r="AA118">
+        <v>0.9997197451456383</v>
+      </c>
+      <c r="AB118">
+        <v>0.9660824341024499</v>
+      </c>
+      <c r="AC118">
+        <v>0.8845333089085399</v>
+      </c>
+      <c r="AD118">
+        <v>0.9982147774761528</v>
+      </c>
+      <c r="AE118">
+        <v>0.8232871744991254</v>
+      </c>
+      <c r="AF118">
+        <v>0.8663069565383469</v>
+      </c>
+      <c r="AG118">
+        <v>0.001542048874828544</v>
+      </c>
+      <c r="AH118">
+        <v>0.008099477647247812</v>
+      </c>
+      <c r="AI118">
+        <v>0.9997197451456383</v>
+      </c>
+      <c r="AJ118">
+        <v>0.9982147774761528</v>
+      </c>
+      <c r="AK118">
+        <v>0.001542048874828544</v>
+      </c>
+      <c r="AL118">
+        <v>0.008099477647247812</v>
+      </c>
+      <c r="AM118" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN118">
+        <v>0.006704310341163472</v>
+      </c>
+      <c r="AO118">
+        <v>0.04899000398163822</v>
+      </c>
+      <c r="AP118">
+        <v>-375.79069566</v>
+      </c>
+      <c r="AQ118">
+        <v>-412.78013622</v>
+      </c>
+      <c r="AR118">
+        <v>18887.36440434008</v>
+      </c>
+      <c r="AS118">
+        <v>19533.98276378008</v>
+      </c>
+      <c r="AT118">
+        <v>18887.36440434008</v>
+      </c>
+      <c r="AU118">
+        <v>19533.98276378008</v>
+      </c>
+      <c r="AV118">
+        <v>0.8887364404340079</v>
+      </c>
+      <c r="AW118">
+        <v>0.9533982763780084</v>
+      </c>
+      <c r="AX118">
+        <v>3.44354609929078</v>
+      </c>
+      <c r="AY118">
+        <v>3.047065450924907</v>
+      </c>
+      <c r="AZ118">
+        <v>103.45</v>
+      </c>
+      <c r="BA118">
+        <v>101.4666666666667</v>
+      </c>
+      <c r="BB118">
+        <v>0.003909031555751341</v>
+      </c>
+      <c r="BC118">
+        <v>0.008242114210051747</v>
+      </c>
+      <c r="BD118">
+        <v>-36.3520669686161</v>
+      </c>
+      <c r="BE118">
+        <v>-82.66367932815118</v>
+      </c>
+      <c r="BF118">
+        <v>2582</v>
+      </c>
+      <c r="BG118">
+        <v>2827</v>
+      </c>
+      <c r="BH118">
+        <v>809.8333333333334</v>
+      </c>
+      <c r="BI118">
+        <v>3059</v>
+      </c>
+      <c r="BJ118">
+        <v>3535</v>
+      </c>
+      <c r="BK118">
+        <v>5641</v>
+      </c>
+      <c r="BL118">
+        <v>6362</v>
+      </c>
+      <c r="BM118">
+        <v>2547</v>
+      </c>
+      <c r="BN118">
+        <v>2150</v>
+      </c>
+      <c r="BO118">
+        <v>2578</v>
+      </c>
+      <c r="BP118">
+        <v>2513</v>
+      </c>
+      <c r="BQ118">
+        <v>512</v>
+      </c>
+      <c r="BR118">
+        <v>1385</v>
+      </c>
+      <c r="BS118">
+        <v>4</v>
+      </c>
+      <c r="BT118">
+        <v>314</v>
+      </c>
+      <c r="BU118">
+        <v>0</v>
+      </c>
+      <c r="BV118">
+        <v>0</v>
+      </c>
+      <c r="BW118">
+        <v>8887.364404340005</v>
+      </c>
+      <c r="BX118">
+        <v>9533.982763779992</v>
+      </c>
+      <c r="BY118">
+        <v>0.05274203025906914</v>
+      </c>
+      <c r="BZ118">
+        <v>0.07131693675439353</v>
+      </c>
+      <c r="CA118">
+        <v>0.1094381913783278</v>
+      </c>
+      <c r="CB118">
+        <v>0.1179237259716363</v>
+      </c>
+      <c r="CC118">
+        <v>0.01578000976636629</v>
+      </c>
+      <c r="CD118">
+        <v>0.01641427643114183</v>
+      </c>
+      <c r="CE118">
+        <v>0.01284992941167513</v>
+      </c>
+      <c r="CF118">
+        <v>0.01395921786232813</v>
+      </c>
+      <c r="CG118">
+        <v>9263.155100000005</v>
+      </c>
+      <c r="CH118">
+        <v>9946.762899999992</v>
+      </c>
+      <c r="CI118">
+        <v>9299.507166968622</v>
+      </c>
+      <c r="CJ118">
+        <v>10029.42657932814</v>
+      </c>
+      <c r="CK118">
+        <v>0.1482370635785899</v>
+      </c>
+      <c r="CL118">
+        <v>0.1057251422234848</v>
+      </c>
+      <c r="CM118">
+        <v>10000</v>
+      </c>
+      <c r="CO118">
+        <v>0.0002057930750630241</v>
+      </c>
+      <c r="CP118">
+        <v>0.009672274527962134</v>
+      </c>
+      <c r="CQ118">
+        <v>1583196.426444974</v>
+      </c>
+      <c r="CR118">
+        <v>8613700.914603613</v>
+      </c>
+      <c r="CS118" s="2">
+        <v>45413.52350057764</v>
+      </c>
+      <c r="CT118">
+        <v>-0.9326775287918465</v>
+      </c>
+      <c r="CU118">
+        <v>-0.819328101924633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSRUSDT.json at 2024-05-01_20-27-04 bestfile_scores 0.0005777682291534664 bestfile_sharp 0.1313121280384654
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1008" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="325">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1350,7 +1350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU118"/>
+  <dimension ref="A1:CU119"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -34131,6 +34131,275 @@
       </c>
       <c r="CU118">
         <v>-0.819328101924633</v>
+      </c>
+    </row>
+    <row r="119" spans="10:99">
+      <c r="J119" t="s">
+        <v>240</v>
+      </c>
+      <c r="K119">
+        <v>0.000586848041296939</v>
+      </c>
+      <c r="L119">
+        <v>0.0002934240206484695</v>
+      </c>
+      <c r="M119">
+        <v>0.0007602977885132756</v>
+      </c>
+      <c r="N119">
+        <v>0.0007602977885132756</v>
+      </c>
+      <c r="O119">
+        <v>0.001340336445264678</v>
+      </c>
+      <c r="P119">
+        <v>0.0006701682226323391</v>
+      </c>
+      <c r="Q119">
+        <v>0.0006870380296517764</v>
+      </c>
+      <c r="R119">
+        <v>0.0006870380296517764</v>
+      </c>
+      <c r="S119">
+        <v>17.30437131062155</v>
+      </c>
+      <c r="T119">
+        <v>10.96523785639878</v>
+      </c>
+      <c r="U119">
+        <v>0.3767461410131815</v>
+      </c>
+      <c r="V119">
+        <v>0.6482188329708638</v>
+      </c>
+      <c r="W119">
+        <v>0.01286153515563114</v>
+      </c>
+      <c r="X119">
+        <v>0.05437285660502358</v>
+      </c>
+      <c r="Y119">
+        <v>0.08136983366983706</v>
+      </c>
+      <c r="Z119">
+        <v>0.1679471309132682</v>
+      </c>
+      <c r="AA119">
+        <v>0.9996026900145027</v>
+      </c>
+      <c r="AB119">
+        <v>0.9440554904385013</v>
+      </c>
+      <c r="AC119">
+        <v>0.8503510239806825</v>
+      </c>
+      <c r="AD119">
+        <v>0.999160814888832</v>
+      </c>
+      <c r="AE119">
+        <v>0.8107907355508887</v>
+      </c>
+      <c r="AF119">
+        <v>0.8330220560037468</v>
+      </c>
+      <c r="AG119">
+        <v>0.001759085417154263</v>
+      </c>
+      <c r="AH119">
+        <v>0.006855097123469433</v>
+      </c>
+      <c r="AI119">
+        <v>0.9996026900145027</v>
+      </c>
+      <c r="AJ119">
+        <v>0.999160814888832</v>
+      </c>
+      <c r="AK119">
+        <v>0.001759085417154263</v>
+      </c>
+      <c r="AL119">
+        <v>0.006855097123469433</v>
+      </c>
+      <c r="AM119" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN119">
+        <v>0.009392776226783691</v>
+      </c>
+      <c r="AO119">
+        <v>0.02058650428729426</v>
+      </c>
+      <c r="AP119">
+        <v>-994.8875814959999</v>
+      </c>
+      <c r="AQ119">
+        <v>-661.2946131260001</v>
+      </c>
+      <c r="AR119">
+        <v>18843.54913850419</v>
+      </c>
+      <c r="AS119">
+        <v>22722.668696874</v>
+      </c>
+      <c r="AT119">
+        <v>18772.83768850419</v>
+      </c>
+      <c r="AU119">
+        <v>22722.668696874</v>
+      </c>
+      <c r="AV119">
+        <v>0.8843549138504194</v>
+      </c>
+      <c r="AW119">
+        <v>1.2722668696874</v>
+      </c>
+      <c r="AX119">
+        <v>1.386309555662582</v>
+      </c>
+      <c r="AY119">
+        <v>2.188194972271486</v>
+      </c>
+      <c r="AZ119">
+        <v>87.05</v>
+      </c>
+      <c r="BA119">
+        <v>109.5333333333333</v>
+      </c>
+      <c r="BB119">
+        <v>0.003751602177814708</v>
+      </c>
+      <c r="BC119">
+        <v>0.01787462162478973</v>
+      </c>
+      <c r="BD119">
+        <v>-37.04889333396146</v>
+      </c>
+      <c r="BE119">
+        <v>-243.5873110234629</v>
+      </c>
+      <c r="BF119">
+        <v>8924</v>
+      </c>
+      <c r="BG119">
+        <v>4860</v>
+      </c>
+      <c r="BH119">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI119">
+        <v>9764</v>
+      </c>
+      <c r="BJ119">
+        <v>6982</v>
+      </c>
+      <c r="BK119">
+        <v>18688</v>
+      </c>
+      <c r="BL119">
+        <v>11842</v>
+      </c>
+      <c r="BM119">
+        <v>8914</v>
+      </c>
+      <c r="BN119">
+        <v>4832</v>
+      </c>
+      <c r="BO119">
+        <v>8923</v>
+      </c>
+      <c r="BP119">
+        <v>4853</v>
+      </c>
+      <c r="BQ119">
+        <v>850</v>
+      </c>
+      <c r="BR119">
+        <v>2150</v>
+      </c>
+      <c r="BS119">
+        <v>1</v>
+      </c>
+      <c r="BT119">
+        <v>7</v>
+      </c>
+      <c r="BU119">
+        <v>0</v>
+      </c>
+      <c r="BV119">
+        <v>0</v>
+      </c>
+      <c r="BW119">
+        <v>8843.549138503988</v>
+      </c>
+      <c r="BX119">
+        <v>12722.66869687401</v>
+      </c>
+      <c r="BY119">
+        <v>0.05041162690277504</v>
+      </c>
+      <c r="BZ119">
+        <v>0.0901653305231279</v>
+      </c>
+      <c r="CA119">
+        <v>0.07285788512160295</v>
+      </c>
+      <c r="CB119">
+        <v>0.1467186596893149</v>
+      </c>
+      <c r="CC119">
+        <v>0.01752174807539791</v>
+      </c>
+      <c r="CD119">
+        <v>0.01058747663655681</v>
+      </c>
+      <c r="CE119">
+        <v>0.01254871868624434</v>
+      </c>
+      <c r="CF119">
+        <v>0.01513503020828842</v>
+      </c>
+      <c r="CG119">
+        <v>9838.436719999987</v>
+      </c>
+      <c r="CH119">
+        <v>13383.96331000001</v>
+      </c>
+      <c r="CI119">
+        <v>9875.485613333949</v>
+      </c>
+      <c r="CJ119">
+        <v>13627.55062102347</v>
+      </c>
+      <c r="CK119">
+        <v>0.1101247433019342</v>
+      </c>
+      <c r="CL119">
+        <v>0.102601789899034</v>
+      </c>
+      <c r="CM119">
+        <v>10000</v>
+      </c>
+      <c r="CO119">
+        <v>0.0005015432098765432</v>
+      </c>
+      <c r="CP119">
+        <v>0.004706790123456791</v>
+      </c>
+      <c r="CQ119">
+        <v>3091816.902562582</v>
+      </c>
+      <c r="CR119">
+        <v>2380328.733367264</v>
+      </c>
+      <c r="CS119" s="2">
+        <v>45413.67610922761</v>
+      </c>
+      <c r="CT119">
+        <v>-0.955941339278515</v>
+      </c>
+      <c r="CU119">
+        <v>-0.8444144380590699</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update HNTUSDT.json at 2024-05-02_17-22-54 bestfile_scores 0.0004373382157628808 bestfile_sharp 0.17735538728753586
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1050" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="361">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1458,7 +1458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU121"/>
+  <dimension ref="A1:CU122"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -35046,6 +35046,275 @@
       </c>
       <c r="CU121">
         <v>-0.8453122650833704</v>
+      </c>
+    </row>
+    <row r="122" spans="10:99">
+      <c r="J122" t="s">
+        <v>236</v>
+      </c>
+      <c r="K122">
+        <v>0.001728903964315354</v>
+      </c>
+      <c r="L122">
+        <v>0.0008644519821576768</v>
+      </c>
+      <c r="M122">
+        <v>0.0004287261639606132</v>
+      </c>
+      <c r="N122">
+        <v>0.0004287261639606132</v>
+      </c>
+      <c r="O122">
+        <v>0.001908969392300564</v>
+      </c>
+      <c r="P122">
+        <v>0.0009544846961502818</v>
+      </c>
+      <c r="Q122">
+        <v>0.0003620626646210434</v>
+      </c>
+      <c r="R122">
+        <v>0.0003620626646210434</v>
+      </c>
+      <c r="S122">
+        <v>15.5826221278239</v>
+      </c>
+      <c r="T122">
+        <v>41.69391774473837</v>
+      </c>
+      <c r="U122">
+        <v>0.4040347838832489</v>
+      </c>
+      <c r="V122">
+        <v>1</v>
+      </c>
+      <c r="W122">
+        <v>0.06714253843568732</v>
+      </c>
+      <c r="X122">
+        <v>0.04289001470941213</v>
+      </c>
+      <c r="Y122">
+        <v>0.1837206490800225</v>
+      </c>
+      <c r="Z122">
+        <v>0.09944049512904625</v>
+      </c>
+      <c r="AA122">
+        <v>0.998836257784695</v>
+      </c>
+      <c r="AB122">
+        <v>0.8393340151777245</v>
+      </c>
+      <c r="AC122">
+        <v>0.9199713071139491</v>
+      </c>
+      <c r="AD122">
+        <v>0.9985371762155364</v>
+      </c>
+      <c r="AE122">
+        <v>0.816602362743289</v>
+      </c>
+      <c r="AF122">
+        <v>0.9006492048194443</v>
+      </c>
+      <c r="AG122">
+        <v>0.007722970938455328</v>
+      </c>
+      <c r="AH122">
+        <v>0.005386378023791972</v>
+      </c>
+      <c r="AI122">
+        <v>0.998836257784695</v>
+      </c>
+      <c r="AJ122">
+        <v>0.9985371762155364</v>
+      </c>
+      <c r="AK122">
+        <v>0.007722970938455328</v>
+      </c>
+      <c r="AL122">
+        <v>0.005386378023791972</v>
+      </c>
+      <c r="AM122" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN122">
+        <v>0.03182171184361936</v>
+      </c>
+      <c r="AO122">
+        <v>0.04398480244716741</v>
+      </c>
+      <c r="AP122">
+        <v>-3661.709861474</v>
+      </c>
+      <c r="AQ122">
+        <v>-993.082788608</v>
+      </c>
+      <c r="AR122">
+        <v>64482.23290852636</v>
+      </c>
+      <c r="AS122">
+        <v>15880.05039139202</v>
+      </c>
+      <c r="AT122">
+        <v>64470.57916852636</v>
+      </c>
+      <c r="AU122">
+        <v>15875.69333139202</v>
+      </c>
+      <c r="AV122">
+        <v>5.448223290852637</v>
+      </c>
+      <c r="AW122">
+        <v>0.5880050391392022</v>
+      </c>
+      <c r="AX122">
+        <v>1.537845983027996</v>
+      </c>
+      <c r="AY122">
+        <v>0.575422177762958</v>
+      </c>
+      <c r="AZ122">
+        <v>119.8166666666667</v>
+      </c>
+      <c r="BA122">
+        <v>118.8166666666667</v>
+      </c>
+      <c r="BB122">
+        <v>0.002892679559724969</v>
+      </c>
+      <c r="BC122">
+        <v>0</v>
+      </c>
+      <c r="BD122">
+        <v>-168.6797311831305</v>
+      </c>
+      <c r="BE122">
+        <v>0</v>
+      </c>
+      <c r="BF122">
+        <v>6352</v>
+      </c>
+      <c r="BG122">
+        <v>18366</v>
+      </c>
+      <c r="BH122">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI122">
+        <v>10461</v>
+      </c>
+      <c r="BJ122">
+        <v>26620</v>
+      </c>
+      <c r="BK122">
+        <v>16813</v>
+      </c>
+      <c r="BL122">
+        <v>44986</v>
+      </c>
+      <c r="BM122">
+        <v>6229</v>
+      </c>
+      <c r="BN122">
+        <v>18330</v>
+      </c>
+      <c r="BO122">
+        <v>6343</v>
+      </c>
+      <c r="BP122">
+        <v>18366</v>
+      </c>
+      <c r="BQ122">
+        <v>4232</v>
+      </c>
+      <c r="BR122">
+        <v>8290</v>
+      </c>
+      <c r="BS122">
+        <v>9</v>
+      </c>
+      <c r="BT122">
+        <v>0</v>
+      </c>
+      <c r="BU122">
+        <v>0</v>
+      </c>
+      <c r="BV122">
+        <v>0</v>
+      </c>
+      <c r="BW122">
+        <v>54482.2329085259</v>
+      </c>
+      <c r="BX122">
+        <v>5880.050391392</v>
+      </c>
+      <c r="BY122">
+        <v>0.04021654892013991</v>
+      </c>
+      <c r="BZ122">
+        <v>0.08614027692450116</v>
+      </c>
+      <c r="CA122">
+        <v>0.1009521388215714</v>
+      </c>
+      <c r="CB122">
+        <v>0.1329467250439504</v>
+      </c>
+      <c r="CC122">
+        <v>0.009288235855895425</v>
+      </c>
+      <c r="CD122">
+        <v>0.0110460773745595</v>
+      </c>
+      <c r="CE122">
+        <v>0.007931947135435472</v>
+      </c>
+      <c r="CF122">
+        <v>0.01393756865436849</v>
+      </c>
+      <c r="CG122">
+        <v>58143.94276999991</v>
+      </c>
+      <c r="CH122">
+        <v>6873.13318</v>
+      </c>
+      <c r="CI122">
+        <v>58312.62250118304</v>
+      </c>
+      <c r="CJ122">
+        <v>6873.13318</v>
+      </c>
+      <c r="CK122">
+        <v>0.2023433174016643</v>
+      </c>
+      <c r="CL122">
+        <v>0.07165289775989087</v>
+      </c>
+      <c r="CM122">
+        <v>10000</v>
+      </c>
+      <c r="CO122">
+        <v>0.00892029657089898</v>
+      </c>
+      <c r="CP122">
+        <v>0</v>
+      </c>
+      <c r="CQ122">
+        <v>30477928.38179236</v>
+      </c>
+      <c r="CR122">
+        <v>4219262.028734344</v>
+      </c>
+      <c r="CS122" s="2">
+        <v>45414.53661663266</v>
+      </c>
+      <c r="CT122">
+        <v>-0.7390744315992817</v>
+      </c>
+      <c r="CU122">
+        <v>-0.8804699533217299</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update APTUSDT.json at 2024-05-02_20-37-27 bestfile_scores 0.0010850181058817993 bestfile_sharp 0.1232345957418265
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1052" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="362">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -740,6 +740,9 @@
   </si>
   <si>
     <t>RSRUSDT</t>
+  </si>
+  <si>
+    <t>HNTUSDT</t>
   </si>
   <si>
     <t>binance</t>
@@ -1458,7 +1461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU122"/>
+  <dimension ref="A1:CU123"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -1873,7 +1876,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN2">
         <v>0.049606857</v>
@@ -2038,7 +2041,7 @@
         <v>0</v>
       </c>
       <c r="CS2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:99">
@@ -2154,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="AM3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN3">
         <v>0.04006526</v>
@@ -2319,7 +2322,7 @@
         <v>0</v>
       </c>
       <c r="CS3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:99">
@@ -2435,7 +2438,7 @@
         <v>0</v>
       </c>
       <c r="AM4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN4">
         <v>0.092575794</v>
@@ -2600,7 +2603,7 @@
         <v>0</v>
       </c>
       <c r="CS4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:99">
@@ -2716,7 +2719,7 @@
         <v>0</v>
       </c>
       <c r="AM5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN5">
         <v>0.027448502</v>
@@ -2881,7 +2884,7 @@
         <v>0</v>
       </c>
       <c r="CS5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:99">
@@ -2997,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="AM6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN6">
         <v>0.083929868</v>
@@ -3162,7 +3165,7 @@
         <v>0</v>
       </c>
       <c r="CS6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:99">
@@ -3278,7 +3281,7 @@
         <v>0</v>
       </c>
       <c r="AM7" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN7">
         <v>0.145376251</v>
@@ -3443,7 +3446,7 @@
         <v>0</v>
       </c>
       <c r="CS7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:99">
@@ -3559,7 +3562,7 @@
         <v>0</v>
       </c>
       <c r="AM8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN8">
         <v>0.087987204</v>
@@ -3724,7 +3727,7 @@
         <v>0</v>
       </c>
       <c r="CS8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:99">
@@ -3840,7 +3843,7 @@
         <v>0</v>
       </c>
       <c r="AM9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN9">
         <v>0.118237951</v>
@@ -4005,7 +4008,7 @@
         <v>0</v>
       </c>
       <c r="CS9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:99">
@@ -4121,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="AM10" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN10">
         <v>0.08106915200000001</v>
@@ -4286,7 +4289,7 @@
         <v>0</v>
       </c>
       <c r="CS10" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:99">
@@ -4402,7 +4405,7 @@
         <v>0</v>
       </c>
       <c r="AM11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN11">
         <v>0.027960571</v>
@@ -4567,7 +4570,7 @@
         <v>0</v>
       </c>
       <c r="CS11" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:99">
@@ -4683,7 +4686,7 @@
         <v>0</v>
       </c>
       <c r="AM12" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN12">
         <v>0.032951036</v>
@@ -4848,7 +4851,7 @@
         <v>0</v>
       </c>
       <c r="CS12" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:99">
@@ -4964,7 +4967,7 @@
         <v>0</v>
       </c>
       <c r="AM13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN13">
         <v>0.179185242</v>
@@ -5129,7 +5132,7 @@
         <v>0</v>
       </c>
       <c r="CS13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:99">
@@ -5245,7 +5248,7 @@
         <v>0</v>
       </c>
       <c r="AM14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN14">
         <v>0.143233482</v>
@@ -5410,7 +5413,7 @@
         <v>0</v>
       </c>
       <c r="CS14" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:99">
@@ -5526,7 +5529,7 @@
         <v>0</v>
       </c>
       <c r="AM15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN15">
         <v>0.138115134</v>
@@ -5691,7 +5694,7 @@
         <v>0</v>
       </c>
       <c r="CS15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:99">
@@ -5807,7 +5810,7 @@
         <v>0</v>
       </c>
       <c r="AM16" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN16">
         <v>0.09650975000000001</v>
@@ -5972,7 +5975,7 @@
         <v>0</v>
       </c>
       <c r="CS16" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:97">
@@ -6088,7 +6091,7 @@
         <v>0</v>
       </c>
       <c r="AM17" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN17">
         <v>0.060693695</v>
@@ -6253,7 +6256,7 @@
         <v>0</v>
       </c>
       <c r="CS17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:97">
@@ -6369,7 +6372,7 @@
         <v>0</v>
       </c>
       <c r="AM18" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN18">
         <v>0.107514363</v>
@@ -6534,7 +6537,7 @@
         <v>0</v>
       </c>
       <c r="CS18" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:97">
@@ -6650,7 +6653,7 @@
         <v>0</v>
       </c>
       <c r="AM19" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN19">
         <v>0.014898256</v>
@@ -6815,7 +6818,7 @@
         <v>0</v>
       </c>
       <c r="CS19" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:97">
@@ -6931,7 +6934,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN20">
         <v>0.02858403</v>
@@ -7096,7 +7099,7 @@
         <v>0</v>
       </c>
       <c r="CS20" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:97">
@@ -7212,7 +7215,7 @@
         <v>0</v>
       </c>
       <c r="AM21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN21">
         <v>0.082273481</v>
@@ -7377,7 +7380,7 @@
         <v>0</v>
       </c>
       <c r="CS21" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:97">
@@ -7493,7 +7496,7 @@
         <v>0</v>
       </c>
       <c r="AM22" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN22">
         <v>0.012592558</v>
@@ -7658,7 +7661,7 @@
         <v>0</v>
       </c>
       <c r="CS22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:97">
@@ -7774,7 +7777,7 @@
         <v>0</v>
       </c>
       <c r="AM23" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN23">
         <v>0.00903967</v>
@@ -7939,7 +7942,7 @@
         <v>0</v>
       </c>
       <c r="CS23" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:97">
@@ -8055,7 +8058,7 @@
         <v>0</v>
       </c>
       <c r="AM24" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN24">
         <v>0.030046089</v>
@@ -8220,7 +8223,7 @@
         <v>0</v>
       </c>
       <c r="CS24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:97">
@@ -8336,7 +8339,7 @@
         <v>0</v>
       </c>
       <c r="AM25" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN25">
         <v>0.010607012</v>
@@ -8501,7 +8504,7 @@
         <v>0</v>
       </c>
       <c r="CS25" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:97">
@@ -8617,7 +8620,7 @@
         <v>0</v>
       </c>
       <c r="AM26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN26">
         <v>0.053096335</v>
@@ -8782,7 +8785,7 @@
         <v>0</v>
       </c>
       <c r="CS26" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="27" spans="1:97">
@@ -8898,7 +8901,7 @@
         <v>0</v>
       </c>
       <c r="AM27" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN27">
         <v>0.092674047</v>
@@ -9063,7 +9066,7 @@
         <v>0</v>
       </c>
       <c r="CS27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:97">
@@ -9179,7 +9182,7 @@
         <v>0</v>
       </c>
       <c r="AM28" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN28">
         <v>0.03099706</v>
@@ -9344,7 +9347,7 @@
         <v>0</v>
       </c>
       <c r="CS28" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:97">
@@ -9460,7 +9463,7 @@
         <v>0</v>
       </c>
       <c r="AM29" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN29">
         <v>0.069423731</v>
@@ -9625,7 +9628,7 @@
         <v>0</v>
       </c>
       <c r="CS29" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:97">
@@ -9741,7 +9744,7 @@
         <v>0</v>
       </c>
       <c r="AM30" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN30">
         <v>0.060424834</v>
@@ -9906,7 +9909,7 @@
         <v>0</v>
       </c>
       <c r="CS30" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:97">
@@ -10022,7 +10025,7 @@
         <v>0</v>
       </c>
       <c r="AM31" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN31">
         <v>0.056666776</v>
@@ -10187,7 +10190,7 @@
         <v>0</v>
       </c>
       <c r="CS31" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:97">
@@ -10303,7 +10306,7 @@
         <v>0</v>
       </c>
       <c r="AM32" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN32">
         <v>0.098888062</v>
@@ -10468,7 +10471,7 @@
         <v>0</v>
       </c>
       <c r="CS32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:99">
@@ -10584,7 +10587,7 @@
         <v>0</v>
       </c>
       <c r="AM33" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN33">
         <v>0.035815903</v>
@@ -10749,7 +10752,7 @@
         <v>0</v>
       </c>
       <c r="CS33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="34" spans="1:99">
@@ -10865,7 +10868,7 @@
         <v>0</v>
       </c>
       <c r="AM34" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN34">
         <v>0.037311133</v>
@@ -11030,7 +11033,7 @@
         <v>0</v>
       </c>
       <c r="CS34" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="CT34">
         <v>-0.814742818</v>
@@ -11152,7 +11155,7 @@
         <v>0</v>
       </c>
       <c r="AM35" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN35">
         <v>0.041330496</v>
@@ -11317,7 +11320,7 @@
         <v>0</v>
       </c>
       <c r="CS35" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="CT35">
         <v>-0.753066891</v>
@@ -11439,7 +11442,7 @@
         <v>0</v>
       </c>
       <c r="AM36" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN36">
         <v>0.047772102</v>
@@ -11604,7 +11607,7 @@
         <v>0</v>
       </c>
       <c r="CS36" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="CT36">
         <v>-0.872335259</v>
@@ -11726,7 +11729,7 @@
         <v>0</v>
       </c>
       <c r="AM37" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN37">
         <v>0.060484521</v>
@@ -11891,7 +11894,7 @@
         <v>0</v>
       </c>
       <c r="CS37" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="CT37">
         <v>-0.759885442</v>
@@ -12013,7 +12016,7 @@
         <v>0</v>
       </c>
       <c r="AM38" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN38">
         <v>0.061007062</v>
@@ -12178,7 +12181,7 @@
         <v>0</v>
       </c>
       <c r="CS38" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="CT38">
         <v>-0.838900609</v>
@@ -12300,7 +12303,7 @@
         <v>0</v>
       </c>
       <c r="AM39" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN39">
         <v>0.025236369</v>
@@ -12465,7 +12468,7 @@
         <v>0</v>
       </c>
       <c r="CS39" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="CT39">
         <v>-0.780218664</v>
@@ -12587,7 +12590,7 @@
         <v>0</v>
       </c>
       <c r="AM40" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN40">
         <v>0.031804424</v>
@@ -12752,7 +12755,7 @@
         <v>0</v>
       </c>
       <c r="CS40" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="CT40">
         <v>-0.79992089</v>
@@ -12874,7 +12877,7 @@
         <v>0</v>
       </c>
       <c r="AM41" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN41">
         <v>0.072404657</v>
@@ -13039,7 +13042,7 @@
         <v>0</v>
       </c>
       <c r="CS41" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="CT41">
         <v>-0.528089775</v>
@@ -13161,7 +13164,7 @@
         <v>0</v>
       </c>
       <c r="AM42" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN42">
         <v>0.06821192299999999</v>
@@ -13326,7 +13329,7 @@
         <v>0</v>
       </c>
       <c r="CS42" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="CT42">
         <v>-0.754849911</v>
@@ -13448,7 +13451,7 @@
         <v>0</v>
       </c>
       <c r="AM43" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN43">
         <v>0.069326524</v>
@@ -13613,7 +13616,7 @@
         <v>0</v>
       </c>
       <c r="CS43" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="CT43">
         <v>-0.7655395739999999</v>
@@ -13735,7 +13738,7 @@
         <v>0</v>
       </c>
       <c r="AM44" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN44">
         <v>0.036991009</v>
@@ -13900,7 +13903,7 @@
         <v>0</v>
       </c>
       <c r="CS44" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="CT44">
         <v>-0.829764531</v>
@@ -14022,7 +14025,7 @@
         <v>0</v>
       </c>
       <c r="AM45" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN45">
         <v>0.036729519</v>
@@ -14187,7 +14190,7 @@
         <v>0</v>
       </c>
       <c r="CS45" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="CT45">
         <v>-0.404237806</v>
@@ -14309,7 +14312,7 @@
         <v>0</v>
       </c>
       <c r="AM46" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN46">
         <v>0.045071814</v>
@@ -14474,7 +14477,7 @@
         <v>0</v>
       </c>
       <c r="CS46" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="CT46">
         <v>-0.703677808</v>
@@ -14596,7 +14599,7 @@
         <v>0</v>
       </c>
       <c r="AM47" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN47">
         <v>0.0580535</v>
@@ -14761,7 +14764,7 @@
         <v>0</v>
       </c>
       <c r="CS47" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="CT47">
         <v>-0.753715321</v>
@@ -14883,7 +14886,7 @@
         <v>0</v>
       </c>
       <c r="AM48" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN48">
         <v>0.056639031</v>
@@ -15048,7 +15051,7 @@
         <v>0</v>
       </c>
       <c r="CS48" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="CT48">
         <v>-0.71793867</v>
@@ -15170,7 +15173,7 @@
         <v>0</v>
       </c>
       <c r="AM49" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN49">
         <v>0.074241638</v>
@@ -15335,7 +15338,7 @@
         <v>0</v>
       </c>
       <c r="CS49" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="CT49">
         <v>-0.655169358</v>
@@ -15457,7 +15460,7 @@
         <v>0</v>
       </c>
       <c r="AM50" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN50">
         <v>0.05430774</v>
@@ -15622,7 +15625,7 @@
         <v>0</v>
       </c>
       <c r="CS50" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="CT50">
         <v>-0.6872439380000001</v>
@@ -15744,7 +15747,7 @@
         <v>0</v>
       </c>
       <c r="AM51" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN51">
         <v>0.080539377</v>
@@ -15909,7 +15912,7 @@
         <v>0</v>
       </c>
       <c r="CS51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="CT51">
         <v>-0.596275172</v>
@@ -16031,7 +16034,7 @@
         <v>0</v>
       </c>
       <c r="AM52" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN52">
         <v>0.032588051</v>
@@ -16196,7 +16199,7 @@
         <v>0</v>
       </c>
       <c r="CS52" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="CT52">
         <v>-0.808081961</v>
@@ -16318,7 +16321,7 @@
         <v>0</v>
       </c>
       <c r="AM53" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN53">
         <v>0.026475554</v>
@@ -16483,7 +16486,7 @@
         <v>0</v>
       </c>
       <c r="CS53" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="CT53">
         <v>-0.77227813</v>
@@ -16605,7 +16608,7 @@
         <v>0</v>
       </c>
       <c r="AM54" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN54">
         <v>0.0245106310926154</v>
@@ -16770,7 +16773,7 @@
         <v>0</v>
       </c>
       <c r="CS54" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="CT54">
         <v>-0.8664117478627688</v>
@@ -16889,7 +16892,7 @@
         <v>0</v>
       </c>
       <c r="AM55" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN55">
         <v>0.0779439577559576</v>
@@ -17054,7 +17057,7 @@
         <v>0</v>
       </c>
       <c r="CS55" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="CT55">
         <v>-0.7108907987632488</v>
@@ -17170,7 +17173,7 @@
         <v>0</v>
       </c>
       <c r="AM56" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN56">
         <v>0.0402740604837066</v>
@@ -17335,7 +17338,7 @@
         <v>0</v>
       </c>
       <c r="CS56" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="CT56">
         <v>-0.7447372903525753</v>
@@ -17448,7 +17451,7 @@
         <v>0</v>
       </c>
       <c r="AM57" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN57">
         <v>0.0441363962743036</v>
@@ -17613,7 +17616,7 @@
         <v>0</v>
       </c>
       <c r="CS57" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="CT57">
         <v>-0.7777179486581601</v>
@@ -17726,7 +17729,7 @@
         <v>0</v>
       </c>
       <c r="AM58" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN58">
         <v>0.0589646348207879</v>
@@ -17891,7 +17894,7 @@
         <v>0</v>
       </c>
       <c r="CS58" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="CT58">
         <v>-0.7757098341832183</v>
@@ -18004,7 +18007,7 @@
         <v>0</v>
       </c>
       <c r="AM59" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN59">
         <v>0.0088498418945465</v>
@@ -18169,7 +18172,7 @@
         <v>0</v>
       </c>
       <c r="CS59" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="CT59">
         <v>-0.9614802262041642</v>
@@ -18282,7 +18285,7 @@
         <v>0</v>
       </c>
       <c r="AM60" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN60">
         <v>0.0438527807624406</v>
@@ -18447,7 +18450,7 @@
         <v>0</v>
       </c>
       <c r="CS60" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="CT60">
         <v>-0.6569921650581255</v>
@@ -18560,7 +18563,7 @@
         <v>0</v>
       </c>
       <c r="AM61" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN61">
         <v>0.0175722673111926</v>
@@ -18725,7 +18728,7 @@
         <v>0</v>
       </c>
       <c r="CS61" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="CT61">
         <v>-0.924044412704054</v>
@@ -18838,7 +18841,7 @@
         <v>0</v>
       </c>
       <c r="AM62" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN62">
         <v>0.0551224625318549</v>
@@ -19003,7 +19006,7 @@
         <v>0</v>
       </c>
       <c r="CS62" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="CT62">
         <v>-0.6213262971882773</v>
@@ -19116,7 +19119,7 @@
         <v>0</v>
       </c>
       <c r="AM63" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN63">
         <v>0.0157574961492794</v>
@@ -19281,7 +19284,7 @@
         <v>0</v>
       </c>
       <c r="CS63" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="CT63">
         <v>-0.9477002142299265</v>
@@ -19394,7 +19397,7 @@
         <v>0</v>
       </c>
       <c r="AM64" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN64">
         <v>0.0348775184726272</v>
@@ -19559,7 +19562,7 @@
         <v>0</v>
       </c>
       <c r="CS64" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="CT64">
         <v>-0.7774025388699596</v>
@@ -19672,7 +19675,7 @@
         <v>0</v>
       </c>
       <c r="AM65" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN65">
         <v>0.0617007650932976</v>
@@ -19837,7 +19840,7 @@
         <v>0</v>
       </c>
       <c r="CS65" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="CT65">
         <v>-0.8140402180385446</v>
@@ -19950,7 +19953,7 @@
         <v>0.0108330657640134</v>
       </c>
       <c r="AM66" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN66">
         <v>0.0122896465671382</v>
@@ -20121,7 +20124,7 @@
         <v>28802806.1197283</v>
       </c>
       <c r="CS66" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="CT66">
         <v>-0.7661604887809055</v>
@@ -20234,7 +20237,7 @@
         <v>0.009662114019183699</v>
       </c>
       <c r="AM67" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN67">
         <v>0.0157075521173083</v>
@@ -20405,7 +20408,7 @@
         <v>12816652.38654842</v>
       </c>
       <c r="CS67" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="CT67">
         <v>-0.843107865610227</v>
@@ -20518,7 +20521,7 @@
         <v>0.009682496602030599</v>
       </c>
       <c r="AM68" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN68">
         <v>0.019453807476403</v>
@@ -20689,7 +20692,7 @@
         <v>362119.31393403</v>
       </c>
       <c r="CS68" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="CT68">
         <v>-0.7040504011377985</v>
@@ -20802,7 +20805,7 @@
         <v>0.009502809785555901</v>
       </c>
       <c r="AM69" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN69">
         <v>0.0467996269477206</v>
@@ -20973,7 +20976,7 @@
         <v>3444392.687119505</v>
       </c>
       <c r="CS69" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="CT69">
         <v>-0.5814104972412503</v>
@@ -21083,7 +21086,7 @@
         <v>0.0100375716524098</v>
       </c>
       <c r="AM70" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN70">
         <v>0.0260012684361012</v>
@@ -21254,7 +21257,7 @@
         <v>8020410.490554446</v>
       </c>
       <c r="CS70" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="CT70">
         <v>-0.1225754953154068</v>
@@ -21361,7 +21364,7 @@
         <v>0.0030270679524292</v>
       </c>
       <c r="AM71" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN71">
         <v>0.007629803458883</v>
@@ -21532,7 +21535,7 @@
         <v>6690404.196816532</v>
       </c>
       <c r="CS71" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="CT71">
         <v>-0.943556327266077</v>
@@ -21636,7 +21639,7 @@
         <v>0.0071318120684325</v>
       </c>
       <c r="AM72" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN72">
         <v>0.0106438024257861</v>
@@ -21807,7 +21810,7 @@
         <v>2333580.086114224</v>
       </c>
       <c r="CS72" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="CT72">
         <v>-0.9017649135974464</v>
@@ -21911,7 +21914,7 @@
         <v>0.008671749707596699</v>
       </c>
       <c r="AM73" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN73">
         <v>0.008922434565822699</v>
@@ -22082,7 +22085,7 @@
         <v>4050354.030474017</v>
       </c>
       <c r="CS73" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="CT73">
         <v>-0.9011542748767548</v>
@@ -22186,7 +22189,7 @@
         <v>0.0061287699408089</v>
       </c>
       <c r="AM74" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN74">
         <v>0.0100444206462455</v>
@@ -22357,7 +22360,7 @@
         <v>284228.7150822567</v>
       </c>
       <c r="CS74" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="CT74">
         <v>-0.9022640234515124</v>
@@ -22461,7 +22464,7 @@
         <v>0.009112086818146899</v>
       </c>
       <c r="AM75" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN75">
         <v>0.0105885988628848</v>
@@ -22632,7 +22635,7 @@
         <v>9238253.926865038</v>
       </c>
       <c r="CS75" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="CT75">
         <v>-0.8442464713130005</v>
@@ -22736,7 +22739,7 @@
         <v>0.0120332146147572</v>
       </c>
       <c r="AM76" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN76">
         <v>0.005689041712621</v>
@@ -22907,7 +22910,7 @@
         <v>103761437.1558867</v>
       </c>
       <c r="CS76" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="CT76">
         <v>-0.9172425776350784</v>
@@ -23011,7 +23014,7 @@
         <v>0.009980777925547499</v>
       </c>
       <c r="AM77" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN77">
         <v>0.0213191472253163</v>
@@ -23182,7 +23185,7 @@
         <v>11075597.03060125</v>
       </c>
       <c r="CS77" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="CT77">
         <v>-0.7048134977852135</v>
@@ -23283,7 +23286,7 @@
         <v>0.008640349693688199</v>
       </c>
       <c r="AM78" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN78">
         <v>0.0310379691662141</v>
@@ -23454,7 +23457,7 @@
         <v>4941591.885046311</v>
       </c>
       <c r="CS78" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="CT78">
         <v>-0.6921566954508142</v>
@@ -23555,7 +23558,7 @@
         <v>0.0052151469726826</v>
       </c>
       <c r="AM79" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN79">
         <v>0.0187749711217366</v>
@@ -23726,7 +23729,7 @@
         <v>13794144.77050867</v>
       </c>
       <c r="CS79" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="CT79">
         <v>-0.6546270123512354</v>
@@ -23827,7 +23830,7 @@
         <v>0.0083235819058295</v>
       </c>
       <c r="AM80" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN80">
         <v>0.0531066176371749</v>
@@ -23998,7 +24001,7 @@
         <v>1271425.087705649</v>
       </c>
       <c r="CS80" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="CT80">
         <v>-0.3384511866527668</v>
@@ -24099,7 +24102,7 @@
         <v>0.0041067346844988</v>
       </c>
       <c r="AM81" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN81">
         <v>0.0376358519870464</v>
@@ -24270,7 +24273,7 @@
         <v>8472790.733285822</v>
       </c>
       <c r="CS81" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="CT81">
         <v>-0.5869016106017596</v>
@@ -24371,7 +24374,7 @@
         <v>0.0055266741344329</v>
       </c>
       <c r="AM82" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN82">
         <v>0.0047447694558675</v>
@@ -24542,7 +24545,7 @@
         <v>6299784.652790904</v>
       </c>
       <c r="CS82" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="CT82">
         <v>-0.9571664073286058</v>
@@ -24643,7 +24646,7 @@
         <v>0.0083610158619657</v>
       </c>
       <c r="AM83" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN83">
         <v>0.0075895877096284</v>
@@ -24814,7 +24817,7 @@
         <v>9553962.229671104</v>
       </c>
       <c r="CS83" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="CT83">
         <v>-0.7975627900619038</v>
@@ -24915,7 +24918,7 @@
         <v>0.0110102665992773</v>
       </c>
       <c r="AM84" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN84">
         <v>0.0289129415567337</v>
@@ -25086,7 +25089,7 @@
         <v>9017755.465507764</v>
       </c>
       <c r="CS84" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="CT84">
         <v>-0.641321453686593</v>
@@ -25184,7 +25187,7 @@
         <v>0.001235474151197</v>
       </c>
       <c r="AM85" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN85">
         <v>0.0236860634403801</v>
@@ -25355,7 +25358,7 @@
         <v>395804.1998002621</v>
       </c>
       <c r="CS85" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="CT85">
         <v>-0.8468525619890503</v>
@@ -25453,7 +25456,7 @@
         <v>0.0069339646256509</v>
       </c>
       <c r="AM86" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN86">
         <v>0.0046798420774097</v>
@@ -25624,7 +25627,7 @@
         <v>5470308.140646266</v>
       </c>
       <c r="CS86" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="CT86">
         <v>-0.9414869172232342</v>
@@ -25722,7 +25725,7 @@
         <v>0.0084303895709902</v>
       </c>
       <c r="AM87" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN87">
         <v>0.0220548762227611</v>
@@ -25893,7 +25896,7 @@
         <v>10570112.91971009</v>
       </c>
       <c r="CS87" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="CT87">
         <v>-0.8207903291654746</v>
@@ -25991,7 +25994,7 @@
         <v>0.0046858616922062</v>
       </c>
       <c r="AM88" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN88">
         <v>0.0514935425696241</v>
@@ -26162,7 +26165,7 @@
         <v>5725644.496349121</v>
       </c>
       <c r="CS88" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="CT88">
         <v>-0.561712415905279</v>
@@ -26260,7 +26263,7 @@
         <v>0.0039939215766598</v>
       </c>
       <c r="AM89" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN89">
         <v>0.012222058764571</v>
@@ -26431,7 +26434,7 @@
         <v>1429804.32644608</v>
       </c>
       <c r="CS89" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="CT89">
         <v>-0.9176379634509604</v>
@@ -26529,7 +26532,7 @@
         <v>0.0042088758977745</v>
       </c>
       <c r="AM90" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN90">
         <v>0.019939030911244</v>
@@ -26700,7 +26703,7 @@
         <v>4722406.067514317</v>
       </c>
       <c r="CS90" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="CT90">
         <v>-0.9278452363120948</v>
@@ -26798,7 +26801,7 @@
         <v>0.0090603002679094</v>
       </c>
       <c r="AM91" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN91">
         <v>0.0130335524359802</v>
@@ -26969,7 +26972,7 @@
         <v>2899232.912138085</v>
       </c>
       <c r="CS91" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="CT91">
         <v>-0.8179686291978085</v>
@@ -27067,7 +27070,7 @@
         <v>0.0034278853232647</v>
       </c>
       <c r="AM92" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN92">
         <v>0.0267226315229668</v>
@@ -27238,7 +27241,7 @@
         <v>1448171.53934798</v>
       </c>
       <c r="CS92" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="CT92">
         <v>-0.8215150584575165</v>
@@ -27336,7 +27339,7 @@
         <v>0.0078801601208179</v>
       </c>
       <c r="AM93" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN93">
         <v>0.0221393128933173</v>
@@ -27507,7 +27510,7 @@
         <v>16635452.15900955</v>
       </c>
       <c r="CS93" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="CT93">
         <v>-0.7542388832888753</v>
@@ -27605,7 +27608,7 @@
         <v>0.0148358454007108</v>
       </c>
       <c r="AM94" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN94">
         <v>0.0142895129437342</v>
@@ -27776,7 +27779,7 @@
         <v>118847.66881</v>
       </c>
       <c r="CS94" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="CT94">
         <v>-0.8706219162560768</v>
@@ -27874,7 +27877,7 @@
         <v>0.00777307269066</v>
       </c>
       <c r="AM95" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN95">
         <v>0.028345432375321</v>
@@ -28045,7 +28048,7 @@
         <v>9989976.067409206</v>
       </c>
       <c r="CS95" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="CT95">
         <v>-0.7702665229627835</v>
@@ -28143,7 +28146,7 @@
         <v>0.005069566938105</v>
       </c>
       <c r="AM96" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN96">
         <v>0.0378882038525435</v>
@@ -28314,7 +28317,7 @@
         <v>4195010.116009732</v>
       </c>
       <c r="CS96" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="CT96">
         <v>-0.6208027078099908</v>
@@ -28412,7 +28415,7 @@
         <v>0.0109181034800677</v>
       </c>
       <c r="AM97" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN97">
         <v>0.0464479162381462</v>
@@ -28583,7 +28586,7 @@
         <v>1753546.300271091</v>
       </c>
       <c r="CS97" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="CT97">
         <v>-0.6637406607330143</v>
@@ -28681,7 +28684,7 @@
         <v>0.0073561352130028</v>
       </c>
       <c r="AM98" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN98">
         <v>0.0129973328606765</v>
@@ -28852,7 +28855,7 @@
         <v>8525723.260530123</v>
       </c>
       <c r="CS98" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="CT98">
         <v>-0.6066396906320848</v>
@@ -28950,7 +28953,7 @@
         <v>0.0010483764611907</v>
       </c>
       <c r="AM99" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN99">
         <v>0.0224095392580651</v>
@@ -29121,7 +29124,7 @@
         <v>555000.5818001842</v>
       </c>
       <c r="CS99" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="CT99">
         <v>-0.7930559623825889</v>
@@ -29219,7 +29222,7 @@
         <v>0.0034227206580065</v>
       </c>
       <c r="AM100" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN100">
         <v>0.0120356538583077</v>
@@ -29390,7 +29393,7 @@
         <v>8829982.660321526</v>
       </c>
       <c r="CS100" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="CT100">
         <v>-0.8625963918106255</v>
@@ -29488,7 +29491,7 @@
         <v>0.0024512168149686</v>
       </c>
       <c r="AM101" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN101">
         <v>0.0237148028402029</v>
@@ -29659,7 +29662,7 @@
         <v>3109464.939265249</v>
       </c>
       <c r="CS101" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="CT101">
         <v>-0.8320151516141147</v>
@@ -29757,7 +29760,7 @@
         <v>0.0013136523187938</v>
       </c>
       <c r="AM102" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN102">
         <v>0.0039597254802618</v>
@@ -29928,7 +29931,7 @@
         <v>1199182.410839436</v>
       </c>
       <c r="CS102" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="CT102">
         <v>-0.9034091343725908</v>
@@ -30026,7 +30029,7 @@
         <v>0.0026660229792492</v>
       </c>
       <c r="AM103" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN103">
         <v>0.0062754689148565</v>
@@ -30197,7 +30200,7 @@
         <v>5608278.16173986</v>
       </c>
       <c r="CS103" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="CT103">
         <v>-0.8495964311677586</v>
@@ -30295,7 +30298,7 @@
         <v>0.0095889911638783</v>
       </c>
       <c r="AM104" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN104">
         <v>0.0276610340172863</v>
@@ -30466,7 +30469,7 @@
         <v>16198187.75410762</v>
       </c>
       <c r="CS104" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="CT104">
         <v>-0.8581350323980486</v>
@@ -30564,7 +30567,7 @@
         <v>0.0090102837599302</v>
       </c>
       <c r="AM105" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN105">
         <v>0.0216087690726687</v>
@@ -30735,7 +30738,7 @@
         <v>10577375.81046865</v>
       </c>
       <c r="CS105" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="CT105">
         <v>-0.8842562871250494</v>
@@ -30833,7 +30836,7 @@
         <v>0.0050995967216395</v>
       </c>
       <c r="AM106" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN106">
         <v>0.0064663828879011</v>
@@ -31004,7 +31007,7 @@
         <v>8161103.390277231</v>
       </c>
       <c r="CS106" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="CT106">
         <v>-0.8751724322696175</v>
@@ -31102,7 +31105,7 @@
         <v>0.008368149950938699</v>
       </c>
       <c r="AM107" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN107">
         <v>0.0044562593205472</v>
@@ -31273,7 +31276,7 @@
         <v>8562542.046147738</v>
       </c>
       <c r="CS107" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="CT107">
         <v>-0.9169005340500024</v>
@@ -31371,7 +31374,7 @@
         <v>0.0065618399294816</v>
       </c>
       <c r="AM108" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN108">
         <v>0.0115970759513037</v>
@@ -31542,7 +31545,7 @@
         <v>5094802.189709073</v>
       </c>
       <c r="CS108" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="CT108">
         <v>-0.807087633056609</v>
@@ -31640,7 +31643,7 @@
         <v>0.0039283848188842</v>
       </c>
       <c r="AM109" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN109">
         <v>0.0506122383924143</v>
@@ -31811,7 +31814,7 @@
         <v>2688942.923710383</v>
       </c>
       <c r="CS109" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="CT109">
         <v>-0.6156032480827009</v>
@@ -31909,7 +31912,7 @@
         <v>0.0110575018573894</v>
       </c>
       <c r="AM110" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN110">
         <v>0.0182408073926103</v>
@@ -32080,7 +32083,7 @@
         <v>7113237.577421894</v>
       </c>
       <c r="CS110" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="CT110">
         <v>-0.7629790982692873</v>
@@ -32178,7 +32181,7 @@
         <v>0.0079211631943229</v>
       </c>
       <c r="AM111" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN111">
         <v>0.0160665598628607</v>
@@ -32349,7 +32352,7 @@
         <v>7296357.590261763</v>
       </c>
       <c r="CS111" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="CT111">
         <v>-0.8942723506201351</v>
@@ -32447,7 +32450,7 @@
         <v>0.0045682228774332</v>
       </c>
       <c r="AM112" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN112">
         <v>0.037886406926907</v>
@@ -32618,7 +32621,7 @@
         <v>646350.5069878154</v>
       </c>
       <c r="CS112" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="CT112">
         <v>-0.0916621825765546</v>
@@ -32716,7 +32719,7 @@
         <v>0.0103540243512939</v>
       </c>
       <c r="AM113" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN113">
         <v>0.0123420077084287</v>
@@ -32887,7 +32890,7 @@
         <v>16980708.42353759</v>
       </c>
       <c r="CS113" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="CT113">
         <v>-0.8006705745635164</v>
@@ -32985,7 +32988,7 @@
         <v>0.0064839021721033</v>
       </c>
       <c r="AM114" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN114">
         <v>0.0163921516174475</v>
@@ -33156,7 +33159,7 @@
         <v>778558.4127862654</v>
       </c>
       <c r="CS114" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="CT114">
         <v>-0.7935423347142916</v>
@@ -33254,7 +33257,7 @@
         <v>0.0115121978063762</v>
       </c>
       <c r="AM115" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN115">
         <v>0.0122833373375532</v>
@@ -33425,7 +33428,7 @@
         <v>22312718.74654885</v>
       </c>
       <c r="CS115" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="CT115">
         <v>-0.833943178203995</v>
@@ -33523,7 +33526,7 @@
         <v>0.0085575638145724</v>
       </c>
       <c r="AM116" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN116">
         <v>0.0253654749054445</v>
@@ -33694,7 +33697,7 @@
         <v>55051148.20247716</v>
       </c>
       <c r="CS116" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="CT116">
         <v>-0.7450076808546802</v>
@@ -33792,7 +33795,7 @@
         <v>0.0073550550024841</v>
       </c>
       <c r="AM117" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN117">
         <v>0.0189839179655455</v>
@@ -33963,7 +33966,7 @@
         <v>7593228.666961946</v>
       </c>
       <c r="CS117" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="CT117">
         <v>-0.5920454049159357</v>
@@ -34061,7 +34064,7 @@
         <v>0.0080994776472478</v>
       </c>
       <c r="AM118" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN118">
         <v>0.0067043103411634</v>
@@ -34232,7 +34235,7 @@
         <v>8613700.914603613</v>
       </c>
       <c r="CS118" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="CT118">
         <v>-0.9326775287918464</v>
@@ -34330,7 +34333,7 @@
         <v>0.0068550971234694</v>
       </c>
       <c r="AM119" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN119">
         <v>0.009392776226783601</v>
@@ -34501,7 +34504,7 @@
         <v>2380328.733367264</v>
       </c>
       <c r="CS119" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="CT119">
         <v>-0.955941339278515</v>
@@ -34599,7 +34602,7 @@
         <v>0.0038610240640448</v>
       </c>
       <c r="AM120" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN120">
         <v>0.0077083561528932</v>
@@ -34770,7 +34773,7 @@
         <v>872704.4135421006</v>
       </c>
       <c r="CS120" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="CT120">
         <v>-0.8980421674690441</v>
@@ -34868,7 +34871,7 @@
         <v>0.007825344507998084</v>
       </c>
       <c r="AM121" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN121">
         <v>0.03277088542105122</v>
@@ -35137,7 +35140,7 @@
         <v>0.005386378023791972</v>
       </c>
       <c r="AM122" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AN122">
         <v>0.03182171184361936</v>
@@ -35315,6 +35318,275 @@
       </c>
       <c r="CU122">
         <v>-0.8804699533217299</v>
+      </c>
+    </row>
+    <row r="123" spans="10:99">
+      <c r="J123" t="s">
+        <v>242</v>
+      </c>
+      <c r="K123">
+        <v>0.001785314458846887</v>
+      </c>
+      <c r="L123">
+        <v>0.0008926572294234436</v>
+      </c>
+      <c r="M123">
+        <v>0.0006467199131070522</v>
+      </c>
+      <c r="N123">
+        <v>0.0006467199131070522</v>
+      </c>
+      <c r="O123">
+        <v>0.0002396546589475745</v>
+      </c>
+      <c r="P123">
+        <v>0.0001198273294737873</v>
+      </c>
+      <c r="Q123">
+        <v>9.014839104724005E-05</v>
+      </c>
+      <c r="R123">
+        <v>9.014839104724005E-05</v>
+      </c>
+      <c r="S123">
+        <v>1.313013619352599</v>
+      </c>
+      <c r="T123">
+        <v>14.09869207916972</v>
+      </c>
+      <c r="U123">
+        <v>0.3708479406564303</v>
+      </c>
+      <c r="V123">
+        <v>0.6147942487421032</v>
+      </c>
+      <c r="W123">
+        <v>0.06019585150578459</v>
+      </c>
+      <c r="X123">
+        <v>0.08357693879873554</v>
+      </c>
+      <c r="Y123">
+        <v>0.2335240912364382</v>
+      </c>
+      <c r="Z123">
+        <v>0.2100276427291388</v>
+      </c>
+      <c r="AA123">
+        <v>1.000115767193069</v>
+      </c>
+      <c r="AB123">
+        <v>0.7870020448599038</v>
+      </c>
+      <c r="AC123">
+        <v>0.8226106454706089</v>
+      </c>
+      <c r="AD123">
+        <v>0.9990863121554732</v>
+      </c>
+      <c r="AE123">
+        <v>0.7658334593314265</v>
+      </c>
+      <c r="AF123">
+        <v>0.790095414307164</v>
+      </c>
+      <c r="AG123">
+        <v>0.008806131174539798</v>
+      </c>
+      <c r="AH123">
+        <v>0.008317099460099979</v>
+      </c>
+      <c r="AI123">
+        <v>1.000115767193069</v>
+      </c>
+      <c r="AJ123">
+        <v>0.9990863121554732</v>
+      </c>
+      <c r="AK123">
+        <v>0.008806131174539798</v>
+      </c>
+      <c r="AL123">
+        <v>0.008317099460099979</v>
+      </c>
+      <c r="AM123" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN123">
+        <v>0.04125443667646698</v>
+      </c>
+      <c r="AO123">
+        <v>0.02358191317826254</v>
+      </c>
+      <c r="AP123">
+        <v>-2391.81231976</v>
+      </c>
+      <c r="AQ123">
+        <v>-497.64963618</v>
+      </c>
+      <c r="AR123">
+        <v>68643.83088023993</v>
+      </c>
+      <c r="AS123">
+        <v>20101.40886382014</v>
+      </c>
+      <c r="AT123">
+        <v>68791.42288023993</v>
+      </c>
+      <c r="AU123">
+        <v>20101.40886382014</v>
+      </c>
+      <c r="AV123">
+        <v>5.864383088023993</v>
+      </c>
+      <c r="AW123">
+        <v>1.010140886382013</v>
+      </c>
+      <c r="AX123">
+        <v>11.34508350976241</v>
+      </c>
+      <c r="AY123">
+        <v>1.055588396278051</v>
+      </c>
+      <c r="AZ123">
+        <v>349.8833333333333</v>
+      </c>
+      <c r="BA123">
+        <v>67.5</v>
+      </c>
+      <c r="BB123">
+        <v>1.518081002546836E-05</v>
+      </c>
+      <c r="BC123">
+        <v>0.1469929822054601</v>
+      </c>
+      <c r="BD123">
+        <v>-0.926584570505808</v>
+      </c>
+      <c r="BE123">
+        <v>-1826.464712463123</v>
+      </c>
+      <c r="BF123">
+        <v>650</v>
+      </c>
+      <c r="BG123">
+        <v>4495</v>
+      </c>
+      <c r="BH123">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI123">
+        <v>768</v>
+      </c>
+      <c r="BJ123">
+        <v>10731</v>
+      </c>
+      <c r="BK123">
+        <v>1418</v>
+      </c>
+      <c r="BL123">
+        <v>15226</v>
+      </c>
+      <c r="BM123">
+        <v>647</v>
+      </c>
+      <c r="BN123">
+        <v>4449</v>
+      </c>
+      <c r="BO123">
+        <v>648</v>
+      </c>
+      <c r="BP123">
+        <v>4455</v>
+      </c>
+      <c r="BQ123">
+        <v>121</v>
+      </c>
+      <c r="BR123">
+        <v>6282</v>
+      </c>
+      <c r="BS123">
+        <v>2</v>
+      </c>
+      <c r="BT123">
+        <v>40</v>
+      </c>
+      <c r="BU123">
+        <v>0</v>
+      </c>
+      <c r="BV123">
+        <v>0</v>
+      </c>
+      <c r="BW123">
+        <v>58643.83088024005</v>
+      </c>
+      <c r="BX123">
+        <v>10101.40886382</v>
+      </c>
+      <c r="BY123">
+        <v>0.05224686226551298</v>
+      </c>
+      <c r="BZ123">
+        <v>0.06786443963120219</v>
+      </c>
+      <c r="CA123">
+        <v>0.132584003710414</v>
+      </c>
+      <c r="CB123">
+        <v>0.1734711724531849</v>
+      </c>
+      <c r="CC123">
+        <v>0.01411464095025058</v>
+      </c>
+      <c r="CD123">
+        <v>0.01222143382320495</v>
+      </c>
+      <c r="CE123">
+        <v>0.007342535571779663</v>
+      </c>
+      <c r="CF123">
+        <v>0.01136365030126063</v>
+      </c>
+      <c r="CG123">
+        <v>61035.64320000005</v>
+      </c>
+      <c r="CH123">
+        <v>10599.0585</v>
+      </c>
+      <c r="CI123">
+        <v>61036.56978457056</v>
+      </c>
+      <c r="CJ123">
+        <v>12425.52321246312</v>
+      </c>
+      <c r="CK123">
+        <v>0.1773553872875359</v>
+      </c>
+      <c r="CL123">
+        <v>0.06087146872493719</v>
+      </c>
+      <c r="CM123">
+        <v>10000</v>
+      </c>
+      <c r="CO123">
+        <v>0.005671296296296297</v>
+      </c>
+      <c r="CP123">
+        <v>0.008371913580246913</v>
+      </c>
+      <c r="CQ123">
+        <v>7291912.694569973</v>
+      </c>
+      <c r="CR123">
+        <v>7884481.26725769</v>
+      </c>
+      <c r="CS123" s="2">
+        <v>45414.72426311563</v>
+      </c>
+      <c r="CT123">
+        <v>-0.7831546722232047</v>
+      </c>
+      <c r="CU123">
+        <v>-0.680300068663037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update THETAUSDT.json at 2024-05-03_06-34-53 bestfile_scores 0.0011774354556709971 bestfile_sharp 0.05424559650284209
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="362">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1461,7 +1461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU123"/>
+  <dimension ref="A1:CU124"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -35587,6 +35587,275 @@
       </c>
       <c r="CU123">
         <v>-0.680300068663037</v>
+      </c>
+    </row>
+    <row r="124" spans="10:99">
+      <c r="J124" t="s">
+        <v>205</v>
+      </c>
+      <c r="K124">
+        <v>0.001296366046547259</v>
+      </c>
+      <c r="L124">
+        <v>0.0006481830232736296</v>
+      </c>
+      <c r="M124">
+        <v>0.001294169521785848</v>
+      </c>
+      <c r="N124">
+        <v>0.001294169521785848</v>
+      </c>
+      <c r="O124">
+        <v>0.002017927231782202</v>
+      </c>
+      <c r="P124">
+        <v>0.001008963615891101</v>
+      </c>
+      <c r="Q124">
+        <v>0.001388756262576618</v>
+      </c>
+      <c r="R124">
+        <v>0.001388756262576618</v>
+      </c>
+      <c r="S124">
+        <v>13.08312903944729</v>
+      </c>
+      <c r="T124">
+        <v>24.80231780699799</v>
+      </c>
+      <c r="U124">
+        <v>0.4088247325637866</v>
+      </c>
+      <c r="V124">
+        <v>0.7881816830606417</v>
+      </c>
+      <c r="W124">
+        <v>0.09870847566697016</v>
+      </c>
+      <c r="X124">
+        <v>0.03399379553683892</v>
+      </c>
+      <c r="Y124">
+        <v>0.2025773374631408</v>
+      </c>
+      <c r="Z124">
+        <v>0.09521239980310614</v>
+      </c>
+      <c r="AA124">
+        <v>0.9971077765755076</v>
+      </c>
+      <c r="AB124">
+        <v>0.8327013213607222</v>
+      </c>
+      <c r="AC124">
+        <v>0.9313896181416321</v>
+      </c>
+      <c r="AD124">
+        <v>0.9995397866079424</v>
+      </c>
+      <c r="AE124">
+        <v>0.7993344529087333</v>
+      </c>
+      <c r="AF124">
+        <v>0.9049529935275081</v>
+      </c>
+      <c r="AG124">
+        <v>0.01112370496280496</v>
+      </c>
+      <c r="AH124">
+        <v>0.003241839375530565</v>
+      </c>
+      <c r="AI124">
+        <v>0.9971077765755076</v>
+      </c>
+      <c r="AJ124">
+        <v>0.9995397866079424</v>
+      </c>
+      <c r="AK124">
+        <v>0.01112370496280496</v>
+      </c>
+      <c r="AL124">
+        <v>0.003241839375530565</v>
+      </c>
+      <c r="AM124" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN124">
+        <v>0.0499292345312228</v>
+      </c>
+      <c r="AO124">
+        <v>0.02696095414200189</v>
+      </c>
+      <c r="AP124">
+        <v>-1069.132693214</v>
+      </c>
+      <c r="AQ124">
+        <v>-767.802456396</v>
+      </c>
+      <c r="AR124">
+        <v>20680.96088132593</v>
+      </c>
+      <c r="AS124">
+        <v>20655.53104360435</v>
+      </c>
+      <c r="AT124">
+        <v>20680.25978132593</v>
+      </c>
+      <c r="AU124">
+        <v>20652.36094360435</v>
+      </c>
+      <c r="AV124">
+        <v>1.068096088132593</v>
+      </c>
+      <c r="AW124">
+        <v>1.065553104360435</v>
+      </c>
+      <c r="AX124">
+        <v>1.829928217709327</v>
+      </c>
+      <c r="AY124">
+        <v>0.9663467529355381</v>
+      </c>
+      <c r="AZ124">
+        <v>117.0333333333333</v>
+      </c>
+      <c r="BA124">
+        <v>49.15</v>
+      </c>
+      <c r="BB124">
+        <v>0.06548780083544982</v>
+      </c>
+      <c r="BC124">
+        <v>0.0590359085568859</v>
+      </c>
+      <c r="BD124">
+        <v>-823.6252625158032</v>
+      </c>
+      <c r="BE124">
+        <v>-716.6977763057191</v>
+      </c>
+      <c r="BF124">
+        <v>3532</v>
+      </c>
+      <c r="BG124">
+        <v>5904</v>
+      </c>
+      <c r="BH124">
+        <v>560.875</v>
+      </c>
+      <c r="BI124">
+        <v>3806</v>
+      </c>
+      <c r="BJ124">
+        <v>8007</v>
+      </c>
+      <c r="BK124">
+        <v>7338</v>
+      </c>
+      <c r="BL124">
+        <v>13911</v>
+      </c>
+      <c r="BM124">
+        <v>3369</v>
+      </c>
+      <c r="BN124">
+        <v>5761</v>
+      </c>
+      <c r="BO124">
+        <v>3503</v>
+      </c>
+      <c r="BP124">
+        <v>5815</v>
+      </c>
+      <c r="BQ124">
+        <v>437</v>
+      </c>
+      <c r="BR124">
+        <v>2246</v>
+      </c>
+      <c r="BS124">
+        <v>29</v>
+      </c>
+      <c r="BT124">
+        <v>89</v>
+      </c>
+      <c r="BU124">
+        <v>0</v>
+      </c>
+      <c r="BV124">
+        <v>0</v>
+      </c>
+      <c r="BW124">
+        <v>10684.01591678599</v>
+      </c>
+      <c r="BX124">
+        <v>10655.531043604</v>
+      </c>
+      <c r="BY124">
+        <v>0.07166894429972837</v>
+      </c>
+      <c r="BZ124">
+        <v>0.03522008980499606</v>
+      </c>
+      <c r="CA124">
+        <v>0.1114915290739781</v>
+      </c>
+      <c r="CB124">
+        <v>0.08678444205212817</v>
+      </c>
+      <c r="CC124">
+        <v>0.01858384506952434</v>
+      </c>
+      <c r="CD124">
+        <v>0.009105693921035841</v>
+      </c>
+      <c r="CE124">
+        <v>0.01381502710228896</v>
+      </c>
+      <c r="CF124">
+        <v>0.006640182413336976</v>
+      </c>
+      <c r="CG124">
+        <v>11753.14860999999</v>
+      </c>
+      <c r="CH124">
+        <v>11423.3335</v>
+      </c>
+      <c r="CI124">
+        <v>12576.77387251579</v>
+      </c>
+      <c r="CJ124">
+        <v>12140.03127630572</v>
+      </c>
+      <c r="CK124">
+        <v>0.1232345957418265</v>
+      </c>
+      <c r="CL124">
+        <v>0.259391251439734</v>
+      </c>
+      <c r="CM124">
+        <v>10000</v>
+      </c>
+      <c r="CO124">
+        <v>0.008319714752637052</v>
+      </c>
+      <c r="CP124">
+        <v>0.005496954390135195</v>
+      </c>
+      <c r="CQ124">
+        <v>4940876.349740313</v>
+      </c>
+      <c r="CR124">
+        <v>4199685.074142367</v>
+      </c>
+      <c r="CS124" s="2">
+        <v>45414.85936401004</v>
+      </c>
+      <c r="CT124">
+        <v>-0.7053510752114568</v>
+      </c>
+      <c r="CU124">
+        <v>-0.8831403389490625</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update UNIUSDT.json at 2024-05-03_11-06-17 bestfile_scores 0.0006006963246286051 bestfile_sharp 0.19062790724995132
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1100,6 +1100,18 @@
   </si>
   <si>
     <t>2024-05-01 20:27:05.950210</t>
+  </si>
+  <si>
+    <t>2024-05-02 06:24:58.447368</t>
+  </si>
+  <si>
+    <t>2024-05-02 12:52:43.677062</t>
+  </si>
+  <si>
+    <t>2024-05-02 17:22:56.333191</t>
+  </si>
+  <si>
+    <t>2024-05-02 20:37:29.050468</t>
   </si>
 </sst>
 </file>
@@ -1461,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU124"/>
+  <dimension ref="A1:CU125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -32591,7 +32603,7 @@
         <v>373133.5807200004</v>
       </c>
       <c r="CH112">
-        <v>1892.879620000002</v>
+        <v>1892.879620000001</v>
       </c>
       <c r="CI112">
         <v>373730.1845249833</v>
@@ -34787,28 +34799,28 @@
         <v>219</v>
       </c>
       <c r="K121">
-        <v>0.001287317064583293</v>
+        <v>0.0012873170645832</v>
       </c>
       <c r="L121">
-        <v>0.0006436585322916466</v>
+        <v>0.0006436585322916</v>
       </c>
       <c r="M121">
-        <v>0.0006799091577396332</v>
+        <v>0.0006799091577396001</v>
       </c>
       <c r="N121">
-        <v>0.0006799091577396332</v>
+        <v>0.0006799091577396001</v>
       </c>
       <c r="O121">
-        <v>0.0009902915176535298</v>
+        <v>0.0009902915176535001</v>
       </c>
       <c r="P121">
-        <v>0.0004951457588267649</v>
+        <v>0.0004951457588267</v>
       </c>
       <c r="Q121">
-        <v>0.0006339568585719713</v>
+        <v>0.0006339568585719</v>
       </c>
       <c r="R121">
-        <v>0.0006339568585719713</v>
+        <v>0.0006339568585719</v>
       </c>
       <c r="S121">
         <v>21.97953272832593</v>
@@ -34823,10 +34835,10 @@
         <v>0.6389886006561238</v>
       </c>
       <c r="W121">
-        <v>0.08195591941729946</v>
+        <v>0.08195591941729941</v>
       </c>
       <c r="X121">
-        <v>0.06670474817370561</v>
+        <v>0.0667047481737056</v>
       </c>
       <c r="Y121">
         <v>0.2498599487734504</v>
@@ -34835,7 +34847,7 @@
         <v>0.2061626732634882</v>
       </c>
       <c r="AA121">
-        <v>0.9983439768090353</v>
+        <v>0.9983439768090352</v>
       </c>
       <c r="AB121">
         <v>0.7797450068714336</v>
@@ -34844,7 +34856,7 @@
         <v>0.8256733722696264</v>
       </c>
       <c r="AD121">
-        <v>0.9988193430591729</v>
+        <v>0.9988193430591727</v>
       </c>
       <c r="AE121">
         <v>0.5977027100792138</v>
@@ -34853,28 +34865,28 @@
         <v>0.793993084219069</v>
       </c>
       <c r="AG121">
-        <v>0.008944569579459443</v>
+        <v>0.0089445695794594</v>
       </c>
       <c r="AH121">
-        <v>0.007825344507998084</v>
+        <v>0.007825344507997999</v>
       </c>
       <c r="AI121">
-        <v>0.9983439768090353</v>
+        <v>0.9983439768090352</v>
       </c>
       <c r="AJ121">
-        <v>0.9988193430591729</v>
+        <v>0.9988193430591727</v>
       </c>
       <c r="AK121">
-        <v>0.008944569579459443</v>
+        <v>0.0089445695794594</v>
       </c>
       <c r="AL121">
-        <v>0.007825344507998084</v>
+        <v>0.007825344507997999</v>
       </c>
       <c r="AM121" t="s">
         <v>243</v>
       </c>
       <c r="AN121">
-        <v>0.03277088542105122</v>
+        <v>0.0327708854210512</v>
       </c>
       <c r="AO121">
         <v>0.0431808012405876</v>
@@ -34889,7 +34901,7 @@
         <v>40071.01748765797</v>
       </c>
       <c r="AS121">
-        <v>20820.32075378027</v>
+        <v>20820.32075378028</v>
       </c>
       <c r="AT121">
         <v>40068.48348765797</v>
@@ -34916,10 +34928,10 @@
         <v>63.08333333333334</v>
       </c>
       <c r="BB121">
-        <v>0.06268979707003425</v>
+        <v>0.06268979707003421</v>
       </c>
       <c r="BC121">
-        <v>0.02630327241826978</v>
+        <v>0.0263032724182697</v>
       </c>
       <c r="BD121">
         <v>-2140.823386776186</v>
@@ -34985,10 +34997,10 @@
         <v>10822.43945418001</v>
       </c>
       <c r="BY121">
-        <v>0.07013149967937063</v>
+        <v>0.0701314996793706</v>
       </c>
       <c r="BZ121">
-        <v>0.06787028640737212</v>
+        <v>0.0678702864073721</v>
       </c>
       <c r="CA121">
         <v>0.1570542719009034</v>
@@ -34997,19 +35009,19 @@
         <v>0.1707999223242642</v>
       </c>
       <c r="CC121">
-        <v>0.01008427941720721</v>
+        <v>0.0100842794172072</v>
       </c>
       <c r="CD121">
-        <v>0.008914617079175888</v>
+        <v>0.008914617079175799</v>
       </c>
       <c r="CE121">
-        <v>0.00984779131712857</v>
+        <v>0.0098477913171285</v>
       </c>
       <c r="CF121">
-        <v>0.009664114879300885</v>
+        <v>0.0096641148793008</v>
       </c>
       <c r="CG121">
-        <v>32008.64729000003</v>
+        <v>32008.64729000004</v>
       </c>
       <c r="CH121">
         <v>12317.16710000001</v>
@@ -35021,28 +35033,28 @@
         <v>12649.90088915147</v>
       </c>
       <c r="CK121">
-        <v>0.08236456576079598</v>
+        <v>0.0823645657607959</v>
       </c>
       <c r="CL121">
-        <v>0.09050962913854409</v>
+        <v>0.090509629138544</v>
       </c>
       <c r="CM121">
         <v>10000</v>
       </c>
       <c r="CO121">
-        <v>0.0009654000617856039</v>
+        <v>0.0009654000617856</v>
       </c>
       <c r="CP121">
-        <v>0.01625733704046957</v>
+        <v>0.0162573370404695</v>
       </c>
       <c r="CQ121">
-        <v>24126158.54265907</v>
+        <v>24126158.54265908</v>
       </c>
       <c r="CR121">
         <v>10271258.08902804</v>
       </c>
-      <c r="CS121" s="2">
-        <v>45414.26734314083</v>
+      <c r="CS121" t="s">
+        <v>362</v>
       </c>
       <c r="CT121">
         <v>-0.7644558396778582</v>
@@ -35056,28 +35068,28 @@
         <v>236</v>
       </c>
       <c r="K122">
-        <v>0.001728903964315354</v>
+        <v>0.0017289039643153</v>
       </c>
       <c r="L122">
-        <v>0.0008644519821576768</v>
+        <v>0.0008644519821576</v>
       </c>
       <c r="M122">
-        <v>0.0004287261639606132</v>
+        <v>0.0004287261639606</v>
       </c>
       <c r="N122">
-        <v>0.0004287261639606132</v>
+        <v>0.0004287261639606</v>
       </c>
       <c r="O122">
-        <v>0.001908969392300564</v>
+        <v>0.0019089693923005</v>
       </c>
       <c r="P122">
-        <v>0.0009544846961502818</v>
+        <v>0.0009544846961502</v>
       </c>
       <c r="Q122">
-        <v>0.0003620626646210434</v>
+        <v>0.000362062664621</v>
       </c>
       <c r="R122">
-        <v>0.0003620626646210434</v>
+        <v>0.000362062664621</v>
       </c>
       <c r="S122">
         <v>15.5826221278239</v>
@@ -35086,22 +35098,22 @@
         <v>41.69391774473837</v>
       </c>
       <c r="U122">
-        <v>0.4040347838832489</v>
+        <v>0.4040347838832488</v>
       </c>
       <c r="V122">
         <v>1</v>
       </c>
       <c r="W122">
-        <v>0.06714253843568732</v>
+        <v>0.06714253843568729</v>
       </c>
       <c r="X122">
-        <v>0.04289001470941213</v>
+        <v>0.0428900147094121</v>
       </c>
       <c r="Y122">
-        <v>0.1837206490800225</v>
+        <v>0.1837206490800224</v>
       </c>
       <c r="Z122">
-        <v>0.09944049512904625</v>
+        <v>0.09944049512904619</v>
       </c>
       <c r="AA122">
         <v>0.998836257784695</v>
@@ -35110,7 +35122,7 @@
         <v>0.8393340151777245</v>
       </c>
       <c r="AC122">
-        <v>0.9199713071139491</v>
+        <v>0.9199713071139493</v>
       </c>
       <c r="AD122">
         <v>0.9985371762155364</v>
@@ -35122,10 +35134,10 @@
         <v>0.9006492048194443</v>
       </c>
       <c r="AG122">
-        <v>0.007722970938455328</v>
+        <v>0.0077229709384553</v>
       </c>
       <c r="AH122">
-        <v>0.005386378023791972</v>
+        <v>0.0053863780237919</v>
       </c>
       <c r="AI122">
         <v>0.998836257784695</v>
@@ -35134,19 +35146,19 @@
         <v>0.9985371762155364</v>
       </c>
       <c r="AK122">
-        <v>0.007722970938455328</v>
+        <v>0.0077229709384553</v>
       </c>
       <c r="AL122">
-        <v>0.005386378023791972</v>
+        <v>0.0053863780237919</v>
       </c>
       <c r="AM122" t="s">
         <v>243</v>
       </c>
       <c r="AN122">
-        <v>0.03182171184361936</v>
+        <v>0.0318217118436193</v>
       </c>
       <c r="AO122">
-        <v>0.04398480244716741</v>
+        <v>0.0439848024471674</v>
       </c>
       <c r="AP122">
         <v>-3661.709861474</v>
@@ -35185,7 +35197,7 @@
         <v>118.8166666666667</v>
       </c>
       <c r="BB122">
-        <v>0.002892679559724969</v>
+        <v>0.0028926795597249</v>
       </c>
       <c r="BC122">
         <v>0</v>
@@ -35254,28 +35266,28 @@
         <v>5880.050391392</v>
       </c>
       <c r="BY122">
-        <v>0.04021654892013991</v>
+        <v>0.0402165489201399</v>
       </c>
       <c r="BZ122">
-        <v>0.08614027692450116</v>
+        <v>0.0861402769245011</v>
       </c>
       <c r="CA122">
-        <v>0.1009521388215714</v>
+        <v>0.1009521388215713</v>
       </c>
       <c r="CB122">
         <v>0.1329467250439504</v>
       </c>
       <c r="CC122">
-        <v>0.009288235855895425</v>
+        <v>0.0092882358558954</v>
       </c>
       <c r="CD122">
         <v>0.0110460773745595</v>
       </c>
       <c r="CE122">
-        <v>0.007931947135435472</v>
+        <v>0.007931947135435401</v>
       </c>
       <c r="CF122">
-        <v>0.01393756865436849</v>
+        <v>0.0139375686543684</v>
       </c>
       <c r="CG122">
         <v>58143.94276999991</v>
@@ -35293,13 +35305,13 @@
         <v>0.2023433174016643</v>
       </c>
       <c r="CL122">
-        <v>0.07165289775989087</v>
+        <v>0.0716528977598908</v>
       </c>
       <c r="CM122">
         <v>10000</v>
       </c>
       <c r="CO122">
-        <v>0.00892029657089898</v>
+        <v>0.008920296570898901</v>
       </c>
       <c r="CP122">
         <v>0</v>
@@ -35310,8 +35322,8 @@
       <c r="CR122">
         <v>4219262.028734344</v>
       </c>
-      <c r="CS122" s="2">
-        <v>45414.53661663266</v>
+      <c r="CS122" t="s">
+        <v>363</v>
       </c>
       <c r="CT122">
         <v>-0.7390744315992817</v>
@@ -35325,22 +35337,22 @@
         <v>242</v>
       </c>
       <c r="K123">
-        <v>0.001785314458846887</v>
+        <v>0.0017853144588468</v>
       </c>
       <c r="L123">
-        <v>0.0008926572294234436</v>
+        <v>0.0008926572294234</v>
       </c>
       <c r="M123">
-        <v>0.0006467199131070522</v>
+        <v>0.000646719913107</v>
       </c>
       <c r="N123">
-        <v>0.0006467199131070522</v>
+        <v>0.000646719913107</v>
       </c>
       <c r="O123">
-        <v>0.0002396546589475745</v>
+        <v>0.0002396546589475</v>
       </c>
       <c r="P123">
-        <v>0.0001198273294737873</v>
+        <v>0.0001198273294737</v>
       </c>
       <c r="Q123">
         <v>9.014839104724005E-05</v>
@@ -35349,7 +35361,7 @@
         <v>9.014839104724005E-05</v>
       </c>
       <c r="S123">
-        <v>1.313013619352599</v>
+        <v>1.313013619352598</v>
       </c>
       <c r="T123">
         <v>14.09869207916972</v>
@@ -35361,16 +35373,16 @@
         <v>0.6147942487421032</v>
       </c>
       <c r="W123">
-        <v>0.06019585150578459</v>
+        <v>0.0601958515057845</v>
       </c>
       <c r="X123">
-        <v>0.08357693879873554</v>
+        <v>0.0835769387987355</v>
       </c>
       <c r="Y123">
         <v>0.2335240912364382</v>
       </c>
       <c r="Z123">
-        <v>0.2100276427291388</v>
+        <v>0.2100276427291387</v>
       </c>
       <c r="AA123">
         <v>1.000115767193069</v>
@@ -35391,10 +35403,10 @@
         <v>0.790095414307164</v>
       </c>
       <c r="AG123">
-        <v>0.008806131174539798</v>
+        <v>0.0088061311745397</v>
       </c>
       <c r="AH123">
-        <v>0.008317099460099979</v>
+        <v>0.008317099460099901</v>
       </c>
       <c r="AI123">
         <v>1.000115767193069</v>
@@ -35403,19 +35415,19 @@
         <v>0.9990863121554732</v>
       </c>
       <c r="AK123">
-        <v>0.008806131174539798</v>
+        <v>0.0088061311745397</v>
       </c>
       <c r="AL123">
-        <v>0.008317099460099979</v>
+        <v>0.008317099460099901</v>
       </c>
       <c r="AM123" t="s">
         <v>243</v>
       </c>
       <c r="AN123">
-        <v>0.04125443667646698</v>
+        <v>0.0412544366764669</v>
       </c>
       <c r="AO123">
-        <v>0.02358191317826254</v>
+        <v>0.0235819131782625</v>
       </c>
       <c r="AP123">
         <v>-2391.81231976</v>
@@ -35445,7 +35457,7 @@
         <v>11.34508350976241</v>
       </c>
       <c r="AY123">
-        <v>1.055588396278051</v>
+        <v>1.055588396278052</v>
       </c>
       <c r="AZ123">
         <v>349.8833333333333</v>
@@ -35523,28 +35535,28 @@
         <v>10101.40886382</v>
       </c>
       <c r="BY123">
-        <v>0.05224686226551298</v>
+        <v>0.0522468622655129</v>
       </c>
       <c r="BZ123">
-        <v>0.06786443963120219</v>
+        <v>0.0678644396312021</v>
       </c>
       <c r="CA123">
-        <v>0.132584003710414</v>
+        <v>0.1325840037104139</v>
       </c>
       <c r="CB123">
         <v>0.1734711724531849</v>
       </c>
       <c r="CC123">
-        <v>0.01411464095025058</v>
+        <v>0.0141146409502505</v>
       </c>
       <c r="CD123">
-        <v>0.01222143382320495</v>
+        <v>0.0122214338232049</v>
       </c>
       <c r="CE123">
-        <v>0.007342535571779663</v>
+        <v>0.0073425355717796</v>
       </c>
       <c r="CF123">
-        <v>0.01136365030126063</v>
+        <v>0.0113636503012606</v>
       </c>
       <c r="CG123">
         <v>61035.64320000005</v>
@@ -35559,19 +35571,19 @@
         <v>12425.52321246312</v>
       </c>
       <c r="CK123">
-        <v>0.1773553872875359</v>
+        <v>0.1773553872875358</v>
       </c>
       <c r="CL123">
-        <v>0.06087146872493719</v>
+        <v>0.0608714687249371</v>
       </c>
       <c r="CM123">
         <v>10000</v>
       </c>
       <c r="CO123">
-        <v>0.005671296296296297</v>
+        <v>0.0056712962962962</v>
       </c>
       <c r="CP123">
-        <v>0.008371913580246913</v>
+        <v>0.008371913580246901</v>
       </c>
       <c r="CQ123">
         <v>7291912.694569973</v>
@@ -35579,8 +35591,8 @@
       <c r="CR123">
         <v>7884481.26725769</v>
       </c>
-      <c r="CS123" s="2">
-        <v>45414.72426311563</v>
+      <c r="CS123" t="s">
+        <v>364</v>
       </c>
       <c r="CT123">
         <v>-0.7831546722232047</v>
@@ -35594,34 +35606,34 @@
         <v>205</v>
       </c>
       <c r="K124">
-        <v>0.001296366046547259</v>
+        <v>0.0012963660465472</v>
       </c>
       <c r="L124">
-        <v>0.0006481830232736296</v>
+        <v>0.0006481830232736</v>
       </c>
       <c r="M124">
-        <v>0.001294169521785848</v>
+        <v>0.0012941695217858</v>
       </c>
       <c r="N124">
-        <v>0.001294169521785848</v>
+        <v>0.0012941695217858</v>
       </c>
       <c r="O124">
-        <v>0.002017927231782202</v>
+        <v>0.0020179272317822</v>
       </c>
       <c r="P124">
-        <v>0.001008963615891101</v>
+        <v>0.0010089636158911</v>
       </c>
       <c r="Q124">
-        <v>0.001388756262576618</v>
+        <v>0.0013887562625766</v>
       </c>
       <c r="R124">
-        <v>0.001388756262576618</v>
+        <v>0.0013887562625766</v>
       </c>
       <c r="S124">
         <v>13.08312903944729</v>
       </c>
       <c r="T124">
-        <v>24.80231780699799</v>
+        <v>24.802317806998</v>
       </c>
       <c r="U124">
         <v>0.4088247325637866</v>
@@ -35630,16 +35642,16 @@
         <v>0.7881816830606417</v>
       </c>
       <c r="W124">
-        <v>0.09870847566697016</v>
+        <v>0.09870847566697009</v>
       </c>
       <c r="X124">
-        <v>0.03399379553683892</v>
+        <v>0.0339937955368389</v>
       </c>
       <c r="Y124">
         <v>0.2025773374631408</v>
       </c>
       <c r="Z124">
-        <v>0.09521239980310614</v>
+        <v>0.0952123998031061</v>
       </c>
       <c r="AA124">
         <v>0.9971077765755076</v>
@@ -35648,7 +35660,7 @@
         <v>0.8327013213607222</v>
       </c>
       <c r="AC124">
-        <v>0.9313896181416321</v>
+        <v>0.931389618141632</v>
       </c>
       <c r="AD124">
         <v>0.9995397866079424</v>
@@ -35657,13 +35669,13 @@
         <v>0.7993344529087333</v>
       </c>
       <c r="AF124">
-        <v>0.9049529935275081</v>
+        <v>0.904952993527508</v>
       </c>
       <c r="AG124">
-        <v>0.01112370496280496</v>
+        <v>0.0111237049628049</v>
       </c>
       <c r="AH124">
-        <v>0.003241839375530565</v>
+        <v>0.0032418393755305</v>
       </c>
       <c r="AI124">
         <v>0.9971077765755076</v>
@@ -35672,10 +35684,10 @@
         <v>0.9995397866079424</v>
       </c>
       <c r="AK124">
-        <v>0.01112370496280496</v>
+        <v>0.0111237049628049</v>
       </c>
       <c r="AL124">
-        <v>0.003241839375530565</v>
+        <v>0.0032418393755305</v>
       </c>
       <c r="AM124" t="s">
         <v>243</v>
@@ -35684,7 +35696,7 @@
         <v>0.0499292345312228</v>
       </c>
       <c r="AO124">
-        <v>0.02696095414200189</v>
+        <v>0.0269609541420018</v>
       </c>
       <c r="AP124">
         <v>-1069.132693214</v>
@@ -35714,7 +35726,7 @@
         <v>1.829928217709327</v>
       </c>
       <c r="AY124">
-        <v>0.9663467529355381</v>
+        <v>0.966346752935538</v>
       </c>
       <c r="AZ124">
         <v>117.0333333333333</v>
@@ -35723,7 +35735,7 @@
         <v>49.15</v>
       </c>
       <c r="BB124">
-        <v>0.06548780083544982</v>
+        <v>0.06548780083544981</v>
       </c>
       <c r="BC124">
         <v>0.0590359085568859</v>
@@ -35792,28 +35804,28 @@
         <v>10655.531043604</v>
       </c>
       <c r="BY124">
-        <v>0.07166894429972837</v>
+        <v>0.0716689442997283</v>
       </c>
       <c r="BZ124">
-        <v>0.03522008980499606</v>
+        <v>0.035220089804996</v>
       </c>
       <c r="CA124">
-        <v>0.1114915290739781</v>
+        <v>0.111491529073978</v>
       </c>
       <c r="CB124">
-        <v>0.08678444205212817</v>
+        <v>0.0867844420521281</v>
       </c>
       <c r="CC124">
-        <v>0.01858384506952434</v>
+        <v>0.0185838450695243</v>
       </c>
       <c r="CD124">
-        <v>0.009105693921035841</v>
+        <v>0.009105693921035799</v>
       </c>
       <c r="CE124">
-        <v>0.01381502710228896</v>
+        <v>0.0138150271022889</v>
       </c>
       <c r="CF124">
-        <v>0.006640182413336976</v>
+        <v>0.0066401824133369</v>
       </c>
       <c r="CG124">
         <v>11753.14860999999</v>
@@ -35831,16 +35843,16 @@
         <v>0.1232345957418265</v>
       </c>
       <c r="CL124">
-        <v>0.259391251439734</v>
+        <v>0.2593912514397339</v>
       </c>
       <c r="CM124">
         <v>10000</v>
       </c>
       <c r="CO124">
-        <v>0.008319714752637052</v>
+        <v>0.008319714752637</v>
       </c>
       <c r="CP124">
-        <v>0.005496954390135195</v>
+        <v>0.0054969543901351</v>
       </c>
       <c r="CQ124">
         <v>4940876.349740313</v>
@@ -35848,14 +35860,283 @@
       <c r="CR124">
         <v>4199685.074142367</v>
       </c>
-      <c r="CS124" s="2">
-        <v>45414.85936401004</v>
+      <c r="CS124" t="s">
+        <v>365</v>
       </c>
       <c r="CT124">
         <v>-0.7053510752114568</v>
       </c>
       <c r="CU124">
         <v>-0.8831403389490625</v>
+      </c>
+    </row>
+    <row r="125" spans="10:99">
+      <c r="J125" t="s">
+        <v>202</v>
+      </c>
+      <c r="K125">
+        <v>0.002236939357510792</v>
+      </c>
+      <c r="L125">
+        <v>0.001118469678755396</v>
+      </c>
+      <c r="M125">
+        <v>0.001236671099455799</v>
+      </c>
+      <c r="N125">
+        <v>0.001236671099455799</v>
+      </c>
+      <c r="O125">
+        <v>0.001839711725944437</v>
+      </c>
+      <c r="P125">
+        <v>0.0009198558629722187</v>
+      </c>
+      <c r="Q125">
+        <v>0.001434745181500574</v>
+      </c>
+      <c r="R125">
+        <v>0.001434745181500574</v>
+      </c>
+      <c r="S125">
+        <v>11.72360044754813</v>
+      </c>
+      <c r="T125">
+        <v>9.218874184960841</v>
+      </c>
+      <c r="U125">
+        <v>0.3073806958778552</v>
+      </c>
+      <c r="V125">
+        <v>0.5954825002586427</v>
+      </c>
+      <c r="W125">
+        <v>0.03031893049282055</v>
+      </c>
+      <c r="X125">
+        <v>0.09013365192788314</v>
+      </c>
+      <c r="Y125">
+        <v>0.1454939486875937</v>
+      </c>
+      <c r="Z125">
+        <v>0.2026782245235637</v>
+      </c>
+      <c r="AA125">
+        <v>0.9992673609594271</v>
+      </c>
+      <c r="AB125">
+        <v>0.8910212382727811</v>
+      </c>
+      <c r="AC125">
+        <v>0.8304744576577544</v>
+      </c>
+      <c r="AD125">
+        <v>0.9973579260301606</v>
+      </c>
+      <c r="AE125">
+        <v>0.8202504119047692</v>
+      </c>
+      <c r="AF125">
+        <v>0.7981920349549094</v>
+      </c>
+      <c r="AG125">
+        <v>0.003859202734480985</v>
+      </c>
+      <c r="AH125">
+        <v>0.01053076937279949</v>
+      </c>
+      <c r="AI125">
+        <v>0.9992673609594271</v>
+      </c>
+      <c r="AJ125">
+        <v>0.9973579260301606</v>
+      </c>
+      <c r="AK125">
+        <v>0.003859202734480985</v>
+      </c>
+      <c r="AL125">
+        <v>0.01053076937279949</v>
+      </c>
+      <c r="AM125" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN125">
+        <v>0.02093695864100079</v>
+      </c>
+      <c r="AO125">
+        <v>0.07852190783920794</v>
+      </c>
+      <c r="AP125">
+        <v>-3159.000605748</v>
+      </c>
+      <c r="AQ125">
+        <v>-934.5695654580001</v>
+      </c>
+      <c r="AR125">
+        <v>111685.6708642515</v>
+      </c>
+      <c r="AS125">
+        <v>37989.62942454188</v>
+      </c>
+      <c r="AT125">
+        <v>111671.3915542515</v>
+      </c>
+      <c r="AU125">
+        <v>37959.54686454187</v>
+      </c>
+      <c r="AV125">
+        <v>10.16856708642515</v>
+      </c>
+      <c r="AW125">
+        <v>2.798962942454188</v>
+      </c>
+      <c r="AX125">
+        <v>2.045950500263297</v>
+      </c>
+      <c r="AY125">
+        <v>2.602918131592165</v>
+      </c>
+      <c r="AZ125">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="BA125">
+        <v>119.2</v>
+      </c>
+      <c r="BB125">
+        <v>0.003224980594379225</v>
+      </c>
+      <c r="BC125">
+        <v>0.06441365475871964</v>
+      </c>
+      <c r="BD125">
+        <v>-339.2159959189568</v>
+      </c>
+      <c r="BE125">
+        <v>-1991.385805693739</v>
+      </c>
+      <c r="BF125">
+        <v>4791</v>
+      </c>
+      <c r="BG125">
+        <v>3080</v>
+      </c>
+      <c r="BH125">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI125">
+        <v>7870</v>
+      </c>
+      <c r="BJ125">
+        <v>6876</v>
+      </c>
+      <c r="BK125">
+        <v>12661</v>
+      </c>
+      <c r="BL125">
+        <v>9956</v>
+      </c>
+      <c r="BM125">
+        <v>4179</v>
+      </c>
+      <c r="BN125">
+        <v>2874</v>
+      </c>
+      <c r="BO125">
+        <v>4788</v>
+      </c>
+      <c r="BP125">
+        <v>2982</v>
+      </c>
+      <c r="BQ125">
+        <v>3691</v>
+      </c>
+      <c r="BR125">
+        <v>4002</v>
+      </c>
+      <c r="BS125">
+        <v>3</v>
+      </c>
+      <c r="BT125">
+        <v>98</v>
+      </c>
+      <c r="BU125">
+        <v>0</v>
+      </c>
+      <c r="BV125">
+        <v>0</v>
+      </c>
+      <c r="BW125">
+        <v>101685.670864252</v>
+      </c>
+      <c r="BX125">
+        <v>27989.629424542</v>
+      </c>
+      <c r="BY125">
+        <v>0.04183586437192352</v>
+      </c>
+      <c r="BZ125">
+        <v>0.07999316210968833</v>
+      </c>
+      <c r="CA125">
+        <v>0.0782810542988181</v>
+      </c>
+      <c r="CB125">
+        <v>0.1679184055700101</v>
+      </c>
+      <c r="CC125">
+        <v>0.01403797457625645</v>
+      </c>
+      <c r="CD125">
+        <v>0.01758184801232305</v>
+      </c>
+      <c r="CE125">
+        <v>0.01023140492613323</v>
+      </c>
+      <c r="CF125">
+        <v>0.01265517397784129</v>
+      </c>
+      <c r="CG125">
+        <v>104844.67147</v>
+      </c>
+      <c r="CH125">
+        <v>28924.19899</v>
+      </c>
+      <c r="CI125">
+        <v>105183.8874659189</v>
+      </c>
+      <c r="CJ125">
+        <v>30915.58479569374</v>
+      </c>
+      <c r="CK125">
+        <v>0.05424559650284209</v>
+      </c>
+      <c r="CL125">
+        <v>0.1141280869522103</v>
+      </c>
+      <c r="CM125">
+        <v>10000</v>
+      </c>
+      <c r="CO125">
+        <v>0.001003086419753086</v>
+      </c>
+      <c r="CP125">
+        <v>0.02299382716049383</v>
+      </c>
+      <c r="CQ125">
+        <v>42201373.71041539</v>
+      </c>
+      <c r="CR125">
+        <v>14590537.25038491</v>
+      </c>
+      <c r="CS125" s="2">
+        <v>45415.27426109111</v>
+      </c>
+      <c r="CT125">
+        <v>-0.7252315072660098</v>
+      </c>
+      <c r="CU125">
+        <v>-0.6865130387546091</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MATICUSDT.json at 2024-05-03_17-38-09 bestfile_scores 0.0009313642327829802 bestfile_sharp 0.27554595873084214
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU125"/>
+  <dimension ref="A1:CU126"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -36137,6 +36137,275 @@
       </c>
       <c r="CU125">
         <v>-0.6865130387546091</v>
+      </c>
+    </row>
+    <row r="126" spans="10:99">
+      <c r="J126" t="s">
+        <v>199</v>
+      </c>
+      <c r="K126">
+        <v>0.001383012923460658</v>
+      </c>
+      <c r="L126">
+        <v>0.000691506461730329</v>
+      </c>
+      <c r="M126">
+        <v>0.0002290439155725466</v>
+      </c>
+      <c r="N126">
+        <v>0.0002290439155725466</v>
+      </c>
+      <c r="O126">
+        <v>0.002361505883074533</v>
+      </c>
+      <c r="P126">
+        <v>0.001180752941537266</v>
+      </c>
+      <c r="Q126">
+        <v>0.0003014819796742785</v>
+      </c>
+      <c r="R126">
+        <v>0.0003014819796742785</v>
+      </c>
+      <c r="S126">
+        <v>9.849314539486388</v>
+      </c>
+      <c r="T126">
+        <v>3.98532535238463</v>
+      </c>
+      <c r="U126">
+        <v>0.4366783408293085</v>
+      </c>
+      <c r="V126">
+        <v>0.6853692467580166</v>
+      </c>
+      <c r="W126">
+        <v>0.01152384743583983</v>
+      </c>
+      <c r="X126">
+        <v>0.03760503838204008</v>
+      </c>
+      <c r="Y126">
+        <v>0.133659095203956</v>
+      </c>
+      <c r="Z126">
+        <v>0.1662778902372808</v>
+      </c>
+      <c r="AA126">
+        <v>0.9997103948208556</v>
+      </c>
+      <c r="AB126">
+        <v>0.9241437817360305</v>
+      </c>
+      <c r="AC126">
+        <v>0.8686276318450761</v>
+      </c>
+      <c r="AD126">
+        <v>0.9994260410307935</v>
+      </c>
+      <c r="AE126">
+        <v>0.8666932819991978</v>
+      </c>
+      <c r="AF126">
+        <v>0.8338887911389863</v>
+      </c>
+      <c r="AG126">
+        <v>0.001956828295282353</v>
+      </c>
+      <c r="AH126">
+        <v>0.00511308770784138</v>
+      </c>
+      <c r="AI126">
+        <v>0.9997103948208556</v>
+      </c>
+      <c r="AJ126">
+        <v>0.9994260410307935</v>
+      </c>
+      <c r="AK126">
+        <v>0.001956828295282353</v>
+      </c>
+      <c r="AL126">
+        <v>0.00511308770784138</v>
+      </c>
+      <c r="AM126" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN126">
+        <v>0.01238684019763216</v>
+      </c>
+      <c r="AO126">
+        <v>0.01546350412039389</v>
+      </c>
+      <c r="AP126">
+        <v>-1358.599824</v>
+      </c>
+      <c r="AQ126">
+        <v>-130.7696636</v>
+      </c>
+      <c r="AR126">
+        <v>44423.45017599994</v>
+      </c>
+      <c r="AS126">
+        <v>12803.07833639999</v>
+      </c>
+      <c r="AT126">
+        <v>44421.59417599994</v>
+      </c>
+      <c r="AU126">
+        <v>12803.46233639999</v>
+      </c>
+      <c r="AV126">
+        <v>3.442345017599994</v>
+      </c>
+      <c r="AW126">
+        <v>0.2803078336399987</v>
+      </c>
+      <c r="AX126">
+        <v>2.432773386034256</v>
+      </c>
+      <c r="AY126">
+        <v>6.01494145925409</v>
+      </c>
+      <c r="AZ126">
+        <v>105.45</v>
+      </c>
+      <c r="BA126">
+        <v>107.2666666666667</v>
+      </c>
+      <c r="BB126">
+        <v>0</v>
+      </c>
+      <c r="BC126">
+        <v>0.003969329704302422</v>
+      </c>
+      <c r="BD126">
+        <v>0</v>
+      </c>
+      <c r="BE126">
+        <v>-11.69181869756181</v>
+      </c>
+      <c r="BF126">
+        <v>4529</v>
+      </c>
+      <c r="BG126">
+        <v>1860</v>
+      </c>
+      <c r="BH126">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI126">
+        <v>6098</v>
+      </c>
+      <c r="BJ126">
+        <v>2440</v>
+      </c>
+      <c r="BK126">
+        <v>10627</v>
+      </c>
+      <c r="BL126">
+        <v>4300</v>
+      </c>
+      <c r="BM126">
+        <v>4387</v>
+      </c>
+      <c r="BN126">
+        <v>1809</v>
+      </c>
+      <c r="BO126">
+        <v>4529</v>
+      </c>
+      <c r="BP126">
+        <v>1854</v>
+      </c>
+      <c r="BQ126">
+        <v>1711</v>
+      </c>
+      <c r="BR126">
+        <v>631</v>
+      </c>
+      <c r="BS126">
+        <v>0</v>
+      </c>
+      <c r="BT126">
+        <v>6</v>
+      </c>
+      <c r="BU126">
+        <v>0</v>
+      </c>
+      <c r="BV126">
+        <v>0</v>
+      </c>
+      <c r="BW126">
+        <v>34423.45017600005</v>
+      </c>
+      <c r="BX126">
+        <v>2803.078336400003</v>
+      </c>
+      <c r="BY126">
+        <v>0.0341364664259203</v>
+      </c>
+      <c r="BZ126">
+        <v>0.06706763821893927</v>
+      </c>
+      <c r="CA126">
+        <v>0.07138856039561405</v>
+      </c>
+      <c r="CB126">
+        <v>0.1424950593520785</v>
+      </c>
+      <c r="CC126">
+        <v>0.01075237522634257</v>
+      </c>
+      <c r="CD126">
+        <v>0.01511947735761453</v>
+      </c>
+      <c r="CE126">
+        <v>0.00841073551070542</v>
+      </c>
+      <c r="CF126">
+        <v>0.01330377112179511</v>
+      </c>
+      <c r="CG126">
+        <v>35782.05000000005</v>
+      </c>
+      <c r="CH126">
+        <v>2933.848000000003</v>
+      </c>
+      <c r="CI126">
+        <v>35782.05000000005</v>
+      </c>
+      <c r="CJ126">
+        <v>2945.539818697564</v>
+      </c>
+      <c r="CK126">
+        <v>0.1906279072499513</v>
+      </c>
+      <c r="CL126">
+        <v>0.04355217853927245</v>
+      </c>
+      <c r="CM126">
+        <v>10000</v>
+      </c>
+      <c r="CO126">
+        <v>0.001699104108742663</v>
+      </c>
+      <c r="CP126">
+        <v>0.00390021624961384</v>
+      </c>
+      <c r="CQ126">
+        <v>7118836.508650885</v>
+      </c>
+      <c r="CR126">
+        <v>716228.3326648935</v>
+      </c>
+      <c r="CS126" s="2">
+        <v>45415.46273133369</v>
+      </c>
+      <c r="CT126">
+        <v>-0.892232561911074</v>
+      </c>
+      <c r="CU126">
+        <v>-0.8971938325335068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MANAUSDT.json at 2024-05-03_21-38-16 bestfile_scores 0.0005740547238169719 bestfile_sharp 0.0972711357319691
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1064" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU126"/>
+  <dimension ref="A1:CU127"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -36406,6 +36406,275 @@
       </c>
       <c r="CU126">
         <v>-0.8971938325335068</v>
+      </c>
+    </row>
+    <row r="127" spans="10:99">
+      <c r="J127" t="s">
+        <v>188</v>
+      </c>
+      <c r="K127">
+        <v>0.002527200832158849</v>
+      </c>
+      <c r="L127">
+        <v>0.001263600416079425</v>
+      </c>
+      <c r="M127">
+        <v>0.000864585709725807</v>
+      </c>
+      <c r="N127">
+        <v>0.000864585709725807</v>
+      </c>
+      <c r="O127">
+        <v>0.002010600907909965</v>
+      </c>
+      <c r="P127">
+        <v>0.001005300453954983</v>
+      </c>
+      <c r="Q127">
+        <v>0.0005919703513717067</v>
+      </c>
+      <c r="R127">
+        <v>0.0005919703513717067</v>
+      </c>
+      <c r="S127">
+        <v>11.98472163277904</v>
+      </c>
+      <c r="T127">
+        <v>18.10718006095914</v>
+      </c>
+      <c r="U127">
+        <v>0.3889019653822828</v>
+      </c>
+      <c r="V127">
+        <v>0.6262798079011247</v>
+      </c>
+      <c r="W127">
+        <v>0.0528228472482147</v>
+      </c>
+      <c r="X127">
+        <v>0.09631323286308821</v>
+      </c>
+      <c r="Y127">
+        <v>0.2192686139069459</v>
+      </c>
+      <c r="Z127">
+        <v>0.2173845172835257</v>
+      </c>
+      <c r="AA127">
+        <v>0.9991045081436382</v>
+      </c>
+      <c r="AB127">
+        <v>0.814661727548742</v>
+      </c>
+      <c r="AC127">
+        <v>0.811840490138626</v>
+      </c>
+      <c r="AD127">
+        <v>0.9979048278191958</v>
+      </c>
+      <c r="AE127">
+        <v>0.7809869082245915</v>
+      </c>
+      <c r="AF127">
+        <v>0.7886800389953728</v>
+      </c>
+      <c r="AG127">
+        <v>0.006955633552441099</v>
+      </c>
+      <c r="AH127">
+        <v>0.01032672546198395</v>
+      </c>
+      <c r="AI127">
+        <v>0.9991045081436382</v>
+      </c>
+      <c r="AJ127">
+        <v>0.9979048278191958</v>
+      </c>
+      <c r="AK127">
+        <v>0.006955633552441099</v>
+      </c>
+      <c r="AL127">
+        <v>0.01032672546198395</v>
+      </c>
+      <c r="AM127" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN127">
+        <v>0.02767415259442773</v>
+      </c>
+      <c r="AO127">
+        <v>0.06217967383121285</v>
+      </c>
+      <c r="AP127">
+        <v>-7121.356162382001</v>
+      </c>
+      <c r="AQ127">
+        <v>-1321.439869042</v>
+      </c>
+      <c r="AR127">
+        <v>152690.6199476184</v>
+      </c>
+      <c r="AS127">
+        <v>25429.20276095791</v>
+      </c>
+      <c r="AT127">
+        <v>152690.6199476184</v>
+      </c>
+      <c r="AU127">
+        <v>25181.80066095791</v>
+      </c>
+      <c r="AV127">
+        <v>14.26906199476184</v>
+      </c>
+      <c r="AW127">
+        <v>1.542920276095791</v>
+      </c>
+      <c r="AX127">
+        <v>1.999603358574151</v>
+      </c>
+      <c r="AY127">
+        <v>1.32465480208653</v>
+      </c>
+      <c r="AZ127">
+        <v>85.68333333333334</v>
+      </c>
+      <c r="BA127">
+        <v>108.2333333333333</v>
+      </c>
+      <c r="BB127">
+        <v>0.00234278296984482</v>
+      </c>
+      <c r="BC127">
+        <v>0.09022560182748188</v>
+      </c>
+      <c r="BD127">
+        <v>-351.8011400289388</v>
+      </c>
+      <c r="BE127">
+        <v>-1661.22152406649</v>
+      </c>
+      <c r="BF127">
+        <v>5757</v>
+      </c>
+      <c r="BG127">
+        <v>8191</v>
+      </c>
+      <c r="BH127">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI127">
+        <v>7186</v>
+      </c>
+      <c r="BJ127">
+        <v>11364</v>
+      </c>
+      <c r="BK127">
+        <v>12943</v>
+      </c>
+      <c r="BL127">
+        <v>19555</v>
+      </c>
+      <c r="BM127">
+        <v>5176</v>
+      </c>
+      <c r="BN127">
+        <v>8106</v>
+      </c>
+      <c r="BO127">
+        <v>5737</v>
+      </c>
+      <c r="BP127">
+        <v>8140</v>
+      </c>
+      <c r="BQ127">
+        <v>2010</v>
+      </c>
+      <c r="BR127">
+        <v>3258</v>
+      </c>
+      <c r="BS127">
+        <v>20</v>
+      </c>
+      <c r="BT127">
+        <v>51</v>
+      </c>
+      <c r="BU127">
+        <v>0</v>
+      </c>
+      <c r="BV127">
+        <v>0</v>
+      </c>
+      <c r="BW127">
+        <v>142690.619947618</v>
+      </c>
+      <c r="BX127">
+        <v>15429.20276095801</v>
+      </c>
+      <c r="BY127">
+        <v>0.04365272898899163</v>
+      </c>
+      <c r="BZ127">
+        <v>0.08212539615751041</v>
+      </c>
+      <c r="CA127">
+        <v>0.1229319602606669</v>
+      </c>
+      <c r="CB127">
+        <v>0.1744545373326135</v>
+      </c>
+      <c r="CC127">
+        <v>0.009299389898866391</v>
+      </c>
+      <c r="CD127">
+        <v>0.01616222911983619</v>
+      </c>
+      <c r="CE127">
+        <v>0.008363201522622345</v>
+      </c>
+      <c r="CF127">
+        <v>0.01188052573500747</v>
+      </c>
+      <c r="CG127">
+        <v>149811.97611</v>
+      </c>
+      <c r="CH127">
+        <v>16750.64263000001</v>
+      </c>
+      <c r="CI127">
+        <v>150163.7772500289</v>
+      </c>
+      <c r="CJ127">
+        <v>18411.8641540665</v>
+      </c>
+      <c r="CK127">
+        <v>0.2755459587308421</v>
+      </c>
+      <c r="CL127">
+        <v>0.08624386399016262</v>
+      </c>
+      <c r="CM127">
+        <v>10000</v>
+      </c>
+      <c r="CO127">
+        <v>0.007677469135802469</v>
+      </c>
+      <c r="CP127">
+        <v>0.01990740740740741</v>
+      </c>
+      <c r="CQ127">
+        <v>47790589.85561877</v>
+      </c>
+      <c r="CR127">
+        <v>7960049.437302528</v>
+      </c>
+      <c r="CS127" s="2">
+        <v>45415.73485744271</v>
+      </c>
+      <c r="CT127">
+        <v>-0.7368411844597273</v>
+      </c>
+      <c r="CU127">
+        <v>-0.7671793576642513</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update EOSUSDT.json at 2024-05-06_04-05-59 bestfile_scores 0.0007650253768974075 bestfile_sharp 0.1430856857822173
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU127"/>
+  <dimension ref="A1:CU128"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -36675,6 +36675,275 @@
       </c>
       <c r="CU127">
         <v>-0.7671793576642513</v>
+      </c>
+    </row>
+    <row r="128" spans="10:99">
+      <c r="J128" t="s">
+        <v>223</v>
+      </c>
+      <c r="K128">
+        <v>0.0009916708039618971</v>
+      </c>
+      <c r="L128">
+        <v>0.0004958354019809486</v>
+      </c>
+      <c r="M128">
+        <v>0.0004334120936875241</v>
+      </c>
+      <c r="N128">
+        <v>0.0004334120936875241</v>
+      </c>
+      <c r="O128">
+        <v>0.002243446688982042</v>
+      </c>
+      <c r="P128">
+        <v>0.001121723344491021</v>
+      </c>
+      <c r="Q128">
+        <v>0.0002452480551083935</v>
+      </c>
+      <c r="R128">
+        <v>0.0002452480551083935</v>
+      </c>
+      <c r="S128">
+        <v>37.21347274200394</v>
+      </c>
+      <c r="T128">
+        <v>5.266869863806474</v>
+      </c>
+      <c r="U128">
+        <v>0.4445259378977388</v>
+      </c>
+      <c r="V128">
+        <v>0.7853980331305344</v>
+      </c>
+      <c r="W128">
+        <v>0.0125379628764633</v>
+      </c>
+      <c r="X128">
+        <v>0.008883600048393513</v>
+      </c>
+      <c r="Y128">
+        <v>0.09006475387533798</v>
+      </c>
+      <c r="Z128">
+        <v>0.03394554869229915</v>
+      </c>
+      <c r="AA128">
+        <v>0.9998017683325096</v>
+      </c>
+      <c r="AB128">
+        <v>0.9356801672223101</v>
+      </c>
+      <c r="AC128">
+        <v>0.9812863454314013</v>
+      </c>
+      <c r="AD128">
+        <v>0.9997023184492735</v>
+      </c>
+      <c r="AE128">
+        <v>0.8827086764609655</v>
+      </c>
+      <c r="AF128">
+        <v>0.8851121996733892</v>
+      </c>
+      <c r="AG128">
+        <v>0.002106263143805456</v>
+      </c>
+      <c r="AH128">
+        <v>0.001129927884937069</v>
+      </c>
+      <c r="AI128">
+        <v>0.9998017683325096</v>
+      </c>
+      <c r="AJ128">
+        <v>0.9997023184492735</v>
+      </c>
+      <c r="AK128">
+        <v>0.002106263143805456</v>
+      </c>
+      <c r="AL128">
+        <v>0.001129927884937069</v>
+      </c>
+      <c r="AM128" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN128">
+        <v>0.006949816448382135</v>
+      </c>
+      <c r="AO128">
+        <v>0.01124501323719901</v>
+      </c>
+      <c r="AP128">
+        <v>-2171.26219778</v>
+      </c>
+      <c r="AQ128">
+        <v>-277.67608284</v>
+      </c>
+      <c r="AR128">
+        <v>29166.40610222029</v>
+      </c>
+      <c r="AS128">
+        <v>15967.42471715995</v>
+      </c>
+      <c r="AT128">
+        <v>29166.40610222029</v>
+      </c>
+      <c r="AU128">
+        <v>15963.01471715995</v>
+      </c>
+      <c r="AV128">
+        <v>1.916640610222029</v>
+      </c>
+      <c r="AW128">
+        <v>0.5967424717159953</v>
+      </c>
+      <c r="AX128">
+        <v>0.6439554925184964</v>
+      </c>
+      <c r="AY128">
+        <v>4.548267979602603</v>
+      </c>
+      <c r="AZ128">
+        <v>118.15</v>
+      </c>
+      <c r="BA128">
+        <v>107.4333333333333</v>
+      </c>
+      <c r="BB128">
+        <v>0.002977066823538635</v>
+      </c>
+      <c r="BC128">
+        <v>0</v>
+      </c>
+      <c r="BD128">
+        <v>-63.71334326806215</v>
+      </c>
+      <c r="BE128">
+        <v>0</v>
+      </c>
+      <c r="BF128">
+        <v>19235</v>
+      </c>
+      <c r="BG128">
+        <v>2604</v>
+      </c>
+      <c r="BH128">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI128">
+        <v>20954</v>
+      </c>
+      <c r="BJ128">
+        <v>3084</v>
+      </c>
+      <c r="BK128">
+        <v>40189</v>
+      </c>
+      <c r="BL128">
+        <v>5688</v>
+      </c>
+      <c r="BM128">
+        <v>19221</v>
+      </c>
+      <c r="BN128">
+        <v>2533</v>
+      </c>
+      <c r="BO128">
+        <v>19230</v>
+      </c>
+      <c r="BP128">
+        <v>2604</v>
+      </c>
+      <c r="BQ128">
+        <v>1733</v>
+      </c>
+      <c r="BR128">
+        <v>551</v>
+      </c>
+      <c r="BS128">
+        <v>5</v>
+      </c>
+      <c r="BT128">
+        <v>0</v>
+      </c>
+      <c r="BU128">
+        <v>0</v>
+      </c>
+      <c r="BV128">
+        <v>0</v>
+      </c>
+      <c r="BW128">
+        <v>19166.40610222001</v>
+      </c>
+      <c r="BX128">
+        <v>5967.42471716</v>
+      </c>
+      <c r="BY128">
+        <v>0.03039765112958839</v>
+      </c>
+      <c r="BZ128">
+        <v>0.0727068207574246</v>
+      </c>
+      <c r="CA128">
+        <v>0.04694679727294592</v>
+      </c>
+      <c r="CB128">
+        <v>0.1186010659433643</v>
+      </c>
+      <c r="CC128">
+        <v>0.01021563002336573</v>
+      </c>
+      <c r="CD128">
+        <v>0.01685222400259557</v>
+      </c>
+      <c r="CE128">
+        <v>0.007489848548474887</v>
+      </c>
+      <c r="CF128">
+        <v>0.01524264633852101</v>
+      </c>
+      <c r="CG128">
+        <v>21337.66830000001</v>
+      </c>
+      <c r="CH128">
+        <v>6245.1008</v>
+      </c>
+      <c r="CI128">
+        <v>21401.38164326808</v>
+      </c>
+      <c r="CJ128">
+        <v>6245.1008</v>
+      </c>
+      <c r="CK128">
+        <v>0.09727113573196911</v>
+      </c>
+      <c r="CL128">
+        <v>0.1645134634887986</v>
+      </c>
+      <c r="CM128">
+        <v>10000</v>
+      </c>
+      <c r="CO128">
+        <v>0.002237654320987654</v>
+      </c>
+      <c r="CP128">
+        <v>0.0005401234567901234</v>
+      </c>
+      <c r="CQ128">
+        <v>6564078.281929377</v>
+      </c>
+      <c r="CR128">
+        <v>1259981.153790825</v>
+      </c>
+      <c r="CS128" s="2">
+        <v>45415.90160276014</v>
+      </c>
+      <c r="CT128">
+        <v>-0.9143802706411295</v>
+      </c>
+      <c r="CU128">
+        <v>-0.9714369186341948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 1INCHUSDT.json at 2024-05-06_07-53-49 bestfile_scores 0.001016014221184683 bestfile_sharp 0.18367785429652245
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU128"/>
+  <dimension ref="A1:CU129"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -36944,6 +36944,275 @@
       </c>
       <c r="CU128">
         <v>-0.9714369186341948</v>
+      </c>
+    </row>
+    <row r="129" spans="10:99">
+      <c r="J129" t="s">
+        <v>225</v>
+      </c>
+      <c r="K129">
+        <v>0.0008442804144459526</v>
+      </c>
+      <c r="L129">
+        <v>0.0004221402072229763</v>
+      </c>
+      <c r="M129">
+        <v>0.001085110189479765</v>
+      </c>
+      <c r="N129">
+        <v>0.001085110189479765</v>
+      </c>
+      <c r="O129">
+        <v>0.0008512421775949575</v>
+      </c>
+      <c r="P129">
+        <v>0.0004256210887974788</v>
+      </c>
+      <c r="Q129">
+        <v>0.001127230022089409</v>
+      </c>
+      <c r="R129">
+        <v>0.001127230022089409</v>
+      </c>
+      <c r="S129">
+        <v>8.785524132875498</v>
+      </c>
+      <c r="T129">
+        <v>13.91164782591921</v>
+      </c>
+      <c r="U129">
+        <v>0.4003236475284112</v>
+      </c>
+      <c r="V129">
+        <v>0.5589109973727375</v>
+      </c>
+      <c r="W129">
+        <v>0.05352168823328322</v>
+      </c>
+      <c r="X129">
+        <v>0.08258862992555079</v>
+      </c>
+      <c r="Y129">
+        <v>0.1318918477338805</v>
+      </c>
+      <c r="Z129">
+        <v>0.234691237232178</v>
+      </c>
+      <c r="AA129">
+        <v>0.9989424313782471</v>
+      </c>
+      <c r="AB129">
+        <v>0.8992973485146749</v>
+      </c>
+      <c r="AC129">
+        <v>0.7864883954783682</v>
+      </c>
+      <c r="AD129">
+        <v>0.9980516147377282</v>
+      </c>
+      <c r="AE129">
+        <v>0.6369384261288934</v>
+      </c>
+      <c r="AF129">
+        <v>0.7678936348016684</v>
+      </c>
+      <c r="AG129">
+        <v>0.005325052147641551</v>
+      </c>
+      <c r="AH129">
+        <v>0.009728832881625836</v>
+      </c>
+      <c r="AI129">
+        <v>0.9989424313782471</v>
+      </c>
+      <c r="AJ129">
+        <v>0.9980516147377282</v>
+      </c>
+      <c r="AK129">
+        <v>0.005325052147641551</v>
+      </c>
+      <c r="AL129">
+        <v>0.009728832881625836</v>
+      </c>
+      <c r="AM129" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN129">
+        <v>0.02756269827294157</v>
+      </c>
+      <c r="AO129">
+        <v>0.07443085699132103</v>
+      </c>
+      <c r="AP129">
+        <v>-784.2830687000001</v>
+      </c>
+      <c r="AQ129">
+        <v>-880.8663830600001</v>
+      </c>
+      <c r="AR129">
+        <v>24878.10443129996</v>
+      </c>
+      <c r="AS129">
+        <v>32259.85371693991</v>
+      </c>
+      <c r="AT129">
+        <v>24878.10443129996</v>
+      </c>
+      <c r="AU129">
+        <v>32086.41841693991</v>
+      </c>
+      <c r="AV129">
+        <v>1.487810443129996</v>
+      </c>
+      <c r="AW129">
+        <v>2.225985371693991</v>
+      </c>
+      <c r="AX129">
+        <v>2.728916763290116</v>
+      </c>
+      <c r="AY129">
+        <v>1.722684106592114</v>
+      </c>
+      <c r="AZ129">
+        <v>116.3166666666667</v>
+      </c>
+      <c r="BA129">
+        <v>86.63333333333334</v>
+      </c>
+      <c r="BB129">
+        <v>0.04375585519857265</v>
+      </c>
+      <c r="BC129">
+        <v>0.07952053879597674</v>
+      </c>
+      <c r="BD129">
+        <v>-716.6801106596547</v>
+      </c>
+      <c r="BE129">
+        <v>-1999.13480749683</v>
+      </c>
+      <c r="BF129">
+        <v>3179</v>
+      </c>
+      <c r="BG129">
+        <v>2815</v>
+      </c>
+      <c r="BH129">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI129">
+        <v>6309</v>
+      </c>
+      <c r="BJ129">
+        <v>12209</v>
+      </c>
+      <c r="BK129">
+        <v>9488</v>
+      </c>
+      <c r="BL129">
+        <v>15024</v>
+      </c>
+      <c r="BM129">
+        <v>2890</v>
+      </c>
+      <c r="BN129">
+        <v>2489</v>
+      </c>
+      <c r="BO129">
+        <v>3151</v>
+      </c>
+      <c r="BP129">
+        <v>2688</v>
+      </c>
+      <c r="BQ129">
+        <v>3419</v>
+      </c>
+      <c r="BR129">
+        <v>9720</v>
+      </c>
+      <c r="BS129">
+        <v>28</v>
+      </c>
+      <c r="BT129">
+        <v>127</v>
+      </c>
+      <c r="BU129">
+        <v>0</v>
+      </c>
+      <c r="BV129">
+        <v>0</v>
+      </c>
+      <c r="BW129">
+        <v>14878.10443129999</v>
+      </c>
+      <c r="BX129">
+        <v>22259.85371694002</v>
+      </c>
+      <c r="BY129">
+        <v>0.05119753308813837</v>
+      </c>
+      <c r="BZ129">
+        <v>0.07338592518482537</v>
+      </c>
+      <c r="CA129">
+        <v>0.1007517646434705</v>
+      </c>
+      <c r="CB129">
+        <v>0.1883847376217125</v>
+      </c>
+      <c r="CC129">
+        <v>0.009808961510069625</v>
+      </c>
+      <c r="CD129">
+        <v>0.007969733953587571</v>
+      </c>
+      <c r="CE129">
+        <v>0.00918904401224825</v>
+      </c>
+      <c r="CF129">
+        <v>0.01124691232412593</v>
+      </c>
+      <c r="CG129">
+        <v>15662.38749999999</v>
+      </c>
+      <c r="CH129">
+        <v>23140.72010000002</v>
+      </c>
+      <c r="CI129">
+        <v>16379.06761065964</v>
+      </c>
+      <c r="CJ129">
+        <v>25139.85490749685</v>
+      </c>
+      <c r="CK129">
+        <v>0.1430856857822173</v>
+      </c>
+      <c r="CL129">
+        <v>0.0861003690194944</v>
+      </c>
+      <c r="CM129">
+        <v>10000</v>
+      </c>
+      <c r="CO129">
+        <v>0.0002700617283950617</v>
+      </c>
+      <c r="CP129">
+        <v>0.01697530864197531</v>
+      </c>
+      <c r="CQ129">
+        <v>13221633.21657962</v>
+      </c>
+      <c r="CR129">
+        <v>16803825.65057263</v>
+      </c>
+      <c r="CS129" s="2">
+        <v>45418.17086291177</v>
+      </c>
+      <c r="CT129">
+        <v>-0.8590793790924167</v>
+      </c>
+      <c r="CU129">
+        <v>-0.664722383588948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ARUSDT.json at 2024-05-06_15-44-39 bestfile_scores 0.000791116930251376 bestfile_sharp 0.1670495380138063
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU129"/>
+  <dimension ref="A1:CU130"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -37213,6 +37213,275 @@
       </c>
       <c r="CU129">
         <v>-0.664722383588948</v>
+      </c>
+    </row>
+    <row r="130" spans="10:99">
+      <c r="J130" t="s">
+        <v>231</v>
+      </c>
+      <c r="K130">
+        <v>0.001974030175498021</v>
+      </c>
+      <c r="L130">
+        <v>0.0009870150877490103</v>
+      </c>
+      <c r="M130">
+        <v>0.0007664952070594033</v>
+      </c>
+      <c r="N130">
+        <v>0.0007664952070594033</v>
+      </c>
+      <c r="O130">
+        <v>0.003173515670422167</v>
+      </c>
+      <c r="P130">
+        <v>0.001586757835211083</v>
+      </c>
+      <c r="Q130">
+        <v>0.0007237887547192345</v>
+      </c>
+      <c r="R130">
+        <v>0.0007237887547192345</v>
+      </c>
+      <c r="S130">
+        <v>17.059046147905</v>
+      </c>
+      <c r="T130">
+        <v>18.80980884340606</v>
+      </c>
+      <c r="U130">
+        <v>0.2783519362819384</v>
+      </c>
+      <c r="V130">
+        <v>0.4268606631339594</v>
+      </c>
+      <c r="W130">
+        <v>0.038189920225125</v>
+      </c>
+      <c r="X130">
+        <v>0.09148465699256171</v>
+      </c>
+      <c r="Y130">
+        <v>0.2376398340586393</v>
+      </c>
+      <c r="Z130">
+        <v>0.2497684200301903</v>
+      </c>
+      <c r="AA130">
+        <v>0.9996187056501427</v>
+      </c>
+      <c r="AB130">
+        <v>0.8061992107897711</v>
+      </c>
+      <c r="AC130">
+        <v>0.8016372527597291</v>
+      </c>
+      <c r="AD130">
+        <v>0.9966353723638919</v>
+      </c>
+      <c r="AE130">
+        <v>0.7625286078451134</v>
+      </c>
+      <c r="AF130">
+        <v>0.6727893426624312</v>
+      </c>
+      <c r="AG130">
+        <v>0.005654459134801621</v>
+      </c>
+      <c r="AH130">
+        <v>0.01156385279379274</v>
+      </c>
+      <c r="AI130">
+        <v>0.9996187056501427</v>
+      </c>
+      <c r="AJ130">
+        <v>0.9966353723638919</v>
+      </c>
+      <c r="AK130">
+        <v>0.005654459134801621</v>
+      </c>
+      <c r="AL130">
+        <v>0.01156385279379274</v>
+      </c>
+      <c r="AM130" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN130">
+        <v>0.009514899377222377</v>
+      </c>
+      <c r="AO130">
+        <v>0.07002115137346268</v>
+      </c>
+      <c r="AP130">
+        <v>-4588.53556124</v>
+      </c>
+      <c r="AQ130">
+        <v>-565.7133034999999</v>
+      </c>
+      <c r="AR130">
+        <v>83963.47843875979</v>
+      </c>
+      <c r="AS130">
+        <v>22857.62349650046</v>
+      </c>
+      <c r="AT130">
+        <v>83963.47843875979</v>
+      </c>
+      <c r="AU130">
+        <v>22787.99569650046</v>
+      </c>
+      <c r="AV130">
+        <v>7.396347843875979</v>
+      </c>
+      <c r="AW130">
+        <v>1.285762349650045</v>
+      </c>
+      <c r="AX130">
+        <v>1.404258806483745</v>
+      </c>
+      <c r="AY130">
+        <v>1.273264675930489</v>
+      </c>
+      <c r="AZ130">
+        <v>111.5833333333333</v>
+      </c>
+      <c r="BA130">
+        <v>109.1666666666667</v>
+      </c>
+      <c r="BB130">
+        <v>0.01167312073209618</v>
+      </c>
+      <c r="BC130">
+        <v>0</v>
+      </c>
+      <c r="BD130">
+        <v>-927.7771984209628</v>
+      </c>
+      <c r="BE130">
+        <v>0</v>
+      </c>
+      <c r="BF130">
+        <v>8231</v>
+      </c>
+      <c r="BG130">
+        <v>5151</v>
+      </c>
+      <c r="BH130">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI130">
+        <v>10175</v>
+      </c>
+      <c r="BJ130">
+        <v>15144</v>
+      </c>
+      <c r="BK130">
+        <v>18406</v>
+      </c>
+      <c r="BL130">
+        <v>20295</v>
+      </c>
+      <c r="BM130">
+        <v>7341</v>
+      </c>
+      <c r="BN130">
+        <v>5148</v>
+      </c>
+      <c r="BO130">
+        <v>8221</v>
+      </c>
+      <c r="BP130">
+        <v>5151</v>
+      </c>
+      <c r="BQ130">
+        <v>2834</v>
+      </c>
+      <c r="BR130">
+        <v>9996</v>
+      </c>
+      <c r="BS130">
+        <v>10</v>
+      </c>
+      <c r="BT130">
+        <v>0</v>
+      </c>
+      <c r="BU130">
+        <v>0</v>
+      </c>
+      <c r="BV130">
+        <v>0</v>
+      </c>
+      <c r="BW130">
+        <v>73963.47843875994</v>
+      </c>
+      <c r="BX130">
+        <v>12857.62349649998</v>
+      </c>
+      <c r="BY130">
+        <v>0.02849449704352394</v>
+      </c>
+      <c r="BZ130">
+        <v>0.1223428777591633</v>
+      </c>
+      <c r="CA130">
+        <v>0.1346813102267796</v>
+      </c>
+      <c r="CB130">
+        <v>0.1997916794785066</v>
+      </c>
+      <c r="CC130">
+        <v>0.005765234951725934</v>
+      </c>
+      <c r="CD130">
+        <v>0.01652623708768868</v>
+      </c>
+      <c r="CE130">
+        <v>0.007299010812043965</v>
+      </c>
+      <c r="CF130">
+        <v>0.02028416007817126</v>
+      </c>
+      <c r="CG130">
+        <v>78552.01399999994</v>
+      </c>
+      <c r="CH130">
+        <v>13423.33679999998</v>
+      </c>
+      <c r="CI130">
+        <v>79479.79119842091</v>
+      </c>
+      <c r="CJ130">
+        <v>13423.33679999998</v>
+      </c>
+      <c r="CK130">
+        <v>0.1836778542965224</v>
+      </c>
+      <c r="CL130">
+        <v>0.08538577050201569</v>
+      </c>
+      <c r="CM130">
+        <v>10000</v>
+      </c>
+      <c r="CO130">
+        <v>0.004402224281742354</v>
+      </c>
+      <c r="CP130">
+        <v>0.002201112140871177</v>
+      </c>
+      <c r="CQ130">
+        <v>36758077.75906376</v>
+      </c>
+      <c r="CR130">
+        <v>7461415.917733567</v>
+      </c>
+      <c r="CS130" s="2">
+        <v>45418.3290608931</v>
+      </c>
+      <c r="CT130">
+        <v>-0.7834455371012616</v>
+      </c>
+      <c r="CU130">
+        <v>-0.7813678870189401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ETCUSDT.json at 2024-05-07_03-28-00 bestfile_scores 0.0007756748300649264 bestfile_sharp 0.18446220892236095
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1072" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU130"/>
+  <dimension ref="A1:CU131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -37482,6 +37482,275 @@
       </c>
       <c r="CU130">
         <v>-0.7813678870189401</v>
+      </c>
+    </row>
+    <row r="131" spans="10:99">
+      <c r="J131" t="s">
+        <v>235</v>
+      </c>
+      <c r="K131">
+        <v>0.001339537874347929</v>
+      </c>
+      <c r="L131">
+        <v>0.0006697689371739646</v>
+      </c>
+      <c r="M131">
+        <v>0.0005374852835609012</v>
+      </c>
+      <c r="N131">
+        <v>0.0005374852835609012</v>
+      </c>
+      <c r="O131">
+        <v>0.002176102086959663</v>
+      </c>
+      <c r="P131">
+        <v>0.001088051043479832</v>
+      </c>
+      <c r="Q131">
+        <v>0.0008691624567908063</v>
+      </c>
+      <c r="R131">
+        <v>0.0008691624567908063</v>
+      </c>
+      <c r="S131">
+        <v>12.16634497280225</v>
+      </c>
+      <c r="T131">
+        <v>8.236181786278294</v>
+      </c>
+      <c r="U131">
+        <v>0.3712811428587015</v>
+      </c>
+      <c r="V131">
+        <v>0.6888497180676669</v>
+      </c>
+      <c r="W131">
+        <v>0.08655526110596123</v>
+      </c>
+      <c r="X131">
+        <v>0.05723982251474728</v>
+      </c>
+      <c r="Y131">
+        <v>0.2344143337672382</v>
+      </c>
+      <c r="Z131">
+        <v>0.1426300321036997</v>
+      </c>
+      <c r="AA131">
+        <v>0.9991700579884613</v>
+      </c>
+      <c r="AB131">
+        <v>0.8011728703136501</v>
+      </c>
+      <c r="AC131">
+        <v>0.8696704621071671</v>
+      </c>
+      <c r="AD131">
+        <v>0.9992041267369297</v>
+      </c>
+      <c r="AE131">
+        <v>0.7665933382226603</v>
+      </c>
+      <c r="AF131">
+        <v>0.857632976502503</v>
+      </c>
+      <c r="AG131">
+        <v>0.007227404012196759</v>
+      </c>
+      <c r="AH131">
+        <v>0.006661789739206238</v>
+      </c>
+      <c r="AI131">
+        <v>0.9991700579884613</v>
+      </c>
+      <c r="AJ131">
+        <v>0.9992041267369297</v>
+      </c>
+      <c r="AK131">
+        <v>0.007227404012196759</v>
+      </c>
+      <c r="AL131">
+        <v>0.006661789739206238</v>
+      </c>
+      <c r="AM131" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN131">
+        <v>0.01752408109593183</v>
+      </c>
+      <c r="AO131">
+        <v>0.01843302335277237</v>
+      </c>
+      <c r="AP131">
+        <v>-1500.0518362</v>
+      </c>
+      <c r="AQ131">
+        <v>-337.4168938</v>
+      </c>
+      <c r="AR131">
+        <v>35661.49036379989</v>
+      </c>
+      <c r="AS131">
+        <v>16659.31270620001</v>
+      </c>
+      <c r="AT131">
+        <v>35661.49036379989</v>
+      </c>
+      <c r="AU131">
+        <v>16659.08950620001</v>
+      </c>
+      <c r="AV131">
+        <v>2.566149036379989</v>
+      </c>
+      <c r="AW131">
+        <v>0.6659312706200007</v>
+      </c>
+      <c r="AX131">
+        <v>1.96876099812491</v>
+      </c>
+      <c r="AY131">
+        <v>2.911256711838405</v>
+      </c>
+      <c r="AZ131">
+        <v>103.3833333333333</v>
+      </c>
+      <c r="BA131">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="BB131">
+        <v>0.08274042588622789</v>
+      </c>
+      <c r="BC131">
+        <v>0.01189502443277505</v>
+      </c>
+      <c r="BD131">
+        <v>-2450.078072530424</v>
+      </c>
+      <c r="BE131">
+        <v>-84.22816562961268</v>
+      </c>
+      <c r="BF131">
+        <v>4704</v>
+      </c>
+      <c r="BG131">
+        <v>3545</v>
+      </c>
+      <c r="BH131">
+        <v>949.8333333333334</v>
+      </c>
+      <c r="BI131">
+        <v>6852</v>
+      </c>
+      <c r="BJ131">
+        <v>4278</v>
+      </c>
+      <c r="BK131">
+        <v>11556</v>
+      </c>
+      <c r="BL131">
+        <v>7823</v>
+      </c>
+      <c r="BM131">
+        <v>4585</v>
+      </c>
+      <c r="BN131">
+        <v>3519</v>
+      </c>
+      <c r="BO131">
+        <v>4657</v>
+      </c>
+      <c r="BP131">
+        <v>3518</v>
+      </c>
+      <c r="BQ131">
+        <v>2267</v>
+      </c>
+      <c r="BR131">
+        <v>759</v>
+      </c>
+      <c r="BS131">
+        <v>47</v>
+      </c>
+      <c r="BT131">
+        <v>27</v>
+      </c>
+      <c r="BU131">
+        <v>0</v>
+      </c>
+      <c r="BV131">
+        <v>0</v>
+      </c>
+      <c r="BW131">
+        <v>25661.49036379996</v>
+      </c>
+      <c r="BX131">
+        <v>6659.312706200015</v>
+      </c>
+      <c r="BY131">
+        <v>0.04965626675578699</v>
+      </c>
+      <c r="BZ131">
+        <v>0.08680051762198861</v>
+      </c>
+      <c r="CA131">
+        <v>0.132084447379597</v>
+      </c>
+      <c r="CB131">
+        <v>0.1255909306850455</v>
+      </c>
+      <c r="CC131">
+        <v>0.009041564726442719</v>
+      </c>
+      <c r="CD131">
+        <v>0.01578562667923071</v>
+      </c>
+      <c r="CE131">
+        <v>0.009649947442705817</v>
+      </c>
+      <c r="CF131">
+        <v>0.01593983778482089</v>
+      </c>
+      <c r="CG131">
+        <v>27161.54219999996</v>
+      </c>
+      <c r="CH131">
+        <v>6996.729600000015</v>
+      </c>
+      <c r="CI131">
+        <v>29611.62027253039</v>
+      </c>
+      <c r="CJ131">
+        <v>7080.957765629628</v>
+      </c>
+      <c r="CK131">
+        <v>0.1670495380138063</v>
+      </c>
+      <c r="CL131">
+        <v>0.09637602883577172</v>
+      </c>
+      <c r="CM131">
+        <v>10000</v>
+      </c>
+      <c r="CO131">
+        <v>0.00307057946220994</v>
+      </c>
+      <c r="CP131">
+        <v>0.009650392595516954</v>
+      </c>
+      <c r="CQ131">
+        <v>8177676.867132748</v>
+      </c>
+      <c r="CR131">
+        <v>1295517.443775632</v>
+      </c>
+      <c r="CS131" s="2">
+        <v>45418.65603952249</v>
+      </c>
+      <c r="CT131">
+        <v>-0.7832286955751367</v>
+      </c>
+      <c r="CU131">
+        <v>-0.8805073825476633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update RSRUSDT.json at 2024-05-07_07-25-06 bestfile_scores 0.0006258996119161641 bestfile_sharp 0.1290194200835246
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1074" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU131"/>
+  <dimension ref="A1:CU132"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -37751,6 +37751,275 @@
       </c>
       <c r="CU131">
         <v>-0.8805073825476633</v>
+      </c>
+    </row>
+    <row r="132" spans="10:99">
+      <c r="J132" t="s">
+        <v>238</v>
+      </c>
+      <c r="K132">
+        <v>0.001619052131043075</v>
+      </c>
+      <c r="L132">
+        <v>0.0008095260655215375</v>
+      </c>
+      <c r="M132">
+        <v>0.0004849124586081555</v>
+      </c>
+      <c r="N132">
+        <v>0.0004849124586081555</v>
+      </c>
+      <c r="O132">
+        <v>0.002865906751505731</v>
+      </c>
+      <c r="P132">
+        <v>0.001432953375752866</v>
+      </c>
+      <c r="Q132">
+        <v>0.0003753074203771467</v>
+      </c>
+      <c r="R132">
+        <v>0.0003753074203771467</v>
+      </c>
+      <c r="S132">
+        <v>49.23430687912342</v>
+      </c>
+      <c r="T132">
+        <v>74.98067055056137</v>
+      </c>
+      <c r="U132">
+        <v>0.3909150932809125</v>
+      </c>
+      <c r="V132">
+        <v>0.6491882734410773</v>
+      </c>
+      <c r="W132">
+        <v>0.04742909684571316</v>
+      </c>
+      <c r="X132">
+        <v>0.06399019998004046</v>
+      </c>
+      <c r="Y132">
+        <v>0.186720952377867</v>
+      </c>
+      <c r="Z132">
+        <v>0.1818627031253102</v>
+      </c>
+      <c r="AA132">
+        <v>0.9994451109296455</v>
+      </c>
+      <c r="AB132">
+        <v>0.8422885164857498</v>
+      </c>
+      <c r="AC132">
+        <v>0.8332007167684943</v>
+      </c>
+      <c r="AD132">
+        <v>0.9990874250882764</v>
+      </c>
+      <c r="AE132">
+        <v>0.8135737049923257</v>
+      </c>
+      <c r="AF132">
+        <v>0.8186404304999623</v>
+      </c>
+      <c r="AG132">
+        <v>0.005712984308084144</v>
+      </c>
+      <c r="AH132">
+        <v>0.007351154378554608</v>
+      </c>
+      <c r="AI132">
+        <v>0.9994451109296455</v>
+      </c>
+      <c r="AJ132">
+        <v>0.9990874250882764</v>
+      </c>
+      <c r="AK132">
+        <v>0.005712984308084144</v>
+      </c>
+      <c r="AL132">
+        <v>0.007351154378554608</v>
+      </c>
+      <c r="AM132" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN132">
+        <v>0.01714805100715212</v>
+      </c>
+      <c r="AO132">
+        <v>0.02867624612728114</v>
+      </c>
+      <c r="AP132">
+        <v>-7368.071834006001</v>
+      </c>
+      <c r="AQ132">
+        <v>-1909.67504913</v>
+      </c>
+      <c r="AR132">
+        <v>57379.09259599377</v>
+      </c>
+      <c r="AS132">
+        <v>16880.23505087064</v>
+      </c>
+      <c r="AT132">
+        <v>57379.09259599377</v>
+      </c>
+      <c r="AU132">
+        <v>16865.38760087064</v>
+      </c>
+      <c r="AV132">
+        <v>4.737909259599377</v>
+      </c>
+      <c r="AW132">
+        <v>0.6880235050870644</v>
+      </c>
+      <c r="AX132">
+        <v>0.4870180552943389</v>
+      </c>
+      <c r="AY132">
+        <v>0.319704847175054</v>
+      </c>
+      <c r="AZ132">
+        <v>59.98333333333333</v>
+      </c>
+      <c r="BA132">
+        <v>63.33333333333334</v>
+      </c>
+      <c r="BB132">
+        <v>0.004789157600066273</v>
+      </c>
+      <c r="BC132">
+        <v>0.03222183572129598</v>
+      </c>
+      <c r="BD132">
+        <v>-263.454523847167</v>
+      </c>
+      <c r="BE132">
+        <v>-292.6569845252222</v>
+      </c>
+      <c r="BF132">
+        <v>24666</v>
+      </c>
+      <c r="BG132">
+        <v>37799</v>
+      </c>
+      <c r="BH132">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI132">
+        <v>28505</v>
+      </c>
+      <c r="BJ132">
+        <v>43177</v>
+      </c>
+      <c r="BK132">
+        <v>53171</v>
+      </c>
+      <c r="BL132">
+        <v>80976</v>
+      </c>
+      <c r="BM132">
+        <v>24600</v>
+      </c>
+      <c r="BN132">
+        <v>37614</v>
+      </c>
+      <c r="BO132">
+        <v>24620</v>
+      </c>
+      <c r="BP132">
+        <v>37714</v>
+      </c>
+      <c r="BQ132">
+        <v>3905</v>
+      </c>
+      <c r="BR132">
+        <v>5563</v>
+      </c>
+      <c r="BS132">
+        <v>46</v>
+      </c>
+      <c r="BT132">
+        <v>85</v>
+      </c>
+      <c r="BU132">
+        <v>0</v>
+      </c>
+      <c r="BV132">
+        <v>0</v>
+      </c>
+      <c r="BW132">
+        <v>47379.09259599402</v>
+      </c>
+      <c r="BX132">
+        <v>6880.235050870009</v>
+      </c>
+      <c r="BY132">
+        <v>0.02765658510849759</v>
+      </c>
+      <c r="BZ132">
+        <v>0.06898786131825328</v>
+      </c>
+      <c r="CA132">
+        <v>0.1027690788009489</v>
+      </c>
+      <c r="CB132">
+        <v>0.1542030494708696</v>
+      </c>
+      <c r="CC132">
+        <v>0.005666643278276891</v>
+      </c>
+      <c r="CD132">
+        <v>0.00823534817457002</v>
+      </c>
+      <c r="CE132">
+        <v>0.005559434035218185</v>
+      </c>
+      <c r="CF132">
+        <v>0.0090508498302827</v>
+      </c>
+      <c r="CG132">
+        <v>54747.16443000002</v>
+      </c>
+      <c r="CH132">
+        <v>8789.91010000001</v>
+      </c>
+      <c r="CI132">
+        <v>55010.61895384719</v>
+      </c>
+      <c r="CJ132">
+        <v>9082.567084525232</v>
+      </c>
+      <c r="CK132">
+        <v>0.184462208922361</v>
+      </c>
+      <c r="CL132">
+        <v>0.07276783020470783</v>
+      </c>
+      <c r="CM132">
+        <v>10000</v>
+      </c>
+      <c r="CO132">
+        <v>0.008912037037037038</v>
+      </c>
+      <c r="CP132">
+        <v>0.01006944444444445</v>
+      </c>
+      <c r="CQ132">
+        <v>26666806.02181739</v>
+      </c>
+      <c r="CR132">
+        <v>7436893.530962305</v>
+      </c>
+      <c r="CS132" s="2">
+        <v>45419.14449996537</v>
+      </c>
+      <c r="CT132">
+        <v>-0.8091587172086132</v>
+      </c>
+      <c r="CU132">
+        <v>-0.8505270497746833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ZECUSDT.json at 2024-05-07_12-28-50 bestfile_scores 0.0008381739950074935 bestfile_sharp 0.23051896190871693
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU132"/>
+  <dimension ref="A1:CU133"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -38020,6 +38020,275 @@
       </c>
       <c r="CU132">
         <v>-0.8505270497746833</v>
+      </c>
+    </row>
+    <row r="133" spans="10:99">
+      <c r="J133" t="s">
+        <v>241</v>
+      </c>
+      <c r="K133">
+        <v>0.00109613729693403</v>
+      </c>
+      <c r="L133">
+        <v>0.000548068648467015</v>
+      </c>
+      <c r="M133">
+        <v>0.0003855285575780076</v>
+      </c>
+      <c r="N133">
+        <v>0.0003855285575780076</v>
+      </c>
+      <c r="O133">
+        <v>0.002113526564414414</v>
+      </c>
+      <c r="P133">
+        <v>0.001056763282207207</v>
+      </c>
+      <c r="Q133">
+        <v>0.000513237959412427</v>
+      </c>
+      <c r="R133">
+        <v>0.000513237959412427</v>
+      </c>
+      <c r="S133">
+        <v>6.797296775439275</v>
+      </c>
+      <c r="T133">
+        <v>2.696118941880672</v>
+      </c>
+      <c r="U133">
+        <v>0.4296603952494842</v>
+      </c>
+      <c r="V133">
+        <v>0.6158266826889449</v>
+      </c>
+      <c r="W133">
+        <v>0.02190812671745069</v>
+      </c>
+      <c r="X133">
+        <v>0.02930266156908121</v>
+      </c>
+      <c r="Y133">
+        <v>0.1006605505523412</v>
+      </c>
+      <c r="Z133">
+        <v>0.115378037190302</v>
+      </c>
+      <c r="AA133">
+        <v>0.9996795065910724</v>
+      </c>
+      <c r="AB133">
+        <v>0.9322605002468208</v>
+      </c>
+      <c r="AC133">
+        <v>0.9097093464615931</v>
+      </c>
+      <c r="AD133">
+        <v>0.9994606671523855</v>
+      </c>
+      <c r="AE133">
+        <v>0.8737986469747442</v>
+      </c>
+      <c r="AF133">
+        <v>0.8853173226108123</v>
+      </c>
+      <c r="AG133">
+        <v>0.002554463849785888</v>
+      </c>
+      <c r="AH133">
+        <v>0.003373041808746848</v>
+      </c>
+      <c r="AI133">
+        <v>0.9996795065910724</v>
+      </c>
+      <c r="AJ133">
+        <v>0.9994606671523855</v>
+      </c>
+      <c r="AK133">
+        <v>0.002554463849785888</v>
+      </c>
+      <c r="AL133">
+        <v>0.003373041808746848</v>
+      </c>
+      <c r="AM133" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN133">
+        <v>0.009616489085314019</v>
+      </c>
+      <c r="AO133">
+        <v>0.01397628572330174</v>
+      </c>
+      <c r="AP133">
+        <v>-758.5693892524</v>
+      </c>
+      <c r="AQ133">
+        <v>-126.149852718</v>
+      </c>
+      <c r="AR133">
+        <v>32610.15829274761</v>
+      </c>
+      <c r="AS133">
+        <v>15157.177460282</v>
+      </c>
+      <c r="AT133">
+        <v>32610.15829274761</v>
+      </c>
+      <c r="AU133">
+        <v>14902.212547282</v>
+      </c>
+      <c r="AV133">
+        <v>2.261015829274761</v>
+      </c>
+      <c r="AW133">
+        <v>0.5157177460281999</v>
+      </c>
+      <c r="AX133">
+        <v>3.527062593754261</v>
+      </c>
+      <c r="AY133">
+        <v>8.89139156350298</v>
+      </c>
+      <c r="AZ133">
+        <v>107.3333333333333</v>
+      </c>
+      <c r="BA133">
+        <v>112.3166666666667</v>
+      </c>
+      <c r="BB133">
+        <v>0.01085916950552062</v>
+      </c>
+      <c r="BC133">
+        <v>0.00789172942731734</v>
+      </c>
+      <c r="BD133">
+        <v>-256.5509047890893</v>
+      </c>
+      <c r="BE133">
+        <v>-42.02624941941458</v>
+      </c>
+      <c r="BF133">
+        <v>3001</v>
+      </c>
+      <c r="BG133">
+        <v>1172</v>
+      </c>
+      <c r="BH133">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI133">
+        <v>4333</v>
+      </c>
+      <c r="BJ133">
+        <v>1737</v>
+      </c>
+      <c r="BK133">
+        <v>7334</v>
+      </c>
+      <c r="BL133">
+        <v>2909</v>
+      </c>
+      <c r="BM133">
+        <v>2911</v>
+      </c>
+      <c r="BN133">
+        <v>1106</v>
+      </c>
+      <c r="BO133">
+        <v>2992</v>
+      </c>
+      <c r="BP133">
+        <v>1165</v>
+      </c>
+      <c r="BQ133">
+        <v>1422</v>
+      </c>
+      <c r="BR133">
+        <v>631</v>
+      </c>
+      <c r="BS133">
+        <v>9</v>
+      </c>
+      <c r="BT133">
+        <v>7</v>
+      </c>
+      <c r="BU133">
+        <v>0</v>
+      </c>
+      <c r="BV133">
+        <v>0</v>
+      </c>
+      <c r="BW133">
+        <v>22610.1582927476</v>
+      </c>
+      <c r="BX133">
+        <v>5157.177460282007</v>
+      </c>
+      <c r="BY133">
+        <v>0.03740348296837005</v>
+      </c>
+      <c r="BZ133">
+        <v>0.1019111071106316</v>
+      </c>
+      <c r="CA133">
+        <v>0.07487268591233054</v>
+      </c>
+      <c r="CB133">
+        <v>0.1673053259867567</v>
+      </c>
+      <c r="CC133">
+        <v>0.01231132187437749</v>
+      </c>
+      <c r="CD133">
+        <v>0.01875398931966051</v>
+      </c>
+      <c r="CE133">
+        <v>0.009624575333654458</v>
+      </c>
+      <c r="CF133">
+        <v>0.01810812085591623</v>
+      </c>
+      <c r="CG133">
+        <v>23368.727682</v>
+      </c>
+      <c r="CH133">
+        <v>5283.327313000007</v>
+      </c>
+      <c r="CI133">
+        <v>23625.27858678909</v>
+      </c>
+      <c r="CJ133">
+        <v>5325.353562419422</v>
+      </c>
+      <c r="CK133">
+        <v>0.1290194200835246</v>
+      </c>
+      <c r="CL133">
+        <v>0.06417092565268021</v>
+      </c>
+      <c r="CM133">
+        <v>10000</v>
+      </c>
+      <c r="CO133">
+        <v>0.0009654000617856039</v>
+      </c>
+      <c r="CP133">
+        <v>0.002587272165585418</v>
+      </c>
+      <c r="CQ133">
+        <v>4329727.394136436</v>
+      </c>
+      <c r="CR133">
+        <v>867003.1587181734</v>
+      </c>
+      <c r="CS133" s="2">
+        <v>45419.30912299596</v>
+      </c>
+      <c r="CT133">
+        <v>-0.9000180936758766</v>
+      </c>
+      <c r="CU133">
+        <v>-0.8989378715702173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update HNTUSDT.json at 2024-05-07_17-50-13 bestfile_scores 0.00045886020101453543 bestfile_sharp 0.23629281165583188
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU133"/>
+  <dimension ref="A1:CU134"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -38289,6 +38289,275 @@
       </c>
       <c r="CU133">
         <v>-0.8989378715702173</v>
+      </c>
+    </row>
+    <row r="134" spans="10:99">
+      <c r="J134" t="s">
+        <v>236</v>
+      </c>
+      <c r="K134">
+        <v>0.002101848400442918</v>
+      </c>
+      <c r="L134">
+        <v>0.001050924200221459</v>
+      </c>
+      <c r="M134">
+        <v>0.0006313105550932452</v>
+      </c>
+      <c r="N134">
+        <v>0.0006313105550932452</v>
+      </c>
+      <c r="O134">
+        <v>0.002227915942938385</v>
+      </c>
+      <c r="P134">
+        <v>0.001113957971469193</v>
+      </c>
+      <c r="Q134">
+        <v>0.0005565032532460767</v>
+      </c>
+      <c r="R134">
+        <v>0.0005565032532460767</v>
+      </c>
+      <c r="S134">
+        <v>11.08939949797258</v>
+      </c>
+      <c r="T134">
+        <v>17.26943425371693</v>
+      </c>
+      <c r="U134">
+        <v>0.3609445505025619</v>
+      </c>
+      <c r="V134">
+        <v>0.7628755660380135</v>
+      </c>
+      <c r="W134">
+        <v>0.07497471142276969</v>
+      </c>
+      <c r="X134">
+        <v>0.09191635575593667</v>
+      </c>
+      <c r="Y134">
+        <v>0.1819636019003284</v>
+      </c>
+      <c r="Z134">
+        <v>0.16595411714472</v>
+      </c>
+      <c r="AA134">
+        <v>0.9986188553281209</v>
+      </c>
+      <c r="AB134">
+        <v>0.8388196141906518</v>
+      </c>
+      <c r="AC134">
+        <v>0.8762201460207655</v>
+      </c>
+      <c r="AD134">
+        <v>0.9986760497381962</v>
+      </c>
+      <c r="AE134">
+        <v>0.8184393040007297</v>
+      </c>
+      <c r="AF134">
+        <v>0.8648435249412598</v>
+      </c>
+      <c r="AG134">
+        <v>0.008452667068119072</v>
+      </c>
+      <c r="AH134">
+        <v>0.0074087938346481</v>
+      </c>
+      <c r="AI134">
+        <v>0.9986188553281209</v>
+      </c>
+      <c r="AJ134">
+        <v>0.9986760497381962</v>
+      </c>
+      <c r="AK134">
+        <v>0.008452667068119072</v>
+      </c>
+      <c r="AL134">
+        <v>0.0074087938346481</v>
+      </c>
+      <c r="AM134" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN134">
+        <v>0.0409391807131387</v>
+      </c>
+      <c r="AO134">
+        <v>0.04359215015688549</v>
+      </c>
+      <c r="AP134">
+        <v>-3992.23056225</v>
+      </c>
+      <c r="AQ134">
+        <v>-582.436653732</v>
+      </c>
+      <c r="AR134">
+        <v>96352.36892775018</v>
+      </c>
+      <c r="AS134">
+        <v>19757.39707626811</v>
+      </c>
+      <c r="AT134">
+        <v>96346.46882775018</v>
+      </c>
+      <c r="AU134">
+        <v>19560.63988626811</v>
+      </c>
+      <c r="AV134">
+        <v>8.635236892775019</v>
+      </c>
+      <c r="AW134">
+        <v>0.9757397076268113</v>
+      </c>
+      <c r="AX134">
+        <v>2.157427839072774</v>
+      </c>
+      <c r="AY134">
+        <v>1.38510895234006</v>
+      </c>
+      <c r="AZ134">
+        <v>119.0666666666667</v>
+      </c>
+      <c r="BA134">
+        <v>112.9833333333333</v>
+      </c>
+      <c r="BB134">
+        <v>0.00671778289806858</v>
+      </c>
+      <c r="BC134">
+        <v>0.07546925217090274</v>
+      </c>
+      <c r="BD134">
+        <v>-611.0201058039232</v>
+      </c>
+      <c r="BE134">
+        <v>-844.0384714157984</v>
+      </c>
+      <c r="BF134">
+        <v>3550</v>
+      </c>
+      <c r="BG134">
+        <v>6781</v>
+      </c>
+      <c r="BH134">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI134">
+        <v>8415</v>
+      </c>
+      <c r="BJ134">
+        <v>11852</v>
+      </c>
+      <c r="BK134">
+        <v>11965</v>
+      </c>
+      <c r="BL134">
+        <v>18633</v>
+      </c>
+      <c r="BM134">
+        <v>3292</v>
+      </c>
+      <c r="BN134">
+        <v>6772</v>
+      </c>
+      <c r="BO134">
+        <v>3539</v>
+      </c>
+      <c r="BP134">
+        <v>6772</v>
+      </c>
+      <c r="BQ134">
+        <v>5123</v>
+      </c>
+      <c r="BR134">
+        <v>5080</v>
+      </c>
+      <c r="BS134">
+        <v>11</v>
+      </c>
+      <c r="BT134">
+        <v>9</v>
+      </c>
+      <c r="BU134">
+        <v>0</v>
+      </c>
+      <c r="BV134">
+        <v>0</v>
+      </c>
+      <c r="BW134">
+        <v>86352.36892775004</v>
+      </c>
+      <c r="BX134">
+        <v>9757.397076268004</v>
+      </c>
+      <c r="BY134">
+        <v>0.04261636952293211</v>
+      </c>
+      <c r="BZ134">
+        <v>0.07123040629672342</v>
+      </c>
+      <c r="CA134">
+        <v>0.09984147157001007</v>
+      </c>
+      <c r="CB134">
+        <v>0.1204562214465475</v>
+      </c>
+      <c r="CC134">
+        <v>0.008774411655161492</v>
+      </c>
+      <c r="CD134">
+        <v>0.01139401041874235</v>
+      </c>
+      <c r="CE134">
+        <v>0.00794777925724508</v>
+      </c>
+      <c r="CF134">
+        <v>0.009742705404139029</v>
+      </c>
+      <c r="CG134">
+        <v>90344.59949000004</v>
+      </c>
+      <c r="CH134">
+        <v>10339.83373</v>
+      </c>
+      <c r="CI134">
+        <v>90955.61959580396</v>
+      </c>
+      <c r="CJ134">
+        <v>11183.8722014158</v>
+      </c>
+      <c r="CK134">
+        <v>0.2305189619087169</v>
+      </c>
+      <c r="CL134">
+        <v>0.08413465918659893</v>
+      </c>
+      <c r="CM134">
+        <v>10000</v>
+      </c>
+      <c r="CO134">
+        <v>0.01015600864998455</v>
+      </c>
+      <c r="CP134">
+        <v>0.008611368551127587</v>
+      </c>
+      <c r="CQ134">
+        <v>66742737.91777743</v>
+      </c>
+      <c r="CR134">
+        <v>3390202.150984915</v>
+      </c>
+      <c r="CS134" s="2">
+        <v>45419.52005372911</v>
+      </c>
+      <c r="CT134">
+        <v>-0.6893066803315582</v>
+      </c>
+      <c r="CU134">
+        <v>-0.8315269425441832</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ENSUSDT.json at 2024-05-07_23-17-23 bestfile_scores 0.0016640323351273523 bestfile_sharp 0.13749305769804276
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU134"/>
+  <dimension ref="A1:CU135"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -38558,6 +38558,275 @@
       </c>
       <c r="CU134">
         <v>-0.8315269425441832</v>
+      </c>
+    </row>
+    <row r="135" spans="10:99">
+      <c r="J135" t="s">
+        <v>242</v>
+      </c>
+      <c r="K135">
+        <v>0.001848957601374712</v>
+      </c>
+      <c r="L135">
+        <v>0.0009244788006873561</v>
+      </c>
+      <c r="M135">
+        <v>0.0006897374777841137</v>
+      </c>
+      <c r="N135">
+        <v>0.0006897374777841137</v>
+      </c>
+      <c r="O135">
+        <v>0.0002519402379465907</v>
+      </c>
+      <c r="P135">
+        <v>0.0001259701189732953</v>
+      </c>
+      <c r="Q135">
+        <v>9.525440661337648E-05</v>
+      </c>
+      <c r="R135">
+        <v>9.525440661337648E-05</v>
+      </c>
+      <c r="S135">
+        <v>1.318569389251129</v>
+      </c>
+      <c r="T135">
+        <v>11.76156487518809</v>
+      </c>
+      <c r="U135">
+        <v>0.3620987196628432</v>
+      </c>
+      <c r="V135">
+        <v>0.6240297615846883</v>
+      </c>
+      <c r="W135">
+        <v>0.04483228600930598</v>
+      </c>
+      <c r="X135">
+        <v>0.08392388039386765</v>
+      </c>
+      <c r="Y135">
+        <v>0.2375959329469452</v>
+      </c>
+      <c r="Z135">
+        <v>0.2022545722996491</v>
+      </c>
+      <c r="AA135">
+        <v>1.000313892475625</v>
+      </c>
+      <c r="AB135">
+        <v>0.825763021135087</v>
+      </c>
+      <c r="AC135">
+        <v>0.8297340005497663</v>
+      </c>
+      <c r="AD135">
+        <v>0.9989870165198325</v>
+      </c>
+      <c r="AE135">
+        <v>0.7627092298595899</v>
+      </c>
+      <c r="AF135">
+        <v>0.7978945436031236</v>
+      </c>
+      <c r="AG135">
+        <v>0.006220720603331166</v>
+      </c>
+      <c r="AH135">
+        <v>0.008384924165057999</v>
+      </c>
+      <c r="AI135">
+        <v>1.000313892475625</v>
+      </c>
+      <c r="AJ135">
+        <v>0.9989870165198325</v>
+      </c>
+      <c r="AK135">
+        <v>0.006220720603331166</v>
+      </c>
+      <c r="AL135">
+        <v>0.008384924165057999</v>
+      </c>
+      <c r="AM135" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN135">
+        <v>0.0422126511911422</v>
+      </c>
+      <c r="AO135">
+        <v>0.02670053916945107</v>
+      </c>
+      <c r="AP135">
+        <v>-2577.8704428</v>
+      </c>
+      <c r="AQ135">
+        <v>-458.5997903000001</v>
+      </c>
+      <c r="AR135">
+        <v>73518.60755720014</v>
+      </c>
+      <c r="AS135">
+        <v>21056.64230969984</v>
+      </c>
+      <c r="AT135">
+        <v>73676.66855720014</v>
+      </c>
+      <c r="AU135">
+        <v>21056.64230969984</v>
+      </c>
+      <c r="AV135">
+        <v>6.351860755720014</v>
+      </c>
+      <c r="AW135">
+        <v>1.105664230969984</v>
+      </c>
+      <c r="AX135">
+        <v>11.20309205903022</v>
+      </c>
+      <c r="AY135">
+        <v>1.255911608009868</v>
+      </c>
+      <c r="AZ135">
+        <v>287.15</v>
+      </c>
+      <c r="BA135">
+        <v>67.76666666666667</v>
+      </c>
+      <c r="BB135">
+        <v>2.37308580809025E-05</v>
+      </c>
+      <c r="BC135">
+        <v>0.1380446255025033</v>
+      </c>
+      <c r="BD135">
+        <v>-1.56856336242004</v>
+      </c>
+      <c r="BE135">
+        <v>-1844.199050550466</v>
+      </c>
+      <c r="BF135">
+        <v>643</v>
+      </c>
+      <c r="BG135">
+        <v>3682</v>
+      </c>
+      <c r="BH135">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI135">
+        <v>781</v>
+      </c>
+      <c r="BJ135">
+        <v>9020</v>
+      </c>
+      <c r="BK135">
+        <v>1424</v>
+      </c>
+      <c r="BL135">
+        <v>12702</v>
+      </c>
+      <c r="BM135">
+        <v>639</v>
+      </c>
+      <c r="BN135">
+        <v>3425</v>
+      </c>
+      <c r="BO135">
+        <v>640</v>
+      </c>
+      <c r="BP135">
+        <v>3635</v>
+      </c>
+      <c r="BQ135">
+        <v>142</v>
+      </c>
+      <c r="BR135">
+        <v>5595</v>
+      </c>
+      <c r="BS135">
+        <v>3</v>
+      </c>
+      <c r="BT135">
+        <v>47</v>
+      </c>
+      <c r="BU135">
+        <v>0</v>
+      </c>
+      <c r="BV135">
+        <v>0</v>
+      </c>
+      <c r="BW135">
+        <v>63518.60755720003</v>
+      </c>
+      <c r="BX135">
+        <v>11056.64230969996</v>
+      </c>
+      <c r="BY135">
+        <v>0.03684354716871903</v>
+      </c>
+      <c r="BZ135">
+        <v>0.06940029673870404</v>
+      </c>
+      <c r="CA135">
+        <v>0.1345163957012951</v>
+      </c>
+      <c r="CB135">
+        <v>0.1681132500281438</v>
+      </c>
+      <c r="CC135">
+        <v>0.01352934217609617</v>
+      </c>
+      <c r="CD135">
+        <v>0.01247992650366996</v>
+      </c>
+      <c r="CE135">
+        <v>0.004839755024427521</v>
+      </c>
+      <c r="CF135">
+        <v>0.01151226577087958</v>
+      </c>
+      <c r="CG135">
+        <v>66096.47800000003</v>
+      </c>
+      <c r="CH135">
+        <v>11515.24209999996</v>
+      </c>
+      <c r="CI135">
+        <v>66098.04656336246</v>
+      </c>
+      <c r="CJ135">
+        <v>13359.44115055043</v>
+      </c>
+      <c r="CK135">
+        <v>0.2362928116558319</v>
+      </c>
+      <c r="CL135">
+        <v>0.06475128703067912</v>
+      </c>
+      <c r="CM135">
+        <v>10000</v>
+      </c>
+      <c r="CO135">
+        <v>0.006790123456790123</v>
+      </c>
+      <c r="CP135">
+        <v>0.01053240740740741</v>
+      </c>
+      <c r="CQ135">
+        <v>7948953.840563923</v>
+      </c>
+      <c r="CR135">
+        <v>8715912.703511165</v>
+      </c>
+      <c r="CS135" s="2">
+        <v>45419.7432346184</v>
+      </c>
+      <c r="CT135">
+        <v>-0.8034449984146571</v>
+      </c>
+      <c r="CU135">
+        <v>-0.6787553663736624</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update OCEANUSDT.json at 2024-05-08_04-21-53 bestfile_scores 0.0010264438880224712 bestfile_sharp 0.21243705432646331
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU135"/>
+  <dimension ref="A1:CU136"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -38827,6 +38827,275 @@
       </c>
       <c r="CU135">
         <v>-0.6787553663736624</v>
+      </c>
+    </row>
+    <row r="136" spans="10:99">
+      <c r="J136" t="s">
+        <v>197</v>
+      </c>
+      <c r="K136">
+        <v>0.001564964211886233</v>
+      </c>
+      <c r="L136">
+        <v>0.0007824821059431164</v>
+      </c>
+      <c r="M136">
+        <v>0.001934162331862277</v>
+      </c>
+      <c r="N136">
+        <v>0.001934162331862277</v>
+      </c>
+      <c r="O136">
+        <v>0.003644722717055559</v>
+      </c>
+      <c r="P136">
+        <v>0.00182236135852778</v>
+      </c>
+      <c r="Q136">
+        <v>0.002117123544176236</v>
+      </c>
+      <c r="R136">
+        <v>0.002117123544176236</v>
+      </c>
+      <c r="S136">
+        <v>11.14382148884305</v>
+      </c>
+      <c r="T136">
+        <v>13.8203637727358</v>
+      </c>
+      <c r="U136">
+        <v>0.4172793261047438</v>
+      </c>
+      <c r="V136">
+        <v>0.6954412932967299</v>
+      </c>
+      <c r="W136">
+        <v>0.06660305564760288</v>
+      </c>
+      <c r="X136">
+        <v>0.07428647687703471</v>
+      </c>
+      <c r="Y136">
+        <v>0.181465014282819</v>
+      </c>
+      <c r="Z136">
+        <v>0.1813368999734138</v>
+      </c>
+      <c r="AA136">
+        <v>0.999200058456911</v>
+      </c>
+      <c r="AB136">
+        <v>0.8341440188953619</v>
+      </c>
+      <c r="AC136">
+        <v>0.8476045088759191</v>
+      </c>
+      <c r="AD136">
+        <v>0.9988154694670831</v>
+      </c>
+      <c r="AE136">
+        <v>0.7220270555159511</v>
+      </c>
+      <c r="AF136">
+        <v>0.8225972088743163</v>
+      </c>
+      <c r="AG136">
+        <v>0.006047226374347921</v>
+      </c>
+      <c r="AH136">
+        <v>0.008401051909799786</v>
+      </c>
+      <c r="AI136">
+        <v>0.999200058456911</v>
+      </c>
+      <c r="AJ136">
+        <v>0.9988154694670831</v>
+      </c>
+      <c r="AK136">
+        <v>0.006047226374347921</v>
+      </c>
+      <c r="AL136">
+        <v>0.008401051909799786</v>
+      </c>
+      <c r="AM136" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN136">
+        <v>0.02071059035954705</v>
+      </c>
+      <c r="AO136">
+        <v>0.03916270565598065</v>
+      </c>
+      <c r="AP136">
+        <v>-947.5506029400001</v>
+      </c>
+      <c r="AQ136">
+        <v>-2329.87511666</v>
+      </c>
+      <c r="AR136">
+        <v>40144.68919706011</v>
+      </c>
+      <c r="AS136">
+        <v>55705.15158333984</v>
+      </c>
+      <c r="AT136">
+        <v>40087.18569706011</v>
+      </c>
+      <c r="AU136">
+        <v>55705.15158333984</v>
+      </c>
+      <c r="AV136">
+        <v>3.014468919706012</v>
+      </c>
+      <c r="AW136">
+        <v>4.570515158333984</v>
+      </c>
+      <c r="AX136">
+        <v>2.152194399569197</v>
+      </c>
+      <c r="AY136">
+        <v>1.734064696463947</v>
+      </c>
+      <c r="AZ136">
+        <v>115.2333333333333</v>
+      </c>
+      <c r="BA136">
+        <v>108.55</v>
+      </c>
+      <c r="BB136">
+        <v>0.03146441057511846</v>
+      </c>
+      <c r="BC136">
+        <v>0.01388779845003036</v>
+      </c>
+      <c r="BD136">
+        <v>-1010.080589137829</v>
+      </c>
+      <c r="BE136">
+        <v>-676.4958067681125</v>
+      </c>
+      <c r="BF136">
+        <v>3852</v>
+      </c>
+      <c r="BG136">
+        <v>5432</v>
+      </c>
+      <c r="BH136">
+        <v>888.8333333333334</v>
+      </c>
+      <c r="BI136">
+        <v>6053</v>
+      </c>
+      <c r="BJ136">
+        <v>6852</v>
+      </c>
+      <c r="BK136">
+        <v>9905</v>
+      </c>
+      <c r="BL136">
+        <v>12284</v>
+      </c>
+      <c r="BM136">
+        <v>3491</v>
+      </c>
+      <c r="BN136">
+        <v>4852</v>
+      </c>
+      <c r="BO136">
+        <v>3813</v>
+      </c>
+      <c r="BP136">
+        <v>5319</v>
+      </c>
+      <c r="BQ136">
+        <v>2562</v>
+      </c>
+      <c r="BR136">
+        <v>2000</v>
+      </c>
+      <c r="BS136">
+        <v>39</v>
+      </c>
+      <c r="BT136">
+        <v>113</v>
+      </c>
+      <c r="BU136">
+        <v>0</v>
+      </c>
+      <c r="BV136">
+        <v>0</v>
+      </c>
+      <c r="BW136">
+        <v>30144.68919705999</v>
+      </c>
+      <c r="BX136">
+        <v>45705.15158333995</v>
+      </c>
+      <c r="BY136">
+        <v>0.04350067991540129</v>
+      </c>
+      <c r="BZ136">
+        <v>0.07252438773486469</v>
+      </c>
+      <c r="CA136">
+        <v>0.09956682142091351</v>
+      </c>
+      <c r="CB136">
+        <v>0.1552798022947827</v>
+      </c>
+      <c r="CC136">
+        <v>0.01351076095108594</v>
+      </c>
+      <c r="CD136">
+        <v>0.009159890304105233</v>
+      </c>
+      <c r="CE136">
+        <v>0.009959032424960084</v>
+      </c>
+      <c r="CF136">
+        <v>0.01079765222490636</v>
+      </c>
+      <c r="CG136">
+        <v>31092.23979999998</v>
+      </c>
+      <c r="CH136">
+        <v>48035.02669999995</v>
+      </c>
+      <c r="CI136">
+        <v>32102.32038913781</v>
+      </c>
+      <c r="CJ136">
+        <v>48711.52250676807</v>
+      </c>
+      <c r="CK136">
+        <v>0.1374930576980428</v>
+      </c>
+      <c r="CL136">
+        <v>0.1781842249304145</v>
+      </c>
+      <c r="CM136">
+        <v>10000</v>
+      </c>
+      <c r="CO136">
+        <v>0.003515679932498945</v>
+      </c>
+      <c r="CP136">
+        <v>0.02526601978155909</v>
+      </c>
+      <c r="CQ136">
+        <v>12244854.11437261</v>
+      </c>
+      <c r="CR136">
+        <v>15549669.36335931</v>
+      </c>
+      <c r="CS136" s="2">
+        <v>45419.97042807396</v>
+      </c>
+      <c r="CT136">
+        <v>-0.8182238609422743</v>
+      </c>
+      <c r="CU136">
+        <v>-0.6710409609013362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update COMPUSDT.json at 2024-05-08_12-46-00 bestfile_scores 0.0006659242816574595 bestfile_sharp 0.16567858772048902
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU136"/>
+  <dimension ref="A1:CU137"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -39096,6 +39096,275 @@
       </c>
       <c r="CU136">
         <v>-0.6710409609013362</v>
+      </c>
+    </row>
+    <row r="137" spans="10:99">
+      <c r="J137" t="s">
+        <v>193</v>
+      </c>
+      <c r="K137">
+        <v>0.001217491149924532</v>
+      </c>
+      <c r="L137">
+        <v>0.0006087455749622661</v>
+      </c>
+      <c r="M137">
+        <v>0.001184876067757301</v>
+      </c>
+      <c r="N137">
+        <v>0.001184876067757301</v>
+      </c>
+      <c r="O137">
+        <v>0.001673189857006729</v>
+      </c>
+      <c r="P137">
+        <v>0.0008365949285033647</v>
+      </c>
+      <c r="Q137">
+        <v>0.001475558980866953</v>
+      </c>
+      <c r="R137">
+        <v>0.001475558980866953</v>
+      </c>
+      <c r="S137">
+        <v>22.96755276052317</v>
+      </c>
+      <c r="T137">
+        <v>10.03094255179598</v>
+      </c>
+      <c r="U137">
+        <v>0.3427582819226099</v>
+      </c>
+      <c r="V137">
+        <v>0.6490382772370177</v>
+      </c>
+      <c r="W137">
+        <v>0.03941166836131144</v>
+      </c>
+      <c r="X137">
+        <v>0.08420756506361381</v>
+      </c>
+      <c r="Y137">
+        <v>0.2451823427515543</v>
+      </c>
+      <c r="Z137">
+        <v>0.1799211959084611</v>
+      </c>
+      <c r="AA137">
+        <v>0.9993037129652775</v>
+      </c>
+      <c r="AB137">
+        <v>0.8135701670258909</v>
+      </c>
+      <c r="AC137">
+        <v>0.8447918632195609</v>
+      </c>
+      <c r="AD137">
+        <v>0.9989020543192647</v>
+      </c>
+      <c r="AE137">
+        <v>0.7622756828827902</v>
+      </c>
+      <c r="AF137">
+        <v>0.8202428385925584</v>
+      </c>
+      <c r="AG137">
+        <v>0.00531010094103464</v>
+      </c>
+      <c r="AH137">
+        <v>0.007733055159483883</v>
+      </c>
+      <c r="AI137">
+        <v>0.9993037129652775</v>
+      </c>
+      <c r="AJ137">
+        <v>0.9989020543192647</v>
+      </c>
+      <c r="AK137">
+        <v>0.00531010094103464</v>
+      </c>
+      <c r="AL137">
+        <v>0.007733055159483883</v>
+      </c>
+      <c r="AM137" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN137">
+        <v>0.01907285100274631</v>
+      </c>
+      <c r="AO137">
+        <v>0.03386295006012625</v>
+      </c>
+      <c r="AP137">
+        <v>-1700.99573232</v>
+      </c>
+      <c r="AQ137">
+        <v>-1134.343039136</v>
+      </c>
+      <c r="AR137">
+        <v>37211.76788767998</v>
+      </c>
+      <c r="AS137">
+        <v>35925.39334566384</v>
+      </c>
+      <c r="AT137">
+        <v>37210.27588767998</v>
+      </c>
+      <c r="AU137">
+        <v>35926.00054566384</v>
+      </c>
+      <c r="AV137">
+        <v>2.721176788767998</v>
+      </c>
+      <c r="AW137">
+        <v>2.592539334566384</v>
+      </c>
+      <c r="AX137">
+        <v>1.044791624669059</v>
+      </c>
+      <c r="AY137">
+        <v>2.390108013293944</v>
+      </c>
+      <c r="AZ137">
+        <v>119.4</v>
+      </c>
+      <c r="BA137">
+        <v>96.41666666666667</v>
+      </c>
+      <c r="BB137">
+        <v>0.04955123066412238</v>
+      </c>
+      <c r="BC137">
+        <v>0.05917543686255724</v>
+      </c>
+      <c r="BD137">
+        <v>-1507.354278834968</v>
+      </c>
+      <c r="BE137">
+        <v>-1702.111445414625</v>
+      </c>
+      <c r="BF137">
+        <v>8739</v>
+      </c>
+      <c r="BG137">
+        <v>4063</v>
+      </c>
+      <c r="BH137">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI137">
+        <v>16065</v>
+      </c>
+      <c r="BJ137">
+        <v>6770</v>
+      </c>
+      <c r="BK137">
+        <v>24804</v>
+      </c>
+      <c r="BL137">
+        <v>10833</v>
+      </c>
+      <c r="BM137">
+        <v>8618</v>
+      </c>
+      <c r="BN137">
+        <v>3611</v>
+      </c>
+      <c r="BO137">
+        <v>8716</v>
+      </c>
+      <c r="BP137">
+        <v>3924</v>
+      </c>
+      <c r="BQ137">
+        <v>7447</v>
+      </c>
+      <c r="BR137">
+        <v>3159</v>
+      </c>
+      <c r="BS137">
+        <v>23</v>
+      </c>
+      <c r="BT137">
+        <v>139</v>
+      </c>
+      <c r="BU137">
+        <v>0</v>
+      </c>
+      <c r="BV137">
+        <v>0</v>
+      </c>
+      <c r="BW137">
+        <v>27211.76788767998</v>
+      </c>
+      <c r="BX137">
+        <v>25927.362660864</v>
+      </c>
+      <c r="BY137">
+        <v>0.03659170191701504</v>
+      </c>
+      <c r="BZ137">
+        <v>0.07486011898151482</v>
+      </c>
+      <c r="CA137">
+        <v>0.1348926464408769</v>
+      </c>
+      <c r="CB137">
+        <v>0.1523531788027705</v>
+      </c>
+      <c r="CC137">
+        <v>0.01125470134018188</v>
+      </c>
+      <c r="CD137">
+        <v>0.009550008042014151</v>
+      </c>
+      <c r="CE137">
+        <v>0.00832321001373682</v>
+      </c>
+      <c r="CF137">
+        <v>0.01342814664270862</v>
+      </c>
+      <c r="CG137">
+        <v>28912.76361999998</v>
+      </c>
+      <c r="CH137">
+        <v>27061.70570000001</v>
+      </c>
+      <c r="CI137">
+        <v>30420.11789883495</v>
+      </c>
+      <c r="CJ137">
+        <v>28763.81714541463</v>
+      </c>
+      <c r="CK137">
+        <v>0.2124370543264633</v>
+      </c>
+      <c r="CL137">
+        <v>0.1605069873709463</v>
+      </c>
+      <c r="CM137">
+        <v>10000</v>
+      </c>
+      <c r="CO137">
+        <v>0.002083333333333333</v>
+      </c>
+      <c r="CP137">
+        <v>0.01084104938271605</v>
+      </c>
+      <c r="CQ137">
+        <v>21761654.04353544</v>
+      </c>
+      <c r="CR137">
+        <v>8185952.559251163</v>
+      </c>
+      <c r="CS137" s="2">
+        <v>45420.18189431339</v>
+      </c>
+      <c r="CT137">
+        <v>-0.8729982178980289</v>
+      </c>
+      <c r="CU137">
+        <v>-0.7970453694758551</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update AUDIOUSDT.json at 2024-05-08_17-49-51 bestfile_scores 0.000501503197691 bestfile_sharp 0.07840001921789688
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1086" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU137"/>
+  <dimension ref="A1:CU138"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -39365,6 +39365,275 @@
       </c>
       <c r="CU137">
         <v>-0.7970453694758551</v>
+      </c>
+    </row>
+    <row r="138" spans="10:99">
+      <c r="J138" t="s">
+        <v>218</v>
+      </c>
+      <c r="K138">
+        <v>0.001616295145627999</v>
+      </c>
+      <c r="L138">
+        <v>0.0008081475728139997</v>
+      </c>
+      <c r="M138">
+        <v>0.0005424826786097903</v>
+      </c>
+      <c r="N138">
+        <v>0.0005424826786097903</v>
+      </c>
+      <c r="O138">
+        <v>0.001638286806134648</v>
+      </c>
+      <c r="P138">
+        <v>0.0008191434030673239</v>
+      </c>
+      <c r="Q138">
+        <v>0.0004939234721387242</v>
+      </c>
+      <c r="R138">
+        <v>0.0004939234721387242</v>
+      </c>
+      <c r="S138">
+        <v>12.24607067001352</v>
+      </c>
+      <c r="T138">
+        <v>6.21525391002124</v>
+      </c>
+      <c r="U138">
+        <v>0.3641976643148658</v>
+      </c>
+      <c r="V138">
+        <v>0.5985076305299992</v>
+      </c>
+      <c r="W138">
+        <v>0.09974849098706609</v>
+      </c>
+      <c r="X138">
+        <v>0.09922477486083482</v>
+      </c>
+      <c r="Y138">
+        <v>0.210038073330966</v>
+      </c>
+      <c r="Z138">
+        <v>0.239814662913279</v>
+      </c>
+      <c r="AA138">
+        <v>0.9984001233491039</v>
+      </c>
+      <c r="AB138">
+        <v>0.8308989142500899</v>
+      </c>
+      <c r="AC138">
+        <v>0.785443057028523</v>
+      </c>
+      <c r="AD138">
+        <v>0.9981128241810232</v>
+      </c>
+      <c r="AE138">
+        <v>0.7903062253854946</v>
+      </c>
+      <c r="AF138">
+        <v>0.7605786850402809</v>
+      </c>
+      <c r="AG138">
+        <v>0.009786131271804402</v>
+      </c>
+      <c r="AH138">
+        <v>0.01089881053102703</v>
+      </c>
+      <c r="AI138">
+        <v>0.9984001233491039</v>
+      </c>
+      <c r="AJ138">
+        <v>0.9981128241810232</v>
+      </c>
+      <c r="AK138">
+        <v>0.009786131271804402</v>
+      </c>
+      <c r="AL138">
+        <v>0.01089881053102703</v>
+      </c>
+      <c r="AM138" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN138">
+        <v>0.03502844843258101</v>
+      </c>
+      <c r="AO138">
+        <v>0.04133791735064998</v>
+      </c>
+      <c r="AP138">
+        <v>-1999.707157332</v>
+      </c>
+      <c r="AQ138">
+        <v>-393.063430352</v>
+      </c>
+      <c r="AR138">
+        <v>57116.46252310804</v>
+      </c>
+      <c r="AS138">
+        <v>17952.73722964806</v>
+      </c>
+      <c r="AT138">
+        <v>57065.70149310803</v>
+      </c>
+      <c r="AU138">
+        <v>17952.73722964806</v>
+      </c>
+      <c r="AV138">
+        <v>4.711646252310803</v>
+      </c>
+      <c r="AW138">
+        <v>0.7952737229648064</v>
+      </c>
+      <c r="AX138">
+        <v>1.957552477545665</v>
+      </c>
+      <c r="AY138">
+        <v>3.857129008202834</v>
+      </c>
+      <c r="AZ138">
+        <v>102.1333333333333</v>
+      </c>
+      <c r="BA138">
+        <v>109.9833333333333</v>
+      </c>
+      <c r="BB138">
+        <v>0.07403854728522574</v>
+      </c>
+      <c r="BC138">
+        <v>0.003762263843969289</v>
+      </c>
+      <c r="BD138">
+        <v>-3927.248035266852</v>
+      </c>
+      <c r="BE138">
+        <v>-31.51768190717812</v>
+      </c>
+      <c r="BF138">
+        <v>4652</v>
+      </c>
+      <c r="BG138">
+        <v>2807</v>
+      </c>
+      <c r="BH138">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI138">
+        <v>8561</v>
+      </c>
+      <c r="BJ138">
+        <v>3899</v>
+      </c>
+      <c r="BK138">
+        <v>13213</v>
+      </c>
+      <c r="BL138">
+        <v>6706</v>
+      </c>
+      <c r="BM138">
+        <v>4262</v>
+      </c>
+      <c r="BN138">
+        <v>2786</v>
+      </c>
+      <c r="BO138">
+        <v>4608</v>
+      </c>
+      <c r="BP138">
+        <v>2793</v>
+      </c>
+      <c r="BQ138">
+        <v>4299</v>
+      </c>
+      <c r="BR138">
+        <v>1113</v>
+      </c>
+      <c r="BS138">
+        <v>44</v>
+      </c>
+      <c r="BT138">
+        <v>14</v>
+      </c>
+      <c r="BU138">
+        <v>0</v>
+      </c>
+      <c r="BV138">
+        <v>0</v>
+      </c>
+      <c r="BW138">
+        <v>47116.33346266799</v>
+      </c>
+      <c r="BX138">
+        <v>7952.737229647995</v>
+      </c>
+      <c r="BY138">
+        <v>0.05108887826035292</v>
+      </c>
+      <c r="BZ138">
+        <v>0.1041739946233573</v>
+      </c>
+      <c r="CA138">
+        <v>0.1171145070205996</v>
+      </c>
+      <c r="CB138">
+        <v>0.1931574060944746</v>
+      </c>
+      <c r="CC138">
+        <v>0.01144537069773439</v>
+      </c>
+      <c r="CD138">
+        <v>0.01748469138926716</v>
+      </c>
+      <c r="CE138">
+        <v>0.009081701505211407</v>
+      </c>
+      <c r="CF138">
+        <v>0.01664488388571054</v>
+      </c>
+      <c r="CG138">
+        <v>49116.04061999999</v>
+      </c>
+      <c r="CH138">
+        <v>8345.800659999995</v>
+      </c>
+      <c r="CI138">
+        <v>53043.28865526684</v>
+      </c>
+      <c r="CJ138">
+        <v>8377.318341907174</v>
+      </c>
+      <c r="CK138">
+        <v>0.165678587720489</v>
+      </c>
+      <c r="CL138">
+        <v>0.06650993724584395</v>
+      </c>
+      <c r="CM138">
+        <v>10000</v>
+      </c>
+      <c r="CO138">
+        <v>0.008804448563484708</v>
+      </c>
+      <c r="CP138">
+        <v>0.007645968489341983</v>
+      </c>
+      <c r="CQ138">
+        <v>22037322.50646456</v>
+      </c>
+      <c r="CR138">
+        <v>1792741.222718281</v>
+      </c>
+      <c r="CS138" s="2">
+        <v>45420.53197429089</v>
+      </c>
+      <c r="CT138">
+        <v>-0.7176955593761354</v>
+      </c>
+      <c r="CU138">
+        <v>-0.798053640692689</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update FETUSDT.json at 2024-05-08_21-44-28 bestfile_scores 0.002632085177329213 bestfile_sharp 0.24431337451463206
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU138"/>
+  <dimension ref="A1:CU139"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -39634,6 +39634,275 @@
       </c>
       <c r="CU138">
         <v>-0.798053640692689</v>
+      </c>
+    </row>
+    <row r="139" spans="10:99">
+      <c r="J139" t="s">
+        <v>200</v>
+      </c>
+      <c r="K139">
+        <v>0.0005551911911603202</v>
+      </c>
+      <c r="L139">
+        <v>0.0002775955955801601</v>
+      </c>
+      <c r="M139">
+        <v>0.0004692890892952217</v>
+      </c>
+      <c r="N139">
+        <v>0.0004692890892952217</v>
+      </c>
+      <c r="O139">
+        <v>0.001607036844155463</v>
+      </c>
+      <c r="P139">
+        <v>0.0008035184220777314</v>
+      </c>
+      <c r="Q139">
+        <v>0.000455609683810887</v>
+      </c>
+      <c r="R139">
+        <v>0.000455609683810887</v>
+      </c>
+      <c r="S139">
+        <v>29.68776229645795</v>
+      </c>
+      <c r="T139">
+        <v>14.59660903139164</v>
+      </c>
+      <c r="U139">
+        <v>0.4526394484804169</v>
+      </c>
+      <c r="V139">
+        <v>0.4971530328389945</v>
+      </c>
+      <c r="W139">
+        <v>0.0605768602510894</v>
+      </c>
+      <c r="X139">
+        <v>0.07520935172115532</v>
+      </c>
+      <c r="Y139">
+        <v>0.2009656300029838</v>
+      </c>
+      <c r="Z139">
+        <v>0.2380676372192553</v>
+      </c>
+      <c r="AA139">
+        <v>0.9994369707886128</v>
+      </c>
+      <c r="AB139">
+        <v>0.8381853843411072</v>
+      </c>
+      <c r="AC139">
+        <v>0.8181417174975338</v>
+      </c>
+      <c r="AD139">
+        <v>0.9995840573300672</v>
+      </c>
+      <c r="AE139">
+        <v>0.818155607382553</v>
+      </c>
+      <c r="AF139">
+        <v>0.7621018232123975</v>
+      </c>
+      <c r="AG139">
+        <v>0.0063660737988839</v>
+      </c>
+      <c r="AH139">
+        <v>0.004994708056206319</v>
+      </c>
+      <c r="AI139">
+        <v>0.9994369707886128</v>
+      </c>
+      <c r="AJ139">
+        <v>0.9995840573300672</v>
+      </c>
+      <c r="AK139">
+        <v>0.0063660737988839</v>
+      </c>
+      <c r="AL139">
+        <v>0.004994708056206319</v>
+      </c>
+      <c r="AM139" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN139">
+        <v>0.009022449129326478</v>
+      </c>
+      <c r="AO139">
+        <v>0.01480636412508247</v>
+      </c>
+      <c r="AP139">
+        <v>-1072.4217431</v>
+      </c>
+      <c r="AQ139">
+        <v>-313.18608208</v>
+      </c>
+      <c r="AR139">
+        <v>17350.90135690009</v>
+      </c>
+      <c r="AS139">
+        <v>15933.14691792001</v>
+      </c>
+      <c r="AT139">
+        <v>17344.05655690009</v>
+      </c>
+      <c r="AU139">
+        <v>15933.14691792001</v>
+      </c>
+      <c r="AV139">
+        <v>0.7350901356900086</v>
+      </c>
+      <c r="AW139">
+        <v>0.5933146917920014</v>
+      </c>
+      <c r="AX139">
+        <v>0.8073245346180815</v>
+      </c>
+      <c r="AY139">
+        <v>1.641699445632921</v>
+      </c>
+      <c r="AZ139">
+        <v>93.63333333333334</v>
+      </c>
+      <c r="BA139">
+        <v>86.09999999999999</v>
+      </c>
+      <c r="BB139">
+        <v>0.05111999284176391</v>
+      </c>
+      <c r="BC139">
+        <v>0.1327208817859857</v>
+      </c>
+      <c r="BD139">
+        <v>-453.7983868639545</v>
+      </c>
+      <c r="BE139">
+        <v>-955.8846815038005</v>
+      </c>
+      <c r="BF139">
+        <v>14274</v>
+      </c>
+      <c r="BG139">
+        <v>3947</v>
+      </c>
+      <c r="BH139">
+        <v>992.8333333333334</v>
+      </c>
+      <c r="BI139">
+        <v>15201</v>
+      </c>
+      <c r="BJ139">
+        <v>10545</v>
+      </c>
+      <c r="BK139">
+        <v>29475</v>
+      </c>
+      <c r="BL139">
+        <v>14492</v>
+      </c>
+      <c r="BM139">
+        <v>14247</v>
+      </c>
+      <c r="BN139">
+        <v>3928</v>
+      </c>
+      <c r="BO139">
+        <v>14264</v>
+      </c>
+      <c r="BP139">
+        <v>3928</v>
+      </c>
+      <c r="BQ139">
+        <v>954</v>
+      </c>
+      <c r="BR139">
+        <v>6617</v>
+      </c>
+      <c r="BS139">
+        <v>10</v>
+      </c>
+      <c r="BT139">
+        <v>19</v>
+      </c>
+      <c r="BU139">
+        <v>0</v>
+      </c>
+      <c r="BV139">
+        <v>0</v>
+      </c>
+      <c r="BW139">
+        <v>7350.901356900011</v>
+      </c>
+      <c r="BX139">
+        <v>5933.14691791999</v>
+      </c>
+      <c r="BY139">
+        <v>0.0531108811854462</v>
+      </c>
+      <c r="BZ139">
+        <v>0.05651699429784502</v>
+      </c>
+      <c r="CA139">
+        <v>0.1220301622258644</v>
+      </c>
+      <c r="CB139">
+        <v>0.1921757179627456</v>
+      </c>
+      <c r="CC139">
+        <v>0.01484278818008808</v>
+      </c>
+      <c r="CD139">
+        <v>0.008818750494495474</v>
+      </c>
+      <c r="CE139">
+        <v>0.01179606047862717</v>
+      </c>
+      <c r="CF139">
+        <v>0.009930364247942761</v>
+      </c>
+      <c r="CG139">
+        <v>8423.323100000011</v>
+      </c>
+      <c r="CH139">
+        <v>6246.332999999991</v>
+      </c>
+      <c r="CI139">
+        <v>8877.121486863965</v>
+      </c>
+      <c r="CJ139">
+        <v>7202.217681503791</v>
+      </c>
+      <c r="CK139">
+        <v>0.07840001921789688</v>
+      </c>
+      <c r="CL139">
+        <v>0.07874972869677671</v>
+      </c>
+      <c r="CM139">
+        <v>10000</v>
+      </c>
+      <c r="CO139">
+        <v>0.001762558227370011</v>
+      </c>
+      <c r="CP139">
+        <v>0.001007176129925721</v>
+      </c>
+      <c r="CQ139">
+        <v>3389577.188059013</v>
+      </c>
+      <c r="CR139">
+        <v>4157882.239708048</v>
+      </c>
+      <c r="CS139" s="2">
+        <v>45420.74298430007</v>
+      </c>
+      <c r="CT139">
+        <v>-0.8723102032515645</v>
+      </c>
+      <c r="CU139">
+        <v>-0.8623508172721044</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ALGOUSDT.json at 2024-05-09_05-18-06 bestfile_scores 0.0009860611521964075 bestfile_sharp 0.2270903940784514
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU139"/>
+  <dimension ref="A1:CU140"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -39903,6 +39903,275 @@
       </c>
       <c r="CU139">
         <v>-0.8623508172721044</v>
+      </c>
+    </row>
+    <row r="140" spans="10:99">
+      <c r="J140" t="s">
+        <v>221</v>
+      </c>
+      <c r="K140">
+        <v>0.003718905936362926</v>
+      </c>
+      <c r="L140">
+        <v>0.001859452968181463</v>
+      </c>
+      <c r="M140">
+        <v>0.002110936175253375</v>
+      </c>
+      <c r="N140">
+        <v>0.002110936175253375</v>
+      </c>
+      <c r="O140">
+        <v>0.006998008485984153</v>
+      </c>
+      <c r="P140">
+        <v>0.003499004242992077</v>
+      </c>
+      <c r="Q140">
+        <v>0.003058947322889938</v>
+      </c>
+      <c r="R140">
+        <v>0.003058947322889938</v>
+      </c>
+      <c r="S140">
+        <v>18.51218872870249</v>
+      </c>
+      <c r="T140">
+        <v>14.06028833551769</v>
+      </c>
+      <c r="U140">
+        <v>0.429742099549777</v>
+      </c>
+      <c r="V140">
+        <v>0.6734776902693198</v>
+      </c>
+      <c r="W140">
+        <v>0.07930280188374478</v>
+      </c>
+      <c r="X140">
+        <v>0.05421403518520693</v>
+      </c>
+      <c r="Y140">
+        <v>0.1525248830962414</v>
+      </c>
+      <c r="Z140">
+        <v>0.188901023245988</v>
+      </c>
+      <c r="AA140">
+        <v>0.9979202098307671</v>
+      </c>
+      <c r="AB140">
+        <v>0.8757283040954551</v>
+      </c>
+      <c r="AC140">
+        <v>0.8502010504998111</v>
+      </c>
+      <c r="AD140">
+        <v>0.9992838939352033</v>
+      </c>
+      <c r="AE140">
+        <v>0.8478141619703143</v>
+      </c>
+      <c r="AF140">
+        <v>0.8028982906883085</v>
+      </c>
+      <c r="AG140">
+        <v>0.009094062282386057</v>
+      </c>
+      <c r="AH140">
+        <v>0.006652001977027054</v>
+      </c>
+      <c r="AI140">
+        <v>0.9979202098307671</v>
+      </c>
+      <c r="AJ140">
+        <v>0.9992838939352033</v>
+      </c>
+      <c r="AK140">
+        <v>0.009094062282386057</v>
+      </c>
+      <c r="AL140">
+        <v>0.006652001977027054</v>
+      </c>
+      <c r="AM140" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN140">
+        <v>0.04867905274594962</v>
+      </c>
+      <c r="AO140">
+        <v>0.03036220516941307</v>
+      </c>
+      <c r="AP140">
+        <v>-1765.84659052</v>
+      </c>
+      <c r="AQ140">
+        <v>-746.67212126</v>
+      </c>
+      <c r="AR140">
+        <v>58718.1490094801</v>
+      </c>
+      <c r="AS140">
+        <v>27335.24197873989</v>
+      </c>
+      <c r="AT140">
+        <v>58640.0158094801</v>
+      </c>
+      <c r="AU140">
+        <v>27335.24197873989</v>
+      </c>
+      <c r="AV140">
+        <v>4.87181490094801</v>
+      </c>
+      <c r="AW140">
+        <v>1.733524197873989</v>
+      </c>
+      <c r="AX140">
+        <v>1.294052339413164</v>
+      </c>
+      <c r="AY140">
+        <v>1.701456841686555</v>
+      </c>
+      <c r="AZ140">
+        <v>89.86666666666666</v>
+      </c>
+      <c r="BA140">
+        <v>78.56666666666666</v>
+      </c>
+      <c r="BB140">
+        <v>0.001490638169435649</v>
+      </c>
+      <c r="BC140">
+        <v>0.03772158664895737</v>
+      </c>
+      <c r="BD140">
+        <v>-75.36571379663336</v>
+      </c>
+      <c r="BE140">
+        <v>-708.816159688007</v>
+      </c>
+      <c r="BF140">
+        <v>3400</v>
+      </c>
+      <c r="BG140">
+        <v>2877</v>
+      </c>
+      <c r="BH140">
+        <v>476.875</v>
+      </c>
+      <c r="BI140">
+        <v>5428</v>
+      </c>
+      <c r="BJ140">
+        <v>3828</v>
+      </c>
+      <c r="BK140">
+        <v>8828</v>
+      </c>
+      <c r="BL140">
+        <v>6705</v>
+      </c>
+      <c r="BM140">
+        <v>3391</v>
+      </c>
+      <c r="BN140">
+        <v>2225</v>
+      </c>
+      <c r="BO140">
+        <v>3394</v>
+      </c>
+      <c r="BP140">
+        <v>2839</v>
+      </c>
+      <c r="BQ140">
+        <v>2037</v>
+      </c>
+      <c r="BR140">
+        <v>1603</v>
+      </c>
+      <c r="BS140">
+        <v>6</v>
+      </c>
+      <c r="BT140">
+        <v>38</v>
+      </c>
+      <c r="BU140">
+        <v>0</v>
+      </c>
+      <c r="BV140">
+        <v>0</v>
+      </c>
+      <c r="BW140">
+        <v>48718.14900948</v>
+      </c>
+      <c r="BX140">
+        <v>17335.24197874002</v>
+      </c>
+      <c r="BY140">
+        <v>0.05656088652193964</v>
+      </c>
+      <c r="BZ140">
+        <v>0.0615210542963856</v>
+      </c>
+      <c r="CA140">
+        <v>0.083091751722095</v>
+      </c>
+      <c r="CB140">
+        <v>0.1631263269236074</v>
+      </c>
+      <c r="CC140">
+        <v>0.01165736331538616</v>
+      </c>
+      <c r="CD140">
+        <v>0.007804936301286026</v>
+      </c>
+      <c r="CE140">
+        <v>0.00931958981462256</v>
+      </c>
+      <c r="CF140">
+        <v>0.009903473811885413</v>
+      </c>
+      <c r="CG140">
+        <v>50483.99559999999</v>
+      </c>
+      <c r="CH140">
+        <v>18081.91410000002</v>
+      </c>
+      <c r="CI140">
+        <v>50559.36131379663</v>
+      </c>
+      <c r="CJ140">
+        <v>18790.73025968803</v>
+      </c>
+      <c r="CK140">
+        <v>0.2443133745146321</v>
+      </c>
+      <c r="CL140">
+        <v>0.2445254674396609</v>
+      </c>
+      <c r="CM140">
+        <v>10000</v>
+      </c>
+      <c r="CO140">
+        <v>0.007600908614363096</v>
+      </c>
+      <c r="CP140">
+        <v>0.0078630089114101</v>
+      </c>
+      <c r="CQ140">
+        <v>8210618.622884387</v>
+      </c>
+      <c r="CR140">
+        <v>7172478.294001529</v>
+      </c>
+      <c r="CS140" s="2">
+        <v>45420.90591002226</v>
+      </c>
+      <c r="CT140">
+        <v>-0.5365809810110987</v>
+      </c>
+      <c r="CU140">
+        <v>-0.7136512022352061</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update NEARUSDT.json at 2024-05-09_10-27-25 bestfile_scores 0.0004170361666574945 bestfile_sharp 0.1424579767085579
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU140"/>
+  <dimension ref="A1:CU141"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -40172,6 +40172,275 @@
       </c>
       <c r="CU140">
         <v>-0.7136512022352061</v>
+      </c>
+    </row>
+    <row r="141" spans="10:99">
+      <c r="J141" t="s">
+        <v>208</v>
+      </c>
+      <c r="K141">
+        <v>0.001889330797239408</v>
+      </c>
+      <c r="L141">
+        <v>0.000944665398619704</v>
+      </c>
+      <c r="M141">
+        <v>0.001012125649365148</v>
+      </c>
+      <c r="N141">
+        <v>0.001012125649365148</v>
+      </c>
+      <c r="O141">
+        <v>0.002163337531366749</v>
+      </c>
+      <c r="P141">
+        <v>0.001081668765683375</v>
+      </c>
+      <c r="Q141">
+        <v>0.0009057847951174036</v>
+      </c>
+      <c r="R141">
+        <v>0.0009057847951174036</v>
+      </c>
+      <c r="S141">
+        <v>38.96446622169066</v>
+      </c>
+      <c r="T141">
+        <v>18.38404259423589</v>
+      </c>
+      <c r="U141">
+        <v>0.3848109461512561</v>
+      </c>
+      <c r="V141">
+        <v>0.2618970158658526</v>
+      </c>
+      <c r="W141">
+        <v>0.0510891128087686</v>
+      </c>
+      <c r="X141">
+        <v>0.08141601234937086</v>
+      </c>
+      <c r="Y141">
+        <v>0.2401885115006192</v>
+      </c>
+      <c r="Z141">
+        <v>0.1522426977783748</v>
+      </c>
+      <c r="AA141">
+        <v>0.9991904239821255</v>
+      </c>
+      <c r="AB141">
+        <v>0.8002590982672541</v>
+      </c>
+      <c r="AC141">
+        <v>0.8595760973147339</v>
+      </c>
+      <c r="AD141">
+        <v>0.9977690736692849</v>
+      </c>
+      <c r="AE141">
+        <v>0.7598054036874696</v>
+      </c>
+      <c r="AF141">
+        <v>0.7556757921170245</v>
+      </c>
+      <c r="AG141">
+        <v>0.006771783071722543</v>
+      </c>
+      <c r="AH141">
+        <v>0.009892196288343594</v>
+      </c>
+      <c r="AI141">
+        <v>0.9991904239821255</v>
+      </c>
+      <c r="AJ141">
+        <v>0.9977690736692849</v>
+      </c>
+      <c r="AK141">
+        <v>0.006771783071722543</v>
+      </c>
+      <c r="AL141">
+        <v>0.009892196288343594</v>
+      </c>
+      <c r="AM141" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN141">
+        <v>0.02620457929351563</v>
+      </c>
+      <c r="AO141">
+        <v>0.068528665289134</v>
+      </c>
+      <c r="AP141">
+        <v>-5554.755204474</v>
+      </c>
+      <c r="AQ141">
+        <v>-2146.338908248</v>
+      </c>
+      <c r="AR141">
+        <v>76788.78204362186</v>
+      </c>
+      <c r="AS141">
+        <v>29817.21292256788</v>
+      </c>
+      <c r="AT141">
+        <v>76758.81870362186</v>
+      </c>
+      <c r="AU141">
+        <v>29818.12722256788</v>
+      </c>
+      <c r="AV141">
+        <v>6.678878204362186</v>
+      </c>
+      <c r="AW141">
+        <v>1.981721292256788</v>
+      </c>
+      <c r="AX141">
+        <v>0.6159568906105183</v>
+      </c>
+      <c r="AY141">
+        <v>1.304436776977451</v>
+      </c>
+      <c r="AZ141">
+        <v>64.66666666666667</v>
+      </c>
+      <c r="BA141">
+        <v>93.46666666666667</v>
+      </c>
+      <c r="BB141">
+        <v>0.000261991631371721</v>
+      </c>
+      <c r="BC141">
+        <v>0.04495178928464983</v>
+      </c>
+      <c r="BD141">
+        <v>-18.9583280299423</v>
+      </c>
+      <c r="BE141">
+        <v>-1033.930240969375</v>
+      </c>
+      <c r="BF141">
+        <v>14556</v>
+      </c>
+      <c r="BG141">
+        <v>8923</v>
+      </c>
+      <c r="BH141">
+        <v>1079.958333333333</v>
+      </c>
+      <c r="BI141">
+        <v>27524</v>
+      </c>
+      <c r="BJ141">
+        <v>10931</v>
+      </c>
+      <c r="BK141">
+        <v>42080</v>
+      </c>
+      <c r="BL141">
+        <v>19854</v>
+      </c>
+      <c r="BM141">
+        <v>13431</v>
+      </c>
+      <c r="BN141">
+        <v>8578</v>
+      </c>
+      <c r="BO141">
+        <v>14510</v>
+      </c>
+      <c r="BP141">
+        <v>8815</v>
+      </c>
+      <c r="BQ141">
+        <v>14093</v>
+      </c>
+      <c r="BR141">
+        <v>2353</v>
+      </c>
+      <c r="BS141">
+        <v>46</v>
+      </c>
+      <c r="BT141">
+        <v>108</v>
+      </c>
+      <c r="BU141">
+        <v>0</v>
+      </c>
+      <c r="BV141">
+        <v>0</v>
+      </c>
+      <c r="BW141">
+        <v>66788.62846552613</v>
+      </c>
+      <c r="BX141">
+        <v>19820.60039175199</v>
+      </c>
+      <c r="BY141">
+        <v>0.03269554087442854</v>
+      </c>
+      <c r="BZ141">
+        <v>0.0813820812434381</v>
+      </c>
+      <c r="CA141">
+        <v>0.1365346925870581</v>
+      </c>
+      <c r="CB141">
+        <v>0.132065655384105</v>
+      </c>
+      <c r="CC141">
+        <v>0.007910900721258907</v>
+      </c>
+      <c r="CD141">
+        <v>0.01238629491717968</v>
+      </c>
+      <c r="CE141">
+        <v>0.006233454372999068</v>
+      </c>
+      <c r="CF141">
+        <v>0.01338162793170816</v>
+      </c>
+      <c r="CG141">
+        <v>72343.38367000013</v>
+      </c>
+      <c r="CH141">
+        <v>21966.93929999999</v>
+      </c>
+      <c r="CI141">
+        <v>72362.34199803007</v>
+      </c>
+      <c r="CJ141">
+        <v>23000.86954096936</v>
+      </c>
+      <c r="CK141">
+        <v>0.2270903940784514</v>
+      </c>
+      <c r="CL141">
+        <v>0.108982459461117</v>
+      </c>
+      <c r="CM141">
+        <v>10000</v>
+      </c>
+      <c r="CO141">
+        <v>0.00625</v>
+      </c>
+      <c r="CP141">
+        <v>0.02650462962962963</v>
+      </c>
+      <c r="CQ141">
+        <v>98712179.16011865</v>
+      </c>
+      <c r="CR141">
+        <v>10598803.27492217</v>
+      </c>
+      <c r="CS141" s="2">
+        <v>45421.22093259679</v>
+      </c>
+      <c r="CT141">
+        <v>-0.8043091815774359</v>
+      </c>
+      <c r="CU141">
+        <v>-0.7574299323150953</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GALAUSDT.json at 2024-05-10_00-57-30 bestfile_scores 0.00047529234133492635 bestfile_sharp 0.2258812048432976
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="366">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1473,7 +1473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU141"/>
+  <dimension ref="A1:CU142"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -40441,6 +40441,275 @@
       </c>
       <c r="CU141">
         <v>-0.7574299323150953</v>
+      </c>
+    </row>
+    <row r="142" spans="10:99">
+      <c r="J142" t="s">
+        <v>213</v>
+      </c>
+      <c r="K142">
+        <v>0.0009791614490426426</v>
+      </c>
+      <c r="L142">
+        <v>0.0004895807245213213</v>
+      </c>
+      <c r="M142">
+        <v>0.0002051275288859067</v>
+      </c>
+      <c r="N142">
+        <v>0.0002051275288859067</v>
+      </c>
+      <c r="O142">
+        <v>0.001373646392256345</v>
+      </c>
+      <c r="P142">
+        <v>0.0006868231961281723</v>
+      </c>
+      <c r="Q142">
+        <v>0.0002866132170945779</v>
+      </c>
+      <c r="R142">
+        <v>0.0002866132170945779</v>
+      </c>
+      <c r="S142">
+        <v>25.53852094999035</v>
+      </c>
+      <c r="T142">
+        <v>10.97169337709983</v>
+      </c>
+      <c r="U142">
+        <v>0.444720364470454</v>
+      </c>
+      <c r="V142">
+        <v>0.5515009125369736</v>
+      </c>
+      <c r="W142">
+        <v>0.01994749617820258</v>
+      </c>
+      <c r="X142">
+        <v>0.02326205019476134</v>
+      </c>
+      <c r="Y142">
+        <v>0.1075313106787391</v>
+      </c>
+      <c r="Z142">
+        <v>0.2443951890819016</v>
+      </c>
+      <c r="AA142">
+        <v>0.9996573305302862</v>
+      </c>
+      <c r="AB142">
+        <v>0.9029732090806061</v>
+      </c>
+      <c r="AC142">
+        <v>0.9220750597495151</v>
+      </c>
+      <c r="AD142">
+        <v>0.9994682435618946</v>
+      </c>
+      <c r="AE142">
+        <v>0.8520702778678207</v>
+      </c>
+      <c r="AF142">
+        <v>0.6751199983546743</v>
+      </c>
+      <c r="AG142">
+        <v>0.003006973066287996</v>
+      </c>
+      <c r="AH142">
+        <v>0.003284008719121437</v>
+      </c>
+      <c r="AI142">
+        <v>0.9996573305302862</v>
+      </c>
+      <c r="AJ142">
+        <v>0.9994682435618946</v>
+      </c>
+      <c r="AK142">
+        <v>0.003006973066287996</v>
+      </c>
+      <c r="AL142">
+        <v>0.003284008719121437</v>
+      </c>
+      <c r="AM142" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN142">
+        <v>0.01102459909290902</v>
+      </c>
+      <c r="AO142">
+        <v>0.01107060651290055</v>
+      </c>
+      <c r="AP142">
+        <v>-3178.4995556</v>
+      </c>
+      <c r="AQ142">
+        <v>-256.96699448</v>
+      </c>
+      <c r="AR142">
+        <v>28747.26424439966</v>
+      </c>
+      <c r="AS142">
+        <v>12476.99380552017</v>
+      </c>
+      <c r="AT142">
+        <v>28722.73124439966</v>
+      </c>
+      <c r="AU142">
+        <v>12476.99380552017</v>
+      </c>
+      <c r="AV142">
+        <v>1.874726424439966</v>
+      </c>
+      <c r="AW142">
+        <v>0.2476993805520167</v>
+      </c>
+      <c r="AX142">
+        <v>0.9385503617139677</v>
+      </c>
+      <c r="AY142">
+        <v>2.184575202050069</v>
+      </c>
+      <c r="AZ142">
+        <v>116.9333333333333</v>
+      </c>
+      <c r="BA142">
+        <v>111.15</v>
+      </c>
+      <c r="BB142">
+        <v>0.0009090456825400375</v>
+      </c>
+      <c r="BC142">
+        <v>0.02047830360591597</v>
+      </c>
+      <c r="BD142">
+        <v>-19.949656067499</v>
+      </c>
+      <c r="BE142">
+        <v>-57.15736518667998</v>
+      </c>
+      <c r="BF142">
+        <v>12137</v>
+      </c>
+      <c r="BG142">
+        <v>5781</v>
+      </c>
+      <c r="BH142">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI142">
+        <v>15418</v>
+      </c>
+      <c r="BJ142">
+        <v>6057</v>
+      </c>
+      <c r="BK142">
+        <v>27555</v>
+      </c>
+      <c r="BL142">
+        <v>11838</v>
+      </c>
+      <c r="BM142">
+        <v>11961</v>
+      </c>
+      <c r="BN142">
+        <v>5524</v>
+      </c>
+      <c r="BO142">
+        <v>12133</v>
+      </c>
+      <c r="BP142">
+        <v>5772</v>
+      </c>
+      <c r="BQ142">
+        <v>3457</v>
+      </c>
+      <c r="BR142">
+        <v>533</v>
+      </c>
+      <c r="BS142">
+        <v>4</v>
+      </c>
+      <c r="BT142">
+        <v>9</v>
+      </c>
+      <c r="BU142">
+        <v>0</v>
+      </c>
+      <c r="BV142">
+        <v>0</v>
+      </c>
+      <c r="BW142">
+        <v>18747.26424440003</v>
+      </c>
+      <c r="BX142">
+        <v>2476.993805520001</v>
+      </c>
+      <c r="BY142">
+        <v>0.0282675234131565</v>
+      </c>
+      <c r="BZ142">
+        <v>0.133234483195606</v>
+      </c>
+      <c r="CA142">
+        <v>0.05732285058476774</v>
+      </c>
+      <c r="CB142">
+        <v>0.2358065693923901</v>
+      </c>
+      <c r="CC142">
+        <v>0.01049894086122908</v>
+      </c>
+      <c r="CD142">
+        <v>0.02191929943834858</v>
+      </c>
+      <c r="CE142">
+        <v>0.007419192349491326</v>
+      </c>
+      <c r="CF142">
+        <v>0.02274835599314671</v>
+      </c>
+      <c r="CG142">
+        <v>21925.76380000003</v>
+      </c>
+      <c r="CH142">
+        <v>2733.960800000001</v>
+      </c>
+      <c r="CI142">
+        <v>21945.71345606753</v>
+      </c>
+      <c r="CJ142">
+        <v>2791.118165186681</v>
+      </c>
+      <c r="CK142">
+        <v>0.1424579767085579</v>
+      </c>
+      <c r="CL142">
+        <v>0.07385941677269116</v>
+      </c>
+      <c r="CM142">
+        <v>10000</v>
+      </c>
+      <c r="CO142">
+        <v>0.002239728143342601</v>
+      </c>
+      <c r="CP142">
+        <v>0.001544640098856966</v>
+      </c>
+      <c r="CQ142">
+        <v>21946958.71626803</v>
+      </c>
+      <c r="CR142">
+        <v>1954441.87495541</v>
+      </c>
+      <c r="CS142" s="2">
+        <v>45421.43573098649</v>
+      </c>
+      <c r="CT142">
+        <v>-0.892071333585829</v>
+      </c>
+      <c r="CU142">
+        <v>-0.9702031259092914</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update ENJUSDT.json at 2024-05-10_07-02-58 bestfile_scores 0.0007992648502826134 bestfile_sharp 0.17822742776233916
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="384">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1113,6 +1113,60 @@
   <si>
     <t>2024-05-02 20:37:29.050468</t>
   </si>
+  <si>
+    <t>2024-05-03 06:34:56.158272</t>
+  </si>
+  <si>
+    <t>2024-05-03 11:06:19.987231</t>
+  </si>
+  <si>
+    <t>2024-05-03 17:38:11.683050</t>
+  </si>
+  <si>
+    <t>2024-05-03 21:38:18.478476</t>
+  </si>
+  <si>
+    <t>2024-05-06 04:06:02.555577</t>
+  </si>
+  <si>
+    <t>2024-05-06 07:53:50.861164</t>
+  </si>
+  <si>
+    <t>2024-05-06 15:44:41.814743</t>
+  </si>
+  <si>
+    <t>2024-05-07 03:28:04.797008</t>
+  </si>
+  <si>
+    <t>2024-05-07 07:25:08.226851</t>
+  </si>
+  <si>
+    <t>2024-05-07 12:28:52.642195</t>
+  </si>
+  <si>
+    <t>2024-05-07 17:50:15.471030</t>
+  </si>
+  <si>
+    <t>2024-05-07 23:17:24.985590</t>
+  </si>
+  <si>
+    <t>2024-05-08 04:21:55.668677</t>
+  </si>
+  <si>
+    <t>2024-05-08 12:46:02.578733</t>
+  </si>
+  <si>
+    <t>2024-05-08 17:49:53.843526</t>
+  </si>
+  <si>
+    <t>2024-05-08 21:44:30.625923</t>
+  </si>
+  <si>
+    <t>2024-05-09 05:18:08.576362</t>
+  </si>
+  <si>
+    <t>2024-05-09 10:27:27.157233</t>
+  </si>
 </sst>
 </file>
 
@@ -1473,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU142"/>
+  <dimension ref="A1:CU143"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -35875,28 +35929,28 @@
         <v>202</v>
       </c>
       <c r="K125">
-        <v>0.002236939357510792</v>
+        <v>0.0022369393575107</v>
       </c>
       <c r="L125">
-        <v>0.001118469678755396</v>
+        <v>0.0011184696787553</v>
       </c>
       <c r="M125">
-        <v>0.001236671099455799</v>
+        <v>0.0012366710994557</v>
       </c>
       <c r="N125">
-        <v>0.001236671099455799</v>
+        <v>0.0012366710994557</v>
       </c>
       <c r="O125">
-        <v>0.001839711725944437</v>
+        <v>0.0018397117259444</v>
       </c>
       <c r="P125">
-        <v>0.0009198558629722187</v>
+        <v>0.0009198558629722</v>
       </c>
       <c r="Q125">
-        <v>0.001434745181500574</v>
+        <v>0.0014347451815005</v>
       </c>
       <c r="R125">
-        <v>0.001434745181500574</v>
+        <v>0.0014347451815005</v>
       </c>
       <c r="S125">
         <v>11.72360044754813</v>
@@ -35911,19 +35965,19 @@
         <v>0.5954825002586427</v>
       </c>
       <c r="W125">
-        <v>0.03031893049282055</v>
+        <v>0.0303189304928205</v>
       </c>
       <c r="X125">
-        <v>0.09013365192788314</v>
+        <v>0.0901336519278831</v>
       </c>
       <c r="Y125">
         <v>0.1454939486875937</v>
       </c>
       <c r="Z125">
-        <v>0.2026782245235637</v>
+        <v>0.2026782245235636</v>
       </c>
       <c r="AA125">
-        <v>0.9992673609594271</v>
+        <v>0.9992673609594273</v>
       </c>
       <c r="AB125">
         <v>0.8910212382727811</v>
@@ -35941,31 +35995,31 @@
         <v>0.7981920349549094</v>
       </c>
       <c r="AG125">
-        <v>0.003859202734480985</v>
+        <v>0.0038592027344809</v>
       </c>
       <c r="AH125">
-        <v>0.01053076937279949</v>
+        <v>0.0105307693727994</v>
       </c>
       <c r="AI125">
-        <v>0.9992673609594271</v>
+        <v>0.9992673609594273</v>
       </c>
       <c r="AJ125">
         <v>0.9973579260301606</v>
       </c>
       <c r="AK125">
-        <v>0.003859202734480985</v>
+        <v>0.0038592027344809</v>
       </c>
       <c r="AL125">
-        <v>0.01053076937279949</v>
+        <v>0.0105307693727994</v>
       </c>
       <c r="AM125" t="s">
         <v>243</v>
       </c>
       <c r="AN125">
-        <v>0.02093695864100079</v>
+        <v>0.0209369586410007</v>
       </c>
       <c r="AO125">
-        <v>0.07852190783920794</v>
+        <v>0.0785219078392079</v>
       </c>
       <c r="AP125">
         <v>-3159.000605748</v>
@@ -36004,16 +36058,16 @@
         <v>119.2</v>
       </c>
       <c r="BB125">
-        <v>0.003224980594379225</v>
+        <v>0.0032249805943792</v>
       </c>
       <c r="BC125">
-        <v>0.06441365475871964</v>
+        <v>0.0644136547587196</v>
       </c>
       <c r="BD125">
         <v>-339.2159959189568</v>
       </c>
       <c r="BE125">
-        <v>-1991.385805693739</v>
+        <v>-1991.385805693738</v>
       </c>
       <c r="BF125">
         <v>4791</v>
@@ -36073,10 +36127,10 @@
         <v>27989.629424542</v>
       </c>
       <c r="BY125">
-        <v>0.04183586437192352</v>
+        <v>0.0418358643719235</v>
       </c>
       <c r="BZ125">
-        <v>0.07999316210968833</v>
+        <v>0.07999316210968831</v>
       </c>
       <c r="CA125">
         <v>0.0782810542988181</v>
@@ -36085,16 +36139,16 @@
         <v>0.1679184055700101</v>
       </c>
       <c r="CC125">
-        <v>0.01403797457625645</v>
+        <v>0.0140379745762564</v>
       </c>
       <c r="CD125">
-        <v>0.01758184801232305</v>
+        <v>0.017581848012323</v>
       </c>
       <c r="CE125">
-        <v>0.01023140492613323</v>
+        <v>0.0102314049261332</v>
       </c>
       <c r="CF125">
-        <v>0.01265517397784129</v>
+        <v>0.0126551739778412</v>
       </c>
       <c r="CG125">
         <v>104844.67147</v>
@@ -36109,19 +36163,19 @@
         <v>30915.58479569374</v>
       </c>
       <c r="CK125">
-        <v>0.05424559650284209</v>
+        <v>0.054245596502842</v>
       </c>
       <c r="CL125">
-        <v>0.1141280869522103</v>
+        <v>0.1141280869522102</v>
       </c>
       <c r="CM125">
         <v>10000</v>
       </c>
       <c r="CO125">
-        <v>0.001003086419753086</v>
+        <v>0.001003086419753</v>
       </c>
       <c r="CP125">
-        <v>0.02299382716049383</v>
+        <v>0.0229938271604938</v>
       </c>
       <c r="CQ125">
         <v>42201373.71041539</v>
@@ -36129,8 +36183,8 @@
       <c r="CR125">
         <v>14590537.25038491</v>
       </c>
-      <c r="CS125" s="2">
-        <v>45415.27426109111</v>
+      <c r="CS125" t="s">
+        <v>366</v>
       </c>
       <c r="CT125">
         <v>-0.7252315072660098</v>
@@ -36144,28 +36198,28 @@
         <v>199</v>
       </c>
       <c r="K126">
-        <v>0.001383012923460658</v>
+        <v>0.0013830129234606</v>
       </c>
       <c r="L126">
-        <v>0.000691506461730329</v>
+        <v>0.0006915064617303</v>
       </c>
       <c r="M126">
-        <v>0.0002290439155725466</v>
+        <v>0.0002290439155725</v>
       </c>
       <c r="N126">
-        <v>0.0002290439155725466</v>
+        <v>0.0002290439155725</v>
       </c>
       <c r="O126">
-        <v>0.002361505883074533</v>
+        <v>0.0023615058830745</v>
       </c>
       <c r="P126">
-        <v>0.001180752941537266</v>
+        <v>0.0011807529415372</v>
       </c>
       <c r="Q126">
-        <v>0.0003014819796742785</v>
+        <v>0.0003014819796742</v>
       </c>
       <c r="R126">
-        <v>0.0003014819796742785</v>
+        <v>0.0003014819796742</v>
       </c>
       <c r="S126">
         <v>9.849314539486388</v>
@@ -36174,16 +36228,16 @@
         <v>3.98532535238463</v>
       </c>
       <c r="U126">
-        <v>0.4366783408293085</v>
+        <v>0.4366783408293084</v>
       </c>
       <c r="V126">
         <v>0.6853692467580166</v>
       </c>
       <c r="W126">
-        <v>0.01152384743583983</v>
+        <v>0.0115238474358398</v>
       </c>
       <c r="X126">
-        <v>0.03760503838204008</v>
+        <v>0.03760503838204</v>
       </c>
       <c r="Y126">
         <v>0.133659095203956</v>
@@ -36195,13 +36249,13 @@
         <v>0.9997103948208556</v>
       </c>
       <c r="AB126">
-        <v>0.9241437817360305</v>
+        <v>0.9241437817360304</v>
       </c>
       <c r="AC126">
         <v>0.8686276318450761</v>
       </c>
       <c r="AD126">
-        <v>0.9994260410307935</v>
+        <v>0.9994260410307936</v>
       </c>
       <c r="AE126">
         <v>0.8666932819991978</v>
@@ -36210,31 +36264,31 @@
         <v>0.8338887911389863</v>
       </c>
       <c r="AG126">
-        <v>0.001956828295282353</v>
+        <v>0.0019568282952823</v>
       </c>
       <c r="AH126">
-        <v>0.00511308770784138</v>
+        <v>0.0051130877078413</v>
       </c>
       <c r="AI126">
         <v>0.9997103948208556</v>
       </c>
       <c r="AJ126">
-        <v>0.9994260410307935</v>
+        <v>0.9994260410307936</v>
       </c>
       <c r="AK126">
-        <v>0.001956828295282353</v>
+        <v>0.0019568282952823</v>
       </c>
       <c r="AL126">
-        <v>0.00511308770784138</v>
+        <v>0.0051130877078413</v>
       </c>
       <c r="AM126" t="s">
         <v>243</v>
       </c>
       <c r="AN126">
-        <v>0.01238684019763216</v>
+        <v>0.0123868401976321</v>
       </c>
       <c r="AO126">
-        <v>0.01546350412039389</v>
+        <v>0.0154635041203938</v>
       </c>
       <c r="AP126">
         <v>-1358.599824</v>
@@ -36258,7 +36312,7 @@
         <v>3.442345017599994</v>
       </c>
       <c r="AW126">
-        <v>0.2803078336399987</v>
+        <v>0.2803078336399986</v>
       </c>
       <c r="AX126">
         <v>2.432773386034256</v>
@@ -36276,7 +36330,7 @@
         <v>0</v>
       </c>
       <c r="BC126">
-        <v>0.003969329704302422</v>
+        <v>0.0039693297043024</v>
       </c>
       <c r="BD126">
         <v>0</v>
@@ -36345,25 +36399,25 @@
         <v>0.0341364664259203</v>
       </c>
       <c r="BZ126">
-        <v>0.06706763821893927</v>
+        <v>0.0670676382189392</v>
       </c>
       <c r="CA126">
-        <v>0.07138856039561405</v>
+        <v>0.071388560395614</v>
       </c>
       <c r="CB126">
         <v>0.1424950593520785</v>
       </c>
       <c r="CC126">
-        <v>0.01075237522634257</v>
+        <v>0.0107523752263425</v>
       </c>
       <c r="CD126">
-        <v>0.01511947735761453</v>
+        <v>0.0151194773576145</v>
       </c>
       <c r="CE126">
-        <v>0.00841073551070542</v>
+        <v>0.008410735510705401</v>
       </c>
       <c r="CF126">
-        <v>0.01330377112179511</v>
+        <v>0.0133037711217951</v>
       </c>
       <c r="CG126">
         <v>35782.05000000005</v>
@@ -36381,16 +36435,16 @@
         <v>0.1906279072499513</v>
       </c>
       <c r="CL126">
-        <v>0.04355217853927245</v>
+        <v>0.0435521785392724</v>
       </c>
       <c r="CM126">
         <v>10000</v>
       </c>
       <c r="CO126">
-        <v>0.001699104108742663</v>
+        <v>0.0016991041087426</v>
       </c>
       <c r="CP126">
-        <v>0.00390021624961384</v>
+        <v>0.0039002162496138</v>
       </c>
       <c r="CQ126">
         <v>7118836.508650885</v>
@@ -36398,8 +36452,8 @@
       <c r="CR126">
         <v>716228.3326648935</v>
       </c>
-      <c r="CS126" s="2">
-        <v>45415.46273133369</v>
+      <c r="CS126" t="s">
+        <v>367</v>
       </c>
       <c r="CT126">
         <v>-0.892232561911074</v>
@@ -36413,28 +36467,28 @@
         <v>188</v>
       </c>
       <c r="K127">
-        <v>0.002527200832158849</v>
+        <v>0.0025272008321588</v>
       </c>
       <c r="L127">
-        <v>0.001263600416079425</v>
+        <v>0.0012636004160794</v>
       </c>
       <c r="M127">
-        <v>0.000864585709725807</v>
+        <v>0.0008645857097258</v>
       </c>
       <c r="N127">
-        <v>0.000864585709725807</v>
+        <v>0.0008645857097258</v>
       </c>
       <c r="O127">
-        <v>0.002010600907909965</v>
+        <v>0.0020106009079099</v>
       </c>
       <c r="P127">
-        <v>0.001005300453954983</v>
+        <v>0.0010053004539549</v>
       </c>
       <c r="Q127">
-        <v>0.0005919703513717067</v>
+        <v>0.0005919703513717</v>
       </c>
       <c r="R127">
-        <v>0.0005919703513717067</v>
+        <v>0.0005919703513717</v>
       </c>
       <c r="S127">
         <v>11.98472163277904</v>
@@ -36452,13 +36506,13 @@
         <v>0.0528228472482147</v>
       </c>
       <c r="X127">
-        <v>0.09631323286308821</v>
+        <v>0.0963132328630882</v>
       </c>
       <c r="Y127">
         <v>0.2192686139069459</v>
       </c>
       <c r="Z127">
-        <v>0.2173845172835257</v>
+        <v>0.2173845172835256</v>
       </c>
       <c r="AA127">
         <v>0.9991045081436382</v>
@@ -36479,10 +36533,10 @@
         <v>0.7886800389953728</v>
       </c>
       <c r="AG127">
-        <v>0.006955633552441099</v>
+        <v>0.006955633552441</v>
       </c>
       <c r="AH127">
-        <v>0.01032672546198395</v>
+        <v>0.0103267254619839</v>
       </c>
       <c r="AI127">
         <v>0.9991045081436382</v>
@@ -36491,19 +36545,19 @@
         <v>0.9979048278191958</v>
       </c>
       <c r="AK127">
-        <v>0.006955633552441099</v>
+        <v>0.006955633552441</v>
       </c>
       <c r="AL127">
-        <v>0.01032672546198395</v>
+        <v>0.0103267254619839</v>
       </c>
       <c r="AM127" t="s">
         <v>243</v>
       </c>
       <c r="AN127">
-        <v>0.02767415259442773</v>
+        <v>0.0276741525944277</v>
       </c>
       <c r="AO127">
-        <v>0.06217967383121285</v>
+        <v>0.0621796738312128</v>
       </c>
       <c r="AP127">
         <v>-7121.356162382001</v>
@@ -36521,7 +36575,7 @@
         <v>152690.6199476184</v>
       </c>
       <c r="AU127">
-        <v>25181.80066095791</v>
+        <v>25181.8006609579</v>
       </c>
       <c r="AV127">
         <v>14.26906199476184</v>
@@ -36530,7 +36584,7 @@
         <v>1.542920276095791</v>
       </c>
       <c r="AX127">
-        <v>1.999603358574151</v>
+        <v>1.999603358574152</v>
       </c>
       <c r="AY127">
         <v>1.32465480208653</v>
@@ -36542,10 +36596,10 @@
         <v>108.2333333333333</v>
       </c>
       <c r="BB127">
-        <v>0.00234278296984482</v>
+        <v>0.0023427829698448</v>
       </c>
       <c r="BC127">
-        <v>0.09022560182748188</v>
+        <v>0.09022560182748179</v>
       </c>
       <c r="BD127">
         <v>-351.8011400289388</v>
@@ -36608,13 +36662,13 @@
         <v>142690.619947618</v>
       </c>
       <c r="BX127">
-        <v>15429.20276095801</v>
+        <v>15429.202760958</v>
       </c>
       <c r="BY127">
-        <v>0.04365272898899163</v>
+        <v>0.0436527289889916</v>
       </c>
       <c r="BZ127">
-        <v>0.08212539615751041</v>
+        <v>0.0821253961575104</v>
       </c>
       <c r="CA127">
         <v>0.1229319602606669</v>
@@ -36623,16 +36677,16 @@
         <v>0.1744545373326135</v>
       </c>
       <c r="CC127">
-        <v>0.009299389898866391</v>
+        <v>0.009299389898866301</v>
       </c>
       <c r="CD127">
-        <v>0.01616222911983619</v>
+        <v>0.0161622291198361</v>
       </c>
       <c r="CE127">
-        <v>0.008363201522622345</v>
+        <v>0.0083632015226223</v>
       </c>
       <c r="CF127">
-        <v>0.01188052573500747</v>
+        <v>0.0118805257350074</v>
       </c>
       <c r="CG127">
         <v>149811.97611</v>
@@ -36650,16 +36704,16 @@
         <v>0.2755459587308421</v>
       </c>
       <c r="CL127">
-        <v>0.08624386399016262</v>
+        <v>0.08624386399016259</v>
       </c>
       <c r="CM127">
         <v>10000</v>
       </c>
       <c r="CO127">
-        <v>0.007677469135802469</v>
+        <v>0.0076774691358024</v>
       </c>
       <c r="CP127">
-        <v>0.01990740740740741</v>
+        <v>0.0199074074074074</v>
       </c>
       <c r="CQ127">
         <v>47790589.85561877</v>
@@ -36667,8 +36721,8 @@
       <c r="CR127">
         <v>7960049.437302528</v>
       </c>
-      <c r="CS127" s="2">
-        <v>45415.73485744271</v>
+      <c r="CS127" t="s">
+        <v>368</v>
       </c>
       <c r="CT127">
         <v>-0.7368411844597273</v>
@@ -36682,28 +36736,28 @@
         <v>223</v>
       </c>
       <c r="K128">
-        <v>0.0009916708039618971</v>
+        <v>0.0009916708039618</v>
       </c>
       <c r="L128">
-        <v>0.0004958354019809486</v>
+        <v>0.0004958354019809</v>
       </c>
       <c r="M128">
-        <v>0.0004334120936875241</v>
+        <v>0.0004334120936875</v>
       </c>
       <c r="N128">
-        <v>0.0004334120936875241</v>
+        <v>0.0004334120936875</v>
       </c>
       <c r="O128">
-        <v>0.002243446688982042</v>
+        <v>0.002243446688982</v>
       </c>
       <c r="P128">
-        <v>0.001121723344491021</v>
+        <v>0.001121723344491</v>
       </c>
       <c r="Q128">
-        <v>0.0002452480551083935</v>
+        <v>0.0002452480551083</v>
       </c>
       <c r="R128">
-        <v>0.0002452480551083935</v>
+        <v>0.0002452480551083</v>
       </c>
       <c r="S128">
         <v>37.21347274200394</v>
@@ -36712,7 +36766,7 @@
         <v>5.266869863806474</v>
       </c>
       <c r="U128">
-        <v>0.4445259378977388</v>
+        <v>0.4445259378977387</v>
       </c>
       <c r="V128">
         <v>0.7853980331305344</v>
@@ -36721,25 +36775,25 @@
         <v>0.0125379628764633</v>
       </c>
       <c r="X128">
-        <v>0.008883600048393513</v>
+        <v>0.008883600048393499</v>
       </c>
       <c r="Y128">
-        <v>0.09006475387533798</v>
+        <v>0.0900647538753379</v>
       </c>
       <c r="Z128">
-        <v>0.03394554869229915</v>
+        <v>0.0339455486922991</v>
       </c>
       <c r="AA128">
         <v>0.9998017683325096</v>
       </c>
       <c r="AB128">
-        <v>0.9356801672223101</v>
+        <v>0.93568016722231</v>
       </c>
       <c r="AC128">
         <v>0.9812863454314013</v>
       </c>
       <c r="AD128">
-        <v>0.9997023184492735</v>
+        <v>0.9997023184492736</v>
       </c>
       <c r="AE128">
         <v>0.8827086764609655</v>
@@ -36748,31 +36802,31 @@
         <v>0.8851121996733892</v>
       </c>
       <c r="AG128">
-        <v>0.002106263143805456</v>
+        <v>0.0021062631438054</v>
       </c>
       <c r="AH128">
-        <v>0.001129927884937069</v>
+        <v>0.001129927884937</v>
       </c>
       <c r="AI128">
         <v>0.9998017683325096</v>
       </c>
       <c r="AJ128">
-        <v>0.9997023184492735</v>
+        <v>0.9997023184492736</v>
       </c>
       <c r="AK128">
-        <v>0.002106263143805456</v>
+        <v>0.0021062631438054</v>
       </c>
       <c r="AL128">
-        <v>0.001129927884937069</v>
+        <v>0.001129927884937</v>
       </c>
       <c r="AM128" t="s">
         <v>243</v>
       </c>
       <c r="AN128">
-        <v>0.006949816448382135</v>
+        <v>0.0069498164483821</v>
       </c>
       <c r="AO128">
-        <v>0.01124501323719901</v>
+        <v>0.011245013237199</v>
       </c>
       <c r="AP128">
         <v>-2171.26219778</v>
@@ -36811,7 +36865,7 @@
         <v>107.4333333333333</v>
       </c>
       <c r="BB128">
-        <v>0.002977066823538635</v>
+        <v>0.0029770668235386</v>
       </c>
       <c r="BC128">
         <v>0</v>
@@ -36880,28 +36934,28 @@
         <v>5967.42471716</v>
       </c>
       <c r="BY128">
-        <v>0.03039765112958839</v>
+        <v>0.0303976511295883</v>
       </c>
       <c r="BZ128">
         <v>0.0727068207574246</v>
       </c>
       <c r="CA128">
-        <v>0.04694679727294592</v>
+        <v>0.0469467972729459</v>
       </c>
       <c r="CB128">
-        <v>0.1186010659433643</v>
+        <v>0.1186010659433642</v>
       </c>
       <c r="CC128">
-        <v>0.01021563002336573</v>
+        <v>0.0102156300233657</v>
       </c>
       <c r="CD128">
-        <v>0.01685222400259557</v>
+        <v>0.0168522240025955</v>
       </c>
       <c r="CE128">
-        <v>0.007489848548474887</v>
+        <v>0.0074898485484748</v>
       </c>
       <c r="CF128">
-        <v>0.01524264633852101</v>
+        <v>0.015242646338521</v>
       </c>
       <c r="CG128">
         <v>21337.66830000001</v>
@@ -36919,16 +36973,16 @@
         <v>0.09727113573196911</v>
       </c>
       <c r="CL128">
-        <v>0.1645134634887986</v>
+        <v>0.1645134634887985</v>
       </c>
       <c r="CM128">
         <v>10000</v>
       </c>
       <c r="CO128">
-        <v>0.002237654320987654</v>
+        <v>0.0022376543209876</v>
       </c>
       <c r="CP128">
-        <v>0.0005401234567901234</v>
+        <v>0.0005401234567901</v>
       </c>
       <c r="CQ128">
         <v>6564078.281929377</v>
@@ -36936,11 +36990,11 @@
       <c r="CR128">
         <v>1259981.153790825</v>
       </c>
-      <c r="CS128" s="2">
-        <v>45415.90160276014</v>
+      <c r="CS128" t="s">
+        <v>369</v>
       </c>
       <c r="CT128">
-        <v>-0.9143802706411295</v>
+        <v>-0.9143802706411296</v>
       </c>
       <c r="CU128">
         <v>-0.9714369186341948</v>
@@ -36951,28 +37005,28 @@
         <v>225</v>
       </c>
       <c r="K129">
-        <v>0.0008442804144459526</v>
+        <v>0.0008442804144459</v>
       </c>
       <c r="L129">
-        <v>0.0004221402072229763</v>
+        <v>0.0004221402072229</v>
       </c>
       <c r="M129">
-        <v>0.001085110189479765</v>
+        <v>0.0010851101894797</v>
       </c>
       <c r="N129">
-        <v>0.001085110189479765</v>
+        <v>0.0010851101894797</v>
       </c>
       <c r="O129">
-        <v>0.0008512421775949575</v>
+        <v>0.0008512421775949</v>
       </c>
       <c r="P129">
-        <v>0.0004256210887974788</v>
+        <v>0.0004256210887974</v>
       </c>
       <c r="Q129">
-        <v>0.001127230022089409</v>
+        <v>0.0011272300220894</v>
       </c>
       <c r="R129">
-        <v>0.001127230022089409</v>
+        <v>0.0011272300220894</v>
       </c>
       <c r="S129">
         <v>8.785524132875498</v>
@@ -36981,16 +37035,16 @@
         <v>13.91164782591921</v>
       </c>
       <c r="U129">
-        <v>0.4003236475284112</v>
+        <v>0.4003236475284111</v>
       </c>
       <c r="V129">
         <v>0.5589109973727375</v>
       </c>
       <c r="W129">
-        <v>0.05352168823328322</v>
+        <v>0.0535216882332832</v>
       </c>
       <c r="X129">
-        <v>0.08258862992555079</v>
+        <v>0.0825886299255507</v>
       </c>
       <c r="Y129">
         <v>0.1318918477338805</v>
@@ -36999,7 +37053,7 @@
         <v>0.234691237232178</v>
       </c>
       <c r="AA129">
-        <v>0.9989424313782471</v>
+        <v>0.9989424313782472</v>
       </c>
       <c r="AB129">
         <v>0.8992973485146749</v>
@@ -37017,31 +37071,31 @@
         <v>0.7678936348016684</v>
       </c>
       <c r="AG129">
-        <v>0.005325052147641551</v>
+        <v>0.0053250521476415</v>
       </c>
       <c r="AH129">
-        <v>0.009728832881625836</v>
+        <v>0.0097288328816258</v>
       </c>
       <c r="AI129">
-        <v>0.9989424313782471</v>
+        <v>0.9989424313782472</v>
       </c>
       <c r="AJ129">
         <v>0.9980516147377282</v>
       </c>
       <c r="AK129">
-        <v>0.005325052147641551</v>
+        <v>0.0053250521476415</v>
       </c>
       <c r="AL129">
-        <v>0.009728832881625836</v>
+        <v>0.0097288328816258</v>
       </c>
       <c r="AM129" t="s">
         <v>243</v>
       </c>
       <c r="AN129">
-        <v>0.02756269827294157</v>
+        <v>0.0275626982729415</v>
       </c>
       <c r="AO129">
-        <v>0.07443085699132103</v>
+        <v>0.074430856991321</v>
       </c>
       <c r="AP129">
         <v>-784.2830687000001</v>
@@ -37080,10 +37134,10 @@
         <v>86.63333333333334</v>
       </c>
       <c r="BB129">
-        <v>0.04375585519857265</v>
+        <v>0.0437558551985726</v>
       </c>
       <c r="BC129">
-        <v>0.07952053879597674</v>
+        <v>0.0795205387959767</v>
       </c>
       <c r="BD129">
         <v>-716.6801106596547</v>
@@ -37149,28 +37203,28 @@
         <v>22259.85371694002</v>
       </c>
       <c r="BY129">
-        <v>0.05119753308813837</v>
+        <v>0.0511975330881383</v>
       </c>
       <c r="BZ129">
-        <v>0.07338592518482537</v>
+        <v>0.0733859251848253</v>
       </c>
       <c r="CA129">
-        <v>0.1007517646434705</v>
+        <v>0.1007517646434704</v>
       </c>
       <c r="CB129">
-        <v>0.1883847376217125</v>
+        <v>0.1883847376217124</v>
       </c>
       <c r="CC129">
-        <v>0.009808961510069625</v>
+        <v>0.009808961510069601</v>
       </c>
       <c r="CD129">
-        <v>0.007969733953587571</v>
+        <v>0.0079697339535875</v>
       </c>
       <c r="CE129">
-        <v>0.00918904401224825</v>
+        <v>0.009189044012248199</v>
       </c>
       <c r="CF129">
-        <v>0.01124691232412593</v>
+        <v>0.0112469123241259</v>
       </c>
       <c r="CG129">
         <v>15662.38749999999</v>
@@ -37194,10 +37248,10 @@
         <v>10000</v>
       </c>
       <c r="CO129">
-        <v>0.0002700617283950617</v>
+        <v>0.000270061728395</v>
       </c>
       <c r="CP129">
-        <v>0.01697530864197531</v>
+        <v>0.0169753086419753</v>
       </c>
       <c r="CQ129">
         <v>13221633.21657962</v>
@@ -37205,8 +37259,8 @@
       <c r="CR129">
         <v>16803825.65057263</v>
       </c>
-      <c r="CS129" s="2">
-        <v>45418.17086291177</v>
+      <c r="CS129" t="s">
+        <v>370</v>
       </c>
       <c r="CT129">
         <v>-0.8590793790924167</v>
@@ -37220,28 +37274,28 @@
         <v>231</v>
       </c>
       <c r="K130">
-        <v>0.001974030175498021</v>
+        <v>0.001974030175498</v>
       </c>
       <c r="L130">
-        <v>0.0009870150877490103</v>
+        <v>0.0009870150877490001</v>
       </c>
       <c r="M130">
-        <v>0.0007664952070594033</v>
+        <v>0.0007664952070594</v>
       </c>
       <c r="N130">
-        <v>0.0007664952070594033</v>
+        <v>0.0007664952070594</v>
       </c>
       <c r="O130">
-        <v>0.003173515670422167</v>
+        <v>0.0031735156704221</v>
       </c>
       <c r="P130">
-        <v>0.001586757835211083</v>
+        <v>0.001586757835211</v>
       </c>
       <c r="Q130">
-        <v>0.0007237887547192345</v>
+        <v>0.0007237887547192</v>
       </c>
       <c r="R130">
-        <v>0.0007237887547192345</v>
+        <v>0.0007237887547192</v>
       </c>
       <c r="S130">
         <v>17.059046147905</v>
@@ -37259,7 +37313,7 @@
         <v>0.038189920225125</v>
       </c>
       <c r="X130">
-        <v>0.09148465699256171</v>
+        <v>0.0914846569925617</v>
       </c>
       <c r="Y130">
         <v>0.2376398340586393</v>
@@ -37268,7 +37322,7 @@
         <v>0.2497684200301903</v>
       </c>
       <c r="AA130">
-        <v>0.9996187056501427</v>
+        <v>0.9996187056501428</v>
       </c>
       <c r="AB130">
         <v>0.8061992107897711</v>
@@ -37277,7 +37331,7 @@
         <v>0.8016372527597291</v>
       </c>
       <c r="AD130">
-        <v>0.9966353723638919</v>
+        <v>0.996635372363892</v>
       </c>
       <c r="AE130">
         <v>0.7625286078451134</v>
@@ -37286,31 +37340,31 @@
         <v>0.6727893426624312</v>
       </c>
       <c r="AG130">
-        <v>0.005654459134801621</v>
+        <v>0.0056544591348016</v>
       </c>
       <c r="AH130">
-        <v>0.01156385279379274</v>
+        <v>0.0115638527937927</v>
       </c>
       <c r="AI130">
-        <v>0.9996187056501427</v>
+        <v>0.9996187056501428</v>
       </c>
       <c r="AJ130">
-        <v>0.9966353723638919</v>
+        <v>0.996635372363892</v>
       </c>
       <c r="AK130">
-        <v>0.005654459134801621</v>
+        <v>0.0056544591348016</v>
       </c>
       <c r="AL130">
-        <v>0.01156385279379274</v>
+        <v>0.0115638527937927</v>
       </c>
       <c r="AM130" t="s">
         <v>243</v>
       </c>
       <c r="AN130">
-        <v>0.009514899377222377</v>
+        <v>0.009514899377222301</v>
       </c>
       <c r="AO130">
-        <v>0.07002115137346268</v>
+        <v>0.0700211513734626</v>
       </c>
       <c r="AP130">
         <v>-4588.53556124</v>
@@ -37322,7 +37376,7 @@
         <v>83963.47843875979</v>
       </c>
       <c r="AS130">
-        <v>22857.62349650046</v>
+        <v>22857.62349650045</v>
       </c>
       <c r="AT130">
         <v>83963.47843875979</v>
@@ -37349,7 +37403,7 @@
         <v>109.1666666666667</v>
       </c>
       <c r="BB130">
-        <v>0.01167312073209618</v>
+        <v>0.0116731207320961</v>
       </c>
       <c r="BC130">
         <v>0</v>
@@ -37418,7 +37472,7 @@
         <v>12857.62349649998</v>
       </c>
       <c r="BY130">
-        <v>0.02849449704352394</v>
+        <v>0.0284944970435239</v>
       </c>
       <c r="BZ130">
         <v>0.1223428777591633</v>
@@ -37430,16 +37484,16 @@
         <v>0.1997916794785066</v>
       </c>
       <c r="CC130">
-        <v>0.005765234951725934</v>
+        <v>0.0057652349517259</v>
       </c>
       <c r="CD130">
-        <v>0.01652623708768868</v>
+        <v>0.0165262370876886</v>
       </c>
       <c r="CE130">
-        <v>0.007299010812043965</v>
+        <v>0.0072990108120439</v>
       </c>
       <c r="CF130">
-        <v>0.02028416007817126</v>
+        <v>0.0202841600781712</v>
       </c>
       <c r="CG130">
         <v>78552.01399999994</v>
@@ -37457,16 +37511,16 @@
         <v>0.1836778542965224</v>
       </c>
       <c r="CL130">
-        <v>0.08538577050201569</v>
+        <v>0.0853857705020156</v>
       </c>
       <c r="CM130">
         <v>10000</v>
       </c>
       <c r="CO130">
-        <v>0.004402224281742354</v>
+        <v>0.0044022242817423</v>
       </c>
       <c r="CP130">
-        <v>0.002201112140871177</v>
+        <v>0.0022011121408711</v>
       </c>
       <c r="CQ130">
         <v>36758077.75906376</v>
@@ -37474,8 +37528,8 @@
       <c r="CR130">
         <v>7461415.917733567</v>
       </c>
-      <c r="CS130" s="2">
-        <v>45418.3290608931</v>
+      <c r="CS130" t="s">
+        <v>371</v>
       </c>
       <c r="CT130">
         <v>-0.7834455371012616</v>
@@ -37489,28 +37543,28 @@
         <v>235</v>
       </c>
       <c r="K131">
-        <v>0.001339537874347929</v>
+        <v>0.0013395378743479</v>
       </c>
       <c r="L131">
-        <v>0.0006697689371739646</v>
+        <v>0.0006697689371739</v>
       </c>
       <c r="M131">
-        <v>0.0005374852835609012</v>
+        <v>0.0005374852835609</v>
       </c>
       <c r="N131">
-        <v>0.0005374852835609012</v>
+        <v>0.0005374852835609</v>
       </c>
       <c r="O131">
-        <v>0.002176102086959663</v>
+        <v>0.0021761020869596</v>
       </c>
       <c r="P131">
-        <v>0.001088051043479832</v>
+        <v>0.0010880510434798</v>
       </c>
       <c r="Q131">
-        <v>0.0008691624567908063</v>
+        <v>0.0008691624567908</v>
       </c>
       <c r="R131">
-        <v>0.0008691624567908063</v>
+        <v>0.0008691624567908</v>
       </c>
       <c r="S131">
         <v>12.16634497280225</v>
@@ -37519,16 +37573,16 @@
         <v>8.236181786278294</v>
       </c>
       <c r="U131">
-        <v>0.3712811428587015</v>
+        <v>0.3712811428587014</v>
       </c>
       <c r="V131">
         <v>0.6888497180676669</v>
       </c>
       <c r="W131">
-        <v>0.08655526110596123</v>
+        <v>0.08655526110596121</v>
       </c>
       <c r="X131">
-        <v>0.05723982251474728</v>
+        <v>0.0572398225147472</v>
       </c>
       <c r="Y131">
         <v>0.2344143337672382</v>
@@ -37537,7 +37591,7 @@
         <v>0.1426300321036997</v>
       </c>
       <c r="AA131">
-        <v>0.9991700579884613</v>
+        <v>0.9991700579884611</v>
       </c>
       <c r="AB131">
         <v>0.8011728703136501</v>
@@ -37546,7 +37600,7 @@
         <v>0.8696704621071671</v>
       </c>
       <c r="AD131">
-        <v>0.9992041267369297</v>
+        <v>0.9992041267369296</v>
       </c>
       <c r="AE131">
         <v>0.7665933382226603</v>
@@ -37555,31 +37609,31 @@
         <v>0.857632976502503</v>
       </c>
       <c r="AG131">
-        <v>0.007227404012196759</v>
+        <v>0.0072274040121967</v>
       </c>
       <c r="AH131">
-        <v>0.006661789739206238</v>
+        <v>0.0066617897392062</v>
       </c>
       <c r="AI131">
-        <v>0.9991700579884613</v>
+        <v>0.9991700579884611</v>
       </c>
       <c r="AJ131">
-        <v>0.9992041267369297</v>
+        <v>0.9992041267369296</v>
       </c>
       <c r="AK131">
-        <v>0.007227404012196759</v>
+        <v>0.0072274040121967</v>
       </c>
       <c r="AL131">
-        <v>0.006661789739206238</v>
+        <v>0.0066617897392062</v>
       </c>
       <c r="AM131" t="s">
         <v>243</v>
       </c>
       <c r="AN131">
-        <v>0.01752408109593183</v>
+        <v>0.0175240810959318</v>
       </c>
       <c r="AO131">
-        <v>0.01843302335277237</v>
+        <v>0.0184330233527723</v>
       </c>
       <c r="AP131">
         <v>-1500.0518362</v>
@@ -37618,10 +37672,10 @@
         <v>95.40000000000001</v>
       </c>
       <c r="BB131">
-        <v>0.08274042588622789</v>
+        <v>0.08274042588622781</v>
       </c>
       <c r="BC131">
-        <v>0.01189502443277505</v>
+        <v>0.011895024432775</v>
       </c>
       <c r="BD131">
         <v>-2450.078072530424</v>
@@ -37687,28 +37741,28 @@
         <v>6659.312706200015</v>
       </c>
       <c r="BY131">
-        <v>0.04965626675578699</v>
+        <v>0.0496562667557869</v>
       </c>
       <c r="BZ131">
-        <v>0.08680051762198861</v>
+        <v>0.08680051762198859</v>
       </c>
       <c r="CA131">
-        <v>0.132084447379597</v>
+        <v>0.1320844473795969</v>
       </c>
       <c r="CB131">
         <v>0.1255909306850455</v>
       </c>
       <c r="CC131">
-        <v>0.009041564726442719</v>
+        <v>0.0090415647264427</v>
       </c>
       <c r="CD131">
-        <v>0.01578562667923071</v>
+        <v>0.0157856266792307</v>
       </c>
       <c r="CE131">
-        <v>0.009649947442705817</v>
+        <v>0.0096499474427058</v>
       </c>
       <c r="CF131">
-        <v>0.01593983778482089</v>
+        <v>0.0159398377848208</v>
       </c>
       <c r="CG131">
         <v>27161.54219999996</v>
@@ -37726,16 +37780,16 @@
         <v>0.1670495380138063</v>
       </c>
       <c r="CL131">
-        <v>0.09637602883577172</v>
+        <v>0.0963760288357717</v>
       </c>
       <c r="CM131">
         <v>10000</v>
       </c>
       <c r="CO131">
-        <v>0.00307057946220994</v>
+        <v>0.0030705794622099</v>
       </c>
       <c r="CP131">
-        <v>0.009650392595516954</v>
+        <v>0.0096503925955169</v>
       </c>
       <c r="CQ131">
         <v>8177676.867132748</v>
@@ -37743,8 +37797,8 @@
       <c r="CR131">
         <v>1295517.443775632</v>
       </c>
-      <c r="CS131" s="2">
-        <v>45418.65603952249</v>
+      <c r="CS131" t="s">
+        <v>372</v>
       </c>
       <c r="CT131">
         <v>-0.7832286955751367</v>
@@ -37758,28 +37812,28 @@
         <v>238</v>
       </c>
       <c r="K132">
-        <v>0.001619052131043075</v>
+        <v>0.001619052131043</v>
       </c>
       <c r="L132">
-        <v>0.0008095260655215375</v>
+        <v>0.0008095260655215</v>
       </c>
       <c r="M132">
-        <v>0.0004849124586081555</v>
+        <v>0.0004849124586081</v>
       </c>
       <c r="N132">
-        <v>0.0004849124586081555</v>
+        <v>0.0004849124586081</v>
       </c>
       <c r="O132">
-        <v>0.002865906751505731</v>
+        <v>0.0028659067515057</v>
       </c>
       <c r="P132">
-        <v>0.001432953375752866</v>
+        <v>0.0014329533757528</v>
       </c>
       <c r="Q132">
-        <v>0.0003753074203771467</v>
+        <v>0.0003753074203771</v>
       </c>
       <c r="R132">
-        <v>0.0003753074203771467</v>
+        <v>0.0003753074203771</v>
       </c>
       <c r="S132">
         <v>49.23430687912342</v>
@@ -37794,19 +37848,19 @@
         <v>0.6491882734410773</v>
       </c>
       <c r="W132">
-        <v>0.04742909684571316</v>
+        <v>0.0474290968457131</v>
       </c>
       <c r="X132">
-        <v>0.06399019998004046</v>
+        <v>0.06399019998004039</v>
       </c>
       <c r="Y132">
-        <v>0.186720952377867</v>
+        <v>0.1867209523778669</v>
       </c>
       <c r="Z132">
         <v>0.1818627031253102</v>
       </c>
       <c r="AA132">
-        <v>0.9994451109296455</v>
+        <v>0.9994451109296456</v>
       </c>
       <c r="AB132">
         <v>0.8422885164857498</v>
@@ -37824,31 +37878,31 @@
         <v>0.8186404304999623</v>
       </c>
       <c r="AG132">
-        <v>0.005712984308084144</v>
+        <v>0.0057129843080841</v>
       </c>
       <c r="AH132">
-        <v>0.007351154378554608</v>
+        <v>0.0073511543785546</v>
       </c>
       <c r="AI132">
-        <v>0.9994451109296455</v>
+        <v>0.9994451109296456</v>
       </c>
       <c r="AJ132">
         <v>0.9990874250882764</v>
       </c>
       <c r="AK132">
-        <v>0.005712984308084144</v>
+        <v>0.0057129843080841</v>
       </c>
       <c r="AL132">
-        <v>0.007351154378554608</v>
+        <v>0.0073511543785546</v>
       </c>
       <c r="AM132" t="s">
         <v>243</v>
       </c>
       <c r="AN132">
-        <v>0.01714805100715212</v>
+        <v>0.0171480510071521</v>
       </c>
       <c r="AO132">
-        <v>0.02867624612728114</v>
+        <v>0.0286762461272811</v>
       </c>
       <c r="AP132">
         <v>-7368.071834006001</v>
@@ -37887,10 +37941,10 @@
         <v>63.33333333333334</v>
       </c>
       <c r="BB132">
-        <v>0.004789157600066273</v>
+        <v>0.0047891576000662</v>
       </c>
       <c r="BC132">
-        <v>0.03222183572129598</v>
+        <v>0.0322218357212959</v>
       </c>
       <c r="BD132">
         <v>-263.454523847167</v>
@@ -37956,10 +38010,10 @@
         <v>6880.235050870009</v>
       </c>
       <c r="BY132">
-        <v>0.02765658510849759</v>
+        <v>0.0276565851084975</v>
       </c>
       <c r="BZ132">
-        <v>0.06898786131825328</v>
+        <v>0.0689878613182532</v>
       </c>
       <c r="CA132">
         <v>0.1027690788009489</v>
@@ -37968,13 +38022,13 @@
         <v>0.1542030494708696</v>
       </c>
       <c r="CC132">
-        <v>0.005666643278276891</v>
+        <v>0.0056666432782768</v>
       </c>
       <c r="CD132">
-        <v>0.00823534817457002</v>
+        <v>0.008235348174570001</v>
       </c>
       <c r="CE132">
-        <v>0.005559434035218185</v>
+        <v>0.0055594340352181</v>
       </c>
       <c r="CF132">
         <v>0.0090508498302827</v>
@@ -37992,28 +38046,28 @@
         <v>9082.567084525232</v>
       </c>
       <c r="CK132">
-        <v>0.184462208922361</v>
+        <v>0.1844622089223609</v>
       </c>
       <c r="CL132">
-        <v>0.07276783020470783</v>
+        <v>0.0727678302047078</v>
       </c>
       <c r="CM132">
         <v>10000</v>
       </c>
       <c r="CO132">
-        <v>0.008912037037037038</v>
+        <v>0.008912037037037</v>
       </c>
       <c r="CP132">
-        <v>0.01006944444444445</v>
+        <v>0.0100694444444444</v>
       </c>
       <c r="CQ132">
-        <v>26666806.02181739</v>
+        <v>26666806.02181738</v>
       </c>
       <c r="CR132">
         <v>7436893.530962305</v>
       </c>
-      <c r="CS132" s="2">
-        <v>45419.14449996537</v>
+      <c r="CS132" t="s">
+        <v>373</v>
       </c>
       <c r="CT132">
         <v>-0.8091587172086132</v>
@@ -38027,28 +38081,28 @@
         <v>241</v>
       </c>
       <c r="K133">
-        <v>0.00109613729693403</v>
+        <v>0.001096137296934</v>
       </c>
       <c r="L133">
-        <v>0.000548068648467015</v>
+        <v>0.000548068648467</v>
       </c>
       <c r="M133">
-        <v>0.0003855285575780076</v>
+        <v>0.000385528557578</v>
       </c>
       <c r="N133">
-        <v>0.0003855285575780076</v>
+        <v>0.000385528557578</v>
       </c>
       <c r="O133">
-        <v>0.002113526564414414</v>
+        <v>0.0021135265644144</v>
       </c>
       <c r="P133">
-        <v>0.001056763282207207</v>
+        <v>0.0010567632822072</v>
       </c>
       <c r="Q133">
-        <v>0.000513237959412427</v>
+        <v>0.0005132379594124</v>
       </c>
       <c r="R133">
-        <v>0.000513237959412427</v>
+        <v>0.0005132379594124</v>
       </c>
       <c r="S133">
         <v>6.797296775439275</v>
@@ -38063,16 +38117,16 @@
         <v>0.6158266826889449</v>
       </c>
       <c r="W133">
-        <v>0.02190812671745069</v>
+        <v>0.0219081267174506</v>
       </c>
       <c r="X133">
-        <v>0.02930266156908121</v>
+        <v>0.0293026615690812</v>
       </c>
       <c r="Y133">
         <v>0.1006605505523412</v>
       </c>
       <c r="Z133">
-        <v>0.115378037190302</v>
+        <v>0.1153780371903019</v>
       </c>
       <c r="AA133">
         <v>0.9996795065910724</v>
@@ -38081,10 +38135,10 @@
         <v>0.9322605002468208</v>
       </c>
       <c r="AC133">
-        <v>0.9097093464615931</v>
+        <v>0.9097093464615932</v>
       </c>
       <c r="AD133">
-        <v>0.9994606671523855</v>
+        <v>0.9994606671523856</v>
       </c>
       <c r="AE133">
         <v>0.8737986469747442</v>
@@ -38093,31 +38147,31 @@
         <v>0.8853173226108123</v>
       </c>
       <c r="AG133">
-        <v>0.002554463849785888</v>
+        <v>0.0025544638497858</v>
       </c>
       <c r="AH133">
-        <v>0.003373041808746848</v>
+        <v>0.0033730418087468</v>
       </c>
       <c r="AI133">
         <v>0.9996795065910724</v>
       </c>
       <c r="AJ133">
-        <v>0.9994606671523855</v>
+        <v>0.9994606671523856</v>
       </c>
       <c r="AK133">
-        <v>0.002554463849785888</v>
+        <v>0.0025544638497858</v>
       </c>
       <c r="AL133">
-        <v>0.003373041808746848</v>
+        <v>0.0033730418087468</v>
       </c>
       <c r="AM133" t="s">
         <v>243</v>
       </c>
       <c r="AN133">
-        <v>0.009616489085314019</v>
+        <v>0.009616489085314</v>
       </c>
       <c r="AO133">
-        <v>0.01397628572330174</v>
+        <v>0.0139762857233017</v>
       </c>
       <c r="AP133">
         <v>-758.5693892524</v>
@@ -38156,10 +38210,10 @@
         <v>112.3166666666667</v>
       </c>
       <c r="BB133">
-        <v>0.01085916950552062</v>
+        <v>0.0108591695055206</v>
       </c>
       <c r="BC133">
-        <v>0.00789172942731734</v>
+        <v>0.0078917294273173</v>
       </c>
       <c r="BD133">
         <v>-256.5509047890893</v>
@@ -38225,28 +38279,28 @@
         <v>5157.177460282007</v>
       </c>
       <c r="BY133">
-        <v>0.03740348296837005</v>
+        <v>0.03740348296837</v>
       </c>
       <c r="BZ133">
         <v>0.1019111071106316</v>
       </c>
       <c r="CA133">
-        <v>0.07487268591233054</v>
+        <v>0.0748726859123305</v>
       </c>
       <c r="CB133">
         <v>0.1673053259867567</v>
       </c>
       <c r="CC133">
-        <v>0.01231132187437749</v>
+        <v>0.0123113218743774</v>
       </c>
       <c r="CD133">
-        <v>0.01875398931966051</v>
+        <v>0.0187539893196605</v>
       </c>
       <c r="CE133">
-        <v>0.009624575333654458</v>
+        <v>0.009624575333654401</v>
       </c>
       <c r="CF133">
-        <v>0.01810812085591623</v>
+        <v>0.0181081208559162</v>
       </c>
       <c r="CG133">
         <v>23368.727682</v>
@@ -38270,10 +38324,10 @@
         <v>10000</v>
       </c>
       <c r="CO133">
-        <v>0.0009654000617856039</v>
+        <v>0.0009654000617856</v>
       </c>
       <c r="CP133">
-        <v>0.002587272165585418</v>
+        <v>0.0025872721655854</v>
       </c>
       <c r="CQ133">
         <v>4329727.394136436</v>
@@ -38281,8 +38335,8 @@
       <c r="CR133">
         <v>867003.1587181734</v>
       </c>
-      <c r="CS133" s="2">
-        <v>45419.30912299596</v>
+      <c r="CS133" t="s">
+        <v>374</v>
       </c>
       <c r="CT133">
         <v>-0.9000180936758766</v>
@@ -38296,28 +38350,28 @@
         <v>236</v>
       </c>
       <c r="K134">
-        <v>0.002101848400442918</v>
+        <v>0.0021018484004429</v>
       </c>
       <c r="L134">
-        <v>0.001050924200221459</v>
+        <v>0.0010509242002214</v>
       </c>
       <c r="M134">
-        <v>0.0006313105550932452</v>
+        <v>0.0006313105550932</v>
       </c>
       <c r="N134">
-        <v>0.0006313105550932452</v>
+        <v>0.0006313105550932</v>
       </c>
       <c r="O134">
-        <v>0.002227915942938385</v>
+        <v>0.0022279159429383</v>
       </c>
       <c r="P134">
-        <v>0.001113957971469193</v>
+        <v>0.0011139579714691</v>
       </c>
       <c r="Q134">
-        <v>0.0005565032532460767</v>
+        <v>0.000556503253246</v>
       </c>
       <c r="R134">
-        <v>0.0005565032532460767</v>
+        <v>0.000556503253246</v>
       </c>
       <c r="S134">
         <v>11.08939949797258</v>
@@ -38326,7 +38380,7 @@
         <v>17.26943425371693</v>
       </c>
       <c r="U134">
-        <v>0.3609445505025619</v>
+        <v>0.3609445505025618</v>
       </c>
       <c r="V134">
         <v>0.7628755660380135</v>
@@ -38335,7 +38389,7 @@
         <v>0.07497471142276969</v>
       </c>
       <c r="X134">
-        <v>0.09191635575593667</v>
+        <v>0.0919163557559366</v>
       </c>
       <c r="Y134">
         <v>0.1819636019003284</v>
@@ -38344,7 +38398,7 @@
         <v>0.16595411714472</v>
       </c>
       <c r="AA134">
-        <v>0.9986188553281209</v>
+        <v>0.9986188553281208</v>
       </c>
       <c r="AB134">
         <v>0.8388196141906518</v>
@@ -38362,19 +38416,19 @@
         <v>0.8648435249412598</v>
       </c>
       <c r="AG134">
-        <v>0.008452667068119072</v>
+        <v>0.008452667068119001</v>
       </c>
       <c r="AH134">
         <v>0.0074087938346481</v>
       </c>
       <c r="AI134">
-        <v>0.9986188553281209</v>
+        <v>0.9986188553281208</v>
       </c>
       <c r="AJ134">
         <v>0.9986760497381962</v>
       </c>
       <c r="AK134">
-        <v>0.008452667068119072</v>
+        <v>0.008452667068119001</v>
       </c>
       <c r="AL134">
         <v>0.0074087938346481</v>
@@ -38386,7 +38440,7 @@
         <v>0.0409391807131387</v>
       </c>
       <c r="AO134">
-        <v>0.04359215015688549</v>
+        <v>0.0435921501568854</v>
       </c>
       <c r="AP134">
         <v>-3992.23056225</v>
@@ -38398,19 +38452,19 @@
         <v>96352.36892775018</v>
       </c>
       <c r="AS134">
-        <v>19757.39707626811</v>
+        <v>19757.39707626812</v>
       </c>
       <c r="AT134">
         <v>96346.46882775018</v>
       </c>
       <c r="AU134">
-        <v>19560.63988626811</v>
+        <v>19560.63988626812</v>
       </c>
       <c r="AV134">
         <v>8.635236892775019</v>
       </c>
       <c r="AW134">
-        <v>0.9757397076268113</v>
+        <v>0.9757397076268112</v>
       </c>
       <c r="AX134">
         <v>2.157427839072774</v>
@@ -38425,10 +38479,10 @@
         <v>112.9833333333333</v>
       </c>
       <c r="BB134">
-        <v>0.00671778289806858</v>
+        <v>0.0067177828980685</v>
       </c>
       <c r="BC134">
-        <v>0.07546925217090274</v>
+        <v>0.0754692521709027</v>
       </c>
       <c r="BD134">
         <v>-611.0201058039232</v>
@@ -38494,28 +38548,28 @@
         <v>9757.397076268004</v>
       </c>
       <c r="BY134">
-        <v>0.04261636952293211</v>
+        <v>0.0426163695229321</v>
       </c>
       <c r="BZ134">
-        <v>0.07123040629672342</v>
+        <v>0.07123040629672341</v>
       </c>
       <c r="CA134">
-        <v>0.09984147157001007</v>
+        <v>0.09984147157001</v>
       </c>
       <c r="CB134">
-        <v>0.1204562214465475</v>
+        <v>0.1204562214465474</v>
       </c>
       <c r="CC134">
-        <v>0.008774411655161492</v>
+        <v>0.0087744116551614</v>
       </c>
       <c r="CD134">
-        <v>0.01139401041874235</v>
+        <v>0.0113940104187423</v>
       </c>
       <c r="CE134">
-        <v>0.00794777925724508</v>
+        <v>0.007947779257245</v>
       </c>
       <c r="CF134">
-        <v>0.009742705404139029</v>
+        <v>0.009742705404139001</v>
       </c>
       <c r="CG134">
         <v>90344.59949000004</v>
@@ -38533,25 +38587,25 @@
         <v>0.2305189619087169</v>
       </c>
       <c r="CL134">
-        <v>0.08413465918659893</v>
+        <v>0.0841346591865989</v>
       </c>
       <c r="CM134">
         <v>10000</v>
       </c>
       <c r="CO134">
-        <v>0.01015600864998455</v>
+        <v>0.0101560086499845</v>
       </c>
       <c r="CP134">
-        <v>0.008611368551127587</v>
+        <v>0.008611368551127501</v>
       </c>
       <c r="CQ134">
-        <v>66742737.91777743</v>
+        <v>66742737.91777744</v>
       </c>
       <c r="CR134">
         <v>3390202.150984915</v>
       </c>
-      <c r="CS134" s="2">
-        <v>45419.52005372911</v>
+      <c r="CS134" t="s">
+        <v>375</v>
       </c>
       <c r="CT134">
         <v>-0.6893066803315582</v>
@@ -38565,22 +38619,22 @@
         <v>242</v>
       </c>
       <c r="K135">
-        <v>0.001848957601374712</v>
+        <v>0.0018489576013747</v>
       </c>
       <c r="L135">
-        <v>0.0009244788006873561</v>
+        <v>0.0009244788006873001</v>
       </c>
       <c r="M135">
-        <v>0.0006897374777841137</v>
+        <v>0.0006897374777841</v>
       </c>
       <c r="N135">
-        <v>0.0006897374777841137</v>
+        <v>0.0006897374777841</v>
       </c>
       <c r="O135">
-        <v>0.0002519402379465907</v>
+        <v>0.0002519402379465</v>
       </c>
       <c r="P135">
-        <v>0.0001259701189732953</v>
+        <v>0.0001259701189732</v>
       </c>
       <c r="Q135">
         <v>9.525440661337648E-05</v>
@@ -38589,7 +38643,7 @@
         <v>9.525440661337648E-05</v>
       </c>
       <c r="S135">
-        <v>1.318569389251129</v>
+        <v>1.318569389251128</v>
       </c>
       <c r="T135">
         <v>11.76156487518809</v>
@@ -38601,10 +38655,10 @@
         <v>0.6240297615846883</v>
       </c>
       <c r="W135">
-        <v>0.04483228600930598</v>
+        <v>0.0448322860093059</v>
       </c>
       <c r="X135">
-        <v>0.08392388039386765</v>
+        <v>0.0839238803938676</v>
       </c>
       <c r="Y135">
         <v>0.2375959329469452</v>
@@ -38613,7 +38667,7 @@
         <v>0.2022545722996491</v>
       </c>
       <c r="AA135">
-        <v>1.000313892475625</v>
+        <v>1.000313892475624</v>
       </c>
       <c r="AB135">
         <v>0.825763021135087</v>
@@ -38622,7 +38676,7 @@
         <v>0.8297340005497663</v>
       </c>
       <c r="AD135">
-        <v>0.9989870165198325</v>
+        <v>0.9989870165198323</v>
       </c>
       <c r="AE135">
         <v>0.7627092298595899</v>
@@ -38631,22 +38685,22 @@
         <v>0.7978945436031236</v>
       </c>
       <c r="AG135">
-        <v>0.006220720603331166</v>
+        <v>0.0062207206033311</v>
       </c>
       <c r="AH135">
-        <v>0.008384924165057999</v>
+        <v>0.0083849241650579</v>
       </c>
       <c r="AI135">
-        <v>1.000313892475625</v>
+        <v>1.000313892475624</v>
       </c>
       <c r="AJ135">
-        <v>0.9989870165198325</v>
+        <v>0.9989870165198323</v>
       </c>
       <c r="AK135">
-        <v>0.006220720603331166</v>
+        <v>0.0062207206033311</v>
       </c>
       <c r="AL135">
-        <v>0.008384924165057999</v>
+        <v>0.0083849241650579</v>
       </c>
       <c r="AM135" t="s">
         <v>243</v>
@@ -38655,7 +38709,7 @@
         <v>0.0422126511911422</v>
       </c>
       <c r="AO135">
-        <v>0.02670053916945107</v>
+        <v>0.026700539169451</v>
       </c>
       <c r="AP135">
         <v>-2577.8704428</v>
@@ -38763,10 +38817,10 @@
         <v>11056.64230969996</v>
       </c>
       <c r="BY135">
-        <v>0.03684354716871903</v>
+        <v>0.036843547168719</v>
       </c>
       <c r="BZ135">
-        <v>0.06940029673870404</v>
+        <v>0.069400296738704</v>
       </c>
       <c r="CA135">
         <v>0.1345163957012951</v>
@@ -38775,16 +38829,16 @@
         <v>0.1681132500281438</v>
       </c>
       <c r="CC135">
-        <v>0.01352934217609617</v>
+        <v>0.0135293421760961</v>
       </c>
       <c r="CD135">
-        <v>0.01247992650366996</v>
+        <v>0.0124799265036699</v>
       </c>
       <c r="CE135">
-        <v>0.004839755024427521</v>
+        <v>0.0048397550244275</v>
       </c>
       <c r="CF135">
-        <v>0.01151226577087958</v>
+        <v>0.0115122657708795</v>
       </c>
       <c r="CG135">
         <v>66096.47800000003</v>
@@ -38799,19 +38853,19 @@
         <v>13359.44115055043</v>
       </c>
       <c r="CK135">
-        <v>0.2362928116558319</v>
+        <v>0.2362928116558318</v>
       </c>
       <c r="CL135">
-        <v>0.06475128703067912</v>
+        <v>0.0647512870306791</v>
       </c>
       <c r="CM135">
         <v>10000</v>
       </c>
       <c r="CO135">
-        <v>0.006790123456790123</v>
+        <v>0.0067901234567901</v>
       </c>
       <c r="CP135">
-        <v>0.01053240740740741</v>
+        <v>0.0105324074074074</v>
       </c>
       <c r="CQ135">
         <v>7948953.840563923</v>
@@ -38819,8 +38873,8 @@
       <c r="CR135">
         <v>8715912.703511165</v>
       </c>
-      <c r="CS135" s="2">
-        <v>45419.7432346184</v>
+      <c r="CS135" t="s">
+        <v>376</v>
       </c>
       <c r="CT135">
         <v>-0.8034449984146571</v>
@@ -38834,28 +38888,28 @@
         <v>197</v>
       </c>
       <c r="K136">
-        <v>0.001564964211886233</v>
+        <v>0.0015649642118862</v>
       </c>
       <c r="L136">
-        <v>0.0007824821059431164</v>
+        <v>0.0007824821059431</v>
       </c>
       <c r="M136">
-        <v>0.001934162331862277</v>
+        <v>0.0019341623318622</v>
       </c>
       <c r="N136">
-        <v>0.001934162331862277</v>
+        <v>0.0019341623318622</v>
       </c>
       <c r="O136">
-        <v>0.003644722717055559</v>
+        <v>0.0036447227170555</v>
       </c>
       <c r="P136">
-        <v>0.00182236135852778</v>
+        <v>0.0018223613585277</v>
       </c>
       <c r="Q136">
-        <v>0.002117123544176236</v>
+        <v>0.0021171235441762</v>
       </c>
       <c r="R136">
-        <v>0.002117123544176236</v>
+        <v>0.0021171235441762</v>
       </c>
       <c r="S136">
         <v>11.14382148884305</v>
@@ -38870,10 +38924,10 @@
         <v>0.6954412932967299</v>
       </c>
       <c r="W136">
-        <v>0.06660305564760288</v>
+        <v>0.0666030556476028</v>
       </c>
       <c r="X136">
-        <v>0.07428647687703471</v>
+        <v>0.0742864768770347</v>
       </c>
       <c r="Y136">
         <v>0.181465014282819</v>
@@ -38891,7 +38945,7 @@
         <v>0.8476045088759191</v>
       </c>
       <c r="AD136">
-        <v>0.9988154694670831</v>
+        <v>0.9988154694670832</v>
       </c>
       <c r="AE136">
         <v>0.7220270555159511</v>
@@ -38900,34 +38954,34 @@
         <v>0.8225972088743163</v>
       </c>
       <c r="AG136">
-        <v>0.006047226374347921</v>
+        <v>0.0060472263743479</v>
       </c>
       <c r="AH136">
-        <v>0.008401051909799786</v>
+        <v>0.008401051909799701</v>
       </c>
       <c r="AI136">
         <v>0.999200058456911</v>
       </c>
       <c r="AJ136">
-        <v>0.9988154694670831</v>
+        <v>0.9988154694670832</v>
       </c>
       <c r="AK136">
-        <v>0.006047226374347921</v>
+        <v>0.0060472263743479</v>
       </c>
       <c r="AL136">
-        <v>0.008401051909799786</v>
+        <v>0.008401051909799701</v>
       </c>
       <c r="AM136" t="s">
         <v>243</v>
       </c>
       <c r="AN136">
-        <v>0.02071059035954705</v>
+        <v>0.020710590359547</v>
       </c>
       <c r="AO136">
-        <v>0.03916270565598065</v>
+        <v>0.0391627056559806</v>
       </c>
       <c r="AP136">
-        <v>-947.5506029400001</v>
+        <v>-947.55060294</v>
       </c>
       <c r="AQ136">
         <v>-2329.87511666</v>
@@ -38939,7 +38993,7 @@
         <v>55705.15158333984</v>
       </c>
       <c r="AT136">
-        <v>40087.18569706011</v>
+        <v>40087.18569706012</v>
       </c>
       <c r="AU136">
         <v>55705.15158333984</v>
@@ -38954,7 +39008,7 @@
         <v>2.152194399569197</v>
       </c>
       <c r="AY136">
-        <v>1.734064696463947</v>
+        <v>1.734064696463948</v>
       </c>
       <c r="AZ136">
         <v>115.2333333333333</v>
@@ -38963,10 +39017,10 @@
         <v>108.55</v>
       </c>
       <c r="BB136">
-        <v>0.03146441057511846</v>
+        <v>0.0314644105751184</v>
       </c>
       <c r="BC136">
-        <v>0.01388779845003036</v>
+        <v>0.0138877984500303</v>
       </c>
       <c r="BD136">
         <v>-1010.080589137829</v>
@@ -39026,34 +39080,34 @@
         <v>0</v>
       </c>
       <c r="BW136">
-        <v>30144.68919705999</v>
+        <v>30144.68919705998</v>
       </c>
       <c r="BX136">
         <v>45705.15158333995</v>
       </c>
       <c r="BY136">
-        <v>0.04350067991540129</v>
+        <v>0.0435006799154012</v>
       </c>
       <c r="BZ136">
-        <v>0.07252438773486469</v>
+        <v>0.0725243877348646</v>
       </c>
       <c r="CA136">
-        <v>0.09956682142091351</v>
+        <v>0.0995668214209135</v>
       </c>
       <c r="CB136">
-        <v>0.1552798022947827</v>
+        <v>0.1552798022947826</v>
       </c>
       <c r="CC136">
-        <v>0.01351076095108594</v>
+        <v>0.0135107609510859</v>
       </c>
       <c r="CD136">
-        <v>0.009159890304105233</v>
+        <v>0.0091598903041052</v>
       </c>
       <c r="CE136">
-        <v>0.009959032424960084</v>
+        <v>0.009959032424960001</v>
       </c>
       <c r="CF136">
-        <v>0.01079765222490636</v>
+        <v>0.0107976522249063</v>
       </c>
       <c r="CG136">
         <v>31092.23979999998</v>
@@ -39068,28 +39122,28 @@
         <v>48711.52250676807</v>
       </c>
       <c r="CK136">
-        <v>0.1374930576980428</v>
+        <v>0.1374930576980427</v>
       </c>
       <c r="CL136">
-        <v>0.1781842249304145</v>
+        <v>0.1781842249304144</v>
       </c>
       <c r="CM136">
         <v>10000</v>
       </c>
       <c r="CO136">
-        <v>0.003515679932498945</v>
+        <v>0.0035156799324989</v>
       </c>
       <c r="CP136">
-        <v>0.02526601978155909</v>
+        <v>0.025266019781559</v>
       </c>
       <c r="CQ136">
-        <v>12244854.11437261</v>
+        <v>12244854.11437262</v>
       </c>
       <c r="CR136">
         <v>15549669.36335931</v>
       </c>
-      <c r="CS136" s="2">
-        <v>45419.97042807396</v>
+      <c r="CS136" t="s">
+        <v>377</v>
       </c>
       <c r="CT136">
         <v>-0.8182238609422743</v>
@@ -39103,28 +39157,28 @@
         <v>193</v>
       </c>
       <c r="K137">
-        <v>0.001217491149924532</v>
+        <v>0.0012174911499245</v>
       </c>
       <c r="L137">
-        <v>0.0006087455749622661</v>
+        <v>0.0006087455749622</v>
       </c>
       <c r="M137">
-        <v>0.001184876067757301</v>
+        <v>0.0011848760677573</v>
       </c>
       <c r="N137">
-        <v>0.001184876067757301</v>
+        <v>0.0011848760677573</v>
       </c>
       <c r="O137">
-        <v>0.001673189857006729</v>
+        <v>0.0016731898570067</v>
       </c>
       <c r="P137">
-        <v>0.0008365949285033647</v>
+        <v>0.0008365949285033</v>
       </c>
       <c r="Q137">
-        <v>0.001475558980866953</v>
+        <v>0.0014755589808669</v>
       </c>
       <c r="R137">
-        <v>0.001475558980866953</v>
+        <v>0.0014755589808669</v>
       </c>
       <c r="S137">
         <v>22.96755276052317</v>
@@ -39139,7 +39193,7 @@
         <v>0.6490382772370177</v>
       </c>
       <c r="W137">
-        <v>0.03941166836131144</v>
+        <v>0.0394116683613114</v>
       </c>
       <c r="X137">
         <v>0.08420756506361381</v>
@@ -39151,7 +39205,7 @@
         <v>0.1799211959084611</v>
       </c>
       <c r="AA137">
-        <v>0.9993037129652775</v>
+        <v>0.9993037129652776</v>
       </c>
       <c r="AB137">
         <v>0.8135701670258909</v>
@@ -39160,7 +39214,7 @@
         <v>0.8447918632195609</v>
       </c>
       <c r="AD137">
-        <v>0.9989020543192647</v>
+        <v>0.9989020543192648</v>
       </c>
       <c r="AE137">
         <v>0.7622756828827902</v>
@@ -39169,31 +39223,31 @@
         <v>0.8202428385925584</v>
       </c>
       <c r="AG137">
-        <v>0.00531010094103464</v>
+        <v>0.0053101009410346</v>
       </c>
       <c r="AH137">
-        <v>0.007733055159483883</v>
+        <v>0.0077330551594838</v>
       </c>
       <c r="AI137">
-        <v>0.9993037129652775</v>
+        <v>0.9993037129652776</v>
       </c>
       <c r="AJ137">
-        <v>0.9989020543192647</v>
+        <v>0.9989020543192648</v>
       </c>
       <c r="AK137">
-        <v>0.00531010094103464</v>
+        <v>0.0053101009410346</v>
       </c>
       <c r="AL137">
-        <v>0.007733055159483883</v>
+        <v>0.0077330551594838</v>
       </c>
       <c r="AM137" t="s">
         <v>243</v>
       </c>
       <c r="AN137">
-        <v>0.01907285100274631</v>
+        <v>0.0190728510027463</v>
       </c>
       <c r="AO137">
-        <v>0.03386295006012625</v>
+        <v>0.0338629500601262</v>
       </c>
       <c r="AP137">
         <v>-1700.99573232</v>
@@ -39229,13 +39283,13 @@
         <v>119.4</v>
       </c>
       <c r="BA137">
-        <v>96.41666666666667</v>
+        <v>96.41666666666669</v>
       </c>
       <c r="BB137">
-        <v>0.04955123066412238</v>
+        <v>0.0495512306641223</v>
       </c>
       <c r="BC137">
-        <v>0.05917543686255724</v>
+        <v>0.0591754368625572</v>
       </c>
       <c r="BD137">
         <v>-1507.354278834968</v>
@@ -39301,10 +39355,10 @@
         <v>25927.362660864</v>
       </c>
       <c r="BY137">
-        <v>0.03659170191701504</v>
+        <v>0.036591701917015</v>
       </c>
       <c r="BZ137">
-        <v>0.07486011898151482</v>
+        <v>0.0748601189815148</v>
       </c>
       <c r="CA137">
         <v>0.1348926464408769</v>
@@ -39313,16 +39367,16 @@
         <v>0.1523531788027705</v>
       </c>
       <c r="CC137">
-        <v>0.01125470134018188</v>
+        <v>0.0112547013401818</v>
       </c>
       <c r="CD137">
-        <v>0.009550008042014151</v>
+        <v>0.009550008042014099</v>
       </c>
       <c r="CE137">
-        <v>0.00832321001373682</v>
+        <v>0.008323210013736799</v>
       </c>
       <c r="CF137">
-        <v>0.01342814664270862</v>
+        <v>0.0134281466427086</v>
       </c>
       <c r="CG137">
         <v>28912.76361999998</v>
@@ -39346,10 +39400,10 @@
         <v>10000</v>
       </c>
       <c r="CO137">
-        <v>0.002083333333333333</v>
+        <v>0.0020833333333333</v>
       </c>
       <c r="CP137">
-        <v>0.01084104938271605</v>
+        <v>0.010841049382716</v>
       </c>
       <c r="CQ137">
         <v>21761654.04353544</v>
@@ -39357,8 +39411,8 @@
       <c r="CR137">
         <v>8185952.559251163</v>
       </c>
-      <c r="CS137" s="2">
-        <v>45420.18189431339</v>
+      <c r="CS137" t="s">
+        <v>378</v>
       </c>
       <c r="CT137">
         <v>-0.8729982178980289</v>
@@ -39372,28 +39426,28 @@
         <v>218</v>
       </c>
       <c r="K138">
-        <v>0.001616295145627999</v>
+        <v>0.0016162951456279</v>
       </c>
       <c r="L138">
-        <v>0.0008081475728139997</v>
+        <v>0.0008081475728139</v>
       </c>
       <c r="M138">
-        <v>0.0005424826786097903</v>
+        <v>0.0005424826786097</v>
       </c>
       <c r="N138">
-        <v>0.0005424826786097903</v>
+        <v>0.0005424826786097</v>
       </c>
       <c r="O138">
-        <v>0.001638286806134648</v>
+        <v>0.0016382868061346</v>
       </c>
       <c r="P138">
-        <v>0.0008191434030673239</v>
+        <v>0.0008191434030673</v>
       </c>
       <c r="Q138">
-        <v>0.0004939234721387242</v>
+        <v>0.0004939234721387001</v>
       </c>
       <c r="R138">
-        <v>0.0004939234721387242</v>
+        <v>0.0004939234721387001</v>
       </c>
       <c r="S138">
         <v>12.24607067001352</v>
@@ -39408,10 +39462,10 @@
         <v>0.5985076305299992</v>
       </c>
       <c r="W138">
-        <v>0.09974849098706609</v>
+        <v>0.09974849098706599</v>
       </c>
       <c r="X138">
-        <v>0.09922477486083482</v>
+        <v>0.09922477486083479</v>
       </c>
       <c r="Y138">
         <v>0.210038073330966</v>
@@ -39420,7 +39474,7 @@
         <v>0.239814662913279</v>
       </c>
       <c r="AA138">
-        <v>0.9984001233491039</v>
+        <v>0.998400123349104</v>
       </c>
       <c r="AB138">
         <v>0.8308989142500899</v>
@@ -39438,31 +39492,31 @@
         <v>0.7605786850402809</v>
       </c>
       <c r="AG138">
-        <v>0.009786131271804402</v>
+        <v>0.0097861312718044</v>
       </c>
       <c r="AH138">
-        <v>0.01089881053102703</v>
+        <v>0.010898810531027</v>
       </c>
       <c r="AI138">
-        <v>0.9984001233491039</v>
+        <v>0.998400123349104</v>
       </c>
       <c r="AJ138">
         <v>0.9981128241810232</v>
       </c>
       <c r="AK138">
-        <v>0.009786131271804402</v>
+        <v>0.0097861312718044</v>
       </c>
       <c r="AL138">
-        <v>0.01089881053102703</v>
+        <v>0.010898810531027</v>
       </c>
       <c r="AM138" t="s">
         <v>243</v>
       </c>
       <c r="AN138">
-        <v>0.03502844843258101</v>
+        <v>0.035028448432581</v>
       </c>
       <c r="AO138">
-        <v>0.04133791735064998</v>
+        <v>0.0413379173506499</v>
       </c>
       <c r="AP138">
         <v>-1999.707157332</v>
@@ -39501,10 +39555,10 @@
         <v>109.9833333333333</v>
       </c>
       <c r="BB138">
-        <v>0.07403854728522574</v>
+        <v>0.0740385472852257</v>
       </c>
       <c r="BC138">
-        <v>0.003762263843969289</v>
+        <v>0.0037622638439692</v>
       </c>
       <c r="BD138">
         <v>-3927.248035266852</v>
@@ -39570,7 +39624,7 @@
         <v>7952.737229647995</v>
       </c>
       <c r="BY138">
-        <v>0.05108887826035292</v>
+        <v>0.0510888782603529</v>
       </c>
       <c r="BZ138">
         <v>0.1041739946233573</v>
@@ -39582,16 +39636,16 @@
         <v>0.1931574060944746</v>
       </c>
       <c r="CC138">
-        <v>0.01144537069773439</v>
+        <v>0.0114453706977343</v>
       </c>
       <c r="CD138">
-        <v>0.01748469138926716</v>
+        <v>0.0174846913892671</v>
       </c>
       <c r="CE138">
-        <v>0.009081701505211407</v>
+        <v>0.0090817015052114</v>
       </c>
       <c r="CF138">
-        <v>0.01664488388571054</v>
+        <v>0.0166448838857105</v>
       </c>
       <c r="CG138">
         <v>49116.04061999999</v>
@@ -39609,16 +39663,16 @@
         <v>0.165678587720489</v>
       </c>
       <c r="CL138">
-        <v>0.06650993724584395</v>
+        <v>0.06650993724584391</v>
       </c>
       <c r="CM138">
         <v>10000</v>
       </c>
       <c r="CO138">
-        <v>0.008804448563484708</v>
+        <v>0.008804448563484699</v>
       </c>
       <c r="CP138">
-        <v>0.007645968489341983</v>
+        <v>0.0076459684893419</v>
       </c>
       <c r="CQ138">
         <v>22037322.50646456</v>
@@ -39626,8 +39680,8 @@
       <c r="CR138">
         <v>1792741.222718281</v>
       </c>
-      <c r="CS138" s="2">
-        <v>45420.53197429089</v>
+      <c r="CS138" t="s">
+        <v>379</v>
       </c>
       <c r="CT138">
         <v>-0.7176955593761354</v>
@@ -39641,28 +39695,28 @@
         <v>200</v>
       </c>
       <c r="K139">
-        <v>0.0005551911911603202</v>
+        <v>0.0005551911911603</v>
       </c>
       <c r="L139">
-        <v>0.0002775955955801601</v>
+        <v>0.0002775955955801</v>
       </c>
       <c r="M139">
-        <v>0.0004692890892952217</v>
+        <v>0.0004692890892952</v>
       </c>
       <c r="N139">
-        <v>0.0004692890892952217</v>
+        <v>0.0004692890892952</v>
       </c>
       <c r="O139">
-        <v>0.001607036844155463</v>
+        <v>0.0016070368441554</v>
       </c>
       <c r="P139">
-        <v>0.0008035184220777314</v>
+        <v>0.0008035184220777</v>
       </c>
       <c r="Q139">
-        <v>0.000455609683810887</v>
+        <v>0.0004556096838108</v>
       </c>
       <c r="R139">
-        <v>0.000455609683810887</v>
+        <v>0.0004556096838108</v>
       </c>
       <c r="S139">
         <v>29.68776229645795</v>
@@ -39677,13 +39731,13 @@
         <v>0.4971530328389945</v>
       </c>
       <c r="W139">
-        <v>0.0605768602510894</v>
+        <v>0.0605768602510893</v>
       </c>
       <c r="X139">
-        <v>0.07520935172115532</v>
+        <v>0.0752093517211553</v>
       </c>
       <c r="Y139">
-        <v>0.2009656300029838</v>
+        <v>0.2009656300029837</v>
       </c>
       <c r="Z139">
         <v>0.2380676372192553</v>
@@ -39710,7 +39764,7 @@
         <v>0.0063660737988839</v>
       </c>
       <c r="AH139">
-        <v>0.004994708056206319</v>
+        <v>0.0049947080562063</v>
       </c>
       <c r="AI139">
         <v>0.9994369707886128</v>
@@ -39722,16 +39776,16 @@
         <v>0.0063660737988839</v>
       </c>
       <c r="AL139">
-        <v>0.004994708056206319</v>
+        <v>0.0049947080562063</v>
       </c>
       <c r="AM139" t="s">
         <v>243</v>
       </c>
       <c r="AN139">
-        <v>0.009022449129326478</v>
+        <v>0.0090224491293264</v>
       </c>
       <c r="AO139">
-        <v>0.01480636412508247</v>
+        <v>0.0148063641250824</v>
       </c>
       <c r="AP139">
         <v>-1072.4217431</v>
@@ -39761,7 +39815,7 @@
         <v>0.8073245346180815</v>
       </c>
       <c r="AY139">
-        <v>1.641699445632921</v>
+        <v>1.641699445632922</v>
       </c>
       <c r="AZ139">
         <v>93.63333333333334</v>
@@ -39770,16 +39824,16 @@
         <v>86.09999999999999</v>
       </c>
       <c r="BB139">
-        <v>0.05111999284176391</v>
+        <v>0.0511199928417639</v>
       </c>
       <c r="BC139">
-        <v>0.1327208817859857</v>
+        <v>0.1327208817859856</v>
       </c>
       <c r="BD139">
         <v>-453.7983868639545</v>
       </c>
       <c r="BE139">
-        <v>-955.8846815038005</v>
+        <v>-955.8846815038004</v>
       </c>
       <c r="BF139">
         <v>14274</v>
@@ -39842,25 +39896,25 @@
         <v>0.0531108811854462</v>
       </c>
       <c r="BZ139">
-        <v>0.05651699429784502</v>
+        <v>0.056516994297845</v>
       </c>
       <c r="CA139">
         <v>0.1220301622258644</v>
       </c>
       <c r="CB139">
-        <v>0.1921757179627456</v>
+        <v>0.1921757179627455</v>
       </c>
       <c r="CC139">
-        <v>0.01484278818008808</v>
+        <v>0.014842788180088</v>
       </c>
       <c r="CD139">
-        <v>0.008818750494495474</v>
+        <v>0.0088187504944954</v>
       </c>
       <c r="CE139">
-        <v>0.01179606047862717</v>
+        <v>0.0117960604786271</v>
       </c>
       <c r="CF139">
-        <v>0.009930364247942761</v>
+        <v>0.0099303642479427</v>
       </c>
       <c r="CG139">
         <v>8423.323100000011</v>
@@ -39875,19 +39929,19 @@
         <v>7202.217681503791</v>
       </c>
       <c r="CK139">
-        <v>0.07840001921789688</v>
+        <v>0.0784000192178968</v>
       </c>
       <c r="CL139">
-        <v>0.07874972869677671</v>
+        <v>0.0787497286967767</v>
       </c>
       <c r="CM139">
         <v>10000</v>
       </c>
       <c r="CO139">
-        <v>0.001762558227370011</v>
+        <v>0.00176255822737</v>
       </c>
       <c r="CP139">
-        <v>0.001007176129925721</v>
+        <v>0.0010071761299257</v>
       </c>
       <c r="CQ139">
         <v>3389577.188059013</v>
@@ -39895,8 +39949,8 @@
       <c r="CR139">
         <v>4157882.239708048</v>
       </c>
-      <c r="CS139" s="2">
-        <v>45420.74298430007</v>
+      <c r="CS139" t="s">
+        <v>380</v>
       </c>
       <c r="CT139">
         <v>-0.8723102032515645</v>
@@ -39910,28 +39964,28 @@
         <v>221</v>
       </c>
       <c r="K140">
-        <v>0.003718905936362926</v>
+        <v>0.0037189059363629</v>
       </c>
       <c r="L140">
-        <v>0.001859452968181463</v>
+        <v>0.0018594529681814</v>
       </c>
       <c r="M140">
-        <v>0.002110936175253375</v>
+        <v>0.0021109361752533</v>
       </c>
       <c r="N140">
-        <v>0.002110936175253375</v>
+        <v>0.0021109361752533</v>
       </c>
       <c r="O140">
-        <v>0.006998008485984153</v>
+        <v>0.0069980084859841</v>
       </c>
       <c r="P140">
-        <v>0.003499004242992077</v>
+        <v>0.003499004242992</v>
       </c>
       <c r="Q140">
-        <v>0.003058947322889938</v>
+        <v>0.0030589473228899</v>
       </c>
       <c r="R140">
-        <v>0.003058947322889938</v>
+        <v>0.0030589473228899</v>
       </c>
       <c r="S140">
         <v>18.51218872870249</v>
@@ -39946,19 +40000,19 @@
         <v>0.6734776902693198</v>
       </c>
       <c r="W140">
-        <v>0.07930280188374478</v>
+        <v>0.07930280188374469</v>
       </c>
       <c r="X140">
-        <v>0.05421403518520693</v>
+        <v>0.0542140351852069</v>
       </c>
       <c r="Y140">
-        <v>0.1525248830962414</v>
+        <v>0.1525248830962413</v>
       </c>
       <c r="Z140">
-        <v>0.188901023245988</v>
+        <v>0.1889010232459879</v>
       </c>
       <c r="AA140">
-        <v>0.9979202098307671</v>
+        <v>0.9979202098307672</v>
       </c>
       <c r="AB140">
         <v>0.8757283040954551</v>
@@ -39967,7 +40021,7 @@
         <v>0.8502010504998111</v>
       </c>
       <c r="AD140">
-        <v>0.9992838939352033</v>
+        <v>0.9992838939352032</v>
       </c>
       <c r="AE140">
         <v>0.8478141619703143</v>
@@ -39976,31 +40030,31 @@
         <v>0.8028982906883085</v>
       </c>
       <c r="AG140">
-        <v>0.009094062282386057</v>
+        <v>0.009094062282386</v>
       </c>
       <c r="AH140">
-        <v>0.006652001977027054</v>
+        <v>0.006652001977027</v>
       </c>
       <c r="AI140">
-        <v>0.9979202098307671</v>
+        <v>0.9979202098307672</v>
       </c>
       <c r="AJ140">
-        <v>0.9992838939352033</v>
+        <v>0.9992838939352032</v>
       </c>
       <c r="AK140">
-        <v>0.009094062282386057</v>
+        <v>0.009094062282386</v>
       </c>
       <c r="AL140">
-        <v>0.006652001977027054</v>
+        <v>0.006652001977027</v>
       </c>
       <c r="AM140" t="s">
         <v>243</v>
       </c>
       <c r="AN140">
-        <v>0.04867905274594962</v>
+        <v>0.0486790527459496</v>
       </c>
       <c r="AO140">
-        <v>0.03036220516941307</v>
+        <v>0.030362205169413</v>
       </c>
       <c r="AP140">
         <v>-1765.84659052</v>
@@ -40039,10 +40093,10 @@
         <v>78.56666666666666</v>
       </c>
       <c r="BB140">
-        <v>0.001490638169435649</v>
+        <v>0.0014906381694356</v>
       </c>
       <c r="BC140">
-        <v>0.03772158664895737</v>
+        <v>0.0377215866489573</v>
       </c>
       <c r="BD140">
         <v>-75.36571379663336</v>
@@ -40108,10 +40162,10 @@
         <v>17335.24197874002</v>
       </c>
       <c r="BY140">
-        <v>0.05656088652193964</v>
+        <v>0.0565608865219396</v>
       </c>
       <c r="BZ140">
-        <v>0.0615210542963856</v>
+        <v>0.0615210542963855</v>
       </c>
       <c r="CA140">
         <v>0.083091751722095</v>
@@ -40120,19 +40174,19 @@
         <v>0.1631263269236074</v>
       </c>
       <c r="CC140">
-        <v>0.01165736331538616</v>
+        <v>0.0116573633153861</v>
       </c>
       <c r="CD140">
-        <v>0.007804936301286026</v>
+        <v>0.007804936301286</v>
       </c>
       <c r="CE140">
-        <v>0.00931958981462256</v>
+        <v>0.009319589814622499</v>
       </c>
       <c r="CF140">
-        <v>0.009903473811885413</v>
+        <v>0.0099034738118854</v>
       </c>
       <c r="CG140">
-        <v>50483.99559999999</v>
+        <v>50483.9956</v>
       </c>
       <c r="CH140">
         <v>18081.91410000002</v>
@@ -40144,7 +40198,7 @@
         <v>18790.73025968803</v>
       </c>
       <c r="CK140">
-        <v>0.2443133745146321</v>
+        <v>0.244313374514632</v>
       </c>
       <c r="CL140">
         <v>0.2445254674396609</v>
@@ -40153,7 +40207,7 @@
         <v>10000</v>
       </c>
       <c r="CO140">
-        <v>0.007600908614363096</v>
+        <v>0.007600908614363</v>
       </c>
       <c r="CP140">
         <v>0.0078630089114101</v>
@@ -40164,8 +40218,8 @@
       <c r="CR140">
         <v>7172478.294001529</v>
       </c>
-      <c r="CS140" s="2">
-        <v>45420.90591002226</v>
+      <c r="CS140" t="s">
+        <v>381</v>
       </c>
       <c r="CT140">
         <v>-0.5365809810110987</v>
@@ -40179,28 +40233,28 @@
         <v>208</v>
       </c>
       <c r="K141">
-        <v>0.001889330797239408</v>
+        <v>0.0018893307972394</v>
       </c>
       <c r="L141">
-        <v>0.000944665398619704</v>
+        <v>0.0009446653986197</v>
       </c>
       <c r="M141">
-        <v>0.001012125649365148</v>
+        <v>0.0010121256493651</v>
       </c>
       <c r="N141">
-        <v>0.001012125649365148</v>
+        <v>0.0010121256493651</v>
       </c>
       <c r="O141">
-        <v>0.002163337531366749</v>
+        <v>0.0021633375313667</v>
       </c>
       <c r="P141">
-        <v>0.001081668765683375</v>
+        <v>0.0010816687656833</v>
       </c>
       <c r="Q141">
-        <v>0.0009057847951174036</v>
+        <v>0.0009057847951174</v>
       </c>
       <c r="R141">
-        <v>0.0009057847951174036</v>
+        <v>0.0009057847951174</v>
       </c>
       <c r="S141">
         <v>38.96446622169066</v>
@@ -40209,7 +40263,7 @@
         <v>18.38404259423589</v>
       </c>
       <c r="U141">
-        <v>0.3848109461512561</v>
+        <v>0.384810946151256</v>
       </c>
       <c r="V141">
         <v>0.2618970158658526</v>
@@ -40218,7 +40272,7 @@
         <v>0.0510891128087686</v>
       </c>
       <c r="X141">
-        <v>0.08141601234937086</v>
+        <v>0.08141601234937081</v>
       </c>
       <c r="Y141">
         <v>0.2401885115006192</v>
@@ -40227,7 +40281,7 @@
         <v>0.1522426977783748</v>
       </c>
       <c r="AA141">
-        <v>0.9991904239821255</v>
+        <v>0.9991904239821257</v>
       </c>
       <c r="AB141">
         <v>0.8002590982672541</v>
@@ -40236,7 +40290,7 @@
         <v>0.8595760973147339</v>
       </c>
       <c r="AD141">
-        <v>0.9977690736692849</v>
+        <v>0.9977690736692848</v>
       </c>
       <c r="AE141">
         <v>0.7598054036874696</v>
@@ -40245,28 +40299,28 @@
         <v>0.7556757921170245</v>
       </c>
       <c r="AG141">
-        <v>0.006771783071722543</v>
+        <v>0.0067717830717225</v>
       </c>
       <c r="AH141">
-        <v>0.009892196288343594</v>
+        <v>0.009892196288343501</v>
       </c>
       <c r="AI141">
-        <v>0.9991904239821255</v>
+        <v>0.9991904239821257</v>
       </c>
       <c r="AJ141">
-        <v>0.9977690736692849</v>
+        <v>0.9977690736692848</v>
       </c>
       <c r="AK141">
-        <v>0.006771783071722543</v>
+        <v>0.0067717830717225</v>
       </c>
       <c r="AL141">
-        <v>0.009892196288343594</v>
+        <v>0.009892196288343501</v>
       </c>
       <c r="AM141" t="s">
         <v>243</v>
       </c>
       <c r="AN141">
-        <v>0.02620457929351563</v>
+        <v>0.0262045792935156</v>
       </c>
       <c r="AO141">
         <v>0.068528665289134</v>
@@ -40305,13 +40359,13 @@
         <v>64.66666666666667</v>
       </c>
       <c r="BA141">
-        <v>93.46666666666667</v>
+        <v>93.46666666666668</v>
       </c>
       <c r="BB141">
-        <v>0.000261991631371721</v>
+        <v>0.0002619916313717</v>
       </c>
       <c r="BC141">
-        <v>0.04495178928464983</v>
+        <v>0.0449517892846498</v>
       </c>
       <c r="BD141">
         <v>-18.9583280299423</v>
@@ -40377,28 +40431,28 @@
         <v>19820.60039175199</v>
       </c>
       <c r="BY141">
-        <v>0.03269554087442854</v>
+        <v>0.0326955408744285</v>
       </c>
       <c r="BZ141">
         <v>0.0813820812434381</v>
       </c>
       <c r="CA141">
-        <v>0.1365346925870581</v>
+        <v>0.136534692587058</v>
       </c>
       <c r="CB141">
         <v>0.132065655384105</v>
       </c>
       <c r="CC141">
-        <v>0.007910900721258907</v>
+        <v>0.0079109007212589</v>
       </c>
       <c r="CD141">
-        <v>0.01238629491717968</v>
+        <v>0.0123862949171796</v>
       </c>
       <c r="CE141">
-        <v>0.006233454372999068</v>
+        <v>0.006233454372999</v>
       </c>
       <c r="CF141">
-        <v>0.01338162793170816</v>
+        <v>0.0133816279317081</v>
       </c>
       <c r="CG141">
         <v>72343.38367000013</v>
@@ -40425,16 +40479,16 @@
         <v>0.00625</v>
       </c>
       <c r="CP141">
-        <v>0.02650462962962963</v>
+        <v>0.0265046296296296</v>
       </c>
       <c r="CQ141">
-        <v>98712179.16011865</v>
+        <v>98712179.16011864</v>
       </c>
       <c r="CR141">
         <v>10598803.27492217</v>
       </c>
-      <c r="CS141" s="2">
-        <v>45421.22093259679</v>
+      <c r="CS141" t="s">
+        <v>382</v>
       </c>
       <c r="CT141">
         <v>-0.8043091815774359</v>
@@ -40448,31 +40502,31 @@
         <v>213</v>
       </c>
       <c r="K142">
-        <v>0.0009791614490426426</v>
+        <v>0.0009791614490426001</v>
       </c>
       <c r="L142">
-        <v>0.0004895807245213213</v>
+        <v>0.0004895807245213</v>
       </c>
       <c r="M142">
-        <v>0.0002051275288859067</v>
+        <v>0.0002051275288859</v>
       </c>
       <c r="N142">
-        <v>0.0002051275288859067</v>
+        <v>0.0002051275288859</v>
       </c>
       <c r="O142">
-        <v>0.001373646392256345</v>
+        <v>0.0013736463922563</v>
       </c>
       <c r="P142">
-        <v>0.0006868231961281723</v>
+        <v>0.0006868231961281</v>
       </c>
       <c r="Q142">
-        <v>0.0002866132170945779</v>
+        <v>0.0002866132170945</v>
       </c>
       <c r="R142">
-        <v>0.0002866132170945779</v>
+        <v>0.0002866132170945</v>
       </c>
       <c r="S142">
-        <v>25.53852094999035</v>
+        <v>25.53852094999034</v>
       </c>
       <c r="T142">
         <v>10.97169337709983</v>
@@ -40484,13 +40538,13 @@
         <v>0.5515009125369736</v>
       </c>
       <c r="W142">
-        <v>0.01994749617820258</v>
+        <v>0.0199474961782025</v>
       </c>
       <c r="X142">
-        <v>0.02326205019476134</v>
+        <v>0.0232620501947613</v>
       </c>
       <c r="Y142">
-        <v>0.1075313106787391</v>
+        <v>0.107531310678739</v>
       </c>
       <c r="Z142">
         <v>0.2443951890819016</v>
@@ -40499,10 +40553,10 @@
         <v>0.9996573305302862</v>
       </c>
       <c r="AB142">
-        <v>0.9029732090806061</v>
+        <v>0.902973209080606</v>
       </c>
       <c r="AC142">
-        <v>0.9220750597495151</v>
+        <v>0.9220750597495152</v>
       </c>
       <c r="AD142">
         <v>0.9994682435618946</v>
@@ -40514,10 +40568,10 @@
         <v>0.6751199983546743</v>
       </c>
       <c r="AG142">
-        <v>0.003006973066287996</v>
+        <v>0.0030069730662879</v>
       </c>
       <c r="AH142">
-        <v>0.003284008719121437</v>
+        <v>0.0032840087191214</v>
       </c>
       <c r="AI142">
         <v>0.9996573305302862</v>
@@ -40526,19 +40580,19 @@
         <v>0.9994682435618946</v>
       </c>
       <c r="AK142">
-        <v>0.003006973066287996</v>
+        <v>0.0030069730662879</v>
       </c>
       <c r="AL142">
-        <v>0.003284008719121437</v>
+        <v>0.0032840087191214</v>
       </c>
       <c r="AM142" t="s">
         <v>243</v>
       </c>
       <c r="AN142">
-        <v>0.01102459909290902</v>
+        <v>0.011024599092909</v>
       </c>
       <c r="AO142">
-        <v>0.01107060651290055</v>
+        <v>0.0110706065129005</v>
       </c>
       <c r="AP142">
         <v>-3178.4995556</v>
@@ -40562,10 +40616,10 @@
         <v>1.874726424439966</v>
       </c>
       <c r="AW142">
-        <v>0.2476993805520167</v>
+        <v>0.2476993805520166</v>
       </c>
       <c r="AX142">
-        <v>0.9385503617139677</v>
+        <v>0.9385503617139676</v>
       </c>
       <c r="AY142">
         <v>2.184575202050069</v>
@@ -40577,10 +40631,10 @@
         <v>111.15</v>
       </c>
       <c r="BB142">
-        <v>0.0009090456825400375</v>
+        <v>0.00090904568254</v>
       </c>
       <c r="BC142">
-        <v>0.02047830360591597</v>
+        <v>0.0204783036059159</v>
       </c>
       <c r="BD142">
         <v>-19.949656067499</v>
@@ -40640,37 +40694,37 @@
         <v>0</v>
       </c>
       <c r="BW142">
-        <v>18747.26424440003</v>
+        <v>18747.26424440004</v>
       </c>
       <c r="BX142">
         <v>2476.993805520001</v>
       </c>
       <c r="BY142">
-        <v>0.0282675234131565</v>
+        <v>0.0282675234131564</v>
       </c>
       <c r="BZ142">
         <v>0.133234483195606</v>
       </c>
       <c r="CA142">
-        <v>0.05732285058476774</v>
+        <v>0.0573228505847677</v>
       </c>
       <c r="CB142">
         <v>0.2358065693923901</v>
       </c>
       <c r="CC142">
-        <v>0.01049894086122908</v>
+        <v>0.010498940861229</v>
       </c>
       <c r="CD142">
-        <v>0.02191929943834858</v>
+        <v>0.0219192994383485</v>
       </c>
       <c r="CE142">
-        <v>0.007419192349491326</v>
+        <v>0.0074191923494913</v>
       </c>
       <c r="CF142">
-        <v>0.02274835599314671</v>
+        <v>0.0227483559931467</v>
       </c>
       <c r="CG142">
-        <v>21925.76380000003</v>
+        <v>21925.76380000004</v>
       </c>
       <c r="CH142">
         <v>2733.960800000001</v>
@@ -40685,16 +40739,16 @@
         <v>0.1424579767085579</v>
       </c>
       <c r="CL142">
-        <v>0.07385941677269116</v>
+        <v>0.0738594167726911</v>
       </c>
       <c r="CM142">
         <v>10000</v>
       </c>
       <c r="CO142">
-        <v>0.002239728143342601</v>
+        <v>0.0022397281433426</v>
       </c>
       <c r="CP142">
-        <v>0.001544640098856966</v>
+        <v>0.0015446400988569</v>
       </c>
       <c r="CQ142">
         <v>21946958.71626803</v>
@@ -40702,14 +40756,283 @@
       <c r="CR142">
         <v>1954441.87495541</v>
       </c>
-      <c r="CS142" s="2">
-        <v>45421.43573098649</v>
+      <c r="CS142" t="s">
+        <v>383</v>
       </c>
       <c r="CT142">
         <v>-0.892071333585829</v>
       </c>
       <c r="CU142">
         <v>-0.9702031259092914</v>
+      </c>
+    </row>
+    <row r="143" spans="10:99">
+      <c r="J143" t="s">
+        <v>229</v>
+      </c>
+      <c r="K143">
+        <v>0.00193214450120216</v>
+      </c>
+      <c r="L143">
+        <v>0.0009660722506010799</v>
+      </c>
+      <c r="M143">
+        <v>8.37950510610419E-05</v>
+      </c>
+      <c r="N143">
+        <v>8.37950510610419E-05</v>
+      </c>
+      <c r="O143">
+        <v>0.002643764250178249</v>
+      </c>
+      <c r="P143">
+        <v>0.001321882125089124</v>
+      </c>
+      <c r="Q143">
+        <v>-0.0004705800614115407</v>
+      </c>
+      <c r="R143">
+        <v>-0.0004705800614115407</v>
+      </c>
+      <c r="S143">
+        <v>50.66954867715718</v>
+      </c>
+      <c r="T143">
+        <v>2.476569254712087</v>
+      </c>
+      <c r="U143">
+        <v>0.356953318363645</v>
+      </c>
+      <c r="V143">
+        <v>0.6609584430027773</v>
+      </c>
+      <c r="W143">
+        <v>0.08817679151966575</v>
+      </c>
+      <c r="X143">
+        <v>0.1937966801738117</v>
+      </c>
+      <c r="Y143">
+        <v>0.2165157390776833</v>
+      </c>
+      <c r="Z143">
+        <v>0.2357281216500317</v>
+      </c>
+      <c r="AA143">
+        <v>0.9988163507549001</v>
+      </c>
+      <c r="AB143">
+        <v>0.8413080191888497</v>
+      </c>
+      <c r="AC143">
+        <v>0.9559177821172404</v>
+      </c>
+      <c r="AD143">
+        <v>0.9988410574348235</v>
+      </c>
+      <c r="AE143">
+        <v>0.7835828345029785</v>
+      </c>
+      <c r="AF143">
+        <v>0.9077416915928269</v>
+      </c>
+      <c r="AG143">
+        <v>0.008083679347870168</v>
+      </c>
+      <c r="AH143">
+        <v>0.004292438417556189</v>
+      </c>
+      <c r="AI143">
+        <v>0.9988163507549001</v>
+      </c>
+      <c r="AJ143">
+        <v>0.9988410574348235</v>
+      </c>
+      <c r="AK143">
+        <v>0.008083679347870168</v>
+      </c>
+      <c r="AL143">
+        <v>0.004292438417556189</v>
+      </c>
+      <c r="AM143" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN143">
+        <v>0.0289399933126468</v>
+      </c>
+      <c r="AO143">
+        <v>0.06509103312343041</v>
+      </c>
+      <c r="AP143">
+        <v>-6448.347372574</v>
+      </c>
+      <c r="AQ143">
+        <v>-403.47856664</v>
+      </c>
+      <c r="AR143">
+        <v>64267.47037742582</v>
+      </c>
+      <c r="AS143">
+        <v>10841.11849335998</v>
+      </c>
+      <c r="AT143">
+        <v>64231.39955742582</v>
+      </c>
+      <c r="AU143">
+        <v>10841.29425335998</v>
+      </c>
+      <c r="AV143">
+        <v>5.426747037742582</v>
+      </c>
+      <c r="AW143">
+        <v>0.08411184933599802</v>
+      </c>
+      <c r="AX143">
+        <v>0.4730584677969804</v>
+      </c>
+      <c r="AY143">
+        <v>9.689249790444258</v>
+      </c>
+      <c r="AZ143">
+        <v>93.43333333333334</v>
+      </c>
+      <c r="BA143">
+        <v>266.1</v>
+      </c>
+      <c r="BB143">
+        <v>0.02197118240507638</v>
+      </c>
+      <c r="BC143">
+        <v>0.9424083587269209</v>
+      </c>
+      <c r="BD143">
+        <v>-1363.966258109926</v>
+      </c>
+      <c r="BE143">
+        <v>-20366.12686603919</v>
+      </c>
+      <c r="BF143">
+        <v>21450</v>
+      </c>
+      <c r="BG143">
+        <v>1014</v>
+      </c>
+      <c r="BH143">
+        <v>963.8333333333334</v>
+      </c>
+      <c r="BI143">
+        <v>27387</v>
+      </c>
+      <c r="BJ143">
+        <v>1373</v>
+      </c>
+      <c r="BK143">
+        <v>48837</v>
+      </c>
+      <c r="BL143">
+        <v>2387</v>
+      </c>
+      <c r="BM143">
+        <v>20856</v>
+      </c>
+      <c r="BN143">
+        <v>530</v>
+      </c>
+      <c r="BO143">
+        <v>21434</v>
+      </c>
+      <c r="BP143">
+        <v>929</v>
+      </c>
+      <c r="BQ143">
+        <v>6531</v>
+      </c>
+      <c r="BR143">
+        <v>843</v>
+      </c>
+      <c r="BS143">
+        <v>16</v>
+      </c>
+      <c r="BT143">
+        <v>85</v>
+      </c>
+      <c r="BU143">
+        <v>0</v>
+      </c>
+      <c r="BV143">
+        <v>0</v>
+      </c>
+      <c r="BW143">
+        <v>54267.47037742598</v>
+      </c>
+      <c r="BX143">
+        <v>841.1184933599964</v>
+      </c>
+      <c r="BY143">
+        <v>0.0424123549502184</v>
+      </c>
+      <c r="BZ143">
+        <v>0.08953268876482108</v>
+      </c>
+      <c r="CA143">
+        <v>0.1213054764188839</v>
+      </c>
+      <c r="CB143">
+        <v>0.1236047181424523</v>
+      </c>
+      <c r="CC143">
+        <v>0.008536267636315162</v>
+      </c>
+      <c r="CD143">
+        <v>0.0197220836342179</v>
+      </c>
+      <c r="CE143">
+        <v>0.006691607230672424</v>
+      </c>
+      <c r="CF143">
+        <v>0.015544617392975</v>
+      </c>
+      <c r="CG143">
+        <v>60715.81774999998</v>
+      </c>
+      <c r="CH143">
+        <v>1244.597059999996</v>
+      </c>
+      <c r="CI143">
+        <v>62079.78400810991</v>
+      </c>
+      <c r="CJ143">
+        <v>21610.72392603919</v>
+      </c>
+      <c r="CK143">
+        <v>0.2258812048432976</v>
+      </c>
+      <c r="CL143">
+        <v>0.01207027251126699</v>
+      </c>
+      <c r="CM143">
+        <v>10000</v>
+      </c>
+      <c r="CO143">
+        <v>0.01110967016815804</v>
+      </c>
+      <c r="CP143">
+        <v>0.0001296848657761639</v>
+      </c>
+      <c r="CQ143">
+        <v>33087506.84221106</v>
+      </c>
+      <c r="CR143">
+        <v>2325567.261086872</v>
+      </c>
+      <c r="CS143" s="2">
+        <v>45422.03995614562</v>
+      </c>
+      <c r="CT143">
+        <v>-0.7586823863673019</v>
+      </c>
+      <c r="CU143">
+        <v>-0.6309820022477655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update SNXUSDT.json at 2024-05-10_12-33-42 bestfile_scores 0.0007361347603016099 bestfile_sharp 0.1295939074773077
</commit_message>
<xml_diff>
--- a/optimized/logs/analysis.xlsx
+++ b/optimized/logs/analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="384">
   <si>
     <t>Unnamed: 0.8</t>
   </si>
@@ -1527,7 +1527,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CU143"/>
+  <dimension ref="A1:CU144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:99">
@@ -41033,6 +41033,275 @@
       </c>
       <c r="CU143">
         <v>-0.6309820022477655</v>
+      </c>
+    </row>
+    <row r="144" spans="10:99">
+      <c r="J144" t="s">
+        <v>232</v>
+      </c>
+      <c r="K144">
+        <v>0.0008564447837671185</v>
+      </c>
+      <c r="L144">
+        <v>0.0004282223918835593</v>
+      </c>
+      <c r="M144">
+        <v>0.001230368064804921</v>
+      </c>
+      <c r="N144">
+        <v>0.001230368064804921</v>
+      </c>
+      <c r="O144">
+        <v>0.001039794012279516</v>
+      </c>
+      <c r="P144">
+        <v>0.0005198970061397578</v>
+      </c>
+      <c r="Q144">
+        <v>0.001018571938302215</v>
+      </c>
+      <c r="R144">
+        <v>0.001018571938302215</v>
+      </c>
+      <c r="S144">
+        <v>21.20378451438502</v>
+      </c>
+      <c r="T144">
+        <v>8.456304305850551</v>
+      </c>
+      <c r="U144">
+        <v>0.3993724528347143</v>
+      </c>
+      <c r="V144">
+        <v>0.4911138929337072</v>
+      </c>
+      <c r="W144">
+        <v>0.03070961689024167</v>
+      </c>
+      <c r="X144">
+        <v>0.05885322586989666</v>
+      </c>
+      <c r="Y144">
+        <v>0.09035268331842589</v>
+      </c>
+      <c r="Z144">
+        <v>0.2159920043500735</v>
+      </c>
+      <c r="AA144">
+        <v>0.999266920953653</v>
+      </c>
+      <c r="AB144">
+        <v>0.9267249864417888</v>
+      </c>
+      <c r="AC144">
+        <v>0.8399637340489251</v>
+      </c>
+      <c r="AD144">
+        <v>0.9988521374689359</v>
+      </c>
+      <c r="AE144">
+        <v>0.8893059015420908</v>
+      </c>
+      <c r="AF144">
+        <v>0.7841648299790046</v>
+      </c>
+      <c r="AG144">
+        <v>0.003520479632482199</v>
+      </c>
+      <c r="AH144">
+        <v>0.006649957649046283</v>
+      </c>
+      <c r="AI144">
+        <v>0.999266920953653</v>
+      </c>
+      <c r="AJ144">
+        <v>0.9988521374689359</v>
+      </c>
+      <c r="AK144">
+        <v>0.003520479632482199</v>
+      </c>
+      <c r="AL144">
+        <v>0.006649957649046283</v>
+      </c>
+      <c r="AM144" t="s">
+        <v>243</v>
+      </c>
+      <c r="AN144">
+        <v>0.01737508200941965</v>
+      </c>
+      <c r="AO144">
+        <v>0.04850452589890775</v>
+      </c>
+      <c r="AP144">
+        <v>-1262.02125008</v>
+      </c>
+      <c r="AQ144">
+        <v>-1894.94275446</v>
+      </c>
+      <c r="AR144">
+        <v>25185.23344992034</v>
+      </c>
+      <c r="AS144">
+        <v>37685.86054554013</v>
+      </c>
+      <c r="AT144">
+        <v>25007.92934992034</v>
+      </c>
+      <c r="AU144">
+        <v>37685.86054554013</v>
+      </c>
+      <c r="AV144">
+        <v>1.518523344992034</v>
+      </c>
+      <c r="AW144">
+        <v>2.768586054554013</v>
+      </c>
+      <c r="AX144">
+        <v>1.12935699610963</v>
+      </c>
+      <c r="AY144">
+        <v>2.8312762614637</v>
+      </c>
+      <c r="AZ144">
+        <v>119.3833333333333</v>
+      </c>
+      <c r="BA144">
+        <v>117.7166666666667</v>
+      </c>
+      <c r="BB144">
+        <v>0.02820468021647839</v>
+      </c>
+      <c r="BC144">
+        <v>0.04794759988816061</v>
+      </c>
+      <c r="BD144">
+        <v>-477.3531522623584</v>
+      </c>
+      <c r="BE144">
+        <v>-1489.758883893541</v>
+      </c>
+      <c r="BF144">
+        <v>10115</v>
+      </c>
+      <c r="BG144">
+        <v>4759</v>
+      </c>
+      <c r="BH144">
+        <v>1078.958333333333</v>
+      </c>
+      <c r="BI144">
+        <v>12763</v>
+      </c>
+      <c r="BJ144">
+        <v>4365</v>
+      </c>
+      <c r="BK144">
+        <v>22878</v>
+      </c>
+      <c r="BL144">
+        <v>9124</v>
+      </c>
+      <c r="BM144">
+        <v>9937</v>
+      </c>
+      <c r="BN144">
+        <v>3357</v>
+      </c>
+      <c r="BO144">
+        <v>10086</v>
+      </c>
+      <c r="BP144">
+        <v>4706</v>
+      </c>
+      <c r="BQ144">
+        <v>2826</v>
+      </c>
+      <c r="BR144">
+        <v>1008</v>
+      </c>
+      <c r="BS144">
+        <v>29</v>
+      </c>
+      <c r="BT144">
+        <v>53</v>
+      </c>
+      <c r="BU144">
+        <v>0</v>
+      </c>
+      <c r="BV144">
+        <v>0</v>
+      </c>
+      <c r="BW144">
+        <v>15185.23344991998</v>
+      </c>
+      <c r="BX144">
+        <v>27685.86054553998</v>
+      </c>
+      <c r="BY144">
+        <v>0.05510436529948603</v>
+      </c>
+      <c r="BZ144">
+        <v>0.05486713722109745</v>
+      </c>
+      <c r="CA144">
+        <v>0.130912942887533</v>
+      </c>
+      <c r="CB144">
+        <v>0.1774896195509062</v>
+      </c>
+      <c r="CC144">
+        <v>0.01233236703338586</v>
+      </c>
+      <c r="CD144">
+        <v>0.0137071162315677</v>
+      </c>
+      <c r="CE144">
+        <v>0.009716525330802424</v>
+      </c>
+      <c r="CF144">
+        <v>0.01141596959170899</v>
+      </c>
+      <c r="CG144">
+        <v>16447.25469999998</v>
+      </c>
+      <c r="CH144">
+        <v>29580.80329999999</v>
+      </c>
+      <c r="CI144">
+        <v>16924.60785226234</v>
+      </c>
+      <c r="CJ144">
+        <v>31070.56218389353</v>
+      </c>
+      <c r="CK144">
+        <v>0.1782274277623392</v>
+      </c>
+      <c r="CL144">
+        <v>0.134202331601194</v>
+      </c>
+      <c r="CM144">
+        <v>10000</v>
+      </c>
+      <c r="CO144">
+        <v>0.0001930800123571208</v>
+      </c>
+      <c r="CP144">
+        <v>0.01865152919369787</v>
+      </c>
+      <c r="CQ144">
+        <v>6384727.126174739</v>
+      </c>
+      <c r="CR144">
+        <v>17826610.98082536</v>
+      </c>
+      <c r="CS144" s="2">
+        <v>45422.29376685802</v>
+      </c>
+      <c r="CT144">
+        <v>-0.9111405881388873</v>
+      </c>
+      <c r="CU144">
+        <v>-0.7572294378445733</v>
       </c>
     </row>
   </sheetData>

</xml_diff>